<commit_message>
Update clean template (master_template_custom.xlsx) without baked-in images
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82D3C60-F672-496C-ABD6-7110C327D5E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ACDF7D1-95D0-46A0-A9AD-70C65F9748F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="harga satuan terpakai" sheetId="8" r:id="rId1"/>
@@ -428,134 +428,27 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color rgb="FFFFC000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color rgb="FFFFC000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <font>
         <b/>
@@ -607,6 +500,65 @@
       </border>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color rgb="FFFFC000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i/>
@@ -629,153 +581,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>37141</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>129540</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>555173</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1504411</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>75337</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>126902</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>511339</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>126688</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="155548" y="126902"/>
-          <a:ext cx="12998975" cy="1874707"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>15240</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>53339</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>908798</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>21771</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="102326" y="53339"/>
-          <a:ext cx="10364129" cy="1535975"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1111,37 +916,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -1149,10 +954,10 @@
       <c r="B5" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="60" t="s">
+      <c r="C5" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="60"/>
+      <c r="D5" s="59"/>
       <c r="E5" s="11" t="s">
         <v>4</v>
       </c>
@@ -9506,13 +9311,12 @@
     <mergeCell ref="C5:D5"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="14" priority="2">
+    <cfRule type="expression" dxfId="9" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="10000" scale="49" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -9541,48 +9345,48 @@
     <row r="1" spans="2:14" ht="147.6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:14" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:14" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="56" t="s">
+      <c r="B3" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="56"/>
-      <c r="N3" s="56"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="57"/>
+      <c r="L3" s="57"/>
+      <c r="M3" s="57"/>
+      <c r="N3" s="57"/>
     </row>
     <row r="4" spans="2:14" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="57" t="s">
+      <c r="B4" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="57"/>
-      <c r="J4" s="57"/>
-      <c r="K4" s="57"/>
-      <c r="L4" s="57"/>
-      <c r="M4" s="57"/>
-      <c r="N4" s="57"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="58"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="58"/>
     </row>
     <row r="5" spans="2:14" ht="7.2" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="6" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="58" t="s">
+      <c r="C6" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="58"/>
+      <c r="D6" s="60"/>
       <c r="E6" s="38" t="s">
         <v>18</v>
       </c>
@@ -11748,26 +11552,25 @@
     <cfRule type="expression" dxfId="7" priority="3">
       <formula>$C7&lt;&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="5">
+    <cfRule type="expression" dxfId="6" priority="4">
+      <formula>AND(LEN($B7)=1,$D7&lt;&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="5">
       <formula>AND(LEN($B7)&lt;&gt;0,$D7&lt;&gt;0)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="5" priority="4">
-      <formula>AND(LEN($B7)=1,$D7&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:H16998">
-    <cfRule type="expression" dxfId="10" priority="8">
+    <cfRule type="expression" dxfId="4" priority="8">
       <formula>IF(G7&lt;&gt;"", NOT(AND(OR(LEFT($E7,2)="L.", LEFT($E7,2)="A.", LEFT($E7,2)="B.", LEFT($E7,2)="M."), $H7&lt;&gt;"", $E7&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:K16998">
-    <cfRule type="notContainsBlanks" dxfId="9" priority="7">
+    <cfRule type="notContainsBlanks" dxfId="3" priority="7">
       <formula>LEN(TRIM(H7))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="10000" scale="44" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -11794,26 +11597,26 @@
       <c r="G2" s="52"/>
     </row>
     <row r="3" spans="2:10" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="56" t="s">
+      <c r="B3" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
     </row>
     <row r="4" spans="2:10" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="57" t="s">
+      <c r="B4" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
     </row>
     <row r="5" spans="2:10" ht="8.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G5" s="52"/>
@@ -35860,20 +35663,19 @@
     <mergeCell ref="B4:H4"/>
   </mergeCells>
   <conditionalFormatting sqref="B7:B996 E7:H996">
-    <cfRule type="expression" dxfId="13" priority="6">
+    <cfRule type="expression" dxfId="2" priority="6">
       <formula>$J7=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:H996">
-    <cfRule type="expression" dxfId="12" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>AND(LEN($B7)=1,$C7&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>$C7&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="55" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update: Shift data start to Row 6 and adjust header logic due to Row 2 deletion in template
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ACDF7D1-95D0-46A0-A9AD-70C65F9748F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{167D0C76-2304-47F0-9E16-6226E9691BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <definedName name="_xlnm.Print_Area" localSheetId="1">ahsp!$A1:$O16326</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'harga satuan terpakai'!$A1:$J2646</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">hsp!$A1:$I2674</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">ahsp!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">hsp!$1:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">ahsp!$1:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">hsp!$1:$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -69,9 +69,6 @@
     <t>HSP (HARGA SATUAN PEKERJAAN)</t>
   </si>
   <si>
-    <t>Surat Edaran Direktur Jenderal Bina Konstruksi Nomor 182/SE/Dk/2025</t>
-  </si>
-  <si>
     <t>Kode AHSP-CK</t>
   </si>
   <si>
@@ -118,6 +115,9 @@
   </si>
   <si>
     <t>TOTAL HARGA</t>
+  </si>
+  <si>
+    <t>AHSP CIPTA KARYA SE BINA KONSTRUKSI SE DJBK NO 47 TAHUN 2026</t>
   </si>
 </sst>
 </file>
@@ -428,13 +428,13 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -916,37 +916,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -9322,7 +9322,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="B1:S5014"/>
+  <dimension ref="B1:S5013"/>
   <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="1.21875" customWidth="1"/>
@@ -9343,10 +9343,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:14" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:14" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:14" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="56" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="M2" s="56"/>
+      <c r="N2" s="56"/>
+    </row>
+    <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="57" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C3" s="57"/>
       <c r="D3" s="57"/>
@@ -9361,62 +9377,60 @@
       <c r="M3" s="57"/>
       <c r="N3" s="57"/>
     </row>
-    <row r="4" spans="2:14" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="58" t="s">
-        <v>10</v>
+    <row r="4" spans="2:14" ht="7.2" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="38" t="s">
+        <v>15</v>
       </c>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
-      <c r="J4" s="58"/>
-      <c r="K4" s="58"/>
-      <c r="L4" s="58"/>
-      <c r="M4" s="58"/>
-      <c r="N4" s="58"/>
-    </row>
-    <row r="5" spans="2:14" ht="7.2" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="38" t="s">
+      <c r="C5" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="60" t="s">
+      <c r="D5" s="60"/>
+      <c r="E5" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="60"/>
-      <c r="E6" s="38" t="s">
+      <c r="F5" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="38" t="s">
+      <c r="G5" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="39" t="s">
+      <c r="H5" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="40" t="s">
+      <c r="I5" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="40" t="s">
+      <c r="J5" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="J6" s="40" t="s">
+      <c r="K5" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="K6" s="40" t="s">
+      <c r="L5" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="L6" s="41" t="s">
+      <c r="M5" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="40" t="s">
-        <v>26</v>
-      </c>
-      <c r="N6" s="41" t="s">
+      <c r="N5" s="41" t="s">
         <v>8</v>
       </c>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="45"/>
+      <c r="H6" s="46"/>
+      <c r="I6" s="46"/>
+      <c r="J6" s="46"/>
+      <c r="K6" s="46"/>
+      <c r="L6" s="47"/>
+      <c r="M6" s="46"/>
+      <c r="N6" s="47"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B7" s="42"/>
@@ -11488,26 +11502,14 @@
       <c r="M144" s="46"/>
       <c r="N144" s="47"/>
     </row>
-    <row r="145" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B145" s="42"/>
-      <c r="C145" s="42"/>
-      <c r="D145" s="43"/>
-      <c r="E145" s="44"/>
-      <c r="F145" s="44"/>
-      <c r="G145" s="45"/>
-      <c r="H145" s="46"/>
-      <c r="I145" s="46"/>
-      <c r="J145" s="46"/>
-      <c r="K145" s="46"/>
-      <c r="L145" s="47"/>
-      <c r="M145" s="46"/>
-      <c r="N145" s="47"/>
-    </row>
-    <row r="2633" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D2633" s="48"/>
-    </row>
-    <row r="4861" spans="19:19" x14ac:dyDescent="0.3">
-      <c r="S4861" s="49"/>
+    <row r="2632" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D2632" s="48"/>
+    </row>
+    <row r="4860" spans="19:19" x14ac:dyDescent="0.3">
+      <c r="S4860" s="49"/>
+    </row>
+    <row r="4877" spans="17:17" x14ac:dyDescent="0.3">
+      <c r="Q4877" s="49"/>
     </row>
     <row r="4878" spans="17:17" x14ac:dyDescent="0.3">
       <c r="Q4878" s="49"/>
@@ -11524,49 +11526,46 @@
     <row r="4882" spans="17:17" x14ac:dyDescent="0.3">
       <c r="Q4882" s="49"/>
     </row>
-    <row r="4883" spans="17:17" x14ac:dyDescent="0.3">
-      <c r="Q4883" s="49"/>
+    <row r="4884" spans="17:17" x14ac:dyDescent="0.3">
+      <c r="Q4884" s="49"/>
     </row>
     <row r="4885" spans="17:17" x14ac:dyDescent="0.3">
       <c r="Q4885" s="49"/>
     </row>
-    <row r="4886" spans="17:17" x14ac:dyDescent="0.3">
-      <c r="Q4886" s="49"/>
-    </row>
-    <row r="5009" spans="17:19" x14ac:dyDescent="0.3">
-      <c r="S5009" s="49"/>
-    </row>
-    <row r="5014" spans="17:19" x14ac:dyDescent="0.3">
-      <c r="Q5014" s="49"/>
+    <row r="5008" spans="19:19" x14ac:dyDescent="0.3">
+      <c r="S5008" s="49"/>
+    </row>
+    <row r="5013" spans="17:17" x14ac:dyDescent="0.3">
+      <c r="Q5013" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="B2:N2"/>
     <mergeCell ref="B3:N3"/>
-    <mergeCell ref="B4:N4"/>
-    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C5:D5"/>
   </mergeCells>
-  <conditionalFormatting sqref="B7:N16998">
+  <conditionalFormatting sqref="B6:N16997">
     <cfRule type="expression" dxfId="8" priority="1">
-      <formula>AND(LEN($B7)=1,$C7&lt;&gt;0)</formula>
+      <formula>AND(LEN($B6)=1,$C6&lt;&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="7" priority="3">
-      <formula>$C7&lt;&gt;0</formula>
+      <formula>$C6&lt;&gt;0</formula>
     </cfRule>
     <cfRule type="expression" dxfId="6" priority="4">
-      <formula>AND(LEN($B7)=1,$D7&lt;&gt;0)</formula>
+      <formula>AND(LEN($B6)=1,$D6&lt;&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="5" priority="5">
-      <formula>AND(LEN($B7)&lt;&gt;0,$D7&lt;&gt;0)</formula>
+      <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7:H16998">
+  <conditionalFormatting sqref="H6:H16997">
     <cfRule type="expression" dxfId="4" priority="8">
-      <formula>IF(G7&lt;&gt;"", NOT(AND(OR(LEFT($E7,2)="L.", LEFT($E7,2)="A.", LEFT($E7,2)="B.", LEFT($E7,2)="M."), $H7&lt;&gt;"", $E7&lt;&gt;"")),FALSE)</formula>
+      <formula>IF(G6&lt;&gt;"", NOT(AND(OR(LEFT($E6,2)="L.", LEFT($E6,2)="A.", LEFT($E6,2)="B.", LEFT($E6,2)="M."), $H6&lt;&gt;"", $E6&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7:K16998">
+  <conditionalFormatting sqref="H6:K16997">
     <cfRule type="notContainsBlanks" dxfId="3" priority="7">
-      <formula>LEN(TRIM(H7))&gt;0</formula>
+      <formula>LEN(TRIM(H6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -11576,7 +11575,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B1:J2674"/>
+  <dimension ref="B1:J2673"/>
   <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="1.33203125" customWidth="1"/>
@@ -11593,12 +11592,20 @@
     <row r="1" spans="2:10" ht="123" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G1" s="52"/>
     </row>
-    <row r="2" spans="2:10" ht="6.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G2" s="52"/>
-    </row>
-    <row r="3" spans="2:10" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:10" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="56" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+    </row>
+    <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="57" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="C3" s="57"/>
       <c r="D3" s="57"/>
@@ -11607,43 +11614,41 @@
       <c r="G3" s="57"/>
       <c r="H3" s="57"/>
     </row>
-    <row r="4" spans="2:10" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="58" t="s">
+    <row r="4" spans="2:10" ht="8.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G4" s="52"/>
+    </row>
+    <row r="5" spans="2:10" s="5" customFormat="1" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-    </row>
-    <row r="5" spans="2:10" ht="8.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G5" s="52"/>
-    </row>
-    <row r="6" spans="2:10" s="5" customFormat="1" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="27" t="s">
+      <c r="C5" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="D5" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="27" t="s">
-        <v>3</v>
+      <c r="G5" s="50" t="s">
+        <v>8</v>
       </c>
-      <c r="E6" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="F6" s="28" t="s">
+      <c r="H5" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="50" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="J6" s="29"/>
+      <c r="J5" s="29"/>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B6" s="30"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="53"/>
+      <c r="H6" s="33"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B7" s="30"/>
@@ -11652,7 +11657,7 @@
       <c r="E7" s="32"/>
       <c r="F7" s="33"/>
       <c r="G7" s="53"/>
-      <c r="H7" s="33"/>
+      <c r="H7" s="34"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B8" s="30"/>
@@ -11661,7 +11666,7 @@
       <c r="E8" s="32"/>
       <c r="F8" s="33"/>
       <c r="G8" s="53"/>
-      <c r="H8" s="34"/>
+      <c r="H8" s="33"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B9" s="30"/>
@@ -11669,7 +11674,7 @@
       <c r="D9" s="30"/>
       <c r="E9" s="32"/>
       <c r="F9" s="33"/>
-      <c r="G9" s="53"/>
+      <c r="G9" s="54"/>
       <c r="H9" s="33"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.3">
@@ -35635,7 +35640,7 @@
       <c r="C2672" s="31"/>
       <c r="D2672" s="30"/>
       <c r="E2672" s="32"/>
-      <c r="F2672" s="33"/>
+      <c r="F2672" s="51"/>
       <c r="G2672" s="54"/>
       <c r="H2672" s="33"/>
     </row>
@@ -35648,31 +35653,22 @@
       <c r="G2673" s="54"/>
       <c r="H2673" s="33"/>
     </row>
-    <row r="2674" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2674" s="30"/>
-      <c r="C2674" s="31"/>
-      <c r="D2674" s="30"/>
-      <c r="E2674" s="32"/>
-      <c r="F2674" s="51"/>
-      <c r="G2674" s="54"/>
-      <c r="H2674" s="33"/>
-    </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="B2:H2"/>
     <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B4:H4"/>
   </mergeCells>
-  <conditionalFormatting sqref="B7:B996 E7:H996">
+  <conditionalFormatting sqref="B6:B995 E6:H995">
     <cfRule type="expression" dxfId="2" priority="6">
-      <formula>$J7=",..,"</formula>
+      <formula>$J6=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B7:H996">
+  <conditionalFormatting sqref="B6:H995">
     <cfRule type="expression" dxfId="1" priority="1">
-      <formula>AND(LEN($B7)=1,$C7&lt;&gt;0)</formula>
+      <formula>AND(LEN($B6)=1,$C6&lt;&gt;0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="2">
-      <formula>$C7&lt;&gt;0</formula>
+      <formula>$C6&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
Update master template: Set Print Areas and Print Titles programmatically
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8D50CE-4FA8-4A5E-A023-0030E2B248E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C9367F-6ABE-491E-9D40-D2163DEF5F93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cover" sheetId="15" r:id="rId1"/>
@@ -33,22 +33,6 @@
     <definedName name="_1__123Graph_ACHART_1" hidden="1">[2]RAB!#REF!</definedName>
     <definedName name="_2__123Graph_XCHART_1" hidden="1">[3]RAB!#REF!</definedName>
     <definedName name="_Fill" hidden="1">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">ahsp!$A:$O</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">cover!$A$1:$I$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'harga satuan'!$A1:$J2646</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">hsp!$A:$I</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="10">'laporan bulanan'!$A:$Q</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'laporan harian'!$A$1:$N$72</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'laporan mingguan'!$A:$Q</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">rab!$A:$L</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'rekap rab'!$A:$I</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">ahsp!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">hsp!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="10">'laporan bulanan'!$1:$12</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="9">'laporan mingguan'!$1:$12</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">rab!$1:$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'rekap rab'!$1:$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">schedule!$1:$7</definedName>
     <definedName name="RAB" hidden="1">[4]RAB!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -5401,7 +5385,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="49" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="50" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Excel: Updated Cover print area to A1:N65 and updated master template
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C9367F-6ABE-491E-9D40-D2163DEF5F93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC133508-303C-4B58-9BB9-5E5B2B0AAC0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="cover" sheetId="15" r:id="rId1"/>
+    <sheet name="cover" sheetId="21" r:id="rId1"/>
     <sheet name="harga satuan" sheetId="8" r:id="rId2"/>
     <sheet name="ahsp" sheetId="10" r:id="rId3"/>
     <sheet name="hsp" sheetId="9" r:id="rId4"/>
@@ -2349,12 +2349,6 @@
       <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2366,6 +2360,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2390,220 +2390,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="25" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="25" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="67" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="60" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="69" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="45" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="47" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="48" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2664,6 +2450,220 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="67" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="60" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="69" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="45" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="47" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="48" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="25" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="25" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2976,22 +2976,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>207818</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>25400</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>7620</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>581891</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>166254</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB98596D-37B2-F7E7-2C12-EE5BDBFEEB76}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD7C1E0E-1C77-474E-B419-75DBA472442C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3013,8 +3013,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="5511800" cy="8054340"/>
+          <a:off x="207818" y="0"/>
+          <a:ext cx="8298873" cy="11870574"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3025,18 +3025,18 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>47913</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>523010</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>12005</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="3611880" cy="487313"/>
+    <xdr:ext cx="3611880" cy="559127"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="TextBox 4">
+        <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{20D9D429-0026-F84C-4FB3-FDE9E67E7E01}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43B8B549-0B64-4AB3-BC23-4CE8CEA4B6B3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3044,8 +3044,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1714500" y="4802793"/>
-          <a:ext cx="3611880" cy="487313"/>
+          <a:off x="4790210" y="7144325"/>
+          <a:ext cx="3611880" cy="559127"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3074,7 +3074,7 @@
         <a:p>
           <a:pPr algn="r"/>
           <a:r>
-            <a:rPr lang="en-ID" sz="2200">
+            <a:rPr lang="en-ID" sz="2600">
               <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
@@ -3090,18 +3090,18 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>563880</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>175260</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>356061</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>64423</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4244340" cy="269369"/>
+    <xdr:ext cx="4244340" cy="343043"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="TextBox 5">
+        <xdr:cNvPr id="4" name="TextBox 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2AFE071-5F99-49A4-8FDB-1EB893E01495}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21FBB679-DCBE-424E-87C2-C7E31AB18AC1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3109,8 +3109,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1173480" y="2735580"/>
-          <a:ext cx="4244340" cy="269369"/>
+          <a:off x="2184861" y="3904903"/>
+          <a:ext cx="4244340" cy="343043"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3139,7 +3139,7 @@
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-ID" sz="1200">
+            <a:rPr lang="en-ID" sz="1700">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -3150,7 +3150,7 @@
             <a:t>&lt;NOMOR</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-ID" sz="1200" baseline="0">
+            <a:rPr lang="en-ID" sz="1700" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -3161,7 +3161,7 @@
             <a:t> KONTRAK</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-ID" sz="1200">
+            <a:rPr lang="en-ID" sz="1700">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -3178,18 +3178,18 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>243840</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>105293</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>114299</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="3886200" cy="307777"/>
+    <xdr:ext cx="3886200" cy="397545"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="TextBox 6">
+        <xdr:cNvPr id="5" name="TextBox 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{298A06E9-E717-48DF-BF68-B77C2505DACF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DABE1740-54A7-4C93-9214-CAE17FAF4603}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3197,8 +3197,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1463040" y="3040380"/>
-          <a:ext cx="3886200" cy="307777"/>
+          <a:off x="2543693" y="4320539"/>
+          <a:ext cx="3886200" cy="397545"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3227,7 +3227,7 @@
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-ID" sz="1200">
+            <a:rPr lang="en-ID" sz="1700">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -3243,18 +3243,18 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>541020</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>471746</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>34636</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3596640" cy="739140"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="TextBox 7">
+        <xdr:cNvPr id="6" name="TextBox 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A4D76212-7FBD-44A1-80A5-569D8E6272BC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06876812-38F7-4955-9BD4-110DB833B14C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3262,7 +3262,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1760220" y="3368040"/>
+          <a:off x="2910146" y="4789516"/>
           <a:ext cx="3596640" cy="739140"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3292,7 +3292,7 @@
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-ID" sz="1200">
+            <a:rPr lang="en-ID" sz="1700">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -3309,17 +3309,17 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>121920</xdr:rowOff>
+      <xdr:colOff>429491</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>94209</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4244340" cy="269369"/>
+    <xdr:ext cx="4244340" cy="343043"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="9" name="TextBox 8">
+        <xdr:cNvPr id="7" name="TextBox 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2A332286-966C-4468-8C0B-CF0FE16445F1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90FA7ED3-C7AC-40DD-94FC-2227072A3933}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3327,8 +3327,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="670560"/>
-          <a:ext cx="4244340" cy="269369"/>
+          <a:off x="429491" y="1008609"/>
+          <a:ext cx="4244340" cy="343043"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3357,7 +3357,7 @@
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="en-ID" sz="1200">
+            <a:rPr lang="en-ID" sz="1700">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -3374,23 +3374,23 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>263236</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>124691</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>579120</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>68580</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>412866</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>27017</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="10" name="Rectangle 9">
+        <xdr:cNvPr id="8" name="Rectangle 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D89724DF-F7D8-C015-AB29-37A7DA90B337}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94936248-7E7B-4068-A679-09B719D54E0C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3398,8 +3398,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2133600" y="5318760"/>
-          <a:ext cx="3322320" cy="53340"/>
+          <a:off x="5140036" y="7622771"/>
+          <a:ext cx="3197630" cy="85206"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3943,12 +3943,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B97B6B6-7C65-4193-8D4E-4DE87F8A1BF2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B5CA0D6-1917-471F-936D-582F74ECBB81}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="82" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -3982,40 +3985,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="179"/>
-      <c r="C1" s="179"/>
-      <c r="D1" s="179"/>
-      <c r="E1" s="179"/>
-      <c r="F1" s="179"/>
-      <c r="G1" s="179"/>
-      <c r="H1" s="179"/>
-      <c r="I1" s="179"/>
-      <c r="J1" s="179"/>
-      <c r="K1" s="179"/>
-      <c r="L1" s="179"/>
-      <c r="M1" s="179"/>
-      <c r="N1" s="179"/>
-      <c r="O1" s="179"/>
-      <c r="P1" s="179"/>
+      <c r="B1" s="177"/>
+      <c r="C1" s="177"/>
+      <c r="D1" s="177"/>
+      <c r="E1" s="177"/>
+      <c r="F1" s="177"/>
+      <c r="G1" s="177"/>
+      <c r="H1" s="177"/>
+      <c r="I1" s="177"/>
+      <c r="J1" s="177"/>
+      <c r="K1" s="177"/>
+      <c r="L1" s="177"/>
+      <c r="M1" s="177"/>
+      <c r="N1" s="177"/>
+      <c r="O1" s="177"/>
+      <c r="P1" s="177"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="180" t="s">
+      <c r="B2" s="178" t="s">
         <v>142</v>
       </c>
-      <c r="C2" s="181"/>
-      <c r="D2" s="181"/>
-      <c r="E2" s="181"/>
-      <c r="F2" s="181"/>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="181"/>
-      <c r="J2" s="181"/>
-      <c r="K2" s="181"/>
-      <c r="L2" s="181"/>
-      <c r="M2" s="181"/>
-      <c r="N2" s="181"/>
-      <c r="O2" s="181"/>
-      <c r="P2" s="181"/>
+      <c r="C2" s="179"/>
+      <c r="D2" s="179"/>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="179"/>
+      <c r="H2" s="179"/>
+      <c r="I2" s="179"/>
+      <c r="J2" s="179"/>
+      <c r="K2" s="179"/>
+      <c r="L2" s="179"/>
+      <c r="M2" s="179"/>
+      <c r="N2" s="179"/>
+      <c r="O2" s="179"/>
+      <c r="P2" s="179"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4207,70 +4210,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="178" t="s">
+      <c r="B12" s="176" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="178" t="s">
+      <c r="C12" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="178"/>
-      <c r="E12" s="178"/>
-      <c r="F12" s="178" t="s">
+      <c r="D12" s="176"/>
+      <c r="E12" s="176"/>
+      <c r="F12" s="176" t="s">
         <v>148</v>
       </c>
-      <c r="G12" s="178" t="s">
+      <c r="G12" s="176" t="s">
         <v>150</v>
       </c>
-      <c r="H12" s="178" t="s">
+      <c r="H12" s="176" t="s">
         <v>149</v>
       </c>
-      <c r="I12" s="178" t="s">
+      <c r="I12" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="J12" s="178" t="s">
+      <c r="J12" s="176" t="s">
         <v>155</v>
       </c>
-      <c r="K12" s="178"/>
-      <c r="L12" s="178"/>
-      <c r="M12" s="178"/>
-      <c r="N12" s="178"/>
-      <c r="O12" s="178"/>
-      <c r="P12" s="176" t="s">
+      <c r="K12" s="176"/>
+      <c r="L12" s="176"/>
+      <c r="M12" s="176"/>
+      <c r="N12" s="176"/>
+      <c r="O12" s="176"/>
+      <c r="P12" s="181" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="178"/>
-      <c r="C13" s="178"/>
-      <c r="D13" s="178"/>
-      <c r="E13" s="178"/>
-      <c r="F13" s="178"/>
-      <c r="G13" s="178"/>
-      <c r="H13" s="178"/>
-      <c r="I13" s="178"/>
-      <c r="J13" s="177" t="s">
+      <c r="B13" s="176"/>
+      <c r="C13" s="176"/>
+      <c r="D13" s="176"/>
+      <c r="E13" s="176"/>
+      <c r="F13" s="176"/>
+      <c r="G13" s="176"/>
+      <c r="H13" s="176"/>
+      <c r="I13" s="176"/>
+      <c r="J13" s="180" t="s">
         <v>152</v>
       </c>
-      <c r="K13" s="177"/>
-      <c r="L13" s="177" t="s">
+      <c r="K13" s="180"/>
+      <c r="L13" s="180" t="s">
         <v>157</v>
       </c>
-      <c r="M13" s="177"/>
-      <c r="N13" s="177" t="s">
+      <c r="M13" s="180"/>
+      <c r="N13" s="180" t="s">
         <v>158</v>
       </c>
-      <c r="O13" s="177"/>
-      <c r="P13" s="176"/>
+      <c r="O13" s="180"/>
+      <c r="P13" s="181"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="178"/>
-      <c r="C14" s="178"/>
-      <c r="D14" s="178"/>
-      <c r="E14" s="178"/>
-      <c r="F14" s="178"/>
-      <c r="G14" s="178"/>
-      <c r="H14" s="178"/>
-      <c r="I14" s="178"/>
+      <c r="B14" s="176"/>
+      <c r="C14" s="176"/>
+      <c r="D14" s="176"/>
+      <c r="E14" s="176"/>
+      <c r="F14" s="176"/>
+      <c r="G14" s="176"/>
+      <c r="H14" s="176"/>
+      <c r="I14" s="176"/>
       <c r="J14" s="38" t="s">
         <v>120</v>
       </c>
@@ -4289,7 +4292,7 @@
       <c r="O14" s="40" t="s">
         <v>121</v>
       </c>
-      <c r="P14" s="176"/>
+      <c r="P14" s="181"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -4677,40 +4680,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="179"/>
-      <c r="C1" s="179"/>
-      <c r="D1" s="179"/>
-      <c r="E1" s="179"/>
-      <c r="F1" s="179"/>
-      <c r="G1" s="179"/>
-      <c r="H1" s="179"/>
-      <c r="I1" s="179"/>
-      <c r="J1" s="179"/>
-      <c r="K1" s="179"/>
-      <c r="L1" s="179"/>
-      <c r="M1" s="179"/>
-      <c r="N1" s="179"/>
-      <c r="O1" s="179"/>
-      <c r="P1" s="179"/>
+      <c r="B1" s="177"/>
+      <c r="C1" s="177"/>
+      <c r="D1" s="177"/>
+      <c r="E1" s="177"/>
+      <c r="F1" s="177"/>
+      <c r="G1" s="177"/>
+      <c r="H1" s="177"/>
+      <c r="I1" s="177"/>
+      <c r="J1" s="177"/>
+      <c r="K1" s="177"/>
+      <c r="L1" s="177"/>
+      <c r="M1" s="177"/>
+      <c r="N1" s="177"/>
+      <c r="O1" s="177"/>
+      <c r="P1" s="177"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="180" t="s">
+      <c r="B2" s="178" t="s">
         <v>161</v>
       </c>
-      <c r="C2" s="181"/>
-      <c r="D2" s="181"/>
-      <c r="E2" s="181"/>
-      <c r="F2" s="181"/>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="181"/>
-      <c r="J2" s="181"/>
-      <c r="K2" s="181"/>
-      <c r="L2" s="181"/>
-      <c r="M2" s="181"/>
-      <c r="N2" s="181"/>
-      <c r="O2" s="181"/>
-      <c r="P2" s="181"/>
+      <c r="C2" s="179"/>
+      <c r="D2" s="179"/>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="179"/>
+      <c r="H2" s="179"/>
+      <c r="I2" s="179"/>
+      <c r="J2" s="179"/>
+      <c r="K2" s="179"/>
+      <c r="L2" s="179"/>
+      <c r="M2" s="179"/>
+      <c r="N2" s="179"/>
+      <c r="O2" s="179"/>
+      <c r="P2" s="179"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4902,70 +4905,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="178" t="s">
+      <c r="B12" s="176" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="178" t="s">
+      <c r="C12" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="178"/>
-      <c r="E12" s="178"/>
-      <c r="F12" s="178" t="s">
+      <c r="D12" s="176"/>
+      <c r="E12" s="176"/>
+      <c r="F12" s="176" t="s">
         <v>148</v>
       </c>
-      <c r="G12" s="178" t="s">
+      <c r="G12" s="176" t="s">
         <v>150</v>
       </c>
-      <c r="H12" s="178" t="s">
+      <c r="H12" s="176" t="s">
         <v>149</v>
       </c>
-      <c r="I12" s="178" t="s">
+      <c r="I12" s="176" t="s">
         <v>151</v>
       </c>
-      <c r="J12" s="178" t="s">
+      <c r="J12" s="176" t="s">
         <v>155</v>
       </c>
-      <c r="K12" s="178"/>
-      <c r="L12" s="178"/>
-      <c r="M12" s="178"/>
-      <c r="N12" s="178"/>
-      <c r="O12" s="178"/>
-      <c r="P12" s="176" t="s">
+      <c r="K12" s="176"/>
+      <c r="L12" s="176"/>
+      <c r="M12" s="176"/>
+      <c r="N12" s="176"/>
+      <c r="O12" s="176"/>
+      <c r="P12" s="181" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="178"/>
-      <c r="C13" s="178"/>
-      <c r="D13" s="178"/>
-      <c r="E13" s="178"/>
-      <c r="F13" s="178"/>
-      <c r="G13" s="178"/>
-      <c r="H13" s="178"/>
-      <c r="I13" s="178"/>
-      <c r="J13" s="177" t="s">
+      <c r="B13" s="176"/>
+      <c r="C13" s="176"/>
+      <c r="D13" s="176"/>
+      <c r="E13" s="176"/>
+      <c r="F13" s="176"/>
+      <c r="G13" s="176"/>
+      <c r="H13" s="176"/>
+      <c r="I13" s="176"/>
+      <c r="J13" s="180" t="s">
         <v>152</v>
       </c>
-      <c r="K13" s="177"/>
-      <c r="L13" s="177" t="s">
+      <c r="K13" s="180"/>
+      <c r="L13" s="180" t="s">
         <v>153</v>
       </c>
-      <c r="M13" s="177"/>
-      <c r="N13" s="177" t="s">
+      <c r="M13" s="180"/>
+      <c r="N13" s="180" t="s">
         <v>154</v>
       </c>
-      <c r="O13" s="177"/>
-      <c r="P13" s="176"/>
+      <c r="O13" s="180"/>
+      <c r="P13" s="181"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="178"/>
-      <c r="C14" s="178"/>
-      <c r="D14" s="178"/>
-      <c r="E14" s="178"/>
-      <c r="F14" s="178"/>
-      <c r="G14" s="178"/>
-      <c r="H14" s="178"/>
-      <c r="I14" s="178"/>
+      <c r="B14" s="176"/>
+      <c r="C14" s="176"/>
+      <c r="D14" s="176"/>
+      <c r="E14" s="176"/>
+      <c r="F14" s="176"/>
+      <c r="G14" s="176"/>
+      <c r="H14" s="176"/>
+      <c r="I14" s="176"/>
       <c r="J14" s="38" t="s">
         <v>120</v>
       </c>
@@ -4984,7 +4987,7 @@
       <c r="O14" s="40" t="s">
         <v>121</v>
       </c>
-      <c r="P14" s="176"/>
+      <c r="P14" s="181"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -13890,10 +13893,10 @@
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="178" t="s">
+      <c r="C5" s="176" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="178"/>
+      <c r="D5" s="176"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -40216,30 +40219,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="179"/>
-      <c r="C1" s="179"/>
-      <c r="D1" s="179"/>
-      <c r="E1" s="179"/>
-      <c r="F1" s="179"/>
-      <c r="G1" s="179"/>
-      <c r="H1" s="179"/>
-      <c r="I1" s="179"/>
-      <c r="J1" s="179"/>
-      <c r="K1" s="179"/>
+      <c r="B1" s="177"/>
+      <c r="C1" s="177"/>
+      <c r="D1" s="177"/>
+      <c r="E1" s="177"/>
+      <c r="F1" s="177"/>
+      <c r="G1" s="177"/>
+      <c r="H1" s="177"/>
+      <c r="I1" s="177"/>
+      <c r="J1" s="177"/>
+      <c r="K1" s="177"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="180" t="s">
+      <c r="B2" s="178" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="181"/>
-      <c r="D2" s="181"/>
-      <c r="E2" s="181"/>
-      <c r="F2" s="181"/>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="181"/>
-      <c r="J2" s="181"/>
-      <c r="K2" s="181"/>
+      <c r="C2" s="179"/>
+      <c r="D2" s="179"/>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="179"/>
+      <c r="H2" s="179"/>
+      <c r="I2" s="179"/>
+      <c r="J2" s="179"/>
+      <c r="K2" s="179"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40359,11 +40362,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="178" t="s">
+      <c r="C11" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="178"/>
-      <c r="E11" s="178"/>
+      <c r="D11" s="176"/>
+      <c r="E11" s="176"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -41792,24 +41795,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="111.6" customHeight="1">
-      <c r="B1" s="179"/>
-      <c r="C1" s="179"/>
-      <c r="D1" s="179"/>
-      <c r="E1" s="179"/>
-      <c r="F1" s="179"/>
-      <c r="G1" s="179"/>
-      <c r="H1" s="179"/>
+      <c r="B1" s="177"/>
+      <c r="C1" s="177"/>
+      <c r="D1" s="177"/>
+      <c r="E1" s="177"/>
+      <c r="F1" s="177"/>
+      <c r="G1" s="177"/>
+      <c r="H1" s="177"/>
     </row>
     <row r="2" spans="2:8" ht="22.95" customHeight="1">
-      <c r="B2" s="180" t="s">
+      <c r="B2" s="178" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="181"/>
-      <c r="D2" s="181"/>
-      <c r="E2" s="181"/>
-      <c r="F2" s="181"/>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
+      <c r="C2" s="179"/>
+      <c r="D2" s="179"/>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="179"/>
+      <c r="H2" s="179"/>
     </row>
     <row r="3" spans="2:8" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -41911,11 +41914,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="178" t="s">
+      <c r="C11" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="178"/>
-      <c r="E11" s="178"/>
+      <c r="D11" s="176"/>
+      <c r="E11" s="176"/>
       <c r="F11" s="40" t="s">
         <v>29</v>
       </c>
@@ -43145,11 +43148,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="179"/>
-      <c r="C1" s="179"/>
-      <c r="D1" s="179"/>
-      <c r="E1" s="179"/>
-      <c r="F1" s="179"/>
+      <c r="B1" s="177"/>
+      <c r="C1" s="177"/>
+      <c r="D1" s="177"/>
+      <c r="E1" s="177"/>
+      <c r="F1" s="177"/>
     </row>
     <row r="2" spans="2:12" ht="18">
       <c r="B2" s="189" t="s">
@@ -43161,11 +43164,11 @@
       <c r="F2" s="189"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="179"/>
-      <c r="C3" s="179"/>
-      <c r="D3" s="179"/>
-      <c r="E3" s="179"/>
-      <c r="F3" s="179"/>
+      <c r="B3" s="177"/>
+      <c r="C3" s="177"/>
+      <c r="D3" s="177"/>
+      <c r="E3" s="177"/>
+      <c r="F3" s="177"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
       <c r="B5" s="187" t="s">
@@ -43327,50 +43330,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="253"/>
-      <c r="C1" s="254"/>
-      <c r="D1" s="254"/>
-      <c r="E1" s="254"/>
-      <c r="F1" s="254"/>
-      <c r="G1" s="254"/>
-      <c r="H1" s="254"/>
-      <c r="I1" s="254"/>
-      <c r="J1" s="254"/>
-      <c r="K1" s="254"/>
-      <c r="L1" s="254"/>
-      <c r="M1" s="255"/>
+      <c r="B1" s="190"/>
+      <c r="C1" s="191"/>
+      <c r="D1" s="191"/>
+      <c r="E1" s="191"/>
+      <c r="F1" s="191"/>
+      <c r="G1" s="191"/>
+      <c r="H1" s="191"/>
+      <c r="I1" s="191"/>
+      <c r="J1" s="191"/>
+      <c r="K1" s="191"/>
+      <c r="L1" s="191"/>
+      <c r="M1" s="192"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="256" t="s">
+      <c r="B2" s="193" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="257"/>
-      <c r="F2" s="257"/>
-      <c r="G2" s="257"/>
-      <c r="H2" s="257"/>
-      <c r="I2" s="258"/>
-      <c r="J2" s="262" t="s">
+      <c r="C2" s="194"/>
+      <c r="D2" s="194"/>
+      <c r="E2" s="194"/>
+      <c r="F2" s="194"/>
+      <c r="G2" s="194"/>
+      <c r="H2" s="194"/>
+      <c r="I2" s="195"/>
+      <c r="J2" s="199" t="s">
         <v>86</v>
       </c>
-      <c r="K2" s="263"/>
-      <c r="L2" s="263"/>
-      <c r="M2" s="264"/>
+      <c r="K2" s="200"/>
+      <c r="L2" s="200"/>
+      <c r="M2" s="201"/>
     </row>
     <row r="3" spans="1:14" ht="14.4" customHeight="1">
-      <c r="B3" s="259"/>
-      <c r="C3" s="260"/>
-      <c r="D3" s="260"/>
-      <c r="E3" s="260"/>
-      <c r="F3" s="260"/>
-      <c r="G3" s="260"/>
-      <c r="H3" s="260"/>
-      <c r="I3" s="261"/>
-      <c r="J3" s="265"/>
-      <c r="K3" s="266"/>
-      <c r="L3" s="266"/>
-      <c r="M3" s="267"/>
+      <c r="B3" s="196"/>
+      <c r="C3" s="197"/>
+      <c r="D3" s="197"/>
+      <c r="E3" s="197"/>
+      <c r="F3" s="197"/>
+      <c r="G3" s="197"/>
+      <c r="H3" s="197"/>
+      <c r="I3" s="198"/>
+      <c r="J3" s="202"/>
+      <c r="K3" s="203"/>
+      <c r="L3" s="203"/>
+      <c r="M3" s="204"/>
     </row>
     <row r="4" spans="1:14" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -43381,10 +43384,10 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="265"/>
-      <c r="K4" s="266"/>
-      <c r="L4" s="266"/>
-      <c r="M4" s="267"/>
+      <c r="J4" s="202"/>
+      <c r="K4" s="203"/>
+      <c r="L4" s="203"/>
+      <c r="M4" s="204"/>
     </row>
     <row r="5" spans="1:14" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -43401,10 +43404,10 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="265"/>
-      <c r="K5" s="266"/>
-      <c r="L5" s="266"/>
-      <c r="M5" s="267"/>
+      <c r="J5" s="202"/>
+      <c r="K5" s="203"/>
+      <c r="L5" s="203"/>
+      <c r="M5" s="204"/>
     </row>
     <row r="6" spans="1:14" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -43421,10 +43424,10 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="268"/>
-      <c r="K6" s="269"/>
-      <c r="L6" s="269"/>
-      <c r="M6" s="270"/>
+      <c r="J6" s="205"/>
+      <c r="K6" s="206"/>
+      <c r="L6" s="206"/>
+      <c r="M6" s="207"/>
     </row>
     <row r="7" spans="1:14" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -43499,52 +43502,52 @@
       <c r="M9" s="89"/>
     </row>
     <row r="10" spans="1:14" ht="15.6">
-      <c r="B10" s="213" t="s">
+      <c r="B10" s="208" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="200"/>
-      <c r="D10" s="200"/>
-      <c r="E10" s="200"/>
-      <c r="F10" s="200"/>
-      <c r="G10" s="200" t="s">
+      <c r="C10" s="209"/>
+      <c r="D10" s="209"/>
+      <c r="E10" s="209"/>
+      <c r="F10" s="209"/>
+      <c r="G10" s="209" t="s">
         <v>95</v>
       </c>
-      <c r="H10" s="200"/>
-      <c r="I10" s="200"/>
-      <c r="J10" s="214"/>
-      <c r="K10" s="199" t="s">
+      <c r="H10" s="209"/>
+      <c r="I10" s="209"/>
+      <c r="J10" s="210"/>
+      <c r="K10" s="234" t="s">
         <v>96</v>
       </c>
-      <c r="L10" s="200"/>
-      <c r="M10" s="201"/>
+      <c r="L10" s="209"/>
+      <c r="M10" s="235"/>
     </row>
     <row r="11" spans="1:14" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="202" t="s">
+      <c r="C11" s="220" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="241"/>
-      <c r="E11" s="241"/>
+      <c r="D11" s="221"/>
+      <c r="E11" s="221"/>
       <c r="F11" s="92" t="s">
         <v>98</v>
       </c>
-      <c r="G11" s="202" t="s">
+      <c r="G11" s="220" t="s">
         <v>99</v>
       </c>
-      <c r="H11" s="203"/>
+      <c r="H11" s="222"/>
       <c r="I11" s="93" t="s">
         <v>27</v>
       </c>
       <c r="J11" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="202" t="s">
+      <c r="K11" s="220" t="s">
         <v>100</v>
       </c>
-      <c r="L11" s="203"/>
+      <c r="L11" s="222"/>
       <c r="M11" s="94" t="s">
         <v>101</v>
       </c>
@@ -43813,58 +43816,58 @@
       <c r="M22" s="123"/>
     </row>
     <row r="23" spans="1:13" ht="16.2" thickBot="1">
-      <c r="B23" s="242"/>
-      <c r="C23" s="243"/>
-      <c r="D23" s="243"/>
-      <c r="E23" s="243"/>
+      <c r="B23" s="223"/>
+      <c r="C23" s="224"/>
+      <c r="D23" s="224"/>
+      <c r="E23" s="224"/>
       <c r="F23" s="124"/>
       <c r="G23" s="124"/>
       <c r="H23" s="125"/>
       <c r="I23" s="125"/>
-      <c r="J23" s="244"/>
-      <c r="K23" s="244"/>
-      <c r="L23" s="244"/>
-      <c r="M23" s="245"/>
+      <c r="J23" s="225"/>
+      <c r="K23" s="225"/>
+      <c r="L23" s="225"/>
+      <c r="M23" s="226"/>
     </row>
     <row r="24" spans="1:13" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="160" t="s">
         <v>118</v>
       </c>
-      <c r="B24" s="246" t="s">
+      <c r="B24" s="227" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="248" t="s">
+      <c r="C24" s="229" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="248"/>
-      <c r="E24" s="248"/>
-      <c r="F24" s="248"/>
-      <c r="G24" s="248"/>
-      <c r="H24" s="248"/>
-      <c r="I24" s="248"/>
-      <c r="J24" s="250" t="s">
+      <c r="D24" s="229"/>
+      <c r="E24" s="229"/>
+      <c r="F24" s="229"/>
+      <c r="G24" s="229"/>
+      <c r="H24" s="229"/>
+      <c r="I24" s="229"/>
+      <c r="J24" s="231" t="s">
         <v>119</v>
       </c>
-      <c r="K24" s="251"/>
-      <c r="L24" s="251"/>
-      <c r="M24" s="252"/>
+      <c r="K24" s="232"/>
+      <c r="L24" s="232"/>
+      <c r="M24" s="233"/>
     </row>
     <row r="25" spans="1:13" ht="31.2">
-      <c r="B25" s="247"/>
-      <c r="C25" s="249"/>
-      <c r="D25" s="249"/>
-      <c r="E25" s="249"/>
-      <c r="F25" s="249"/>
-      <c r="G25" s="249"/>
-      <c r="H25" s="249"/>
-      <c r="I25" s="249"/>
+      <c r="B25" s="228"/>
+      <c r="C25" s="230"/>
+      <c r="D25" s="230"/>
+      <c r="E25" s="230"/>
+      <c r="F25" s="230"/>
+      <c r="G25" s="230"/>
+      <c r="H25" s="230"/>
+      <c r="I25" s="230"/>
       <c r="J25" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="193" t="s">
+      <c r="K25" s="248" t="s">
         <v>120</v>
       </c>
-      <c r="L25" s="194"/>
+      <c r="L25" s="249"/>
       <c r="M25" s="126" t="s">
         <v>121</v>
       </c>
@@ -44422,64 +44425,64 @@
       </c>
     </row>
     <row r="49" spans="2:13" ht="16.2" thickTop="1">
-      <c r="B49" s="226" t="s">
+      <c r="B49" s="265" t="s">
         <v>122</v>
       </c>
-      <c r="C49" s="227"/>
-      <c r="D49" s="227"/>
-      <c r="E49" s="227"/>
-      <c r="F49" s="227"/>
-      <c r="G49" s="227"/>
-      <c r="H49" s="227"/>
-      <c r="I49" s="227"/>
-      <c r="J49" s="228"/>
-      <c r="K49" s="238" t="s">
+      <c r="C49" s="266"/>
+      <c r="D49" s="266"/>
+      <c r="E49" s="266"/>
+      <c r="F49" s="266"/>
+      <c r="G49" s="266"/>
+      <c r="H49" s="266"/>
+      <c r="I49" s="266"/>
+      <c r="J49" s="267"/>
+      <c r="K49" s="217" t="s">
         <v>123</v>
       </c>
-      <c r="L49" s="239"/>
-      <c r="M49" s="240"/>
+      <c r="L49" s="218"/>
+      <c r="M49" s="219"/>
     </row>
     <row r="50" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B50" s="229"/>
-      <c r="C50" s="230"/>
-      <c r="D50" s="230"/>
-      <c r="E50" s="230"/>
-      <c r="F50" s="230"/>
-      <c r="G50" s="230"/>
-      <c r="H50" s="230"/>
-      <c r="I50" s="230"/>
-      <c r="J50" s="231"/>
-      <c r="K50" s="235" t="s">
+      <c r="B50" s="268"/>
+      <c r="C50" s="269"/>
+      <c r="D50" s="269"/>
+      <c r="E50" s="269"/>
+      <c r="F50" s="269"/>
+      <c r="G50" s="269"/>
+      <c r="H50" s="269"/>
+      <c r="I50" s="269"/>
+      <c r="J50" s="270"/>
+      <c r="K50" s="214" t="s">
         <v>124</v>
       </c>
-      <c r="L50" s="236"/>
-      <c r="M50" s="237"/>
+      <c r="L50" s="215"/>
+      <c r="M50" s="216"/>
     </row>
     <row r="51" spans="2:13" ht="15.6">
       <c r="B51" s="138"/>
-      <c r="C51" s="232"/>
-      <c r="D51" s="232"/>
-      <c r="E51" s="232"/>
-      <c r="F51" s="232"/>
-      <c r="G51" s="232"/>
-      <c r="H51" s="232"/>
-      <c r="I51" s="232"/>
+      <c r="C51" s="211"/>
+      <c r="D51" s="211"/>
+      <c r="E51" s="211"/>
+      <c r="F51" s="211"/>
+      <c r="G51" s="211"/>
+      <c r="H51" s="211"/>
+      <c r="I51" s="211"/>
       <c r="J51" s="139"/>
-      <c r="K51" s="210" t="s">
+      <c r="K51" s="242" t="s">
         <v>86</v>
       </c>
-      <c r="L51" s="211"/>
-      <c r="M51" s="212"/>
+      <c r="L51" s="243"/>
+      <c r="M51" s="244"/>
     </row>
     <row r="52" spans="2:13" ht="15.6">
       <c r="B52" s="140"/>
-      <c r="C52" s="233"/>
-      <c r="D52" s="233"/>
-      <c r="E52" s="233"/>
-      <c r="F52" s="233"/>
-      <c r="G52" s="233"/>
-      <c r="H52" s="233"/>
-      <c r="I52" s="233"/>
+      <c r="C52" s="212"/>
+      <c r="D52" s="212"/>
+      <c r="E52" s="212"/>
+      <c r="F52" s="212"/>
+      <c r="G52" s="212"/>
+      <c r="H52" s="212"/>
+      <c r="I52" s="212"/>
       <c r="J52" s="141"/>
       <c r="K52" s="172"/>
       <c r="L52" s="169"/>
@@ -44487,13 +44490,13 @@
     </row>
     <row r="53" spans="2:13" ht="15.6">
       <c r="B53" s="140"/>
-      <c r="C53" s="233"/>
-      <c r="D53" s="233"/>
-      <c r="E53" s="233"/>
-      <c r="F53" s="233"/>
-      <c r="G53" s="233"/>
-      <c r="H53" s="233"/>
-      <c r="I53" s="233"/>
+      <c r="C53" s="212"/>
+      <c r="D53" s="212"/>
+      <c r="E53" s="212"/>
+      <c r="F53" s="212"/>
+      <c r="G53" s="212"/>
+      <c r="H53" s="212"/>
+      <c r="I53" s="212"/>
       <c r="J53" s="141"/>
       <c r="K53" s="172"/>
       <c r="L53" s="169"/>
@@ -44501,13 +44504,13 @@
     </row>
     <row r="54" spans="2:13" ht="15.6">
       <c r="B54" s="140"/>
-      <c r="C54" s="233"/>
-      <c r="D54" s="233"/>
-      <c r="E54" s="233"/>
-      <c r="F54" s="233"/>
-      <c r="G54" s="233"/>
-      <c r="H54" s="233"/>
-      <c r="I54" s="233"/>
+      <c r="C54" s="212"/>
+      <c r="D54" s="212"/>
+      <c r="E54" s="212"/>
+      <c r="F54" s="212"/>
+      <c r="G54" s="212"/>
+      <c r="H54" s="212"/>
+      <c r="I54" s="212"/>
       <c r="J54" s="141"/>
       <c r="K54" s="172"/>
       <c r="L54" s="169"/>
@@ -44515,13 +44518,13 @@
     </row>
     <row r="55" spans="2:13" ht="15.6">
       <c r="B55" s="143"/>
-      <c r="C55" s="233"/>
-      <c r="D55" s="233"/>
-      <c r="E55" s="233"/>
-      <c r="F55" s="233"/>
-      <c r="G55" s="233"/>
-      <c r="H55" s="233"/>
-      <c r="I55" s="233"/>
+      <c r="C55" s="212"/>
+      <c r="D55" s="212"/>
+      <c r="E55" s="212"/>
+      <c r="F55" s="212"/>
+      <c r="G55" s="212"/>
+      <c r="H55" s="212"/>
+      <c r="I55" s="212"/>
       <c r="J55" s="144"/>
       <c r="K55" s="172"/>
       <c r="L55" s="145"/>
@@ -44529,13 +44532,13 @@
     </row>
     <row r="56" spans="2:13" ht="15.6">
       <c r="B56" s="143"/>
-      <c r="C56" s="233"/>
-      <c r="D56" s="233"/>
-      <c r="E56" s="233"/>
-      <c r="F56" s="233"/>
-      <c r="G56" s="233"/>
-      <c r="H56" s="233"/>
-      <c r="I56" s="233"/>
+      <c r="C56" s="212"/>
+      <c r="D56" s="212"/>
+      <c r="E56" s="212"/>
+      <c r="F56" s="212"/>
+      <c r="G56" s="212"/>
+      <c r="H56" s="212"/>
+      <c r="I56" s="212"/>
       <c r="J56" s="144"/>
       <c r="K56" s="172"/>
       <c r="L56" s="145"/>
@@ -44543,45 +44546,45 @@
     </row>
     <row r="57" spans="2:13" ht="15.6">
       <c r="B57" s="143"/>
-      <c r="C57" s="233"/>
-      <c r="D57" s="233"/>
-      <c r="E57" s="233"/>
-      <c r="F57" s="233"/>
-      <c r="G57" s="233"/>
-      <c r="H57" s="233"/>
-      <c r="I57" s="233"/>
+      <c r="C57" s="212"/>
+      <c r="D57" s="212"/>
+      <c r="E57" s="212"/>
+      <c r="F57" s="212"/>
+      <c r="G57" s="212"/>
+      <c r="H57" s="212"/>
+      <c r="I57" s="212"/>
       <c r="J57" s="144"/>
-      <c r="K57" s="204" t="s">
+      <c r="K57" s="236" t="s">
         <v>125</v>
       </c>
-      <c r="L57" s="205"/>
-      <c r="M57" s="206"/>
+      <c r="L57" s="237"/>
+      <c r="M57" s="238"/>
     </row>
     <row r="58" spans="2:13" ht="15.6">
       <c r="B58" s="143"/>
-      <c r="C58" s="233"/>
-      <c r="D58" s="233"/>
-      <c r="E58" s="233"/>
-      <c r="F58" s="233"/>
-      <c r="G58" s="233"/>
-      <c r="H58" s="233"/>
-      <c r="I58" s="233"/>
+      <c r="C58" s="212"/>
+      <c r="D58" s="212"/>
+      <c r="E58" s="212"/>
+      <c r="F58" s="212"/>
+      <c r="G58" s="212"/>
+      <c r="H58" s="212"/>
+      <c r="I58" s="212"/>
       <c r="J58" s="144"/>
-      <c r="K58" s="207" t="s">
+      <c r="K58" s="239" t="s">
         <v>126</v>
       </c>
-      <c r="L58" s="208"/>
-      <c r="M58" s="209"/>
+      <c r="L58" s="240"/>
+      <c r="M58" s="241"/>
     </row>
     <row r="59" spans="2:13" ht="15.6">
       <c r="B59" s="143"/>
-      <c r="C59" s="233"/>
-      <c r="D59" s="233"/>
-      <c r="E59" s="233"/>
-      <c r="F59" s="233"/>
-      <c r="G59" s="233"/>
-      <c r="H59" s="233"/>
-      <c r="I59" s="233"/>
+      <c r="C59" s="212"/>
+      <c r="D59" s="212"/>
+      <c r="E59" s="212"/>
+      <c r="F59" s="212"/>
+      <c r="G59" s="212"/>
+      <c r="H59" s="212"/>
+      <c r="I59" s="212"/>
       <c r="J59" s="144"/>
       <c r="K59" s="172"/>
       <c r="L59" s="170"/>
@@ -44589,13 +44592,13 @@
     </row>
     <row r="60" spans="2:13" ht="15.6">
       <c r="B60" s="143"/>
-      <c r="C60" s="233"/>
-      <c r="D60" s="233"/>
-      <c r="E60" s="233"/>
-      <c r="F60" s="233"/>
-      <c r="G60" s="233"/>
-      <c r="H60" s="233"/>
-      <c r="I60" s="233"/>
+      <c r="C60" s="212"/>
+      <c r="D60" s="212"/>
+      <c r="E60" s="212"/>
+      <c r="F60" s="212"/>
+      <c r="G60" s="212"/>
+      <c r="H60" s="212"/>
+      <c r="I60" s="212"/>
       <c r="J60" s="144"/>
       <c r="K60" s="172"/>
       <c r="L60" s="170"/>
@@ -44603,13 +44606,13 @@
     </row>
     <row r="61" spans="2:13" ht="15.6">
       <c r="B61" s="143"/>
-      <c r="C61" s="234"/>
-      <c r="D61" s="234"/>
-      <c r="E61" s="234"/>
-      <c r="F61" s="234"/>
-      <c r="G61" s="234"/>
-      <c r="H61" s="234"/>
-      <c r="I61" s="234"/>
+      <c r="C61" s="213"/>
+      <c r="D61" s="213"/>
+      <c r="E61" s="213"/>
+      <c r="F61" s="213"/>
+      <c r="G61" s="213"/>
+      <c r="H61" s="213"/>
+      <c r="I61" s="213"/>
       <c r="J61" s="144"/>
       <c r="K61" s="172"/>
       <c r="L61" s="170"/>
@@ -44630,41 +44633,41 @@
       <c r="M62" s="175"/>
     </row>
     <row r="63" spans="2:13" ht="15.6">
-      <c r="B63" s="213" t="s">
+      <c r="B63" s="208" t="s">
         <v>127</v>
       </c>
-      <c r="C63" s="200"/>
-      <c r="D63" s="200"/>
-      <c r="E63" s="214"/>
-      <c r="F63" s="199" t="s">
+      <c r="C63" s="209"/>
+      <c r="D63" s="209"/>
+      <c r="E63" s="210"/>
+      <c r="F63" s="234" t="s">
         <v>128</v>
       </c>
-      <c r="G63" s="214"/>
-      <c r="H63" s="199" t="s">
+      <c r="G63" s="210"/>
+      <c r="H63" s="234" t="s">
         <v>129</v>
       </c>
-      <c r="I63" s="200"/>
-      <c r="J63" s="214"/>
+      <c r="I63" s="209"/>
+      <c r="J63" s="210"/>
       <c r="K63" s="173"/>
       <c r="L63" s="145"/>
       <c r="M63" s="146"/>
     </row>
     <row r="64" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B64" s="215" t="s">
+      <c r="B64" s="254" t="s">
         <v>130</v>
       </c>
-      <c r="C64" s="216"/>
-      <c r="D64" s="216"/>
-      <c r="E64" s="216"/>
-      <c r="F64" s="217" t="s">
+      <c r="C64" s="255"/>
+      <c r="D64" s="255"/>
+      <c r="E64" s="255"/>
+      <c r="F64" s="256" t="s">
         <v>131</v>
       </c>
-      <c r="G64" s="218"/>
-      <c r="H64" s="219" t="s">
+      <c r="G64" s="257"/>
+      <c r="H64" s="258" t="s">
         <v>132</v>
       </c>
-      <c r="I64" s="220"/>
-      <c r="J64" s="221"/>
+      <c r="I64" s="259"/>
+      <c r="J64" s="260"/>
       <c r="K64" s="151"/>
       <c r="L64" s="145"/>
       <c r="M64" s="146"/>
@@ -44676,27 +44679,27 @@
       <c r="E65" s="80"/>
       <c r="F65" s="150"/>
       <c r="G65" s="145"/>
-      <c r="H65" s="190"/>
-      <c r="I65" s="191"/>
-      <c r="J65" s="222"/>
+      <c r="H65" s="245"/>
+      <c r="I65" s="246"/>
+      <c r="J65" s="261"/>
       <c r="K65" s="151"/>
       <c r="L65" s="171"/>
       <c r="M65" s="146"/>
     </row>
     <row r="66" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B66" s="197" t="s">
+      <c r="B66" s="252" t="s">
         <v>133</v>
       </c>
-      <c r="C66" s="198"/>
-      <c r="D66" s="198"/>
-      <c r="E66" s="198"/>
-      <c r="F66" s="195" t="s">
+      <c r="C66" s="253"/>
+      <c r="D66" s="253"/>
+      <c r="E66" s="253"/>
+      <c r="F66" s="250" t="s">
         <v>134</v>
       </c>
-      <c r="G66" s="196"/>
-      <c r="H66" s="190"/>
-      <c r="I66" s="191"/>
-      <c r="J66" s="222"/>
+      <c r="G66" s="251"/>
+      <c r="H66" s="245"/>
+      <c r="I66" s="246"/>
+      <c r="J66" s="261"/>
       <c r="K66" s="151"/>
       <c r="L66" s="145"/>
       <c r="M66" s="146"/>
@@ -44708,27 +44711,27 @@
       <c r="E67" s="145"/>
       <c r="F67" s="148"/>
       <c r="G67" s="145"/>
-      <c r="H67" s="190"/>
-      <c r="I67" s="191"/>
-      <c r="J67" s="222"/>
+      <c r="H67" s="245"/>
+      <c r="I67" s="246"/>
+      <c r="J67" s="261"/>
       <c r="K67" s="151"/>
       <c r="L67" s="170"/>
       <c r="M67" s="76"/>
     </row>
     <row r="68" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B68" s="197" t="s">
+      <c r="B68" s="252" t="s">
         <v>135</v>
       </c>
-      <c r="C68" s="198"/>
-      <c r="D68" s="198"/>
-      <c r="E68" s="198"/>
-      <c r="F68" s="195" t="s">
+      <c r="C68" s="253"/>
+      <c r="D68" s="253"/>
+      <c r="E68" s="253"/>
+      <c r="F68" s="250" t="s">
         <v>136</v>
       </c>
-      <c r="G68" s="196"/>
-      <c r="H68" s="190"/>
-      <c r="I68" s="191"/>
-      <c r="J68" s="222"/>
+      <c r="G68" s="251"/>
+      <c r="H68" s="245"/>
+      <c r="I68" s="246"/>
+      <c r="J68" s="261"/>
       <c r="K68" s="151"/>
       <c r="L68" s="170"/>
       <c r="M68" s="76"/>
@@ -44740,30 +44743,30 @@
       <c r="E69" s="80"/>
       <c r="F69" s="150"/>
       <c r="G69" s="153"/>
-      <c r="H69" s="190"/>
-      <c r="I69" s="191"/>
-      <c r="J69" s="222"/>
-      <c r="K69" s="190"/>
-      <c r="L69" s="191"/>
-      <c r="M69" s="192"/>
+      <c r="H69" s="245"/>
+      <c r="I69" s="246"/>
+      <c r="J69" s="261"/>
+      <c r="K69" s="245"/>
+      <c r="L69" s="246"/>
+      <c r="M69" s="247"/>
     </row>
     <row r="70" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B70" s="197" t="s">
+      <c r="B70" s="252" t="s">
         <v>137</v>
       </c>
-      <c r="C70" s="198"/>
-      <c r="D70" s="198"/>
-      <c r="E70" s="198"/>
-      <c r="F70" s="195" t="s">
+      <c r="C70" s="253"/>
+      <c r="D70" s="253"/>
+      <c r="E70" s="253"/>
+      <c r="F70" s="250" t="s">
         <v>138</v>
       </c>
-      <c r="G70" s="196"/>
-      <c r="H70" s="190"/>
-      <c r="I70" s="191"/>
-      <c r="J70" s="222"/>
-      <c r="K70" s="190"/>
-      <c r="L70" s="191"/>
-      <c r="M70" s="192"/>
+      <c r="G70" s="251"/>
+      <c r="H70" s="245"/>
+      <c r="I70" s="246"/>
+      <c r="J70" s="261"/>
+      <c r="K70" s="245"/>
+      <c r="L70" s="246"/>
+      <c r="M70" s="247"/>
     </row>
     <row r="71" spans="2:13" ht="16.2" customHeight="1" thickBot="1">
       <c r="B71" s="154"/>
@@ -44772,9 +44775,9 @@
       <c r="E71" s="155"/>
       <c r="F71" s="156"/>
       <c r="G71" s="157"/>
-      <c r="H71" s="223"/>
-      <c r="I71" s="224"/>
-      <c r="J71" s="225"/>
+      <c r="H71" s="262"/>
+      <c r="I71" s="263"/>
+      <c r="J71" s="264"/>
       <c r="K71" s="158"/>
       <c r="L71" s="157"/>
       <c r="M71" s="159"/>
@@ -44787,26 +44790,6 @@
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="J2:M6"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="C51:I61"/>
-    <mergeCell ref="K50:M50"/>
-    <mergeCell ref="K49:M49"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="J23:M23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:I25"/>
-    <mergeCell ref="J24:M24"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="K57:M57"/>
-    <mergeCell ref="K58:M58"/>
-    <mergeCell ref="K51:M51"/>
     <mergeCell ref="K70:M70"/>
     <mergeCell ref="K69:M69"/>
     <mergeCell ref="K25:L25"/>
@@ -44823,6 +44806,26 @@
     <mergeCell ref="F66:G66"/>
     <mergeCell ref="B68:E68"/>
     <mergeCell ref="B49:J50"/>
+    <mergeCell ref="C51:I61"/>
+    <mergeCell ref="K50:M50"/>
+    <mergeCell ref="K49:M49"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="J23:M23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:I25"/>
+    <mergeCell ref="J24:M24"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="K58:M58"/>
+    <mergeCell ref="K51:M51"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="J2:M6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="K10:M10"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:I48">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
System: Integrated weather tracking and consolidated Reporting Engine (Static & Formula) using Master Template
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC133508-303C-4B58-9BB9-5E5B2B0AAC0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA863D6A-620F-4132-BAA4-F72D4C809F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cover" sheetId="21" r:id="rId1"/>
@@ -33,6 +33,7 @@
     <definedName name="_1__123Graph_ACHART_1" hidden="1">[2]RAB!#REF!</definedName>
     <definedName name="_2__123Graph_XCHART_1" hidden="1">[3]RAB!#REF!</definedName>
     <definedName name="_Fill" hidden="1">#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'laporan harian'!$A$1:$N$71</definedName>
     <definedName name="RAB" hidden="1">[4]RAB!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="145">
   <si>
     <t>HARGA SATUAN BAHAN, ALAT DAN UPAH</t>
   </si>
@@ -370,12 +371,6 @@
     <t>Mandor</t>
   </si>
   <si>
-    <t>- Org</t>
-  </si>
-  <si>
-    <t>(blank)</t>
-  </si>
-  <si>
     <t>Kepala Tukang</t>
   </si>
   <si>
@@ -427,15 +422,6 @@
     <t>Dibuat Oleh</t>
   </si>
   <si>
-    <t>Site Engineer</t>
-  </si>
-  <si>
-    <t>Nama Lengkap</t>
-  </si>
-  <si>
-    <t>NIP. 1234567890</t>
-  </si>
-  <si>
     <t>Index Cuaca</t>
   </si>
   <si>
@@ -443,42 +429,6 @@
   </si>
   <si>
     <t>Kondisi Cuaca Hari Ini</t>
-  </si>
-  <si>
-    <t>0 mm</t>
-  </si>
-  <si>
-    <t>cerah</t>
-  </si>
-  <si>
-    <t>Cerah / Berawan</t>
-  </si>
-  <si>
-    <t>0 - 0,5 mm</t>
-  </si>
-  <si>
-    <t>Berawan</t>
-  </si>
-  <si>
-    <t>0,5 - 50 mm</t>
-  </si>
-  <si>
-    <t>Hujan Sedang</t>
-  </si>
-  <si>
-    <t>50 - 100 mm</t>
-  </si>
-  <si>
-    <t>Hujan Lebat</t>
-  </si>
-  <si>
-    <t>Kamis</t>
-  </si>
-  <si>
-    <t>PEMBANGUNAN RUMAH PRIBADI 2 LANTAI</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>LAPORAN MINGGUAN</t>
@@ -555,7 +505,7 @@
     <numFmt numFmtId="170" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="171" formatCode="0.000"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -739,12 +689,6 @@
     </font>
     <font>
       <sz val="14"/>
-      <name val="Arial Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
       <name val="Arial Narrow"/>
       <family val="2"/>
     </font>
@@ -1763,7 +1707,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="169" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="271">
+  <cellXfs count="269">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2246,40 +2190,8 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2349,27 +2261,6 @@
       <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2382,6 +2273,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2391,65 +2294,29 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="79" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="25" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="171" fontId="25" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2459,6 +2326,64 @@
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2537,12 +2462,6 @@
     <xf numFmtId="0" fontId="25" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
@@ -2579,91 +2498,106 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="79" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="25" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="25" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -3985,40 +3919,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
+      <c r="B1" s="175"/>
+      <c r="C1" s="175"/>
+      <c r="D1" s="175"/>
+      <c r="E1" s="175"/>
+      <c r="F1" s="175"/>
+      <c r="G1" s="175"/>
+      <c r="H1" s="175"/>
+      <c r="I1" s="175"/>
+      <c r="J1" s="175"/>
+      <c r="K1" s="175"/>
+      <c r="L1" s="175"/>
+      <c r="M1" s="175"/>
+      <c r="N1" s="175"/>
+      <c r="O1" s="175"/>
+      <c r="P1" s="175"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="178" t="s">
-        <v>142</v>
+      <c r="B2" s="173" t="s">
+        <v>125</v>
       </c>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="179"/>
-      <c r="I2" s="179"/>
-      <c r="J2" s="179"/>
-      <c r="K2" s="179"/>
-      <c r="L2" s="179"/>
-      <c r="M2" s="179"/>
-      <c r="N2" s="179"/>
-      <c r="O2" s="179"/>
-      <c r="P2" s="179"/>
+      <c r="C2" s="174"/>
+      <c r="D2" s="174"/>
+      <c r="E2" s="174"/>
+      <c r="F2" s="174"/>
+      <c r="G2" s="174"/>
+      <c r="H2" s="174"/>
+      <c r="I2" s="174"/>
+      <c r="J2" s="174"/>
+      <c r="K2" s="174"/>
+      <c r="L2" s="174"/>
+      <c r="M2" s="174"/>
+      <c r="N2" s="174"/>
+      <c r="O2" s="174"/>
+      <c r="P2" s="174"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4045,16 +3979,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="182" t="s">
+      <c r="I4" s="260" t="s">
         <v>86</v>
       </c>
-      <c r="J4" s="182"/>
-      <c r="K4" s="182"/>
-      <c r="L4" s="182"/>
-      <c r="M4" s="182"/>
-      <c r="N4" s="182"/>
-      <c r="O4" s="182"/>
-      <c r="P4" s="182"/>
+      <c r="J4" s="260"/>
+      <c r="K4" s="260"/>
+      <c r="L4" s="260"/>
+      <c r="M4" s="260"/>
+      <c r="N4" s="260"/>
+      <c r="O4" s="260"/>
+      <c r="P4" s="260"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4068,14 +4002,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="182"/>
-      <c r="J5" s="182"/>
-      <c r="K5" s="182"/>
-      <c r="L5" s="182"/>
-      <c r="M5" s="182"/>
-      <c r="N5" s="182"/>
-      <c r="O5" s="182"/>
-      <c r="P5" s="182"/>
+      <c r="I5" s="260"/>
+      <c r="J5" s="260"/>
+      <c r="K5" s="260"/>
+      <c r="L5" s="260"/>
+      <c r="M5" s="260"/>
+      <c r="N5" s="260"/>
+      <c r="O5" s="260"/>
+      <c r="P5" s="260"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4090,7 +4024,7 @@
       <c r="G6" s="56"/>
       <c r="H6" s="56"/>
       <c r="I6" s="56" t="s">
-        <v>160</v>
+        <v>143</v>
       </c>
       <c r="J6" s="58"/>
       <c r="K6" s="56"/>
@@ -4113,7 +4047,7 @@
       <c r="G7" s="56"/>
       <c r="H7" s="56"/>
       <c r="I7" s="56" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="J7" s="58"/>
       <c r="K7" s="56"/>
@@ -4136,7 +4070,7 @@
       <c r="G8" s="56"/>
       <c r="H8" s="56"/>
       <c r="I8" s="56" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="J8" s="58"/>
       <c r="K8" s="56"/>
@@ -4159,7 +4093,7 @@
       <c r="G9" s="56"/>
       <c r="H9" s="56"/>
       <c r="I9" s="56" t="s">
-        <v>159</v>
+        <v>142</v>
       </c>
       <c r="J9" s="58"/>
       <c r="K9" s="56"/>
@@ -4182,7 +4116,7 @@
       <c r="G10" s="56"/>
       <c r="H10" s="56"/>
       <c r="I10" s="56" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
       <c r="J10" s="58"/>
       <c r="K10" s="56"/>
@@ -4210,89 +4144,89 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="176" t="s">
+      <c r="B12" s="172" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="176" t="s">
+      <c r="C12" s="172" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="176"/>
-      <c r="E12" s="176"/>
-      <c r="F12" s="176" t="s">
-        <v>148</v>
+      <c r="D12" s="172"/>
+      <c r="E12" s="172"/>
+      <c r="F12" s="172" t="s">
+        <v>131</v>
       </c>
-      <c r="G12" s="176" t="s">
-        <v>150</v>
+      <c r="G12" s="172" t="s">
+        <v>133</v>
       </c>
-      <c r="H12" s="176" t="s">
-        <v>149</v>
+      <c r="H12" s="172" t="s">
+        <v>132</v>
       </c>
-      <c r="I12" s="176" t="s">
-        <v>151</v>
+      <c r="I12" s="172" t="s">
+        <v>134</v>
       </c>
-      <c r="J12" s="176" t="s">
-        <v>155</v>
+      <c r="J12" s="172" t="s">
+        <v>138</v>
       </c>
-      <c r="K12" s="176"/>
-      <c r="L12" s="176"/>
-      <c r="M12" s="176"/>
-      <c r="N12" s="176"/>
-      <c r="O12" s="176"/>
-      <c r="P12" s="181" t="s">
-        <v>156</v>
+      <c r="K12" s="172"/>
+      <c r="L12" s="172"/>
+      <c r="M12" s="172"/>
+      <c r="N12" s="172"/>
+      <c r="O12" s="172"/>
+      <c r="P12" s="259" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="176"/>
-      <c r="C13" s="176"/>
-      <c r="D13" s="176"/>
-      <c r="E13" s="176"/>
-      <c r="F13" s="176"/>
-      <c r="G13" s="176"/>
-      <c r="H13" s="176"/>
-      <c r="I13" s="176"/>
-      <c r="J13" s="180" t="s">
-        <v>152</v>
+      <c r="B13" s="172"/>
+      <c r="C13" s="172"/>
+      <c r="D13" s="172"/>
+      <c r="E13" s="172"/>
+      <c r="F13" s="172"/>
+      <c r="G13" s="172"/>
+      <c r="H13" s="172"/>
+      <c r="I13" s="172"/>
+      <c r="J13" s="258" t="s">
+        <v>135</v>
       </c>
-      <c r="K13" s="180"/>
-      <c r="L13" s="180" t="s">
-        <v>157</v>
+      <c r="K13" s="258"/>
+      <c r="L13" s="258" t="s">
+        <v>140</v>
       </c>
-      <c r="M13" s="180"/>
-      <c r="N13" s="180" t="s">
-        <v>158</v>
+      <c r="M13" s="258"/>
+      <c r="N13" s="258" t="s">
+        <v>141</v>
       </c>
-      <c r="O13" s="180"/>
-      <c r="P13" s="181"/>
+      <c r="O13" s="258"/>
+      <c r="P13" s="259"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="176"/>
-      <c r="C14" s="176"/>
-      <c r="D14" s="176"/>
-      <c r="E14" s="176"/>
-      <c r="F14" s="176"/>
-      <c r="G14" s="176"/>
-      <c r="H14" s="176"/>
-      <c r="I14" s="176"/>
+      <c r="B14" s="172"/>
+      <c r="C14" s="172"/>
+      <c r="D14" s="172"/>
+      <c r="E14" s="172"/>
+      <c r="F14" s="172"/>
+      <c r="G14" s="172"/>
+      <c r="H14" s="172"/>
+      <c r="I14" s="172"/>
       <c r="J14" s="38" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="K14" s="39" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="L14" s="39" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="M14" s="39" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N14" s="40" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="O14" s="40" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
-      <c r="P14" s="181"/>
+      <c r="P14" s="259"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -4680,40 +4614,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
-      <c r="P1" s="177"/>
+      <c r="B1" s="175"/>
+      <c r="C1" s="175"/>
+      <c r="D1" s="175"/>
+      <c r="E1" s="175"/>
+      <c r="F1" s="175"/>
+      <c r="G1" s="175"/>
+      <c r="H1" s="175"/>
+      <c r="I1" s="175"/>
+      <c r="J1" s="175"/>
+      <c r="K1" s="175"/>
+      <c r="L1" s="175"/>
+      <c r="M1" s="175"/>
+      <c r="N1" s="175"/>
+      <c r="O1" s="175"/>
+      <c r="P1" s="175"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="178" t="s">
-        <v>161</v>
+      <c r="B2" s="173" t="s">
+        <v>144</v>
       </c>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="179"/>
-      <c r="I2" s="179"/>
-      <c r="J2" s="179"/>
-      <c r="K2" s="179"/>
-      <c r="L2" s="179"/>
-      <c r="M2" s="179"/>
-      <c r="N2" s="179"/>
-      <c r="O2" s="179"/>
-      <c r="P2" s="179"/>
+      <c r="C2" s="174"/>
+      <c r="D2" s="174"/>
+      <c r="E2" s="174"/>
+      <c r="F2" s="174"/>
+      <c r="G2" s="174"/>
+      <c r="H2" s="174"/>
+      <c r="I2" s="174"/>
+      <c r="J2" s="174"/>
+      <c r="K2" s="174"/>
+      <c r="L2" s="174"/>
+      <c r="M2" s="174"/>
+      <c r="N2" s="174"/>
+      <c r="O2" s="174"/>
+      <c r="P2" s="174"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4740,16 +4674,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="182" t="s">
+      <c r="I4" s="260" t="s">
         <v>86</v>
       </c>
-      <c r="J4" s="182"/>
-      <c r="K4" s="182"/>
-      <c r="L4" s="182"/>
-      <c r="M4" s="182"/>
-      <c r="N4" s="182"/>
-      <c r="O4" s="182"/>
-      <c r="P4" s="182"/>
+      <c r="J4" s="260"/>
+      <c r="K4" s="260"/>
+      <c r="L4" s="260"/>
+      <c r="M4" s="260"/>
+      <c r="N4" s="260"/>
+      <c r="O4" s="260"/>
+      <c r="P4" s="260"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4763,14 +4697,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="182"/>
-      <c r="J5" s="182"/>
-      <c r="K5" s="182"/>
-      <c r="L5" s="182"/>
-      <c r="M5" s="182"/>
-      <c r="N5" s="182"/>
-      <c r="O5" s="182"/>
-      <c r="P5" s="182"/>
+      <c r="I5" s="260"/>
+      <c r="J5" s="260"/>
+      <c r="K5" s="260"/>
+      <c r="L5" s="260"/>
+      <c r="M5" s="260"/>
+      <c r="N5" s="260"/>
+      <c r="O5" s="260"/>
+      <c r="P5" s="260"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4785,7 +4719,7 @@
       <c r="G6" s="56"/>
       <c r="H6" s="56"/>
       <c r="I6" s="56" t="s">
-        <v>143</v>
+        <v>126</v>
       </c>
       <c r="J6" s="58"/>
       <c r="K6" s="56"/>
@@ -4808,7 +4742,7 @@
       <c r="G7" s="56"/>
       <c r="H7" s="56"/>
       <c r="I7" s="56" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="J7" s="58"/>
       <c r="K7" s="56"/>
@@ -4831,7 +4765,7 @@
       <c r="G8" s="56"/>
       <c r="H8" s="56"/>
       <c r="I8" s="56" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="J8" s="58"/>
       <c r="K8" s="56"/>
@@ -4854,7 +4788,7 @@
       <c r="G9" s="56"/>
       <c r="H9" s="56"/>
       <c r="I9" s="56" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="J9" s="58"/>
       <c r="K9" s="56"/>
@@ -4877,7 +4811,7 @@
       <c r="G10" s="56"/>
       <c r="H10" s="56"/>
       <c r="I10" s="56" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
       <c r="J10" s="58"/>
       <c r="K10" s="56"/>
@@ -4905,89 +4839,89 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="176" t="s">
+      <c r="B12" s="172" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="176" t="s">
+      <c r="C12" s="172" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="176"/>
-      <c r="E12" s="176"/>
-      <c r="F12" s="176" t="s">
-        <v>148</v>
+      <c r="D12" s="172"/>
+      <c r="E12" s="172"/>
+      <c r="F12" s="172" t="s">
+        <v>131</v>
       </c>
-      <c r="G12" s="176" t="s">
-        <v>150</v>
+      <c r="G12" s="172" t="s">
+        <v>133</v>
       </c>
-      <c r="H12" s="176" t="s">
-        <v>149</v>
+      <c r="H12" s="172" t="s">
+        <v>132</v>
       </c>
-      <c r="I12" s="176" t="s">
-        <v>151</v>
+      <c r="I12" s="172" t="s">
+        <v>134</v>
       </c>
-      <c r="J12" s="176" t="s">
-        <v>155</v>
+      <c r="J12" s="172" t="s">
+        <v>138</v>
       </c>
-      <c r="K12" s="176"/>
-      <c r="L12" s="176"/>
-      <c r="M12" s="176"/>
-      <c r="N12" s="176"/>
-      <c r="O12" s="176"/>
-      <c r="P12" s="181" t="s">
-        <v>156</v>
+      <c r="K12" s="172"/>
+      <c r="L12" s="172"/>
+      <c r="M12" s="172"/>
+      <c r="N12" s="172"/>
+      <c r="O12" s="172"/>
+      <c r="P12" s="259" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="176"/>
-      <c r="C13" s="176"/>
-      <c r="D13" s="176"/>
-      <c r="E13" s="176"/>
-      <c r="F13" s="176"/>
-      <c r="G13" s="176"/>
-      <c r="H13" s="176"/>
-      <c r="I13" s="176"/>
-      <c r="J13" s="180" t="s">
-        <v>152</v>
+      <c r="B13" s="172"/>
+      <c r="C13" s="172"/>
+      <c r="D13" s="172"/>
+      <c r="E13" s="172"/>
+      <c r="F13" s="172"/>
+      <c r="G13" s="172"/>
+      <c r="H13" s="172"/>
+      <c r="I13" s="172"/>
+      <c r="J13" s="258" t="s">
+        <v>135</v>
       </c>
-      <c r="K13" s="180"/>
-      <c r="L13" s="180" t="s">
-        <v>153</v>
+      <c r="K13" s="258"/>
+      <c r="L13" s="258" t="s">
+        <v>136</v>
       </c>
-      <c r="M13" s="180"/>
-      <c r="N13" s="180" t="s">
-        <v>154</v>
+      <c r="M13" s="258"/>
+      <c r="N13" s="258" t="s">
+        <v>137</v>
       </c>
-      <c r="O13" s="180"/>
-      <c r="P13" s="181"/>
+      <c r="O13" s="258"/>
+      <c r="P13" s="259"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="176"/>
-      <c r="C14" s="176"/>
-      <c r="D14" s="176"/>
-      <c r="E14" s="176"/>
-      <c r="F14" s="176"/>
-      <c r="G14" s="176"/>
-      <c r="H14" s="176"/>
-      <c r="I14" s="176"/>
+      <c r="B14" s="172"/>
+      <c r="C14" s="172"/>
+      <c r="D14" s="172"/>
+      <c r="E14" s="172"/>
+      <c r="F14" s="172"/>
+      <c r="G14" s="172"/>
+      <c r="H14" s="172"/>
+      <c r="I14" s="172"/>
       <c r="J14" s="38" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="K14" s="39" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="L14" s="39" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="M14" s="39" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N14" s="40" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="O14" s="40" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
-      <c r="P14" s="181"/>
+      <c r="P14" s="259"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -5411,38 +5345,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="186"/>
-      <c r="C1" s="186"/>
-      <c r="D1" s="186"/>
-      <c r="E1" s="186"/>
-      <c r="F1" s="186"/>
-      <c r="G1" s="186"/>
-      <c r="H1" s="186"/>
-      <c r="I1" s="186"/>
+      <c r="B1" s="171"/>
+      <c r="C1" s="171"/>
+      <c r="D1" s="171"/>
+      <c r="E1" s="171"/>
+      <c r="F1" s="171"/>
+      <c r="G1" s="171"/>
+      <c r="H1" s="171"/>
+      <c r="I1" s="171"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="168" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="183"/>
-      <c r="D2" s="183"/>
-      <c r="E2" s="183"/>
-      <c r="F2" s="183"/>
-      <c r="G2" s="183"/>
-      <c r="H2" s="183"/>
-      <c r="I2" s="183"/>
+      <c r="C2" s="168"/>
+      <c r="D2" s="168"/>
+      <c r="E2" s="168"/>
+      <c r="F2" s="168"/>
+      <c r="G2" s="168"/>
+      <c r="H2" s="168"/>
+      <c r="I2" s="168"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="184" t="s">
+      <c r="B3" s="169" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="184"/>
-      <c r="D3" s="184"/>
-      <c r="E3" s="184"/>
-      <c r="F3" s="184"/>
-      <c r="G3" s="184"/>
-      <c r="H3" s="184"/>
-      <c r="I3" s="184"/>
+      <c r="C3" s="169"/>
+      <c r="D3" s="169"/>
+      <c r="E3" s="169"/>
+      <c r="F3" s="169"/>
+      <c r="G3" s="169"/>
+      <c r="H3" s="169"/>
+      <c r="I3" s="169"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -5450,10 +5384,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="185" t="s">
+      <c r="C5" s="170" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="185"/>
+      <c r="D5" s="170"/>
       <c r="E5" s="11" t="s">
         <v>80</v>
       </c>
@@ -13840,63 +13774,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="186"/>
-      <c r="C1" s="186"/>
-      <c r="D1" s="186"/>
-      <c r="E1" s="186"/>
-      <c r="F1" s="186"/>
-      <c r="G1" s="186"/>
-      <c r="H1" s="186"/>
-      <c r="I1" s="186"/>
-      <c r="J1" s="186"/>
-      <c r="K1" s="186"/>
-      <c r="L1" s="186"/>
-      <c r="M1" s="186"/>
-      <c r="N1" s="186"/>
+      <c r="B1" s="171"/>
+      <c r="C1" s="171"/>
+      <c r="D1" s="171"/>
+      <c r="E1" s="171"/>
+      <c r="F1" s="171"/>
+      <c r="G1" s="171"/>
+      <c r="H1" s="171"/>
+      <c r="I1" s="171"/>
+      <c r="J1" s="171"/>
+      <c r="K1" s="171"/>
+      <c r="L1" s="171"/>
+      <c r="M1" s="171"/>
+      <c r="N1" s="171"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="168" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="183"/>
-      <c r="D2" s="183"/>
-      <c r="E2" s="183"/>
-      <c r="F2" s="183"/>
-      <c r="G2" s="183"/>
-      <c r="H2" s="183"/>
-      <c r="I2" s="183"/>
-      <c r="J2" s="183"/>
-      <c r="K2" s="183"/>
-      <c r="L2" s="183"/>
-      <c r="M2" s="183"/>
-      <c r="N2" s="183"/>
+      <c r="C2" s="168"/>
+      <c r="D2" s="168"/>
+      <c r="E2" s="168"/>
+      <c r="F2" s="168"/>
+      <c r="G2" s="168"/>
+      <c r="H2" s="168"/>
+      <c r="I2" s="168"/>
+      <c r="J2" s="168"/>
+      <c r="K2" s="168"/>
+      <c r="L2" s="168"/>
+      <c r="M2" s="168"/>
+      <c r="N2" s="168"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="184" t="s">
+      <c r="B3" s="169" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="184"/>
-      <c r="D3" s="184"/>
-      <c r="E3" s="184"/>
-      <c r="F3" s="184"/>
-      <c r="G3" s="184"/>
-      <c r="H3" s="184"/>
-      <c r="I3" s="184"/>
-      <c r="J3" s="184"/>
-      <c r="K3" s="184"/>
-      <c r="L3" s="184"/>
-      <c r="M3" s="184"/>
-      <c r="N3" s="184"/>
+      <c r="C3" s="169"/>
+      <c r="D3" s="169"/>
+      <c r="E3" s="169"/>
+      <c r="F3" s="169"/>
+      <c r="G3" s="169"/>
+      <c r="H3" s="169"/>
+      <c r="I3" s="169"/>
+      <c r="J3" s="169"/>
+      <c r="K3" s="169"/>
+      <c r="L3" s="169"/>
+      <c r="M3" s="169"/>
+      <c r="N3" s="169"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="176" t="s">
+      <c r="C5" s="172" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="176"/>
+      <c r="D5" s="172"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -16100,35 +16034,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="186"/>
-      <c r="C1" s="186"/>
-      <c r="D1" s="186"/>
-      <c r="E1" s="186"/>
-      <c r="F1" s="186"/>
-      <c r="G1" s="186"/>
-      <c r="H1" s="186"/>
+      <c r="B1" s="171"/>
+      <c r="C1" s="171"/>
+      <c r="D1" s="171"/>
+      <c r="E1" s="171"/>
+      <c r="F1" s="171"/>
+      <c r="G1" s="171"/>
+      <c r="H1" s="171"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="168" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="183"/>
-      <c r="D2" s="183"/>
-      <c r="E2" s="183"/>
-      <c r="F2" s="183"/>
-      <c r="G2" s="183"/>
-      <c r="H2" s="183"/>
+      <c r="C2" s="168"/>
+      <c r="D2" s="168"/>
+      <c r="E2" s="168"/>
+      <c r="F2" s="168"/>
+      <c r="G2" s="168"/>
+      <c r="H2" s="168"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="184" t="s">
+      <c r="B3" s="169" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="184"/>
-      <c r="D3" s="184"/>
-      <c r="E3" s="184"/>
-      <c r="F3" s="184"/>
-      <c r="G3" s="184"/>
-      <c r="H3" s="184"/>
+      <c r="C3" s="169"/>
+      <c r="D3" s="169"/>
+      <c r="E3" s="169"/>
+      <c r="F3" s="169"/>
+      <c r="G3" s="169"/>
+      <c r="H3" s="169"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -40219,30 +40153,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
+      <c r="B1" s="175"/>
+      <c r="C1" s="175"/>
+      <c r="D1" s="175"/>
+      <c r="E1" s="175"/>
+      <c r="F1" s="175"/>
+      <c r="G1" s="175"/>
+      <c r="H1" s="175"/>
+      <c r="I1" s="175"/>
+      <c r="J1" s="175"/>
+      <c r="K1" s="175"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="178" t="s">
+      <c r="B2" s="173" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="179"/>
-      <c r="I2" s="179"/>
-      <c r="J2" s="179"/>
-      <c r="K2" s="179"/>
+      <c r="C2" s="174"/>
+      <c r="D2" s="174"/>
+      <c r="E2" s="174"/>
+      <c r="F2" s="174"/>
+      <c r="G2" s="174"/>
+      <c r="H2" s="174"/>
+      <c r="I2" s="174"/>
+      <c r="J2" s="174"/>
+      <c r="K2" s="174"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40362,11 +40296,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="176" t="s">
+      <c r="C11" s="172" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="176"/>
-      <c r="E11" s="176"/>
+      <c r="D11" s="172"/>
+      <c r="E11" s="172"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -41795,24 +41729,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="111.6" customHeight="1">
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
+      <c r="B1" s="175"/>
+      <c r="C1" s="175"/>
+      <c r="D1" s="175"/>
+      <c r="E1" s="175"/>
+      <c r="F1" s="175"/>
+      <c r="G1" s="175"/>
+      <c r="H1" s="175"/>
     </row>
     <row r="2" spans="2:8" ht="22.95" customHeight="1">
-      <c r="B2" s="178" t="s">
+      <c r="B2" s="173" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="179"/>
+      <c r="C2" s="174"/>
+      <c r="D2" s="174"/>
+      <c r="E2" s="174"/>
+      <c r="F2" s="174"/>
+      <c r="G2" s="174"/>
+      <c r="H2" s="174"/>
     </row>
     <row r="3" spans="2:8" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -41914,11 +41848,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="176" t="s">
+      <c r="C11" s="172" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="176"/>
-      <c r="E11" s="176"/>
+      <c r="D11" s="172"/>
+      <c r="E11" s="172"/>
       <c r="F11" s="40" t="s">
         <v>29</v>
       </c>
@@ -43148,58 +43082,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
+      <c r="B1" s="175"/>
+      <c r="C1" s="175"/>
+      <c r="D1" s="175"/>
+      <c r="E1" s="175"/>
+      <c r="F1" s="175"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="189" t="s">
+      <c r="B2" s="178" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="189"/>
-      <c r="D2" s="189"/>
-      <c r="E2" s="189"/>
-      <c r="F2" s="189"/>
+      <c r="C2" s="178"/>
+      <c r="D2" s="178"/>
+      <c r="E2" s="178"/>
+      <c r="F2" s="178"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="177"/>
-      <c r="C3" s="177"/>
-      <c r="D3" s="177"/>
-      <c r="E3" s="177"/>
-      <c r="F3" s="177"/>
+      <c r="B3" s="175"/>
+      <c r="C3" s="175"/>
+      <c r="D3" s="175"/>
+      <c r="E3" s="175"/>
+      <c r="F3" s="175"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="187" t="s">
+      <c r="B5" s="176" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="187" t="s">
+      <c r="C5" s="176" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="187" t="s">
+      <c r="D5" s="176" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="188" t="s">
+      <c r="E5" s="177" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="188" t="s">
+      <c r="F5" s="177" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="187"/>
-      <c r="C6" s="187"/>
-      <c r="D6" s="187"/>
-      <c r="E6" s="188"/>
-      <c r="F6" s="188"/>
+      <c r="B6" s="176"/>
+      <c r="C6" s="176"/>
+      <c r="D6" s="176"/>
+      <c r="E6" s="177"/>
+      <c r="F6" s="177"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="187"/>
-      <c r="C7" s="187"/>
-      <c r="D7" s="187"/>
-      <c r="E7" s="188"/>
-      <c r="F7" s="188"/>
+      <c r="B7" s="176"/>
+      <c r="C7" s="176"/>
+      <c r="D7" s="176"/>
+      <c r="E7" s="177"/>
+      <c r="F7" s="177"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -43330,50 +43264,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="190"/>
-      <c r="C1" s="191"/>
-      <c r="D1" s="191"/>
-      <c r="E1" s="191"/>
-      <c r="F1" s="191"/>
-      <c r="G1" s="191"/>
-      <c r="H1" s="191"/>
-      <c r="I1" s="191"/>
-      <c r="J1" s="191"/>
-      <c r="K1" s="191"/>
-      <c r="L1" s="191"/>
-      <c r="M1" s="192"/>
+      <c r="B1" s="239"/>
+      <c r="C1" s="240"/>
+      <c r="D1" s="240"/>
+      <c r="E1" s="240"/>
+      <c r="F1" s="240"/>
+      <c r="G1" s="240"/>
+      <c r="H1" s="240"/>
+      <c r="I1" s="240"/>
+      <c r="J1" s="240"/>
+      <c r="K1" s="240"/>
+      <c r="L1" s="240"/>
+      <c r="M1" s="241"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="193" t="s">
+      <c r="B2" s="242" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="194"/>
-      <c r="D2" s="194"/>
-      <c r="E2" s="194"/>
-      <c r="F2" s="194"/>
-      <c r="G2" s="194"/>
-      <c r="H2" s="194"/>
-      <c r="I2" s="195"/>
-      <c r="J2" s="199" t="s">
-        <v>86</v>
-      </c>
-      <c r="K2" s="200"/>
-      <c r="L2" s="200"/>
-      <c r="M2" s="201"/>
+      <c r="C2" s="243"/>
+      <c r="D2" s="243"/>
+      <c r="E2" s="243"/>
+      <c r="F2" s="243"/>
+      <c r="G2" s="243"/>
+      <c r="H2" s="243"/>
+      <c r="I2" s="244"/>
+      <c r="J2" s="248"/>
+      <c r="K2" s="249"/>
+      <c r="L2" s="249"/>
+      <c r="M2" s="250"/>
     </row>
     <row r="3" spans="1:14" ht="14.4" customHeight="1">
-      <c r="B3" s="196"/>
-      <c r="C3" s="197"/>
-      <c r="D3" s="197"/>
-      <c r="E3" s="197"/>
-      <c r="F3" s="197"/>
-      <c r="G3" s="197"/>
-      <c r="H3" s="197"/>
-      <c r="I3" s="198"/>
-      <c r="J3" s="202"/>
-      <c r="K3" s="203"/>
-      <c r="L3" s="203"/>
-      <c r="M3" s="204"/>
+      <c r="B3" s="245"/>
+      <c r="C3" s="246"/>
+      <c r="D3" s="246"/>
+      <c r="E3" s="246"/>
+      <c r="F3" s="246"/>
+      <c r="G3" s="246"/>
+      <c r="H3" s="246"/>
+      <c r="I3" s="247"/>
+      <c r="J3" s="251"/>
+      <c r="K3" s="252"/>
+      <c r="L3" s="252"/>
+      <c r="M3" s="253"/>
     </row>
     <row r="4" spans="1:14" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -43384,10 +43316,10 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="202"/>
-      <c r="K4" s="203"/>
-      <c r="L4" s="203"/>
-      <c r="M4" s="204"/>
+      <c r="J4" s="251"/>
+      <c r="K4" s="252"/>
+      <c r="L4" s="252"/>
+      <c r="M4" s="253"/>
     </row>
     <row r="5" spans="1:14" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -43397,17 +43329,15 @@
       <c r="D5" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="80" t="s">
-        <v>140</v>
-      </c>
+      <c r="E5" s="80"/>
       <c r="F5" s="80"/>
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="202"/>
-      <c r="K5" s="203"/>
-      <c r="L5" s="203"/>
-      <c r="M5" s="204"/>
+      <c r="J5" s="251"/>
+      <c r="K5" s="252"/>
+      <c r="L5" s="252"/>
+      <c r="M5" s="253"/>
     </row>
     <row r="6" spans="1:14" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -43417,17 +43347,15 @@
       <c r="D6" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="80" t="s">
-        <v>141</v>
-      </c>
+      <c r="E6" s="80"/>
       <c r="F6" s="80"/>
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="205"/>
-      <c r="K6" s="206"/>
-      <c r="L6" s="206"/>
-      <c r="M6" s="207"/>
+      <c r="J6" s="254"/>
+      <c r="K6" s="255"/>
+      <c r="L6" s="255"/>
+      <c r="M6" s="256"/>
     </row>
     <row r="7" spans="1:14" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -43437,9 +43365,7 @@
       <c r="D7" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="80" t="s">
-        <v>141</v>
-      </c>
+      <c r="E7" s="80"/>
       <c r="F7" s="80"/>
       <c r="G7" s="80"/>
       <c r="H7" s="80"/>
@@ -43450,9 +43376,7 @@
       <c r="K7" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="L7" s="85">
-        <v>1</v>
-      </c>
+      <c r="L7" s="85"/>
       <c r="M7" s="86"/>
     </row>
     <row r="8" spans="1:14" ht="15.6">
@@ -43463,9 +43387,7 @@
       <c r="D8" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="85">
-        <v>2025</v>
-      </c>
+      <c r="E8" s="85"/>
       <c r="F8" s="80"/>
       <c r="G8" s="80"/>
       <c r="H8" s="80"/>
@@ -43476,9 +43398,7 @@
       <c r="K8" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="L8" s="85" t="s">
-        <v>139</v>
-      </c>
+      <c r="L8" s="85"/>
       <c r="M8" s="87"/>
     </row>
     <row r="9" spans="1:14" ht="15.6">
@@ -43496,58 +43416,56 @@
       <c r="K9" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="L9" s="164">
-        <v>46204</v>
-      </c>
+      <c r="L9" s="156"/>
       <c r="M9" s="89"/>
     </row>
     <row r="10" spans="1:14" ht="15.6">
-      <c r="B10" s="208" t="s">
+      <c r="B10" s="186" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="209"/>
-      <c r="D10" s="209"/>
-      <c r="E10" s="209"/>
-      <c r="F10" s="209"/>
-      <c r="G10" s="209" t="s">
+      <c r="C10" s="187"/>
+      <c r="D10" s="187"/>
+      <c r="E10" s="187"/>
+      <c r="F10" s="187"/>
+      <c r="G10" s="187" t="s">
         <v>95</v>
       </c>
-      <c r="H10" s="209"/>
-      <c r="I10" s="209"/>
-      <c r="J10" s="210"/>
-      <c r="K10" s="234" t="s">
+      <c r="H10" s="187"/>
+      <c r="I10" s="187"/>
+      <c r="J10" s="188"/>
+      <c r="K10" s="189" t="s">
         <v>96</v>
       </c>
-      <c r="L10" s="209"/>
-      <c r="M10" s="235"/>
+      <c r="L10" s="187"/>
+      <c r="M10" s="257"/>
     </row>
     <row r="11" spans="1:14" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="220" t="s">
+      <c r="C11" s="216" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="221"/>
-      <c r="E11" s="221"/>
+      <c r="D11" s="217"/>
+      <c r="E11" s="217"/>
       <c r="F11" s="92" t="s">
         <v>98</v>
       </c>
-      <c r="G11" s="220" t="s">
+      <c r="G11" s="216" t="s">
         <v>99</v>
       </c>
-      <c r="H11" s="222"/>
+      <c r="H11" s="218"/>
       <c r="I11" s="93" t="s">
         <v>27</v>
       </c>
       <c r="J11" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="220" t="s">
+      <c r="K11" s="216" t="s">
         <v>100</v>
       </c>
-      <c r="L11" s="222"/>
+      <c r="L11" s="218"/>
       <c r="M11" s="94" t="s">
         <v>101</v>
       </c>
@@ -43567,7 +43485,7 @@
       <c r="H12" s="100"/>
       <c r="I12" s="101"/>
       <c r="J12" s="101"/>
-      <c r="K12" s="161"/>
+      <c r="K12" s="153"/>
       <c r="L12" s="102"/>
       <c r="M12" s="103"/>
     </row>
@@ -43580,20 +43498,12 @@
       </c>
       <c r="D13" s="106"/>
       <c r="E13" s="106"/>
-      <c r="F13" s="107" t="s">
-        <v>105</v>
-      </c>
-      <c r="G13" s="108" t="s">
-        <v>106</v>
-      </c>
+      <c r="F13" s="107"/>
+      <c r="G13" s="108"/>
       <c r="H13" s="109"/>
-      <c r="I13" s="110">
-        <v>1</v>
-      </c>
-      <c r="J13" s="111" t="s">
-        <v>106</v>
-      </c>
-      <c r="K13" s="162"/>
+      <c r="I13" s="110"/>
+      <c r="J13" s="111"/>
+      <c r="K13" s="154"/>
       <c r="L13" s="112"/>
       <c r="M13" s="113"/>
     </row>
@@ -43602,24 +43512,16 @@
         <v>2</v>
       </c>
       <c r="C14" s="105" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D14" s="106"/>
       <c r="E14" s="106"/>
-      <c r="F14" s="107" t="s">
-        <v>105</v>
-      </c>
-      <c r="G14" s="108">
-        <v>0</v>
-      </c>
+      <c r="F14" s="107"/>
+      <c r="G14" s="108"/>
       <c r="H14" s="109"/>
-      <c r="I14" s="110" t="s">
-        <v>108</v>
-      </c>
-      <c r="J14" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="K14" s="162"/>
+      <c r="I14" s="110"/>
+      <c r="J14" s="111"/>
+      <c r="K14" s="154"/>
       <c r="L14" s="112"/>
       <c r="M14" s="113"/>
     </row>
@@ -43628,24 +43530,16 @@
         <v>3</v>
       </c>
       <c r="C15" s="105" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D15" s="106"/>
       <c r="E15" s="106"/>
-      <c r="F15" s="107" t="s">
-        <v>105</v>
-      </c>
-      <c r="G15" s="108">
-        <v>0</v>
-      </c>
+      <c r="F15" s="107"/>
+      <c r="G15" s="108"/>
       <c r="H15" s="114"/>
-      <c r="I15" s="110" t="s">
-        <v>108</v>
-      </c>
-      <c r="J15" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="K15" s="162"/>
+      <c r="I15" s="110"/>
+      <c r="J15" s="111"/>
+      <c r="K15" s="154"/>
       <c r="L15" s="112"/>
       <c r="M15" s="113"/>
     </row>
@@ -43654,22 +43548,16 @@
         <v>4</v>
       </c>
       <c r="C16" s="105" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D16" s="106"/>
       <c r="E16" s="106"/>
-      <c r="F16" s="107" t="s">
-        <v>105</v>
-      </c>
+      <c r="F16" s="107"/>
       <c r="G16" s="108"/>
       <c r="H16" s="109"/>
-      <c r="I16" s="110" t="s">
-        <v>108</v>
-      </c>
-      <c r="J16" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="K16" s="162"/>
+      <c r="I16" s="110"/>
+      <c r="J16" s="111"/>
+      <c r="K16" s="154"/>
       <c r="L16" s="112"/>
       <c r="M16" s="113"/>
     </row>
@@ -43678,22 +43566,16 @@
         <v>5</v>
       </c>
       <c r="C17" s="105" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D17" s="106"/>
       <c r="E17" s="106"/>
-      <c r="F17" s="107" t="s">
-        <v>105</v>
-      </c>
+      <c r="F17" s="107"/>
       <c r="G17" s="108"/>
       <c r="H17" s="109"/>
-      <c r="I17" s="110" t="s">
-        <v>108</v>
-      </c>
-      <c r="J17" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="K17" s="162"/>
+      <c r="I17" s="110"/>
+      <c r="J17" s="111"/>
+      <c r="K17" s="154"/>
       <c r="L17" s="112"/>
       <c r="M17" s="113"/>
     </row>
@@ -43702,44 +43584,34 @@
         <v>6</v>
       </c>
       <c r="C18" s="105" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D18" s="106"/>
       <c r="E18" s="106"/>
-      <c r="F18" s="107" t="s">
-        <v>105</v>
-      </c>
+      <c r="F18" s="107"/>
       <c r="G18" s="108"/>
       <c r="H18" s="115"/>
-      <c r="I18" s="110" t="s">
-        <v>108</v>
-      </c>
-      <c r="J18" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="K18" s="162"/>
+      <c r="I18" s="110"/>
+      <c r="J18" s="111"/>
+      <c r="K18" s="154"/>
       <c r="L18" s="112"/>
       <c r="M18" s="113"/>
     </row>
     <row r="19" spans="1:13" ht="15.6">
       <c r="B19" s="116" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C19" s="117" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D19" s="118"/>
       <c r="E19" s="118"/>
       <c r="F19" s="107"/>
       <c r="G19" s="119"/>
       <c r="H19" s="115"/>
-      <c r="I19" s="110" t="s">
-        <v>108</v>
-      </c>
-      <c r="J19" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="K19" s="162"/>
+      <c r="I19" s="110"/>
+      <c r="J19" s="111"/>
+      <c r="K19" s="154"/>
       <c r="L19" s="112"/>
       <c r="M19" s="113"/>
     </row>
@@ -43748,22 +43620,16 @@
         <v>1</v>
       </c>
       <c r="C20" s="105" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D20" s="106"/>
       <c r="E20" s="106"/>
-      <c r="F20" s="107" t="s">
-        <v>105</v>
-      </c>
+      <c r="F20" s="107"/>
       <c r="G20" s="119"/>
       <c r="H20" s="115"/>
-      <c r="I20" s="110" t="s">
-        <v>108</v>
-      </c>
-      <c r="J20" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="K20" s="162"/>
+      <c r="I20" s="110"/>
+      <c r="J20" s="111"/>
+      <c r="K20" s="154"/>
       <c r="L20" s="112"/>
       <c r="M20" s="113"/>
     </row>
@@ -43772,22 +43638,16 @@
         <v>2</v>
       </c>
       <c r="C21" s="105" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D21" s="106"/>
       <c r="E21" s="106"/>
-      <c r="F21" s="107" t="s">
-        <v>105</v>
-      </c>
+      <c r="F21" s="107"/>
       <c r="G21" s="119"/>
       <c r="H21" s="115"/>
-      <c r="I21" s="110" t="s">
-        <v>108</v>
-      </c>
-      <c r="J21" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="K21" s="162"/>
+      <c r="I21" s="110"/>
+      <c r="J21" s="111"/>
+      <c r="K21" s="154"/>
       <c r="L21" s="112"/>
       <c r="M21" s="113"/>
     </row>
@@ -43796,826 +43656,812 @@
         <v>3</v>
       </c>
       <c r="C22" s="105" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D22" s="106"/>
       <c r="E22" s="106"/>
-      <c r="F22" s="107" t="s">
-        <v>105</v>
-      </c>
+      <c r="F22" s="107"/>
       <c r="G22" s="120"/>
       <c r="H22" s="121"/>
-      <c r="I22" s="110" t="s">
-        <v>108</v>
-      </c>
-      <c r="J22" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="K22" s="163"/>
+      <c r="I22" s="110"/>
+      <c r="J22" s="111"/>
+      <c r="K22" s="155"/>
       <c r="L22" s="122"/>
       <c r="M22" s="123"/>
     </row>
     <row r="23" spans="1:13" ht="16.2" thickBot="1">
-      <c r="B23" s="223"/>
-      <c r="C23" s="224"/>
-      <c r="D23" s="224"/>
-      <c r="E23" s="224"/>
+      <c r="B23" s="219"/>
+      <c r="C23" s="220"/>
+      <c r="D23" s="220"/>
+      <c r="E23" s="220"/>
       <c r="F23" s="124"/>
       <c r="G23" s="124"/>
       <c r="H23" s="125"/>
       <c r="I23" s="125"/>
-      <c r="J23" s="225"/>
-      <c r="K23" s="225"/>
-      <c r="L23" s="225"/>
-      <c r="M23" s="226"/>
+      <c r="J23" s="221"/>
+      <c r="K23" s="221"/>
+      <c r="L23" s="221"/>
+      <c r="M23" s="222"/>
     </row>
     <row r="24" spans="1:13" ht="16.2" customHeight="1" thickTop="1">
-      <c r="A24" s="160" t="s">
-        <v>118</v>
+      <c r="A24" s="152" t="s">
+        <v>116</v>
       </c>
-      <c r="B24" s="227" t="s">
+      <c r="B24" s="223" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="229" t="s">
+      <c r="C24" s="225" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="229"/>
-      <c r="E24" s="229"/>
-      <c r="F24" s="229"/>
-      <c r="G24" s="229"/>
-      <c r="H24" s="229"/>
-      <c r="I24" s="229"/>
-      <c r="J24" s="231" t="s">
-        <v>119</v>
+      <c r="D24" s="225"/>
+      <c r="E24" s="225"/>
+      <c r="F24" s="225"/>
+      <c r="G24" s="225"/>
+      <c r="H24" s="225"/>
+      <c r="I24" s="225"/>
+      <c r="J24" s="227" t="s">
+        <v>117</v>
       </c>
-      <c r="K24" s="232"/>
-      <c r="L24" s="232"/>
-      <c r="M24" s="233"/>
+      <c r="K24" s="228"/>
+      <c r="L24" s="228"/>
+      <c r="M24" s="229"/>
     </row>
     <row r="25" spans="1:13" ht="31.2">
-      <c r="B25" s="228"/>
-      <c r="C25" s="230"/>
-      <c r="D25" s="230"/>
-      <c r="E25" s="230"/>
-      <c r="F25" s="230"/>
-      <c r="G25" s="230"/>
-      <c r="H25" s="230"/>
-      <c r="I25" s="230"/>
+      <c r="B25" s="224"/>
+      <c r="C25" s="226"/>
+      <c r="D25" s="226"/>
+      <c r="E25" s="226"/>
+      <c r="F25" s="226"/>
+      <c r="G25" s="226"/>
+      <c r="H25" s="226"/>
+      <c r="I25" s="226"/>
       <c r="J25" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="248" t="s">
-        <v>120</v>
+      <c r="K25" s="181" t="s">
+        <v>118</v>
       </c>
-      <c r="L25" s="249"/>
+      <c r="L25" s="182"/>
       <c r="M25" s="126" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="15.6">
       <c r="B26" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C26" s="128" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D26" s="165"/>
+      <c r="D26" s="157"/>
       <c r="E26" s="129"/>
       <c r="F26" s="129"/>
       <c r="G26" s="129"/>
       <c r="H26" s="129"/>
       <c r="I26" s="130"/>
       <c r="J26" s="131" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K26" s="131"/>
-      <c r="L26" s="167" t="s">
-        <v>108</v>
+      <c r="L26" s="159" t="s">
+        <v>106</v>
       </c>
       <c r="M26" s="132" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="15.6">
       <c r="B27" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C27" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D27" s="166"/>
+      <c r="D27" s="158"/>
       <c r="E27" s="134"/>
       <c r="F27" s="134"/>
       <c r="G27" s="134"/>
       <c r="H27" s="134"/>
       <c r="I27" s="135"/>
       <c r="J27" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K27" s="136"/>
-      <c r="L27" s="168" t="s">
-        <v>108</v>
+      <c r="L27" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M27" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="15.6">
       <c r="B28" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C28" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D28" s="166"/>
+      <c r="D28" s="158"/>
       <c r="E28" s="134"/>
       <c r="F28" s="134"/>
       <c r="G28" s="134"/>
       <c r="H28" s="134"/>
       <c r="I28" s="135"/>
       <c r="J28" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K28" s="136"/>
-      <c r="L28" s="168" t="s">
-        <v>108</v>
+      <c r="L28" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M28" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="15.6">
       <c r="B29" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C29" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D29" s="166"/>
+      <c r="D29" s="158"/>
       <c r="E29" s="134"/>
       <c r="F29" s="134"/>
       <c r="G29" s="134"/>
       <c r="H29" s="134"/>
       <c r="I29" s="135"/>
       <c r="J29" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K29" s="136"/>
-      <c r="L29" s="168" t="s">
-        <v>108</v>
+      <c r="L29" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M29" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="15.6">
       <c r="B30" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C30" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D30" s="166"/>
+      <c r="D30" s="158"/>
       <c r="E30" s="134"/>
       <c r="F30" s="134"/>
       <c r="G30" s="134"/>
       <c r="H30" s="134"/>
       <c r="I30" s="135"/>
       <c r="J30" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K30" s="136"/>
-      <c r="L30" s="168" t="s">
-        <v>108</v>
+      <c r="L30" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M30" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="15.6">
       <c r="B31" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C31" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D31" s="166"/>
+      <c r="D31" s="158"/>
       <c r="E31" s="134"/>
       <c r="F31" s="134"/>
       <c r="G31" s="134"/>
       <c r="H31" s="134"/>
       <c r="I31" s="135"/>
       <c r="J31" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K31" s="136"/>
-      <c r="L31" s="168" t="s">
-        <v>108</v>
+      <c r="L31" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M31" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="15.6">
       <c r="B32" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C32" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D32" s="166"/>
+      <c r="D32" s="158"/>
       <c r="E32" s="134"/>
       <c r="F32" s="134"/>
       <c r="G32" s="134"/>
       <c r="H32" s="134"/>
       <c r="I32" s="135"/>
       <c r="J32" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K32" s="136"/>
-      <c r="L32" s="168" t="s">
-        <v>108</v>
+      <c r="L32" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M32" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="33" spans="2:13" ht="15.6">
       <c r="B33" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C33" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D33" s="166"/>
+      <c r="D33" s="158"/>
       <c r="E33" s="134"/>
       <c r="F33" s="134"/>
       <c r="G33" s="134"/>
       <c r="H33" s="134"/>
       <c r="I33" s="135"/>
       <c r="J33" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K33" s="136"/>
-      <c r="L33" s="168" t="s">
-        <v>108</v>
+      <c r="L33" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M33" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="34" spans="2:13" ht="15.6">
       <c r="B34" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C34" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D34" s="166"/>
+      <c r="D34" s="158"/>
       <c r="E34" s="134"/>
       <c r="F34" s="134"/>
       <c r="G34" s="134"/>
       <c r="H34" s="134"/>
       <c r="I34" s="135"/>
       <c r="J34" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K34" s="136"/>
-      <c r="L34" s="168" t="s">
-        <v>108</v>
+      <c r="L34" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M34" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="35" spans="2:13" ht="15.6">
       <c r="B35" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C35" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D35" s="166"/>
+      <c r="D35" s="158"/>
       <c r="E35" s="134"/>
       <c r="F35" s="134"/>
       <c r="G35" s="134"/>
       <c r="H35" s="134"/>
       <c r="I35" s="135"/>
       <c r="J35" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K35" s="136"/>
-      <c r="L35" s="168" t="s">
-        <v>108</v>
+      <c r="L35" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M35" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="36" spans="2:13" ht="15.6">
       <c r="B36" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C36" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D36" s="166"/>
+      <c r="D36" s="158"/>
       <c r="E36" s="134"/>
       <c r="F36" s="134"/>
       <c r="G36" s="134"/>
       <c r="H36" s="134"/>
       <c r="I36" s="135"/>
       <c r="J36" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K36" s="136"/>
-      <c r="L36" s="168" t="s">
-        <v>108</v>
+      <c r="L36" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M36" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="37" spans="2:13" ht="15.6">
       <c r="B37" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C37" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D37" s="166"/>
+      <c r="D37" s="158"/>
       <c r="E37" s="134"/>
       <c r="F37" s="134"/>
       <c r="G37" s="134"/>
       <c r="H37" s="134"/>
       <c r="I37" s="135"/>
       <c r="J37" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K37" s="136"/>
-      <c r="L37" s="168" t="s">
-        <v>108</v>
+      <c r="L37" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M37" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="38" spans="2:13" ht="15.6">
       <c r="B38" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C38" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D38" s="166"/>
+      <c r="D38" s="158"/>
       <c r="E38" s="134"/>
       <c r="F38" s="134"/>
       <c r="G38" s="134"/>
       <c r="H38" s="134"/>
       <c r="I38" s="135"/>
       <c r="J38" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K38" s="136"/>
-      <c r="L38" s="168" t="s">
-        <v>108</v>
+      <c r="L38" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M38" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="39" spans="2:13" ht="15.6">
       <c r="B39" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C39" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D39" s="166"/>
+      <c r="D39" s="158"/>
       <c r="E39" s="134"/>
       <c r="F39" s="134"/>
       <c r="G39" s="134"/>
       <c r="H39" s="134"/>
       <c r="I39" s="135"/>
       <c r="J39" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K39" s="136"/>
-      <c r="L39" s="168" t="s">
-        <v>108</v>
+      <c r="L39" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M39" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="40" spans="2:13" ht="15.6">
       <c r="B40" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C40" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D40" s="166"/>
+      <c r="D40" s="158"/>
       <c r="E40" s="134"/>
       <c r="F40" s="134"/>
       <c r="G40" s="134"/>
       <c r="H40" s="134"/>
       <c r="I40" s="135"/>
       <c r="J40" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K40" s="136"/>
-      <c r="L40" s="168" t="s">
-        <v>108</v>
+      <c r="L40" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M40" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="41" spans="2:13" ht="15.6">
       <c r="B41" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C41" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D41" s="166"/>
+      <c r="D41" s="158"/>
       <c r="E41" s="134"/>
       <c r="F41" s="134"/>
       <c r="G41" s="134"/>
       <c r="H41" s="134"/>
       <c r="I41" s="135"/>
       <c r="J41" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K41" s="136"/>
-      <c r="L41" s="168" t="s">
-        <v>108</v>
+      <c r="L41" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M41" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="2:13" ht="15.6">
       <c r="B42" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C42" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D42" s="166"/>
+      <c r="D42" s="158"/>
       <c r="E42" s="134"/>
       <c r="F42" s="134"/>
       <c r="G42" s="134"/>
       <c r="H42" s="134"/>
       <c r="I42" s="135"/>
       <c r="J42" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K42" s="136"/>
-      <c r="L42" s="168" t="s">
-        <v>108</v>
+      <c r="L42" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M42" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="43" spans="2:13" ht="15.6">
       <c r="B43" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C43" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D43" s="166"/>
+      <c r="D43" s="158"/>
       <c r="E43" s="134"/>
       <c r="F43" s="134"/>
       <c r="G43" s="134"/>
       <c r="H43" s="134"/>
       <c r="I43" s="135"/>
       <c r="J43" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K43" s="136"/>
-      <c r="L43" s="168" t="s">
-        <v>108</v>
+      <c r="L43" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M43" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="44" spans="2:13" ht="15.6">
       <c r="B44" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C44" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D44" s="166"/>
+      <c r="D44" s="158"/>
       <c r="E44" s="134"/>
       <c r="F44" s="134"/>
       <c r="G44" s="134"/>
       <c r="H44" s="134"/>
       <c r="I44" s="135"/>
       <c r="J44" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K44" s="136"/>
-      <c r="L44" s="168" t="s">
-        <v>108</v>
+      <c r="L44" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M44" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="45" spans="2:13" ht="15.6">
       <c r="B45" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C45" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D45" s="166"/>
+      <c r="D45" s="158"/>
       <c r="E45" s="134"/>
       <c r="F45" s="134"/>
       <c r="G45" s="134"/>
       <c r="H45" s="134"/>
       <c r="I45" s="135"/>
       <c r="J45" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K45" s="136"/>
-      <c r="L45" s="168" t="s">
-        <v>108</v>
+      <c r="L45" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M45" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="46" spans="2:13" ht="15.6">
       <c r="B46" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C46" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D46" s="166"/>
+      <c r="D46" s="158"/>
       <c r="E46" s="134"/>
       <c r="F46" s="134"/>
       <c r="G46" s="134"/>
       <c r="H46" s="134"/>
       <c r="I46" s="135"/>
       <c r="J46" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K46" s="136"/>
-      <c r="L46" s="168" t="s">
-        <v>108</v>
+      <c r="L46" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M46" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="47" spans="2:13" ht="15.6">
       <c r="B47" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C47" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D47" s="166"/>
+      <c r="D47" s="158"/>
       <c r="E47" s="134"/>
       <c r="F47" s="134"/>
       <c r="G47" s="134"/>
       <c r="H47" s="134"/>
       <c r="I47" s="135"/>
       <c r="J47" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K47" s="136"/>
-      <c r="L47" s="168" t="s">
-        <v>108</v>
+      <c r="L47" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M47" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="48" spans="2:13" ht="16.2" thickBot="1">
       <c r="B48" s="127" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C48" s="133" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
-      <c r="D48" s="166"/>
+      <c r="D48" s="158"/>
       <c r="E48" s="134"/>
       <c r="F48" s="134"/>
       <c r="G48" s="134"/>
       <c r="H48" s="134"/>
       <c r="I48" s="135"/>
       <c r="J48" s="136" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K48" s="136"/>
-      <c r="L48" s="168" t="s">
-        <v>108</v>
+      <c r="L48" s="160" t="s">
+        <v>106</v>
       </c>
       <c r="M48" s="137" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="49" spans="2:13" ht="16.2" thickTop="1">
-      <c r="B49" s="265" t="s">
-        <v>122</v>
+      <c r="B49" s="201" t="s">
+        <v>120</v>
       </c>
-      <c r="C49" s="266"/>
-      <c r="D49" s="266"/>
-      <c r="E49" s="266"/>
-      <c r="F49" s="266"/>
-      <c r="G49" s="266"/>
-      <c r="H49" s="266"/>
-      <c r="I49" s="266"/>
-      <c r="J49" s="267"/>
-      <c r="K49" s="217" t="s">
-        <v>123</v>
+      <c r="C49" s="202"/>
+      <c r="D49" s="202"/>
+      <c r="E49" s="202"/>
+      <c r="F49" s="202"/>
+      <c r="G49" s="202"/>
+      <c r="H49" s="202"/>
+      <c r="I49" s="202"/>
+      <c r="J49" s="203"/>
+      <c r="K49" s="213" t="s">
+        <v>121</v>
       </c>
-      <c r="L49" s="218"/>
-      <c r="M49" s="219"/>
+      <c r="L49" s="214"/>
+      <c r="M49" s="215"/>
     </row>
     <row r="50" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B50" s="268"/>
-      <c r="C50" s="269"/>
-      <c r="D50" s="269"/>
-      <c r="E50" s="269"/>
-      <c r="F50" s="269"/>
-      <c r="G50" s="269"/>
-      <c r="H50" s="269"/>
-      <c r="I50" s="269"/>
-      <c r="J50" s="270"/>
-      <c r="K50" s="214" t="s">
-        <v>124</v>
-      </c>
-      <c r="L50" s="215"/>
-      <c r="M50" s="216"/>
+      <c r="B50" s="204"/>
+      <c r="C50" s="205"/>
+      <c r="D50" s="205"/>
+      <c r="E50" s="205"/>
+      <c r="F50" s="205"/>
+      <c r="G50" s="205"/>
+      <c r="H50" s="205"/>
+      <c r="I50" s="205"/>
+      <c r="J50" s="206"/>
+      <c r="K50" s="210"/>
+      <c r="L50" s="211"/>
+      <c r="M50" s="212"/>
     </row>
     <row r="51" spans="2:13" ht="15.6">
       <c r="B51" s="138"/>
-      <c r="C51" s="211"/>
-      <c r="D51" s="211"/>
-      <c r="E51" s="211"/>
-      <c r="F51" s="211"/>
-      <c r="G51" s="211"/>
-      <c r="H51" s="211"/>
-      <c r="I51" s="211"/>
+      <c r="C51" s="207"/>
+      <c r="D51" s="207"/>
+      <c r="E51" s="207"/>
+      <c r="F51" s="207"/>
+      <c r="G51" s="207"/>
+      <c r="H51" s="207"/>
+      <c r="I51" s="207"/>
       <c r="J51" s="139"/>
-      <c r="K51" s="242" t="s">
-        <v>86</v>
-      </c>
-      <c r="L51" s="243"/>
-      <c r="M51" s="244"/>
+      <c r="K51" s="236"/>
+      <c r="L51" s="237"/>
+      <c r="M51" s="238"/>
     </row>
     <row r="52" spans="2:13" ht="15.6">
       <c r="B52" s="140"/>
-      <c r="C52" s="212"/>
-      <c r="D52" s="212"/>
-      <c r="E52" s="212"/>
-      <c r="F52" s="212"/>
-      <c r="G52" s="212"/>
-      <c r="H52" s="212"/>
-      <c r="I52" s="212"/>
+      <c r="C52" s="208"/>
+      <c r="D52" s="208"/>
+      <c r="E52" s="208"/>
+      <c r="F52" s="208"/>
+      <c r="G52" s="208"/>
+      <c r="H52" s="208"/>
+      <c r="I52" s="208"/>
       <c r="J52" s="141"/>
-      <c r="K52" s="172"/>
-      <c r="L52" s="169"/>
+      <c r="K52" s="164"/>
+      <c r="L52" s="161"/>
       <c r="M52" s="142"/>
     </row>
     <row r="53" spans="2:13" ht="15.6">
       <c r="B53" s="140"/>
-      <c r="C53" s="212"/>
-      <c r="D53" s="212"/>
-      <c r="E53" s="212"/>
-      <c r="F53" s="212"/>
-      <c r="G53" s="212"/>
-      <c r="H53" s="212"/>
-      <c r="I53" s="212"/>
+      <c r="C53" s="208"/>
+      <c r="D53" s="208"/>
+      <c r="E53" s="208"/>
+      <c r="F53" s="208"/>
+      <c r="G53" s="208"/>
+      <c r="H53" s="208"/>
+      <c r="I53" s="208"/>
       <c r="J53" s="141"/>
-      <c r="K53" s="172"/>
-      <c r="L53" s="169"/>
+      <c r="K53" s="164"/>
+      <c r="L53" s="161"/>
       <c r="M53" s="142"/>
     </row>
     <row r="54" spans="2:13" ht="15.6">
       <c r="B54" s="140"/>
-      <c r="C54" s="212"/>
-      <c r="D54" s="212"/>
-      <c r="E54" s="212"/>
-      <c r="F54" s="212"/>
-      <c r="G54" s="212"/>
-      <c r="H54" s="212"/>
-      <c r="I54" s="212"/>
+      <c r="C54" s="208"/>
+      <c r="D54" s="208"/>
+      <c r="E54" s="208"/>
+      <c r="F54" s="208"/>
+      <c r="G54" s="208"/>
+      <c r="H54" s="208"/>
+      <c r="I54" s="208"/>
       <c r="J54" s="141"/>
-      <c r="K54" s="172"/>
-      <c r="L54" s="169"/>
+      <c r="K54" s="164"/>
+      <c r="L54" s="161"/>
       <c r="M54" s="142"/>
     </row>
     <row r="55" spans="2:13" ht="15.6">
       <c r="B55" s="143"/>
-      <c r="C55" s="212"/>
-      <c r="D55" s="212"/>
-      <c r="E55" s="212"/>
-      <c r="F55" s="212"/>
-      <c r="G55" s="212"/>
-      <c r="H55" s="212"/>
-      <c r="I55" s="212"/>
+      <c r="C55" s="208"/>
+      <c r="D55" s="208"/>
+      <c r="E55" s="208"/>
+      <c r="F55" s="208"/>
+      <c r="G55" s="208"/>
+      <c r="H55" s="208"/>
+      <c r="I55" s="208"/>
       <c r="J55" s="144"/>
-      <c r="K55" s="172"/>
+      <c r="K55" s="164"/>
       <c r="L55" s="145"/>
       <c r="M55" s="146"/>
     </row>
     <row r="56" spans="2:13" ht="15.6">
       <c r="B56" s="143"/>
-      <c r="C56" s="212"/>
-      <c r="D56" s="212"/>
-      <c r="E56" s="212"/>
-      <c r="F56" s="212"/>
-      <c r="G56" s="212"/>
-      <c r="H56" s="212"/>
-      <c r="I56" s="212"/>
+      <c r="C56" s="208"/>
+      <c r="D56" s="208"/>
+      <c r="E56" s="208"/>
+      <c r="F56" s="208"/>
+      <c r="G56" s="208"/>
+      <c r="H56" s="208"/>
+      <c r="I56" s="208"/>
       <c r="J56" s="144"/>
-      <c r="K56" s="172"/>
+      <c r="K56" s="164"/>
       <c r="L56" s="145"/>
       <c r="M56" s="146"/>
     </row>
     <row r="57" spans="2:13" ht="15.6">
       <c r="B57" s="143"/>
-      <c r="C57" s="212"/>
-      <c r="D57" s="212"/>
-      <c r="E57" s="212"/>
-      <c r="F57" s="212"/>
-      <c r="G57" s="212"/>
-      <c r="H57" s="212"/>
-      <c r="I57" s="212"/>
+      <c r="C57" s="208"/>
+      <c r="D57" s="208"/>
+      <c r="E57" s="208"/>
+      <c r="F57" s="208"/>
+      <c r="G57" s="208"/>
+      <c r="H57" s="208"/>
+      <c r="I57" s="208"/>
       <c r="J57" s="144"/>
-      <c r="K57" s="236" t="s">
-        <v>125</v>
-      </c>
-      <c r="L57" s="237"/>
-      <c r="M57" s="238"/>
+      <c r="K57" s="230"/>
+      <c r="L57" s="231"/>
+      <c r="M57" s="232"/>
     </row>
     <row r="58" spans="2:13" ht="15.6">
       <c r="B58" s="143"/>
-      <c r="C58" s="212"/>
-      <c r="D58" s="212"/>
-      <c r="E58" s="212"/>
-      <c r="F58" s="212"/>
-      <c r="G58" s="212"/>
-      <c r="H58" s="212"/>
-      <c r="I58" s="212"/>
+      <c r="C58" s="208"/>
+      <c r="D58" s="208"/>
+      <c r="E58" s="208"/>
+      <c r="F58" s="208"/>
+      <c r="G58" s="208"/>
+      <c r="H58" s="208"/>
+      <c r="I58" s="208"/>
       <c r="J58" s="144"/>
-      <c r="K58" s="239" t="s">
-        <v>126</v>
-      </c>
-      <c r="L58" s="240"/>
-      <c r="M58" s="241"/>
+      <c r="K58" s="233"/>
+      <c r="L58" s="234"/>
+      <c r="M58" s="235"/>
     </row>
     <row r="59" spans="2:13" ht="15.6">
       <c r="B59" s="143"/>
-      <c r="C59" s="212"/>
-      <c r="D59" s="212"/>
-      <c r="E59" s="212"/>
-      <c r="F59" s="212"/>
-      <c r="G59" s="212"/>
-      <c r="H59" s="212"/>
-      <c r="I59" s="212"/>
+      <c r="C59" s="208"/>
+      <c r="D59" s="208"/>
+      <c r="E59" s="208"/>
+      <c r="F59" s="208"/>
+      <c r="G59" s="208"/>
+      <c r="H59" s="208"/>
+      <c r="I59" s="208"/>
       <c r="J59" s="144"/>
-      <c r="K59" s="172"/>
-      <c r="L59" s="170"/>
+      <c r="K59" s="164"/>
+      <c r="L59" s="162"/>
       <c r="M59" s="76"/>
     </row>
     <row r="60" spans="2:13" ht="15.6">
       <c r="B60" s="143"/>
-      <c r="C60" s="212"/>
-      <c r="D60" s="212"/>
-      <c r="E60" s="212"/>
-      <c r="F60" s="212"/>
-      <c r="G60" s="212"/>
-      <c r="H60" s="212"/>
-      <c r="I60" s="212"/>
+      <c r="C60" s="208"/>
+      <c r="D60" s="208"/>
+      <c r="E60" s="208"/>
+      <c r="F60" s="208"/>
+      <c r="G60" s="208"/>
+      <c r="H60" s="208"/>
+      <c r="I60" s="208"/>
       <c r="J60" s="144"/>
-      <c r="K60" s="172"/>
-      <c r="L60" s="170"/>
+      <c r="K60" s="164"/>
+      <c r="L60" s="162"/>
       <c r="M60" s="76"/>
     </row>
     <row r="61" spans="2:13" ht="15.6">
       <c r="B61" s="143"/>
-      <c r="C61" s="213"/>
-      <c r="D61" s="213"/>
-      <c r="E61" s="213"/>
-      <c r="F61" s="213"/>
-      <c r="G61" s="213"/>
-      <c r="H61" s="213"/>
-      <c r="I61" s="213"/>
+      <c r="C61" s="209"/>
+      <c r="D61" s="209"/>
+      <c r="E61" s="209"/>
+      <c r="F61" s="209"/>
+      <c r="G61" s="209"/>
+      <c r="H61" s="209"/>
+      <c r="I61" s="209"/>
       <c r="J61" s="144"/>
-      <c r="K61" s="172"/>
-      <c r="L61" s="170"/>
+      <c r="K61" s="164"/>
+      <c r="L61" s="162"/>
       <c r="M61" s="76"/>
     </row>
     <row r="62" spans="2:13" ht="15.6">
@@ -44628,159 +44474,141 @@
       <c r="H62" s="147"/>
       <c r="I62" s="147"/>
       <c r="J62" s="144"/>
-      <c r="K62" s="172"/>
-      <c r="L62" s="174"/>
-      <c r="M62" s="175"/>
+      <c r="K62" s="164"/>
+      <c r="L62" s="166"/>
+      <c r="M62" s="167"/>
     </row>
     <row r="63" spans="2:13" ht="15.6">
-      <c r="B63" s="208" t="s">
-        <v>127</v>
+      <c r="B63" s="186" t="s">
+        <v>122</v>
       </c>
-      <c r="C63" s="209"/>
-      <c r="D63" s="209"/>
-      <c r="E63" s="210"/>
-      <c r="F63" s="234" t="s">
-        <v>128</v>
+      <c r="C63" s="187"/>
+      <c r="D63" s="187"/>
+      <c r="E63" s="188"/>
+      <c r="F63" s="189" t="s">
+        <v>123</v>
       </c>
-      <c r="G63" s="210"/>
-      <c r="H63" s="234" t="s">
-        <v>129</v>
+      <c r="G63" s="188"/>
+      <c r="H63" s="189" t="s">
+        <v>124</v>
       </c>
-      <c r="I63" s="209"/>
-      <c r="J63" s="210"/>
-      <c r="K63" s="173"/>
+      <c r="I63" s="187"/>
+      <c r="J63" s="188"/>
+      <c r="K63" s="165"/>
       <c r="L63" s="145"/>
       <c r="M63" s="146"/>
     </row>
     <row r="64" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B64" s="254" t="s">
-        <v>130</v>
-      </c>
-      <c r="C64" s="255"/>
-      <c r="D64" s="255"/>
-      <c r="E64" s="255"/>
-      <c r="F64" s="256" t="s">
-        <v>131</v>
-      </c>
-      <c r="G64" s="257"/>
-      <c r="H64" s="258" t="s">
-        <v>132</v>
-      </c>
-      <c r="I64" s="259"/>
-      <c r="J64" s="260"/>
-      <c r="K64" s="151"/>
+      <c r="B64" s="190"/>
+      <c r="C64" s="191"/>
+      <c r="D64" s="191"/>
+      <c r="E64" s="193"/>
+      <c r="F64" s="192"/>
+      <c r="G64" s="193"/>
+      <c r="H64" s="194"/>
+      <c r="I64" s="195"/>
+      <c r="J64" s="196"/>
+      <c r="K64" s="148"/>
       <c r="L64" s="145"/>
       <c r="M64" s="146"/>
     </row>
     <row r="65" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B65" s="149"/>
-      <c r="C65" s="80"/>
-      <c r="D65" s="80"/>
-      <c r="E65" s="80"/>
-      <c r="F65" s="150"/>
-      <c r="G65" s="145"/>
-      <c r="H65" s="245"/>
-      <c r="I65" s="246"/>
-      <c r="J65" s="261"/>
-      <c r="K65" s="151"/>
-      <c r="L65" s="171"/>
+      <c r="B65" s="185"/>
+      <c r="C65" s="263"/>
+      <c r="D65" s="263"/>
+      <c r="E65" s="184"/>
+      <c r="F65" s="183"/>
+      <c r="G65" s="184"/>
+      <c r="H65" s="179"/>
+      <c r="I65" s="180"/>
+      <c r="J65" s="197"/>
+      <c r="K65" s="148"/>
+      <c r="L65" s="163"/>
       <c r="M65" s="146"/>
     </row>
     <row r="66" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B66" s="252" t="s">
-        <v>133</v>
-      </c>
-      <c r="C66" s="253"/>
-      <c r="D66" s="253"/>
-      <c r="E66" s="253"/>
-      <c r="F66" s="250" t="s">
-        <v>134</v>
-      </c>
-      <c r="G66" s="251"/>
-      <c r="H66" s="245"/>
-      <c r="I66" s="246"/>
-      <c r="J66" s="261"/>
-      <c r="K66" s="151"/>
+      <c r="B66" s="185"/>
+      <c r="C66" s="263"/>
+      <c r="D66" s="263"/>
+      <c r="E66" s="184"/>
+      <c r="F66" s="183"/>
+      <c r="G66" s="184"/>
+      <c r="H66" s="179"/>
+      <c r="I66" s="180"/>
+      <c r="J66" s="197"/>
+      <c r="K66" s="148"/>
       <c r="L66" s="145"/>
       <c r="M66" s="146"/>
     </row>
     <row r="67" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B67" s="152"/>
-      <c r="C67" s="145"/>
-      <c r="D67" s="145"/>
-      <c r="E67" s="145"/>
-      <c r="F67" s="148"/>
-      <c r="G67" s="145"/>
-      <c r="H67" s="245"/>
-      <c r="I67" s="246"/>
-      <c r="J67" s="261"/>
-      <c r="K67" s="151"/>
-      <c r="L67" s="170"/>
+      <c r="B67" s="185"/>
+      <c r="C67" s="263"/>
+      <c r="D67" s="263"/>
+      <c r="E67" s="184"/>
+      <c r="F67" s="183"/>
+      <c r="G67" s="184"/>
+      <c r="H67" s="179"/>
+      <c r="I67" s="180"/>
+      <c r="J67" s="197"/>
+      <c r="K67" s="148"/>
+      <c r="L67" s="162"/>
       <c r="M67" s="76"/>
     </row>
     <row r="68" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B68" s="252" t="s">
-        <v>135</v>
-      </c>
-      <c r="C68" s="253"/>
-      <c r="D68" s="253"/>
-      <c r="E68" s="253"/>
-      <c r="F68" s="250" t="s">
-        <v>136</v>
-      </c>
-      <c r="G68" s="251"/>
-      <c r="H68" s="245"/>
-      <c r="I68" s="246"/>
-      <c r="J68" s="261"/>
-      <c r="K68" s="151"/>
-      <c r="L68" s="170"/>
+      <c r="B68" s="185"/>
+      <c r="C68" s="263"/>
+      <c r="D68" s="263"/>
+      <c r="E68" s="184"/>
+      <c r="F68" s="183"/>
+      <c r="G68" s="184"/>
+      <c r="H68" s="179"/>
+      <c r="I68" s="180"/>
+      <c r="J68" s="197"/>
+      <c r="K68" s="148"/>
+      <c r="L68" s="162"/>
       <c r="M68" s="76"/>
     </row>
     <row r="69" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B69" s="149"/>
-      <c r="C69" s="80"/>
-      <c r="D69" s="80"/>
-      <c r="E69" s="80"/>
-      <c r="F69" s="150"/>
-      <c r="G69" s="153"/>
-      <c r="H69" s="245"/>
-      <c r="I69" s="246"/>
-      <c r="J69" s="261"/>
-      <c r="K69" s="245"/>
-      <c r="L69" s="246"/>
-      <c r="M69" s="247"/>
+      <c r="B69" s="185"/>
+      <c r="C69" s="263"/>
+      <c r="D69" s="263"/>
+      <c r="E69" s="184"/>
+      <c r="F69" s="183"/>
+      <c r="G69" s="184"/>
+      <c r="H69" s="179"/>
+      <c r="I69" s="180"/>
+      <c r="J69" s="197"/>
+      <c r="K69" s="266"/>
+      <c r="L69" s="267"/>
+      <c r="M69" s="268"/>
     </row>
     <row r="70" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B70" s="252" t="s">
-        <v>137</v>
-      </c>
-      <c r="C70" s="253"/>
-      <c r="D70" s="253"/>
-      <c r="E70" s="253"/>
-      <c r="F70" s="250" t="s">
-        <v>138</v>
-      </c>
-      <c r="G70" s="251"/>
-      <c r="H70" s="245"/>
-      <c r="I70" s="246"/>
-      <c r="J70" s="261"/>
-      <c r="K70" s="245"/>
-      <c r="L70" s="246"/>
-      <c r="M70" s="247"/>
+      <c r="B70" s="185"/>
+      <c r="C70" s="263"/>
+      <c r="D70" s="263"/>
+      <c r="E70" s="184"/>
+      <c r="F70" s="183"/>
+      <c r="G70" s="184"/>
+      <c r="H70" s="179"/>
+      <c r="I70" s="180"/>
+      <c r="J70" s="197"/>
+      <c r="K70" s="266"/>
+      <c r="L70" s="267"/>
+      <c r="M70" s="268"/>
     </row>
     <row r="71" spans="2:13" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B71" s="154"/>
-      <c r="C71" s="155"/>
-      <c r="D71" s="155"/>
-      <c r="E71" s="155"/>
-      <c r="F71" s="156"/>
-      <c r="G71" s="157"/>
-      <c r="H71" s="262"/>
-      <c r="I71" s="263"/>
-      <c r="J71" s="264"/>
-      <c r="K71" s="158"/>
-      <c r="L71" s="157"/>
-      <c r="M71" s="159"/>
+      <c r="B71" s="264"/>
+      <c r="C71" s="265"/>
+      <c r="D71" s="265"/>
+      <c r="E71" s="262"/>
+      <c r="F71" s="261"/>
+      <c r="G71" s="262"/>
+      <c r="H71" s="198"/>
+      <c r="I71" s="199"/>
+      <c r="J71" s="200"/>
+      <c r="K71" s="150"/>
+      <c r="L71" s="149"/>
+      <c r="M71" s="151"/>
     </row>
     <row r="72" spans="2:13" ht="15" thickTop="1">
       <c r="J72" s="61"/>
@@ -44789,23 +44617,15 @@
       <c r="M72" s="61"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
-    <mergeCell ref="K70:M70"/>
-    <mergeCell ref="K69:M69"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="F68:G68"/>
-    <mergeCell ref="B70:E70"/>
-    <mergeCell ref="F70:G70"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="H63:J63"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="F64:G64"/>
-    <mergeCell ref="H64:J71"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="B68:E68"/>
-    <mergeCell ref="B49:J50"/>
+  <mergeCells count="28">
+    <mergeCell ref="F64:G71"/>
+    <mergeCell ref="B64:E71"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="J2:M6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="K10:M10"/>
     <mergeCell ref="C51:I61"/>
     <mergeCell ref="K50:M50"/>
     <mergeCell ref="K49:M49"/>
@@ -44820,12 +44640,12 @@
     <mergeCell ref="K57:M57"/>
     <mergeCell ref="K58:M58"/>
     <mergeCell ref="K51:M51"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="J2:M6"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="H63:J63"/>
+    <mergeCell ref="H64:J71"/>
+    <mergeCell ref="B49:J50"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:I48">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
feat: implement stakeholder signatures and fix HSP sheet columns/TKDN
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56BF3937-DD37-4286-8397-5164CF8460A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BD47DD-0F8D-4CFE-B84F-7799C638DD60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cover" sheetId="21" r:id="rId1"/>
@@ -2265,6 +2265,15 @@
       <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2298,17 +2307,13 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="25" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="25" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2318,9 +2323,97 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="79" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2334,60 +2427,8 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2502,68 +2543,56 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="25" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="25" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="79" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2574,35 +2603,6 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma [0] 2" xfId="3" xr:uid="{5950E916-03C9-42B5-8F65-57AD3DC32531}"/>
@@ -2610,7 +2610,203 @@
     <cellStyle name="Normal 2 2 3" xfId="2" xr:uid="{25DAB206-4C06-437D-BFFA-FD21FFA5A242}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="42">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -2835,54 +3031,6 @@
           <color auto="1"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -3940,48 +4088,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="239"/>
-      <c r="C1" s="240"/>
-      <c r="D1" s="240"/>
-      <c r="E1" s="240"/>
-      <c r="F1" s="240"/>
-      <c r="G1" s="240"/>
-      <c r="H1" s="240"/>
-      <c r="I1" s="240"/>
-      <c r="J1" s="240"/>
-      <c r="K1" s="240"/>
-      <c r="L1" s="240"/>
-      <c r="M1" s="241"/>
+      <c r="B1" s="194"/>
+      <c r="C1" s="195"/>
+      <c r="D1" s="195"/>
+      <c r="E1" s="195"/>
+      <c r="F1" s="195"/>
+      <c r="G1" s="195"/>
+      <c r="H1" s="195"/>
+      <c r="I1" s="195"/>
+      <c r="J1" s="195"/>
+      <c r="K1" s="195"/>
+      <c r="L1" s="195"/>
+      <c r="M1" s="196"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="242" t="s">
+      <c r="B2" s="197" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="243"/>
-      <c r="D2" s="243"/>
-      <c r="E2" s="243"/>
-      <c r="F2" s="243"/>
-      <c r="G2" s="243"/>
-      <c r="H2" s="243"/>
-      <c r="I2" s="244"/>
-      <c r="J2" s="248"/>
-      <c r="K2" s="249"/>
-      <c r="L2" s="249"/>
-      <c r="M2" s="250"/>
+      <c r="C2" s="198"/>
+      <c r="D2" s="198"/>
+      <c r="E2" s="198"/>
+      <c r="F2" s="198"/>
+      <c r="G2" s="198"/>
+      <c r="H2" s="198"/>
+      <c r="I2" s="199"/>
+      <c r="J2" s="203"/>
+      <c r="K2" s="204"/>
+      <c r="L2" s="204"/>
+      <c r="M2" s="205"/>
     </row>
     <row r="3" spans="1:14" ht="14.4" customHeight="1">
-      <c r="B3" s="245"/>
-      <c r="C3" s="246"/>
-      <c r="D3" s="246"/>
-      <c r="E3" s="246"/>
-      <c r="F3" s="246"/>
-      <c r="G3" s="246"/>
-      <c r="H3" s="246"/>
-      <c r="I3" s="247"/>
-      <c r="J3" s="251"/>
-      <c r="K3" s="252"/>
-      <c r="L3" s="252"/>
-      <c r="M3" s="253"/>
+      <c r="B3" s="200"/>
+      <c r="C3" s="201"/>
+      <c r="D3" s="201"/>
+      <c r="E3" s="201"/>
+      <c r="F3" s="201"/>
+      <c r="G3" s="201"/>
+      <c r="H3" s="201"/>
+      <c r="I3" s="202"/>
+      <c r="J3" s="206"/>
+      <c r="K3" s="207"/>
+      <c r="L3" s="207"/>
+      <c r="M3" s="208"/>
     </row>
     <row r="4" spans="1:14" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -3992,10 +4140,10 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="251"/>
-      <c r="K4" s="252"/>
-      <c r="L4" s="252"/>
-      <c r="M4" s="253"/>
+      <c r="J4" s="206"/>
+      <c r="K4" s="207"/>
+      <c r="L4" s="207"/>
+      <c r="M4" s="208"/>
     </row>
     <row r="5" spans="1:14" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -4010,10 +4158,10 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="251"/>
-      <c r="K5" s="252"/>
-      <c r="L5" s="252"/>
-      <c r="M5" s="253"/>
+      <c r="J5" s="206"/>
+      <c r="K5" s="207"/>
+      <c r="L5" s="207"/>
+      <c r="M5" s="208"/>
     </row>
     <row r="6" spans="1:14" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -4028,10 +4176,10 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="254"/>
-      <c r="K6" s="255"/>
-      <c r="L6" s="255"/>
-      <c r="M6" s="256"/>
+      <c r="J6" s="209"/>
+      <c r="K6" s="210"/>
+      <c r="L6" s="210"/>
+      <c r="M6" s="211"/>
     </row>
     <row r="7" spans="1:14" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -4096,52 +4244,52 @@
       <c r="M9" s="89"/>
     </row>
     <row r="10" spans="1:14" ht="15.6">
-      <c r="B10" s="186" t="s">
+      <c r="B10" s="212" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="187"/>
-      <c r="D10" s="187"/>
-      <c r="E10" s="187"/>
-      <c r="F10" s="187"/>
-      <c r="G10" s="187" t="s">
+      <c r="C10" s="213"/>
+      <c r="D10" s="213"/>
+      <c r="E10" s="213"/>
+      <c r="F10" s="213"/>
+      <c r="G10" s="213" t="s">
         <v>95</v>
       </c>
-      <c r="H10" s="187"/>
-      <c r="I10" s="187"/>
-      <c r="J10" s="188"/>
-      <c r="K10" s="189" t="s">
+      <c r="H10" s="213"/>
+      <c r="I10" s="213"/>
+      <c r="J10" s="214"/>
+      <c r="K10" s="215" t="s">
         <v>96</v>
       </c>
-      <c r="L10" s="187"/>
-      <c r="M10" s="257"/>
+      <c r="L10" s="213"/>
+      <c r="M10" s="216"/>
     </row>
     <row r="11" spans="1:14" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="216" t="s">
+      <c r="C11" s="226" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="217"/>
-      <c r="E11" s="217"/>
+      <c r="D11" s="227"/>
+      <c r="E11" s="227"/>
       <c r="F11" s="92" t="s">
         <v>98</v>
       </c>
-      <c r="G11" s="216" t="s">
+      <c r="G11" s="226" t="s">
         <v>99</v>
       </c>
-      <c r="H11" s="218"/>
+      <c r="H11" s="228"/>
       <c r="I11" s="93" t="s">
         <v>27</v>
       </c>
       <c r="J11" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="216" t="s">
+      <c r="K11" s="226" t="s">
         <v>100</v>
       </c>
-      <c r="L11" s="218"/>
+      <c r="L11" s="228"/>
       <c r="M11" s="94" t="s">
         <v>101</v>
       </c>
@@ -4346,58 +4494,58 @@
       <c r="M22" s="123"/>
     </row>
     <row r="23" spans="1:13" ht="16.2" thickBot="1">
-      <c r="B23" s="219"/>
-      <c r="C23" s="220"/>
-      <c r="D23" s="220"/>
-      <c r="E23" s="220"/>
+      <c r="B23" s="229"/>
+      <c r="C23" s="230"/>
+      <c r="D23" s="230"/>
+      <c r="E23" s="230"/>
       <c r="F23" s="124"/>
       <c r="G23" s="124"/>
       <c r="H23" s="125"/>
       <c r="I23" s="125"/>
-      <c r="J23" s="221"/>
-      <c r="K23" s="221"/>
-      <c r="L23" s="221"/>
-      <c r="M23" s="222"/>
+      <c r="J23" s="231"/>
+      <c r="K23" s="231"/>
+      <c r="L23" s="231"/>
+      <c r="M23" s="232"/>
     </row>
     <row r="24" spans="1:13" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="152" t="s">
         <v>116</v>
       </c>
-      <c r="B24" s="223" t="s">
+      <c r="B24" s="233" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="225" t="s">
+      <c r="C24" s="235" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="225"/>
-      <c r="E24" s="225"/>
-      <c r="F24" s="225"/>
-      <c r="G24" s="225"/>
-      <c r="H24" s="225"/>
-      <c r="I24" s="225"/>
-      <c r="J24" s="227" t="s">
+      <c r="D24" s="235"/>
+      <c r="E24" s="235"/>
+      <c r="F24" s="235"/>
+      <c r="G24" s="235"/>
+      <c r="H24" s="235"/>
+      <c r="I24" s="235"/>
+      <c r="J24" s="237" t="s">
         <v>117</v>
       </c>
-      <c r="K24" s="228"/>
-      <c r="L24" s="228"/>
-      <c r="M24" s="229"/>
+      <c r="K24" s="238"/>
+      <c r="L24" s="238"/>
+      <c r="M24" s="239"/>
     </row>
     <row r="25" spans="1:13" ht="31.2">
-      <c r="B25" s="224"/>
-      <c r="C25" s="226"/>
-      <c r="D25" s="226"/>
-      <c r="E25" s="226"/>
-      <c r="F25" s="226"/>
-      <c r="G25" s="226"/>
-      <c r="H25" s="226"/>
-      <c r="I25" s="226"/>
+      <c r="B25" s="234"/>
+      <c r="C25" s="236"/>
+      <c r="D25" s="236"/>
+      <c r="E25" s="236"/>
+      <c r="F25" s="236"/>
+      <c r="G25" s="236"/>
+      <c r="H25" s="236"/>
+      <c r="I25" s="236"/>
       <c r="J25" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="181" t="s">
+      <c r="K25" s="249" t="s">
         <v>118</v>
       </c>
-      <c r="L25" s="182"/>
+      <c r="L25" s="250"/>
       <c r="M25" s="126" t="s">
         <v>119</v>
       </c>
@@ -4955,60 +5103,60 @@
       </c>
     </row>
     <row r="49" spans="2:13" ht="16.2" thickTop="1">
-      <c r="B49" s="201" t="s">
+      <c r="B49" s="260" t="s">
         <v>120</v>
       </c>
-      <c r="C49" s="202"/>
-      <c r="D49" s="202"/>
-      <c r="E49" s="202"/>
-      <c r="F49" s="202"/>
-      <c r="G49" s="202"/>
-      <c r="H49" s="202"/>
-      <c r="I49" s="202"/>
-      <c r="J49" s="203"/>
-      <c r="K49" s="213" t="s">
+      <c r="C49" s="261"/>
+      <c r="D49" s="261"/>
+      <c r="E49" s="261"/>
+      <c r="F49" s="261"/>
+      <c r="G49" s="261"/>
+      <c r="H49" s="261"/>
+      <c r="I49" s="261"/>
+      <c r="J49" s="262"/>
+      <c r="K49" s="223" t="s">
         <v>121</v>
       </c>
-      <c r="L49" s="214"/>
-      <c r="M49" s="215"/>
+      <c r="L49" s="224"/>
+      <c r="M49" s="225"/>
     </row>
     <row r="50" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B50" s="204"/>
-      <c r="C50" s="205"/>
-      <c r="D50" s="205"/>
-      <c r="E50" s="205"/>
-      <c r="F50" s="205"/>
-      <c r="G50" s="205"/>
-      <c r="H50" s="205"/>
-      <c r="I50" s="205"/>
-      <c r="J50" s="206"/>
-      <c r="K50" s="210"/>
-      <c r="L50" s="211"/>
-      <c r="M50" s="212"/>
+      <c r="B50" s="263"/>
+      <c r="C50" s="264"/>
+      <c r="D50" s="264"/>
+      <c r="E50" s="264"/>
+      <c r="F50" s="264"/>
+      <c r="G50" s="264"/>
+      <c r="H50" s="264"/>
+      <c r="I50" s="264"/>
+      <c r="J50" s="265"/>
+      <c r="K50" s="220"/>
+      <c r="L50" s="221"/>
+      <c r="M50" s="222"/>
     </row>
     <row r="51" spans="2:13" ht="15.6">
       <c r="B51" s="138"/>
-      <c r="C51" s="207"/>
-      <c r="D51" s="207"/>
-      <c r="E51" s="207"/>
-      <c r="F51" s="207"/>
-      <c r="G51" s="207"/>
-      <c r="H51" s="207"/>
-      <c r="I51" s="207"/>
+      <c r="C51" s="217"/>
+      <c r="D51" s="217"/>
+      <c r="E51" s="217"/>
+      <c r="F51" s="217"/>
+      <c r="G51" s="217"/>
+      <c r="H51" s="217"/>
+      <c r="I51" s="217"/>
       <c r="J51" s="139"/>
-      <c r="K51" s="236"/>
-      <c r="L51" s="237"/>
-      <c r="M51" s="238"/>
+      <c r="K51" s="246"/>
+      <c r="L51" s="247"/>
+      <c r="M51" s="248"/>
     </row>
     <row r="52" spans="2:13" ht="15.6">
       <c r="B52" s="140"/>
-      <c r="C52" s="208"/>
-      <c r="D52" s="208"/>
-      <c r="E52" s="208"/>
-      <c r="F52" s="208"/>
-      <c r="G52" s="208"/>
-      <c r="H52" s="208"/>
-      <c r="I52" s="208"/>
+      <c r="C52" s="218"/>
+      <c r="D52" s="218"/>
+      <c r="E52" s="218"/>
+      <c r="F52" s="218"/>
+      <c r="G52" s="218"/>
+      <c r="H52" s="218"/>
+      <c r="I52" s="218"/>
       <c r="J52" s="141"/>
       <c r="K52" s="164"/>
       <c r="L52" s="161"/>
@@ -5016,13 +5164,13 @@
     </row>
     <row r="53" spans="2:13" ht="15.6">
       <c r="B53" s="140"/>
-      <c r="C53" s="208"/>
-      <c r="D53" s="208"/>
-      <c r="E53" s="208"/>
-      <c r="F53" s="208"/>
-      <c r="G53" s="208"/>
-      <c r="H53" s="208"/>
-      <c r="I53" s="208"/>
+      <c r="C53" s="218"/>
+      <c r="D53" s="218"/>
+      <c r="E53" s="218"/>
+      <c r="F53" s="218"/>
+      <c r="G53" s="218"/>
+      <c r="H53" s="218"/>
+      <c r="I53" s="218"/>
       <c r="J53" s="141"/>
       <c r="K53" s="164"/>
       <c r="L53" s="161"/>
@@ -5030,13 +5178,13 @@
     </row>
     <row r="54" spans="2:13" ht="15.6">
       <c r="B54" s="140"/>
-      <c r="C54" s="208"/>
-      <c r="D54" s="208"/>
-      <c r="E54" s="208"/>
-      <c r="F54" s="208"/>
-      <c r="G54" s="208"/>
-      <c r="H54" s="208"/>
-      <c r="I54" s="208"/>
+      <c r="C54" s="218"/>
+      <c r="D54" s="218"/>
+      <c r="E54" s="218"/>
+      <c r="F54" s="218"/>
+      <c r="G54" s="218"/>
+      <c r="H54" s="218"/>
+      <c r="I54" s="218"/>
       <c r="J54" s="141"/>
       <c r="K54" s="164"/>
       <c r="L54" s="161"/>
@@ -5044,13 +5192,13 @@
     </row>
     <row r="55" spans="2:13" ht="15.6">
       <c r="B55" s="143"/>
-      <c r="C55" s="208"/>
-      <c r="D55" s="208"/>
-      <c r="E55" s="208"/>
-      <c r="F55" s="208"/>
-      <c r="G55" s="208"/>
-      <c r="H55" s="208"/>
-      <c r="I55" s="208"/>
+      <c r="C55" s="218"/>
+      <c r="D55" s="218"/>
+      <c r="E55" s="218"/>
+      <c r="F55" s="218"/>
+      <c r="G55" s="218"/>
+      <c r="H55" s="218"/>
+      <c r="I55" s="218"/>
       <c r="J55" s="144"/>
       <c r="K55" s="164"/>
       <c r="L55" s="145"/>
@@ -5058,13 +5206,13 @@
     </row>
     <row r="56" spans="2:13" ht="15.6">
       <c r="B56" s="143"/>
-      <c r="C56" s="208"/>
-      <c r="D56" s="208"/>
-      <c r="E56" s="208"/>
-      <c r="F56" s="208"/>
-      <c r="G56" s="208"/>
-      <c r="H56" s="208"/>
-      <c r="I56" s="208"/>
+      <c r="C56" s="218"/>
+      <c r="D56" s="218"/>
+      <c r="E56" s="218"/>
+      <c r="F56" s="218"/>
+      <c r="G56" s="218"/>
+      <c r="H56" s="218"/>
+      <c r="I56" s="218"/>
       <c r="J56" s="144"/>
       <c r="K56" s="164"/>
       <c r="L56" s="145"/>
@@ -5072,41 +5220,41 @@
     </row>
     <row r="57" spans="2:13" ht="15.6">
       <c r="B57" s="143"/>
-      <c r="C57" s="208"/>
-      <c r="D57" s="208"/>
-      <c r="E57" s="208"/>
-      <c r="F57" s="208"/>
-      <c r="G57" s="208"/>
-      <c r="H57" s="208"/>
-      <c r="I57" s="208"/>
+      <c r="C57" s="218"/>
+      <c r="D57" s="218"/>
+      <c r="E57" s="218"/>
+      <c r="F57" s="218"/>
+      <c r="G57" s="218"/>
+      <c r="H57" s="218"/>
+      <c r="I57" s="218"/>
       <c r="J57" s="144"/>
-      <c r="K57" s="230"/>
-      <c r="L57" s="231"/>
-      <c r="M57" s="232"/>
+      <c r="K57" s="240"/>
+      <c r="L57" s="241"/>
+      <c r="M57" s="242"/>
     </row>
     <row r="58" spans="2:13" ht="15.6">
       <c r="B58" s="143"/>
-      <c r="C58" s="208"/>
-      <c r="D58" s="208"/>
-      <c r="E58" s="208"/>
-      <c r="F58" s="208"/>
-      <c r="G58" s="208"/>
-      <c r="H58" s="208"/>
-      <c r="I58" s="208"/>
+      <c r="C58" s="218"/>
+      <c r="D58" s="218"/>
+      <c r="E58" s="218"/>
+      <c r="F58" s="218"/>
+      <c r="G58" s="218"/>
+      <c r="H58" s="218"/>
+      <c r="I58" s="218"/>
       <c r="J58" s="144"/>
-      <c r="K58" s="233"/>
-      <c r="L58" s="234"/>
-      <c r="M58" s="235"/>
+      <c r="K58" s="243"/>
+      <c r="L58" s="244"/>
+      <c r="M58" s="245"/>
     </row>
     <row r="59" spans="2:13" ht="15.6">
       <c r="B59" s="143"/>
-      <c r="C59" s="208"/>
-      <c r="D59" s="208"/>
-      <c r="E59" s="208"/>
-      <c r="F59" s="208"/>
-      <c r="G59" s="208"/>
-      <c r="H59" s="208"/>
-      <c r="I59" s="208"/>
+      <c r="C59" s="218"/>
+      <c r="D59" s="218"/>
+      <c r="E59" s="218"/>
+      <c r="F59" s="218"/>
+      <c r="G59" s="218"/>
+      <c r="H59" s="218"/>
+      <c r="I59" s="218"/>
       <c r="J59" s="144"/>
       <c r="K59" s="164"/>
       <c r="L59" s="162"/>
@@ -5114,13 +5262,13 @@
     </row>
     <row r="60" spans="2:13" ht="15.6">
       <c r="B60" s="143"/>
-      <c r="C60" s="208"/>
-      <c r="D60" s="208"/>
-      <c r="E60" s="208"/>
-      <c r="F60" s="208"/>
-      <c r="G60" s="208"/>
-      <c r="H60" s="208"/>
-      <c r="I60" s="208"/>
+      <c r="C60" s="218"/>
+      <c r="D60" s="218"/>
+      <c r="E60" s="218"/>
+      <c r="F60" s="218"/>
+      <c r="G60" s="218"/>
+      <c r="H60" s="218"/>
+      <c r="I60" s="218"/>
       <c r="J60" s="144"/>
       <c r="K60" s="164"/>
       <c r="L60" s="162"/>
@@ -5128,13 +5276,13 @@
     </row>
     <row r="61" spans="2:13" ht="15.6">
       <c r="B61" s="143"/>
-      <c r="C61" s="209"/>
-      <c r="D61" s="209"/>
-      <c r="E61" s="209"/>
-      <c r="F61" s="209"/>
-      <c r="G61" s="209"/>
-      <c r="H61" s="209"/>
-      <c r="I61" s="209"/>
+      <c r="C61" s="219"/>
+      <c r="D61" s="219"/>
+      <c r="E61" s="219"/>
+      <c r="F61" s="219"/>
+      <c r="G61" s="219"/>
+      <c r="H61" s="219"/>
+      <c r="I61" s="219"/>
       <c r="J61" s="144"/>
       <c r="K61" s="164"/>
       <c r="L61" s="162"/>
@@ -5155,133 +5303,133 @@
       <c r="M62" s="167"/>
     </row>
     <row r="63" spans="2:13" ht="15.6">
-      <c r="B63" s="186" t="s">
+      <c r="B63" s="212" t="s">
         <v>122</v>
       </c>
-      <c r="C63" s="187"/>
-      <c r="D63" s="187"/>
-      <c r="E63" s="188"/>
-      <c r="F63" s="189" t="s">
+      <c r="C63" s="213"/>
+      <c r="D63" s="213"/>
+      <c r="E63" s="214"/>
+      <c r="F63" s="215" t="s">
         <v>123</v>
       </c>
-      <c r="G63" s="188"/>
-      <c r="H63" s="189" t="s">
+      <c r="G63" s="214"/>
+      <c r="H63" s="215" t="s">
         <v>124</v>
       </c>
-      <c r="I63" s="187"/>
-      <c r="J63" s="188"/>
+      <c r="I63" s="213"/>
+      <c r="J63" s="214"/>
       <c r="K63" s="165"/>
       <c r="L63" s="145"/>
       <c r="M63" s="146"/>
     </row>
     <row r="64" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B64" s="190"/>
-      <c r="C64" s="191"/>
-      <c r="D64" s="191"/>
-      <c r="E64" s="193"/>
-      <c r="F64" s="192"/>
-      <c r="G64" s="193"/>
-      <c r="H64" s="194"/>
-      <c r="I64" s="195"/>
-      <c r="J64" s="196"/>
+      <c r="B64" s="188"/>
+      <c r="C64" s="189"/>
+      <c r="D64" s="189"/>
+      <c r="E64" s="183"/>
+      <c r="F64" s="182"/>
+      <c r="G64" s="183"/>
+      <c r="H64" s="251"/>
+      <c r="I64" s="252"/>
+      <c r="J64" s="253"/>
       <c r="K64" s="148"/>
       <c r="L64" s="145"/>
       <c r="M64" s="146"/>
     </row>
     <row r="65" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B65" s="185"/>
-      <c r="C65" s="263"/>
-      <c r="D65" s="263"/>
-      <c r="E65" s="184"/>
-      <c r="F65" s="183"/>
-      <c r="G65" s="184"/>
-      <c r="H65" s="179"/>
-      <c r="I65" s="180"/>
-      <c r="J65" s="197"/>
+      <c r="B65" s="190"/>
+      <c r="C65" s="191"/>
+      <c r="D65" s="191"/>
+      <c r="E65" s="185"/>
+      <c r="F65" s="184"/>
+      <c r="G65" s="185"/>
+      <c r="H65" s="254"/>
+      <c r="I65" s="255"/>
+      <c r="J65" s="256"/>
       <c r="K65" s="148"/>
       <c r="L65" s="163"/>
       <c r="M65" s="146"/>
     </row>
     <row r="66" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B66" s="185"/>
-      <c r="C66" s="263"/>
-      <c r="D66" s="263"/>
-      <c r="E66" s="184"/>
-      <c r="F66" s="183"/>
-      <c r="G66" s="184"/>
-      <c r="H66" s="179"/>
-      <c r="I66" s="180"/>
-      <c r="J66" s="197"/>
+      <c r="B66" s="190"/>
+      <c r="C66" s="191"/>
+      <c r="D66" s="191"/>
+      <c r="E66" s="185"/>
+      <c r="F66" s="184"/>
+      <c r="G66" s="185"/>
+      <c r="H66" s="254"/>
+      <c r="I66" s="255"/>
+      <c r="J66" s="256"/>
       <c r="K66" s="148"/>
       <c r="L66" s="145"/>
       <c r="M66" s="146"/>
     </row>
     <row r="67" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B67" s="185"/>
-      <c r="C67" s="263"/>
-      <c r="D67" s="263"/>
-      <c r="E67" s="184"/>
-      <c r="F67" s="183"/>
-      <c r="G67" s="184"/>
-      <c r="H67" s="179"/>
-      <c r="I67" s="180"/>
-      <c r="J67" s="197"/>
+      <c r="B67" s="190"/>
+      <c r="C67" s="191"/>
+      <c r="D67" s="191"/>
+      <c r="E67" s="185"/>
+      <c r="F67" s="184"/>
+      <c r="G67" s="185"/>
+      <c r="H67" s="254"/>
+      <c r="I67" s="255"/>
+      <c r="J67" s="256"/>
       <c r="K67" s="148"/>
       <c r="L67" s="162"/>
       <c r="M67" s="76"/>
     </row>
     <row r="68" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B68" s="185"/>
-      <c r="C68" s="263"/>
-      <c r="D68" s="263"/>
-      <c r="E68" s="184"/>
-      <c r="F68" s="183"/>
-      <c r="G68" s="184"/>
-      <c r="H68" s="179"/>
-      <c r="I68" s="180"/>
-      <c r="J68" s="197"/>
+      <c r="B68" s="190"/>
+      <c r="C68" s="191"/>
+      <c r="D68" s="191"/>
+      <c r="E68" s="185"/>
+      <c r="F68" s="184"/>
+      <c r="G68" s="185"/>
+      <c r="H68" s="254"/>
+      <c r="I68" s="255"/>
+      <c r="J68" s="256"/>
       <c r="K68" s="148"/>
       <c r="L68" s="162"/>
       <c r="M68" s="76"/>
     </row>
     <row r="69" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B69" s="185"/>
-      <c r="C69" s="263"/>
-      <c r="D69" s="263"/>
-      <c r="E69" s="184"/>
-      <c r="F69" s="183"/>
-      <c r="G69" s="184"/>
-      <c r="H69" s="179"/>
-      <c r="I69" s="180"/>
-      <c r="J69" s="197"/>
-      <c r="K69" s="266"/>
-      <c r="L69" s="267"/>
-      <c r="M69" s="268"/>
+      <c r="B69" s="190"/>
+      <c r="C69" s="191"/>
+      <c r="D69" s="191"/>
+      <c r="E69" s="185"/>
+      <c r="F69" s="184"/>
+      <c r="G69" s="185"/>
+      <c r="H69" s="254"/>
+      <c r="I69" s="255"/>
+      <c r="J69" s="256"/>
+      <c r="K69" s="168"/>
+      <c r="L69" s="169"/>
+      <c r="M69" s="170"/>
     </row>
     <row r="70" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B70" s="185"/>
-      <c r="C70" s="263"/>
-      <c r="D70" s="263"/>
-      <c r="E70" s="184"/>
-      <c r="F70" s="183"/>
-      <c r="G70" s="184"/>
-      <c r="H70" s="179"/>
-      <c r="I70" s="180"/>
-      <c r="J70" s="197"/>
-      <c r="K70" s="266"/>
-      <c r="L70" s="267"/>
-      <c r="M70" s="268"/>
+      <c r="B70" s="190"/>
+      <c r="C70" s="191"/>
+      <c r="D70" s="191"/>
+      <c r="E70" s="185"/>
+      <c r="F70" s="184"/>
+      <c r="G70" s="185"/>
+      <c r="H70" s="254"/>
+      <c r="I70" s="255"/>
+      <c r="J70" s="256"/>
+      <c r="K70" s="168"/>
+      <c r="L70" s="169"/>
+      <c r="M70" s="170"/>
     </row>
     <row r="71" spans="2:13" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B71" s="264"/>
-      <c r="C71" s="265"/>
-      <c r="D71" s="265"/>
-      <c r="E71" s="262"/>
-      <c r="F71" s="261"/>
-      <c r="G71" s="262"/>
-      <c r="H71" s="198"/>
-      <c r="I71" s="199"/>
-      <c r="J71" s="200"/>
+      <c r="B71" s="192"/>
+      <c r="C71" s="193"/>
+      <c r="D71" s="193"/>
+      <c r="E71" s="187"/>
+      <c r="F71" s="186"/>
+      <c r="G71" s="187"/>
+      <c r="H71" s="257"/>
+      <c r="I71" s="258"/>
+      <c r="J71" s="259"/>
       <c r="K71" s="150"/>
       <c r="L71" s="149"/>
       <c r="M71" s="151"/>
@@ -5294,6 +5442,18 @@
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="H63:J63"/>
+    <mergeCell ref="H64:J71"/>
+    <mergeCell ref="B49:J50"/>
+    <mergeCell ref="C24:I25"/>
+    <mergeCell ref="J24:M24"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="K58:M58"/>
+    <mergeCell ref="K51:M51"/>
+    <mergeCell ref="K25:L25"/>
     <mergeCell ref="F64:G71"/>
     <mergeCell ref="B64:E71"/>
     <mergeCell ref="B1:M1"/>
@@ -5310,26 +5470,14 @@
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="J23:M23"/>
     <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:I25"/>
-    <mergeCell ref="J24:M24"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="K57:M57"/>
-    <mergeCell ref="K58:M58"/>
-    <mergeCell ref="K51:M51"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="H63:J63"/>
-    <mergeCell ref="H64:J71"/>
-    <mergeCell ref="B49:J50"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:I48">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="24" priority="1">
       <formula>ISTEXT($C26)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J27:M48">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5367,40 +5515,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="175"/>
-      <c r="C1" s="175"/>
-      <c r="D1" s="175"/>
-      <c r="E1" s="175"/>
-      <c r="F1" s="175"/>
-      <c r="G1" s="175"/>
-      <c r="H1" s="175"/>
-      <c r="I1" s="175"/>
-      <c r="J1" s="175"/>
-      <c r="K1" s="175"/>
-      <c r="L1" s="175"/>
-      <c r="M1" s="175"/>
-      <c r="N1" s="175"/>
-      <c r="O1" s="175"/>
-      <c r="P1" s="175"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="173" t="s">
+      <c r="B2" s="176" t="s">
         <v>125</v>
       </c>
-      <c r="C2" s="174"/>
-      <c r="D2" s="174"/>
-      <c r="E2" s="174"/>
-      <c r="F2" s="174"/>
-      <c r="G2" s="174"/>
-      <c r="H2" s="174"/>
-      <c r="I2" s="174"/>
-      <c r="J2" s="174"/>
-      <c r="K2" s="174"/>
-      <c r="L2" s="174"/>
-      <c r="M2" s="174"/>
-      <c r="N2" s="174"/>
-      <c r="O2" s="174"/>
-      <c r="P2" s="174"/>
+      <c r="C2" s="177"/>
+      <c r="D2" s="177"/>
+      <c r="E2" s="177"/>
+      <c r="F2" s="177"/>
+      <c r="G2" s="177"/>
+      <c r="H2" s="177"/>
+      <c r="I2" s="177"/>
+      <c r="J2" s="177"/>
+      <c r="K2" s="177"/>
+      <c r="L2" s="177"/>
+      <c r="M2" s="177"/>
+      <c r="N2" s="177"/>
+      <c r="O2" s="177"/>
+      <c r="P2" s="177"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -5427,16 +5575,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="260" t="s">
+      <c r="I4" s="268" t="s">
         <v>86</v>
       </c>
-      <c r="J4" s="260"/>
-      <c r="K4" s="260"/>
-      <c r="L4" s="260"/>
-      <c r="M4" s="260"/>
-      <c r="N4" s="260"/>
-      <c r="O4" s="260"/>
-      <c r="P4" s="260"/>
+      <c r="J4" s="268"/>
+      <c r="K4" s="268"/>
+      <c r="L4" s="268"/>
+      <c r="M4" s="268"/>
+      <c r="N4" s="268"/>
+      <c r="O4" s="268"/>
+      <c r="P4" s="268"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -5450,14 +5598,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="260"/>
-      <c r="J5" s="260"/>
-      <c r="K5" s="260"/>
-      <c r="L5" s="260"/>
-      <c r="M5" s="260"/>
-      <c r="N5" s="260"/>
-      <c r="O5" s="260"/>
-      <c r="P5" s="260"/>
+      <c r="I5" s="268"/>
+      <c r="J5" s="268"/>
+      <c r="K5" s="268"/>
+      <c r="L5" s="268"/>
+      <c r="M5" s="268"/>
+      <c r="N5" s="268"/>
+      <c r="O5" s="268"/>
+      <c r="P5" s="268"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -5592,70 +5740,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="172" t="s">
+      <c r="B12" s="175" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="172" t="s">
+      <c r="C12" s="175" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="172"/>
-      <c r="E12" s="172"/>
-      <c r="F12" s="172" t="s">
+      <c r="D12" s="175"/>
+      <c r="E12" s="175"/>
+      <c r="F12" s="175" t="s">
         <v>131</v>
       </c>
-      <c r="G12" s="172" t="s">
+      <c r="G12" s="175" t="s">
         <v>133</v>
       </c>
-      <c r="H12" s="172" t="s">
+      <c r="H12" s="175" t="s">
         <v>132</v>
       </c>
-      <c r="I12" s="172" t="s">
+      <c r="I12" s="175" t="s">
         <v>134</v>
       </c>
-      <c r="J12" s="172" t="s">
+      <c r="J12" s="175" t="s">
         <v>138</v>
       </c>
-      <c r="K12" s="172"/>
-      <c r="L12" s="172"/>
-      <c r="M12" s="172"/>
-      <c r="N12" s="172"/>
-      <c r="O12" s="172"/>
-      <c r="P12" s="259" t="s">
+      <c r="K12" s="175"/>
+      <c r="L12" s="175"/>
+      <c r="M12" s="175"/>
+      <c r="N12" s="175"/>
+      <c r="O12" s="175"/>
+      <c r="P12" s="267" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="172"/>
-      <c r="C13" s="172"/>
-      <c r="D13" s="172"/>
-      <c r="E13" s="172"/>
-      <c r="F13" s="172"/>
-      <c r="G13" s="172"/>
-      <c r="H13" s="172"/>
-      <c r="I13" s="172"/>
-      <c r="J13" s="258" t="s">
+      <c r="B13" s="175"/>
+      <c r="C13" s="175"/>
+      <c r="D13" s="175"/>
+      <c r="E13" s="175"/>
+      <c r="F13" s="175"/>
+      <c r="G13" s="175"/>
+      <c r="H13" s="175"/>
+      <c r="I13" s="175"/>
+      <c r="J13" s="266" t="s">
         <v>135</v>
       </c>
-      <c r="K13" s="258"/>
-      <c r="L13" s="258" t="s">
+      <c r="K13" s="266"/>
+      <c r="L13" s="266" t="s">
         <v>140</v>
       </c>
-      <c r="M13" s="258"/>
-      <c r="N13" s="258" t="s">
+      <c r="M13" s="266"/>
+      <c r="N13" s="266" t="s">
         <v>141</v>
       </c>
-      <c r="O13" s="258"/>
-      <c r="P13" s="259"/>
+      <c r="O13" s="266"/>
+      <c r="P13" s="267"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="172"/>
-      <c r="C14" s="172"/>
-      <c r="D14" s="172"/>
-      <c r="E14" s="172"/>
-      <c r="F14" s="172"/>
-      <c r="G14" s="172"/>
-      <c r="H14" s="172"/>
-      <c r="I14" s="172"/>
+      <c r="B14" s="175"/>
+      <c r="C14" s="175"/>
+      <c r="D14" s="175"/>
+      <c r="E14" s="175"/>
+      <c r="F14" s="175"/>
+      <c r="G14" s="175"/>
+      <c r="H14" s="175"/>
+      <c r="I14" s="175"/>
       <c r="J14" s="38" t="s">
         <v>118</v>
       </c>
@@ -5674,7 +5822,7 @@
       <c r="O14" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="P14" s="259"/>
+      <c r="P14" s="267"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -6024,7 +6172,7 @@
     <mergeCell ref="I4:P5"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P49">
-    <cfRule type="expression" dxfId="1" priority="13">
+    <cfRule type="expression" dxfId="22" priority="13">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6062,40 +6210,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="175"/>
-      <c r="C1" s="175"/>
-      <c r="D1" s="175"/>
-      <c r="E1" s="175"/>
-      <c r="F1" s="175"/>
-      <c r="G1" s="175"/>
-      <c r="H1" s="175"/>
-      <c r="I1" s="175"/>
-      <c r="J1" s="175"/>
-      <c r="K1" s="175"/>
-      <c r="L1" s="175"/>
-      <c r="M1" s="175"/>
-      <c r="N1" s="175"/>
-      <c r="O1" s="175"/>
-      <c r="P1" s="175"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="178"/>
+      <c r="O1" s="178"/>
+      <c r="P1" s="178"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="173" t="s">
+      <c r="B2" s="176" t="s">
         <v>144</v>
       </c>
-      <c r="C2" s="174"/>
-      <c r="D2" s="174"/>
-      <c r="E2" s="174"/>
-      <c r="F2" s="174"/>
-      <c r="G2" s="174"/>
-      <c r="H2" s="174"/>
-      <c r="I2" s="174"/>
-      <c r="J2" s="174"/>
-      <c r="K2" s="174"/>
-      <c r="L2" s="174"/>
-      <c r="M2" s="174"/>
-      <c r="N2" s="174"/>
-      <c r="O2" s="174"/>
-      <c r="P2" s="174"/>
+      <c r="C2" s="177"/>
+      <c r="D2" s="177"/>
+      <c r="E2" s="177"/>
+      <c r="F2" s="177"/>
+      <c r="G2" s="177"/>
+      <c r="H2" s="177"/>
+      <c r="I2" s="177"/>
+      <c r="J2" s="177"/>
+      <c r="K2" s="177"/>
+      <c r="L2" s="177"/>
+      <c r="M2" s="177"/>
+      <c r="N2" s="177"/>
+      <c r="O2" s="177"/>
+      <c r="P2" s="177"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -6122,16 +6270,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="260" t="s">
+      <c r="I4" s="268" t="s">
         <v>86</v>
       </c>
-      <c r="J4" s="260"/>
-      <c r="K4" s="260"/>
-      <c r="L4" s="260"/>
-      <c r="M4" s="260"/>
-      <c r="N4" s="260"/>
-      <c r="O4" s="260"/>
-      <c r="P4" s="260"/>
+      <c r="J4" s="268"/>
+      <c r="K4" s="268"/>
+      <c r="L4" s="268"/>
+      <c r="M4" s="268"/>
+      <c r="N4" s="268"/>
+      <c r="O4" s="268"/>
+      <c r="P4" s="268"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -6145,14 +6293,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="260"/>
-      <c r="J5" s="260"/>
-      <c r="K5" s="260"/>
-      <c r="L5" s="260"/>
-      <c r="M5" s="260"/>
-      <c r="N5" s="260"/>
-      <c r="O5" s="260"/>
-      <c r="P5" s="260"/>
+      <c r="I5" s="268"/>
+      <c r="J5" s="268"/>
+      <c r="K5" s="268"/>
+      <c r="L5" s="268"/>
+      <c r="M5" s="268"/>
+      <c r="N5" s="268"/>
+      <c r="O5" s="268"/>
+      <c r="P5" s="268"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -6287,70 +6435,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="172" t="s">
+      <c r="B12" s="175" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="172" t="s">
+      <c r="C12" s="175" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="172"/>
-      <c r="E12" s="172"/>
-      <c r="F12" s="172" t="s">
+      <c r="D12" s="175"/>
+      <c r="E12" s="175"/>
+      <c r="F12" s="175" t="s">
         <v>131</v>
       </c>
-      <c r="G12" s="172" t="s">
+      <c r="G12" s="175" t="s">
         <v>133</v>
       </c>
-      <c r="H12" s="172" t="s">
+      <c r="H12" s="175" t="s">
         <v>132</v>
       </c>
-      <c r="I12" s="172" t="s">
+      <c r="I12" s="175" t="s">
         <v>134</v>
       </c>
-      <c r="J12" s="172" t="s">
+      <c r="J12" s="175" t="s">
         <v>138</v>
       </c>
-      <c r="K12" s="172"/>
-      <c r="L12" s="172"/>
-      <c r="M12" s="172"/>
-      <c r="N12" s="172"/>
-      <c r="O12" s="172"/>
-      <c r="P12" s="259" t="s">
+      <c r="K12" s="175"/>
+      <c r="L12" s="175"/>
+      <c r="M12" s="175"/>
+      <c r="N12" s="175"/>
+      <c r="O12" s="175"/>
+      <c r="P12" s="267" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="172"/>
-      <c r="C13" s="172"/>
-      <c r="D13" s="172"/>
-      <c r="E13" s="172"/>
-      <c r="F13" s="172"/>
-      <c r="G13" s="172"/>
-      <c r="H13" s="172"/>
-      <c r="I13" s="172"/>
-      <c r="J13" s="258" t="s">
+      <c r="B13" s="175"/>
+      <c r="C13" s="175"/>
+      <c r="D13" s="175"/>
+      <c r="E13" s="175"/>
+      <c r="F13" s="175"/>
+      <c r="G13" s="175"/>
+      <c r="H13" s="175"/>
+      <c r="I13" s="175"/>
+      <c r="J13" s="266" t="s">
         <v>135</v>
       </c>
-      <c r="K13" s="258"/>
-      <c r="L13" s="258" t="s">
+      <c r="K13" s="266"/>
+      <c r="L13" s="266" t="s">
         <v>136</v>
       </c>
-      <c r="M13" s="258"/>
-      <c r="N13" s="258" t="s">
+      <c r="M13" s="266"/>
+      <c r="N13" s="266" t="s">
         <v>137</v>
       </c>
-      <c r="O13" s="258"/>
-      <c r="P13" s="259"/>
+      <c r="O13" s="266"/>
+      <c r="P13" s="267"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="172"/>
-      <c r="C14" s="172"/>
-      <c r="D14" s="172"/>
-      <c r="E14" s="172"/>
-      <c r="F14" s="172"/>
-      <c r="G14" s="172"/>
-      <c r="H14" s="172"/>
-      <c r="I14" s="172"/>
+      <c r="B14" s="175"/>
+      <c r="C14" s="175"/>
+      <c r="D14" s="175"/>
+      <c r="E14" s="175"/>
+      <c r="F14" s="175"/>
+      <c r="G14" s="175"/>
+      <c r="H14" s="175"/>
+      <c r="I14" s="175"/>
       <c r="J14" s="38" t="s">
         <v>118</v>
       </c>
@@ -6369,7 +6517,7 @@
       <c r="O14" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="P14" s="259"/>
+      <c r="P14" s="267"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -6765,7 +6913,7 @@
     <mergeCell ref="G12:G14"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P51">
-    <cfRule type="expression" dxfId="0" priority="14">
+    <cfRule type="expression" dxfId="21" priority="14">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6793,38 +6941,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="171"/>
-      <c r="C1" s="171"/>
-      <c r="D1" s="171"/>
-      <c r="E1" s="171"/>
-      <c r="F1" s="171"/>
-      <c r="G1" s="171"/>
-      <c r="H1" s="171"/>
-      <c r="I1" s="171"/>
+      <c r="B1" s="174"/>
+      <c r="C1" s="174"/>
+      <c r="D1" s="174"/>
+      <c r="E1" s="174"/>
+      <c r="F1" s="174"/>
+      <c r="G1" s="174"/>
+      <c r="H1" s="174"/>
+      <c r="I1" s="174"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="171" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="168"/>
-      <c r="D2" s="168"/>
-      <c r="E2" s="168"/>
-      <c r="F2" s="168"/>
-      <c r="G2" s="168"/>
-      <c r="H2" s="168"/>
-      <c r="I2" s="168"/>
+      <c r="C2" s="171"/>
+      <c r="D2" s="171"/>
+      <c r="E2" s="171"/>
+      <c r="F2" s="171"/>
+      <c r="G2" s="171"/>
+      <c r="H2" s="171"/>
+      <c r="I2" s="171"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="169" t="s">
+      <c r="B3" s="172" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="169"/>
-      <c r="D3" s="169"/>
-      <c r="E3" s="169"/>
-      <c r="F3" s="169"/>
-      <c r="G3" s="169"/>
-      <c r="H3" s="169"/>
-      <c r="I3" s="169"/>
+      <c r="C3" s="172"/>
+      <c r="D3" s="172"/>
+      <c r="E3" s="172"/>
+      <c r="F3" s="172"/>
+      <c r="G3" s="172"/>
+      <c r="H3" s="172"/>
+      <c r="I3" s="172"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -6832,10 +6980,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="170" t="s">
+      <c r="C5" s="173" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="170"/>
+      <c r="D5" s="173"/>
       <c r="E5" s="11" t="s">
         <v>80</v>
       </c>
@@ -15189,7 +15337,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="25" priority="2">
+    <cfRule type="expression" dxfId="41" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15222,63 +15370,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="171"/>
-      <c r="C1" s="171"/>
-      <c r="D1" s="171"/>
-      <c r="E1" s="171"/>
-      <c r="F1" s="171"/>
-      <c r="G1" s="171"/>
-      <c r="H1" s="171"/>
-      <c r="I1" s="171"/>
-      <c r="J1" s="171"/>
-      <c r="K1" s="171"/>
-      <c r="L1" s="171"/>
-      <c r="M1" s="171"/>
-      <c r="N1" s="171"/>
+      <c r="B1" s="174"/>
+      <c r="C1" s="174"/>
+      <c r="D1" s="174"/>
+      <c r="E1" s="174"/>
+      <c r="F1" s="174"/>
+      <c r="G1" s="174"/>
+      <c r="H1" s="174"/>
+      <c r="I1" s="174"/>
+      <c r="J1" s="174"/>
+      <c r="K1" s="174"/>
+      <c r="L1" s="174"/>
+      <c r="M1" s="174"/>
+      <c r="N1" s="174"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="171" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="168"/>
-      <c r="D2" s="168"/>
-      <c r="E2" s="168"/>
-      <c r="F2" s="168"/>
-      <c r="G2" s="168"/>
-      <c r="H2" s="168"/>
-      <c r="I2" s="168"/>
-      <c r="J2" s="168"/>
-      <c r="K2" s="168"/>
-      <c r="L2" s="168"/>
-      <c r="M2" s="168"/>
-      <c r="N2" s="168"/>
+      <c r="C2" s="171"/>
+      <c r="D2" s="171"/>
+      <c r="E2" s="171"/>
+      <c r="F2" s="171"/>
+      <c r="G2" s="171"/>
+      <c r="H2" s="171"/>
+      <c r="I2" s="171"/>
+      <c r="J2" s="171"/>
+      <c r="K2" s="171"/>
+      <c r="L2" s="171"/>
+      <c r="M2" s="171"/>
+      <c r="N2" s="171"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="169" t="s">
+      <c r="B3" s="172" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="169"/>
-      <c r="D3" s="169"/>
-      <c r="E3" s="169"/>
-      <c r="F3" s="169"/>
-      <c r="G3" s="169"/>
-      <c r="H3" s="169"/>
-      <c r="I3" s="169"/>
-      <c r="J3" s="169"/>
-      <c r="K3" s="169"/>
-      <c r="L3" s="169"/>
-      <c r="M3" s="169"/>
-      <c r="N3" s="169"/>
+      <c r="C3" s="172"/>
+      <c r="D3" s="172"/>
+      <c r="E3" s="172"/>
+      <c r="F3" s="172"/>
+      <c r="G3" s="172"/>
+      <c r="H3" s="172"/>
+      <c r="I3" s="172"/>
+      <c r="J3" s="172"/>
+      <c r="K3" s="172"/>
+      <c r="L3" s="172"/>
+      <c r="M3" s="172"/>
+      <c r="N3" s="172"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="172" t="s">
+      <c r="C5" s="175" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="172"/>
+      <c r="D5" s="175"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -17439,23 +17587,20 @@
     <mergeCell ref="B1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:N16997">
-    <cfRule type="expression" dxfId="24" priority="1">
-      <formula>AND(LEN($B6)&lt;&gt;0,$C6&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>AND(LEN($B6)&lt;&gt;0,$D6=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="4">
-      <formula>AND(LEN($B6)=1,$D6&lt;&gt;0)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="5">
-      <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
+    <cfRule type="expression" dxfId="7" priority="4">
+      <formula>AND($B6&lt;&gt;"",$C6&lt;&gt;"",$D6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H16997">
-    <cfRule type="expression" dxfId="21" priority="8">
+    <cfRule type="expression" dxfId="6" priority="8">
       <formula>IF(G6&lt;&gt;"", NOT(AND(OR(LEFT($E6,2)="L.", LEFT($E6,2)="A.", LEFT($E6,2)="B.", LEFT($E6,2)="M."), $H6&lt;&gt;"", $E6&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:K16997">
-    <cfRule type="notContainsBlanks" dxfId="20" priority="7">
+    <cfRule type="notContainsBlanks" dxfId="5" priority="7">
       <formula>LEN(TRIM(H6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17482,35 +17627,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="171"/>
-      <c r="C1" s="171"/>
-      <c r="D1" s="171"/>
-      <c r="E1" s="171"/>
-      <c r="F1" s="171"/>
-      <c r="G1" s="171"/>
-      <c r="H1" s="171"/>
+      <c r="B1" s="174"/>
+      <c r="C1" s="174"/>
+      <c r="D1" s="174"/>
+      <c r="E1" s="174"/>
+      <c r="F1" s="174"/>
+      <c r="G1" s="174"/>
+      <c r="H1" s="174"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="171" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="168"/>
-      <c r="D2" s="168"/>
-      <c r="E2" s="168"/>
-      <c r="F2" s="168"/>
-      <c r="G2" s="168"/>
-      <c r="H2" s="168"/>
+      <c r="C2" s="171"/>
+      <c r="D2" s="171"/>
+      <c r="E2" s="171"/>
+      <c r="F2" s="171"/>
+      <c r="G2" s="171"/>
+      <c r="H2" s="171"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="169" t="s">
+      <c r="B3" s="172" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="169"/>
-      <c r="D3" s="169"/>
-      <c r="E3" s="169"/>
-      <c r="F3" s="169"/>
-      <c r="G3" s="169"/>
-      <c r="H3" s="169"/>
+      <c r="C3" s="172"/>
+      <c r="D3" s="172"/>
+      <c r="E3" s="172"/>
+      <c r="F3" s="172"/>
+      <c r="G3" s="172"/>
+      <c r="H3" s="172"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -41558,15 +41703,15 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B995 E6:H995">
-    <cfRule type="expression" dxfId="19" priority="6">
+    <cfRule type="expression" dxfId="40" priority="6">
       <formula>$J6=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:H995">
-    <cfRule type="expression" dxfId="18" priority="1">
+    <cfRule type="expression" dxfId="39" priority="1">
       <formula>AND(LEN($B6)=1,$C6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="2">
+    <cfRule type="expression" dxfId="38" priority="2">
       <formula>$C6&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -41601,30 +41746,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="175"/>
-      <c r="C1" s="175"/>
-      <c r="D1" s="175"/>
-      <c r="E1" s="175"/>
-      <c r="F1" s="175"/>
-      <c r="G1" s="175"/>
-      <c r="H1" s="175"/>
-      <c r="I1" s="175"/>
-      <c r="J1" s="175"/>
-      <c r="K1" s="175"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
+      <c r="I1" s="178"/>
+      <c r="J1" s="178"/>
+      <c r="K1" s="178"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="173" t="s">
+      <c r="B2" s="176" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="174"/>
-      <c r="D2" s="174"/>
-      <c r="E2" s="174"/>
-      <c r="F2" s="174"/>
-      <c r="G2" s="174"/>
-      <c r="H2" s="174"/>
-      <c r="I2" s="174"/>
-      <c r="J2" s="174"/>
-      <c r="K2" s="174"/>
+      <c r="C2" s="177"/>
+      <c r="D2" s="177"/>
+      <c r="E2" s="177"/>
+      <c r="F2" s="177"/>
+      <c r="G2" s="177"/>
+      <c r="H2" s="177"/>
+      <c r="I2" s="177"/>
+      <c r="J2" s="177"/>
+      <c r="K2" s="177"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -41744,11 +41889,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="172" t="s">
+      <c r="C11" s="175" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="172"/>
-      <c r="E11" s="172"/>
+      <c r="D11" s="175"/>
+      <c r="E11" s="175"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -43144,7 +43289,7 @@
     <mergeCell ref="B1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="B12:K9929">
-    <cfRule type="expression" dxfId="16" priority="1">
+    <cfRule type="expression" dxfId="37" priority="1">
       <formula>AND($B12&lt;&gt;"",$C12&lt;&gt;"",$G12="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -43177,24 +43322,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="111.6" customHeight="1">
-      <c r="B1" s="175"/>
-      <c r="C1" s="175"/>
-      <c r="D1" s="175"/>
-      <c r="E1" s="175"/>
-      <c r="F1" s="175"/>
-      <c r="G1" s="175"/>
-      <c r="H1" s="175"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="178"/>
     </row>
     <row r="2" spans="2:8" ht="22.95" customHeight="1">
-      <c r="B2" s="173" t="s">
+      <c r="B2" s="176" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="174"/>
-      <c r="D2" s="174"/>
-      <c r="E2" s="174"/>
-      <c r="F2" s="174"/>
-      <c r="G2" s="174"/>
-      <c r="H2" s="174"/>
+      <c r="C2" s="177"/>
+      <c r="D2" s="177"/>
+      <c r="E2" s="177"/>
+      <c r="F2" s="177"/>
+      <c r="G2" s="177"/>
+      <c r="H2" s="177"/>
     </row>
     <row r="3" spans="2:8" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -43296,11 +43441,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="172" t="s">
+      <c r="C11" s="175" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="172"/>
-      <c r="E11" s="172"/>
+      <c r="D11" s="175"/>
+      <c r="E11" s="175"/>
       <c r="F11" s="40" t="s">
         <v>29</v>
       </c>
@@ -44505,7 +44650,7 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B12:H9929">
-    <cfRule type="expression" dxfId="15" priority="9">
+    <cfRule type="expression" dxfId="36" priority="9">
       <formula>AND($B12&lt;&gt;"",$C12&lt;&gt;"",#REF!="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -44530,58 +44675,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="175"/>
-      <c r="C1" s="175"/>
-      <c r="D1" s="175"/>
-      <c r="E1" s="175"/>
-      <c r="F1" s="175"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="178" t="s">
+      <c r="B2" s="181" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="178"/>
-      <c r="D2" s="178"/>
-      <c r="E2" s="178"/>
-      <c r="F2" s="178"/>
+      <c r="C2" s="181"/>
+      <c r="D2" s="181"/>
+      <c r="E2" s="181"/>
+      <c r="F2" s="181"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="175"/>
-      <c r="C3" s="175"/>
-      <c r="D3" s="175"/>
-      <c r="E3" s="175"/>
-      <c r="F3" s="175"/>
+      <c r="B3" s="178"/>
+      <c r="C3" s="178"/>
+      <c r="D3" s="178"/>
+      <c r="E3" s="178"/>
+      <c r="F3" s="178"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="176" t="s">
+      <c r="B5" s="179" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="176" t="s">
+      <c r="C5" s="179" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="176" t="s">
+      <c r="D5" s="179" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="177" t="s">
+      <c r="E5" s="180" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="177" t="s">
+      <c r="F5" s="180" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="176"/>
-      <c r="C6" s="176"/>
-      <c r="D6" s="176"/>
-      <c r="E6" s="177"/>
-      <c r="F6" s="177"/>
+      <c r="B6" s="179"/>
+      <c r="C6" s="179"/>
+      <c r="D6" s="179"/>
+      <c r="E6" s="180"/>
+      <c r="F6" s="180"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="176"/>
-      <c r="C7" s="176"/>
-      <c r="D7" s="176"/>
-      <c r="E7" s="177"/>
-      <c r="F7" s="177"/>
+      <c r="B7" s="179"/>
+      <c r="C7" s="179"/>
+      <c r="D7" s="179"/>
+      <c r="E7" s="180"/>
+      <c r="F7" s="180"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -44629,39 +44774,39 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:CE7">
-    <cfRule type="expression" dxfId="14" priority="12">
+    <cfRule type="expression" dxfId="35" priority="12">
       <formula>B5&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:CE201">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="34" priority="1">
       <formula>AND(G8&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="33" priority="2">
       <formula>AND(G$7&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="3">
+    <cfRule type="expression" dxfId="32" priority="3">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="4">
+    <cfRule type="expression" dxfId="31" priority="4">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="30" priority="5">
       <formula>AND(G8&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="29" priority="6">
       <formula>AND(G$7&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="7">
+    <cfRule type="expression" dxfId="28" priority="7">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="8">
+    <cfRule type="expression" dxfId="27" priority="8">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="10">
+    <cfRule type="expression" dxfId="25" priority="10">
       <formula>AND(G$7&lt;&gt;"",$B8="DEVIASI")</formula>
     </cfRule>
     <cfRule type="colorScale" priority="11">

</xml_diff>

<commit_message>
final polish: HSP border B-H, AHSP labels shifted to C, TKDN sync fixed
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BD47DD-0F8D-4CFE-B84F-7799C638DD60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C55029F3-E610-4E08-8A7F-545695E1F8BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2610,7 +2610,41 @@
     <cellStyle name="Normal 2 2 3" xfId="2" xr:uid="{25DAB206-4C06-437D-BFFA-FD21FFA5A242}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="42">
+  <dxfs count="51">
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2649,6 +2683,45 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i/>
@@ -2682,6 +2755,18 @@
       <fill>
         <patternFill patternType="none">
           <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5472,12 +5557,12 @@
     <mergeCell ref="B24:B25"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:I48">
-    <cfRule type="expression" dxfId="24" priority="1">
+    <cfRule type="expression" dxfId="33" priority="1">
       <formula>ISTEXT($C26)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J27:M48">
-    <cfRule type="cellIs" dxfId="23" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6172,7 +6257,7 @@
     <mergeCell ref="I4:P5"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P49">
-    <cfRule type="expression" dxfId="22" priority="13">
+    <cfRule type="expression" dxfId="31" priority="13">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6913,7 +6998,7 @@
     <mergeCell ref="G12:G14"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P51">
-    <cfRule type="expression" dxfId="21" priority="14">
+    <cfRule type="expression" dxfId="30" priority="14">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15337,7 +15422,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="41" priority="2">
+    <cfRule type="expression" dxfId="50" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17587,20 +17672,23 @@
     <mergeCell ref="B1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:N16997">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="4">
-      <formula>AND($B6&lt;&gt;"",$C6&lt;&gt;"",$D6&lt;&gt;"")</formula>
+    <cfRule type="expression" dxfId="1" priority="5">
+      <formula>AND($B6="",$C6&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H16997">
-    <cfRule type="expression" dxfId="6" priority="8">
+    <cfRule type="expression" dxfId="8" priority="9">
       <formula>IF(G6&lt;&gt;"", NOT(AND(OR(LEFT($E6,2)="L.", LEFT($E6,2)="A.", LEFT($E6,2)="B.", LEFT($E6,2)="M."), $H6&lt;&gt;"", $E6&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:K16997">
-    <cfRule type="notContainsBlanks" dxfId="5" priority="7">
+    <cfRule type="notContainsBlanks" dxfId="7" priority="8">
       <formula>LEN(TRIM(H6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -41703,15 +41791,15 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B995 E6:H995">
-    <cfRule type="expression" dxfId="40" priority="6">
+    <cfRule type="expression" dxfId="49" priority="6">
       <formula>$J6=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:H995">
-    <cfRule type="expression" dxfId="39" priority="1">
+    <cfRule type="expression" dxfId="48" priority="1">
       <formula>AND(LEN($B6)=1,$C6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="2">
+    <cfRule type="expression" dxfId="47" priority="2">
       <formula>$C6&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -43289,7 +43377,7 @@
     <mergeCell ref="B1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="B12:K9929">
-    <cfRule type="expression" dxfId="37" priority="1">
+    <cfRule type="expression" dxfId="46" priority="1">
       <formula>AND($B12&lt;&gt;"",$C12&lt;&gt;"",$G12="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -44650,7 +44738,7 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B12:H9929">
-    <cfRule type="expression" dxfId="36" priority="9">
+    <cfRule type="expression" dxfId="45" priority="9">
       <formula>AND($B12&lt;&gt;"",$C12&lt;&gt;"",#REF!="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -44774,39 +44862,39 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:CE7">
-    <cfRule type="expression" dxfId="35" priority="12">
+    <cfRule type="expression" dxfId="44" priority="12">
       <formula>B5&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:CE201">
-    <cfRule type="expression" dxfId="34" priority="1">
+    <cfRule type="expression" dxfId="43" priority="1">
       <formula>AND(G8&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="2">
+    <cfRule type="expression" dxfId="42" priority="2">
       <formula>AND(G$7&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="3">
+    <cfRule type="expression" dxfId="41" priority="3">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="4">
+    <cfRule type="expression" dxfId="40" priority="4">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="5">
+    <cfRule type="expression" dxfId="39" priority="5">
       <formula>AND(G8&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="6">
+    <cfRule type="expression" dxfId="38" priority="6">
       <formula>AND(G$7&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="7">
+    <cfRule type="expression" dxfId="37" priority="7">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="8">
+    <cfRule type="expression" dxfId="36" priority="8">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="10">
+    <cfRule type="expression" dxfId="34" priority="10">
       <formula>AND(G$7&lt;&gt;"",$B8="DEVIASI")</formula>
     </cfRule>
     <cfRule type="colorScale" priority="11">

</xml_diff>

<commit_message>
feat: sync local template and code fixes to github
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C55029F3-E610-4E08-8A7F-545695E1F8BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFBBA769-50B1-427D-B66D-2A677D078FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cover" sheetId="21" r:id="rId1"/>
@@ -2280,14 +2280,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2306,6 +2306,126 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="48" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="25" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="25" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2415,18 +2535,6 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2463,13 +2571,7 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2492,108 +2594,6 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="47" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="48" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="25" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="25" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2610,15 +2610,41 @@
     <cellStyle name="Normal 2 2 3" xfId="2" xr:uid="{25DAB206-4C06-437D-BFFA-FD21FFA5A242}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="51">
+  <dxfs count="30">
     <dxf>
       <font>
         <b/>
         <i/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0" tint="-0.14996795556505021"/>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color rgb="FFFFC000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor theme="7" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2629,7 +2655,33 @@
       </font>
       <fill>
         <patternFill patternType="none">
-          <bgColor auto="1"/>
+          <fgColor indexed="64"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2637,25 +2689,12 @@
       <font>
         <b/>
         <i/>
-        <color auto="1"/>
+        <color rgb="FFFFC000"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <fgColor theme="0"/>
+          <bgColor theme="7" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2666,231 +2705,23 @@
       </font>
       <fill>
         <patternFill patternType="none">
-          <bgColor auto="1"/>
+          <fgColor indexed="64"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -3068,27 +2899,16 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
       <fill>
         <patternFill>
-          <fgColor theme="0"/>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color rgb="FFFFC000"/>
-      </font>
       <fill>
         <patternFill>
-          <fgColor theme="0"/>
-          <bgColor theme="7" tint="-0.499984740745262"/>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3099,23 +2919,32 @@
       </font>
       <fill>
         <patternFill patternType="none">
-          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -4173,48 +4002,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="194"/>
-      <c r="C1" s="195"/>
-      <c r="D1" s="195"/>
-      <c r="E1" s="195"/>
-      <c r="F1" s="195"/>
-      <c r="G1" s="195"/>
-      <c r="H1" s="195"/>
-      <c r="I1" s="195"/>
-      <c r="J1" s="195"/>
-      <c r="K1" s="195"/>
-      <c r="L1" s="195"/>
-      <c r="M1" s="196"/>
+      <c r="B1" s="231"/>
+      <c r="C1" s="232"/>
+      <c r="D1" s="232"/>
+      <c r="E1" s="232"/>
+      <c r="F1" s="232"/>
+      <c r="G1" s="232"/>
+      <c r="H1" s="232"/>
+      <c r="I1" s="232"/>
+      <c r="J1" s="232"/>
+      <c r="K1" s="232"/>
+      <c r="L1" s="232"/>
+      <c r="M1" s="233"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="197" t="s">
+      <c r="B2" s="234" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="198"/>
-      <c r="D2" s="198"/>
-      <c r="E2" s="198"/>
-      <c r="F2" s="198"/>
-      <c r="G2" s="198"/>
-      <c r="H2" s="198"/>
-      <c r="I2" s="199"/>
-      <c r="J2" s="203"/>
-      <c r="K2" s="204"/>
-      <c r="L2" s="204"/>
-      <c r="M2" s="205"/>
+      <c r="C2" s="235"/>
+      <c r="D2" s="235"/>
+      <c r="E2" s="235"/>
+      <c r="F2" s="235"/>
+      <c r="G2" s="235"/>
+      <c r="H2" s="235"/>
+      <c r="I2" s="236"/>
+      <c r="J2" s="240"/>
+      <c r="K2" s="241"/>
+      <c r="L2" s="241"/>
+      <c r="M2" s="242"/>
     </row>
     <row r="3" spans="1:14" ht="14.4" customHeight="1">
-      <c r="B3" s="200"/>
-      <c r="C3" s="201"/>
-      <c r="D3" s="201"/>
-      <c r="E3" s="201"/>
-      <c r="F3" s="201"/>
-      <c r="G3" s="201"/>
-      <c r="H3" s="201"/>
-      <c r="I3" s="202"/>
-      <c r="J3" s="206"/>
-      <c r="K3" s="207"/>
-      <c r="L3" s="207"/>
-      <c r="M3" s="208"/>
+      <c r="B3" s="237"/>
+      <c r="C3" s="238"/>
+      <c r="D3" s="238"/>
+      <c r="E3" s="238"/>
+      <c r="F3" s="238"/>
+      <c r="G3" s="238"/>
+      <c r="H3" s="238"/>
+      <c r="I3" s="239"/>
+      <c r="J3" s="243"/>
+      <c r="K3" s="244"/>
+      <c r="L3" s="244"/>
+      <c r="M3" s="245"/>
     </row>
     <row r="4" spans="1:14" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -4225,10 +4054,10 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="206"/>
-      <c r="K4" s="207"/>
-      <c r="L4" s="207"/>
-      <c r="M4" s="208"/>
+      <c r="J4" s="243"/>
+      <c r="K4" s="244"/>
+      <c r="L4" s="244"/>
+      <c r="M4" s="245"/>
     </row>
     <row r="5" spans="1:14" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -4243,10 +4072,10 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="206"/>
-      <c r="K5" s="207"/>
-      <c r="L5" s="207"/>
-      <c r="M5" s="208"/>
+      <c r="J5" s="243"/>
+      <c r="K5" s="244"/>
+      <c r="L5" s="244"/>
+      <c r="M5" s="245"/>
     </row>
     <row r="6" spans="1:14" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -4261,10 +4090,10 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="209"/>
-      <c r="K6" s="210"/>
-      <c r="L6" s="210"/>
-      <c r="M6" s="211"/>
+      <c r="J6" s="246"/>
+      <c r="K6" s="247"/>
+      <c r="L6" s="247"/>
+      <c r="M6" s="248"/>
     </row>
     <row r="7" spans="1:14" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -4329,52 +4158,52 @@
       <c r="M9" s="89"/>
     </row>
     <row r="10" spans="1:14" ht="15.6">
-      <c r="B10" s="212" t="s">
+      <c r="B10" s="182" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="213"/>
-      <c r="D10" s="213"/>
-      <c r="E10" s="213"/>
-      <c r="F10" s="213"/>
-      <c r="G10" s="213" t="s">
+      <c r="C10" s="183"/>
+      <c r="D10" s="183"/>
+      <c r="E10" s="183"/>
+      <c r="F10" s="183"/>
+      <c r="G10" s="183" t="s">
         <v>95</v>
       </c>
-      <c r="H10" s="213"/>
-      <c r="I10" s="213"/>
-      <c r="J10" s="214"/>
-      <c r="K10" s="215" t="s">
+      <c r="H10" s="183"/>
+      <c r="I10" s="183"/>
+      <c r="J10" s="184"/>
+      <c r="K10" s="185" t="s">
         <v>96</v>
       </c>
-      <c r="L10" s="213"/>
-      <c r="M10" s="216"/>
+      <c r="L10" s="183"/>
+      <c r="M10" s="249"/>
     </row>
     <row r="11" spans="1:14" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="226" t="s">
+      <c r="C11" s="206" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="227"/>
-      <c r="E11" s="227"/>
+      <c r="D11" s="259"/>
+      <c r="E11" s="259"/>
       <c r="F11" s="92" t="s">
         <v>98</v>
       </c>
-      <c r="G11" s="226" t="s">
+      <c r="G11" s="206" t="s">
         <v>99</v>
       </c>
-      <c r="H11" s="228"/>
+      <c r="H11" s="207"/>
       <c r="I11" s="93" t="s">
         <v>27</v>
       </c>
       <c r="J11" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="226" t="s">
+      <c r="K11" s="206" t="s">
         <v>100</v>
       </c>
-      <c r="L11" s="228"/>
+      <c r="L11" s="207"/>
       <c r="M11" s="94" t="s">
         <v>101</v>
       </c>
@@ -4579,58 +4408,58 @@
       <c r="M22" s="123"/>
     </row>
     <row r="23" spans="1:13" ht="16.2" thickBot="1">
-      <c r="B23" s="229"/>
-      <c r="C23" s="230"/>
-      <c r="D23" s="230"/>
-      <c r="E23" s="230"/>
+      <c r="B23" s="260"/>
+      <c r="C23" s="261"/>
+      <c r="D23" s="261"/>
+      <c r="E23" s="261"/>
       <c r="F23" s="124"/>
       <c r="G23" s="124"/>
       <c r="H23" s="125"/>
       <c r="I23" s="125"/>
-      <c r="J23" s="231"/>
-      <c r="K23" s="231"/>
-      <c r="L23" s="231"/>
-      <c r="M23" s="232"/>
+      <c r="J23" s="262"/>
+      <c r="K23" s="262"/>
+      <c r="L23" s="262"/>
+      <c r="M23" s="263"/>
     </row>
     <row r="24" spans="1:13" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="152" t="s">
         <v>116</v>
       </c>
-      <c r="B24" s="233" t="s">
+      <c r="B24" s="264" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="235" t="s">
+      <c r="C24" s="201" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="235"/>
-      <c r="E24" s="235"/>
-      <c r="F24" s="235"/>
-      <c r="G24" s="235"/>
-      <c r="H24" s="235"/>
-      <c r="I24" s="235"/>
-      <c r="J24" s="237" t="s">
+      <c r="D24" s="201"/>
+      <c r="E24" s="201"/>
+      <c r="F24" s="201"/>
+      <c r="G24" s="201"/>
+      <c r="H24" s="201"/>
+      <c r="I24" s="201"/>
+      <c r="J24" s="203" t="s">
         <v>117</v>
       </c>
-      <c r="K24" s="238"/>
-      <c r="L24" s="238"/>
-      <c r="M24" s="239"/>
+      <c r="K24" s="204"/>
+      <c r="L24" s="204"/>
+      <c r="M24" s="205"/>
     </row>
     <row r="25" spans="1:13" ht="31.2">
-      <c r="B25" s="234"/>
-      <c r="C25" s="236"/>
-      <c r="D25" s="236"/>
-      <c r="E25" s="236"/>
-      <c r="F25" s="236"/>
-      <c r="G25" s="236"/>
-      <c r="H25" s="236"/>
-      <c r="I25" s="236"/>
+      <c r="B25" s="265"/>
+      <c r="C25" s="202"/>
+      <c r="D25" s="202"/>
+      <c r="E25" s="202"/>
+      <c r="F25" s="202"/>
+      <c r="G25" s="202"/>
+      <c r="H25" s="202"/>
+      <c r="I25" s="202"/>
       <c r="J25" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="249" t="s">
+      <c r="K25" s="217" t="s">
         <v>118</v>
       </c>
-      <c r="L25" s="250"/>
+      <c r="L25" s="218"/>
       <c r="M25" s="126" t="s">
         <v>119</v>
       </c>
@@ -5188,60 +5017,60 @@
       </c>
     </row>
     <row r="49" spans="2:13" ht="16.2" thickTop="1">
-      <c r="B49" s="260" t="s">
+      <c r="B49" s="195" t="s">
         <v>120</v>
       </c>
-      <c r="C49" s="261"/>
-      <c r="D49" s="261"/>
-      <c r="E49" s="261"/>
-      <c r="F49" s="261"/>
-      <c r="G49" s="261"/>
-      <c r="H49" s="261"/>
-      <c r="I49" s="261"/>
-      <c r="J49" s="262"/>
-      <c r="K49" s="223" t="s">
+      <c r="C49" s="196"/>
+      <c r="D49" s="196"/>
+      <c r="E49" s="196"/>
+      <c r="F49" s="196"/>
+      <c r="G49" s="196"/>
+      <c r="H49" s="196"/>
+      <c r="I49" s="196"/>
+      <c r="J49" s="197"/>
+      <c r="K49" s="256" t="s">
         <v>121</v>
       </c>
-      <c r="L49" s="224"/>
-      <c r="M49" s="225"/>
+      <c r="L49" s="257"/>
+      <c r="M49" s="258"/>
     </row>
     <row r="50" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B50" s="263"/>
-      <c r="C50" s="264"/>
-      <c r="D50" s="264"/>
-      <c r="E50" s="264"/>
-      <c r="F50" s="264"/>
-      <c r="G50" s="264"/>
-      <c r="H50" s="264"/>
-      <c r="I50" s="264"/>
-      <c r="J50" s="265"/>
-      <c r="K50" s="220"/>
-      <c r="L50" s="221"/>
-      <c r="M50" s="222"/>
+      <c r="B50" s="198"/>
+      <c r="C50" s="199"/>
+      <c r="D50" s="199"/>
+      <c r="E50" s="199"/>
+      <c r="F50" s="199"/>
+      <c r="G50" s="199"/>
+      <c r="H50" s="199"/>
+      <c r="I50" s="199"/>
+      <c r="J50" s="200"/>
+      <c r="K50" s="253"/>
+      <c r="L50" s="254"/>
+      <c r="M50" s="255"/>
     </row>
     <row r="51" spans="2:13" ht="15.6">
       <c r="B51" s="138"/>
-      <c r="C51" s="217"/>
-      <c r="D51" s="217"/>
-      <c r="E51" s="217"/>
-      <c r="F51" s="217"/>
-      <c r="G51" s="217"/>
-      <c r="H51" s="217"/>
-      <c r="I51" s="217"/>
+      <c r="C51" s="250"/>
+      <c r="D51" s="250"/>
+      <c r="E51" s="250"/>
+      <c r="F51" s="250"/>
+      <c r="G51" s="250"/>
+      <c r="H51" s="250"/>
+      <c r="I51" s="250"/>
       <c r="J51" s="139"/>
-      <c r="K51" s="246"/>
-      <c r="L51" s="247"/>
-      <c r="M51" s="248"/>
+      <c r="K51" s="214"/>
+      <c r="L51" s="215"/>
+      <c r="M51" s="216"/>
     </row>
     <row r="52" spans="2:13" ht="15.6">
       <c r="B52" s="140"/>
-      <c r="C52" s="218"/>
-      <c r="D52" s="218"/>
-      <c r="E52" s="218"/>
-      <c r="F52" s="218"/>
-      <c r="G52" s="218"/>
-      <c r="H52" s="218"/>
-      <c r="I52" s="218"/>
+      <c r="C52" s="251"/>
+      <c r="D52" s="251"/>
+      <c r="E52" s="251"/>
+      <c r="F52" s="251"/>
+      <c r="G52" s="251"/>
+      <c r="H52" s="251"/>
+      <c r="I52" s="251"/>
       <c r="J52" s="141"/>
       <c r="K52" s="164"/>
       <c r="L52" s="161"/>
@@ -5249,13 +5078,13 @@
     </row>
     <row r="53" spans="2:13" ht="15.6">
       <c r="B53" s="140"/>
-      <c r="C53" s="218"/>
-      <c r="D53" s="218"/>
-      <c r="E53" s="218"/>
-      <c r="F53" s="218"/>
-      <c r="G53" s="218"/>
-      <c r="H53" s="218"/>
-      <c r="I53" s="218"/>
+      <c r="C53" s="251"/>
+      <c r="D53" s="251"/>
+      <c r="E53" s="251"/>
+      <c r="F53" s="251"/>
+      <c r="G53" s="251"/>
+      <c r="H53" s="251"/>
+      <c r="I53" s="251"/>
       <c r="J53" s="141"/>
       <c r="K53" s="164"/>
       <c r="L53" s="161"/>
@@ -5263,13 +5092,13 @@
     </row>
     <row r="54" spans="2:13" ht="15.6">
       <c r="B54" s="140"/>
-      <c r="C54" s="218"/>
-      <c r="D54" s="218"/>
-      <c r="E54" s="218"/>
-      <c r="F54" s="218"/>
-      <c r="G54" s="218"/>
-      <c r="H54" s="218"/>
-      <c r="I54" s="218"/>
+      <c r="C54" s="251"/>
+      <c r="D54" s="251"/>
+      <c r="E54" s="251"/>
+      <c r="F54" s="251"/>
+      <c r="G54" s="251"/>
+      <c r="H54" s="251"/>
+      <c r="I54" s="251"/>
       <c r="J54" s="141"/>
       <c r="K54" s="164"/>
       <c r="L54" s="161"/>
@@ -5277,13 +5106,13 @@
     </row>
     <row r="55" spans="2:13" ht="15.6">
       <c r="B55" s="143"/>
-      <c r="C55" s="218"/>
-      <c r="D55" s="218"/>
-      <c r="E55" s="218"/>
-      <c r="F55" s="218"/>
-      <c r="G55" s="218"/>
-      <c r="H55" s="218"/>
-      <c r="I55" s="218"/>
+      <c r="C55" s="251"/>
+      <c r="D55" s="251"/>
+      <c r="E55" s="251"/>
+      <c r="F55" s="251"/>
+      <c r="G55" s="251"/>
+      <c r="H55" s="251"/>
+      <c r="I55" s="251"/>
       <c r="J55" s="144"/>
       <c r="K55" s="164"/>
       <c r="L55" s="145"/>
@@ -5291,13 +5120,13 @@
     </row>
     <row r="56" spans="2:13" ht="15.6">
       <c r="B56" s="143"/>
-      <c r="C56" s="218"/>
-      <c r="D56" s="218"/>
-      <c r="E56" s="218"/>
-      <c r="F56" s="218"/>
-      <c r="G56" s="218"/>
-      <c r="H56" s="218"/>
-      <c r="I56" s="218"/>
+      <c r="C56" s="251"/>
+      <c r="D56" s="251"/>
+      <c r="E56" s="251"/>
+      <c r="F56" s="251"/>
+      <c r="G56" s="251"/>
+      <c r="H56" s="251"/>
+      <c r="I56" s="251"/>
       <c r="J56" s="144"/>
       <c r="K56" s="164"/>
       <c r="L56" s="145"/>
@@ -5305,41 +5134,41 @@
     </row>
     <row r="57" spans="2:13" ht="15.6">
       <c r="B57" s="143"/>
-      <c r="C57" s="218"/>
-      <c r="D57" s="218"/>
-      <c r="E57" s="218"/>
-      <c r="F57" s="218"/>
-      <c r="G57" s="218"/>
-      <c r="H57" s="218"/>
-      <c r="I57" s="218"/>
+      <c r="C57" s="251"/>
+      <c r="D57" s="251"/>
+      <c r="E57" s="251"/>
+      <c r="F57" s="251"/>
+      <c r="G57" s="251"/>
+      <c r="H57" s="251"/>
+      <c r="I57" s="251"/>
       <c r="J57" s="144"/>
-      <c r="K57" s="240"/>
-      <c r="L57" s="241"/>
-      <c r="M57" s="242"/>
+      <c r="K57" s="208"/>
+      <c r="L57" s="209"/>
+      <c r="M57" s="210"/>
     </row>
     <row r="58" spans="2:13" ht="15.6">
       <c r="B58" s="143"/>
-      <c r="C58" s="218"/>
-      <c r="D58" s="218"/>
-      <c r="E58" s="218"/>
-      <c r="F58" s="218"/>
-      <c r="G58" s="218"/>
-      <c r="H58" s="218"/>
-      <c r="I58" s="218"/>
+      <c r="C58" s="251"/>
+      <c r="D58" s="251"/>
+      <c r="E58" s="251"/>
+      <c r="F58" s="251"/>
+      <c r="G58" s="251"/>
+      <c r="H58" s="251"/>
+      <c r="I58" s="251"/>
       <c r="J58" s="144"/>
-      <c r="K58" s="243"/>
-      <c r="L58" s="244"/>
-      <c r="M58" s="245"/>
+      <c r="K58" s="211"/>
+      <c r="L58" s="212"/>
+      <c r="M58" s="213"/>
     </row>
     <row r="59" spans="2:13" ht="15.6">
       <c r="B59" s="143"/>
-      <c r="C59" s="218"/>
-      <c r="D59" s="218"/>
-      <c r="E59" s="218"/>
-      <c r="F59" s="218"/>
-      <c r="G59" s="218"/>
-      <c r="H59" s="218"/>
-      <c r="I59" s="218"/>
+      <c r="C59" s="251"/>
+      <c r="D59" s="251"/>
+      <c r="E59" s="251"/>
+      <c r="F59" s="251"/>
+      <c r="G59" s="251"/>
+      <c r="H59" s="251"/>
+      <c r="I59" s="251"/>
       <c r="J59" s="144"/>
       <c r="K59" s="164"/>
       <c r="L59" s="162"/>
@@ -5347,13 +5176,13 @@
     </row>
     <row r="60" spans="2:13" ht="15.6">
       <c r="B60" s="143"/>
-      <c r="C60" s="218"/>
-      <c r="D60" s="218"/>
-      <c r="E60" s="218"/>
-      <c r="F60" s="218"/>
-      <c r="G60" s="218"/>
-      <c r="H60" s="218"/>
-      <c r="I60" s="218"/>
+      <c r="C60" s="251"/>
+      <c r="D60" s="251"/>
+      <c r="E60" s="251"/>
+      <c r="F60" s="251"/>
+      <c r="G60" s="251"/>
+      <c r="H60" s="251"/>
+      <c r="I60" s="251"/>
       <c r="J60" s="144"/>
       <c r="K60" s="164"/>
       <c r="L60" s="162"/>
@@ -5361,13 +5190,13 @@
     </row>
     <row r="61" spans="2:13" ht="15.6">
       <c r="B61" s="143"/>
-      <c r="C61" s="219"/>
-      <c r="D61" s="219"/>
-      <c r="E61" s="219"/>
-      <c r="F61" s="219"/>
-      <c r="G61" s="219"/>
-      <c r="H61" s="219"/>
-      <c r="I61" s="219"/>
+      <c r="C61" s="252"/>
+      <c r="D61" s="252"/>
+      <c r="E61" s="252"/>
+      <c r="F61" s="252"/>
+      <c r="G61" s="252"/>
+      <c r="H61" s="252"/>
+      <c r="I61" s="252"/>
       <c r="J61" s="144"/>
       <c r="K61" s="164"/>
       <c r="L61" s="162"/>
@@ -5388,133 +5217,133 @@
       <c r="M62" s="167"/>
     </row>
     <row r="63" spans="2:13" ht="15.6">
-      <c r="B63" s="212" t="s">
+      <c r="B63" s="182" t="s">
         <v>122</v>
       </c>
-      <c r="C63" s="213"/>
-      <c r="D63" s="213"/>
-      <c r="E63" s="214"/>
-      <c r="F63" s="215" t="s">
+      <c r="C63" s="183"/>
+      <c r="D63" s="183"/>
+      <c r="E63" s="184"/>
+      <c r="F63" s="185" t="s">
         <v>123</v>
       </c>
-      <c r="G63" s="214"/>
-      <c r="H63" s="215" t="s">
+      <c r="G63" s="184"/>
+      <c r="H63" s="185" t="s">
         <v>124</v>
       </c>
-      <c r="I63" s="213"/>
-      <c r="J63" s="214"/>
+      <c r="I63" s="183"/>
+      <c r="J63" s="184"/>
       <c r="K63" s="165"/>
       <c r="L63" s="145"/>
       <c r="M63" s="146"/>
     </row>
     <row r="64" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B64" s="188"/>
-      <c r="C64" s="189"/>
-      <c r="D64" s="189"/>
-      <c r="E64" s="183"/>
-      <c r="F64" s="182"/>
-      <c r="G64" s="183"/>
-      <c r="H64" s="251"/>
-      <c r="I64" s="252"/>
-      <c r="J64" s="253"/>
+      <c r="B64" s="225"/>
+      <c r="C64" s="226"/>
+      <c r="D64" s="226"/>
+      <c r="E64" s="220"/>
+      <c r="F64" s="219"/>
+      <c r="G64" s="220"/>
+      <c r="H64" s="186"/>
+      <c r="I64" s="187"/>
+      <c r="J64" s="188"/>
       <c r="K64" s="148"/>
       <c r="L64" s="145"/>
       <c r="M64" s="146"/>
     </row>
     <row r="65" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B65" s="190"/>
-      <c r="C65" s="191"/>
-      <c r="D65" s="191"/>
-      <c r="E65" s="185"/>
-      <c r="F65" s="184"/>
-      <c r="G65" s="185"/>
-      <c r="H65" s="254"/>
-      <c r="I65" s="255"/>
-      <c r="J65" s="256"/>
+      <c r="B65" s="227"/>
+      <c r="C65" s="228"/>
+      <c r="D65" s="228"/>
+      <c r="E65" s="222"/>
+      <c r="F65" s="221"/>
+      <c r="G65" s="222"/>
+      <c r="H65" s="189"/>
+      <c r="I65" s="190"/>
+      <c r="J65" s="191"/>
       <c r="K65" s="148"/>
       <c r="L65" s="163"/>
       <c r="M65" s="146"/>
     </row>
     <row r="66" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B66" s="190"/>
-      <c r="C66" s="191"/>
-      <c r="D66" s="191"/>
-      <c r="E66" s="185"/>
-      <c r="F66" s="184"/>
-      <c r="G66" s="185"/>
-      <c r="H66" s="254"/>
-      <c r="I66" s="255"/>
-      <c r="J66" s="256"/>
+      <c r="B66" s="227"/>
+      <c r="C66" s="228"/>
+      <c r="D66" s="228"/>
+      <c r="E66" s="222"/>
+      <c r="F66" s="221"/>
+      <c r="G66" s="222"/>
+      <c r="H66" s="189"/>
+      <c r="I66" s="190"/>
+      <c r="J66" s="191"/>
       <c r="K66" s="148"/>
       <c r="L66" s="145"/>
       <c r="M66" s="146"/>
     </row>
     <row r="67" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B67" s="190"/>
-      <c r="C67" s="191"/>
-      <c r="D67" s="191"/>
-      <c r="E67" s="185"/>
-      <c r="F67" s="184"/>
-      <c r="G67" s="185"/>
-      <c r="H67" s="254"/>
-      <c r="I67" s="255"/>
-      <c r="J67" s="256"/>
+      <c r="B67" s="227"/>
+      <c r="C67" s="228"/>
+      <c r="D67" s="228"/>
+      <c r="E67" s="222"/>
+      <c r="F67" s="221"/>
+      <c r="G67" s="222"/>
+      <c r="H67" s="189"/>
+      <c r="I67" s="190"/>
+      <c r="J67" s="191"/>
       <c r="K67" s="148"/>
       <c r="L67" s="162"/>
       <c r="M67" s="76"/>
     </row>
     <row r="68" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B68" s="190"/>
-      <c r="C68" s="191"/>
-      <c r="D68" s="191"/>
-      <c r="E68" s="185"/>
-      <c r="F68" s="184"/>
-      <c r="G68" s="185"/>
-      <c r="H68" s="254"/>
-      <c r="I68" s="255"/>
-      <c r="J68" s="256"/>
+      <c r="B68" s="227"/>
+      <c r="C68" s="228"/>
+      <c r="D68" s="228"/>
+      <c r="E68" s="222"/>
+      <c r="F68" s="221"/>
+      <c r="G68" s="222"/>
+      <c r="H68" s="189"/>
+      <c r="I68" s="190"/>
+      <c r="J68" s="191"/>
       <c r="K68" s="148"/>
       <c r="L68" s="162"/>
       <c r="M68" s="76"/>
     </row>
     <row r="69" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B69" s="190"/>
-      <c r="C69" s="191"/>
-      <c r="D69" s="191"/>
-      <c r="E69" s="185"/>
-      <c r="F69" s="184"/>
-      <c r="G69" s="185"/>
-      <c r="H69" s="254"/>
-      <c r="I69" s="255"/>
-      <c r="J69" s="256"/>
+      <c r="B69" s="227"/>
+      <c r="C69" s="228"/>
+      <c r="D69" s="228"/>
+      <c r="E69" s="222"/>
+      <c r="F69" s="221"/>
+      <c r="G69" s="222"/>
+      <c r="H69" s="189"/>
+      <c r="I69" s="190"/>
+      <c r="J69" s="191"/>
       <c r="K69" s="168"/>
       <c r="L69" s="169"/>
       <c r="M69" s="170"/>
     </row>
     <row r="70" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B70" s="190"/>
-      <c r="C70" s="191"/>
-      <c r="D70" s="191"/>
-      <c r="E70" s="185"/>
-      <c r="F70" s="184"/>
-      <c r="G70" s="185"/>
-      <c r="H70" s="254"/>
-      <c r="I70" s="255"/>
-      <c r="J70" s="256"/>
+      <c r="B70" s="227"/>
+      <c r="C70" s="228"/>
+      <c r="D70" s="228"/>
+      <c r="E70" s="222"/>
+      <c r="F70" s="221"/>
+      <c r="G70" s="222"/>
+      <c r="H70" s="189"/>
+      <c r="I70" s="190"/>
+      <c r="J70" s="191"/>
       <c r="K70" s="168"/>
       <c r="L70" s="169"/>
       <c r="M70" s="170"/>
     </row>
     <row r="71" spans="2:13" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B71" s="192"/>
-      <c r="C71" s="193"/>
-      <c r="D71" s="193"/>
-      <c r="E71" s="187"/>
-      <c r="F71" s="186"/>
-      <c r="G71" s="187"/>
-      <c r="H71" s="257"/>
-      <c r="I71" s="258"/>
-      <c r="J71" s="259"/>
+      <c r="B71" s="229"/>
+      <c r="C71" s="230"/>
+      <c r="D71" s="230"/>
+      <c r="E71" s="224"/>
+      <c r="F71" s="223"/>
+      <c r="G71" s="224"/>
+      <c r="H71" s="192"/>
+      <c r="I71" s="193"/>
+      <c r="J71" s="194"/>
       <c r="K71" s="150"/>
       <c r="L71" s="149"/>
       <c r="M71" s="151"/>
@@ -5527,11 +5356,12 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="H63:J63"/>
-    <mergeCell ref="H64:J71"/>
-    <mergeCell ref="B49:J50"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="J2:M6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="K10:M10"/>
     <mergeCell ref="C24:I25"/>
     <mergeCell ref="J24:M24"/>
     <mergeCell ref="K11:L11"/>
@@ -5539,14 +5369,6 @@
     <mergeCell ref="K58:M58"/>
     <mergeCell ref="K51:M51"/>
     <mergeCell ref="K25:L25"/>
-    <mergeCell ref="F64:G71"/>
-    <mergeCell ref="B64:E71"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="J2:M6"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="K10:M10"/>
     <mergeCell ref="C51:I61"/>
     <mergeCell ref="K50:M50"/>
     <mergeCell ref="K49:M49"/>
@@ -5555,14 +5377,21 @@
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="J23:M23"/>
     <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="H63:J63"/>
+    <mergeCell ref="H64:J71"/>
+    <mergeCell ref="B49:J50"/>
+    <mergeCell ref="F64:G71"/>
+    <mergeCell ref="B64:E71"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:I48">
-    <cfRule type="expression" dxfId="33" priority="1">
+    <cfRule type="expression" dxfId="10" priority="1">
       <formula>ISTEXT($C26)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J27:M48">
-    <cfRule type="cellIs" dxfId="32" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5825,47 +5654,47 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="175" t="s">
+      <c r="B12" s="173" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="175" t="s">
+      <c r="C12" s="173" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="175"/>
-      <c r="E12" s="175"/>
-      <c r="F12" s="175" t="s">
+      <c r="D12" s="173"/>
+      <c r="E12" s="173"/>
+      <c r="F12" s="173" t="s">
         <v>131</v>
       </c>
-      <c r="G12" s="175" t="s">
+      <c r="G12" s="173" t="s">
         <v>133</v>
       </c>
-      <c r="H12" s="175" t="s">
+      <c r="H12" s="173" t="s">
         <v>132</v>
       </c>
-      <c r="I12" s="175" t="s">
+      <c r="I12" s="173" t="s">
         <v>134</v>
       </c>
-      <c r="J12" s="175" t="s">
+      <c r="J12" s="173" t="s">
         <v>138</v>
       </c>
-      <c r="K12" s="175"/>
-      <c r="L12" s="175"/>
-      <c r="M12" s="175"/>
-      <c r="N12" s="175"/>
-      <c r="O12" s="175"/>
+      <c r="K12" s="173"/>
+      <c r="L12" s="173"/>
+      <c r="M12" s="173"/>
+      <c r="N12" s="173"/>
+      <c r="O12" s="173"/>
       <c r="P12" s="267" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="175"/>
-      <c r="C13" s="175"/>
-      <c r="D13" s="175"/>
-      <c r="E13" s="175"/>
-      <c r="F13" s="175"/>
-      <c r="G13" s="175"/>
-      <c r="H13" s="175"/>
-      <c r="I13" s="175"/>
+      <c r="B13" s="173"/>
+      <c r="C13" s="173"/>
+      <c r="D13" s="173"/>
+      <c r="E13" s="173"/>
+      <c r="F13" s="173"/>
+      <c r="G13" s="173"/>
+      <c r="H13" s="173"/>
+      <c r="I13" s="173"/>
       <c r="J13" s="266" t="s">
         <v>135</v>
       </c>
@@ -5881,14 +5710,14 @@
       <c r="P13" s="267"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="175"/>
-      <c r="C14" s="175"/>
-      <c r="D14" s="175"/>
-      <c r="E14" s="175"/>
-      <c r="F14" s="175"/>
-      <c r="G14" s="175"/>
-      <c r="H14" s="175"/>
-      <c r="I14" s="175"/>
+      <c r="B14" s="173"/>
+      <c r="C14" s="173"/>
+      <c r="D14" s="173"/>
+      <c r="E14" s="173"/>
+      <c r="F14" s="173"/>
+      <c r="G14" s="173"/>
+      <c r="H14" s="173"/>
+      <c r="I14" s="173"/>
       <c r="J14" s="38" t="s">
         <v>118</v>
       </c>
@@ -6257,7 +6086,7 @@
     <mergeCell ref="I4:P5"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P49">
-    <cfRule type="expression" dxfId="31" priority="13">
+    <cfRule type="expression" dxfId="8" priority="13">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6520,47 +6349,47 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="175" t="s">
+      <c r="B12" s="173" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="175" t="s">
+      <c r="C12" s="173" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="175"/>
-      <c r="E12" s="175"/>
-      <c r="F12" s="175" t="s">
+      <c r="D12" s="173"/>
+      <c r="E12" s="173"/>
+      <c r="F12" s="173" t="s">
         <v>131</v>
       </c>
-      <c r="G12" s="175" t="s">
+      <c r="G12" s="173" t="s">
         <v>133</v>
       </c>
-      <c r="H12" s="175" t="s">
+      <c r="H12" s="173" t="s">
         <v>132</v>
       </c>
-      <c r="I12" s="175" t="s">
+      <c r="I12" s="173" t="s">
         <v>134</v>
       </c>
-      <c r="J12" s="175" t="s">
+      <c r="J12" s="173" t="s">
         <v>138</v>
       </c>
-      <c r="K12" s="175"/>
-      <c r="L12" s="175"/>
-      <c r="M12" s="175"/>
-      <c r="N12" s="175"/>
-      <c r="O12" s="175"/>
+      <c r="K12" s="173"/>
+      <c r="L12" s="173"/>
+      <c r="M12" s="173"/>
+      <c r="N12" s="173"/>
+      <c r="O12" s="173"/>
       <c r="P12" s="267" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="175"/>
-      <c r="C13" s="175"/>
-      <c r="D13" s="175"/>
-      <c r="E13" s="175"/>
-      <c r="F13" s="175"/>
-      <c r="G13" s="175"/>
-      <c r="H13" s="175"/>
-      <c r="I13" s="175"/>
+      <c r="B13" s="173"/>
+      <c r="C13" s="173"/>
+      <c r="D13" s="173"/>
+      <c r="E13" s="173"/>
+      <c r="F13" s="173"/>
+      <c r="G13" s="173"/>
+      <c r="H13" s="173"/>
+      <c r="I13" s="173"/>
       <c r="J13" s="266" t="s">
         <v>135</v>
       </c>
@@ -6576,14 +6405,14 @@
       <c r="P13" s="267"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="175"/>
-      <c r="C14" s="175"/>
-      <c r="D14" s="175"/>
-      <c r="E14" s="175"/>
-      <c r="F14" s="175"/>
-      <c r="G14" s="175"/>
-      <c r="H14" s="175"/>
-      <c r="I14" s="175"/>
+      <c r="B14" s="173"/>
+      <c r="C14" s="173"/>
+      <c r="D14" s="173"/>
+      <c r="E14" s="173"/>
+      <c r="F14" s="173"/>
+      <c r="G14" s="173"/>
+      <c r="H14" s="173"/>
+      <c r="I14" s="173"/>
       <c r="J14" s="38" t="s">
         <v>118</v>
       </c>
@@ -6998,7 +6827,7 @@
     <mergeCell ref="G12:G14"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P51">
-    <cfRule type="expression" dxfId="30" priority="14">
+    <cfRule type="expression" dxfId="7" priority="14">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7065,10 +6894,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="173" t="s">
+      <c r="C5" s="175" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="173"/>
+      <c r="D5" s="175"/>
       <c r="E5" s="11" t="s">
         <v>80</v>
       </c>
@@ -15422,7 +15251,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="50" priority="2">
+    <cfRule type="expression" dxfId="29" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15508,10 +15337,10 @@
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="175" t="s">
+      <c r="C5" s="173" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="175"/>
+      <c r="D5" s="173"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -17672,23 +17501,23 @@
     <mergeCell ref="B1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:N16997">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="28" priority="1">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="5">
+    <cfRule type="expression" dxfId="27" priority="2">
+      <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="26" priority="5">
       <formula>AND($B6="",$C6&lt;&gt;"")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H16997">
-    <cfRule type="expression" dxfId="8" priority="9">
+    <cfRule type="expression" dxfId="25" priority="9">
       <formula>IF(G6&lt;&gt;"", NOT(AND(OR(LEFT($E6,2)="L.", LEFT($E6,2)="A.", LEFT($E6,2)="B.", LEFT($E6,2)="M."), $H6&lt;&gt;"", $E6&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:K16997">
-    <cfRule type="notContainsBlanks" dxfId="7" priority="8">
+    <cfRule type="notContainsBlanks" dxfId="24" priority="8">
       <formula>LEN(TRIM(H6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -41791,16 +41620,19 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B995 E6:H995">
-    <cfRule type="expression" dxfId="49" priority="6">
+    <cfRule type="expression" dxfId="3" priority="7">
       <formula>$J6=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:H995">
-    <cfRule type="expression" dxfId="48" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>AND(LEN($B6)=1,$C6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="47" priority="2">
-      <formula>$C6&lt;&gt;0</formula>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>AND($C6&lt;&gt;"",$B6="")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="3">
+      <formula>AND($B6&lt;&gt;"",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -41977,11 +41809,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="175" t="s">
+      <c r="C11" s="173" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="175"/>
-      <c r="E11" s="175"/>
+      <c r="D11" s="173"/>
+      <c r="E11" s="173"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -43377,7 +43209,7 @@
     <mergeCell ref="B1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="B12:K9929">
-    <cfRule type="expression" dxfId="46" priority="1">
+    <cfRule type="expression" dxfId="23" priority="1">
       <formula>AND($B12&lt;&gt;"",$C12&lt;&gt;"",$G12="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -43529,11 +43361,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="175" t="s">
+      <c r="C11" s="173" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="175"/>
-      <c r="E11" s="175"/>
+      <c r="D11" s="173"/>
+      <c r="E11" s="173"/>
       <c r="F11" s="40" t="s">
         <v>29</v>
       </c>
@@ -44738,7 +44570,7 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B12:H9929">
-    <cfRule type="expression" dxfId="45" priority="9">
+    <cfRule type="expression" dxfId="22" priority="9">
       <formula>AND($B12&lt;&gt;"",$C12&lt;&gt;"",#REF!="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -44862,39 +44694,39 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:CE7">
-    <cfRule type="expression" dxfId="44" priority="12">
+    <cfRule type="expression" dxfId="21" priority="12">
       <formula>B5&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:CE201">
-    <cfRule type="expression" dxfId="43" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>AND(G8&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="2">
+    <cfRule type="expression" dxfId="19" priority="2">
       <formula>AND(G$7&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="3">
+    <cfRule type="expression" dxfId="18" priority="3">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="4">
+    <cfRule type="expression" dxfId="17" priority="4">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="5">
+    <cfRule type="expression" dxfId="16" priority="5">
       <formula>AND(G8&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="6">
+    <cfRule type="expression" dxfId="15" priority="6">
       <formula>AND(G$7&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="7">
+    <cfRule type="expression" dxfId="14" priority="7">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="8">
+    <cfRule type="expression" dxfId="13" priority="8">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="34" priority="10">
+    <cfRule type="expression" dxfId="11" priority="10">
       <formula>AND(G$7&lt;&gt;"",$B8="DEVIASI")</formula>
     </cfRule>
     <cfRule type="colorScale" priority="11">

</xml_diff>

<commit_message>
fix: update AHSP labels and RAB print area as requested by Bos
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C24FCCDA-96F0-4F11-A9F5-E9336DAB58DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F864DAC-065E-4BD1-A3CE-EBEEAD507F97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="150">
   <si>
     <t>HARGA SATUAN BAHAN, ALAT DAN UPAH</t>
   </si>
@@ -493,6 +493,21 @@
   </si>
   <si>
     <t>LAPORAN BULANAN</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>PEKERJAAN PERSIAPAN</t>
+  </si>
+  <si>
+    <t>1.1.1.1</t>
+  </si>
+  <si>
+    <t>Pembuatan 1 m’ pagar sementara dari kayu tinggi 2 meter</t>
+  </si>
+  <si>
+    <t>m'</t>
   </si>
 </sst>
 </file>
@@ -2280,14 +2295,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2307,6 +2322,66 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="79" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2319,50 +2394,8 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2427,117 +2460,6 @@
     <xf numFmtId="171" fontId="25" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="79" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -2594,6 +2516,99 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="47" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2610,7 +2625,7 @@
     <cellStyle name="Normal 2 2 3" xfId="2" xr:uid="{25DAB206-4C06-437D-BFFA-FD21FFA5A242}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="31">
     <dxf>
       <font>
         <b/>
@@ -2619,7 +2634,7 @@
       <fill>
         <patternFill>
           <fgColor theme="0"/>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor theme="0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2631,7 +2646,7 @@
       <fill>
         <patternFill>
           <fgColor theme="0"/>
-          <bgColor theme="0"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2682,6 +2697,18 @@
         <patternFill>
           <fgColor theme="0"/>
           <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor theme="0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4002,48 +4029,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="231"/>
-      <c r="C1" s="232"/>
-      <c r="D1" s="232"/>
-      <c r="E1" s="232"/>
-      <c r="F1" s="232"/>
-      <c r="G1" s="232"/>
-      <c r="H1" s="232"/>
-      <c r="I1" s="232"/>
-      <c r="J1" s="232"/>
-      <c r="K1" s="232"/>
-      <c r="L1" s="232"/>
-      <c r="M1" s="233"/>
+      <c r="B1" s="182"/>
+      <c r="C1" s="183"/>
+      <c r="D1" s="183"/>
+      <c r="E1" s="183"/>
+      <c r="F1" s="183"/>
+      <c r="G1" s="183"/>
+      <c r="H1" s="183"/>
+      <c r="I1" s="183"/>
+      <c r="J1" s="183"/>
+      <c r="K1" s="183"/>
+      <c r="L1" s="183"/>
+      <c r="M1" s="184"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="234" t="s">
+      <c r="B2" s="185" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="235"/>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
-      <c r="G2" s="235"/>
-      <c r="H2" s="235"/>
-      <c r="I2" s="236"/>
-      <c r="J2" s="240"/>
-      <c r="K2" s="241"/>
-      <c r="L2" s="241"/>
-      <c r="M2" s="242"/>
+      <c r="C2" s="186"/>
+      <c r="D2" s="186"/>
+      <c r="E2" s="186"/>
+      <c r="F2" s="186"/>
+      <c r="G2" s="186"/>
+      <c r="H2" s="186"/>
+      <c r="I2" s="187"/>
+      <c r="J2" s="191"/>
+      <c r="K2" s="192"/>
+      <c r="L2" s="192"/>
+      <c r="M2" s="193"/>
     </row>
     <row r="3" spans="1:14" ht="14.4" customHeight="1">
-      <c r="B3" s="237"/>
-      <c r="C3" s="238"/>
-      <c r="D3" s="238"/>
-      <c r="E3" s="238"/>
-      <c r="F3" s="238"/>
-      <c r="G3" s="238"/>
-      <c r="H3" s="238"/>
-      <c r="I3" s="239"/>
-      <c r="J3" s="243"/>
-      <c r="K3" s="244"/>
-      <c r="L3" s="244"/>
-      <c r="M3" s="245"/>
+      <c r="B3" s="188"/>
+      <c r="C3" s="189"/>
+      <c r="D3" s="189"/>
+      <c r="E3" s="189"/>
+      <c r="F3" s="189"/>
+      <c r="G3" s="189"/>
+      <c r="H3" s="189"/>
+      <c r="I3" s="190"/>
+      <c r="J3" s="194"/>
+      <c r="K3" s="195"/>
+      <c r="L3" s="195"/>
+      <c r="M3" s="196"/>
     </row>
     <row r="4" spans="1:14" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -4054,10 +4081,10 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="243"/>
-      <c r="K4" s="244"/>
-      <c r="L4" s="244"/>
-      <c r="M4" s="245"/>
+      <c r="J4" s="194"/>
+      <c r="K4" s="195"/>
+      <c r="L4" s="195"/>
+      <c r="M4" s="196"/>
     </row>
     <row r="5" spans="1:14" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -4072,10 +4099,10 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="243"/>
-      <c r="K5" s="244"/>
-      <c r="L5" s="244"/>
-      <c r="M5" s="245"/>
+      <c r="J5" s="194"/>
+      <c r="K5" s="195"/>
+      <c r="L5" s="195"/>
+      <c r="M5" s="196"/>
     </row>
     <row r="6" spans="1:14" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -4090,10 +4117,10 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="246"/>
-      <c r="K6" s="247"/>
-      <c r="L6" s="247"/>
-      <c r="M6" s="248"/>
+      <c r="J6" s="197"/>
+      <c r="K6" s="198"/>
+      <c r="L6" s="198"/>
+      <c r="M6" s="199"/>
     </row>
     <row r="7" spans="1:14" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -4158,52 +4185,52 @@
       <c r="M9" s="89"/>
     </row>
     <row r="10" spans="1:14" ht="15.6">
-      <c r="B10" s="182" t="s">
+      <c r="B10" s="200" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="183"/>
-      <c r="D10" s="183"/>
-      <c r="E10" s="183"/>
-      <c r="F10" s="183"/>
-      <c r="G10" s="183" t="s">
+      <c r="C10" s="201"/>
+      <c r="D10" s="201"/>
+      <c r="E10" s="201"/>
+      <c r="F10" s="201"/>
+      <c r="G10" s="201" t="s">
         <v>95</v>
       </c>
-      <c r="H10" s="183"/>
-      <c r="I10" s="183"/>
-      <c r="J10" s="184"/>
-      <c r="K10" s="185" t="s">
+      <c r="H10" s="201"/>
+      <c r="I10" s="201"/>
+      <c r="J10" s="202"/>
+      <c r="K10" s="203" t="s">
         <v>96</v>
       </c>
-      <c r="L10" s="183"/>
-      <c r="M10" s="249"/>
+      <c r="L10" s="201"/>
+      <c r="M10" s="204"/>
     </row>
     <row r="11" spans="1:14" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="206" t="s">
+      <c r="C11" s="210" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="259"/>
-      <c r="E11" s="259"/>
+      <c r="D11" s="232"/>
+      <c r="E11" s="232"/>
       <c r="F11" s="92" t="s">
         <v>98</v>
       </c>
-      <c r="G11" s="206" t="s">
+      <c r="G11" s="210" t="s">
         <v>99</v>
       </c>
-      <c r="H11" s="207"/>
+      <c r="H11" s="211"/>
       <c r="I11" s="93" t="s">
         <v>27</v>
       </c>
       <c r="J11" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="206" t="s">
+      <c r="K11" s="210" t="s">
         <v>100</v>
       </c>
-      <c r="L11" s="207"/>
+      <c r="L11" s="211"/>
       <c r="M11" s="94" t="s">
         <v>101</v>
       </c>
@@ -4408,58 +4435,58 @@
       <c r="M22" s="123"/>
     </row>
     <row r="23" spans="1:13" ht="16.2" thickBot="1">
-      <c r="B23" s="260"/>
-      <c r="C23" s="261"/>
-      <c r="D23" s="261"/>
-      <c r="E23" s="261"/>
+      <c r="B23" s="233"/>
+      <c r="C23" s="234"/>
+      <c r="D23" s="234"/>
+      <c r="E23" s="234"/>
       <c r="F23" s="124"/>
       <c r="G23" s="124"/>
       <c r="H23" s="125"/>
       <c r="I23" s="125"/>
-      <c r="J23" s="262"/>
-      <c r="K23" s="262"/>
-      <c r="L23" s="262"/>
-      <c r="M23" s="263"/>
+      <c r="J23" s="235"/>
+      <c r="K23" s="235"/>
+      <c r="L23" s="235"/>
+      <c r="M23" s="236"/>
     </row>
     <row r="24" spans="1:13" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="152" t="s">
         <v>116</v>
       </c>
-      <c r="B24" s="264" t="s">
+      <c r="B24" s="237" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="201" t="s">
+      <c r="C24" s="205" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="201"/>
-      <c r="E24" s="201"/>
-      <c r="F24" s="201"/>
-      <c r="G24" s="201"/>
-      <c r="H24" s="201"/>
-      <c r="I24" s="201"/>
-      <c r="J24" s="203" t="s">
+      <c r="D24" s="205"/>
+      <c r="E24" s="205"/>
+      <c r="F24" s="205"/>
+      <c r="G24" s="205"/>
+      <c r="H24" s="205"/>
+      <c r="I24" s="205"/>
+      <c r="J24" s="207" t="s">
         <v>117</v>
       </c>
-      <c r="K24" s="204"/>
-      <c r="L24" s="204"/>
-      <c r="M24" s="205"/>
+      <c r="K24" s="208"/>
+      <c r="L24" s="208"/>
+      <c r="M24" s="209"/>
     </row>
     <row r="25" spans="1:13" ht="31.2">
-      <c r="B25" s="265"/>
-      <c r="C25" s="202"/>
-      <c r="D25" s="202"/>
-      <c r="E25" s="202"/>
-      <c r="F25" s="202"/>
-      <c r="G25" s="202"/>
-      <c r="H25" s="202"/>
-      <c r="I25" s="202"/>
+      <c r="B25" s="238"/>
+      <c r="C25" s="206"/>
+      <c r="D25" s="206"/>
+      <c r="E25" s="206"/>
+      <c r="F25" s="206"/>
+      <c r="G25" s="206"/>
+      <c r="H25" s="206"/>
+      <c r="I25" s="206"/>
       <c r="J25" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="217" t="s">
+      <c r="K25" s="221" t="s">
         <v>118</v>
       </c>
-      <c r="L25" s="218"/>
+      <c r="L25" s="222"/>
       <c r="M25" s="126" t="s">
         <v>119</v>
       </c>
@@ -5017,60 +5044,60 @@
       </c>
     </row>
     <row r="49" spans="2:13" ht="16.2" thickTop="1">
-      <c r="B49" s="195" t="s">
+      <c r="B49" s="248" t="s">
         <v>120</v>
       </c>
-      <c r="C49" s="196"/>
-      <c r="D49" s="196"/>
-      <c r="E49" s="196"/>
-      <c r="F49" s="196"/>
-      <c r="G49" s="196"/>
-      <c r="H49" s="196"/>
-      <c r="I49" s="196"/>
-      <c r="J49" s="197"/>
-      <c r="K49" s="256" t="s">
+      <c r="C49" s="249"/>
+      <c r="D49" s="249"/>
+      <c r="E49" s="249"/>
+      <c r="F49" s="249"/>
+      <c r="G49" s="249"/>
+      <c r="H49" s="249"/>
+      <c r="I49" s="249"/>
+      <c r="J49" s="250"/>
+      <c r="K49" s="229" t="s">
         <v>121</v>
       </c>
-      <c r="L49" s="257"/>
-      <c r="M49" s="258"/>
+      <c r="L49" s="230"/>
+      <c r="M49" s="231"/>
     </row>
     <row r="50" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B50" s="198"/>
-      <c r="C50" s="199"/>
-      <c r="D50" s="199"/>
-      <c r="E50" s="199"/>
-      <c r="F50" s="199"/>
-      <c r="G50" s="199"/>
-      <c r="H50" s="199"/>
-      <c r="I50" s="199"/>
-      <c r="J50" s="200"/>
-      <c r="K50" s="253"/>
-      <c r="L50" s="254"/>
-      <c r="M50" s="255"/>
+      <c r="B50" s="251"/>
+      <c r="C50" s="252"/>
+      <c r="D50" s="252"/>
+      <c r="E50" s="252"/>
+      <c r="F50" s="252"/>
+      <c r="G50" s="252"/>
+      <c r="H50" s="252"/>
+      <c r="I50" s="252"/>
+      <c r="J50" s="253"/>
+      <c r="K50" s="226"/>
+      <c r="L50" s="227"/>
+      <c r="M50" s="228"/>
     </row>
     <row r="51" spans="2:13" ht="15.6">
       <c r="B51" s="138"/>
-      <c r="C51" s="250"/>
-      <c r="D51" s="250"/>
-      <c r="E51" s="250"/>
-      <c r="F51" s="250"/>
-      <c r="G51" s="250"/>
-      <c r="H51" s="250"/>
-      <c r="I51" s="250"/>
+      <c r="C51" s="223"/>
+      <c r="D51" s="223"/>
+      <c r="E51" s="223"/>
+      <c r="F51" s="223"/>
+      <c r="G51" s="223"/>
+      <c r="H51" s="223"/>
+      <c r="I51" s="223"/>
       <c r="J51" s="139"/>
-      <c r="K51" s="214"/>
-      <c r="L51" s="215"/>
-      <c r="M51" s="216"/>
+      <c r="K51" s="218"/>
+      <c r="L51" s="219"/>
+      <c r="M51" s="220"/>
     </row>
     <row r="52" spans="2:13" ht="15.6">
       <c r="B52" s="140"/>
-      <c r="C52" s="251"/>
-      <c r="D52" s="251"/>
-      <c r="E52" s="251"/>
-      <c r="F52" s="251"/>
-      <c r="G52" s="251"/>
-      <c r="H52" s="251"/>
-      <c r="I52" s="251"/>
+      <c r="C52" s="224"/>
+      <c r="D52" s="224"/>
+      <c r="E52" s="224"/>
+      <c r="F52" s="224"/>
+      <c r="G52" s="224"/>
+      <c r="H52" s="224"/>
+      <c r="I52" s="224"/>
       <c r="J52" s="141"/>
       <c r="K52" s="164"/>
       <c r="L52" s="161"/>
@@ -5078,13 +5105,13 @@
     </row>
     <row r="53" spans="2:13" ht="15.6">
       <c r="B53" s="140"/>
-      <c r="C53" s="251"/>
-      <c r="D53" s="251"/>
-      <c r="E53" s="251"/>
-      <c r="F53" s="251"/>
-      <c r="G53" s="251"/>
-      <c r="H53" s="251"/>
-      <c r="I53" s="251"/>
+      <c r="C53" s="224"/>
+      <c r="D53" s="224"/>
+      <c r="E53" s="224"/>
+      <c r="F53" s="224"/>
+      <c r="G53" s="224"/>
+      <c r="H53" s="224"/>
+      <c r="I53" s="224"/>
       <c r="J53" s="141"/>
       <c r="K53" s="164"/>
       <c r="L53" s="161"/>
@@ -5092,13 +5119,13 @@
     </row>
     <row r="54" spans="2:13" ht="15.6">
       <c r="B54" s="140"/>
-      <c r="C54" s="251"/>
-      <c r="D54" s="251"/>
-      <c r="E54" s="251"/>
-      <c r="F54" s="251"/>
-      <c r="G54" s="251"/>
-      <c r="H54" s="251"/>
-      <c r="I54" s="251"/>
+      <c r="C54" s="224"/>
+      <c r="D54" s="224"/>
+      <c r="E54" s="224"/>
+      <c r="F54" s="224"/>
+      <c r="G54" s="224"/>
+      <c r="H54" s="224"/>
+      <c r="I54" s="224"/>
       <c r="J54" s="141"/>
       <c r="K54" s="164"/>
       <c r="L54" s="161"/>
@@ -5106,13 +5133,13 @@
     </row>
     <row r="55" spans="2:13" ht="15.6">
       <c r="B55" s="143"/>
-      <c r="C55" s="251"/>
-      <c r="D55" s="251"/>
-      <c r="E55" s="251"/>
-      <c r="F55" s="251"/>
-      <c r="G55" s="251"/>
-      <c r="H55" s="251"/>
-      <c r="I55" s="251"/>
+      <c r="C55" s="224"/>
+      <c r="D55" s="224"/>
+      <c r="E55" s="224"/>
+      <c r="F55" s="224"/>
+      <c r="G55" s="224"/>
+      <c r="H55" s="224"/>
+      <c r="I55" s="224"/>
       <c r="J55" s="144"/>
       <c r="K55" s="164"/>
       <c r="L55" s="145"/>
@@ -5120,13 +5147,13 @@
     </row>
     <row r="56" spans="2:13" ht="15.6">
       <c r="B56" s="143"/>
-      <c r="C56" s="251"/>
-      <c r="D56" s="251"/>
-      <c r="E56" s="251"/>
-      <c r="F56" s="251"/>
-      <c r="G56" s="251"/>
-      <c r="H56" s="251"/>
-      <c r="I56" s="251"/>
+      <c r="C56" s="224"/>
+      <c r="D56" s="224"/>
+      <c r="E56" s="224"/>
+      <c r="F56" s="224"/>
+      <c r="G56" s="224"/>
+      <c r="H56" s="224"/>
+      <c r="I56" s="224"/>
       <c r="J56" s="144"/>
       <c r="K56" s="164"/>
       <c r="L56" s="145"/>
@@ -5134,41 +5161,41 @@
     </row>
     <row r="57" spans="2:13" ht="15.6">
       <c r="B57" s="143"/>
-      <c r="C57" s="251"/>
-      <c r="D57" s="251"/>
-      <c r="E57" s="251"/>
-      <c r="F57" s="251"/>
-      <c r="G57" s="251"/>
-      <c r="H57" s="251"/>
-      <c r="I57" s="251"/>
+      <c r="C57" s="224"/>
+      <c r="D57" s="224"/>
+      <c r="E57" s="224"/>
+      <c r="F57" s="224"/>
+      <c r="G57" s="224"/>
+      <c r="H57" s="224"/>
+      <c r="I57" s="224"/>
       <c r="J57" s="144"/>
-      <c r="K57" s="208"/>
-      <c r="L57" s="209"/>
-      <c r="M57" s="210"/>
+      <c r="K57" s="212"/>
+      <c r="L57" s="213"/>
+      <c r="M57" s="214"/>
     </row>
     <row r="58" spans="2:13" ht="15.6">
       <c r="B58" s="143"/>
-      <c r="C58" s="251"/>
-      <c r="D58" s="251"/>
-      <c r="E58" s="251"/>
-      <c r="F58" s="251"/>
-      <c r="G58" s="251"/>
-      <c r="H58" s="251"/>
-      <c r="I58" s="251"/>
+      <c r="C58" s="224"/>
+      <c r="D58" s="224"/>
+      <c r="E58" s="224"/>
+      <c r="F58" s="224"/>
+      <c r="G58" s="224"/>
+      <c r="H58" s="224"/>
+      <c r="I58" s="224"/>
       <c r="J58" s="144"/>
-      <c r="K58" s="211"/>
-      <c r="L58" s="212"/>
-      <c r="M58" s="213"/>
+      <c r="K58" s="215"/>
+      <c r="L58" s="216"/>
+      <c r="M58" s="217"/>
     </row>
     <row r="59" spans="2:13" ht="15.6">
       <c r="B59" s="143"/>
-      <c r="C59" s="251"/>
-      <c r="D59" s="251"/>
-      <c r="E59" s="251"/>
-      <c r="F59" s="251"/>
-      <c r="G59" s="251"/>
-      <c r="H59" s="251"/>
-      <c r="I59" s="251"/>
+      <c r="C59" s="224"/>
+      <c r="D59" s="224"/>
+      <c r="E59" s="224"/>
+      <c r="F59" s="224"/>
+      <c r="G59" s="224"/>
+      <c r="H59" s="224"/>
+      <c r="I59" s="224"/>
       <c r="J59" s="144"/>
       <c r="K59" s="164"/>
       <c r="L59" s="162"/>
@@ -5176,13 +5203,13 @@
     </row>
     <row r="60" spans="2:13" ht="15.6">
       <c r="B60" s="143"/>
-      <c r="C60" s="251"/>
-      <c r="D60" s="251"/>
-      <c r="E60" s="251"/>
-      <c r="F60" s="251"/>
-      <c r="G60" s="251"/>
-      <c r="H60" s="251"/>
-      <c r="I60" s="251"/>
+      <c r="C60" s="224"/>
+      <c r="D60" s="224"/>
+      <c r="E60" s="224"/>
+      <c r="F60" s="224"/>
+      <c r="G60" s="224"/>
+      <c r="H60" s="224"/>
+      <c r="I60" s="224"/>
       <c r="J60" s="144"/>
       <c r="K60" s="164"/>
       <c r="L60" s="162"/>
@@ -5190,13 +5217,13 @@
     </row>
     <row r="61" spans="2:13" ht="15.6">
       <c r="B61" s="143"/>
-      <c r="C61" s="252"/>
-      <c r="D61" s="252"/>
-      <c r="E61" s="252"/>
-      <c r="F61" s="252"/>
-      <c r="G61" s="252"/>
-      <c r="H61" s="252"/>
-      <c r="I61" s="252"/>
+      <c r="C61" s="225"/>
+      <c r="D61" s="225"/>
+      <c r="E61" s="225"/>
+      <c r="F61" s="225"/>
+      <c r="G61" s="225"/>
+      <c r="H61" s="225"/>
+      <c r="I61" s="225"/>
       <c r="J61" s="144"/>
       <c r="K61" s="164"/>
       <c r="L61" s="162"/>
@@ -5217,133 +5244,133 @@
       <c r="M62" s="167"/>
     </row>
     <row r="63" spans="2:13" ht="15.6">
-      <c r="B63" s="182" t="s">
+      <c r="B63" s="200" t="s">
         <v>122</v>
       </c>
-      <c r="C63" s="183"/>
-      <c r="D63" s="183"/>
-      <c r="E63" s="184"/>
-      <c r="F63" s="185" t="s">
+      <c r="C63" s="201"/>
+      <c r="D63" s="201"/>
+      <c r="E63" s="202"/>
+      <c r="F63" s="203" t="s">
         <v>123</v>
       </c>
-      <c r="G63" s="184"/>
-      <c r="H63" s="185" t="s">
+      <c r="G63" s="202"/>
+      <c r="H63" s="203" t="s">
         <v>124</v>
       </c>
-      <c r="I63" s="183"/>
-      <c r="J63" s="184"/>
+      <c r="I63" s="201"/>
+      <c r="J63" s="202"/>
       <c r="K63" s="165"/>
       <c r="L63" s="145"/>
       <c r="M63" s="146"/>
     </row>
     <row r="64" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B64" s="225"/>
-      <c r="C64" s="226"/>
-      <c r="D64" s="226"/>
-      <c r="E64" s="220"/>
-      <c r="F64" s="219"/>
-      <c r="G64" s="220"/>
-      <c r="H64" s="186"/>
-      <c r="I64" s="187"/>
-      <c r="J64" s="188"/>
+      <c r="B64" s="260"/>
+      <c r="C64" s="261"/>
+      <c r="D64" s="261"/>
+      <c r="E64" s="255"/>
+      <c r="F64" s="254"/>
+      <c r="G64" s="255"/>
+      <c r="H64" s="239"/>
+      <c r="I64" s="240"/>
+      <c r="J64" s="241"/>
       <c r="K64" s="148"/>
       <c r="L64" s="145"/>
       <c r="M64" s="146"/>
     </row>
     <row r="65" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B65" s="227"/>
-      <c r="C65" s="228"/>
-      <c r="D65" s="228"/>
-      <c r="E65" s="222"/>
-      <c r="F65" s="221"/>
-      <c r="G65" s="222"/>
-      <c r="H65" s="189"/>
-      <c r="I65" s="190"/>
-      <c r="J65" s="191"/>
+      <c r="B65" s="262"/>
+      <c r="C65" s="263"/>
+      <c r="D65" s="263"/>
+      <c r="E65" s="257"/>
+      <c r="F65" s="256"/>
+      <c r="G65" s="257"/>
+      <c r="H65" s="242"/>
+      <c r="I65" s="243"/>
+      <c r="J65" s="244"/>
       <c r="K65" s="148"/>
       <c r="L65" s="163"/>
       <c r="M65" s="146"/>
     </row>
     <row r="66" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B66" s="227"/>
-      <c r="C66" s="228"/>
-      <c r="D66" s="228"/>
-      <c r="E66" s="222"/>
-      <c r="F66" s="221"/>
-      <c r="G66" s="222"/>
-      <c r="H66" s="189"/>
-      <c r="I66" s="190"/>
-      <c r="J66" s="191"/>
+      <c r="B66" s="262"/>
+      <c r="C66" s="263"/>
+      <c r="D66" s="263"/>
+      <c r="E66" s="257"/>
+      <c r="F66" s="256"/>
+      <c r="G66" s="257"/>
+      <c r="H66" s="242"/>
+      <c r="I66" s="243"/>
+      <c r="J66" s="244"/>
       <c r="K66" s="148"/>
       <c r="L66" s="145"/>
       <c r="M66" s="146"/>
     </row>
     <row r="67" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B67" s="227"/>
-      <c r="C67" s="228"/>
-      <c r="D67" s="228"/>
-      <c r="E67" s="222"/>
-      <c r="F67" s="221"/>
-      <c r="G67" s="222"/>
-      <c r="H67" s="189"/>
-      <c r="I67" s="190"/>
-      <c r="J67" s="191"/>
+      <c r="B67" s="262"/>
+      <c r="C67" s="263"/>
+      <c r="D67" s="263"/>
+      <c r="E67" s="257"/>
+      <c r="F67" s="256"/>
+      <c r="G67" s="257"/>
+      <c r="H67" s="242"/>
+      <c r="I67" s="243"/>
+      <c r="J67" s="244"/>
       <c r="K67" s="148"/>
       <c r="L67" s="162"/>
       <c r="M67" s="76"/>
     </row>
     <row r="68" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B68" s="227"/>
-      <c r="C68" s="228"/>
-      <c r="D68" s="228"/>
-      <c r="E68" s="222"/>
-      <c r="F68" s="221"/>
-      <c r="G68" s="222"/>
-      <c r="H68" s="189"/>
-      <c r="I68" s="190"/>
-      <c r="J68" s="191"/>
+      <c r="B68" s="262"/>
+      <c r="C68" s="263"/>
+      <c r="D68" s="263"/>
+      <c r="E68" s="257"/>
+      <c r="F68" s="256"/>
+      <c r="G68" s="257"/>
+      <c r="H68" s="242"/>
+      <c r="I68" s="243"/>
+      <c r="J68" s="244"/>
       <c r="K68" s="148"/>
       <c r="L68" s="162"/>
       <c r="M68" s="76"/>
     </row>
     <row r="69" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B69" s="227"/>
-      <c r="C69" s="228"/>
-      <c r="D69" s="228"/>
-      <c r="E69" s="222"/>
-      <c r="F69" s="221"/>
-      <c r="G69" s="222"/>
-      <c r="H69" s="189"/>
-      <c r="I69" s="190"/>
-      <c r="J69" s="191"/>
+      <c r="B69" s="262"/>
+      <c r="C69" s="263"/>
+      <c r="D69" s="263"/>
+      <c r="E69" s="257"/>
+      <c r="F69" s="256"/>
+      <c r="G69" s="257"/>
+      <c r="H69" s="242"/>
+      <c r="I69" s="243"/>
+      <c r="J69" s="244"/>
       <c r="K69" s="168"/>
       <c r="L69" s="169"/>
       <c r="M69" s="170"/>
     </row>
     <row r="70" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B70" s="227"/>
-      <c r="C70" s="228"/>
-      <c r="D70" s="228"/>
-      <c r="E70" s="222"/>
-      <c r="F70" s="221"/>
-      <c r="G70" s="222"/>
-      <c r="H70" s="189"/>
-      <c r="I70" s="190"/>
-      <c r="J70" s="191"/>
+      <c r="B70" s="262"/>
+      <c r="C70" s="263"/>
+      <c r="D70" s="263"/>
+      <c r="E70" s="257"/>
+      <c r="F70" s="256"/>
+      <c r="G70" s="257"/>
+      <c r="H70" s="242"/>
+      <c r="I70" s="243"/>
+      <c r="J70" s="244"/>
       <c r="K70" s="168"/>
       <c r="L70" s="169"/>
       <c r="M70" s="170"/>
     </row>
     <row r="71" spans="2:13" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B71" s="229"/>
-      <c r="C71" s="230"/>
-      <c r="D71" s="230"/>
-      <c r="E71" s="224"/>
-      <c r="F71" s="223"/>
-      <c r="G71" s="224"/>
-      <c r="H71" s="192"/>
-      <c r="I71" s="193"/>
-      <c r="J71" s="194"/>
+      <c r="B71" s="264"/>
+      <c r="C71" s="265"/>
+      <c r="D71" s="265"/>
+      <c r="E71" s="259"/>
+      <c r="F71" s="258"/>
+      <c r="G71" s="259"/>
+      <c r="H71" s="245"/>
+      <c r="I71" s="246"/>
+      <c r="J71" s="247"/>
       <c r="K71" s="150"/>
       <c r="L71" s="149"/>
       <c r="M71" s="151"/>
@@ -5356,12 +5383,13 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="J2:M6"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="H63:J63"/>
+    <mergeCell ref="H64:J71"/>
+    <mergeCell ref="B49:J50"/>
+    <mergeCell ref="F64:G71"/>
+    <mergeCell ref="B64:E71"/>
     <mergeCell ref="C24:I25"/>
     <mergeCell ref="J24:M24"/>
     <mergeCell ref="K11:L11"/>
@@ -5377,21 +5405,20 @@
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="J23:M23"/>
     <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="H63:J63"/>
-    <mergeCell ref="H64:J71"/>
-    <mergeCell ref="B49:J50"/>
-    <mergeCell ref="F64:G71"/>
-    <mergeCell ref="B64:E71"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="J2:M6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="K10:M10"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:I48">
-    <cfRule type="expression" dxfId="10" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>ISTEXT($C26)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J27:M48">
-    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5654,47 +5681,47 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="173" t="s">
+      <c r="B12" s="175" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="173" t="s">
+      <c r="C12" s="175" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="173"/>
-      <c r="E12" s="173"/>
-      <c r="F12" s="173" t="s">
+      <c r="D12" s="175"/>
+      <c r="E12" s="175"/>
+      <c r="F12" s="175" t="s">
         <v>131</v>
       </c>
-      <c r="G12" s="173" t="s">
+      <c r="G12" s="175" t="s">
         <v>133</v>
       </c>
-      <c r="H12" s="173" t="s">
+      <c r="H12" s="175" t="s">
         <v>132</v>
       </c>
-      <c r="I12" s="173" t="s">
+      <c r="I12" s="175" t="s">
         <v>134</v>
       </c>
-      <c r="J12" s="173" t="s">
+      <c r="J12" s="175" t="s">
         <v>138</v>
       </c>
-      <c r="K12" s="173"/>
-      <c r="L12" s="173"/>
-      <c r="M12" s="173"/>
-      <c r="N12" s="173"/>
-      <c r="O12" s="173"/>
+      <c r="K12" s="175"/>
+      <c r="L12" s="175"/>
+      <c r="M12" s="175"/>
+      <c r="N12" s="175"/>
+      <c r="O12" s="175"/>
       <c r="P12" s="267" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="173"/>
-      <c r="C13" s="173"/>
-      <c r="D13" s="173"/>
-      <c r="E13" s="173"/>
-      <c r="F13" s="173"/>
-      <c r="G13" s="173"/>
-      <c r="H13" s="173"/>
-      <c r="I13" s="173"/>
+      <c r="B13" s="175"/>
+      <c r="C13" s="175"/>
+      <c r="D13" s="175"/>
+      <c r="E13" s="175"/>
+      <c r="F13" s="175"/>
+      <c r="G13" s="175"/>
+      <c r="H13" s="175"/>
+      <c r="I13" s="175"/>
       <c r="J13" s="266" t="s">
         <v>135</v>
       </c>
@@ -5710,14 +5737,14 @@
       <c r="P13" s="267"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="173"/>
-      <c r="C14" s="173"/>
-      <c r="D14" s="173"/>
-      <c r="E14" s="173"/>
-      <c r="F14" s="173"/>
-      <c r="G14" s="173"/>
-      <c r="H14" s="173"/>
-      <c r="I14" s="173"/>
+      <c r="B14" s="175"/>
+      <c r="C14" s="175"/>
+      <c r="D14" s="175"/>
+      <c r="E14" s="175"/>
+      <c r="F14" s="175"/>
+      <c r="G14" s="175"/>
+      <c r="H14" s="175"/>
+      <c r="I14" s="175"/>
       <c r="J14" s="38" t="s">
         <v>118</v>
       </c>
@@ -6086,7 +6113,7 @@
     <mergeCell ref="I4:P5"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P49">
-    <cfRule type="expression" dxfId="8" priority="13">
+    <cfRule type="expression" dxfId="9" priority="13">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6349,47 +6376,47 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="173" t="s">
+      <c r="B12" s="175" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="173" t="s">
+      <c r="C12" s="175" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="173"/>
-      <c r="E12" s="173"/>
-      <c r="F12" s="173" t="s">
+      <c r="D12" s="175"/>
+      <c r="E12" s="175"/>
+      <c r="F12" s="175" t="s">
         <v>131</v>
       </c>
-      <c r="G12" s="173" t="s">
+      <c r="G12" s="175" t="s">
         <v>133</v>
       </c>
-      <c r="H12" s="173" t="s">
+      <c r="H12" s="175" t="s">
         <v>132</v>
       </c>
-      <c r="I12" s="173" t="s">
+      <c r="I12" s="175" t="s">
         <v>134</v>
       </c>
-      <c r="J12" s="173" t="s">
+      <c r="J12" s="175" t="s">
         <v>138</v>
       </c>
-      <c r="K12" s="173"/>
-      <c r="L12" s="173"/>
-      <c r="M12" s="173"/>
-      <c r="N12" s="173"/>
-      <c r="O12" s="173"/>
+      <c r="K12" s="175"/>
+      <c r="L12" s="175"/>
+      <c r="M12" s="175"/>
+      <c r="N12" s="175"/>
+      <c r="O12" s="175"/>
       <c r="P12" s="267" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="173"/>
-      <c r="C13" s="173"/>
-      <c r="D13" s="173"/>
-      <c r="E13" s="173"/>
-      <c r="F13" s="173"/>
-      <c r="G13" s="173"/>
-      <c r="H13" s="173"/>
-      <c r="I13" s="173"/>
+      <c r="B13" s="175"/>
+      <c r="C13" s="175"/>
+      <c r="D13" s="175"/>
+      <c r="E13" s="175"/>
+      <c r="F13" s="175"/>
+      <c r="G13" s="175"/>
+      <c r="H13" s="175"/>
+      <c r="I13" s="175"/>
       <c r="J13" s="266" t="s">
         <v>135</v>
       </c>
@@ -6405,14 +6432,14 @@
       <c r="P13" s="267"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="173"/>
-      <c r="C14" s="173"/>
-      <c r="D14" s="173"/>
-      <c r="E14" s="173"/>
-      <c r="F14" s="173"/>
-      <c r="G14" s="173"/>
-      <c r="H14" s="173"/>
-      <c r="I14" s="173"/>
+      <c r="B14" s="175"/>
+      <c r="C14" s="175"/>
+      <c r="D14" s="175"/>
+      <c r="E14" s="175"/>
+      <c r="F14" s="175"/>
+      <c r="G14" s="175"/>
+      <c r="H14" s="175"/>
+      <c r="I14" s="175"/>
       <c r="J14" s="38" t="s">
         <v>118</v>
       </c>
@@ -6827,7 +6854,7 @@
     <mergeCell ref="G12:G14"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P51">
-    <cfRule type="expression" dxfId="7" priority="14">
+    <cfRule type="expression" dxfId="8" priority="14">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6855,14 +6882,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
-      <c r="E1" s="174"/>
-      <c r="F1" s="174"/>
-      <c r="G1" s="174"/>
-      <c r="H1" s="174"/>
-      <c r="I1" s="174"/>
+      <c r="B1" s="173"/>
+      <c r="C1" s="173"/>
+      <c r="D1" s="173"/>
+      <c r="E1" s="173"/>
+      <c r="F1" s="173"/>
+      <c r="G1" s="173"/>
+      <c r="H1" s="173"/>
+      <c r="I1" s="173"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
       <c r="B2" s="171" t="s">
@@ -6894,10 +6921,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="175" t="s">
+      <c r="C5" s="174" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="175"/>
+      <c r="D5" s="174"/>
       <c r="E5" s="11" t="s">
         <v>80</v>
       </c>
@@ -15251,7 +15278,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="29" priority="2">
+    <cfRule type="expression" dxfId="30" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15284,19 +15311,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
-      <c r="E1" s="174"/>
-      <c r="F1" s="174"/>
-      <c r="G1" s="174"/>
-      <c r="H1" s="174"/>
-      <c r="I1" s="174"/>
-      <c r="J1" s="174"/>
-      <c r="K1" s="174"/>
-      <c r="L1" s="174"/>
-      <c r="M1" s="174"/>
-      <c r="N1" s="174"/>
+      <c r="B1" s="173"/>
+      <c r="C1" s="173"/>
+      <c r="D1" s="173"/>
+      <c r="E1" s="173"/>
+      <c r="F1" s="173"/>
+      <c r="G1" s="173"/>
+      <c r="H1" s="173"/>
+      <c r="I1" s="173"/>
+      <c r="J1" s="173"/>
+      <c r="K1" s="173"/>
+      <c r="L1" s="173"/>
+      <c r="M1" s="173"/>
+      <c r="N1" s="173"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
       <c r="B2" s="171" t="s">
@@ -15337,10 +15364,10 @@
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="173" t="s">
+      <c r="C5" s="175" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="173"/>
+      <c r="D5" s="175"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -17501,23 +17528,23 @@
     <mergeCell ref="B1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:N16997">
-    <cfRule type="expression" dxfId="28" priority="1">
+    <cfRule type="expression" dxfId="29" priority="1">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="2">
+    <cfRule type="expression" dxfId="28" priority="2">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="5">
+    <cfRule type="expression" dxfId="27" priority="5">
       <formula>AND($B6="",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H16997">
-    <cfRule type="expression" dxfId="25" priority="9">
+    <cfRule type="expression" dxfId="26" priority="9">
       <formula>IF(G6&lt;&gt;"", NOT(AND(OR(LEFT($E6,2)="L.", LEFT($E6,2)="A.", LEFT($E6,2)="B.", LEFT($E6,2)="M."), $H6&lt;&gt;"", $E6&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:K16997">
-    <cfRule type="notContainsBlanks" dxfId="24" priority="8">
+    <cfRule type="notContainsBlanks" dxfId="25" priority="8">
       <formula>LEN(TRIM(H6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17544,13 +17571,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
-      <c r="E1" s="174"/>
-      <c r="F1" s="174"/>
-      <c r="G1" s="174"/>
-      <c r="H1" s="174"/>
+      <c r="B1" s="173"/>
+      <c r="C1" s="173"/>
+      <c r="D1" s="173"/>
+      <c r="E1" s="173"/>
+      <c r="F1" s="173"/>
+      <c r="G1" s="173"/>
+      <c r="H1" s="173"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
       <c r="B2" s="171" t="s">
@@ -17602,22 +17629,38 @@
       <c r="J5" s="29"/>
     </row>
     <row r="6" spans="2:10">
-      <c r="B6" s="30"/>
+      <c r="B6" s="30" t="s">
+        <v>145</v>
+      </c>
       <c r="C6" s="31"/>
-      <c r="D6" s="30"/>
+      <c r="D6" s="30" t="s">
+        <v>146</v>
+      </c>
       <c r="E6" s="32"/>
       <c r="F6" s="33"/>
       <c r="G6" s="53"/>
       <c r="H6" s="33"/>
     </row>
     <row r="7" spans="2:10">
-      <c r="B7" s="30"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="30"/>
+      <c r="B7" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="C7" s="31">
+        <v>1</v>
+      </c>
+      <c r="D7" s="30" t="s">
+        <v>148</v>
+      </c>
       <c r="E7" s="32"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="53"/>
-      <c r="H7" s="34"/>
+      <c r="F7" s="33" t="s">
+        <v>149</v>
+      </c>
+      <c r="G7" s="53">
+        <v>580608</v>
+      </c>
+      <c r="H7" s="34">
+        <v>0.97428571428571431</v>
+      </c>
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="30"/>
@@ -41620,18 +41663,18 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B995 E6:H995">
-    <cfRule type="expression" dxfId="3" priority="7">
+    <cfRule type="expression" dxfId="7" priority="7">
       <formula>$J6=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:H995">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>AND(LEN($B6)=1,$C6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>AND($C6&lt;&gt;"",$B6="")</formula>
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>AND($C6="",$B6&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>AND($B6&lt;&gt;"",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -41809,11 +41852,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="173" t="s">
+      <c r="C11" s="175" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="173"/>
-      <c r="E11" s="173"/>
+      <c r="D11" s="175"/>
+      <c r="E11" s="175"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -43209,7 +43252,7 @@
     <mergeCell ref="B1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="B12:K9929">
-    <cfRule type="expression" dxfId="23" priority="1">
+    <cfRule type="expression" dxfId="24" priority="1">
       <formula>AND($B12&lt;&gt;"",$C12&lt;&gt;"",$G12="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -43361,11 +43404,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="173" t="s">
+      <c r="C11" s="175" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="173"/>
-      <c r="E11" s="173"/>
+      <c r="D11" s="175"/>
+      <c r="E11" s="175"/>
       <c r="F11" s="40" t="s">
         <v>29</v>
       </c>
@@ -44570,7 +44613,7 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B12:H9929">
-    <cfRule type="expression" dxfId="22" priority="9">
+    <cfRule type="expression" dxfId="23" priority="9">
       <formula>AND($B12&lt;&gt;"",$C12&lt;&gt;"",#REF!="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -44694,39 +44737,39 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:CE7">
-    <cfRule type="expression" dxfId="21" priority="12">
+    <cfRule type="expression" dxfId="22" priority="12">
       <formula>B5&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:CE201">
-    <cfRule type="expression" dxfId="20" priority="1">
+    <cfRule type="expression" dxfId="21" priority="1">
       <formula>AND(G8&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="2">
+    <cfRule type="expression" dxfId="20" priority="2">
       <formula>AND(G$7&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="3">
+    <cfRule type="expression" dxfId="19" priority="3">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="4">
+    <cfRule type="expression" dxfId="18" priority="4">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="5">
+    <cfRule type="expression" dxfId="17" priority="5">
       <formula>AND(G8&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="6">
+    <cfRule type="expression" dxfId="16" priority="6">
       <formula>AND(G$7&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="7">
+    <cfRule type="expression" dxfId="15" priority="7">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="8">
+    <cfRule type="expression" dxfId="14" priority="8">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="10">
+    <cfRule type="expression" dxfId="12" priority="10">
       <formula>AND(G$7&lt;&gt;"",$B8="DEVIASI")</formula>
     </cfRule>
     <cfRule type="colorScale" priority="11">

</xml_diff>

<commit_message>
fix: rekap rab column shift, print area A:J, and signature alignment
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F864DAC-065E-4BD1-A3CE-EBEEAD507F97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3F885D-DAB2-4E62-B5B9-F4768715BD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cover" sheetId="21" r:id="rId1"/>
@@ -37,7 +37,6 @@
     <definedName name="_1__123Graph_ACHART_1" hidden="1">[2]RAB!#REF!</definedName>
     <definedName name="_2__123Graph_XCHART_1" hidden="1">[3]RAB!#REF!</definedName>
     <definedName name="_Fill" hidden="1">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="12">'laporan harian'!$A$1:$N$71</definedName>
     <definedName name="RAB" hidden="1">[4]RAB!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -58,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="103">
   <si>
     <t>HARGA SATUAN BAHAN, ALAT DAN UPAH</t>
   </si>
@@ -154,132 +153,6 @@
   </si>
   <si>
     <t>JUMLAH HARGA TKDN (Rp)</t>
-  </si>
-  <si>
-    <t>Papan Nama Kegiatan</t>
-  </si>
-  <si>
-    <t>PEKERJAAN PERLENGKAPAN K3</t>
-  </si>
-  <si>
-    <t>Pengadaan Spanduk K3</t>
-  </si>
-  <si>
-    <t>Pengadaan Helm Safety</t>
-  </si>
-  <si>
-    <t>Pengadaan Rompi Safety</t>
-  </si>
-  <si>
-    <t>Pengadaan Sepatu Boots</t>
-  </si>
-  <si>
-    <t>PEKERJAAN TANKI SEPTIK INDIVIDUAL</t>
-  </si>
-  <si>
-    <t>Penggalian 1 m3 tanah biasa sedalam &gt; 1 s.d. 2 m untuk volume &gt; 200 m3 secara manual</t>
-  </si>
-  <si>
-    <t>1 m3 urukan pasir uruk untuk volume &gt; 200 m3 tanpa pemadatan secara manual</t>
-  </si>
-  <si>
-    <t>1 m3 beton mutu rendah f'c 17 MPa, slump (100 ± 25) mm, agregat maks 19 mm secara manual</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m2 dinding bata merah tebal 1/2 batu dengan mortar tipe O,fc’ 2,4 MPa (Setara Campuran 1SP : 5PP)</t>
-  </si>
-  <si>
-    <t>Tanki Septic Prabrikasi</t>
-  </si>
-  <si>
-    <t>PEKERJAAN JARINGAN PIPA</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m pipa PVC D, DN. 4" (100 mm)</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m' pipa PVC AW, DN. 1" (25 mm) + Isolasi</t>
-  </si>
-  <si>
-    <t>1 m3 urukan kembali galian tanah ( &gt;0 s.d 200 m3) tanpa pemadatan secara manual</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m Pipa PVC, DN. 2" (50 mm)</t>
-  </si>
-  <si>
-    <t>Aksesoris Pipa PVC</t>
-  </si>
-  <si>
-    <t>PEKERJAAN RESAPAN</t>
-  </si>
-  <si>
-    <t>Urukan Batu</t>
-  </si>
-  <si>
-    <t>1m3 Urukan Batu Kerikil Tanpa Pemadatan secara manual</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m2 Lapisan Ijuk tebal 10 cm</t>
-  </si>
-  <si>
-    <t>1 m3 urukan tanah biasa atau tanah liat berpasir tanpa pemadatan secara manual</t>
-  </si>
-  <si>
-    <t>PEKERJAAN PEMBUATAN BILIK WC</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m3 batu kosong (anstamping) untuk pondasi gedung</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m3 pondasi batu belah mortar tipe O 2,4 Mpa (setara 1SP : 5PP), cara manual</t>
-  </si>
-  <si>
-    <t>1 m3 beton mutu rendah f'c 17 MPa, slump (100 ± 25) mm, agregat maks 19 mm secara semi mekanis</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 buah closet jongkok</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 buah floor drain stainless steel</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m2 dinding bata merah tebal 1 batu dengan mortar tipe S,fc’ 12,5 MPa (Setara Campuran 1SP : 3PP)</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m2 plesteran 1SP : 3PP tebal 15 mm</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m2 acian</t>
-  </si>
-  <si>
-    <t>Pengecatan 1 m2 tembok baru Interior( 1 lapis cat dasar, 2 lapis cat penutup)</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m2 plafon serat semen/GRC tebal 4 mm, 5 mm, dan 6 mm</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m3 konstruksi gordeng, kayu kelas II</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m2 atap seng gelombang 105x180 cm</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m2 lantai keramik uk. 20x20 cm (1SP : 2PP) Unpolished</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 buah engsel pintu</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 buah grendel</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 buah kran diameter ½"</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m' pipa PVC AW, DN. 1/2" (15 mm) + Isolasi</t>
-  </si>
-  <si>
-    <t>Pemasangan 1 m2 rangka dinding pemisah 60x120 cm kayu kelas II atau III</t>
   </si>
   <si>
     <t>Rekap RAB</t>
@@ -493,21 +366,6 @@
   </si>
   <si>
     <t>LAPORAN BULANAN</t>
-  </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>PEKERJAAN PERSIAPAN</t>
-  </si>
-  <si>
-    <t>1.1.1.1</t>
-  </si>
-  <si>
-    <t>Pembuatan 1 m’ pagar sementara dari kayu tinggi 2 meter</t>
-  </si>
-  <si>
-    <t>m'</t>
   </si>
 </sst>
 </file>
@@ -2625,131 +2483,7 @@
     <cellStyle name="Normal 2 2 3" xfId="2" xr:uid="{25DAB206-4C06-437D-BFFA-FD21FFA5A242}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="31">
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color rgb="FFFFC000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor theme="7" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color rgb="FFFFC000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor theme="7" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="29">
     <dxf>
       <font>
         <b/>
@@ -2906,24 +2640,64 @@
     <dxf>
       <font>
         <b/>
-        <i val="0"/>
+        <i/>
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
+          <fgColor theme="0"/>
+          <bgColor theme="0"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b/>
-        <i val="0"/>
+        <i/>
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
+          <fgColor theme="0"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color rgb="FFFFC000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor theme="7" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <fill>
@@ -2984,6 +2758,68 @@
           <bgColor theme="7" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color rgb="FFFFC000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor theme="7" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4044,7 +3880,7 @@
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" thickTop="1">
       <c r="B2" s="185" t="s">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="C2" s="186"/>
       <c r="D2" s="186"/>
@@ -4088,7 +3924,7 @@
     </row>
     <row r="5" spans="1:14" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="C5" s="80"/>
       <c r="D5" s="85" t="s">
@@ -4106,7 +3942,7 @@
     </row>
     <row r="6" spans="1:14" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
-        <v>88</v>
+        <v>46</v>
       </c>
       <c r="C6" s="80"/>
       <c r="D6" s="85" t="s">
@@ -4124,7 +3960,7 @@
     </row>
     <row r="7" spans="1:14" ht="15.6">
       <c r="B7" s="79" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="C7" s="80"/>
       <c r="D7" s="85" t="s">
@@ -4136,7 +3972,7 @@
       <c r="H7" s="80"/>
       <c r="I7" s="83"/>
       <c r="J7" s="84" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
       <c r="K7" s="85" t="s">
         <v>20</v>
@@ -4146,7 +3982,7 @@
     </row>
     <row r="8" spans="1:14" ht="15.6">
       <c r="B8" s="79" t="s">
-        <v>91</v>
+        <v>49</v>
       </c>
       <c r="C8" s="80"/>
       <c r="D8" s="85" t="s">
@@ -4158,7 +3994,7 @@
       <c r="H8" s="80"/>
       <c r="I8" s="80"/>
       <c r="J8" s="84" t="s">
-        <v>92</v>
+        <v>50</v>
       </c>
       <c r="K8" s="85" t="s">
         <v>20</v>
@@ -4176,7 +4012,7 @@
       <c r="H9" s="80"/>
       <c r="I9" s="80"/>
       <c r="J9" s="88" t="s">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="K9" s="85" t="s">
         <v>20</v>
@@ -4186,20 +4022,20 @@
     </row>
     <row r="10" spans="1:14" ht="15.6">
       <c r="B10" s="200" t="s">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="C10" s="201"/>
       <c r="D10" s="201"/>
       <c r="E10" s="201"/>
       <c r="F10" s="201"/>
       <c r="G10" s="201" t="s">
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="H10" s="201"/>
       <c r="I10" s="201"/>
       <c r="J10" s="202"/>
       <c r="K10" s="203" t="s">
-        <v>96</v>
+        <v>54</v>
       </c>
       <c r="L10" s="201"/>
       <c r="M10" s="204"/>
@@ -4210,15 +4046,15 @@
         <v>6</v>
       </c>
       <c r="C11" s="210" t="s">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="D11" s="232"/>
       <c r="E11" s="232"/>
       <c r="F11" s="92" t="s">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="G11" s="210" t="s">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="H11" s="211"/>
       <c r="I11" s="93" t="s">
@@ -4228,20 +4064,20 @@
         <v>26</v>
       </c>
       <c r="K11" s="210" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="L11" s="211"/>
       <c r="M11" s="94" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="N11" s="58"/>
     </row>
     <row r="12" spans="1:14" ht="16.2" thickTop="1">
       <c r="B12" s="95" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="C12" s="96" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="D12" s="97"/>
       <c r="E12" s="97"/>
@@ -4259,7 +4095,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="105" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="D13" s="106"/>
       <c r="E13" s="106"/>
@@ -4277,7 +4113,7 @@
         <v>2</v>
       </c>
       <c r="C14" s="105" t="s">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="D14" s="106"/>
       <c r="E14" s="106"/>
@@ -4295,7 +4131,7 @@
         <v>3</v>
       </c>
       <c r="C15" s="105" t="s">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="D15" s="106"/>
       <c r="E15" s="106"/>
@@ -4313,7 +4149,7 @@
         <v>4</v>
       </c>
       <c r="C16" s="105" t="s">
-        <v>108</v>
+        <v>66</v>
       </c>
       <c r="D16" s="106"/>
       <c r="E16" s="106"/>
@@ -4331,7 +4167,7 @@
         <v>5</v>
       </c>
       <c r="C17" s="105" t="s">
-        <v>109</v>
+        <v>67</v>
       </c>
       <c r="D17" s="106"/>
       <c r="E17" s="106"/>
@@ -4349,7 +4185,7 @@
         <v>6</v>
       </c>
       <c r="C18" s="105" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
       <c r="D18" s="106"/>
       <c r="E18" s="106"/>
@@ -4364,10 +4200,10 @@
     </row>
     <row r="19" spans="1:13" ht="15.6">
       <c r="B19" s="116" t="s">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="C19" s="117" t="s">
-        <v>112</v>
+        <v>70</v>
       </c>
       <c r="D19" s="118"/>
       <c r="E19" s="118"/>
@@ -4385,7 +4221,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="105" t="s">
-        <v>113</v>
+        <v>71</v>
       </c>
       <c r="D20" s="106"/>
       <c r="E20" s="106"/>
@@ -4403,7 +4239,7 @@
         <v>2</v>
       </c>
       <c r="C21" s="105" t="s">
-        <v>114</v>
+        <v>72</v>
       </c>
       <c r="D21" s="106"/>
       <c r="E21" s="106"/>
@@ -4421,7 +4257,7 @@
         <v>3</v>
       </c>
       <c r="C22" s="105" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="D22" s="106"/>
       <c r="E22" s="106"/>
@@ -4450,13 +4286,13 @@
     </row>
     <row r="24" spans="1:13" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="152" t="s">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="B24" s="237" t="s">
         <v>6</v>
       </c>
       <c r="C24" s="205" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="D24" s="205"/>
       <c r="E24" s="205"/>
@@ -4465,7 +4301,7 @@
       <c r="H24" s="205"/>
       <c r="I24" s="205"/>
       <c r="J24" s="207" t="s">
-        <v>117</v>
+        <v>75</v>
       </c>
       <c r="K24" s="208"/>
       <c r="L24" s="208"/>
@@ -4484,19 +4320,19 @@
         <v>9</v>
       </c>
       <c r="K25" s="221" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="L25" s="222"/>
       <c r="M25" s="126" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="15.6">
       <c r="B26" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C26" s="128" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D26" s="157"/>
       <c r="E26" s="129"/>
@@ -4505,22 +4341,22 @@
       <c r="H26" s="129"/>
       <c r="I26" s="130"/>
       <c r="J26" s="131" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K26" s="131"/>
       <c r="L26" s="159" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M26" s="132" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="15.6">
       <c r="B27" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C27" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D27" s="158"/>
       <c r="E27" s="134"/>
@@ -4529,22 +4365,22 @@
       <c r="H27" s="134"/>
       <c r="I27" s="135"/>
       <c r="J27" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K27" s="136"/>
       <c r="L27" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M27" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="15.6">
       <c r="B28" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C28" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D28" s="158"/>
       <c r="E28" s="134"/>
@@ -4553,22 +4389,22 @@
       <c r="H28" s="134"/>
       <c r="I28" s="135"/>
       <c r="J28" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K28" s="136"/>
       <c r="L28" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M28" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="15.6">
       <c r="B29" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C29" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D29" s="158"/>
       <c r="E29" s="134"/>
@@ -4577,22 +4413,22 @@
       <c r="H29" s="134"/>
       <c r="I29" s="135"/>
       <c r="J29" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K29" s="136"/>
       <c r="L29" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M29" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="15.6">
       <c r="B30" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C30" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D30" s="158"/>
       <c r="E30" s="134"/>
@@ -4601,22 +4437,22 @@
       <c r="H30" s="134"/>
       <c r="I30" s="135"/>
       <c r="J30" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K30" s="136"/>
       <c r="L30" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M30" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="15.6">
       <c r="B31" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C31" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D31" s="158"/>
       <c r="E31" s="134"/>
@@ -4625,22 +4461,22 @@
       <c r="H31" s="134"/>
       <c r="I31" s="135"/>
       <c r="J31" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K31" s="136"/>
       <c r="L31" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M31" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="15.6">
       <c r="B32" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C32" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D32" s="158"/>
       <c r="E32" s="134"/>
@@ -4649,22 +4485,22 @@
       <c r="H32" s="134"/>
       <c r="I32" s="135"/>
       <c r="J32" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K32" s="136"/>
       <c r="L32" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M32" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="2:13" ht="15.6">
       <c r="B33" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C33" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D33" s="158"/>
       <c r="E33" s="134"/>
@@ -4673,22 +4509,22 @@
       <c r="H33" s="134"/>
       <c r="I33" s="135"/>
       <c r="J33" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K33" s="136"/>
       <c r="L33" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M33" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" spans="2:13" ht="15.6">
       <c r="B34" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C34" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D34" s="158"/>
       <c r="E34" s="134"/>
@@ -4697,22 +4533,22 @@
       <c r="H34" s="134"/>
       <c r="I34" s="135"/>
       <c r="J34" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K34" s="136"/>
       <c r="L34" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M34" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="2:13" ht="15.6">
       <c r="B35" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C35" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D35" s="158"/>
       <c r="E35" s="134"/>
@@ -4721,22 +4557,22 @@
       <c r="H35" s="134"/>
       <c r="I35" s="135"/>
       <c r="J35" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K35" s="136"/>
       <c r="L35" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M35" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36" spans="2:13" ht="15.6">
       <c r="B36" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C36" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D36" s="158"/>
       <c r="E36" s="134"/>
@@ -4745,22 +4581,22 @@
       <c r="H36" s="134"/>
       <c r="I36" s="135"/>
       <c r="J36" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K36" s="136"/>
       <c r="L36" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M36" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="2:13" ht="15.6">
       <c r="B37" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C37" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D37" s="158"/>
       <c r="E37" s="134"/>
@@ -4769,22 +4605,22 @@
       <c r="H37" s="134"/>
       <c r="I37" s="135"/>
       <c r="J37" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K37" s="136"/>
       <c r="L37" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M37" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="38" spans="2:13" ht="15.6">
       <c r="B38" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C38" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D38" s="158"/>
       <c r="E38" s="134"/>
@@ -4793,22 +4629,22 @@
       <c r="H38" s="134"/>
       <c r="I38" s="135"/>
       <c r="J38" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K38" s="136"/>
       <c r="L38" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M38" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39" spans="2:13" ht="15.6">
       <c r="B39" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C39" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D39" s="158"/>
       <c r="E39" s="134"/>
@@ -4817,22 +4653,22 @@
       <c r="H39" s="134"/>
       <c r="I39" s="135"/>
       <c r="J39" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K39" s="136"/>
       <c r="L39" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M39" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" spans="2:13" ht="15.6">
       <c r="B40" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C40" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D40" s="158"/>
       <c r="E40" s="134"/>
@@ -4841,22 +4677,22 @@
       <c r="H40" s="134"/>
       <c r="I40" s="135"/>
       <c r="J40" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K40" s="136"/>
       <c r="L40" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M40" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="41" spans="2:13" ht="15.6">
       <c r="B41" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C41" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D41" s="158"/>
       <c r="E41" s="134"/>
@@ -4865,22 +4701,22 @@
       <c r="H41" s="134"/>
       <c r="I41" s="135"/>
       <c r="J41" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K41" s="136"/>
       <c r="L41" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M41" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="42" spans="2:13" ht="15.6">
       <c r="B42" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C42" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D42" s="158"/>
       <c r="E42" s="134"/>
@@ -4889,22 +4725,22 @@
       <c r="H42" s="134"/>
       <c r="I42" s="135"/>
       <c r="J42" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K42" s="136"/>
       <c r="L42" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M42" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="43" spans="2:13" ht="15.6">
       <c r="B43" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C43" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D43" s="158"/>
       <c r="E43" s="134"/>
@@ -4913,22 +4749,22 @@
       <c r="H43" s="134"/>
       <c r="I43" s="135"/>
       <c r="J43" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K43" s="136"/>
       <c r="L43" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M43" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" spans="2:13" ht="15.6">
       <c r="B44" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C44" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D44" s="158"/>
       <c r="E44" s="134"/>
@@ -4937,22 +4773,22 @@
       <c r="H44" s="134"/>
       <c r="I44" s="135"/>
       <c r="J44" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K44" s="136"/>
       <c r="L44" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M44" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="45" spans="2:13" ht="15.6">
       <c r="B45" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C45" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D45" s="158"/>
       <c r="E45" s="134"/>
@@ -4961,22 +4797,22 @@
       <c r="H45" s="134"/>
       <c r="I45" s="135"/>
       <c r="J45" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K45" s="136"/>
       <c r="L45" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M45" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="46" spans="2:13" ht="15.6">
       <c r="B46" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C46" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D46" s="158"/>
       <c r="E46" s="134"/>
@@ -4985,22 +4821,22 @@
       <c r="H46" s="134"/>
       <c r="I46" s="135"/>
       <c r="J46" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K46" s="136"/>
       <c r="L46" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M46" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="47" spans="2:13" ht="15.6">
       <c r="B47" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C47" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D47" s="158"/>
       <c r="E47" s="134"/>
@@ -5009,22 +4845,22 @@
       <c r="H47" s="134"/>
       <c r="I47" s="135"/>
       <c r="J47" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K47" s="136"/>
       <c r="L47" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M47" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="48" spans="2:13" ht="16.2" thickBot="1">
       <c r="B48" s="127" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="C48" s="133" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="D48" s="158"/>
       <c r="E48" s="134"/>
@@ -5033,19 +4869,19 @@
       <c r="H48" s="134"/>
       <c r="I48" s="135"/>
       <c r="J48" s="136" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="K48" s="136"/>
       <c r="L48" s="160" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M48" s="137" t="s">
-        <v>106</v>
+        <v>64</v>
       </c>
     </row>
     <row r="49" spans="2:13" ht="16.2" thickTop="1">
       <c r="B49" s="248" t="s">
-        <v>120</v>
+        <v>78</v>
       </c>
       <c r="C49" s="249"/>
       <c r="D49" s="249"/>
@@ -5056,7 +4892,7 @@
       <c r="I49" s="249"/>
       <c r="J49" s="250"/>
       <c r="K49" s="229" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="L49" s="230"/>
       <c r="M49" s="231"/>
@@ -5245,17 +5081,17 @@
     </row>
     <row r="63" spans="2:13" ht="15.6">
       <c r="B63" s="200" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="C63" s="201"/>
       <c r="D63" s="201"/>
       <c r="E63" s="202"/>
       <c r="F63" s="203" t="s">
-        <v>123</v>
+        <v>81</v>
       </c>
       <c r="G63" s="202"/>
       <c r="H63" s="203" t="s">
-        <v>124</v>
+        <v>82</v>
       </c>
       <c r="I63" s="201"/>
       <c r="J63" s="202"/>
@@ -5413,12 +5249,12 @@
     <mergeCell ref="K10:M10"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:I48">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>ISTEXT($C26)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J27:M48">
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5474,7 +5310,7 @@
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
       <c r="B2" s="176" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="C2" s="177"/>
       <c r="D2" s="177"/>
@@ -5517,7 +5353,7 @@
       <c r="G4"/>
       <c r="H4"/>
       <c r="I4" s="268" t="s">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="J4" s="268"/>
       <c r="K4" s="268"/>
@@ -5561,7 +5397,7 @@
       <c r="G6" s="56"/>
       <c r="H6" s="56"/>
       <c r="I6" s="56" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="J6" s="58"/>
       <c r="K6" s="56"/>
@@ -5584,7 +5420,7 @@
       <c r="G7" s="56"/>
       <c r="H7" s="56"/>
       <c r="I7" s="56" t="s">
-        <v>127</v>
+        <v>85</v>
       </c>
       <c r="J7" s="58"/>
       <c r="K7" s="56"/>
@@ -5607,7 +5443,7 @@
       <c r="G8" s="56"/>
       <c r="H8" s="56"/>
       <c r="I8" s="56" t="s">
-        <v>128</v>
+        <v>86</v>
       </c>
       <c r="J8" s="58"/>
       <c r="K8" s="56"/>
@@ -5630,7 +5466,7 @@
       <c r="G9" s="56"/>
       <c r="H9" s="56"/>
       <c r="I9" s="56" t="s">
-        <v>142</v>
+        <v>100</v>
       </c>
       <c r="J9" s="58"/>
       <c r="K9" s="56"/>
@@ -5653,7 +5489,7 @@
       <c r="G10" s="56"/>
       <c r="H10" s="56"/>
       <c r="I10" s="56" t="s">
-        <v>130</v>
+        <v>88</v>
       </c>
       <c r="J10" s="58"/>
       <c r="K10" s="56"/>
@@ -5685,24 +5521,24 @@
         <v>6</v>
       </c>
       <c r="C12" s="175" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="D12" s="175"/>
       <c r="E12" s="175"/>
       <c r="F12" s="175" t="s">
-        <v>131</v>
+        <v>89</v>
       </c>
       <c r="G12" s="175" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="H12" s="175" t="s">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="I12" s="175" t="s">
-        <v>134</v>
+        <v>92</v>
       </c>
       <c r="J12" s="175" t="s">
-        <v>138</v>
+        <v>96</v>
       </c>
       <c r="K12" s="175"/>
       <c r="L12" s="175"/>
@@ -5710,7 +5546,7 @@
       <c r="N12" s="175"/>
       <c r="O12" s="175"/>
       <c r="P12" s="267" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
@@ -5723,15 +5559,15 @@
       <c r="H13" s="175"/>
       <c r="I13" s="175"/>
       <c r="J13" s="266" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="K13" s="266"/>
       <c r="L13" s="266" t="s">
-        <v>140</v>
+        <v>98</v>
       </c>
       <c r="M13" s="266"/>
       <c r="N13" s="266" t="s">
-        <v>141</v>
+        <v>99</v>
       </c>
       <c r="O13" s="266"/>
       <c r="P13" s="267"/>
@@ -5746,22 +5582,22 @@
       <c r="H14" s="175"/>
       <c r="I14" s="175"/>
       <c r="J14" s="38" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="K14" s="39" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="L14" s="39" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="M14" s="39" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="N14" s="40" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="O14" s="40" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="P14" s="267"/>
     </row>
@@ -6113,7 +5949,7 @@
     <mergeCell ref="I4:P5"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P49">
-    <cfRule type="expression" dxfId="9" priority="13">
+    <cfRule type="expression" dxfId="1" priority="13">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6169,7 +6005,7 @@
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
       <c r="B2" s="176" t="s">
-        <v>144</v>
+        <v>102</v>
       </c>
       <c r="C2" s="177"/>
       <c r="D2" s="177"/>
@@ -6212,7 +6048,7 @@
       <c r="G4"/>
       <c r="H4"/>
       <c r="I4" s="268" t="s">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="J4" s="268"/>
       <c r="K4" s="268"/>
@@ -6256,7 +6092,7 @@
       <c r="G6" s="56"/>
       <c r="H6" s="56"/>
       <c r="I6" s="56" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="J6" s="58"/>
       <c r="K6" s="56"/>
@@ -6279,7 +6115,7 @@
       <c r="G7" s="56"/>
       <c r="H7" s="56"/>
       <c r="I7" s="56" t="s">
-        <v>127</v>
+        <v>85</v>
       </c>
       <c r="J7" s="58"/>
       <c r="K7" s="56"/>
@@ -6302,7 +6138,7 @@
       <c r="G8" s="56"/>
       <c r="H8" s="56"/>
       <c r="I8" s="56" t="s">
-        <v>128</v>
+        <v>86</v>
       </c>
       <c r="J8" s="58"/>
       <c r="K8" s="56"/>
@@ -6325,7 +6161,7 @@
       <c r="G9" s="56"/>
       <c r="H9" s="56"/>
       <c r="I9" s="56" t="s">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="J9" s="58"/>
       <c r="K9" s="56"/>
@@ -6348,7 +6184,7 @@
       <c r="G10" s="56"/>
       <c r="H10" s="56"/>
       <c r="I10" s="56" t="s">
-        <v>130</v>
+        <v>88</v>
       </c>
       <c r="J10" s="58"/>
       <c r="K10" s="56"/>
@@ -6380,24 +6216,24 @@
         <v>6</v>
       </c>
       <c r="C12" s="175" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="D12" s="175"/>
       <c r="E12" s="175"/>
       <c r="F12" s="175" t="s">
-        <v>131</v>
+        <v>89</v>
       </c>
       <c r="G12" s="175" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="H12" s="175" t="s">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="I12" s="175" t="s">
-        <v>134</v>
+        <v>92</v>
       </c>
       <c r="J12" s="175" t="s">
-        <v>138</v>
+        <v>96</v>
       </c>
       <c r="K12" s="175"/>
       <c r="L12" s="175"/>
@@ -6405,7 +6241,7 @@
       <c r="N12" s="175"/>
       <c r="O12" s="175"/>
       <c r="P12" s="267" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
@@ -6418,15 +6254,15 @@
       <c r="H13" s="175"/>
       <c r="I13" s="175"/>
       <c r="J13" s="266" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="K13" s="266"/>
       <c r="L13" s="266" t="s">
-        <v>136</v>
+        <v>94</v>
       </c>
       <c r="M13" s="266"/>
       <c r="N13" s="266" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
       <c r="O13" s="266"/>
       <c r="P13" s="267"/>
@@ -6441,22 +6277,22 @@
       <c r="H14" s="175"/>
       <c r="I14" s="175"/>
       <c r="J14" s="38" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="K14" s="39" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="L14" s="39" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="M14" s="39" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="N14" s="40" t="s">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="O14" s="40" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="P14" s="267"/>
     </row>
@@ -6854,7 +6690,7 @@
     <mergeCell ref="G12:G14"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P51">
-    <cfRule type="expression" dxfId="8" priority="14">
+    <cfRule type="expression" dxfId="0" priority="14">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6926,16 +6762,16 @@
       </c>
       <c r="D5" s="174"/>
       <c r="E5" s="11" t="s">
-        <v>80</v>
+        <v>38</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>9</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="I5" s="13" t="s">
         <v>3</v>
@@ -15278,7 +15114,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="30" priority="2">
+    <cfRule type="expression" dxfId="24" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17528,23 +17364,23 @@
     <mergeCell ref="B1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:N16997">
-    <cfRule type="expression" dxfId="29" priority="1">
+    <cfRule type="expression" dxfId="23" priority="1">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="2">
+    <cfRule type="expression" dxfId="22" priority="2">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="5">
+    <cfRule type="expression" dxfId="21" priority="5">
       <formula>AND($B6="",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H16997">
-    <cfRule type="expression" dxfId="26" priority="9">
+    <cfRule type="expression" dxfId="20" priority="9">
       <formula>IF(G6&lt;&gt;"", NOT(AND(OR(LEFT($E6,2)="L.", LEFT($E6,2)="A.", LEFT($E6,2)="B.", LEFT($E6,2)="M."), $H6&lt;&gt;"", $E6&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:K16997">
-    <cfRule type="notContainsBlanks" dxfId="25" priority="8">
+    <cfRule type="notContainsBlanks" dxfId="19" priority="8">
       <formula>LEN(TRIM(H6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17606,7 +17442,7 @@
     </row>
     <row r="5" spans="2:10" s="5" customFormat="1" ht="62.4" customHeight="1">
       <c r="B5" s="27" t="s">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="C5" s="27" t="s">
         <v>6</v>
@@ -17618,49 +17454,33 @@
         <v>26</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="G5" s="50" t="s">
         <v>3</v>
       </c>
       <c r="H5" s="28" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="J5" s="29"/>
     </row>
     <row r="6" spans="2:10">
-      <c r="B6" s="30" t="s">
-        <v>145</v>
-      </c>
+      <c r="B6" s="30"/>
       <c r="C6" s="31"/>
-      <c r="D6" s="30" t="s">
-        <v>146</v>
-      </c>
+      <c r="D6" s="30"/>
       <c r="E6" s="32"/>
       <c r="F6" s="33"/>
       <c r="G6" s="53"/>
       <c r="H6" s="33"/>
     </row>
     <row r="7" spans="2:10">
-      <c r="B7" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="C7" s="31">
-        <v>1</v>
-      </c>
-      <c r="D7" s="30" t="s">
-        <v>148</v>
-      </c>
+      <c r="B7" s="30"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="30"/>
       <c r="E7" s="32"/>
-      <c r="F7" s="33" t="s">
-        <v>149</v>
-      </c>
-      <c r="G7" s="53">
-        <v>580608</v>
-      </c>
-      <c r="H7" s="34">
-        <v>0.97428571428571431</v>
-      </c>
+      <c r="F7" s="33"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="34"/>
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="30"/>
@@ -41663,18 +41483,18 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B995 E6:H995">
-    <cfRule type="expression" dxfId="7" priority="7">
+    <cfRule type="expression" dxfId="18" priority="7">
       <formula>$J6=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:H995">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="17" priority="1">
       <formula>AND(LEN($B6)=1,$C6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="16" priority="2">
       <formula>AND($C6="",$B6&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="15" priority="3">
       <formula>AND($B6&lt;&gt;"",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -41688,7 +41508,7 @@
   <sheetPr codeName="Sheet4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q189"/>
+  <dimension ref="B1:K11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="1.21875" customWidth="1"/>
@@ -41853,7 +41673,7 @@
         <v>6</v>
       </c>
       <c r="C11" s="175" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="D11" s="175"/>
       <c r="E11" s="175"/>
@@ -41876,1386 +41696,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="2:11">
-      <c r="B12" s="22"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="64"/>
-      <c r="I12" s="64"/>
-      <c r="J12" s="65"/>
-      <c r="K12" s="64"/>
-    </row>
-    <row r="13" spans="2:11">
-      <c r="C13" s="66"/>
-      <c r="D13" s="66"/>
-      <c r="E13" s="66"/>
-    </row>
-    <row r="14" spans="2:11">
-      <c r="C14" s="59"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-    </row>
-    <row r="15" spans="2:11">
-      <c r="B15" s="22"/>
-      <c r="C15" s="69"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="70"/>
-      <c r="H15" s="64"/>
-      <c r="I15" s="64"/>
-      <c r="J15" s="65"/>
-      <c r="K15" s="64"/>
-    </row>
-    <row r="16" spans="2:11">
-      <c r="C16" s="59"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-    </row>
-    <row r="17" spans="2:11">
-      <c r="C17" s="59"/>
-      <c r="D17" s="66"/>
-      <c r="E17" s="66"/>
-    </row>
-    <row r="18" spans="2:11">
-      <c r="C18"/>
-      <c r="D18"/>
-      <c r="E18"/>
-    </row>
-    <row r="19" spans="2:11">
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19"/>
-    </row>
-    <row r="20" spans="2:11">
-      <c r="C20" s="59"/>
-      <c r="D20" s="66"/>
-      <c r="E20" s="66"/>
-    </row>
-    <row r="21" spans="2:11">
-      <c r="B21" s="22"/>
-      <c r="C21" s="69"/>
-      <c r="D21" s="63"/>
-      <c r="E21" s="63"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="70"/>
-      <c r="H21" s="64"/>
-      <c r="I21" s="64"/>
-      <c r="J21" s="65"/>
-      <c r="K21" s="64"/>
-    </row>
-    <row r="22" spans="2:11">
-      <c r="C22" s="59"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
-    </row>
-    <row r="23" spans="2:11">
-      <c r="C23" s="59"/>
-      <c r="D23" s="66"/>
-      <c r="E23" s="66"/>
-    </row>
-    <row r="24" spans="2:11">
-      <c r="C24" s="59"/>
-      <c r="D24" s="66"/>
-      <c r="E24" s="66"/>
-    </row>
-    <row r="25" spans="2:11">
-      <c r="C25" s="59"/>
-      <c r="D25" s="66"/>
-      <c r="E25" s="66"/>
-    </row>
-    <row r="26" spans="2:11">
-      <c r="C26" s="59"/>
-      <c r="D26" s="66"/>
-      <c r="E26" s="66"/>
-    </row>
-    <row r="27" spans="2:11">
-      <c r="C27" s="59"/>
-      <c r="D27" s="66"/>
-      <c r="E27" s="66"/>
-    </row>
-    <row r="28" spans="2:11">
-      <c r="C28" s="59"/>
-      <c r="D28" s="66"/>
-      <c r="E28" s="66"/>
-    </row>
-    <row r="29" spans="2:11">
-      <c r="C29" s="59"/>
-      <c r="D29" s="66"/>
-      <c r="E29" s="66"/>
-    </row>
-    <row r="30" spans="2:11">
-      <c r="C30" s="59"/>
-      <c r="D30" s="66"/>
-      <c r="E30" s="66"/>
-    </row>
-    <row r="31" spans="2:11">
-      <c r="C31" s="59"/>
-      <c r="D31" s="66"/>
-      <c r="E31" s="66"/>
-    </row>
-    <row r="32" spans="2:11">
-      <c r="B32" s="22"/>
-      <c r="C32" s="69"/>
-      <c r="D32" s="63"/>
-      <c r="E32" s="63"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="70"/>
-      <c r="H32" s="64"/>
-      <c r="I32" s="64"/>
-      <c r="J32" s="65"/>
-      <c r="K32" s="64"/>
-    </row>
-    <row r="33" spans="2:11">
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-    </row>
-    <row r="34" spans="2:11">
-      <c r="C34"/>
-      <c r="D34"/>
-      <c r="E34"/>
-    </row>
-    <row r="35" spans="2:11">
-      <c r="C35"/>
-      <c r="D35"/>
-      <c r="E35"/>
-    </row>
-    <row r="36" spans="2:11">
-      <c r="C36"/>
-      <c r="D36"/>
-      <c r="E36"/>
-    </row>
-    <row r="37" spans="2:11">
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-    </row>
-    <row r="38" spans="2:11">
-      <c r="C38"/>
-      <c r="D38"/>
-      <c r="E38"/>
-      <c r="F38" s="61"/>
-    </row>
-    <row r="39" spans="2:11">
-      <c r="C39" s="59"/>
-      <c r="D39" s="66"/>
-      <c r="E39" s="66"/>
-    </row>
-    <row r="40" spans="2:11">
-      <c r="B40" s="22"/>
-      <c r="C40" s="69"/>
-      <c r="D40" s="63"/>
-      <c r="E40" s="63"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="70"/>
-      <c r="H40" s="64"/>
-      <c r="I40" s="64"/>
-      <c r="J40" s="65"/>
-      <c r="K40" s="64"/>
-    </row>
-    <row r="41" spans="2:11">
-      <c r="C41"/>
-      <c r="D41"/>
-      <c r="E41"/>
-    </row>
-    <row r="42" spans="2:11">
-      <c r="C42"/>
-      <c r="D42"/>
-      <c r="E42"/>
-    </row>
-    <row r="43" spans="2:11">
-      <c r="C43"/>
-      <c r="D43"/>
-      <c r="E43"/>
-    </row>
-    <row r="44" spans="2:11">
-      <c r="C44"/>
-      <c r="D44"/>
-      <c r="E44"/>
-    </row>
-    <row r="45" spans="2:11">
-      <c r="C45"/>
-      <c r="D45"/>
-      <c r="E45"/>
-      <c r="H45" s="71"/>
-      <c r="I45" s="71"/>
-    </row>
-    <row r="46" spans="2:11">
-      <c r="C46"/>
-      <c r="D46"/>
-      <c r="E46"/>
-    </row>
-    <row r="47" spans="2:11">
-      <c r="C47" s="59"/>
-      <c r="D47" s="66"/>
-      <c r="E47" s="66"/>
-    </row>
-    <row r="48" spans="2:11">
-      <c r="B48" s="22"/>
-      <c r="C48" s="69"/>
-      <c r="D48" s="63"/>
-      <c r="E48" s="63"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="70"/>
-      <c r="H48" s="64"/>
-      <c r="I48" s="64"/>
-      <c r="J48" s="65"/>
-      <c r="K48" s="64"/>
-    </row>
-    <row r="49" spans="3:5">
-      <c r="C49" s="59"/>
-      <c r="D49" s="59"/>
-      <c r="E49" s="59"/>
-    </row>
-    <row r="50" spans="3:5">
-      <c r="C50" s="59"/>
-      <c r="D50" s="59"/>
-      <c r="E50" s="59"/>
-    </row>
-    <row r="51" spans="3:5">
-      <c r="C51" s="59"/>
-      <c r="D51" s="59"/>
-      <c r="E51" s="59"/>
-    </row>
-    <row r="52" spans="3:5">
-      <c r="C52" s="59"/>
-      <c r="D52" s="59"/>
-      <c r="E52" s="59"/>
-    </row>
-    <row r="53" spans="3:5">
-      <c r="C53" s="59"/>
-      <c r="D53" s="59"/>
-      <c r="E53" s="59"/>
-    </row>
-    <row r="54" spans="3:5">
-      <c r="C54" s="59"/>
-      <c r="D54" s="59"/>
-      <c r="E54" s="59"/>
-    </row>
-    <row r="55" spans="3:5">
-      <c r="C55" s="59"/>
-      <c r="D55" s="59"/>
-      <c r="E55" s="59"/>
-    </row>
-    <row r="56" spans="3:5">
-      <c r="C56" s="59"/>
-      <c r="D56" s="59"/>
-      <c r="E56" s="59"/>
-    </row>
-    <row r="57" spans="3:5">
-      <c r="C57" s="59"/>
-      <c r="D57" s="59"/>
-      <c r="E57" s="59"/>
-    </row>
-    <row r="58" spans="3:5">
-      <c r="C58" s="59"/>
-      <c r="D58" s="59"/>
-      <c r="E58" s="59"/>
-    </row>
-    <row r="59" spans="3:5">
-      <c r="C59" s="59"/>
-      <c r="D59" s="59"/>
-      <c r="E59" s="59"/>
-    </row>
-    <row r="60" spans="3:5">
-      <c r="C60" s="59"/>
-      <c r="D60" s="59"/>
-      <c r="E60" s="59"/>
-    </row>
-    <row r="61" spans="3:5">
-      <c r="C61" s="59"/>
-      <c r="D61" s="59"/>
-      <c r="E61" s="59"/>
-    </row>
-    <row r="62" spans="3:5">
-      <c r="C62" s="59"/>
-      <c r="D62" s="59"/>
-      <c r="E62" s="59"/>
-    </row>
-    <row r="63" spans="3:5">
-      <c r="C63" s="59"/>
-      <c r="D63" s="59"/>
-      <c r="E63" s="59"/>
-    </row>
-    <row r="64" spans="3:5">
-      <c r="C64" s="59"/>
-      <c r="D64" s="59"/>
-      <c r="E64" s="59"/>
-    </row>
-    <row r="65" spans="3:5">
-      <c r="C65" s="59"/>
-      <c r="D65" s="59"/>
-      <c r="E65" s="59"/>
-    </row>
-    <row r="66" spans="3:5">
-      <c r="C66" s="59"/>
-      <c r="D66" s="59"/>
-      <c r="E66" s="59"/>
-    </row>
-    <row r="67" spans="3:5">
-      <c r="C67" s="59"/>
-      <c r="D67" s="59"/>
-      <c r="E67" s="59"/>
-    </row>
-    <row r="68" spans="3:5">
-      <c r="C68" s="59"/>
-      <c r="D68" s="59"/>
-      <c r="E68" s="59"/>
-    </row>
-    <row r="69" spans="3:5">
-      <c r="C69" s="59"/>
-      <c r="D69" s="59"/>
-      <c r="E69" s="59"/>
-    </row>
-    <row r="70" spans="3:5">
-      <c r="C70" s="59"/>
-      <c r="D70" s="59"/>
-      <c r="E70" s="59"/>
-    </row>
-    <row r="71" spans="3:5">
-      <c r="C71" s="66"/>
-      <c r="D71" s="66"/>
-      <c r="E71" s="66"/>
-    </row>
-    <row r="136" spans="1:17" s="56" customFormat="1">
-      <c r="A136"/>
-      <c r="C136" t="s">
-        <v>32</v>
-      </c>
-      <c r="E136" s="57"/>
-      <c r="F136" s="58"/>
-      <c r="G136" s="67"/>
-      <c r="H136" s="68"/>
-      <c r="I136" s="68"/>
-      <c r="J136" s="60"/>
-      <c r="K136" s="68"/>
-      <c r="L136"/>
-      <c r="M136"/>
-      <c r="N136"/>
-      <c r="O136"/>
-      <c r="P136"/>
-      <c r="Q136"/>
-    </row>
-    <row r="137" spans="1:17" s="56" customFormat="1">
-      <c r="A137"/>
-      <c r="C137" t="s">
-        <v>33</v>
-      </c>
-      <c r="E137" s="57"/>
-      <c r="F137" s="58"/>
-      <c r="G137" s="67"/>
-      <c r="H137" s="68"/>
-      <c r="I137" s="68"/>
-      <c r="J137" s="60"/>
-      <c r="K137" s="68"/>
-      <c r="L137"/>
-      <c r="M137"/>
-      <c r="N137"/>
-      <c r="O137"/>
-      <c r="P137"/>
-      <c r="Q137"/>
-    </row>
-    <row r="138" spans="1:17" s="56" customFormat="1">
-      <c r="A138"/>
-      <c r="C138" t="s">
-        <v>34</v>
-      </c>
-      <c r="E138" s="57"/>
-      <c r="F138" s="58"/>
-      <c r="G138" s="67"/>
-      <c r="H138" s="68"/>
-      <c r="I138" s="68"/>
-      <c r="J138" s="60"/>
-      <c r="K138" s="68"/>
-      <c r="L138"/>
-      <c r="M138"/>
-      <c r="N138"/>
-      <c r="O138"/>
-      <c r="P138"/>
-      <c r="Q138"/>
-    </row>
-    <row r="139" spans="1:17" s="56" customFormat="1">
-      <c r="A139"/>
-      <c r="C139" t="s">
-        <v>35</v>
-      </c>
-      <c r="E139" s="57"/>
-      <c r="F139" s="58"/>
-      <c r="G139" s="67"/>
-      <c r="H139" s="68"/>
-      <c r="I139" s="68"/>
-      <c r="J139" s="60"/>
-      <c r="K139" s="68"/>
-      <c r="L139"/>
-      <c r="M139"/>
-      <c r="N139"/>
-      <c r="O139"/>
-      <c r="P139"/>
-      <c r="Q139"/>
-    </row>
-    <row r="140" spans="1:17" s="56" customFormat="1">
-      <c r="A140"/>
-      <c r="C140" t="s">
-        <v>36</v>
-      </c>
-      <c r="E140" s="57"/>
-      <c r="F140" s="58"/>
-      <c r="G140" s="67"/>
-      <c r="H140" s="68"/>
-      <c r="I140" s="68"/>
-      <c r="J140" s="60"/>
-      <c r="K140" s="68"/>
-      <c r="L140"/>
-      <c r="M140"/>
-      <c r="N140"/>
-      <c r="O140"/>
-      <c r="P140"/>
-      <c r="Q140"/>
-    </row>
-    <row r="141" spans="1:17" s="56" customFormat="1">
-      <c r="A141"/>
-      <c r="C141" t="s">
-        <v>37</v>
-      </c>
-      <c r="E141" s="57"/>
-      <c r="F141" s="58"/>
-      <c r="G141" s="67"/>
-      <c r="H141" s="68"/>
-      <c r="I141" s="68"/>
-      <c r="J141" s="60"/>
-      <c r="K141" s="68"/>
-      <c r="L141"/>
-      <c r="M141"/>
-      <c r="N141"/>
-      <c r="O141"/>
-      <c r="P141"/>
-      <c r="Q141"/>
-    </row>
-    <row r="142" spans="1:17" s="56" customFormat="1">
-      <c r="A142"/>
-      <c r="C142" t="s">
-        <v>38</v>
-      </c>
-      <c r="E142" s="57"/>
-      <c r="F142" s="58"/>
-      <c r="G142" s="67"/>
-      <c r="H142" s="68"/>
-      <c r="I142" s="68"/>
-      <c r="J142" s="60"/>
-      <c r="K142" s="68"/>
-      <c r="L142"/>
-      <c r="M142"/>
-      <c r="N142"/>
-      <c r="O142"/>
-      <c r="P142"/>
-      <c r="Q142"/>
-    </row>
-    <row r="143" spans="1:17" s="56" customFormat="1">
-      <c r="A143"/>
-      <c r="C143" t="s">
-        <v>39</v>
-      </c>
-      <c r="E143" s="57"/>
-      <c r="F143" s="58"/>
-      <c r="G143" s="67"/>
-      <c r="H143" s="68"/>
-      <c r="I143" s="68"/>
-      <c r="J143" s="60"/>
-      <c r="K143" s="68"/>
-      <c r="L143"/>
-      <c r="M143"/>
-      <c r="N143"/>
-      <c r="O143"/>
-      <c r="P143"/>
-      <c r="Q143"/>
-    </row>
-    <row r="144" spans="1:17" s="56" customFormat="1">
-      <c r="A144"/>
-      <c r="C144" t="s">
-        <v>40</v>
-      </c>
-      <c r="E144" s="57"/>
-      <c r="F144" s="58"/>
-      <c r="G144" s="67"/>
-      <c r="H144" s="68"/>
-      <c r="I144" s="68"/>
-      <c r="J144" s="60"/>
-      <c r="K144" s="68"/>
-      <c r="L144"/>
-      <c r="M144"/>
-      <c r="N144"/>
-      <c r="O144"/>
-      <c r="P144"/>
-      <c r="Q144"/>
-    </row>
-    <row r="145" spans="1:17" s="56" customFormat="1">
-      <c r="A145"/>
-      <c r="C145" t="s">
-        <v>40</v>
-      </c>
-      <c r="E145" s="57"/>
-      <c r="F145" s="58"/>
-      <c r="G145" s="67"/>
-      <c r="H145" s="68"/>
-      <c r="I145" s="68"/>
-      <c r="J145" s="60"/>
-      <c r="K145" s="68"/>
-      <c r="L145"/>
-      <c r="M145"/>
-      <c r="N145"/>
-      <c r="O145"/>
-      <c r="P145"/>
-      <c r="Q145"/>
-    </row>
-    <row r="146" spans="1:17" s="56" customFormat="1">
-      <c r="A146"/>
-      <c r="C146" t="s">
-        <v>41</v>
-      </c>
-      <c r="E146" s="57"/>
-      <c r="F146" s="58"/>
-      <c r="G146" s="67"/>
-      <c r="H146" s="68"/>
-      <c r="I146" s="68"/>
-      <c r="J146" s="60"/>
-      <c r="K146" s="68"/>
-      <c r="L146"/>
-      <c r="M146"/>
-      <c r="N146"/>
-      <c r="O146"/>
-      <c r="P146"/>
-      <c r="Q146"/>
-    </row>
-    <row r="147" spans="1:17" s="56" customFormat="1">
-      <c r="A147"/>
-      <c r="C147" t="s">
-        <v>42</v>
-      </c>
-      <c r="E147" s="57"/>
-      <c r="F147" s="58"/>
-      <c r="G147" s="67"/>
-      <c r="H147" s="68"/>
-      <c r="I147" s="68"/>
-      <c r="J147" s="60"/>
-      <c r="K147" s="68"/>
-      <c r="L147"/>
-      <c r="M147"/>
-      <c r="N147"/>
-      <c r="O147"/>
-      <c r="P147"/>
-      <c r="Q147"/>
-    </row>
-    <row r="148" spans="1:17" s="56" customFormat="1">
-      <c r="A148"/>
-      <c r="C148" t="s">
-        <v>41</v>
-      </c>
-      <c r="E148" s="57"/>
-      <c r="F148" s="58"/>
-      <c r="G148" s="67"/>
-      <c r="H148" s="68"/>
-      <c r="I148" s="68"/>
-      <c r="J148" s="60"/>
-      <c r="K148" s="68"/>
-      <c r="L148"/>
-      <c r="M148"/>
-      <c r="N148"/>
-      <c r="O148"/>
-      <c r="P148"/>
-      <c r="Q148"/>
-    </row>
-    <row r="149" spans="1:17" s="56" customFormat="1">
-      <c r="A149"/>
-      <c r="C149" t="s">
-        <v>41</v>
-      </c>
-      <c r="E149" s="57"/>
-      <c r="F149" s="58"/>
-      <c r="G149" s="67"/>
-      <c r="H149" s="68"/>
-      <c r="I149" s="68"/>
-      <c r="J149" s="60"/>
-      <c r="K149" s="68"/>
-      <c r="L149"/>
-      <c r="M149"/>
-      <c r="N149"/>
-      <c r="O149"/>
-      <c r="P149"/>
-      <c r="Q149"/>
-    </row>
-    <row r="150" spans="1:17" s="56" customFormat="1">
-      <c r="A150"/>
-      <c r="C150" t="s">
-        <v>41</v>
-      </c>
-      <c r="E150" s="57"/>
-      <c r="F150" s="58"/>
-      <c r="G150" s="67"/>
-      <c r="H150" s="68"/>
-      <c r="I150" s="68"/>
-      <c r="J150" s="60"/>
-      <c r="K150" s="68"/>
-      <c r="L150"/>
-      <c r="M150"/>
-      <c r="N150"/>
-      <c r="O150"/>
-      <c r="P150"/>
-      <c r="Q150"/>
-    </row>
-    <row r="151" spans="1:17" s="56" customFormat="1">
-      <c r="A151"/>
-      <c r="C151" t="s">
-        <v>43</v>
-      </c>
-      <c r="E151" s="57"/>
-      <c r="F151" s="58"/>
-      <c r="G151" s="67"/>
-      <c r="H151" s="68"/>
-      <c r="I151" s="68"/>
-      <c r="J151" s="60"/>
-      <c r="K151" s="68"/>
-      <c r="L151"/>
-      <c r="M151"/>
-      <c r="N151"/>
-      <c r="O151"/>
-      <c r="P151"/>
-      <c r="Q151"/>
-    </row>
-    <row r="152" spans="1:17" s="56" customFormat="1">
-      <c r="A152"/>
-      <c r="C152" t="s">
-        <v>44</v>
-      </c>
-      <c r="E152" s="57"/>
-      <c r="F152" s="58"/>
-      <c r="G152" s="67"/>
-      <c r="H152" s="68"/>
-      <c r="I152" s="68"/>
-      <c r="J152" s="60"/>
-      <c r="K152" s="68"/>
-      <c r="L152"/>
-      <c r="M152"/>
-      <c r="N152"/>
-      <c r="O152"/>
-      <c r="P152"/>
-      <c r="Q152"/>
-    </row>
-    <row r="153" spans="1:17" s="56" customFormat="1">
-      <c r="A153"/>
-      <c r="C153" t="s">
-        <v>39</v>
-      </c>
-      <c r="E153" s="57"/>
-      <c r="F153" s="58"/>
-      <c r="G153" s="67"/>
-      <c r="H153" s="68"/>
-      <c r="I153" s="68"/>
-      <c r="J153" s="60"/>
-      <c r="K153" s="68"/>
-      <c r="L153"/>
-      <c r="M153"/>
-      <c r="N153"/>
-      <c r="O153"/>
-      <c r="P153"/>
-      <c r="Q153"/>
-    </row>
-    <row r="154" spans="1:17" s="56" customFormat="1">
-      <c r="A154"/>
-      <c r="C154" t="s">
-        <v>45</v>
-      </c>
-      <c r="E154" s="57"/>
-      <c r="F154" s="58"/>
-      <c r="G154" s="67"/>
-      <c r="H154" s="68"/>
-      <c r="I154" s="68"/>
-      <c r="J154" s="60"/>
-      <c r="K154" s="68"/>
-      <c r="L154"/>
-      <c r="M154"/>
-      <c r="N154"/>
-      <c r="O154"/>
-      <c r="P154"/>
-      <c r="Q154"/>
-    </row>
-    <row r="155" spans="1:17" s="56" customFormat="1">
-      <c r="A155"/>
-      <c r="C155" t="s">
-        <v>46</v>
-      </c>
-      <c r="E155" s="57"/>
-      <c r="F155" s="58"/>
-      <c r="G155" s="67"/>
-      <c r="H155" s="68"/>
-      <c r="I155" s="68"/>
-      <c r="J155" s="60"/>
-      <c r="K155" s="68"/>
-      <c r="L155"/>
-      <c r="M155"/>
-      <c r="N155"/>
-      <c r="O155"/>
-      <c r="P155"/>
-      <c r="Q155"/>
-    </row>
-    <row r="156" spans="1:17" s="56" customFormat="1">
-      <c r="A156"/>
-      <c r="C156" t="s">
-        <v>47</v>
-      </c>
-      <c r="E156" s="57"/>
-      <c r="F156" s="58"/>
-      <c r="G156" s="67"/>
-      <c r="H156" s="68"/>
-      <c r="I156" s="68"/>
-      <c r="J156" s="60"/>
-      <c r="K156" s="68"/>
-      <c r="L156"/>
-      <c r="M156"/>
-      <c r="N156"/>
-      <c r="O156"/>
-      <c r="P156"/>
-      <c r="Q156"/>
-    </row>
-    <row r="157" spans="1:17" s="56" customFormat="1">
-      <c r="A157"/>
-      <c r="C157" t="s">
-        <v>48</v>
-      </c>
-      <c r="E157" s="57"/>
-      <c r="F157" s="58"/>
-      <c r="G157" s="67"/>
-      <c r="H157" s="68"/>
-      <c r="I157" s="68"/>
-      <c r="J157" s="60"/>
-      <c r="K157" s="68"/>
-      <c r="L157"/>
-      <c r="M157"/>
-      <c r="N157"/>
-      <c r="O157"/>
-      <c r="P157"/>
-      <c r="Q157"/>
-    </row>
-    <row r="158" spans="1:17" s="56" customFormat="1">
-      <c r="A158"/>
-      <c r="C158" t="s">
-        <v>49</v>
-      </c>
-      <c r="E158" s="57"/>
-      <c r="F158" s="58"/>
-      <c r="G158" s="67"/>
-      <c r="H158" s="68"/>
-      <c r="I158" s="68"/>
-      <c r="J158" s="60"/>
-      <c r="K158" s="68"/>
-      <c r="L158"/>
-      <c r="M158"/>
-      <c r="N158"/>
-      <c r="O158"/>
-      <c r="P158"/>
-      <c r="Q158"/>
-    </row>
-    <row r="159" spans="1:17" s="56" customFormat="1">
-      <c r="A159"/>
-      <c r="C159" t="s">
-        <v>50</v>
-      </c>
-      <c r="E159" s="57"/>
-      <c r="F159" s="58"/>
-      <c r="G159" s="67"/>
-      <c r="H159" s="68"/>
-      <c r="I159" s="68"/>
-      <c r="J159" s="60"/>
-      <c r="K159" s="68"/>
-      <c r="L159"/>
-      <c r="M159"/>
-      <c r="N159"/>
-      <c r="O159"/>
-      <c r="P159"/>
-      <c r="Q159"/>
-    </row>
-    <row r="160" spans="1:17" s="56" customFormat="1">
-      <c r="A160"/>
-      <c r="C160" t="s">
-        <v>39</v>
-      </c>
-      <c r="E160" s="57"/>
-      <c r="F160" s="58"/>
-      <c r="G160" s="67"/>
-      <c r="H160" s="68"/>
-      <c r="I160" s="68"/>
-      <c r="J160" s="60"/>
-      <c r="K160" s="68"/>
-      <c r="L160"/>
-      <c r="M160"/>
-      <c r="N160"/>
-      <c r="O160"/>
-      <c r="P160"/>
-      <c r="Q160"/>
-    </row>
-    <row r="161" spans="1:17" s="56" customFormat="1">
-      <c r="A161"/>
-      <c r="C161" t="s">
-        <v>40</v>
-      </c>
-      <c r="E161" s="57"/>
-      <c r="F161" s="58"/>
-      <c r="G161" s="67"/>
-      <c r="H161" s="68"/>
-      <c r="I161" s="68"/>
-      <c r="J161" s="60"/>
-      <c r="K161" s="68"/>
-      <c r="L161"/>
-      <c r="M161"/>
-      <c r="N161"/>
-      <c r="O161"/>
-      <c r="P161"/>
-      <c r="Q161"/>
-    </row>
-    <row r="162" spans="1:17" s="56" customFormat="1">
-      <c r="A162"/>
-      <c r="C162" t="s">
-        <v>51</v>
-      </c>
-      <c r="E162" s="57"/>
-      <c r="F162" s="58"/>
-      <c r="G162" s="67"/>
-      <c r="H162" s="68"/>
-      <c r="I162" s="68"/>
-      <c r="J162" s="60"/>
-      <c r="K162" s="68"/>
-      <c r="L162"/>
-      <c r="M162"/>
-      <c r="N162"/>
-      <c r="O162"/>
-      <c r="P162"/>
-      <c r="Q162"/>
-    </row>
-    <row r="163" spans="1:17" s="56" customFormat="1">
-      <c r="A163"/>
-      <c r="C163" t="s">
-        <v>52</v>
-      </c>
-      <c r="E163" s="57"/>
-      <c r="F163" s="58"/>
-      <c r="G163" s="67"/>
-      <c r="H163" s="68"/>
-      <c r="I163" s="68"/>
-      <c r="J163" s="60"/>
-      <c r="K163" s="68"/>
-      <c r="L163"/>
-      <c r="M163"/>
-      <c r="N163"/>
-      <c r="O163"/>
-      <c r="P163"/>
-      <c r="Q163"/>
-    </row>
-    <row r="164" spans="1:17" s="56" customFormat="1">
-      <c r="A164"/>
-      <c r="C164" t="s">
-        <v>53</v>
-      </c>
-      <c r="E164" s="57"/>
-      <c r="F164" s="58"/>
-      <c r="G164" s="67"/>
-      <c r="H164" s="68"/>
-      <c r="I164" s="68"/>
-      <c r="J164" s="60"/>
-      <c r="K164" s="68"/>
-      <c r="L164"/>
-      <c r="M164"/>
-      <c r="N164"/>
-      <c r="O164"/>
-      <c r="P164"/>
-      <c r="Q164"/>
-    </row>
-    <row r="165" spans="1:17" s="56" customFormat="1">
-      <c r="A165"/>
-      <c r="C165" t="s">
-        <v>54</v>
-      </c>
-      <c r="E165" s="57"/>
-      <c r="F165" s="58"/>
-      <c r="G165" s="67"/>
-      <c r="H165" s="68"/>
-      <c r="I165" s="68"/>
-      <c r="J165" s="60"/>
-      <c r="K165" s="68"/>
-      <c r="L165"/>
-      <c r="M165"/>
-      <c r="N165"/>
-      <c r="O165"/>
-      <c r="P165"/>
-      <c r="Q165"/>
-    </row>
-    <row r="166" spans="1:17" s="56" customFormat="1">
-      <c r="A166"/>
-      <c r="C166" t="s">
-        <v>55</v>
-      </c>
-      <c r="E166" s="57"/>
-      <c r="F166" s="58"/>
-      <c r="G166" s="67"/>
-      <c r="H166" s="68"/>
-      <c r="I166" s="68"/>
-      <c r="J166" s="60"/>
-      <c r="K166" s="68"/>
-      <c r="L166"/>
-      <c r="M166"/>
-      <c r="N166"/>
-      <c r="O166"/>
-      <c r="P166"/>
-      <c r="Q166"/>
-    </row>
-    <row r="167" spans="1:17" s="56" customFormat="1">
-      <c r="A167"/>
-      <c r="C167" t="s">
-        <v>39</v>
-      </c>
-      <c r="E167" s="57"/>
-      <c r="F167" s="58"/>
-      <c r="G167" s="67"/>
-      <c r="H167" s="68"/>
-      <c r="I167" s="68"/>
-      <c r="J167" s="60"/>
-      <c r="K167" s="68"/>
-      <c r="L167"/>
-      <c r="M167"/>
-      <c r="N167"/>
-      <c r="O167"/>
-      <c r="P167"/>
-      <c r="Q167"/>
-    </row>
-    <row r="168" spans="1:17" s="56" customFormat="1">
-      <c r="A168"/>
-      <c r="C168" t="s">
-        <v>40</v>
-      </c>
-      <c r="E168" s="57"/>
-      <c r="F168" s="58"/>
-      <c r="G168" s="67"/>
-      <c r="H168" s="68"/>
-      <c r="I168" s="68"/>
-      <c r="J168" s="60"/>
-      <c r="K168" s="68"/>
-      <c r="L168"/>
-      <c r="M168"/>
-      <c r="N168"/>
-      <c r="O168"/>
-      <c r="P168"/>
-      <c r="Q168"/>
-    </row>
-    <row r="169" spans="1:17" s="56" customFormat="1">
-      <c r="A169"/>
-      <c r="C169" t="s">
-        <v>56</v>
-      </c>
-      <c r="E169" s="57"/>
-      <c r="F169" s="58"/>
-      <c r="G169" s="67"/>
-      <c r="H169" s="68"/>
-      <c r="I169" s="68"/>
-      <c r="J169" s="60"/>
-      <c r="K169" s="68"/>
-      <c r="L169"/>
-      <c r="M169"/>
-      <c r="N169"/>
-      <c r="O169"/>
-      <c r="P169"/>
-      <c r="Q169"/>
-    </row>
-    <row r="170" spans="1:17" s="56" customFormat="1">
-      <c r="A170"/>
-      <c r="C170" t="s">
-        <v>57</v>
-      </c>
-      <c r="E170" s="57"/>
-      <c r="F170" s="58"/>
-      <c r="G170" s="67"/>
-      <c r="H170" s="68"/>
-      <c r="I170" s="68"/>
-      <c r="J170" s="60"/>
-      <c r="K170" s="68"/>
-      <c r="L170"/>
-      <c r="M170"/>
-      <c r="N170"/>
-      <c r="O170"/>
-      <c r="P170"/>
-      <c r="Q170"/>
-    </row>
-    <row r="171" spans="1:17" s="56" customFormat="1">
-      <c r="A171"/>
-      <c r="C171" t="s">
-        <v>40</v>
-      </c>
-      <c r="E171" s="57"/>
-      <c r="F171" s="58"/>
-      <c r="G171" s="67"/>
-      <c r="H171" s="68"/>
-      <c r="I171" s="68"/>
-      <c r="J171" s="60"/>
-      <c r="K171" s="68"/>
-      <c r="L171"/>
-      <c r="M171"/>
-      <c r="N171"/>
-      <c r="O171"/>
-      <c r="P171"/>
-      <c r="Q171"/>
-    </row>
-    <row r="172" spans="1:17" s="56" customFormat="1">
-      <c r="A172"/>
-      <c r="C172" t="s">
-        <v>54</v>
-      </c>
-      <c r="E172" s="57"/>
-      <c r="F172" s="58"/>
-      <c r="G172" s="67"/>
-      <c r="H172" s="68"/>
-      <c r="I172" s="68"/>
-      <c r="J172" s="60"/>
-      <c r="K172" s="68"/>
-      <c r="L172"/>
-      <c r="M172"/>
-      <c r="N172"/>
-      <c r="O172"/>
-      <c r="P172"/>
-      <c r="Q172"/>
-    </row>
-    <row r="173" spans="1:17" s="56" customFormat="1">
-      <c r="A173"/>
-      <c r="C173" t="s">
-        <v>58</v>
-      </c>
-      <c r="E173" s="57"/>
-      <c r="F173" s="58"/>
-      <c r="G173" s="67"/>
-      <c r="H173" s="68"/>
-      <c r="I173" s="68"/>
-      <c r="J173" s="60"/>
-      <c r="K173" s="68"/>
-      <c r="L173"/>
-      <c r="M173"/>
-      <c r="N173"/>
-      <c r="O173"/>
-      <c r="P173"/>
-      <c r="Q173"/>
-    </row>
-    <row r="174" spans="1:17" s="56" customFormat="1">
-      <c r="A174"/>
-      <c r="C174" t="s">
-        <v>59</v>
-      </c>
-      <c r="E174" s="57"/>
-      <c r="F174" s="58"/>
-      <c r="G174" s="67"/>
-      <c r="H174" s="68"/>
-      <c r="I174" s="68"/>
-      <c r="J174" s="60"/>
-      <c r="K174" s="68"/>
-      <c r="L174"/>
-      <c r="M174"/>
-      <c r="N174"/>
-      <c r="O174"/>
-      <c r="P174"/>
-      <c r="Q174"/>
-    </row>
-    <row r="175" spans="1:17" s="56" customFormat="1">
-      <c r="A175"/>
-      <c r="C175" t="s">
-        <v>60</v>
-      </c>
-      <c r="E175" s="57"/>
-      <c r="F175" s="58"/>
-      <c r="G175" s="67"/>
-      <c r="H175" s="68"/>
-      <c r="I175" s="68"/>
-      <c r="J175" s="60"/>
-      <c r="K175" s="68"/>
-      <c r="L175"/>
-      <c r="M175"/>
-      <c r="N175"/>
-      <c r="O175"/>
-      <c r="P175"/>
-      <c r="Q175"/>
-    </row>
-    <row r="176" spans="1:17" s="56" customFormat="1">
-      <c r="A176"/>
-      <c r="C176" t="s">
-        <v>61</v>
-      </c>
-      <c r="E176" s="57"/>
-      <c r="F176" s="58"/>
-      <c r="G176" s="67"/>
-      <c r="H176" s="68"/>
-      <c r="I176" s="68"/>
-      <c r="J176" s="60"/>
-      <c r="K176" s="68"/>
-      <c r="L176"/>
-      <c r="M176"/>
-      <c r="N176"/>
-      <c r="O176"/>
-      <c r="P176"/>
-      <c r="Q176"/>
-    </row>
-    <row r="177" spans="1:17" s="56" customFormat="1">
-      <c r="A177"/>
-      <c r="C177" t="s">
-        <v>62</v>
-      </c>
-      <c r="E177" s="57"/>
-      <c r="F177" s="58"/>
-      <c r="G177" s="67"/>
-      <c r="H177" s="68"/>
-      <c r="I177" s="68"/>
-      <c r="J177" s="60"/>
-      <c r="K177" s="68"/>
-      <c r="L177"/>
-      <c r="M177"/>
-      <c r="N177"/>
-      <c r="O177"/>
-      <c r="P177"/>
-      <c r="Q177"/>
-    </row>
-    <row r="178" spans="1:17" s="56" customFormat="1">
-      <c r="A178"/>
-      <c r="C178" t="s">
-        <v>63</v>
-      </c>
-      <c r="E178" s="57"/>
-      <c r="F178" s="58"/>
-      <c r="G178" s="67"/>
-      <c r="H178" s="68"/>
-      <c r="I178" s="68"/>
-      <c r="J178" s="60"/>
-      <c r="K178" s="68"/>
-      <c r="L178"/>
-      <c r="M178"/>
-      <c r="N178"/>
-      <c r="O178"/>
-      <c r="P178"/>
-      <c r="Q178"/>
-    </row>
-    <row r="179" spans="1:17" s="56" customFormat="1">
-      <c r="A179"/>
-      <c r="C179" t="s">
-        <v>64</v>
-      </c>
-      <c r="E179" s="57"/>
-      <c r="F179" s="58"/>
-      <c r="G179" s="67"/>
-      <c r="H179" s="68"/>
-      <c r="I179" s="68"/>
-      <c r="J179" s="60"/>
-      <c r="K179" s="68"/>
-      <c r="L179"/>
-      <c r="M179"/>
-      <c r="N179"/>
-      <c r="O179"/>
-      <c r="P179"/>
-      <c r="Q179"/>
-    </row>
-    <row r="180" spans="1:17" s="56" customFormat="1">
-      <c r="A180"/>
-      <c r="C180" t="s">
-        <v>65</v>
-      </c>
-      <c r="E180" s="57"/>
-      <c r="F180" s="58"/>
-      <c r="G180" s="67"/>
-      <c r="H180" s="68"/>
-      <c r="I180" s="68"/>
-      <c r="J180" s="60"/>
-      <c r="K180" s="68"/>
-      <c r="L180"/>
-      <c r="M180"/>
-      <c r="N180"/>
-      <c r="O180"/>
-      <c r="P180"/>
-      <c r="Q180"/>
-    </row>
-    <row r="181" spans="1:17" s="56" customFormat="1">
-      <c r="A181"/>
-      <c r="C181" t="s">
-        <v>66</v>
-      </c>
-      <c r="E181" s="57"/>
-      <c r="F181" s="58"/>
-      <c r="G181" s="67"/>
-      <c r="H181" s="68"/>
-      <c r="I181" s="68"/>
-      <c r="J181" s="60"/>
-      <c r="K181" s="68"/>
-      <c r="L181"/>
-      <c r="M181"/>
-      <c r="N181"/>
-      <c r="O181"/>
-      <c r="P181"/>
-      <c r="Q181"/>
-    </row>
-    <row r="182" spans="1:17" s="56" customFormat="1">
-      <c r="A182"/>
-      <c r="C182" t="s">
-        <v>67</v>
-      </c>
-      <c r="E182" s="57"/>
-      <c r="F182" s="58"/>
-      <c r="G182" s="67"/>
-      <c r="H182" s="68"/>
-      <c r="I182" s="68"/>
-      <c r="J182" s="60"/>
-      <c r="K182" s="68"/>
-      <c r="L182"/>
-      <c r="M182"/>
-      <c r="N182"/>
-      <c r="O182"/>
-      <c r="P182"/>
-      <c r="Q182"/>
-    </row>
-    <row r="183" spans="1:17" s="56" customFormat="1">
-      <c r="A183"/>
-      <c r="C183" t="s">
-        <v>68</v>
-      </c>
-      <c r="E183" s="57"/>
-      <c r="F183" s="58"/>
-      <c r="G183" s="67"/>
-      <c r="H183" s="68"/>
-      <c r="I183" s="68"/>
-      <c r="J183" s="60"/>
-      <c r="K183" s="68"/>
-      <c r="L183"/>
-      <c r="M183"/>
-      <c r="N183"/>
-      <c r="O183"/>
-      <c r="P183"/>
-      <c r="Q183"/>
-    </row>
-    <row r="184" spans="1:17" s="56" customFormat="1">
-      <c r="A184"/>
-      <c r="C184" t="s">
-        <v>69</v>
-      </c>
-      <c r="E184" s="57"/>
-      <c r="F184" s="58"/>
-      <c r="G184" s="67"/>
-      <c r="H184" s="68"/>
-      <c r="I184" s="68"/>
-      <c r="J184" s="60"/>
-      <c r="K184" s="68"/>
-      <c r="L184"/>
-      <c r="M184"/>
-      <c r="N184"/>
-      <c r="O184"/>
-      <c r="P184"/>
-      <c r="Q184"/>
-    </row>
-    <row r="185" spans="1:17" s="56" customFormat="1">
-      <c r="A185"/>
-      <c r="C185" t="s">
-        <v>70</v>
-      </c>
-      <c r="E185" s="57"/>
-      <c r="F185" s="58"/>
-      <c r="G185" s="67"/>
-      <c r="H185" s="68"/>
-      <c r="I185" s="68"/>
-      <c r="J185" s="60"/>
-      <c r="K185" s="68"/>
-      <c r="L185"/>
-      <c r="M185"/>
-      <c r="N185"/>
-      <c r="O185"/>
-      <c r="P185"/>
-      <c r="Q185"/>
-    </row>
-    <row r="186" spans="1:17" s="56" customFormat="1">
-      <c r="A186"/>
-      <c r="C186" t="s">
-        <v>71</v>
-      </c>
-      <c r="E186" s="57"/>
-      <c r="F186" s="58"/>
-      <c r="G186" s="67"/>
-      <c r="H186" s="68"/>
-      <c r="I186" s="68"/>
-      <c r="J186" s="60"/>
-      <c r="K186" s="68"/>
-      <c r="L186"/>
-      <c r="M186"/>
-      <c r="N186"/>
-      <c r="O186"/>
-      <c r="P186"/>
-      <c r="Q186"/>
-    </row>
-    <row r="187" spans="1:17" s="56" customFormat="1">
-      <c r="A187"/>
-      <c r="C187" t="s">
-        <v>72</v>
-      </c>
-      <c r="E187" s="57"/>
-      <c r="F187" s="58"/>
-      <c r="G187" s="67"/>
-      <c r="H187" s="68"/>
-      <c r="I187" s="68"/>
-      <c r="J187" s="60"/>
-      <c r="K187" s="68"/>
-      <c r="L187"/>
-      <c r="M187"/>
-      <c r="N187"/>
-      <c r="O187"/>
-      <c r="P187"/>
-      <c r="Q187"/>
-    </row>
-    <row r="188" spans="1:17" s="56" customFormat="1">
-      <c r="A188"/>
-      <c r="C188" t="s">
-        <v>73</v>
-      </c>
-      <c r="E188" s="57"/>
-      <c r="F188" s="58"/>
-      <c r="G188" s="67"/>
-      <c r="H188" s="68"/>
-      <c r="I188" s="68"/>
-      <c r="J188" s="60"/>
-      <c r="K188" s="68"/>
-      <c r="L188"/>
-      <c r="M188"/>
-      <c r="N188"/>
-      <c r="O188"/>
-      <c r="P188"/>
-      <c r="Q188"/>
-    </row>
-    <row r="189" spans="1:17" s="56" customFormat="1">
-      <c r="A189"/>
-      <c r="C189"/>
-      <c r="E189" s="57"/>
-      <c r="F189" s="58"/>
-      <c r="G189" s="67"/>
-      <c r="H189" s="68"/>
-      <c r="I189" s="68"/>
-      <c r="J189" s="60"/>
-      <c r="K189" s="68"/>
-      <c r="L189"/>
-      <c r="M189"/>
-      <c r="N189"/>
-      <c r="O189"/>
-      <c r="P189"/>
-      <c r="Q189"/>
-    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="B1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B12:K9929">
-    <cfRule type="expression" dxfId="24" priority="1">
-      <formula>AND($B12&lt;&gt;"",$C12&lt;&gt;"",$G12="")</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="72" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -43266,25 +41712,26 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N189"/>
+  <dimension ref="B1:I11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="1.21875" customWidth="1"/>
     <col min="2" max="2" width="3.77734375" style="56" customWidth="1"/>
     <col min="3" max="3" width="14" style="56" customWidth="1"/>
     <col min="4" max="4" width="1.44140625" style="56" customWidth="1"/>
-    <col min="5" max="5" width="64.77734375" style="57" customWidth="1"/>
-    <col min="6" max="6" width="19.21875" style="68" customWidth="1"/>
-    <col min="7" max="7" width="11.44140625" style="60" customWidth="1"/>
-    <col min="8" max="8" width="19.21875" style="68" customWidth="1"/>
-    <col min="9" max="9" width="1.21875" customWidth="1"/>
-    <col min="10" max="10" width="8.88671875" customWidth="1"/>
-    <col min="11" max="11" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.88671875" style="56" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" style="57" customWidth="1"/>
+    <col min="7" max="7" width="19.21875" style="68" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" style="60" customWidth="1"/>
+    <col min="9" max="9" width="19.21875" style="68" customWidth="1"/>
+    <col min="10" max="10" width="1.21875" customWidth="1"/>
+    <col min="11" max="11" width="8.88671875" customWidth="1"/>
+    <col min="12" max="12" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="111.6" customHeight="1">
+    <row r="1" spans="2:9" ht="111.6" customHeight="1">
       <c r="B1" s="178"/>
       <c r="C1" s="178"/>
       <c r="D1" s="178"/>
@@ -43292,10 +41739,11 @@
       <c r="F1" s="178"/>
       <c r="G1" s="178"/>
       <c r="H1" s="178"/>
-    </row>
-    <row r="2" spans="2:8" ht="22.95" customHeight="1">
+      <c r="I1" s="178"/>
+    </row>
+    <row r="2" spans="2:9" ht="22.95" customHeight="1">
       <c r="B2" s="176" t="s">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="C2" s="177"/>
       <c r="D2" s="177"/>
@@ -43303,8 +41751,9 @@
       <c r="F2" s="177"/>
       <c r="G2" s="177"/>
       <c r="H2" s="177"/>
-    </row>
-    <row r="3" spans="2:8" ht="4.95" customHeight="1">
+      <c r="I2" s="177"/>
+    </row>
+    <row r="3" spans="2:9" ht="4.95" customHeight="1">
       <c r="B3"/>
       <c r="C3"/>
       <c r="D3"/>
@@ -43312,8 +41761,9 @@
       <c r="F3"/>
       <c r="G3"/>
       <c r="H3"/>
-    </row>
-    <row r="4" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I3"/>
+    </row>
+    <row r="4" spans="2:9" ht="14.4" customHeight="1">
       <c r="B4" t="s">
         <v>19</v>
       </c>
@@ -43321,12 +41771,13 @@
       <c r="D4" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="56"/>
+      <c r="E4"/>
       <c r="F4" s="56"/>
       <c r="G4" s="56"/>
       <c r="H4" s="56"/>
-    </row>
-    <row r="5" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I4" s="56"/>
+    </row>
+    <row r="5" spans="2:9" ht="14.4" customHeight="1">
       <c r="B5" t="s">
         <v>21</v>
       </c>
@@ -43334,12 +41785,13 @@
       <c r="D5" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="56"/>
+      <c r="E5"/>
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-    </row>
-    <row r="6" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I5" s="56"/>
+    </row>
+    <row r="6" spans="2:9" ht="14.4" customHeight="1">
       <c r="B6" t="s">
         <v>22</v>
       </c>
@@ -43347,12 +41799,13 @@
       <c r="D6" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="56"/>
+      <c r="E6"/>
       <c r="F6" s="56"/>
       <c r="G6" s="56"/>
       <c r="H6" s="56"/>
-    </row>
-    <row r="7" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I6" s="56"/>
+    </row>
+    <row r="7" spans="2:9" ht="14.4" customHeight="1">
       <c r="B7" t="s">
         <v>23</v>
       </c>
@@ -43360,12 +41813,13 @@
       <c r="D7" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="56"/>
+      <c r="E7"/>
       <c r="F7" s="56"/>
       <c r="G7" s="56"/>
       <c r="H7" s="56"/>
-    </row>
-    <row r="8" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I7" s="56"/>
+    </row>
+    <row r="8" spans="2:9" ht="14.4" customHeight="1">
       <c r="B8" t="s">
         <v>24</v>
       </c>
@@ -43373,12 +41827,13 @@
       <c r="D8" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="56"/>
+      <c r="E8"/>
       <c r="F8" s="56"/>
       <c r="G8" s="56"/>
       <c r="H8" s="56"/>
-    </row>
-    <row r="9" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I8" s="56"/>
+    </row>
+    <row r="9" spans="2:9" ht="14.4" customHeight="1">
       <c r="B9" t="s">
         <v>25</v>
       </c>
@@ -43386,12 +41841,13 @@
       <c r="D9" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="56"/>
+      <c r="E9"/>
       <c r="F9" s="56"/>
       <c r="G9" s="56"/>
       <c r="H9" s="56"/>
-    </row>
-    <row r="10" spans="2:8" ht="4.95" customHeight="1">
+      <c r="I9" s="56"/>
+    </row>
+    <row r="10" spans="2:9" ht="4.95" customHeight="1">
       <c r="B10"/>
       <c r="C10"/>
       <c r="D10"/>
@@ -43399,1226 +41855,36 @@
       <c r="F10"/>
       <c r="G10"/>
       <c r="H10"/>
-    </row>
-    <row r="11" spans="2:8" s="62" customFormat="1" ht="37.200000000000003" customHeight="1">
+      <c r="I10"/>
+    </row>
+    <row r="11" spans="2:9" s="62" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="175" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="D11" s="175"/>
       <c r="E11" s="175"/>
-      <c r="F11" s="40" t="s">
+      <c r="F11" s="175"/>
+      <c r="G11" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="G11" s="40" t="s">
+      <c r="H11" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="40" t="s">
+      <c r="I11" s="40" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="2:8">
-      <c r="B12" s="22"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="64"/>
-      <c r="G12" s="65"/>
-      <c r="H12" s="64"/>
-    </row>
-    <row r="13" spans="2:8">
-      <c r="C13" s="66"/>
-      <c r="D13" s="66"/>
-      <c r="E13" s="66"/>
-    </row>
-    <row r="14" spans="2:8">
-      <c r="C14" s="59"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-    </row>
-    <row r="15" spans="2:8">
-      <c r="B15" s="22"/>
-      <c r="C15" s="69"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="65"/>
-      <c r="H15" s="64"/>
-    </row>
-    <row r="16" spans="2:8">
-      <c r="C16" s="59"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-    </row>
-    <row r="17" spans="2:8">
-      <c r="C17" s="59"/>
-      <c r="D17" s="66"/>
-      <c r="E17" s="66"/>
-    </row>
-    <row r="18" spans="2:8">
-      <c r="C18"/>
-      <c r="D18"/>
-      <c r="E18"/>
-    </row>
-    <row r="19" spans="2:8">
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19"/>
-    </row>
-    <row r="20" spans="2:8">
-      <c r="C20" s="59"/>
-      <c r="D20" s="66"/>
-      <c r="E20" s="66"/>
-    </row>
-    <row r="21" spans="2:8">
-      <c r="B21" s="22"/>
-      <c r="C21" s="69"/>
-      <c r="D21" s="63"/>
-      <c r="E21" s="63"/>
-      <c r="F21" s="64"/>
-      <c r="G21" s="65"/>
-      <c r="H21" s="64"/>
-    </row>
-    <row r="22" spans="2:8">
-      <c r="C22" s="59"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
-    </row>
-    <row r="23" spans="2:8">
-      <c r="C23" s="59"/>
-      <c r="D23" s="66"/>
-      <c r="E23" s="66"/>
-    </row>
-    <row r="24" spans="2:8">
-      <c r="C24" s="59"/>
-      <c r="D24" s="66"/>
-      <c r="E24" s="66"/>
-    </row>
-    <row r="25" spans="2:8">
-      <c r="C25" s="59"/>
-      <c r="D25" s="66"/>
-      <c r="E25" s="66"/>
-    </row>
-    <row r="26" spans="2:8">
-      <c r="C26" s="59"/>
-      <c r="D26" s="66"/>
-      <c r="E26" s="66"/>
-    </row>
-    <row r="27" spans="2:8">
-      <c r="C27" s="59"/>
-      <c r="D27" s="66"/>
-      <c r="E27" s="66"/>
-    </row>
-    <row r="28" spans="2:8">
-      <c r="C28" s="59"/>
-      <c r="D28" s="66"/>
-      <c r="E28" s="66"/>
-    </row>
-    <row r="29" spans="2:8">
-      <c r="C29" s="59"/>
-      <c r="D29" s="66"/>
-      <c r="E29" s="66"/>
-    </row>
-    <row r="30" spans="2:8">
-      <c r="C30" s="59"/>
-      <c r="D30" s="66"/>
-      <c r="E30" s="66"/>
-    </row>
-    <row r="31" spans="2:8">
-      <c r="C31" s="59"/>
-      <c r="D31" s="66"/>
-      <c r="E31" s="66"/>
-    </row>
-    <row r="32" spans="2:8">
-      <c r="B32" s="22"/>
-      <c r="C32" s="69"/>
-      <c r="D32" s="63"/>
-      <c r="E32" s="63"/>
-      <c r="F32" s="64"/>
-      <c r="G32" s="65"/>
-      <c r="H32" s="64"/>
-    </row>
-    <row r="33" spans="2:8">
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-    </row>
-    <row r="34" spans="2:8">
-      <c r="C34"/>
-      <c r="D34"/>
-      <c r="E34"/>
-    </row>
-    <row r="35" spans="2:8">
-      <c r="C35"/>
-      <c r="D35"/>
-      <c r="E35"/>
-    </row>
-    <row r="36" spans="2:8">
-      <c r="C36"/>
-      <c r="D36"/>
-      <c r="E36"/>
-    </row>
-    <row r="37" spans="2:8">
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-    </row>
-    <row r="38" spans="2:8">
-      <c r="C38"/>
-      <c r="D38"/>
-      <c r="E38"/>
-    </row>
-    <row r="39" spans="2:8">
-      <c r="C39" s="59"/>
-      <c r="D39" s="66"/>
-      <c r="E39" s="66"/>
-    </row>
-    <row r="40" spans="2:8">
-      <c r="B40" s="22"/>
-      <c r="C40" s="69"/>
-      <c r="D40" s="63"/>
-      <c r="E40" s="63"/>
-      <c r="F40" s="64"/>
-      <c r="G40" s="65"/>
-      <c r="H40" s="64"/>
-    </row>
-    <row r="41" spans="2:8">
-      <c r="C41"/>
-      <c r="D41"/>
-      <c r="E41"/>
-    </row>
-    <row r="42" spans="2:8">
-      <c r="C42"/>
-      <c r="D42"/>
-      <c r="E42"/>
-    </row>
-    <row r="43" spans="2:8">
-      <c r="C43"/>
-      <c r="D43"/>
-      <c r="E43"/>
-    </row>
-    <row r="44" spans="2:8">
-      <c r="C44"/>
-      <c r="D44"/>
-      <c r="E44"/>
-    </row>
-    <row r="45" spans="2:8">
-      <c r="C45"/>
-      <c r="D45"/>
-      <c r="E45"/>
-      <c r="F45" s="71"/>
-    </row>
-    <row r="46" spans="2:8">
-      <c r="C46"/>
-      <c r="D46"/>
-      <c r="E46"/>
-    </row>
-    <row r="47" spans="2:8">
-      <c r="C47" s="59"/>
-      <c r="D47" s="66"/>
-      <c r="E47" s="66"/>
-    </row>
-    <row r="48" spans="2:8">
-      <c r="B48" s="22"/>
-      <c r="C48" s="69"/>
-      <c r="D48" s="63"/>
-      <c r="E48" s="63"/>
-      <c r="F48" s="64"/>
-      <c r="G48" s="65"/>
-      <c r="H48" s="64"/>
-    </row>
-    <row r="49" spans="3:5">
-      <c r="C49" s="59"/>
-      <c r="D49" s="59"/>
-      <c r="E49" s="59"/>
-    </row>
-    <row r="50" spans="3:5">
-      <c r="C50" s="59"/>
-      <c r="D50" s="59"/>
-      <c r="E50" s="59"/>
-    </row>
-    <row r="51" spans="3:5">
-      <c r="C51" s="59"/>
-      <c r="D51" s="59"/>
-      <c r="E51" s="59"/>
-    </row>
-    <row r="52" spans="3:5">
-      <c r="C52" s="59"/>
-      <c r="D52" s="59"/>
-      <c r="E52" s="59"/>
-    </row>
-    <row r="53" spans="3:5">
-      <c r="C53" s="59"/>
-      <c r="D53" s="59"/>
-      <c r="E53" s="59"/>
-    </row>
-    <row r="54" spans="3:5">
-      <c r="C54" s="59"/>
-      <c r="D54" s="59"/>
-      <c r="E54" s="59"/>
-    </row>
-    <row r="55" spans="3:5">
-      <c r="C55" s="59"/>
-      <c r="D55" s="59"/>
-      <c r="E55" s="59"/>
-    </row>
-    <row r="56" spans="3:5">
-      <c r="C56" s="59"/>
-      <c r="D56" s="59"/>
-      <c r="E56" s="59"/>
-    </row>
-    <row r="57" spans="3:5">
-      <c r="C57" s="59"/>
-      <c r="D57" s="59"/>
-      <c r="E57" s="59"/>
-    </row>
-    <row r="58" spans="3:5">
-      <c r="C58" s="59"/>
-      <c r="D58" s="59"/>
-      <c r="E58" s="59"/>
-    </row>
-    <row r="59" spans="3:5">
-      <c r="C59" s="59"/>
-      <c r="D59" s="59"/>
-      <c r="E59" s="59"/>
-    </row>
-    <row r="60" spans="3:5">
-      <c r="C60" s="59"/>
-      <c r="D60" s="59"/>
-      <c r="E60" s="59"/>
-    </row>
-    <row r="61" spans="3:5">
-      <c r="C61" s="59"/>
-      <c r="D61" s="59"/>
-      <c r="E61" s="59"/>
-    </row>
-    <row r="62" spans="3:5">
-      <c r="C62" s="59"/>
-      <c r="D62" s="59"/>
-      <c r="E62" s="59"/>
-    </row>
-    <row r="63" spans="3:5">
-      <c r="C63" s="59"/>
-      <c r="D63" s="59"/>
-      <c r="E63" s="59"/>
-    </row>
-    <row r="64" spans="3:5">
-      <c r="C64" s="59"/>
-      <c r="D64" s="59"/>
-      <c r="E64" s="59"/>
-    </row>
-    <row r="65" spans="3:5">
-      <c r="C65" s="59"/>
-      <c r="D65" s="59"/>
-      <c r="E65" s="59"/>
-    </row>
-    <row r="66" spans="3:5">
-      <c r="C66" s="59"/>
-      <c r="D66" s="59"/>
-      <c r="E66" s="59"/>
-    </row>
-    <row r="67" spans="3:5">
-      <c r="C67" s="59"/>
-      <c r="D67" s="59"/>
-      <c r="E67" s="59"/>
-    </row>
-    <row r="68" spans="3:5">
-      <c r="C68" s="59"/>
-      <c r="D68" s="59"/>
-      <c r="E68" s="59"/>
-    </row>
-    <row r="69" spans="3:5">
-      <c r="C69" s="59"/>
-      <c r="D69" s="59"/>
-      <c r="E69" s="59"/>
-    </row>
-    <row r="70" spans="3:5">
-      <c r="C70" s="59"/>
-      <c r="D70" s="59"/>
-      <c r="E70" s="59"/>
-    </row>
-    <row r="71" spans="3:5">
-      <c r="C71" s="66"/>
-      <c r="D71" s="66"/>
-      <c r="E71" s="66"/>
-    </row>
-    <row r="136" spans="1:14" s="56" customFormat="1">
-      <c r="A136"/>
-      <c r="C136" t="s">
-        <v>32</v>
-      </c>
-      <c r="E136" s="57"/>
-      <c r="F136" s="68"/>
-      <c r="G136" s="60"/>
-      <c r="H136" s="68"/>
-      <c r="I136"/>
-      <c r="J136"/>
-      <c r="K136"/>
-      <c r="L136"/>
-      <c r="M136"/>
-      <c r="N136"/>
-    </row>
-    <row r="137" spans="1:14" s="56" customFormat="1">
-      <c r="A137"/>
-      <c r="C137" t="s">
-        <v>33</v>
-      </c>
-      <c r="E137" s="57"/>
-      <c r="F137" s="68"/>
-      <c r="G137" s="60"/>
-      <c r="H137" s="68"/>
-      <c r="I137"/>
-      <c r="J137"/>
-      <c r="K137"/>
-      <c r="L137"/>
-      <c r="M137"/>
-      <c r="N137"/>
-    </row>
-    <row r="138" spans="1:14" s="56" customFormat="1">
-      <c r="A138"/>
-      <c r="C138" t="s">
-        <v>34</v>
-      </c>
-      <c r="E138" s="57"/>
-      <c r="F138" s="68"/>
-      <c r="G138" s="60"/>
-      <c r="H138" s="68"/>
-      <c r="I138"/>
-      <c r="J138"/>
-      <c r="K138"/>
-      <c r="L138"/>
-      <c r="M138"/>
-      <c r="N138"/>
-    </row>
-    <row r="139" spans="1:14" s="56" customFormat="1">
-      <c r="A139"/>
-      <c r="C139" t="s">
-        <v>35</v>
-      </c>
-      <c r="E139" s="57"/>
-      <c r="F139" s="68"/>
-      <c r="G139" s="60"/>
-      <c r="H139" s="68"/>
-      <c r="I139"/>
-      <c r="J139"/>
-      <c r="K139"/>
-      <c r="L139"/>
-      <c r="M139"/>
-      <c r="N139"/>
-    </row>
-    <row r="140" spans="1:14" s="56" customFormat="1">
-      <c r="A140"/>
-      <c r="C140" t="s">
-        <v>36</v>
-      </c>
-      <c r="E140" s="57"/>
-      <c r="F140" s="68"/>
-      <c r="G140" s="60"/>
-      <c r="H140" s="68"/>
-      <c r="I140"/>
-      <c r="J140"/>
-      <c r="K140"/>
-      <c r="L140"/>
-      <c r="M140"/>
-      <c r="N140"/>
-    </row>
-    <row r="141" spans="1:14" s="56" customFormat="1">
-      <c r="A141"/>
-      <c r="C141" t="s">
-        <v>37</v>
-      </c>
-      <c r="E141" s="57"/>
-      <c r="F141" s="68"/>
-      <c r="G141" s="60"/>
-      <c r="H141" s="68"/>
-      <c r="I141"/>
-      <c r="J141"/>
-      <c r="K141"/>
-      <c r="L141"/>
-      <c r="M141"/>
-      <c r="N141"/>
-    </row>
-    <row r="142" spans="1:14" s="56" customFormat="1">
-      <c r="A142"/>
-      <c r="C142" t="s">
-        <v>38</v>
-      </c>
-      <c r="E142" s="57"/>
-      <c r="F142" s="68"/>
-      <c r="G142" s="60"/>
-      <c r="H142" s="68"/>
-      <c r="I142"/>
-      <c r="J142"/>
-      <c r="K142"/>
-      <c r="L142"/>
-      <c r="M142"/>
-      <c r="N142"/>
-    </row>
-    <row r="143" spans="1:14" s="56" customFormat="1">
-      <c r="A143"/>
-      <c r="C143" t="s">
-        <v>39</v>
-      </c>
-      <c r="E143" s="57"/>
-      <c r="F143" s="68"/>
-      <c r="G143" s="60"/>
-      <c r="H143" s="68"/>
-      <c r="I143"/>
-      <c r="J143"/>
-      <c r="K143"/>
-      <c r="L143"/>
-      <c r="M143"/>
-      <c r="N143"/>
-    </row>
-    <row r="144" spans="1:14" s="56" customFormat="1">
-      <c r="A144"/>
-      <c r="C144" t="s">
-        <v>40</v>
-      </c>
-      <c r="E144" s="57"/>
-      <c r="F144" s="68"/>
-      <c r="G144" s="60"/>
-      <c r="H144" s="68"/>
-      <c r="I144"/>
-      <c r="J144"/>
-      <c r="K144"/>
-      <c r="L144"/>
-      <c r="M144"/>
-      <c r="N144"/>
-    </row>
-    <row r="145" spans="1:14" s="56" customFormat="1">
-      <c r="A145"/>
-      <c r="C145" t="s">
-        <v>40</v>
-      </c>
-      <c r="E145" s="57"/>
-      <c r="F145" s="68"/>
-      <c r="G145" s="60"/>
-      <c r="H145" s="68"/>
-      <c r="I145"/>
-      <c r="J145"/>
-      <c r="K145"/>
-      <c r="L145"/>
-      <c r="M145"/>
-      <c r="N145"/>
-    </row>
-    <row r="146" spans="1:14" s="56" customFormat="1">
-      <c r="A146"/>
-      <c r="C146" t="s">
-        <v>41</v>
-      </c>
-      <c r="E146" s="57"/>
-      <c r="F146" s="68"/>
-      <c r="G146" s="60"/>
-      <c r="H146" s="68"/>
-      <c r="I146"/>
-      <c r="J146"/>
-      <c r="K146"/>
-      <c r="L146"/>
-      <c r="M146"/>
-      <c r="N146"/>
-    </row>
-    <row r="147" spans="1:14" s="56" customFormat="1">
-      <c r="A147"/>
-      <c r="C147" t="s">
-        <v>42</v>
-      </c>
-      <c r="E147" s="57"/>
-      <c r="F147" s="68"/>
-      <c r="G147" s="60"/>
-      <c r="H147" s="68"/>
-      <c r="I147"/>
-      <c r="J147"/>
-      <c r="K147"/>
-      <c r="L147"/>
-      <c r="M147"/>
-      <c r="N147"/>
-    </row>
-    <row r="148" spans="1:14" s="56" customFormat="1">
-      <c r="A148"/>
-      <c r="C148" t="s">
-        <v>41</v>
-      </c>
-      <c r="E148" s="57"/>
-      <c r="F148" s="68"/>
-      <c r="G148" s="60"/>
-      <c r="H148" s="68"/>
-      <c r="I148"/>
-      <c r="J148"/>
-      <c r="K148"/>
-      <c r="L148"/>
-      <c r="M148"/>
-      <c r="N148"/>
-    </row>
-    <row r="149" spans="1:14" s="56" customFormat="1">
-      <c r="A149"/>
-      <c r="C149" t="s">
-        <v>41</v>
-      </c>
-      <c r="E149" s="57"/>
-      <c r="F149" s="68"/>
-      <c r="G149" s="60"/>
-      <c r="H149" s="68"/>
-      <c r="I149"/>
-      <c r="J149"/>
-      <c r="K149"/>
-      <c r="L149"/>
-      <c r="M149"/>
-      <c r="N149"/>
-    </row>
-    <row r="150" spans="1:14" s="56" customFormat="1">
-      <c r="A150"/>
-      <c r="C150" t="s">
-        <v>41</v>
-      </c>
-      <c r="E150" s="57"/>
-      <c r="F150" s="68"/>
-      <c r="G150" s="60"/>
-      <c r="H150" s="68"/>
-      <c r="I150"/>
-      <c r="J150"/>
-      <c r="K150"/>
-      <c r="L150"/>
-      <c r="M150"/>
-      <c r="N150"/>
-    </row>
-    <row r="151" spans="1:14" s="56" customFormat="1">
-      <c r="A151"/>
-      <c r="C151" t="s">
-        <v>43</v>
-      </c>
-      <c r="E151" s="57"/>
-      <c r="F151" s="68"/>
-      <c r="G151" s="60"/>
-      <c r="H151" s="68"/>
-      <c r="I151"/>
-      <c r="J151"/>
-      <c r="K151"/>
-      <c r="L151"/>
-      <c r="M151"/>
-      <c r="N151"/>
-    </row>
-    <row r="152" spans="1:14" s="56" customFormat="1">
-      <c r="A152"/>
-      <c r="C152" t="s">
-        <v>44</v>
-      </c>
-      <c r="E152" s="57"/>
-      <c r="F152" s="68"/>
-      <c r="G152" s="60"/>
-      <c r="H152" s="68"/>
-      <c r="I152"/>
-      <c r="J152"/>
-      <c r="K152"/>
-      <c r="L152"/>
-      <c r="M152"/>
-      <c r="N152"/>
-    </row>
-    <row r="153" spans="1:14" s="56" customFormat="1">
-      <c r="A153"/>
-      <c r="C153" t="s">
-        <v>39</v>
-      </c>
-      <c r="E153" s="57"/>
-      <c r="F153" s="68"/>
-      <c r="G153" s="60"/>
-      <c r="H153" s="68"/>
-      <c r="I153"/>
-      <c r="J153"/>
-      <c r="K153"/>
-      <c r="L153"/>
-      <c r="M153"/>
-      <c r="N153"/>
-    </row>
-    <row r="154" spans="1:14" s="56" customFormat="1">
-      <c r="A154"/>
-      <c r="C154" t="s">
-        <v>45</v>
-      </c>
-      <c r="E154" s="57"/>
-      <c r="F154" s="68"/>
-      <c r="G154" s="60"/>
-      <c r="H154" s="68"/>
-      <c r="I154"/>
-      <c r="J154"/>
-      <c r="K154"/>
-      <c r="L154"/>
-      <c r="M154"/>
-      <c r="N154"/>
-    </row>
-    <row r="155" spans="1:14" s="56" customFormat="1">
-      <c r="A155"/>
-      <c r="C155" t="s">
-        <v>46</v>
-      </c>
-      <c r="E155" s="57"/>
-      <c r="F155" s="68"/>
-      <c r="G155" s="60"/>
-      <c r="H155" s="68"/>
-      <c r="I155"/>
-      <c r="J155"/>
-      <c r="K155"/>
-      <c r="L155"/>
-      <c r="M155"/>
-      <c r="N155"/>
-    </row>
-    <row r="156" spans="1:14" s="56" customFormat="1">
-      <c r="A156"/>
-      <c r="C156" t="s">
-        <v>47</v>
-      </c>
-      <c r="E156" s="57"/>
-      <c r="F156" s="68"/>
-      <c r="G156" s="60"/>
-      <c r="H156" s="68"/>
-      <c r="I156"/>
-      <c r="J156"/>
-      <c r="K156"/>
-      <c r="L156"/>
-      <c r="M156"/>
-      <c r="N156"/>
-    </row>
-    <row r="157" spans="1:14" s="56" customFormat="1">
-      <c r="A157"/>
-      <c r="C157" t="s">
-        <v>48</v>
-      </c>
-      <c r="E157" s="57"/>
-      <c r="F157" s="68"/>
-      <c r="G157" s="60"/>
-      <c r="H157" s="68"/>
-      <c r="I157"/>
-      <c r="J157"/>
-      <c r="K157"/>
-      <c r="L157"/>
-      <c r="M157"/>
-      <c r="N157"/>
-    </row>
-    <row r="158" spans="1:14" s="56" customFormat="1">
-      <c r="A158"/>
-      <c r="C158" t="s">
-        <v>49</v>
-      </c>
-      <c r="E158" s="57"/>
-      <c r="F158" s="68"/>
-      <c r="G158" s="60"/>
-      <c r="H158" s="68"/>
-      <c r="I158"/>
-      <c r="J158"/>
-      <c r="K158"/>
-      <c r="L158"/>
-      <c r="M158"/>
-      <c r="N158"/>
-    </row>
-    <row r="159" spans="1:14" s="56" customFormat="1">
-      <c r="A159"/>
-      <c r="C159" t="s">
-        <v>50</v>
-      </c>
-      <c r="E159" s="57"/>
-      <c r="F159" s="68"/>
-      <c r="G159" s="60"/>
-      <c r="H159" s="68"/>
-      <c r="I159"/>
-      <c r="J159"/>
-      <c r="K159"/>
-      <c r="L159"/>
-      <c r="M159"/>
-      <c r="N159"/>
-    </row>
-    <row r="160" spans="1:14" s="56" customFormat="1">
-      <c r="A160"/>
-      <c r="C160" t="s">
-        <v>39</v>
-      </c>
-      <c r="E160" s="57"/>
-      <c r="F160" s="68"/>
-      <c r="G160" s="60"/>
-      <c r="H160" s="68"/>
-      <c r="I160"/>
-      <c r="J160"/>
-      <c r="K160"/>
-      <c r="L160"/>
-      <c r="M160"/>
-      <c r="N160"/>
-    </row>
-    <row r="161" spans="1:14" s="56" customFormat="1">
-      <c r="A161"/>
-      <c r="C161" t="s">
-        <v>40</v>
-      </c>
-      <c r="E161" s="57"/>
-      <c r="F161" s="68"/>
-      <c r="G161" s="60"/>
-      <c r="H161" s="68"/>
-      <c r="I161"/>
-      <c r="J161"/>
-      <c r="K161"/>
-      <c r="L161"/>
-      <c r="M161"/>
-      <c r="N161"/>
-    </row>
-    <row r="162" spans="1:14" s="56" customFormat="1">
-      <c r="A162"/>
-      <c r="C162" t="s">
-        <v>51</v>
-      </c>
-      <c r="E162" s="57"/>
-      <c r="F162" s="68"/>
-      <c r="G162" s="60"/>
-      <c r="H162" s="68"/>
-      <c r="I162"/>
-      <c r="J162"/>
-      <c r="K162"/>
-      <c r="L162"/>
-      <c r="M162"/>
-      <c r="N162"/>
-    </row>
-    <row r="163" spans="1:14" s="56" customFormat="1">
-      <c r="A163"/>
-      <c r="C163" t="s">
-        <v>52</v>
-      </c>
-      <c r="E163" s="57"/>
-      <c r="F163" s="68"/>
-      <c r="G163" s="60"/>
-      <c r="H163" s="68"/>
-      <c r="I163"/>
-      <c r="J163"/>
-      <c r="K163"/>
-      <c r="L163"/>
-      <c r="M163"/>
-      <c r="N163"/>
-    </row>
-    <row r="164" spans="1:14" s="56" customFormat="1">
-      <c r="A164"/>
-      <c r="C164" t="s">
-        <v>53</v>
-      </c>
-      <c r="E164" s="57"/>
-      <c r="F164" s="68"/>
-      <c r="G164" s="60"/>
-      <c r="H164" s="68"/>
-      <c r="I164"/>
-      <c r="J164"/>
-      <c r="K164"/>
-      <c r="L164"/>
-      <c r="M164"/>
-      <c r="N164"/>
-    </row>
-    <row r="165" spans="1:14" s="56" customFormat="1">
-      <c r="A165"/>
-      <c r="C165" t="s">
-        <v>54</v>
-      </c>
-      <c r="E165" s="57"/>
-      <c r="F165" s="68"/>
-      <c r="G165" s="60"/>
-      <c r="H165" s="68"/>
-      <c r="I165"/>
-      <c r="J165"/>
-      <c r="K165"/>
-      <c r="L165"/>
-      <c r="M165"/>
-      <c r="N165"/>
-    </row>
-    <row r="166" spans="1:14" s="56" customFormat="1">
-      <c r="A166"/>
-      <c r="C166" t="s">
-        <v>55</v>
-      </c>
-      <c r="E166" s="57"/>
-      <c r="F166" s="68"/>
-      <c r="G166" s="60"/>
-      <c r="H166" s="68"/>
-      <c r="I166"/>
-      <c r="J166"/>
-      <c r="K166"/>
-      <c r="L166"/>
-      <c r="M166"/>
-      <c r="N166"/>
-    </row>
-    <row r="167" spans="1:14" s="56" customFormat="1">
-      <c r="A167"/>
-      <c r="C167" t="s">
-        <v>39</v>
-      </c>
-      <c r="E167" s="57"/>
-      <c r="F167" s="68"/>
-      <c r="G167" s="60"/>
-      <c r="H167" s="68"/>
-      <c r="I167"/>
-      <c r="J167"/>
-      <c r="K167"/>
-      <c r="L167"/>
-      <c r="M167"/>
-      <c r="N167"/>
-    </row>
-    <row r="168" spans="1:14" s="56" customFormat="1">
-      <c r="A168"/>
-      <c r="C168" t="s">
-        <v>40</v>
-      </c>
-      <c r="E168" s="57"/>
-      <c r="F168" s="68"/>
-      <c r="G168" s="60"/>
-      <c r="H168" s="68"/>
-      <c r="I168"/>
-      <c r="J168"/>
-      <c r="K168"/>
-      <c r="L168"/>
-      <c r="M168"/>
-      <c r="N168"/>
-    </row>
-    <row r="169" spans="1:14" s="56" customFormat="1">
-      <c r="A169"/>
-      <c r="C169" t="s">
-        <v>56</v>
-      </c>
-      <c r="E169" s="57"/>
-      <c r="F169" s="68"/>
-      <c r="G169" s="60"/>
-      <c r="H169" s="68"/>
-      <c r="I169"/>
-      <c r="J169"/>
-      <c r="K169"/>
-      <c r="L169"/>
-      <c r="M169"/>
-      <c r="N169"/>
-    </row>
-    <row r="170" spans="1:14" s="56" customFormat="1">
-      <c r="A170"/>
-      <c r="C170" t="s">
-        <v>57</v>
-      </c>
-      <c r="E170" s="57"/>
-      <c r="F170" s="68"/>
-      <c r="G170" s="60"/>
-      <c r="H170" s="68"/>
-      <c r="I170"/>
-      <c r="J170"/>
-      <c r="K170"/>
-      <c r="L170"/>
-      <c r="M170"/>
-      <c r="N170"/>
-    </row>
-    <row r="171" spans="1:14" s="56" customFormat="1">
-      <c r="A171"/>
-      <c r="C171" t="s">
-        <v>40</v>
-      </c>
-      <c r="E171" s="57"/>
-      <c r="F171" s="68"/>
-      <c r="G171" s="60"/>
-      <c r="H171" s="68"/>
-      <c r="I171"/>
-      <c r="J171"/>
-      <c r="K171"/>
-      <c r="L171"/>
-      <c r="M171"/>
-      <c r="N171"/>
-    </row>
-    <row r="172" spans="1:14" s="56" customFormat="1">
-      <c r="A172"/>
-      <c r="C172" t="s">
-        <v>54</v>
-      </c>
-      <c r="E172" s="57"/>
-      <c r="F172" s="68"/>
-      <c r="G172" s="60"/>
-      <c r="H172" s="68"/>
-      <c r="I172"/>
-      <c r="J172"/>
-      <c r="K172"/>
-      <c r="L172"/>
-      <c r="M172"/>
-      <c r="N172"/>
-    </row>
-    <row r="173" spans="1:14" s="56" customFormat="1">
-      <c r="A173"/>
-      <c r="C173" t="s">
-        <v>58</v>
-      </c>
-      <c r="E173" s="57"/>
-      <c r="F173" s="68"/>
-      <c r="G173" s="60"/>
-      <c r="H173" s="68"/>
-      <c r="I173"/>
-      <c r="J173"/>
-      <c r="K173"/>
-      <c r="L173"/>
-      <c r="M173"/>
-      <c r="N173"/>
-    </row>
-    <row r="174" spans="1:14" s="56" customFormat="1">
-      <c r="A174"/>
-      <c r="C174" t="s">
-        <v>59</v>
-      </c>
-      <c r="E174" s="57"/>
-      <c r="F174" s="68"/>
-      <c r="G174" s="60"/>
-      <c r="H174" s="68"/>
-      <c r="I174"/>
-      <c r="J174"/>
-      <c r="K174"/>
-      <c r="L174"/>
-      <c r="M174"/>
-      <c r="N174"/>
-    </row>
-    <row r="175" spans="1:14" s="56" customFormat="1">
-      <c r="A175"/>
-      <c r="C175" t="s">
-        <v>60</v>
-      </c>
-      <c r="E175" s="57"/>
-      <c r="F175" s="68"/>
-      <c r="G175" s="60"/>
-      <c r="H175" s="68"/>
-      <c r="I175"/>
-      <c r="J175"/>
-      <c r="K175"/>
-      <c r="L175"/>
-      <c r="M175"/>
-      <c r="N175"/>
-    </row>
-    <row r="176" spans="1:14" s="56" customFormat="1">
-      <c r="A176"/>
-      <c r="C176" t="s">
-        <v>61</v>
-      </c>
-      <c r="E176" s="57"/>
-      <c r="F176" s="68"/>
-      <c r="G176" s="60"/>
-      <c r="H176" s="68"/>
-      <c r="I176"/>
-      <c r="J176"/>
-      <c r="K176"/>
-      <c r="L176"/>
-      <c r="M176"/>
-      <c r="N176"/>
-    </row>
-    <row r="177" spans="1:14" s="56" customFormat="1">
-      <c r="A177"/>
-      <c r="C177" t="s">
-        <v>62</v>
-      </c>
-      <c r="E177" s="57"/>
-      <c r="F177" s="68"/>
-      <c r="G177" s="60"/>
-      <c r="H177" s="68"/>
-      <c r="I177"/>
-      <c r="J177"/>
-      <c r="K177"/>
-      <c r="L177"/>
-      <c r="M177"/>
-      <c r="N177"/>
-    </row>
-    <row r="178" spans="1:14" s="56" customFormat="1">
-      <c r="A178"/>
-      <c r="C178" t="s">
-        <v>63</v>
-      </c>
-      <c r="E178" s="57"/>
-      <c r="F178" s="68"/>
-      <c r="G178" s="60"/>
-      <c r="H178" s="68"/>
-      <c r="I178"/>
-      <c r="J178"/>
-      <c r="K178"/>
-      <c r="L178"/>
-      <c r="M178"/>
-      <c r="N178"/>
-    </row>
-    <row r="179" spans="1:14" s="56" customFormat="1">
-      <c r="A179"/>
-      <c r="C179" t="s">
-        <v>64</v>
-      </c>
-      <c r="E179" s="57"/>
-      <c r="F179" s="68"/>
-      <c r="G179" s="60"/>
-      <c r="H179" s="68"/>
-      <c r="I179"/>
-      <c r="J179"/>
-      <c r="K179"/>
-      <c r="L179"/>
-      <c r="M179"/>
-      <c r="N179"/>
-    </row>
-    <row r="180" spans="1:14" s="56" customFormat="1">
-      <c r="A180"/>
-      <c r="C180" t="s">
-        <v>65</v>
-      </c>
-      <c r="E180" s="57"/>
-      <c r="F180" s="68"/>
-      <c r="G180" s="60"/>
-      <c r="H180" s="68"/>
-      <c r="I180"/>
-      <c r="J180"/>
-      <c r="K180"/>
-      <c r="L180"/>
-      <c r="M180"/>
-      <c r="N180"/>
-    </row>
-    <row r="181" spans="1:14" s="56" customFormat="1">
-      <c r="A181"/>
-      <c r="C181" t="s">
-        <v>66</v>
-      </c>
-      <c r="E181" s="57"/>
-      <c r="F181" s="68"/>
-      <c r="G181" s="60"/>
-      <c r="H181" s="68"/>
-      <c r="I181"/>
-      <c r="J181"/>
-      <c r="K181"/>
-      <c r="L181"/>
-      <c r="M181"/>
-      <c r="N181"/>
-    </row>
-    <row r="182" spans="1:14" s="56" customFormat="1">
-      <c r="A182"/>
-      <c r="C182" t="s">
-        <v>67</v>
-      </c>
-      <c r="E182" s="57"/>
-      <c r="F182" s="68"/>
-      <c r="G182" s="60"/>
-      <c r="H182" s="68"/>
-      <c r="I182"/>
-      <c r="J182"/>
-      <c r="K182"/>
-      <c r="L182"/>
-      <c r="M182"/>
-      <c r="N182"/>
-    </row>
-    <row r="183" spans="1:14" s="56" customFormat="1">
-      <c r="A183"/>
-      <c r="C183" t="s">
-        <v>68</v>
-      </c>
-      <c r="E183" s="57"/>
-      <c r="F183" s="68"/>
-      <c r="G183" s="60"/>
-      <c r="H183" s="68"/>
-      <c r="I183"/>
-      <c r="J183"/>
-      <c r="K183"/>
-      <c r="L183"/>
-      <c r="M183"/>
-      <c r="N183"/>
-    </row>
-    <row r="184" spans="1:14" s="56" customFormat="1">
-      <c r="A184"/>
-      <c r="C184" t="s">
-        <v>69</v>
-      </c>
-      <c r="E184" s="57"/>
-      <c r="F184" s="68"/>
-      <c r="G184" s="60"/>
-      <c r="H184" s="68"/>
-      <c r="I184"/>
-      <c r="J184"/>
-      <c r="K184"/>
-      <c r="L184"/>
-      <c r="M184"/>
-      <c r="N184"/>
-    </row>
-    <row r="185" spans="1:14" s="56" customFormat="1">
-      <c r="A185"/>
-      <c r="C185" t="s">
-        <v>70</v>
-      </c>
-      <c r="E185" s="57"/>
-      <c r="F185" s="68"/>
-      <c r="G185" s="60"/>
-      <c r="H185" s="68"/>
-      <c r="I185"/>
-      <c r="J185"/>
-      <c r="K185"/>
-      <c r="L185"/>
-      <c r="M185"/>
-      <c r="N185"/>
-    </row>
-    <row r="186" spans="1:14" s="56" customFormat="1">
-      <c r="A186"/>
-      <c r="C186" t="s">
-        <v>71</v>
-      </c>
-      <c r="E186" s="57"/>
-      <c r="F186" s="68"/>
-      <c r="G186" s="60"/>
-      <c r="H186" s="68"/>
-      <c r="I186"/>
-      <c r="J186"/>
-      <c r="K186"/>
-      <c r="L186"/>
-      <c r="M186"/>
-      <c r="N186"/>
-    </row>
-    <row r="187" spans="1:14" s="56" customFormat="1">
-      <c r="A187"/>
-      <c r="C187" t="s">
-        <v>72</v>
-      </c>
-      <c r="E187" s="57"/>
-      <c r="F187" s="68"/>
-      <c r="G187" s="60"/>
-      <c r="H187" s="68"/>
-      <c r="I187"/>
-      <c r="J187"/>
-      <c r="K187"/>
-      <c r="L187"/>
-      <c r="M187"/>
-      <c r="N187"/>
-    </row>
-    <row r="188" spans="1:14" s="56" customFormat="1">
-      <c r="A188"/>
-      <c r="C188" t="s">
-        <v>73</v>
-      </c>
-      <c r="E188" s="57"/>
-      <c r="F188" s="68"/>
-      <c r="G188" s="60"/>
-      <c r="H188" s="68"/>
-      <c r="I188"/>
-      <c r="J188"/>
-      <c r="K188"/>
-      <c r="L188"/>
-      <c r="M188"/>
-      <c r="N188"/>
-    </row>
-    <row r="189" spans="1:14" s="56" customFormat="1">
-      <c r="A189"/>
-      <c r="C189"/>
-      <c r="E189" s="57"/>
-      <c r="F189" s="68"/>
-      <c r="G189" s="60"/>
-      <c r="H189" s="68"/>
-      <c r="I189"/>
-      <c r="J189"/>
-      <c r="K189"/>
-      <c r="L189"/>
-      <c r="M189"/>
-      <c r="N189"/>
-    </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="B1:I1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B12:H9929">
-    <cfRule type="expression" dxfId="23" priority="9">
-      <formula>AND($B12&lt;&gt;"",$C12&lt;&gt;"",#REF!="")</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="73" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="76" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -44646,7 +41912,7 @@
     </row>
     <row r="2" spans="2:12" ht="18">
       <c r="B2" s="181" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="C2" s="181"/>
       <c r="D2" s="181"/>
@@ -44665,16 +41931,16 @@
         <v>6</v>
       </c>
       <c r="C5" s="179" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="D5" s="179" t="s">
         <v>29</v>
       </c>
       <c r="E5" s="180" t="s">
-        <v>83</v>
+        <v>41</v>
       </c>
       <c r="F5" s="180" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
@@ -44737,39 +42003,39 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:CE7">
-    <cfRule type="expression" dxfId="22" priority="12">
+    <cfRule type="expression" dxfId="14" priority="12">
       <formula>B5&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:CE201">
-    <cfRule type="expression" dxfId="21" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>AND(G8&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="2">
+    <cfRule type="expression" dxfId="12" priority="2">
       <formula>AND(G$7&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="3">
+    <cfRule type="expression" dxfId="11" priority="3">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="4">
+    <cfRule type="expression" dxfId="10" priority="4">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="5">
+    <cfRule type="expression" dxfId="9" priority="5">
       <formula>AND(G8&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="6">
+    <cfRule type="expression" dxfId="8" priority="6">
       <formula>AND(G$7&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="7">
+    <cfRule type="expression" dxfId="7" priority="7">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="8">
+    <cfRule type="expression" dxfId="6" priority="8">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="10">
+    <cfRule type="expression" dxfId="4" priority="10">
       <formula>AND(G$7&lt;&gt;"",$B8="DEVIASI")</formula>
     </cfRule>
     <cfRule type="colorScale" priority="11">

</xml_diff>

<commit_message>
feat(export): update documentation excel layout, print area, and repeating headers
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA70E7DC-8CA8-4115-9B7B-3700769E2C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB359FBF-B014-4B2F-9EF6-15F53CD91CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cover" sheetId="21" r:id="rId1"/>
@@ -5141,7 +5141,7 @@
     <col min="16" max="16" width="1.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:15" ht="75" customHeight="1">
+    <row r="1" spans="2:15" ht="103.2" customHeight="1">
       <c r="B1" s="177"/>
       <c r="C1" s="177"/>
       <c r="D1" s="177"/>

</xml_diff>

<commit_message>
feat(reporting): added dynamic header info in K6:K10 and contractor name in I4 for weekly/monthly reports
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -5,7 +5,7 @@
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB359FBF-B014-4B2F-9EF6-15F53CD91CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cover" sheetId="21" r:id="rId1"/>
@@ -2088,7 +2088,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="169" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="315">
+  <cellXfs count="313">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2651,6 +2651,48 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="90" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="93" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="108" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="100" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="98" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2670,9 +2712,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2683,66 +2722,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="79" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2756,8 +2735,98 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2878,98 +2947,68 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="47" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="79" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2980,25 +3019,32 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="94" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="90" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="93" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="108" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="112" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="106" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="105" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="7" borderId="109" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3009,19 +3055,10 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="100" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="98" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="4" borderId="81" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3033,18 +3070,6 @@
     <xf numFmtId="0" fontId="32" fillId="4" borderId="83" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="32" fillId="4" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3053,6 +3078,9 @@
     </xf>
     <xf numFmtId="0" fontId="32" fillId="4" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="4" borderId="106" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3066,41 +3094,11 @@
     <xf numFmtId="0" fontId="32" fillId="4" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="105" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="112" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="106" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="94" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -4412,40 +4410,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="178"/>
-      <c r="C1" s="178"/>
-      <c r="D1" s="178"/>
-      <c r="E1" s="178"/>
-      <c r="F1" s="178"/>
-      <c r="G1" s="178"/>
-      <c r="H1" s="178"/>
-      <c r="I1" s="178"/>
-      <c r="J1" s="178"/>
-      <c r="K1" s="178"/>
-      <c r="L1" s="178"/>
-      <c r="M1" s="178"/>
-      <c r="N1" s="178"/>
-      <c r="O1" s="178"/>
-      <c r="P1" s="178"/>
+      <c r="B1" s="195"/>
+      <c r="C1" s="195"/>
+      <c r="D1" s="195"/>
+      <c r="E1" s="195"/>
+      <c r="F1" s="195"/>
+      <c r="G1" s="195"/>
+      <c r="H1" s="195"/>
+      <c r="I1" s="195"/>
+      <c r="J1" s="195"/>
+      <c r="K1" s="195"/>
+      <c r="L1" s="195"/>
+      <c r="M1" s="195"/>
+      <c r="N1" s="195"/>
+      <c r="O1" s="195"/>
+      <c r="P1" s="195"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="176" t="s">
+      <c r="B2" s="194" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="177"/>
-      <c r="D2" s="177"/>
-      <c r="E2" s="177"/>
-      <c r="F2" s="177"/>
-      <c r="G2" s="177"/>
-      <c r="H2" s="177"/>
-      <c r="I2" s="177"/>
-      <c r="J2" s="177"/>
-      <c r="K2" s="177"/>
-      <c r="L2" s="177"/>
-      <c r="M2" s="177"/>
-      <c r="N2" s="177"/>
-      <c r="O2" s="177"/>
-      <c r="P2" s="177"/>
+      <c r="C2" s="186"/>
+      <c r="D2" s="186"/>
+      <c r="E2" s="186"/>
+      <c r="F2" s="186"/>
+      <c r="G2" s="186"/>
+      <c r="H2" s="186"/>
+      <c r="I2" s="186"/>
+      <c r="J2" s="186"/>
+      <c r="K2" s="186"/>
+      <c r="L2" s="186"/>
+      <c r="M2" s="186"/>
+      <c r="N2" s="186"/>
+      <c r="O2" s="186"/>
+      <c r="P2" s="186"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4472,16 +4470,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="268" t="s">
+      <c r="I4" s="285" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="268"/>
-      <c r="K4" s="268"/>
-      <c r="L4" s="268"/>
-      <c r="M4" s="268"/>
-      <c r="N4" s="268"/>
-      <c r="O4" s="268"/>
-      <c r="P4" s="268"/>
+      <c r="J4" s="285"/>
+      <c r="K4" s="285"/>
+      <c r="L4" s="285"/>
+      <c r="M4" s="285"/>
+      <c r="N4" s="285"/>
+      <c r="O4" s="285"/>
+      <c r="P4" s="285"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4495,14 +4493,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="268"/>
-      <c r="J5" s="268"/>
-      <c r="K5" s="268"/>
-      <c r="L5" s="268"/>
-      <c r="M5" s="268"/>
-      <c r="N5" s="268"/>
-      <c r="O5" s="268"/>
-      <c r="P5" s="268"/>
+      <c r="I5" s="285"/>
+      <c r="J5" s="285"/>
+      <c r="K5" s="285"/>
+      <c r="L5" s="285"/>
+      <c r="M5" s="285"/>
+      <c r="N5" s="285"/>
+      <c r="O5" s="285"/>
+      <c r="P5" s="285"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4637,70 +4635,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="175" t="s">
+      <c r="B12" s="193" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="175" t="s">
+      <c r="C12" s="193" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="175"/>
-      <c r="E12" s="175"/>
-      <c r="F12" s="175" t="s">
+      <c r="D12" s="193"/>
+      <c r="E12" s="193"/>
+      <c r="F12" s="193" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="175" t="s">
+      <c r="G12" s="193" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="175" t="s">
+      <c r="H12" s="193" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="175" t="s">
+      <c r="I12" s="193" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="175" t="s">
+      <c r="J12" s="193" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="175"/>
-      <c r="L12" s="175"/>
-      <c r="M12" s="175"/>
-      <c r="N12" s="175"/>
-      <c r="O12" s="175"/>
-      <c r="P12" s="267" t="s">
+      <c r="K12" s="193"/>
+      <c r="L12" s="193"/>
+      <c r="M12" s="193"/>
+      <c r="N12" s="193"/>
+      <c r="O12" s="193"/>
+      <c r="P12" s="284" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="175"/>
-      <c r="C13" s="175"/>
-      <c r="D13" s="175"/>
-      <c r="E13" s="175"/>
-      <c r="F13" s="175"/>
-      <c r="G13" s="175"/>
-      <c r="H13" s="175"/>
-      <c r="I13" s="175"/>
-      <c r="J13" s="266" t="s">
+      <c r="B13" s="193"/>
+      <c r="C13" s="193"/>
+      <c r="D13" s="193"/>
+      <c r="E13" s="193"/>
+      <c r="F13" s="193"/>
+      <c r="G13" s="193"/>
+      <c r="H13" s="193"/>
+      <c r="I13" s="193"/>
+      <c r="J13" s="283" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="266"/>
-      <c r="L13" s="266" t="s">
+      <c r="K13" s="283"/>
+      <c r="L13" s="283" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="266"/>
-      <c r="N13" s="266" t="s">
+      <c r="M13" s="283"/>
+      <c r="N13" s="283" t="s">
         <v>95</v>
       </c>
-      <c r="O13" s="266"/>
-      <c r="P13" s="267"/>
+      <c r="O13" s="283"/>
+      <c r="P13" s="284"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="175"/>
-      <c r="C14" s="175"/>
-      <c r="D14" s="175"/>
-      <c r="E14" s="175"/>
-      <c r="F14" s="175"/>
-      <c r="G14" s="175"/>
-      <c r="H14" s="175"/>
-      <c r="I14" s="175"/>
+      <c r="B14" s="193"/>
+      <c r="C14" s="193"/>
+      <c r="D14" s="193"/>
+      <c r="E14" s="193"/>
+      <c r="F14" s="193"/>
+      <c r="G14" s="193"/>
+      <c r="H14" s="193"/>
+      <c r="I14" s="193"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -4719,7 +4717,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="267"/>
+      <c r="P14" s="284"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -5142,24 +5140,297 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="103.2" customHeight="1">
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="177"/>
-      <c r="O1" s="177"/>
+      <c r="B1" s="186"/>
+      <c r="C1" s="186"/>
+      <c r="D1" s="186"/>
+      <c r="E1" s="186"/>
+      <c r="F1" s="186"/>
+      <c r="G1" s="186"/>
+      <c r="H1" s="186"/>
+      <c r="I1" s="186"/>
+      <c r="J1" s="186"/>
+      <c r="K1" s="186"/>
+      <c r="L1" s="186"/>
+      <c r="M1" s="186"/>
+      <c r="N1" s="186"/>
+      <c r="O1" s="186"/>
     </row>
     <row r="2" spans="2:15" ht="22.95" customHeight="1">
-      <c r="B2" s="287" t="s">
+      <c r="B2" s="187" t="s">
         <v>104</v>
+      </c>
+      <c r="C2" s="187"/>
+      <c r="D2" s="187"/>
+      <c r="E2" s="187"/>
+      <c r="F2" s="187"/>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="187"/>
+      <c r="J2" s="187"/>
+      <c r="K2" s="187"/>
+      <c r="L2" s="187"/>
+      <c r="M2" s="187"/>
+      <c r="N2" s="187"/>
+      <c r="O2" s="187"/>
+    </row>
+    <row r="3" spans="2:15">
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15">
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15">
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15">
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15">
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15">
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" ht="4.95" customHeight="1"/>
+    <row r="11" spans="2:15" s="58" customFormat="1">
+      <c r="B11" s="188" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" s="188"/>
+      <c r="D11" s="188"/>
+      <c r="E11" s="188"/>
+      <c r="G11" s="188" t="s">
+        <v>105</v>
+      </c>
+      <c r="H11" s="188"/>
+      <c r="I11" s="188"/>
+      <c r="J11" s="188"/>
+      <c r="L11" s="188" t="s">
+        <v>105</v>
+      </c>
+      <c r="M11" s="188"/>
+      <c r="N11" s="188"/>
+      <c r="O11" s="188"/>
+    </row>
+    <row r="12" spans="2:15" ht="4.95" customHeight="1"/>
+    <row r="13" spans="2:15">
+      <c r="B13" s="186"/>
+      <c r="C13" s="186"/>
+      <c r="D13" s="186"/>
+      <c r="E13" s="186"/>
+      <c r="G13" s="186"/>
+      <c r="H13" s="186"/>
+      <c r="I13" s="186"/>
+      <c r="J13" s="186"/>
+      <c r="L13" s="186"/>
+      <c r="M13" s="186"/>
+      <c r="N13" s="186"/>
+      <c r="O13" s="186"/>
+    </row>
+    <row r="14" spans="2:15">
+      <c r="B14" s="186"/>
+      <c r="C14" s="186"/>
+      <c r="D14" s="186"/>
+      <c r="E14" s="186"/>
+      <c r="G14" s="186"/>
+      <c r="H14" s="186"/>
+      <c r="I14" s="186"/>
+      <c r="J14" s="186"/>
+      <c r="L14" s="186"/>
+      <c r="M14" s="186"/>
+      <c r="N14" s="186"/>
+      <c r="O14" s="186"/>
+    </row>
+    <row r="15" spans="2:15">
+      <c r="B15" s="186"/>
+      <c r="C15" s="186"/>
+      <c r="D15" s="186"/>
+      <c r="E15" s="186"/>
+      <c r="G15" s="186"/>
+      <c r="H15" s="186"/>
+      <c r="I15" s="186"/>
+      <c r="J15" s="186"/>
+      <c r="L15" s="186"/>
+      <c r="M15" s="186"/>
+      <c r="N15" s="186"/>
+      <c r="O15" s="186"/>
+    </row>
+    <row r="16" spans="2:15">
+      <c r="B16" s="186"/>
+      <c r="C16" s="186"/>
+      <c r="D16" s="186"/>
+      <c r="E16" s="186"/>
+      <c r="G16" s="186"/>
+      <c r="H16" s="186"/>
+      <c r="I16" s="186"/>
+      <c r="J16" s="186"/>
+      <c r="L16" s="186"/>
+      <c r="M16" s="186"/>
+      <c r="N16" s="186"/>
+      <c r="O16" s="186"/>
+    </row>
+    <row r="17" spans="2:15">
+      <c r="B17" s="186"/>
+      <c r="C17" s="186"/>
+      <c r="D17" s="186"/>
+      <c r="E17" s="186"/>
+      <c r="G17" s="186"/>
+      <c r="H17" s="186"/>
+      <c r="I17" s="186"/>
+      <c r="J17" s="186"/>
+      <c r="L17" s="186"/>
+      <c r="M17" s="186"/>
+      <c r="N17" s="186"/>
+      <c r="O17" s="186"/>
+    </row>
+    <row r="18" spans="2:15">
+      <c r="B18" s="186"/>
+      <c r="C18" s="186"/>
+      <c r="D18" s="186"/>
+      <c r="E18" s="186"/>
+      <c r="G18" s="186"/>
+      <c r="H18" s="186"/>
+      <c r="I18" s="186"/>
+      <c r="J18" s="186"/>
+      <c r="L18" s="186"/>
+      <c r="M18" s="186"/>
+      <c r="N18" s="186"/>
+      <c r="O18" s="186"/>
+    </row>
+    <row r="19" spans="2:15">
+      <c r="B19" s="186"/>
+      <c r="C19" s="186"/>
+      <c r="D19" s="186"/>
+      <c r="E19" s="186"/>
+      <c r="G19" s="186"/>
+      <c r="H19" s="186"/>
+      <c r="I19" s="186"/>
+      <c r="J19" s="186"/>
+      <c r="L19" s="186"/>
+      <c r="M19" s="186"/>
+      <c r="N19" s="186"/>
+      <c r="O19" s="186"/>
+    </row>
+    <row r="20" spans="2:15">
+      <c r="B20" s="186"/>
+      <c r="C20" s="186"/>
+      <c r="D20" s="186"/>
+      <c r="E20" s="186"/>
+      <c r="G20" s="186"/>
+      <c r="H20" s="186"/>
+      <c r="I20" s="186"/>
+      <c r="J20" s="186"/>
+      <c r="L20" s="186"/>
+      <c r="M20" s="186"/>
+      <c r="N20" s="186"/>
+      <c r="O20" s="186"/>
+    </row>
+    <row r="21" spans="2:15">
+      <c r="B21" s="186"/>
+      <c r="C21" s="186"/>
+      <c r="D21" s="186"/>
+      <c r="E21" s="186"/>
+      <c r="G21" s="186"/>
+      <c r="H21" s="186"/>
+      <c r="I21" s="186"/>
+      <c r="J21" s="186"/>
+      <c r="L21" s="186"/>
+      <c r="M21" s="186"/>
+      <c r="N21" s="186"/>
+      <c r="O21" s="186"/>
+    </row>
+    <row r="22" spans="2:15">
+      <c r="B22" s="186"/>
+      <c r="C22" s="186"/>
+      <c r="D22" s="186"/>
+      <c r="E22" s="186"/>
+      <c r="G22" s="186"/>
+      <c r="H22" s="186"/>
+      <c r="I22" s="186"/>
+      <c r="J22" s="186"/>
+      <c r="L22" s="186"/>
+      <c r="M22" s="186"/>
+      <c r="N22" s="186"/>
+      <c r="O22" s="186"/>
+    </row>
+    <row r="23" spans="2:15">
+      <c r="B23" s="186"/>
+      <c r="C23" s="186"/>
+      <c r="D23" s="186"/>
+      <c r="E23" s="186"/>
+      <c r="G23" s="186"/>
+      <c r="H23" s="186"/>
+      <c r="I23" s="186"/>
+      <c r="J23" s="186"/>
+      <c r="L23" s="186"/>
+      <c r="M23" s="186"/>
+      <c r="N23" s="186"/>
+      <c r="O23" s="186"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B13:E23"/>
+    <mergeCell ref="G13:J23"/>
+    <mergeCell ref="L13:O23"/>
+    <mergeCell ref="B1:O1"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="G11:J11"/>
+    <mergeCell ref="L11:O11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="64" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38D0D34F-A68A-477F-96AD-F50038903927}">
+  <dimension ref="B1:AC15"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="1.21875" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" customWidth="1"/>
+    <col min="4" max="4" width="1.77734375" customWidth="1"/>
+    <col min="13" max="14" width="30" customWidth="1"/>
+    <col min="15" max="28" width="7.21875" customWidth="1"/>
+    <col min="29" max="29" width="1.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:29" ht="4.8" customHeight="1" thickBot="1"/>
+    <row r="2" spans="2:29" ht="19.95" customHeight="1" thickBot="1">
+      <c r="B2" s="286" t="s">
+        <v>106</v>
       </c>
       <c r="C2" s="287"/>
       <c r="D2" s="287"/>
@@ -5174,839 +5445,316 @@
       <c r="M2" s="287"/>
       <c r="N2" s="287"/>
       <c r="O2" s="287"/>
-    </row>
-    <row r="3" spans="2:15">
-      <c r="B3" t="s">
-        <v>19</v>
+      <c r="P2" s="287"/>
+      <c r="Q2" s="287"/>
+      <c r="R2" s="287"/>
+      <c r="S2" s="287"/>
+      <c r="T2" s="287"/>
+      <c r="U2" s="287"/>
+      <c r="V2" s="287"/>
+      <c r="W2" s="287"/>
+      <c r="X2" s="287"/>
+      <c r="Y2" s="287"/>
+      <c r="Z2" s="287"/>
+      <c r="AA2" s="287"/>
+      <c r="AB2" s="288"/>
+      <c r="AC2" s="178"/>
+    </row>
+    <row r="3" spans="2:29" ht="15" customHeight="1">
+      <c r="B3" s="177"/>
+      <c r="AB3" s="172"/>
+    </row>
+    <row r="4" spans="2:29" ht="15" customHeight="1">
+      <c r="B4" s="171" t="s">
+        <v>107</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D4" s="173" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="2:15">
-      <c r="B4" t="s">
-        <v>21</v>
+      <c r="AB4" s="172"/>
+    </row>
+    <row r="5" spans="2:29" ht="15" customHeight="1">
+      <c r="B5" s="171" t="s">
+        <v>108</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D5" s="173" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="2:15">
-      <c r="B5" t="s">
-        <v>22</v>
+      <c r="AB5" s="172"/>
+    </row>
+    <row r="6" spans="2:29" ht="15" customHeight="1">
+      <c r="B6" s="171" t="s">
+        <v>109</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D6" s="173" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="2:15">
-      <c r="B6" t="s">
-        <v>23</v>
+      <c r="AB6" s="172"/>
+    </row>
+    <row r="7" spans="2:29" ht="15" customHeight="1">
+      <c r="B7" s="171" t="s">
+        <v>45</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D7" s="173" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="2:15">
-      <c r="B7" t="s">
-        <v>24</v>
+      <c r="AB7" s="172"/>
+    </row>
+    <row r="8" spans="2:29" ht="15" customHeight="1">
+      <c r="B8" s="171" t="s">
+        <v>47</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D8" s="173" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="2:15">
-      <c r="B8" t="s">
-        <v>25</v>
+      <c r="AB8" s="172"/>
+    </row>
+    <row r="9" spans="2:29" ht="15" customHeight="1">
+      <c r="B9" s="171" t="s">
+        <v>110</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D9" s="173" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="2:15" ht="4.95" customHeight="1"/>
-    <row r="11" spans="2:15" s="58" customFormat="1">
-      <c r="B11" s="269" t="s">
-        <v>105</v>
+      <c r="AB9" s="172"/>
+    </row>
+    <row r="10" spans="2:29" ht="15" customHeight="1">
+      <c r="B10" s="171" t="s">
+        <v>111</v>
       </c>
-      <c r="C11" s="269"/>
-      <c r="D11" s="269"/>
-      <c r="E11" s="269"/>
-      <c r="G11" s="269" t="s">
-        <v>105</v>
-      </c>
-      <c r="H11" s="269"/>
-      <c r="I11" s="269"/>
-      <c r="J11" s="269"/>
-      <c r="L11" s="269" t="s">
-        <v>105</v>
-      </c>
-      <c r="M11" s="269"/>
-      <c r="N11" s="269"/>
-      <c r="O11" s="269"/>
-    </row>
-    <row r="12" spans="2:15" ht="4.95" customHeight="1"/>
-    <row r="13" spans="2:15">
-      <c r="B13" s="177"/>
-      <c r="C13" s="177"/>
-      <c r="D13" s="177"/>
-      <c r="E13" s="177"/>
-      <c r="G13" s="177"/>
-      <c r="H13" s="177"/>
-      <c r="I13" s="177"/>
-      <c r="J13" s="177"/>
-      <c r="L13" s="177"/>
-      <c r="M13" s="177"/>
-      <c r="N13" s="177"/>
-      <c r="O13" s="177"/>
-    </row>
-    <row r="14" spans="2:15">
-      <c r="B14" s="177"/>
-      <c r="C14" s="177"/>
-      <c r="D14" s="177"/>
-      <c r="E14" s="177"/>
-      <c r="G14" s="177"/>
-      <c r="H14" s="177"/>
-      <c r="I14" s="177"/>
-      <c r="J14" s="177"/>
-      <c r="L14" s="177"/>
-      <c r="M14" s="177"/>
-      <c r="N14" s="177"/>
-      <c r="O14" s="177"/>
-    </row>
-    <row r="15" spans="2:15">
-      <c r="B15" s="177"/>
-      <c r="C15" s="177"/>
-      <c r="D15" s="177"/>
-      <c r="E15" s="177"/>
-      <c r="G15" s="177"/>
-      <c r="H15" s="177"/>
-      <c r="I15" s="177"/>
-      <c r="J15" s="177"/>
-      <c r="L15" s="177"/>
-      <c r="M15" s="177"/>
-      <c r="N15" s="177"/>
-      <c r="O15" s="177"/>
-    </row>
-    <row r="16" spans="2:15">
-      <c r="B16" s="177"/>
-      <c r="C16" s="177"/>
-      <c r="D16" s="177"/>
-      <c r="E16" s="177"/>
-      <c r="G16" s="177"/>
-      <c r="H16" s="177"/>
-      <c r="I16" s="177"/>
-      <c r="J16" s="177"/>
-      <c r="L16" s="177"/>
-      <c r="M16" s="177"/>
-      <c r="N16" s="177"/>
-      <c r="O16" s="177"/>
-    </row>
-    <row r="17" spans="2:15">
-      <c r="B17" s="177"/>
-      <c r="C17" s="177"/>
-      <c r="D17" s="177"/>
-      <c r="E17" s="177"/>
-      <c r="G17" s="177"/>
-      <c r="H17" s="177"/>
-      <c r="I17" s="177"/>
-      <c r="J17" s="177"/>
-      <c r="L17" s="177"/>
-      <c r="M17" s="177"/>
-      <c r="N17" s="177"/>
-      <c r="O17" s="177"/>
-    </row>
-    <row r="18" spans="2:15">
-      <c r="B18" s="177"/>
-      <c r="C18" s="177"/>
-      <c r="D18" s="177"/>
-      <c r="E18" s="177"/>
-      <c r="G18" s="177"/>
-      <c r="H18" s="177"/>
-      <c r="I18" s="177"/>
-      <c r="J18" s="177"/>
-      <c r="L18" s="177"/>
-      <c r="M18" s="177"/>
-      <c r="N18" s="177"/>
-      <c r="O18" s="177"/>
-    </row>
-    <row r="19" spans="2:15">
-      <c r="B19" s="177"/>
-      <c r="C19" s="177"/>
-      <c r="D19" s="177"/>
-      <c r="E19" s="177"/>
-      <c r="G19" s="177"/>
-      <c r="H19" s="177"/>
-      <c r="I19" s="177"/>
-      <c r="J19" s="177"/>
-      <c r="L19" s="177"/>
-      <c r="M19" s="177"/>
-      <c r="N19" s="177"/>
-      <c r="O19" s="177"/>
-    </row>
-    <row r="20" spans="2:15">
-      <c r="B20" s="177"/>
-      <c r="C20" s="177"/>
-      <c r="D20" s="177"/>
-      <c r="E20" s="177"/>
-      <c r="G20" s="177"/>
-      <c r="H20" s="177"/>
-      <c r="I20" s="177"/>
-      <c r="J20" s="177"/>
-      <c r="L20" s="177"/>
-      <c r="M20" s="177"/>
-      <c r="N20" s="177"/>
-      <c r="O20" s="177"/>
-    </row>
-    <row r="21" spans="2:15">
-      <c r="B21" s="177"/>
-      <c r="C21" s="177"/>
-      <c r="D21" s="177"/>
-      <c r="E21" s="177"/>
-      <c r="G21" s="177"/>
-      <c r="H21" s="177"/>
-      <c r="I21" s="177"/>
-      <c r="J21" s="177"/>
-      <c r="L21" s="177"/>
-      <c r="M21" s="177"/>
-      <c r="N21" s="177"/>
-      <c r="O21" s="177"/>
-    </row>
-    <row r="22" spans="2:15">
-      <c r="B22" s="177"/>
-      <c r="C22" s="177"/>
-      <c r="D22" s="177"/>
-      <c r="E22" s="177"/>
-      <c r="G22" s="177"/>
-      <c r="H22" s="177"/>
-      <c r="I22" s="177"/>
-      <c r="J22" s="177"/>
-      <c r="L22" s="177"/>
-      <c r="M22" s="177"/>
-      <c r="N22" s="177"/>
-      <c r="O22" s="177"/>
-    </row>
-    <row r="23" spans="2:15">
-      <c r="B23" s="177"/>
-      <c r="C23" s="177"/>
-      <c r="D23" s="177"/>
-      <c r="E23" s="177"/>
-      <c r="G23" s="177"/>
-      <c r="H23" s="177"/>
-      <c r="I23" s="177"/>
-      <c r="J23" s="177"/>
-      <c r="L23" s="177"/>
-      <c r="M23" s="177"/>
-      <c r="N23" s="177"/>
-      <c r="O23" s="177"/>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B1:O1"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="G11:J11"/>
-    <mergeCell ref="L11:O11"/>
-    <mergeCell ref="B13:E23"/>
-    <mergeCell ref="G13:J23"/>
-    <mergeCell ref="L13:O23"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="64" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38D0D34F-A68A-477F-96AD-F50038903927}">
-  <dimension ref="A1:AC15"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="1.21875" customWidth="1"/>
-    <col min="2" max="2" width="4.33203125" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" customWidth="1"/>
-    <col min="4" max="4" width="1.77734375" customWidth="1"/>
-    <col min="13" max="14" width="30" customWidth="1"/>
-    <col min="15" max="28" width="7.21875" customWidth="1"/>
-    <col min="29" max="29" width="1.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:29" ht="4.8" customHeight="1" thickBot="1">
-      <c r="A1" s="270"/>
-      <c r="B1" s="271"/>
-      <c r="C1" s="271"/>
-      <c r="D1" s="271"/>
-      <c r="E1" s="271"/>
-      <c r="F1" s="271"/>
-      <c r="G1" s="271"/>
-      <c r="H1" s="271"/>
-      <c r="I1" s="271"/>
-      <c r="J1" s="271"/>
-      <c r="K1" s="271"/>
-      <c r="L1" s="271"/>
-      <c r="M1" s="271"/>
-      <c r="N1" s="271"/>
-      <c r="O1" s="271"/>
-      <c r="P1" s="271"/>
-      <c r="Q1" s="271"/>
-      <c r="R1" s="271"/>
-      <c r="S1" s="271"/>
-      <c r="T1" s="271"/>
-      <c r="U1" s="271"/>
-      <c r="V1" s="271"/>
-      <c r="W1" s="271"/>
-      <c r="X1" s="271"/>
-      <c r="Y1" s="271"/>
-      <c r="Z1" s="271"/>
-      <c r="AA1" s="271"/>
-      <c r="AB1" s="271"/>
-      <c r="AC1" s="271"/>
-    </row>
-    <row r="2" spans="1:29" ht="19.95" customHeight="1" thickBot="1">
-      <c r="A2" s="270"/>
-      <c r="B2" s="312" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="313"/>
-      <c r="D2" s="313"/>
-      <c r="E2" s="313"/>
-      <c r="F2" s="313"/>
-      <c r="G2" s="313"/>
-      <c r="H2" s="313"/>
-      <c r="I2" s="313"/>
-      <c r="J2" s="313"/>
-      <c r="K2" s="313"/>
-      <c r="L2" s="313"/>
-      <c r="M2" s="313"/>
-      <c r="N2" s="313"/>
-      <c r="O2" s="313"/>
-      <c r="P2" s="313"/>
-      <c r="Q2" s="313"/>
-      <c r="R2" s="313"/>
-      <c r="S2" s="313"/>
-      <c r="T2" s="313"/>
-      <c r="U2" s="313"/>
-      <c r="V2" s="313"/>
-      <c r="W2" s="313"/>
-      <c r="X2" s="313"/>
-      <c r="Y2" s="313"/>
-      <c r="Z2" s="313"/>
-      <c r="AA2" s="313"/>
-      <c r="AB2" s="314"/>
-      <c r="AC2" s="279"/>
-    </row>
-    <row r="3" spans="1:29" ht="15" customHeight="1">
-      <c r="A3" s="270"/>
-      <c r="B3" s="278"/>
-      <c r="C3" s="271"/>
-      <c r="D3" s="271"/>
-      <c r="E3" s="271"/>
-      <c r="F3" s="271"/>
-      <c r="G3" s="271"/>
-      <c r="H3" s="271"/>
-      <c r="I3" s="271"/>
-      <c r="J3" s="271"/>
-      <c r="K3" s="271"/>
-      <c r="L3" s="271"/>
-      <c r="M3" s="271"/>
-      <c r="N3" s="271"/>
-      <c r="O3" s="271"/>
-      <c r="P3" s="271"/>
-      <c r="Q3" s="271"/>
-      <c r="R3" s="271"/>
-      <c r="S3" s="271"/>
-      <c r="T3" s="271"/>
-      <c r="U3" s="271"/>
-      <c r="V3" s="271"/>
-      <c r="W3" s="271"/>
-      <c r="X3" s="271"/>
-      <c r="Y3" s="271"/>
-      <c r="Z3" s="271"/>
-      <c r="AA3" s="271"/>
-      <c r="AB3" s="273"/>
-      <c r="AC3" s="271"/>
-    </row>
-    <row r="4" spans="1:29" ht="15" customHeight="1">
-      <c r="A4" s="270"/>
-      <c r="B4" s="272" t="s">
-        <v>107</v>
-      </c>
-      <c r="C4" s="271"/>
-      <c r="D4" s="274" t="s">
+      <c r="D10" s="173" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="271"/>
-      <c r="F4" s="271"/>
-      <c r="G4" s="271"/>
-      <c r="H4" s="271"/>
-      <c r="I4" s="271"/>
-      <c r="J4" s="271"/>
-      <c r="K4" s="271"/>
-      <c r="L4" s="271"/>
-      <c r="M4" s="271"/>
-      <c r="N4" s="271"/>
-      <c r="O4" s="271"/>
-      <c r="P4" s="271"/>
-      <c r="Q4" s="271"/>
-      <c r="R4" s="271"/>
-      <c r="S4" s="271"/>
-      <c r="T4" s="271"/>
-      <c r="U4" s="271"/>
-      <c r="V4" s="271"/>
-      <c r="W4" s="271"/>
-      <c r="X4" s="271"/>
-      <c r="Y4" s="271"/>
-      <c r="Z4" s="271"/>
-      <c r="AA4" s="271"/>
-      <c r="AB4" s="273"/>
-      <c r="AC4" s="271"/>
-    </row>
-    <row r="5" spans="1:29" ht="15" customHeight="1">
-      <c r="A5" s="270"/>
-      <c r="B5" s="272" t="s">
-        <v>108</v>
-      </c>
-      <c r="C5" s="271"/>
-      <c r="D5" s="274" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="271"/>
-      <c r="F5" s="271"/>
-      <c r="G5" s="271"/>
-      <c r="H5" s="271"/>
-      <c r="I5" s="271"/>
-      <c r="J5" s="271"/>
-      <c r="K5" s="271"/>
-      <c r="L5" s="271"/>
-      <c r="M5" s="271"/>
-      <c r="N5" s="271"/>
-      <c r="O5" s="271"/>
-      <c r="P5" s="271"/>
-      <c r="Q5" s="271"/>
-      <c r="R5" s="271"/>
-      <c r="S5" s="271"/>
-      <c r="T5" s="271"/>
-      <c r="U5" s="271"/>
-      <c r="V5" s="271"/>
-      <c r="W5" s="271"/>
-      <c r="X5" s="271"/>
-      <c r="Y5" s="271"/>
-      <c r="Z5" s="271"/>
-      <c r="AA5" s="271"/>
-      <c r="AB5" s="273"/>
-      <c r="AC5" s="271"/>
-    </row>
-    <row r="6" spans="1:29" ht="15" customHeight="1">
-      <c r="A6" s="270"/>
-      <c r="B6" s="272" t="s">
-        <v>109</v>
-      </c>
-      <c r="C6" s="271"/>
-      <c r="D6" s="274" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="271"/>
-      <c r="F6" s="271"/>
-      <c r="G6" s="271"/>
-      <c r="H6" s="271"/>
-      <c r="I6" s="271"/>
-      <c r="J6" s="271"/>
-      <c r="K6" s="271"/>
-      <c r="L6" s="271"/>
-      <c r="M6" s="271"/>
-      <c r="N6" s="271"/>
-      <c r="O6" s="271"/>
-      <c r="P6" s="271"/>
-      <c r="Q6" s="271"/>
-      <c r="R6" s="271"/>
-      <c r="S6" s="271"/>
-      <c r="T6" s="271"/>
-      <c r="U6" s="271"/>
-      <c r="V6" s="271"/>
-      <c r="W6" s="271"/>
-      <c r="X6" s="271"/>
-      <c r="Y6" s="271"/>
-      <c r="Z6" s="271"/>
-      <c r="AA6" s="271"/>
-      <c r="AB6" s="273"/>
-      <c r="AC6" s="271"/>
-    </row>
-    <row r="7" spans="1:29" ht="15" customHeight="1">
-      <c r="A7" s="270"/>
-      <c r="B7" s="272" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="271"/>
-      <c r="D7" s="274" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="271"/>
-      <c r="F7" s="271"/>
-      <c r="G7" s="271"/>
-      <c r="H7" s="271"/>
-      <c r="I7" s="271"/>
-      <c r="J7" s="271"/>
-      <c r="K7" s="271"/>
-      <c r="L7" s="271"/>
-      <c r="M7" s="271"/>
-      <c r="N7" s="271"/>
-      <c r="O7" s="271"/>
-      <c r="P7" s="271"/>
-      <c r="Q7" s="271"/>
-      <c r="R7" s="271"/>
-      <c r="S7" s="271"/>
-      <c r="T7" s="271"/>
-      <c r="U7" s="271"/>
-      <c r="V7" s="271"/>
-      <c r="W7" s="271"/>
-      <c r="X7" s="271"/>
-      <c r="Y7" s="271"/>
-      <c r="Z7" s="271"/>
-      <c r="AA7" s="271"/>
-      <c r="AB7" s="273"/>
-      <c r="AC7" s="271"/>
-    </row>
-    <row r="8" spans="1:29" ht="15" customHeight="1">
-      <c r="A8" s="270"/>
-      <c r="B8" s="272" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="271"/>
-      <c r="D8" s="274" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="271"/>
-      <c r="F8" s="271"/>
-      <c r="G8" s="271"/>
-      <c r="H8" s="271"/>
-      <c r="I8" s="271"/>
-      <c r="J8" s="271"/>
-      <c r="K8" s="271"/>
-      <c r="L8" s="271"/>
-      <c r="M8" s="271"/>
-      <c r="N8" s="271"/>
-      <c r="O8" s="271"/>
-      <c r="P8" s="271"/>
-      <c r="Q8" s="271"/>
-      <c r="R8" s="271"/>
-      <c r="S8" s="271"/>
-      <c r="T8" s="271"/>
-      <c r="U8" s="271"/>
-      <c r="V8" s="271"/>
-      <c r="W8" s="271"/>
-      <c r="X8" s="271"/>
-      <c r="Y8" s="271"/>
-      <c r="Z8" s="271"/>
-      <c r="AA8" s="271"/>
-      <c r="AB8" s="273"/>
-      <c r="AC8" s="271"/>
-    </row>
-    <row r="9" spans="1:29" ht="15" customHeight="1">
-      <c r="A9" s="270"/>
-      <c r="B9" s="272" t="s">
-        <v>110</v>
-      </c>
-      <c r="C9" s="271"/>
-      <c r="D9" s="274" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="271"/>
-      <c r="F9" s="271"/>
-      <c r="G9" s="271"/>
-      <c r="H9" s="271"/>
-      <c r="I9" s="271"/>
-      <c r="J9" s="271"/>
-      <c r="K9" s="271"/>
-      <c r="L9" s="271"/>
-      <c r="M9" s="271"/>
-      <c r="N9" s="271"/>
-      <c r="O9" s="271"/>
-      <c r="P9" s="271"/>
-      <c r="Q9" s="271"/>
-      <c r="R9" s="271"/>
-      <c r="S9" s="271"/>
-      <c r="T9" s="271"/>
-      <c r="U9" s="271"/>
-      <c r="V9" s="271"/>
-      <c r="W9" s="271"/>
-      <c r="X9" s="271"/>
-      <c r="Y9" s="271"/>
-      <c r="Z9" s="271"/>
-      <c r="AA9" s="271"/>
-      <c r="AB9" s="273"/>
-      <c r="AC9" s="271"/>
-    </row>
-    <row r="10" spans="1:29" ht="15" customHeight="1">
-      <c r="A10" s="270"/>
-      <c r="B10" s="272" t="s">
-        <v>111</v>
-      </c>
-      <c r="C10" s="271"/>
-      <c r="D10" s="274" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="271"/>
-      <c r="F10" s="271"/>
-      <c r="G10" s="271"/>
-      <c r="H10" s="271"/>
-      <c r="I10" s="271"/>
-      <c r="J10" s="271"/>
-      <c r="K10" s="271"/>
-      <c r="L10" s="271"/>
-      <c r="M10" s="271"/>
-      <c r="N10" s="271"/>
-      <c r="O10" s="271"/>
-      <c r="P10" s="271"/>
-      <c r="Q10" s="271"/>
-      <c r="R10" s="271"/>
-      <c r="S10" s="271"/>
-      <c r="T10" s="271"/>
-      <c r="U10" s="271"/>
-      <c r="V10" s="271"/>
-      <c r="W10" s="271"/>
-      <c r="X10" s="271"/>
-      <c r="Y10" s="271"/>
-      <c r="Z10" s="271"/>
-      <c r="AA10" s="271"/>
-      <c r="AB10" s="273"/>
-      <c r="AC10" s="271"/>
-    </row>
-    <row r="11" spans="1:29" ht="15" customHeight="1" thickBot="1">
-      <c r="A11" s="270"/>
-      <c r="B11" s="275"/>
-      <c r="C11" s="276"/>
-      <c r="D11" s="276"/>
-      <c r="E11" s="276"/>
-      <c r="F11" s="276"/>
-      <c r="G11" s="276"/>
-      <c r="H11" s="276"/>
-      <c r="I11" s="276"/>
-      <c r="J11" s="276"/>
-      <c r="K11" s="276"/>
-      <c r="L11" s="276"/>
-      <c r="M11" s="276"/>
-      <c r="N11" s="276"/>
-      <c r="O11" s="276"/>
-      <c r="P11" s="276"/>
-      <c r="Q11" s="276"/>
-      <c r="R11" s="276"/>
-      <c r="S11" s="276"/>
-      <c r="T11" s="276"/>
-      <c r="U11" s="276"/>
-      <c r="V11" s="276"/>
-      <c r="W11" s="276"/>
-      <c r="X11" s="276"/>
-      <c r="Y11" s="276"/>
-      <c r="Z11" s="276"/>
-      <c r="AA11" s="276"/>
-      <c r="AB11" s="277"/>
-      <c r="AC11" s="271"/>
-    </row>
-    <row r="12" spans="1:29" ht="15" customHeight="1">
-      <c r="A12" s="270"/>
-      <c r="B12" s="288" t="s">
+      <c r="AB10" s="172"/>
+    </row>
+    <row r="11" spans="2:29" ht="15" customHeight="1" thickBot="1">
+      <c r="B11" s="174"/>
+      <c r="C11" s="175"/>
+      <c r="D11" s="175"/>
+      <c r="E11" s="175"/>
+      <c r="F11" s="175"/>
+      <c r="G11" s="175"/>
+      <c r="H11" s="175"/>
+      <c r="I11" s="175"/>
+      <c r="J11" s="175"/>
+      <c r="K11" s="175"/>
+      <c r="L11" s="175"/>
+      <c r="M11" s="175"/>
+      <c r="N11" s="175"/>
+      <c r="O11" s="175"/>
+      <c r="P11" s="175"/>
+      <c r="Q11" s="175"/>
+      <c r="R11" s="175"/>
+      <c r="S11" s="175"/>
+      <c r="T11" s="175"/>
+      <c r="U11" s="175"/>
+      <c r="V11" s="175"/>
+      <c r="W11" s="175"/>
+      <c r="X11" s="175"/>
+      <c r="Y11" s="175"/>
+      <c r="Z11" s="175"/>
+      <c r="AA11" s="175"/>
+      <c r="AB11" s="176"/>
+    </row>
+    <row r="12" spans="2:29" ht="15" customHeight="1">
+      <c r="B12" s="298" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="289" t="s">
+      <c r="C12" s="300" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="290"/>
-      <c r="E12" s="290"/>
-      <c r="F12" s="290"/>
-      <c r="G12" s="290"/>
-      <c r="H12" s="290"/>
-      <c r="I12" s="290"/>
-      <c r="J12" s="290"/>
-      <c r="K12" s="290"/>
-      <c r="L12" s="291"/>
-      <c r="M12" s="292" t="s">
+      <c r="D12" s="301"/>
+      <c r="E12" s="301"/>
+      <c r="F12" s="301"/>
+      <c r="G12" s="301"/>
+      <c r="H12" s="301"/>
+      <c r="I12" s="301"/>
+      <c r="J12" s="301"/>
+      <c r="K12" s="301"/>
+      <c r="L12" s="302"/>
+      <c r="M12" s="306" t="s">
         <v>113</v>
       </c>
-      <c r="N12" s="292" t="s">
+      <c r="N12" s="306" t="s">
         <v>34</v>
       </c>
-      <c r="O12" s="293" t="s">
+      <c r="O12" s="311" t="s">
         <v>114</v>
       </c>
-      <c r="P12" s="293"/>
-      <c r="Q12" s="293"/>
-      <c r="R12" s="293"/>
-      <c r="S12" s="293"/>
-      <c r="T12" s="293"/>
-      <c r="U12" s="293"/>
-      <c r="V12" s="293"/>
-      <c r="W12" s="293"/>
-      <c r="X12" s="293"/>
-      <c r="Y12" s="293"/>
-      <c r="Z12" s="293"/>
-      <c r="AA12" s="293"/>
-      <c r="AB12" s="294"/>
-      <c r="AC12" s="271"/>
-    </row>
-    <row r="13" spans="1:29" ht="15" customHeight="1">
-      <c r="A13" s="270"/>
-      <c r="B13" s="295"/>
-      <c r="C13" s="296"/>
-      <c r="D13" s="297"/>
-      <c r="E13" s="297"/>
-      <c r="F13" s="297"/>
-      <c r="G13" s="297"/>
-      <c r="H13" s="297"/>
-      <c r="I13" s="297"/>
-      <c r="J13" s="297"/>
-      <c r="K13" s="297"/>
-      <c r="L13" s="298"/>
-      <c r="M13" s="299"/>
-      <c r="N13" s="299"/>
-      <c r="O13" s="300" t="s">
+      <c r="P12" s="311"/>
+      <c r="Q12" s="311"/>
+      <c r="R12" s="311"/>
+      <c r="S12" s="311"/>
+      <c r="T12" s="311"/>
+      <c r="U12" s="311"/>
+      <c r="V12" s="311"/>
+      <c r="W12" s="311"/>
+      <c r="X12" s="311"/>
+      <c r="Y12" s="311"/>
+      <c r="Z12" s="311"/>
+      <c r="AA12" s="311"/>
+      <c r="AB12" s="312"/>
+    </row>
+    <row r="13" spans="2:29" ht="15" customHeight="1">
+      <c r="B13" s="299"/>
+      <c r="C13" s="303"/>
+      <c r="D13" s="304"/>
+      <c r="E13" s="304"/>
+      <c r="F13" s="304"/>
+      <c r="G13" s="304"/>
+      <c r="H13" s="304"/>
+      <c r="I13" s="304"/>
+      <c r="J13" s="304"/>
+      <c r="K13" s="304"/>
+      <c r="L13" s="305"/>
+      <c r="M13" s="307"/>
+      <c r="N13" s="307"/>
+      <c r="O13" s="308" t="s">
         <v>115</v>
       </c>
-      <c r="P13" s="301"/>
-      <c r="Q13" s="302"/>
-      <c r="R13" s="300" t="s">
+      <c r="P13" s="309"/>
+      <c r="Q13" s="310"/>
+      <c r="R13" s="308" t="s">
         <v>116</v>
       </c>
-      <c r="S13" s="301"/>
-      <c r="T13" s="302"/>
-      <c r="U13" s="300" t="s">
+      <c r="S13" s="309"/>
+      <c r="T13" s="310"/>
+      <c r="U13" s="308" t="s">
         <v>117</v>
       </c>
-      <c r="V13" s="301"/>
-      <c r="W13" s="302"/>
-      <c r="X13" s="303" t="s">
+      <c r="V13" s="309"/>
+      <c r="W13" s="310"/>
+      <c r="X13" s="289" t="s">
         <v>118</v>
       </c>
-      <c r="Y13" s="304" t="s">
+      <c r="Y13" s="183" t="s">
         <v>119</v>
       </c>
-      <c r="Z13" s="305" t="s">
+      <c r="Z13" s="184" t="s">
         <v>119</v>
       </c>
-      <c r="AA13" s="306" t="s">
+      <c r="AA13" s="291" t="s">
         <v>120</v>
       </c>
-      <c r="AB13" s="307" t="s">
+      <c r="AB13" s="293" t="s">
         <v>121</v>
       </c>
-      <c r="AC13" s="271"/>
-    </row>
-    <row r="14" spans="1:29" ht="15" customHeight="1">
-      <c r="A14" s="270"/>
-      <c r="B14" s="295"/>
-      <c r="C14" s="296"/>
-      <c r="D14" s="297"/>
-      <c r="E14" s="297"/>
-      <c r="F14" s="297"/>
-      <c r="G14" s="297"/>
-      <c r="H14" s="297"/>
-      <c r="I14" s="297"/>
-      <c r="J14" s="297"/>
-      <c r="K14" s="297"/>
-      <c r="L14" s="298"/>
-      <c r="M14" s="308"/>
-      <c r="N14" s="308"/>
-      <c r="O14" s="309" t="s">
+    </row>
+    <row r="14" spans="2:29" ht="15" customHeight="1">
+      <c r="B14" s="299"/>
+      <c r="C14" s="303"/>
+      <c r="D14" s="304"/>
+      <c r="E14" s="304"/>
+      <c r="F14" s="304"/>
+      <c r="G14" s="304"/>
+      <c r="H14" s="304"/>
+      <c r="I14" s="304"/>
+      <c r="J14" s="304"/>
+      <c r="K14" s="304"/>
+      <c r="L14" s="305"/>
+      <c r="M14" s="290"/>
+      <c r="N14" s="290"/>
+      <c r="O14" s="185" t="s">
         <v>122</v>
       </c>
-      <c r="P14" s="309" t="s">
+      <c r="P14" s="185" t="s">
         <v>123</v>
       </c>
-      <c r="Q14" s="309" t="s">
+      <c r="Q14" s="185" t="s">
         <v>124</v>
       </c>
-      <c r="R14" s="309" t="s">
+      <c r="R14" s="185" t="s">
         <v>125</v>
       </c>
-      <c r="S14" s="309" t="s">
+      <c r="S14" s="185" t="s">
         <v>126</v>
       </c>
-      <c r="T14" s="309" t="s">
+      <c r="T14" s="185" t="s">
         <v>124</v>
       </c>
-      <c r="U14" s="309" t="s">
+      <c r="U14" s="185" t="s">
         <v>127</v>
       </c>
-      <c r="V14" s="309" t="s">
+      <c r="V14" s="185" t="s">
         <v>128</v>
       </c>
-      <c r="W14" s="309" t="s">
+      <c r="W14" s="185" t="s">
         <v>129</v>
       </c>
-      <c r="X14" s="308"/>
-      <c r="Y14" s="304" t="s">
+      <c r="X14" s="290"/>
+      <c r="Y14" s="183" t="s">
         <v>130</v>
       </c>
-      <c r="Z14" s="309" t="s">
+      <c r="Z14" s="185" t="s">
         <v>131</v>
       </c>
-      <c r="AA14" s="310"/>
-      <c r="AB14" s="311"/>
-      <c r="AC14" s="271"/>
-    </row>
-    <row r="15" spans="1:29" ht="15" customHeight="1" thickBot="1">
-      <c r="A15" s="270"/>
-      <c r="B15" s="280">
+      <c r="AA14" s="292"/>
+      <c r="AB14" s="294"/>
+    </row>
+    <row r="15" spans="2:29" ht="15" customHeight="1" thickBot="1">
+      <c r="B15" s="179">
         <v>1</v>
       </c>
-      <c r="C15" s="281">
+      <c r="C15" s="295">
         <v>2</v>
       </c>
-      <c r="D15" s="282"/>
-      <c r="E15" s="282"/>
-      <c r="F15" s="282"/>
-      <c r="G15" s="282"/>
-      <c r="H15" s="282"/>
-      <c r="I15" s="282"/>
-      <c r="J15" s="282"/>
-      <c r="K15" s="282"/>
-      <c r="L15" s="283"/>
-      <c r="M15" s="284">
+      <c r="D15" s="296"/>
+      <c r="E15" s="296"/>
+      <c r="F15" s="296"/>
+      <c r="G15" s="296"/>
+      <c r="H15" s="296"/>
+      <c r="I15" s="296"/>
+      <c r="J15" s="296"/>
+      <c r="K15" s="296"/>
+      <c r="L15" s="297"/>
+      <c r="M15" s="180">
         <v>3</v>
       </c>
-      <c r="N15" s="284">
+      <c r="N15" s="180">
         <v>4</v>
       </c>
-      <c r="O15" s="285">
+      <c r="O15" s="181">
         <v>5</v>
       </c>
-      <c r="P15" s="285">
+      <c r="P15" s="181">
         <v>6</v>
       </c>
-      <c r="Q15" s="285">
+      <c r="Q15" s="181">
         <v>7</v>
       </c>
-      <c r="R15" s="285">
+      <c r="R15" s="181">
         <v>8</v>
       </c>
-      <c r="S15" s="285">
+      <c r="S15" s="181">
         <v>9</v>
       </c>
-      <c r="T15" s="285">
+      <c r="T15" s="181">
         <v>10</v>
       </c>
-      <c r="U15" s="285">
+      <c r="U15" s="181">
         <v>11</v>
       </c>
-      <c r="V15" s="285">
+      <c r="V15" s="181">
         <v>12</v>
       </c>
-      <c r="W15" s="285">
+      <c r="W15" s="181">
         <v>13</v>
       </c>
-      <c r="X15" s="285">
+      <c r="X15" s="181">
         <v>14</v>
       </c>
-      <c r="Y15" s="285">
+      <c r="Y15" s="181">
         <v>15</v>
       </c>
-      <c r="Z15" s="285">
+      <c r="Z15" s="181">
         <v>16</v>
       </c>
-      <c r="AA15" s="285">
+      <c r="AA15" s="181">
         <v>17</v>
       </c>
-      <c r="AB15" s="286">
+      <c r="AB15" s="182">
         <v>18</v>
       </c>
-      <c r="AC15" s="271"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -6048,38 +5796,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
-      <c r="E1" s="174"/>
-      <c r="F1" s="174"/>
-      <c r="G1" s="174"/>
-      <c r="H1" s="174"/>
-      <c r="I1" s="174"/>
+      <c r="B1" s="192"/>
+      <c r="C1" s="192"/>
+      <c r="D1" s="192"/>
+      <c r="E1" s="192"/>
+      <c r="F1" s="192"/>
+      <c r="G1" s="192"/>
+      <c r="H1" s="192"/>
+      <c r="I1" s="192"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="171" t="s">
+      <c r="B2" s="189" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="171"/>
-      <c r="D2" s="171"/>
-      <c r="E2" s="171"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="171"/>
-      <c r="H2" s="171"/>
-      <c r="I2" s="171"/>
+      <c r="C2" s="189"/>
+      <c r="D2" s="189"/>
+      <c r="E2" s="189"/>
+      <c r="F2" s="189"/>
+      <c r="G2" s="189"/>
+      <c r="H2" s="189"/>
+      <c r="I2" s="189"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="172" t="s">
+      <c r="B3" s="190" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="172"/>
-      <c r="D3" s="172"/>
-      <c r="E3" s="172"/>
-      <c r="F3" s="172"/>
-      <c r="G3" s="172"/>
-      <c r="H3" s="172"/>
-      <c r="I3" s="172"/>
+      <c r="C3" s="190"/>
+      <c r="D3" s="190"/>
+      <c r="E3" s="190"/>
+      <c r="F3" s="190"/>
+      <c r="G3" s="190"/>
+      <c r="H3" s="190"/>
+      <c r="I3" s="190"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -6087,10 +5835,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="173" t="s">
+      <c r="C5" s="191" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="173"/>
+      <c r="D5" s="191"/>
       <c r="E5" s="11" t="s">
         <v>38</v>
       </c>
@@ -14477,63 +14225,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
-      <c r="E1" s="174"/>
-      <c r="F1" s="174"/>
-      <c r="G1" s="174"/>
-      <c r="H1" s="174"/>
-      <c r="I1" s="174"/>
-      <c r="J1" s="174"/>
-      <c r="K1" s="174"/>
-      <c r="L1" s="174"/>
-      <c r="M1" s="174"/>
-      <c r="N1" s="174"/>
+      <c r="B1" s="192"/>
+      <c r="C1" s="192"/>
+      <c r="D1" s="192"/>
+      <c r="E1" s="192"/>
+      <c r="F1" s="192"/>
+      <c r="G1" s="192"/>
+      <c r="H1" s="192"/>
+      <c r="I1" s="192"/>
+      <c r="J1" s="192"/>
+      <c r="K1" s="192"/>
+      <c r="L1" s="192"/>
+      <c r="M1" s="192"/>
+      <c r="N1" s="192"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="171" t="s">
+      <c r="B2" s="189" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="171"/>
-      <c r="D2" s="171"/>
-      <c r="E2" s="171"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="171"/>
-      <c r="H2" s="171"/>
-      <c r="I2" s="171"/>
-      <c r="J2" s="171"/>
-      <c r="K2" s="171"/>
-      <c r="L2" s="171"/>
-      <c r="M2" s="171"/>
-      <c r="N2" s="171"/>
+      <c r="C2" s="189"/>
+      <c r="D2" s="189"/>
+      <c r="E2" s="189"/>
+      <c r="F2" s="189"/>
+      <c r="G2" s="189"/>
+      <c r="H2" s="189"/>
+      <c r="I2" s="189"/>
+      <c r="J2" s="189"/>
+      <c r="K2" s="189"/>
+      <c r="L2" s="189"/>
+      <c r="M2" s="189"/>
+      <c r="N2" s="189"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="172" t="s">
+      <c r="B3" s="190" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="172"/>
-      <c r="D3" s="172"/>
-      <c r="E3" s="172"/>
-      <c r="F3" s="172"/>
-      <c r="G3" s="172"/>
-      <c r="H3" s="172"/>
-      <c r="I3" s="172"/>
-      <c r="J3" s="172"/>
-      <c r="K3" s="172"/>
-      <c r="L3" s="172"/>
-      <c r="M3" s="172"/>
-      <c r="N3" s="172"/>
+      <c r="C3" s="190"/>
+      <c r="D3" s="190"/>
+      <c r="E3" s="190"/>
+      <c r="F3" s="190"/>
+      <c r="G3" s="190"/>
+      <c r="H3" s="190"/>
+      <c r="I3" s="190"/>
+      <c r="J3" s="190"/>
+      <c r="K3" s="190"/>
+      <c r="L3" s="190"/>
+      <c r="M3" s="190"/>
+      <c r="N3" s="190"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="175" t="s">
+      <c r="C5" s="193" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="175"/>
+      <c r="D5" s="193"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -16737,35 +16485,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
-      <c r="E1" s="174"/>
-      <c r="F1" s="174"/>
-      <c r="G1" s="174"/>
-      <c r="H1" s="174"/>
+      <c r="B1" s="192"/>
+      <c r="C1" s="192"/>
+      <c r="D1" s="192"/>
+      <c r="E1" s="192"/>
+      <c r="F1" s="192"/>
+      <c r="G1" s="192"/>
+      <c r="H1" s="192"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="171" t="s">
+      <c r="B2" s="189" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="171"/>
-      <c r="D2" s="171"/>
-      <c r="E2" s="171"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="171"/>
-      <c r="H2" s="171"/>
+      <c r="C2" s="189"/>
+      <c r="D2" s="189"/>
+      <c r="E2" s="189"/>
+      <c r="F2" s="189"/>
+      <c r="G2" s="189"/>
+      <c r="H2" s="189"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="172" t="s">
+      <c r="B3" s="190" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="172"/>
-      <c r="D3" s="172"/>
-      <c r="E3" s="172"/>
-      <c r="F3" s="172"/>
-      <c r="G3" s="172"/>
-      <c r="H3" s="172"/>
+      <c r="C3" s="190"/>
+      <c r="D3" s="190"/>
+      <c r="E3" s="190"/>
+      <c r="F3" s="190"/>
+      <c r="G3" s="190"/>
+      <c r="H3" s="190"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -40859,30 +40607,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="178"/>
-      <c r="C1" s="178"/>
-      <c r="D1" s="178"/>
-      <c r="E1" s="178"/>
-      <c r="F1" s="178"/>
-      <c r="G1" s="178"/>
-      <c r="H1" s="178"/>
-      <c r="I1" s="178"/>
-      <c r="J1" s="178"/>
-      <c r="K1" s="178"/>
+      <c r="B1" s="195"/>
+      <c r="C1" s="195"/>
+      <c r="D1" s="195"/>
+      <c r="E1" s="195"/>
+      <c r="F1" s="195"/>
+      <c r="G1" s="195"/>
+      <c r="H1" s="195"/>
+      <c r="I1" s="195"/>
+      <c r="J1" s="195"/>
+      <c r="K1" s="195"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="176" t="s">
+      <c r="B2" s="194" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="177"/>
-      <c r="D2" s="177"/>
-      <c r="E2" s="177"/>
-      <c r="F2" s="177"/>
-      <c r="G2" s="177"/>
-      <c r="H2" s="177"/>
-      <c r="I2" s="177"/>
-      <c r="J2" s="177"/>
-      <c r="K2" s="177"/>
+      <c r="C2" s="186"/>
+      <c r="D2" s="186"/>
+      <c r="E2" s="186"/>
+      <c r="F2" s="186"/>
+      <c r="G2" s="186"/>
+      <c r="H2" s="186"/>
+      <c r="I2" s="186"/>
+      <c r="J2" s="186"/>
+      <c r="K2" s="186"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -41002,11 +40750,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="175" t="s">
+      <c r="C11" s="193" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="175"/>
-      <c r="E11" s="175"/>
+      <c r="D11" s="193"/>
+      <c r="E11" s="193"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -41062,26 +40810,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="111.6" customHeight="1">
-      <c r="B1" s="178"/>
-      <c r="C1" s="178"/>
-      <c r="D1" s="178"/>
-      <c r="E1" s="178"/>
-      <c r="F1" s="178"/>
-      <c r="G1" s="178"/>
-      <c r="H1" s="178"/>
-      <c r="I1" s="178"/>
+      <c r="B1" s="195"/>
+      <c r="C1" s="195"/>
+      <c r="D1" s="195"/>
+      <c r="E1" s="195"/>
+      <c r="F1" s="195"/>
+      <c r="G1" s="195"/>
+      <c r="H1" s="195"/>
+      <c r="I1" s="195"/>
     </row>
     <row r="2" spans="2:9" ht="22.95" customHeight="1">
-      <c r="B2" s="176" t="s">
+      <c r="B2" s="194" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="177"/>
-      <c r="D2" s="177"/>
-      <c r="E2" s="177"/>
-      <c r="F2" s="177"/>
-      <c r="G2" s="177"/>
-      <c r="H2" s="177"/>
-      <c r="I2" s="177"/>
+      <c r="C2" s="186"/>
+      <c r="D2" s="186"/>
+      <c r="E2" s="186"/>
+      <c r="F2" s="186"/>
+      <c r="G2" s="186"/>
+      <c r="H2" s="186"/>
+      <c r="I2" s="186"/>
     </row>
     <row r="3" spans="2:9" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -41191,12 +40939,12 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="175" t="s">
+      <c r="C11" s="193" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="175"/>
-      <c r="E11" s="175"/>
-      <c r="F11" s="175"/>
+      <c r="D11" s="193"/>
+      <c r="E11" s="193"/>
+      <c r="F11" s="193"/>
       <c r="G11" s="40" t="s">
         <v>29</v>
       </c>
@@ -41234,58 +40982,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="178"/>
-      <c r="C1" s="178"/>
-      <c r="D1" s="178"/>
-      <c r="E1" s="178"/>
-      <c r="F1" s="178"/>
+      <c r="B1" s="195"/>
+      <c r="C1" s="195"/>
+      <c r="D1" s="195"/>
+      <c r="E1" s="195"/>
+      <c r="F1" s="195"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="181" t="s">
+      <c r="B2" s="198" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="181"/>
-      <c r="D2" s="181"/>
-      <c r="E2" s="181"/>
-      <c r="F2" s="181"/>
+      <c r="C2" s="198"/>
+      <c r="D2" s="198"/>
+      <c r="E2" s="198"/>
+      <c r="F2" s="198"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="178"/>
-      <c r="C3" s="178"/>
-      <c r="D3" s="178"/>
-      <c r="E3" s="178"/>
-      <c r="F3" s="178"/>
+      <c r="B3" s="195"/>
+      <c r="C3" s="195"/>
+      <c r="D3" s="195"/>
+      <c r="E3" s="195"/>
+      <c r="F3" s="195"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="179" t="s">
+      <c r="B5" s="196" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="179" t="s">
+      <c r="C5" s="196" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="179" t="s">
+      <c r="D5" s="196" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="180" t="s">
+      <c r="E5" s="197" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="180" t="s">
+      <c r="F5" s="197" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="179"/>
-      <c r="C6" s="179"/>
-      <c r="D6" s="179"/>
-      <c r="E6" s="180"/>
-      <c r="F6" s="180"/>
+      <c r="B6" s="196"/>
+      <c r="C6" s="196"/>
+      <c r="D6" s="196"/>
+      <c r="E6" s="197"/>
+      <c r="F6" s="197"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="179"/>
-      <c r="C7" s="179"/>
-      <c r="D7" s="179"/>
-      <c r="E7" s="180"/>
-      <c r="F7" s="180"/>
+      <c r="B7" s="196"/>
+      <c r="C7" s="196"/>
+      <c r="D7" s="196"/>
+      <c r="E7" s="197"/>
+      <c r="F7" s="197"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -41407,48 +41155,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="182"/>
-      <c r="C1" s="183"/>
-      <c r="D1" s="183"/>
-      <c r="E1" s="183"/>
-      <c r="F1" s="183"/>
-      <c r="G1" s="183"/>
-      <c r="H1" s="183"/>
-      <c r="I1" s="183"/>
-      <c r="J1" s="183"/>
-      <c r="K1" s="183"/>
-      <c r="L1" s="183"/>
-      <c r="M1" s="184"/>
+      <c r="B1" s="264"/>
+      <c r="C1" s="265"/>
+      <c r="D1" s="265"/>
+      <c r="E1" s="265"/>
+      <c r="F1" s="265"/>
+      <c r="G1" s="265"/>
+      <c r="H1" s="265"/>
+      <c r="I1" s="265"/>
+      <c r="J1" s="265"/>
+      <c r="K1" s="265"/>
+      <c r="L1" s="265"/>
+      <c r="M1" s="266"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="185" t="s">
+      <c r="B2" s="267" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="186"/>
-      <c r="D2" s="186"/>
-      <c r="E2" s="186"/>
-      <c r="F2" s="186"/>
-      <c r="G2" s="186"/>
-      <c r="H2" s="186"/>
-      <c r="I2" s="187"/>
-      <c r="J2" s="191"/>
-      <c r="K2" s="192"/>
-      <c r="L2" s="192"/>
-      <c r="M2" s="193"/>
+      <c r="C2" s="268"/>
+      <c r="D2" s="268"/>
+      <c r="E2" s="268"/>
+      <c r="F2" s="268"/>
+      <c r="G2" s="268"/>
+      <c r="H2" s="268"/>
+      <c r="I2" s="269"/>
+      <c r="J2" s="273"/>
+      <c r="K2" s="274"/>
+      <c r="L2" s="274"/>
+      <c r="M2" s="275"/>
     </row>
     <row r="3" spans="1:14" ht="14.4" customHeight="1">
-      <c r="B3" s="188"/>
-      <c r="C3" s="189"/>
-      <c r="D3" s="189"/>
-      <c r="E3" s="189"/>
-      <c r="F3" s="189"/>
-      <c r="G3" s="189"/>
-      <c r="H3" s="189"/>
-      <c r="I3" s="190"/>
-      <c r="J3" s="194"/>
-      <c r="K3" s="195"/>
-      <c r="L3" s="195"/>
-      <c r="M3" s="196"/>
+      <c r="B3" s="270"/>
+      <c r="C3" s="271"/>
+      <c r="D3" s="271"/>
+      <c r="E3" s="271"/>
+      <c r="F3" s="271"/>
+      <c r="G3" s="271"/>
+      <c r="H3" s="271"/>
+      <c r="I3" s="272"/>
+      <c r="J3" s="276"/>
+      <c r="K3" s="277"/>
+      <c r="L3" s="277"/>
+      <c r="M3" s="278"/>
     </row>
     <row r="4" spans="1:14" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -41459,10 +41207,10 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="194"/>
-      <c r="K4" s="195"/>
-      <c r="L4" s="195"/>
-      <c r="M4" s="196"/>
+      <c r="J4" s="276"/>
+      <c r="K4" s="277"/>
+      <c r="L4" s="277"/>
+      <c r="M4" s="278"/>
     </row>
     <row r="5" spans="1:14" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -41477,10 +41225,10 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="194"/>
-      <c r="K5" s="195"/>
-      <c r="L5" s="195"/>
-      <c r="M5" s="196"/>
+      <c r="J5" s="276"/>
+      <c r="K5" s="277"/>
+      <c r="L5" s="277"/>
+      <c r="M5" s="278"/>
     </row>
     <row r="6" spans="1:14" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -41495,10 +41243,10 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="197"/>
-      <c r="K6" s="198"/>
-      <c r="L6" s="198"/>
-      <c r="M6" s="199"/>
+      <c r="J6" s="279"/>
+      <c r="K6" s="280"/>
+      <c r="L6" s="280"/>
+      <c r="M6" s="281"/>
     </row>
     <row r="7" spans="1:14" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -41563,52 +41311,52 @@
       <c r="M9" s="89"/>
     </row>
     <row r="10" spans="1:14" ht="15.6">
-      <c r="B10" s="200" t="s">
+      <c r="B10" s="199" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="201"/>
-      <c r="D10" s="201"/>
-      <c r="E10" s="201"/>
-      <c r="F10" s="201"/>
-      <c r="G10" s="201" t="s">
+      <c r="C10" s="200"/>
+      <c r="D10" s="200"/>
+      <c r="E10" s="200"/>
+      <c r="F10" s="200"/>
+      <c r="G10" s="200" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="201"/>
-      <c r="I10" s="201"/>
-      <c r="J10" s="202"/>
-      <c r="K10" s="203" t="s">
+      <c r="H10" s="200"/>
+      <c r="I10" s="200"/>
+      <c r="J10" s="201"/>
+      <c r="K10" s="202" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="201"/>
-      <c r="M10" s="204"/>
+      <c r="L10" s="200"/>
+      <c r="M10" s="282"/>
     </row>
     <row r="11" spans="1:14" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="210" t="s">
+      <c r="C11" s="235" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="232"/>
-      <c r="E11" s="232"/>
+      <c r="D11" s="257"/>
+      <c r="E11" s="257"/>
       <c r="F11" s="92" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="210" t="s">
+      <c r="G11" s="235" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="211"/>
+      <c r="H11" s="236"/>
       <c r="I11" s="93" t="s">
         <v>27</v>
       </c>
       <c r="J11" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="210" t="s">
+      <c r="K11" s="235" t="s">
         <v>58</v>
       </c>
-      <c r="L11" s="211"/>
+      <c r="L11" s="236"/>
       <c r="M11" s="94" t="s">
         <v>59</v>
       </c>
@@ -41813,58 +41561,58 @@
       <c r="M22" s="123"/>
     </row>
     <row r="23" spans="1:13" ht="16.2" thickBot="1">
-      <c r="B23" s="233"/>
-      <c r="C23" s="234"/>
-      <c r="D23" s="234"/>
-      <c r="E23" s="234"/>
+      <c r="B23" s="258"/>
+      <c r="C23" s="259"/>
+      <c r="D23" s="259"/>
+      <c r="E23" s="259"/>
       <c r="F23" s="124"/>
       <c r="G23" s="124"/>
       <c r="H23" s="125"/>
       <c r="I23" s="125"/>
-      <c r="J23" s="235"/>
-      <c r="K23" s="235"/>
-      <c r="L23" s="235"/>
-      <c r="M23" s="236"/>
+      <c r="J23" s="260"/>
+      <c r="K23" s="260"/>
+      <c r="L23" s="260"/>
+      <c r="M23" s="261"/>
     </row>
     <row r="24" spans="1:13" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="152" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="237" t="s">
+      <c r="B24" s="262" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="205" t="s">
+      <c r="C24" s="230" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="205"/>
-      <c r="E24" s="205"/>
-      <c r="F24" s="205"/>
-      <c r="G24" s="205"/>
-      <c r="H24" s="205"/>
-      <c r="I24" s="205"/>
-      <c r="J24" s="207" t="s">
+      <c r="D24" s="230"/>
+      <c r="E24" s="230"/>
+      <c r="F24" s="230"/>
+      <c r="G24" s="230"/>
+      <c r="H24" s="230"/>
+      <c r="I24" s="230"/>
+      <c r="J24" s="232" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="208"/>
-      <c r="L24" s="208"/>
-      <c r="M24" s="209"/>
+      <c r="K24" s="233"/>
+      <c r="L24" s="233"/>
+      <c r="M24" s="234"/>
     </row>
     <row r="25" spans="1:13" ht="31.2">
-      <c r="B25" s="238"/>
-      <c r="C25" s="206"/>
-      <c r="D25" s="206"/>
-      <c r="E25" s="206"/>
-      <c r="F25" s="206"/>
-      <c r="G25" s="206"/>
-      <c r="H25" s="206"/>
-      <c r="I25" s="206"/>
+      <c r="B25" s="263"/>
+      <c r="C25" s="231"/>
+      <c r="D25" s="231"/>
+      <c r="E25" s="231"/>
+      <c r="F25" s="231"/>
+      <c r="G25" s="231"/>
+      <c r="H25" s="231"/>
+      <c r="I25" s="231"/>
       <c r="J25" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="221" t="s">
+      <c r="K25" s="246" t="s">
         <v>76</v>
       </c>
-      <c r="L25" s="222"/>
+      <c r="L25" s="247"/>
       <c r="M25" s="126" t="s">
         <v>77</v>
       </c>
@@ -42422,62 +42170,62 @@
       </c>
     </row>
     <row r="49" spans="2:13" ht="16.2" thickTop="1">
-      <c r="B49" s="248" t="s">
+      <c r="B49" s="212" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="249"/>
-      <c r="D49" s="249"/>
-      <c r="E49" s="249"/>
-      <c r="F49" s="249"/>
-      <c r="G49" s="249"/>
-      <c r="H49" s="249"/>
-      <c r="I49" s="249"/>
-      <c r="J49" s="250"/>
-      <c r="K49" s="229" t="s">
+      <c r="C49" s="213"/>
+      <c r="D49" s="213"/>
+      <c r="E49" s="213"/>
+      <c r="F49" s="213"/>
+      <c r="G49" s="213"/>
+      <c r="H49" s="213"/>
+      <c r="I49" s="213"/>
+      <c r="J49" s="214"/>
+      <c r="K49" s="254" t="s">
         <v>79</v>
       </c>
-      <c r="L49" s="230"/>
-      <c r="M49" s="231"/>
+      <c r="L49" s="255"/>
+      <c r="M49" s="256"/>
     </row>
     <row r="50" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B50" s="251"/>
-      <c r="C50" s="252"/>
-      <c r="D50" s="252"/>
-      <c r="E50" s="252"/>
-      <c r="F50" s="252"/>
-      <c r="G50" s="252"/>
-      <c r="H50" s="252"/>
-      <c r="I50" s="252"/>
-      <c r="J50" s="253"/>
-      <c r="K50" s="226" t="s">
+      <c r="B50" s="215"/>
+      <c r="C50" s="216"/>
+      <c r="D50" s="216"/>
+      <c r="E50" s="216"/>
+      <c r="F50" s="216"/>
+      <c r="G50" s="216"/>
+      <c r="H50" s="216"/>
+      <c r="I50" s="216"/>
+      <c r="J50" s="217"/>
+      <c r="K50" s="251" t="s">
         <v>103</v>
       </c>
-      <c r="L50" s="227"/>
-      <c r="M50" s="228"/>
+      <c r="L50" s="252"/>
+      <c r="M50" s="253"/>
     </row>
     <row r="51" spans="2:13" ht="15.6">
       <c r="B51" s="138"/>
-      <c r="C51" s="223"/>
-      <c r="D51" s="223"/>
-      <c r="E51" s="223"/>
-      <c r="F51" s="223"/>
-      <c r="G51" s="223"/>
-      <c r="H51" s="223"/>
-      <c r="I51" s="223"/>
+      <c r="C51" s="248"/>
+      <c r="D51" s="248"/>
+      <c r="E51" s="248"/>
+      <c r="F51" s="248"/>
+      <c r="G51" s="248"/>
+      <c r="H51" s="248"/>
+      <c r="I51" s="248"/>
       <c r="J51" s="139"/>
-      <c r="K51" s="218"/>
-      <c r="L51" s="219"/>
-      <c r="M51" s="220"/>
+      <c r="K51" s="243"/>
+      <c r="L51" s="244"/>
+      <c r="M51" s="245"/>
     </row>
     <row r="52" spans="2:13" ht="15.6">
       <c r="B52" s="140"/>
-      <c r="C52" s="224"/>
-      <c r="D52" s="224"/>
-      <c r="E52" s="224"/>
-      <c r="F52" s="224"/>
-      <c r="G52" s="224"/>
-      <c r="H52" s="224"/>
-      <c r="I52" s="224"/>
+      <c r="C52" s="249"/>
+      <c r="D52" s="249"/>
+      <c r="E52" s="249"/>
+      <c r="F52" s="249"/>
+      <c r="G52" s="249"/>
+      <c r="H52" s="249"/>
+      <c r="I52" s="249"/>
       <c r="J52" s="141"/>
       <c r="K52" s="164"/>
       <c r="L52" s="161"/>
@@ -42485,13 +42233,13 @@
     </row>
     <row r="53" spans="2:13" ht="15.6">
       <c r="B53" s="140"/>
-      <c r="C53" s="224"/>
-      <c r="D53" s="224"/>
-      <c r="E53" s="224"/>
-      <c r="F53" s="224"/>
-      <c r="G53" s="224"/>
-      <c r="H53" s="224"/>
-      <c r="I53" s="224"/>
+      <c r="C53" s="249"/>
+      <c r="D53" s="249"/>
+      <c r="E53" s="249"/>
+      <c r="F53" s="249"/>
+      <c r="G53" s="249"/>
+      <c r="H53" s="249"/>
+      <c r="I53" s="249"/>
       <c r="J53" s="141"/>
       <c r="K53" s="164"/>
       <c r="L53" s="161"/>
@@ -42499,13 +42247,13 @@
     </row>
     <row r="54" spans="2:13" ht="15.6">
       <c r="B54" s="140"/>
-      <c r="C54" s="224"/>
-      <c r="D54" s="224"/>
-      <c r="E54" s="224"/>
-      <c r="F54" s="224"/>
-      <c r="G54" s="224"/>
-      <c r="H54" s="224"/>
-      <c r="I54" s="224"/>
+      <c r="C54" s="249"/>
+      <c r="D54" s="249"/>
+      <c r="E54" s="249"/>
+      <c r="F54" s="249"/>
+      <c r="G54" s="249"/>
+      <c r="H54" s="249"/>
+      <c r="I54" s="249"/>
       <c r="J54" s="141"/>
       <c r="K54" s="164"/>
       <c r="L54" s="161"/>
@@ -42513,13 +42261,13 @@
     </row>
     <row r="55" spans="2:13" ht="15.6">
       <c r="B55" s="143"/>
-      <c r="C55" s="224"/>
-      <c r="D55" s="224"/>
-      <c r="E55" s="224"/>
-      <c r="F55" s="224"/>
-      <c r="G55" s="224"/>
-      <c r="H55" s="224"/>
-      <c r="I55" s="224"/>
+      <c r="C55" s="249"/>
+      <c r="D55" s="249"/>
+      <c r="E55" s="249"/>
+      <c r="F55" s="249"/>
+      <c r="G55" s="249"/>
+      <c r="H55" s="249"/>
+      <c r="I55" s="249"/>
       <c r="J55" s="144"/>
       <c r="K55" s="164"/>
       <c r="L55" s="145"/>
@@ -42527,13 +42275,13 @@
     </row>
     <row r="56" spans="2:13" ht="15.6">
       <c r="B56" s="143"/>
-      <c r="C56" s="224"/>
-      <c r="D56" s="224"/>
-      <c r="E56" s="224"/>
-      <c r="F56" s="224"/>
-      <c r="G56" s="224"/>
-      <c r="H56" s="224"/>
-      <c r="I56" s="224"/>
+      <c r="C56" s="249"/>
+      <c r="D56" s="249"/>
+      <c r="E56" s="249"/>
+      <c r="F56" s="249"/>
+      <c r="G56" s="249"/>
+      <c r="H56" s="249"/>
+      <c r="I56" s="249"/>
       <c r="J56" s="144"/>
       <c r="K56" s="164"/>
       <c r="L56" s="145"/>
@@ -42541,41 +42289,41 @@
     </row>
     <row r="57" spans="2:13" ht="15.6">
       <c r="B57" s="143"/>
-      <c r="C57" s="224"/>
-      <c r="D57" s="224"/>
-      <c r="E57" s="224"/>
-      <c r="F57" s="224"/>
-      <c r="G57" s="224"/>
-      <c r="H57" s="224"/>
-      <c r="I57" s="224"/>
+      <c r="C57" s="249"/>
+      <c r="D57" s="249"/>
+      <c r="E57" s="249"/>
+      <c r="F57" s="249"/>
+      <c r="G57" s="249"/>
+      <c r="H57" s="249"/>
+      <c r="I57" s="249"/>
       <c r="J57" s="144"/>
-      <c r="K57" s="212"/>
-      <c r="L57" s="213"/>
-      <c r="M57" s="214"/>
+      <c r="K57" s="237"/>
+      <c r="L57" s="238"/>
+      <c r="M57" s="239"/>
     </row>
     <row r="58" spans="2:13" ht="15.6">
       <c r="B58" s="143"/>
-      <c r="C58" s="224"/>
-      <c r="D58" s="224"/>
-      <c r="E58" s="224"/>
-      <c r="F58" s="224"/>
-      <c r="G58" s="224"/>
-      <c r="H58" s="224"/>
-      <c r="I58" s="224"/>
+      <c r="C58" s="249"/>
+      <c r="D58" s="249"/>
+      <c r="E58" s="249"/>
+      <c r="F58" s="249"/>
+      <c r="G58" s="249"/>
+      <c r="H58" s="249"/>
+      <c r="I58" s="249"/>
       <c r="J58" s="144"/>
-      <c r="K58" s="215"/>
-      <c r="L58" s="216"/>
-      <c r="M58" s="217"/>
+      <c r="K58" s="240"/>
+      <c r="L58" s="241"/>
+      <c r="M58" s="242"/>
     </row>
     <row r="59" spans="2:13" ht="15.6">
       <c r="B59" s="143"/>
-      <c r="C59" s="224"/>
-      <c r="D59" s="224"/>
-      <c r="E59" s="224"/>
-      <c r="F59" s="224"/>
-      <c r="G59" s="224"/>
-      <c r="H59" s="224"/>
-      <c r="I59" s="224"/>
+      <c r="C59" s="249"/>
+      <c r="D59" s="249"/>
+      <c r="E59" s="249"/>
+      <c r="F59" s="249"/>
+      <c r="G59" s="249"/>
+      <c r="H59" s="249"/>
+      <c r="I59" s="249"/>
       <c r="J59" s="144"/>
       <c r="K59" s="164"/>
       <c r="L59" s="162"/>
@@ -42583,13 +42331,13 @@
     </row>
     <row r="60" spans="2:13" ht="15.6">
       <c r="B60" s="143"/>
-      <c r="C60" s="224"/>
-      <c r="D60" s="224"/>
-      <c r="E60" s="224"/>
-      <c r="F60" s="224"/>
-      <c r="G60" s="224"/>
-      <c r="H60" s="224"/>
-      <c r="I60" s="224"/>
+      <c r="C60" s="249"/>
+      <c r="D60" s="249"/>
+      <c r="E60" s="249"/>
+      <c r="F60" s="249"/>
+      <c r="G60" s="249"/>
+      <c r="H60" s="249"/>
+      <c r="I60" s="249"/>
       <c r="J60" s="144"/>
       <c r="K60" s="164"/>
       <c r="L60" s="162"/>
@@ -42597,13 +42345,13 @@
     </row>
     <row r="61" spans="2:13" ht="15.6">
       <c r="B61" s="143"/>
-      <c r="C61" s="225"/>
-      <c r="D61" s="225"/>
-      <c r="E61" s="225"/>
-      <c r="F61" s="225"/>
-      <c r="G61" s="225"/>
-      <c r="H61" s="225"/>
-      <c r="I61" s="225"/>
+      <c r="C61" s="250"/>
+      <c r="D61" s="250"/>
+      <c r="E61" s="250"/>
+      <c r="F61" s="250"/>
+      <c r="G61" s="250"/>
+      <c r="H61" s="250"/>
+      <c r="I61" s="250"/>
       <c r="J61" s="144"/>
       <c r="K61" s="164"/>
       <c r="L61" s="162"/>
@@ -42624,133 +42372,133 @@
       <c r="M62" s="167"/>
     </row>
     <row r="63" spans="2:13" ht="15.6">
-      <c r="B63" s="200" t="s">
+      <c r="B63" s="199" t="s">
         <v>80</v>
       </c>
-      <c r="C63" s="201"/>
-      <c r="D63" s="201"/>
-      <c r="E63" s="202"/>
-      <c r="F63" s="203" t="s">
+      <c r="C63" s="200"/>
+      <c r="D63" s="200"/>
+      <c r="E63" s="201"/>
+      <c r="F63" s="202" t="s">
         <v>81</v>
       </c>
-      <c r="G63" s="202"/>
-      <c r="H63" s="203" t="s">
+      <c r="G63" s="201"/>
+      <c r="H63" s="202" t="s">
         <v>82</v>
       </c>
-      <c r="I63" s="201"/>
-      <c r="J63" s="202"/>
+      <c r="I63" s="200"/>
+      <c r="J63" s="201"/>
       <c r="K63" s="165"/>
       <c r="L63" s="145"/>
       <c r="M63" s="146"/>
     </row>
     <row r="64" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B64" s="260"/>
-      <c r="C64" s="261"/>
-      <c r="D64" s="261"/>
-      <c r="E64" s="255"/>
-      <c r="F64" s="254"/>
-      <c r="G64" s="255"/>
-      <c r="H64" s="239"/>
-      <c r="I64" s="240"/>
-      <c r="J64" s="241"/>
+      <c r="B64" s="224"/>
+      <c r="C64" s="225"/>
+      <c r="D64" s="225"/>
+      <c r="E64" s="219"/>
+      <c r="F64" s="218"/>
+      <c r="G64" s="219"/>
+      <c r="H64" s="203"/>
+      <c r="I64" s="204"/>
+      <c r="J64" s="205"/>
       <c r="K64" s="148"/>
       <c r="L64" s="145"/>
       <c r="M64" s="146"/>
     </row>
     <row r="65" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B65" s="262"/>
-      <c r="C65" s="263"/>
-      <c r="D65" s="263"/>
-      <c r="E65" s="257"/>
-      <c r="F65" s="256"/>
-      <c r="G65" s="257"/>
-      <c r="H65" s="242"/>
-      <c r="I65" s="243"/>
-      <c r="J65" s="244"/>
+      <c r="B65" s="226"/>
+      <c r="C65" s="227"/>
+      <c r="D65" s="227"/>
+      <c r="E65" s="221"/>
+      <c r="F65" s="220"/>
+      <c r="G65" s="221"/>
+      <c r="H65" s="206"/>
+      <c r="I65" s="207"/>
+      <c r="J65" s="208"/>
       <c r="K65" s="148"/>
       <c r="L65" s="163"/>
       <c r="M65" s="146"/>
     </row>
     <row r="66" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B66" s="262"/>
-      <c r="C66" s="263"/>
-      <c r="D66" s="263"/>
-      <c r="E66" s="257"/>
-      <c r="F66" s="256"/>
-      <c r="G66" s="257"/>
-      <c r="H66" s="242"/>
-      <c r="I66" s="243"/>
-      <c r="J66" s="244"/>
+      <c r="B66" s="226"/>
+      <c r="C66" s="227"/>
+      <c r="D66" s="227"/>
+      <c r="E66" s="221"/>
+      <c r="F66" s="220"/>
+      <c r="G66" s="221"/>
+      <c r="H66" s="206"/>
+      <c r="I66" s="207"/>
+      <c r="J66" s="208"/>
       <c r="K66" s="148"/>
       <c r="L66" s="145"/>
       <c r="M66" s="146"/>
     </row>
     <row r="67" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B67" s="262"/>
-      <c r="C67" s="263"/>
-      <c r="D67" s="263"/>
-      <c r="E67" s="257"/>
-      <c r="F67" s="256"/>
-      <c r="G67" s="257"/>
-      <c r="H67" s="242"/>
-      <c r="I67" s="243"/>
-      <c r="J67" s="244"/>
+      <c r="B67" s="226"/>
+      <c r="C67" s="227"/>
+      <c r="D67" s="227"/>
+      <c r="E67" s="221"/>
+      <c r="F67" s="220"/>
+      <c r="G67" s="221"/>
+      <c r="H67" s="206"/>
+      <c r="I67" s="207"/>
+      <c r="J67" s="208"/>
       <c r="K67" s="148"/>
       <c r="L67" s="162"/>
       <c r="M67" s="76"/>
     </row>
     <row r="68" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B68" s="262"/>
-      <c r="C68" s="263"/>
-      <c r="D68" s="263"/>
-      <c r="E68" s="257"/>
-      <c r="F68" s="256"/>
-      <c r="G68" s="257"/>
-      <c r="H68" s="242"/>
-      <c r="I68" s="243"/>
-      <c r="J68" s="244"/>
+      <c r="B68" s="226"/>
+      <c r="C68" s="227"/>
+      <c r="D68" s="227"/>
+      <c r="E68" s="221"/>
+      <c r="F68" s="220"/>
+      <c r="G68" s="221"/>
+      <c r="H68" s="206"/>
+      <c r="I68" s="207"/>
+      <c r="J68" s="208"/>
       <c r="K68" s="148"/>
       <c r="L68" s="162"/>
       <c r="M68" s="76"/>
     </row>
     <row r="69" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B69" s="262"/>
-      <c r="C69" s="263"/>
-      <c r="D69" s="263"/>
-      <c r="E69" s="257"/>
-      <c r="F69" s="256"/>
-      <c r="G69" s="257"/>
-      <c r="H69" s="242"/>
-      <c r="I69" s="243"/>
-      <c r="J69" s="244"/>
+      <c r="B69" s="226"/>
+      <c r="C69" s="227"/>
+      <c r="D69" s="227"/>
+      <c r="E69" s="221"/>
+      <c r="F69" s="220"/>
+      <c r="G69" s="221"/>
+      <c r="H69" s="206"/>
+      <c r="I69" s="207"/>
+      <c r="J69" s="208"/>
       <c r="K69" s="168"/>
       <c r="L69" s="169"/>
       <c r="M69" s="170"/>
     </row>
     <row r="70" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B70" s="262"/>
-      <c r="C70" s="263"/>
-      <c r="D70" s="263"/>
-      <c r="E70" s="257"/>
-      <c r="F70" s="256"/>
-      <c r="G70" s="257"/>
-      <c r="H70" s="242"/>
-      <c r="I70" s="243"/>
-      <c r="J70" s="244"/>
+      <c r="B70" s="226"/>
+      <c r="C70" s="227"/>
+      <c r="D70" s="227"/>
+      <c r="E70" s="221"/>
+      <c r="F70" s="220"/>
+      <c r="G70" s="221"/>
+      <c r="H70" s="206"/>
+      <c r="I70" s="207"/>
+      <c r="J70" s="208"/>
       <c r="K70" s="168"/>
       <c r="L70" s="169"/>
       <c r="M70" s="170"/>
     </row>
     <row r="71" spans="2:13" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B71" s="264"/>
-      <c r="C71" s="265"/>
-      <c r="D71" s="265"/>
-      <c r="E71" s="259"/>
-      <c r="F71" s="258"/>
-      <c r="G71" s="259"/>
-      <c r="H71" s="245"/>
-      <c r="I71" s="246"/>
-      <c r="J71" s="247"/>
+      <c r="B71" s="228"/>
+      <c r="C71" s="229"/>
+      <c r="D71" s="229"/>
+      <c r="E71" s="223"/>
+      <c r="F71" s="222"/>
+      <c r="G71" s="223"/>
+      <c r="H71" s="209"/>
+      <c r="I71" s="210"/>
+      <c r="J71" s="211"/>
       <c r="K71" s="150"/>
       <c r="L71" s="149"/>
       <c r="M71" s="151"/>
@@ -42763,13 +42511,12 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="H63:J63"/>
-    <mergeCell ref="H64:J71"/>
-    <mergeCell ref="B49:J50"/>
-    <mergeCell ref="F64:G71"/>
-    <mergeCell ref="B64:E71"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="J2:M6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="K10:M10"/>
     <mergeCell ref="C24:I25"/>
     <mergeCell ref="J24:M24"/>
     <mergeCell ref="K11:L11"/>
@@ -42785,12 +42532,13 @@
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="J23:M23"/>
     <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="J2:M6"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="H63:J63"/>
+    <mergeCell ref="H64:J71"/>
+    <mergeCell ref="B49:J50"/>
+    <mergeCell ref="F64:G71"/>
+    <mergeCell ref="B64:E71"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:I48">
     <cfRule type="expression" dxfId="3" priority="1">
@@ -42836,40 +42584,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="178"/>
-      <c r="C1" s="178"/>
-      <c r="D1" s="178"/>
-      <c r="E1" s="178"/>
-      <c r="F1" s="178"/>
-      <c r="G1" s="178"/>
-      <c r="H1" s="178"/>
-      <c r="I1" s="178"/>
-      <c r="J1" s="178"/>
-      <c r="K1" s="178"/>
-      <c r="L1" s="178"/>
-      <c r="M1" s="178"/>
-      <c r="N1" s="178"/>
-      <c r="O1" s="178"/>
-      <c r="P1" s="178"/>
+      <c r="B1" s="195"/>
+      <c r="C1" s="195"/>
+      <c r="D1" s="195"/>
+      <c r="E1" s="195"/>
+      <c r="F1" s="195"/>
+      <c r="G1" s="195"/>
+      <c r="H1" s="195"/>
+      <c r="I1" s="195"/>
+      <c r="J1" s="195"/>
+      <c r="K1" s="195"/>
+      <c r="L1" s="195"/>
+      <c r="M1" s="195"/>
+      <c r="N1" s="195"/>
+      <c r="O1" s="195"/>
+      <c r="P1" s="195"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="176" t="s">
+      <c r="B2" s="194" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="177"/>
-      <c r="D2" s="177"/>
-      <c r="E2" s="177"/>
-      <c r="F2" s="177"/>
-      <c r="G2" s="177"/>
-      <c r="H2" s="177"/>
-      <c r="I2" s="177"/>
-      <c r="J2" s="177"/>
-      <c r="K2" s="177"/>
-      <c r="L2" s="177"/>
-      <c r="M2" s="177"/>
-      <c r="N2" s="177"/>
-      <c r="O2" s="177"/>
-      <c r="P2" s="177"/>
+      <c r="C2" s="186"/>
+      <c r="D2" s="186"/>
+      <c r="E2" s="186"/>
+      <c r="F2" s="186"/>
+      <c r="G2" s="186"/>
+      <c r="H2" s="186"/>
+      <c r="I2" s="186"/>
+      <c r="J2" s="186"/>
+      <c r="K2" s="186"/>
+      <c r="L2" s="186"/>
+      <c r="M2" s="186"/>
+      <c r="N2" s="186"/>
+      <c r="O2" s="186"/>
+      <c r="P2" s="186"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -42896,16 +42644,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="268" t="s">
+      <c r="I4" s="285" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="268"/>
-      <c r="K4" s="268"/>
-      <c r="L4" s="268"/>
-      <c r="M4" s="268"/>
-      <c r="N4" s="268"/>
-      <c r="O4" s="268"/>
-      <c r="P4" s="268"/>
+      <c r="J4" s="285"/>
+      <c r="K4" s="285"/>
+      <c r="L4" s="285"/>
+      <c r="M4" s="285"/>
+      <c r="N4" s="285"/>
+      <c r="O4" s="285"/>
+      <c r="P4" s="285"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -42919,14 +42667,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="268"/>
-      <c r="J5" s="268"/>
-      <c r="K5" s="268"/>
-      <c r="L5" s="268"/>
-      <c r="M5" s="268"/>
-      <c r="N5" s="268"/>
-      <c r="O5" s="268"/>
-      <c r="P5" s="268"/>
+      <c r="I5" s="285"/>
+      <c r="J5" s="285"/>
+      <c r="K5" s="285"/>
+      <c r="L5" s="285"/>
+      <c r="M5" s="285"/>
+      <c r="N5" s="285"/>
+      <c r="O5" s="285"/>
+      <c r="P5" s="285"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -43061,70 +42809,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="175" t="s">
+      <c r="B12" s="193" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="175" t="s">
+      <c r="C12" s="193" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="175"/>
-      <c r="E12" s="175"/>
-      <c r="F12" s="175" t="s">
+      <c r="D12" s="193"/>
+      <c r="E12" s="193"/>
+      <c r="F12" s="193" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="175" t="s">
+      <c r="G12" s="193" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="175" t="s">
+      <c r="H12" s="193" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="175" t="s">
+      <c r="I12" s="193" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="175" t="s">
+      <c r="J12" s="193" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="175"/>
-      <c r="L12" s="175"/>
-      <c r="M12" s="175"/>
-      <c r="N12" s="175"/>
-      <c r="O12" s="175"/>
-      <c r="P12" s="267" t="s">
+      <c r="K12" s="193"/>
+      <c r="L12" s="193"/>
+      <c r="M12" s="193"/>
+      <c r="N12" s="193"/>
+      <c r="O12" s="193"/>
+      <c r="P12" s="284" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="175"/>
-      <c r="C13" s="175"/>
-      <c r="D13" s="175"/>
-      <c r="E13" s="175"/>
-      <c r="F13" s="175"/>
-      <c r="G13" s="175"/>
-      <c r="H13" s="175"/>
-      <c r="I13" s="175"/>
-      <c r="J13" s="266" t="s">
+      <c r="B13" s="193"/>
+      <c r="C13" s="193"/>
+      <c r="D13" s="193"/>
+      <c r="E13" s="193"/>
+      <c r="F13" s="193"/>
+      <c r="G13" s="193"/>
+      <c r="H13" s="193"/>
+      <c r="I13" s="193"/>
+      <c r="J13" s="283" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="266"/>
-      <c r="L13" s="266" t="s">
+      <c r="K13" s="283"/>
+      <c r="L13" s="283" t="s">
         <v>98</v>
       </c>
-      <c r="M13" s="266"/>
-      <c r="N13" s="266" t="s">
+      <c r="M13" s="283"/>
+      <c r="N13" s="283" t="s">
         <v>99</v>
       </c>
-      <c r="O13" s="266"/>
-      <c r="P13" s="267"/>
+      <c r="O13" s="283"/>
+      <c r="P13" s="284"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="175"/>
-      <c r="C14" s="175"/>
-      <c r="D14" s="175"/>
-      <c r="E14" s="175"/>
-      <c r="F14" s="175"/>
-      <c r="G14" s="175"/>
-      <c r="H14" s="175"/>
-      <c r="I14" s="175"/>
+      <c r="B14" s="193"/>
+      <c r="C14" s="193"/>
+      <c r="D14" s="193"/>
+      <c r="E14" s="193"/>
+      <c r="F14" s="193"/>
+      <c r="G14" s="193"/>
+      <c r="H14" s="193"/>
+      <c r="I14" s="193"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -43143,7 +42891,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="267"/>
+      <c r="P14" s="284"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>

</xml_diff>

<commit_message>
chore(template): update master template to reflect layout changes
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC58D63-AA6F-40EF-BCDE-6E79639B0123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504B2336-A84A-4373-AF1D-B46D2CDFD889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,20 +21,14 @@
     <sheet name="dokumentasi" sheetId="22" r:id="rId11"/>
     <sheet name="backup data" sheetId="23" r:id="rId12"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId13"/>
-    <externalReference r:id="rId14"/>
-    <externalReference r:id="rId15"/>
-    <externalReference r:id="rId16"/>
-  </externalReferences>
   <definedNames>
-    <definedName name="__123Graph_A" hidden="1">[1]Div2!#REF!</definedName>
-    <definedName name="__123Graph_B" hidden="1">[1]Div2!#REF!</definedName>
-    <definedName name="__123Graph_X" hidden="1">[1]Div2!#REF!</definedName>
-    <definedName name="_1__123Graph_ACHART_1" hidden="1">[2]RAB!#REF!</definedName>
-    <definedName name="_2__123Graph_XCHART_1" hidden="1">[3]RAB!#REF!</definedName>
+    <definedName name="__123Graph_A" hidden="1">#REF!</definedName>
+    <definedName name="__123Graph_B" hidden="1">#REF!</definedName>
+    <definedName name="__123Graph_X" hidden="1">#REF!</definedName>
+    <definedName name="_1__123Graph_ACHART_1" hidden="1">#REF!</definedName>
+    <definedName name="_2__123Graph_XCHART_1" hidden="1">#REF!</definedName>
     <definedName name="_Fill" hidden="1">#REF!</definedName>
-    <definedName name="RAB" hidden="1">[4]RAB!#REF!</definedName>
+    <definedName name="RAB" hidden="1">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2641,44 +2635,179 @@
     <xf numFmtId="0" fontId="32" fillId="4" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="19" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="33" fillId="4" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="33" fillId="4" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="67" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="60" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2785,137 +2914,38 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="67" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="60" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2924,6 +2954,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3006,48 +3042,6 @@
     </xf>
     <xf numFmtId="0" fontId="32" fillId="4" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="19" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="33" fillId="4" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="33" fillId="4" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -3809,198 +3803,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Surat"/>
-      <sheetName val="Div1"/>
-      <sheetName val="Div2"/>
-      <sheetName val="Div 2"/>
-      <sheetName val="Div3"/>
-      <sheetName val="Div5"/>
-      <sheetName val="Div4"/>
-      <sheetName val="Div8b"/>
-      <sheetName val="Div 6"/>
-      <sheetName val="Div 7"/>
-      <sheetName val="Div 8"/>
-      <sheetName val="Jadwal"/>
-      <sheetName val="Utama"/>
-      <sheetName val="Lamp8"/>
-      <sheetName val="Lamp"/>
-      <sheetName val="SKon"/>
-      <sheetName val="Kapasitas AMP.S.C"/>
-      <sheetName val="Staf"/>
-      <sheetName val="Alat"/>
-      <sheetName val="Div_2"/>
-      <sheetName val="Div_6"/>
-      <sheetName val="Div_7"/>
-      <sheetName val="Div_8"/>
-      <sheetName val="Kapasitas_AMP_S_C"/>
-      <sheetName val="upahbahan"/>
-      <sheetName val="analisa"/>
-      <sheetName val="rab1"/>
-      <sheetName val="rekap"/>
-      <sheetName val="OUTPUT"/>
-      <sheetName val="ANAL-"/>
-      <sheetName val="H.Satuan"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24" refreshError="1"/>
-      <sheetData sheetId="25" refreshError="1"/>
-      <sheetData sheetId="26" refreshError="1"/>
-      <sheetData sheetId="27" refreshError="1"/>
-      <sheetData sheetId="28" refreshError="1"/>
-      <sheetData sheetId="29" refreshError="1"/>
-      <sheetData sheetId="30" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Mot"/>
-      <sheetName val="MPU"/>
-      <sheetName val="Jad"/>
-      <sheetName val="RAB"/>
-      <sheetName val="Mob"/>
-      <sheetName val="Ana"/>
-      <sheetName val="Alat"/>
-      <sheetName val="U&amp;B"/>
-      <sheetName val="Sub"/>
-      <sheetName val="Mob. Alat"/>
-      <sheetName val="Mob Alat"/>
-      <sheetName val="Sheet2"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="laroux"/>
-      <sheetName val="Mata"/>
-      <sheetName val="Analisa"/>
-      <sheetName val="Jad"/>
-      <sheetName val="Mat"/>
-      <sheetName val="RAB"/>
-      <sheetName val="Mob"/>
-      <sheetName val="MobAlat"/>
-      <sheetName val="Alat"/>
-      <sheetName val="U &amp; B"/>
-      <sheetName val="Jadwal"/>
-      <sheetName val="Sub"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="laroux"/>
-      <sheetName val="Mata"/>
-      <sheetName val="Analisa"/>
-      <sheetName val="Jad"/>
-      <sheetName val="Mat"/>
-      <sheetName val="RAB"/>
-      <sheetName val="Mob"/>
-      <sheetName val="MobAlat"/>
-      <sheetName val="Alat"/>
-      <sheetName val="U &amp; B"/>
-      <sheetName val="Jadwal"/>
-      <sheetName val="Sub"/>
-      <sheetName val="U_&amp;_B"/>
-      <sheetName val="upah"/>
-      <sheetName val="ANAL-"/>
-      <sheetName val="Kuantitas &amp; Harga"/>
-      <sheetName val="Agregat Halus &amp; Kasar"/>
-      <sheetName val="TPI"/>
-      <sheetName val="H.Satuan"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4359,40 +4161,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="185"/>
-      <c r="C1" s="185"/>
-      <c r="D1" s="185"/>
-      <c r="E1" s="185"/>
-      <c r="F1" s="185"/>
-      <c r="G1" s="185"/>
-      <c r="H1" s="185"/>
-      <c r="I1" s="185"/>
-      <c r="J1" s="185"/>
-      <c r="K1" s="185"/>
-      <c r="L1" s="185"/>
-      <c r="M1" s="185"/>
-      <c r="N1" s="185"/>
-      <c r="O1" s="185"/>
-      <c r="P1" s="185"/>
+      <c r="B1" s="266"/>
+      <c r="C1" s="266"/>
+      <c r="D1" s="266"/>
+      <c r="E1" s="266"/>
+      <c r="F1" s="266"/>
+      <c r="G1" s="266"/>
+      <c r="H1" s="266"/>
+      <c r="I1" s="266"/>
+      <c r="J1" s="266"/>
+      <c r="K1" s="266"/>
+      <c r="L1" s="266"/>
+      <c r="M1" s="266"/>
+      <c r="N1" s="266"/>
+      <c r="O1" s="266"/>
+      <c r="P1" s="266"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="184" t="s">
+      <c r="B2" s="264" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="176"/>
-      <c r="D2" s="176"/>
-      <c r="E2" s="176"/>
-      <c r="F2" s="176"/>
-      <c r="G2" s="176"/>
-      <c r="H2" s="176"/>
-      <c r="I2" s="176"/>
-      <c r="J2" s="176"/>
-      <c r="K2" s="176"/>
-      <c r="L2" s="176"/>
-      <c r="M2" s="176"/>
-      <c r="N2" s="176"/>
-      <c r="O2" s="176"/>
-      <c r="P2" s="176"/>
+      <c r="C2" s="265"/>
+      <c r="D2" s="265"/>
+      <c r="E2" s="265"/>
+      <c r="F2" s="265"/>
+      <c r="G2" s="265"/>
+      <c r="H2" s="265"/>
+      <c r="I2" s="265"/>
+      <c r="J2" s="265"/>
+      <c r="K2" s="265"/>
+      <c r="L2" s="265"/>
+      <c r="M2" s="265"/>
+      <c r="N2" s="265"/>
+      <c r="O2" s="265"/>
+      <c r="P2" s="265"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4419,16 +4221,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="260" t="s">
+      <c r="I4" s="272" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="260"/>
-      <c r="K4" s="260"/>
-      <c r="L4" s="260"/>
-      <c r="M4" s="260"/>
-      <c r="N4" s="260"/>
-      <c r="O4" s="260"/>
-      <c r="P4" s="260"/>
+      <c r="J4" s="272"/>
+      <c r="K4" s="272"/>
+      <c r="L4" s="272"/>
+      <c r="M4" s="272"/>
+      <c r="N4" s="272"/>
+      <c r="O4" s="272"/>
+      <c r="P4" s="272"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4442,14 +4244,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="260"/>
-      <c r="J5" s="260"/>
-      <c r="K5" s="260"/>
-      <c r="L5" s="260"/>
-      <c r="M5" s="260"/>
-      <c r="N5" s="260"/>
-      <c r="O5" s="260"/>
-      <c r="P5" s="260"/>
+      <c r="I5" s="272"/>
+      <c r="J5" s="272"/>
+      <c r="K5" s="272"/>
+      <c r="L5" s="272"/>
+      <c r="M5" s="272"/>
+      <c r="N5" s="272"/>
+      <c r="O5" s="272"/>
+      <c r="P5" s="272"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4584,70 +4386,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="183" t="s">
+      <c r="B12" s="263" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="183" t="s">
+      <c r="C12" s="263" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="183"/>
-      <c r="E12" s="183"/>
-      <c r="F12" s="183" t="s">
+      <c r="D12" s="263"/>
+      <c r="E12" s="263"/>
+      <c r="F12" s="263" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="183" t="s">
+      <c r="G12" s="263" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="183" t="s">
+      <c r="H12" s="263" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="183" t="s">
+      <c r="I12" s="263" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="183" t="s">
+      <c r="J12" s="263" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="183"/>
-      <c r="L12" s="183"/>
-      <c r="M12" s="183"/>
-      <c r="N12" s="183"/>
-      <c r="O12" s="183"/>
-      <c r="P12" s="259" t="s">
+      <c r="K12" s="263"/>
+      <c r="L12" s="263"/>
+      <c r="M12" s="263"/>
+      <c r="N12" s="263"/>
+      <c r="O12" s="263"/>
+      <c r="P12" s="271" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="183"/>
-      <c r="C13" s="183"/>
-      <c r="D13" s="183"/>
-      <c r="E13" s="183"/>
-      <c r="F13" s="183"/>
-      <c r="G13" s="183"/>
-      <c r="H13" s="183"/>
-      <c r="I13" s="183"/>
-      <c r="J13" s="258" t="s">
+      <c r="B13" s="263"/>
+      <c r="C13" s="263"/>
+      <c r="D13" s="263"/>
+      <c r="E13" s="263"/>
+      <c r="F13" s="263"/>
+      <c r="G13" s="263"/>
+      <c r="H13" s="263"/>
+      <c r="I13" s="263"/>
+      <c r="J13" s="270" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="258"/>
-      <c r="L13" s="258" t="s">
+      <c r="K13" s="270"/>
+      <c r="L13" s="270" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="258"/>
-      <c r="N13" s="258" t="s">
+      <c r="M13" s="270"/>
+      <c r="N13" s="270" t="s">
         <v>95</v>
       </c>
-      <c r="O13" s="258"/>
-      <c r="P13" s="259"/>
+      <c r="O13" s="270"/>
+      <c r="P13" s="271"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="183"/>
-      <c r="C14" s="183"/>
-      <c r="D14" s="183"/>
-      <c r="E14" s="183"/>
-      <c r="F14" s="183"/>
-      <c r="G14" s="183"/>
-      <c r="H14" s="183"/>
-      <c r="I14" s="183"/>
+      <c r="B14" s="263"/>
+      <c r="C14" s="263"/>
+      <c r="D14" s="263"/>
+      <c r="E14" s="263"/>
+      <c r="F14" s="263"/>
+      <c r="G14" s="263"/>
+      <c r="H14" s="263"/>
+      <c r="I14" s="263"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -4666,7 +4468,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="259"/>
+      <c r="P14" s="271"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -5089,38 +4891,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="103.2" customHeight="1">
-      <c r="B1" s="176"/>
-      <c r="C1" s="176"/>
-      <c r="D1" s="176"/>
-      <c r="E1" s="176"/>
-      <c r="F1" s="176"/>
-      <c r="G1" s="176"/>
-      <c r="H1" s="176"/>
-      <c r="I1" s="176"/>
-      <c r="J1" s="176"/>
-      <c r="K1" s="176"/>
-      <c r="L1" s="176"/>
-      <c r="M1" s="176"/>
-      <c r="N1" s="176"/>
-      <c r="O1" s="176"/>
+      <c r="B1" s="265"/>
+      <c r="C1" s="265"/>
+      <c r="D1" s="265"/>
+      <c r="E1" s="265"/>
+      <c r="F1" s="265"/>
+      <c r="G1" s="265"/>
+      <c r="H1" s="265"/>
+      <c r="I1" s="265"/>
+      <c r="J1" s="265"/>
+      <c r="K1" s="265"/>
+      <c r="L1" s="265"/>
+      <c r="M1" s="265"/>
+      <c r="N1" s="265"/>
+      <c r="O1" s="265"/>
     </row>
     <row r="2" spans="2:15" ht="22.95" customHeight="1">
-      <c r="B2" s="177" t="s">
+      <c r="B2" s="273" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="177"/>
-      <c r="D2" s="177"/>
-      <c r="E2" s="177"/>
-      <c r="F2" s="177"/>
-      <c r="G2" s="177"/>
-      <c r="H2" s="177"/>
-      <c r="I2" s="177"/>
-      <c r="J2" s="177"/>
-      <c r="K2" s="177"/>
-      <c r="L2" s="177"/>
-      <c r="M2" s="177"/>
-      <c r="N2" s="177"/>
-      <c r="O2" s="177"/>
+      <c r="C2" s="273"/>
+      <c r="D2" s="273"/>
+      <c r="E2" s="273"/>
+      <c r="F2" s="273"/>
+      <c r="G2" s="273"/>
+      <c r="H2" s="273"/>
+      <c r="I2" s="273"/>
+      <c r="J2" s="273"/>
+      <c r="K2" s="273"/>
+      <c r="L2" s="273"/>
+      <c r="M2" s="273"/>
+      <c r="N2" s="273"/>
+      <c r="O2" s="273"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" t="s">
@@ -5172,179 +4974,179 @@
     </row>
     <row r="9" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="11" spans="2:15" s="58" customFormat="1">
-      <c r="B11" s="178" t="s">
+      <c r="B11" s="274" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="178"/>
-      <c r="D11" s="178"/>
-      <c r="E11" s="178"/>
-      <c r="G11" s="178" t="s">
+      <c r="C11" s="274"/>
+      <c r="D11" s="274"/>
+      <c r="E11" s="274"/>
+      <c r="G11" s="274" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="178"/>
-      <c r="I11" s="178"/>
-      <c r="J11" s="178"/>
-      <c r="L11" s="178" t="s">
+      <c r="H11" s="274"/>
+      <c r="I11" s="274"/>
+      <c r="J11" s="274"/>
+      <c r="L11" s="274" t="s">
         <v>105</v>
       </c>
-      <c r="M11" s="178"/>
-      <c r="N11" s="178"/>
-      <c r="O11" s="178"/>
+      <c r="M11" s="274"/>
+      <c r="N11" s="274"/>
+      <c r="O11" s="274"/>
     </row>
     <row r="12" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="13" spans="2:15">
-      <c r="B13" s="176"/>
-      <c r="C13" s="176"/>
-      <c r="D13" s="176"/>
-      <c r="E13" s="176"/>
-      <c r="G13" s="176"/>
-      <c r="H13" s="176"/>
-      <c r="I13" s="176"/>
-      <c r="J13" s="176"/>
-      <c r="L13" s="176"/>
-      <c r="M13" s="176"/>
-      <c r="N13" s="176"/>
-      <c r="O13" s="176"/>
+      <c r="B13" s="265"/>
+      <c r="C13" s="265"/>
+      <c r="D13" s="265"/>
+      <c r="E13" s="265"/>
+      <c r="G13" s="265"/>
+      <c r="H13" s="265"/>
+      <c r="I13" s="265"/>
+      <c r="J13" s="265"/>
+      <c r="L13" s="265"/>
+      <c r="M13" s="265"/>
+      <c r="N13" s="265"/>
+      <c r="O13" s="265"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="176"/>
-      <c r="C14" s="176"/>
-      <c r="D14" s="176"/>
-      <c r="E14" s="176"/>
-      <c r="G14" s="176"/>
-      <c r="H14" s="176"/>
-      <c r="I14" s="176"/>
-      <c r="J14" s="176"/>
-      <c r="L14" s="176"/>
-      <c r="M14" s="176"/>
-      <c r="N14" s="176"/>
-      <c r="O14" s="176"/>
+      <c r="B14" s="265"/>
+      <c r="C14" s="265"/>
+      <c r="D14" s="265"/>
+      <c r="E14" s="265"/>
+      <c r="G14" s="265"/>
+      <c r="H14" s="265"/>
+      <c r="I14" s="265"/>
+      <c r="J14" s="265"/>
+      <c r="L14" s="265"/>
+      <c r="M14" s="265"/>
+      <c r="N14" s="265"/>
+      <c r="O14" s="265"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="176"/>
-      <c r="C15" s="176"/>
-      <c r="D15" s="176"/>
-      <c r="E15" s="176"/>
-      <c r="G15" s="176"/>
-      <c r="H15" s="176"/>
-      <c r="I15" s="176"/>
-      <c r="J15" s="176"/>
-      <c r="L15" s="176"/>
-      <c r="M15" s="176"/>
-      <c r="N15" s="176"/>
-      <c r="O15" s="176"/>
+      <c r="B15" s="265"/>
+      <c r="C15" s="265"/>
+      <c r="D15" s="265"/>
+      <c r="E15" s="265"/>
+      <c r="G15" s="265"/>
+      <c r="H15" s="265"/>
+      <c r="I15" s="265"/>
+      <c r="J15" s="265"/>
+      <c r="L15" s="265"/>
+      <c r="M15" s="265"/>
+      <c r="N15" s="265"/>
+      <c r="O15" s="265"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="176"/>
-      <c r="C16" s="176"/>
-      <c r="D16" s="176"/>
-      <c r="E16" s="176"/>
-      <c r="G16" s="176"/>
-      <c r="H16" s="176"/>
-      <c r="I16" s="176"/>
-      <c r="J16" s="176"/>
-      <c r="L16" s="176"/>
-      <c r="M16" s="176"/>
-      <c r="N16" s="176"/>
-      <c r="O16" s="176"/>
+      <c r="B16" s="265"/>
+      <c r="C16" s="265"/>
+      <c r="D16" s="265"/>
+      <c r="E16" s="265"/>
+      <c r="G16" s="265"/>
+      <c r="H16" s="265"/>
+      <c r="I16" s="265"/>
+      <c r="J16" s="265"/>
+      <c r="L16" s="265"/>
+      <c r="M16" s="265"/>
+      <c r="N16" s="265"/>
+      <c r="O16" s="265"/>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="176"/>
-      <c r="C17" s="176"/>
-      <c r="D17" s="176"/>
-      <c r="E17" s="176"/>
-      <c r="G17" s="176"/>
-      <c r="H17" s="176"/>
-      <c r="I17" s="176"/>
-      <c r="J17" s="176"/>
-      <c r="L17" s="176"/>
-      <c r="M17" s="176"/>
-      <c r="N17" s="176"/>
-      <c r="O17" s="176"/>
+      <c r="B17" s="265"/>
+      <c r="C17" s="265"/>
+      <c r="D17" s="265"/>
+      <c r="E17" s="265"/>
+      <c r="G17" s="265"/>
+      <c r="H17" s="265"/>
+      <c r="I17" s="265"/>
+      <c r="J17" s="265"/>
+      <c r="L17" s="265"/>
+      <c r="M17" s="265"/>
+      <c r="N17" s="265"/>
+      <c r="O17" s="265"/>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="176"/>
-      <c r="C18" s="176"/>
-      <c r="D18" s="176"/>
-      <c r="E18" s="176"/>
-      <c r="G18" s="176"/>
-      <c r="H18" s="176"/>
-      <c r="I18" s="176"/>
-      <c r="J18" s="176"/>
-      <c r="L18" s="176"/>
-      <c r="M18" s="176"/>
-      <c r="N18" s="176"/>
-      <c r="O18" s="176"/>
+      <c r="B18" s="265"/>
+      <c r="C18" s="265"/>
+      <c r="D18" s="265"/>
+      <c r="E18" s="265"/>
+      <c r="G18" s="265"/>
+      <c r="H18" s="265"/>
+      <c r="I18" s="265"/>
+      <c r="J18" s="265"/>
+      <c r="L18" s="265"/>
+      <c r="M18" s="265"/>
+      <c r="N18" s="265"/>
+      <c r="O18" s="265"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="B19" s="176"/>
-      <c r="C19" s="176"/>
-      <c r="D19" s="176"/>
-      <c r="E19" s="176"/>
-      <c r="G19" s="176"/>
-      <c r="H19" s="176"/>
-      <c r="I19" s="176"/>
-      <c r="J19" s="176"/>
-      <c r="L19" s="176"/>
-      <c r="M19" s="176"/>
-      <c r="N19" s="176"/>
-      <c r="O19" s="176"/>
+      <c r="B19" s="265"/>
+      <c r="C19" s="265"/>
+      <c r="D19" s="265"/>
+      <c r="E19" s="265"/>
+      <c r="G19" s="265"/>
+      <c r="H19" s="265"/>
+      <c r="I19" s="265"/>
+      <c r="J19" s="265"/>
+      <c r="L19" s="265"/>
+      <c r="M19" s="265"/>
+      <c r="N19" s="265"/>
+      <c r="O19" s="265"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="B20" s="176"/>
-      <c r="C20" s="176"/>
-      <c r="D20" s="176"/>
-      <c r="E20" s="176"/>
-      <c r="G20" s="176"/>
-      <c r="H20" s="176"/>
-      <c r="I20" s="176"/>
-      <c r="J20" s="176"/>
-      <c r="L20" s="176"/>
-      <c r="M20" s="176"/>
-      <c r="N20" s="176"/>
-      <c r="O20" s="176"/>
+      <c r="B20" s="265"/>
+      <c r="C20" s="265"/>
+      <c r="D20" s="265"/>
+      <c r="E20" s="265"/>
+      <c r="G20" s="265"/>
+      <c r="H20" s="265"/>
+      <c r="I20" s="265"/>
+      <c r="J20" s="265"/>
+      <c r="L20" s="265"/>
+      <c r="M20" s="265"/>
+      <c r="N20" s="265"/>
+      <c r="O20" s="265"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="B21" s="176"/>
-      <c r="C21" s="176"/>
-      <c r="D21" s="176"/>
-      <c r="E21" s="176"/>
-      <c r="G21" s="176"/>
-      <c r="H21" s="176"/>
-      <c r="I21" s="176"/>
-      <c r="J21" s="176"/>
-      <c r="L21" s="176"/>
-      <c r="M21" s="176"/>
-      <c r="N21" s="176"/>
-      <c r="O21" s="176"/>
+      <c r="B21" s="265"/>
+      <c r="C21" s="265"/>
+      <c r="D21" s="265"/>
+      <c r="E21" s="265"/>
+      <c r="G21" s="265"/>
+      <c r="H21" s="265"/>
+      <c r="I21" s="265"/>
+      <c r="J21" s="265"/>
+      <c r="L21" s="265"/>
+      <c r="M21" s="265"/>
+      <c r="N21" s="265"/>
+      <c r="O21" s="265"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="B22" s="176"/>
-      <c r="C22" s="176"/>
-      <c r="D22" s="176"/>
-      <c r="E22" s="176"/>
-      <c r="G22" s="176"/>
-      <c r="H22" s="176"/>
-      <c r="I22" s="176"/>
-      <c r="J22" s="176"/>
-      <c r="L22" s="176"/>
-      <c r="M22" s="176"/>
-      <c r="N22" s="176"/>
-      <c r="O22" s="176"/>
+      <c r="B22" s="265"/>
+      <c r="C22" s="265"/>
+      <c r="D22" s="265"/>
+      <c r="E22" s="265"/>
+      <c r="G22" s="265"/>
+      <c r="H22" s="265"/>
+      <c r="I22" s="265"/>
+      <c r="J22" s="265"/>
+      <c r="L22" s="265"/>
+      <c r="M22" s="265"/>
+      <c r="N22" s="265"/>
+      <c r="O22" s="265"/>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="176"/>
-      <c r="C23" s="176"/>
-      <c r="D23" s="176"/>
-      <c r="E23" s="176"/>
-      <c r="G23" s="176"/>
-      <c r="H23" s="176"/>
-      <c r="I23" s="176"/>
-      <c r="J23" s="176"/>
-      <c r="L23" s="176"/>
-      <c r="M23" s="176"/>
-      <c r="N23" s="176"/>
-      <c r="O23" s="176"/>
+      <c r="B23" s="265"/>
+      <c r="C23" s="265"/>
+      <c r="D23" s="265"/>
+      <c r="E23" s="265"/>
+      <c r="G23" s="265"/>
+      <c r="H23" s="265"/>
+      <c r="I23" s="265"/>
+      <c r="J23" s="265"/>
+      <c r="L23" s="265"/>
+      <c r="M23" s="265"/>
+      <c r="N23" s="265"/>
+      <c r="O23" s="265"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5378,35 +5180,35 @@
   <sheetData>
     <row r="1" spans="2:29" ht="4.8" customHeight="1" thickBot="1"/>
     <row r="2" spans="2:29" ht="19.95" customHeight="1" thickBot="1">
-      <c r="B2" s="261" t="s">
+      <c r="B2" s="275" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="262"/>
-      <c r="D2" s="262"/>
-      <c r="E2" s="262"/>
-      <c r="F2" s="262"/>
-      <c r="G2" s="262"/>
-      <c r="H2" s="262"/>
-      <c r="I2" s="262"/>
-      <c r="J2" s="262"/>
-      <c r="K2" s="262"/>
-      <c r="L2" s="262"/>
-      <c r="M2" s="262"/>
-      <c r="N2" s="262"/>
-      <c r="O2" s="262"/>
-      <c r="P2" s="262"/>
-      <c r="Q2" s="262"/>
-      <c r="R2" s="262"/>
-      <c r="S2" s="262"/>
-      <c r="T2" s="262"/>
-      <c r="U2" s="262"/>
-      <c r="V2" s="262"/>
-      <c r="W2" s="262"/>
-      <c r="X2" s="262"/>
-      <c r="Y2" s="262"/>
-      <c r="Z2" s="262"/>
-      <c r="AA2" s="262"/>
-      <c r="AB2" s="263"/>
+      <c r="C2" s="276"/>
+      <c r="D2" s="276"/>
+      <c r="E2" s="276"/>
+      <c r="F2" s="276"/>
+      <c r="G2" s="276"/>
+      <c r="H2" s="276"/>
+      <c r="I2" s="276"/>
+      <c r="J2" s="276"/>
+      <c r="K2" s="276"/>
+      <c r="L2" s="276"/>
+      <c r="M2" s="276"/>
+      <c r="N2" s="276"/>
+      <c r="O2" s="276"/>
+      <c r="P2" s="276"/>
+      <c r="Q2" s="276"/>
+      <c r="R2" s="276"/>
+      <c r="S2" s="276"/>
+      <c r="T2" s="276"/>
+      <c r="U2" s="276"/>
+      <c r="V2" s="276"/>
+      <c r="W2" s="276"/>
+      <c r="X2" s="276"/>
+      <c r="Y2" s="276"/>
+      <c r="Z2" s="276"/>
+      <c r="AA2" s="276"/>
+      <c r="AB2" s="277"/>
       <c r="AC2" s="168"/>
     </row>
     <row r="3" spans="2:29" ht="15" customHeight="1">
@@ -5506,74 +5308,74 @@
       <c r="AB11" s="166"/>
     </row>
     <row r="12" spans="2:29" ht="15" customHeight="1">
-      <c r="B12" s="273" t="s">
+      <c r="B12" s="287" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="275" t="s">
+      <c r="C12" s="289" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="276"/>
-      <c r="E12" s="276"/>
-      <c r="F12" s="276"/>
-      <c r="G12" s="276"/>
-      <c r="H12" s="276"/>
-      <c r="I12" s="276"/>
-      <c r="J12" s="276"/>
-      <c r="K12" s="276"/>
-      <c r="L12" s="277"/>
-      <c r="M12" s="281" t="s">
+      <c r="D12" s="290"/>
+      <c r="E12" s="290"/>
+      <c r="F12" s="290"/>
+      <c r="G12" s="290"/>
+      <c r="H12" s="290"/>
+      <c r="I12" s="290"/>
+      <c r="J12" s="290"/>
+      <c r="K12" s="290"/>
+      <c r="L12" s="291"/>
+      <c r="M12" s="295" t="s">
         <v>113</v>
       </c>
-      <c r="N12" s="281" t="s">
+      <c r="N12" s="295" t="s">
         <v>34</v>
       </c>
-      <c r="O12" s="286" t="s">
+      <c r="O12" s="300" t="s">
         <v>114</v>
       </c>
-      <c r="P12" s="286"/>
-      <c r="Q12" s="286"/>
-      <c r="R12" s="286"/>
-      <c r="S12" s="286"/>
-      <c r="T12" s="286"/>
-      <c r="U12" s="286"/>
-      <c r="V12" s="286"/>
-      <c r="W12" s="286"/>
-      <c r="X12" s="286"/>
-      <c r="Y12" s="286"/>
-      <c r="Z12" s="286"/>
-      <c r="AA12" s="286"/>
-      <c r="AB12" s="287"/>
+      <c r="P12" s="300"/>
+      <c r="Q12" s="300"/>
+      <c r="R12" s="300"/>
+      <c r="S12" s="300"/>
+      <c r="T12" s="300"/>
+      <c r="U12" s="300"/>
+      <c r="V12" s="300"/>
+      <c r="W12" s="300"/>
+      <c r="X12" s="300"/>
+      <c r="Y12" s="300"/>
+      <c r="Z12" s="300"/>
+      <c r="AA12" s="300"/>
+      <c r="AB12" s="301"/>
     </row>
     <row r="13" spans="2:29" ht="15" customHeight="1">
-      <c r="B13" s="274"/>
-      <c r="C13" s="278"/>
-      <c r="D13" s="279"/>
-      <c r="E13" s="279"/>
-      <c r="F13" s="279"/>
-      <c r="G13" s="279"/>
-      <c r="H13" s="279"/>
-      <c r="I13" s="279"/>
-      <c r="J13" s="279"/>
-      <c r="K13" s="279"/>
-      <c r="L13" s="280"/>
-      <c r="M13" s="282"/>
-      <c r="N13" s="282"/>
-      <c r="O13" s="283" t="s">
+      <c r="B13" s="288"/>
+      <c r="C13" s="292"/>
+      <c r="D13" s="293"/>
+      <c r="E13" s="293"/>
+      <c r="F13" s="293"/>
+      <c r="G13" s="293"/>
+      <c r="H13" s="293"/>
+      <c r="I13" s="293"/>
+      <c r="J13" s="293"/>
+      <c r="K13" s="293"/>
+      <c r="L13" s="294"/>
+      <c r="M13" s="296"/>
+      <c r="N13" s="296"/>
+      <c r="O13" s="297" t="s">
         <v>115</v>
       </c>
-      <c r="P13" s="284"/>
-      <c r="Q13" s="285"/>
-      <c r="R13" s="283" t="s">
+      <c r="P13" s="298"/>
+      <c r="Q13" s="299"/>
+      <c r="R13" s="297" t="s">
         <v>116</v>
       </c>
-      <c r="S13" s="284"/>
-      <c r="T13" s="285"/>
-      <c r="U13" s="283" t="s">
+      <c r="S13" s="298"/>
+      <c r="T13" s="299"/>
+      <c r="U13" s="297" t="s">
         <v>117</v>
       </c>
-      <c r="V13" s="284"/>
-      <c r="W13" s="285"/>
-      <c r="X13" s="264" t="s">
+      <c r="V13" s="298"/>
+      <c r="W13" s="299"/>
+      <c r="X13" s="278" t="s">
         <v>118</v>
       </c>
       <c r="Y13" s="173" t="s">
@@ -5582,27 +5384,27 @@
       <c r="Z13" s="174" t="s">
         <v>119</v>
       </c>
-      <c r="AA13" s="266" t="s">
+      <c r="AA13" s="280" t="s">
         <v>120</v>
       </c>
-      <c r="AB13" s="268" t="s">
+      <c r="AB13" s="282" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="14" spans="2:29" ht="15" customHeight="1">
-      <c r="B14" s="274"/>
-      <c r="C14" s="278"/>
-      <c r="D14" s="279"/>
-      <c r="E14" s="279"/>
-      <c r="F14" s="279"/>
-      <c r="G14" s="279"/>
-      <c r="H14" s="279"/>
-      <c r="I14" s="279"/>
-      <c r="J14" s="279"/>
-      <c r="K14" s="279"/>
-      <c r="L14" s="280"/>
-      <c r="M14" s="265"/>
-      <c r="N14" s="265"/>
+      <c r="B14" s="288"/>
+      <c r="C14" s="292"/>
+      <c r="D14" s="293"/>
+      <c r="E14" s="293"/>
+      <c r="F14" s="293"/>
+      <c r="G14" s="293"/>
+      <c r="H14" s="293"/>
+      <c r="I14" s="293"/>
+      <c r="J14" s="293"/>
+      <c r="K14" s="293"/>
+      <c r="L14" s="294"/>
+      <c r="M14" s="279"/>
+      <c r="N14" s="279"/>
       <c r="O14" s="175" t="s">
         <v>122</v>
       </c>
@@ -5630,32 +5432,32 @@
       <c r="W14" s="175" t="s">
         <v>129</v>
       </c>
-      <c r="X14" s="265"/>
+      <c r="X14" s="279"/>
       <c r="Y14" s="173" t="s">
         <v>130</v>
       </c>
       <c r="Z14" s="175" t="s">
         <v>131</v>
       </c>
-      <c r="AA14" s="267"/>
-      <c r="AB14" s="269"/>
+      <c r="AA14" s="281"/>
+      <c r="AB14" s="283"/>
     </row>
     <row r="15" spans="2:29" ht="15" customHeight="1" thickBot="1">
       <c r="B15" s="169">
         <v>1</v>
       </c>
-      <c r="C15" s="270">
+      <c r="C15" s="284">
         <v>2</v>
       </c>
-      <c r="D15" s="271"/>
-      <c r="E15" s="271"/>
-      <c r="F15" s="271"/>
-      <c r="G15" s="271"/>
-      <c r="H15" s="271"/>
-      <c r="I15" s="271"/>
-      <c r="J15" s="271"/>
-      <c r="K15" s="271"/>
-      <c r="L15" s="272"/>
+      <c r="D15" s="285"/>
+      <c r="E15" s="285"/>
+      <c r="F15" s="285"/>
+      <c r="G15" s="285"/>
+      <c r="H15" s="285"/>
+      <c r="I15" s="285"/>
+      <c r="J15" s="285"/>
+      <c r="K15" s="285"/>
+      <c r="L15" s="286"/>
       <c r="M15" s="170">
         <v>3</v>
       </c>
@@ -5745,38 +5547,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="182"/>
-      <c r="C1" s="182"/>
-      <c r="D1" s="182"/>
-      <c r="E1" s="182"/>
-      <c r="F1" s="182"/>
-      <c r="G1" s="182"/>
-      <c r="H1" s="182"/>
-      <c r="I1" s="182"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="262"/>
+      <c r="I1" s="262"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="179" t="s">
+      <c r="B2" s="259" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="179"/>
-      <c r="I2" s="179"/>
+      <c r="C2" s="259"/>
+      <c r="D2" s="259"/>
+      <c r="E2" s="259"/>
+      <c r="F2" s="259"/>
+      <c r="G2" s="259"/>
+      <c r="H2" s="259"/>
+      <c r="I2" s="259"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="180" t="s">
+      <c r="B3" s="260" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="180"/>
-      <c r="D3" s="180"/>
-      <c r="E3" s="180"/>
-      <c r="F3" s="180"/>
-      <c r="G3" s="180"/>
-      <c r="H3" s="180"/>
-      <c r="I3" s="180"/>
+      <c r="C3" s="260"/>
+      <c r="D3" s="260"/>
+      <c r="E3" s="260"/>
+      <c r="F3" s="260"/>
+      <c r="G3" s="260"/>
+      <c r="H3" s="260"/>
+      <c r="I3" s="260"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -5784,10 +5586,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="181" t="s">
+      <c r="C5" s="261" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="181"/>
+      <c r="D5" s="261"/>
       <c r="E5" s="11" t="s">
         <v>38</v>
       </c>
@@ -14174,63 +13976,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="182"/>
-      <c r="C1" s="182"/>
-      <c r="D1" s="182"/>
-      <c r="E1" s="182"/>
-      <c r="F1" s="182"/>
-      <c r="G1" s="182"/>
-      <c r="H1" s="182"/>
-      <c r="I1" s="182"/>
-      <c r="J1" s="182"/>
-      <c r="K1" s="182"/>
-      <c r="L1" s="182"/>
-      <c r="M1" s="182"/>
-      <c r="N1" s="182"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="262"/>
+      <c r="I1" s="262"/>
+      <c r="J1" s="262"/>
+      <c r="K1" s="262"/>
+      <c r="L1" s="262"/>
+      <c r="M1" s="262"/>
+      <c r="N1" s="262"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="179" t="s">
+      <c r="B2" s="259" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="179"/>
-      <c r="I2" s="179"/>
-      <c r="J2" s="179"/>
-      <c r="K2" s="179"/>
-      <c r="L2" s="179"/>
-      <c r="M2" s="179"/>
-      <c r="N2" s="179"/>
+      <c r="C2" s="259"/>
+      <c r="D2" s="259"/>
+      <c r="E2" s="259"/>
+      <c r="F2" s="259"/>
+      <c r="G2" s="259"/>
+      <c r="H2" s="259"/>
+      <c r="I2" s="259"/>
+      <c r="J2" s="259"/>
+      <c r="K2" s="259"/>
+      <c r="L2" s="259"/>
+      <c r="M2" s="259"/>
+      <c r="N2" s="259"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="180" t="s">
+      <c r="B3" s="260" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="180"/>
-      <c r="D3" s="180"/>
-      <c r="E3" s="180"/>
-      <c r="F3" s="180"/>
-      <c r="G3" s="180"/>
-      <c r="H3" s="180"/>
-      <c r="I3" s="180"/>
-      <c r="J3" s="180"/>
-      <c r="K3" s="180"/>
-      <c r="L3" s="180"/>
-      <c r="M3" s="180"/>
-      <c r="N3" s="180"/>
+      <c r="C3" s="260"/>
+      <c r="D3" s="260"/>
+      <c r="E3" s="260"/>
+      <c r="F3" s="260"/>
+      <c r="G3" s="260"/>
+      <c r="H3" s="260"/>
+      <c r="I3" s="260"/>
+      <c r="J3" s="260"/>
+      <c r="K3" s="260"/>
+      <c r="L3" s="260"/>
+      <c r="M3" s="260"/>
+      <c r="N3" s="260"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="183" t="s">
+      <c r="C5" s="263" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="183"/>
+      <c r="D5" s="263"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -16434,35 +16236,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="182"/>
-      <c r="C1" s="182"/>
-      <c r="D1" s="182"/>
-      <c r="E1" s="182"/>
-      <c r="F1" s="182"/>
-      <c r="G1" s="182"/>
-      <c r="H1" s="182"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="262"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="179" t="s">
+      <c r="B2" s="259" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="179"/>
+      <c r="C2" s="259"/>
+      <c r="D2" s="259"/>
+      <c r="E2" s="259"/>
+      <c r="F2" s="259"/>
+      <c r="G2" s="259"/>
+      <c r="H2" s="259"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="180" t="s">
+      <c r="B3" s="260" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="180"/>
-      <c r="D3" s="180"/>
-      <c r="E3" s="180"/>
-      <c r="F3" s="180"/>
-      <c r="G3" s="180"/>
-      <c r="H3" s="180"/>
+      <c r="C3" s="260"/>
+      <c r="D3" s="260"/>
+      <c r="E3" s="260"/>
+      <c r="F3" s="260"/>
+      <c r="G3" s="260"/>
+      <c r="H3" s="260"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -40556,30 +40358,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="185"/>
-      <c r="C1" s="185"/>
-      <c r="D1" s="185"/>
-      <c r="E1" s="185"/>
-      <c r="F1" s="185"/>
-      <c r="G1" s="185"/>
-      <c r="H1" s="185"/>
-      <c r="I1" s="185"/>
-      <c r="J1" s="185"/>
-      <c r="K1" s="185"/>
+      <c r="B1" s="266"/>
+      <c r="C1" s="266"/>
+      <c r="D1" s="266"/>
+      <c r="E1" s="266"/>
+      <c r="F1" s="266"/>
+      <c r="G1" s="266"/>
+      <c r="H1" s="266"/>
+      <c r="I1" s="266"/>
+      <c r="J1" s="266"/>
+      <c r="K1" s="266"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="184" t="s">
+      <c r="B2" s="264" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="176"/>
-      <c r="D2" s="176"/>
-      <c r="E2" s="176"/>
-      <c r="F2" s="176"/>
-      <c r="G2" s="176"/>
-      <c r="H2" s="176"/>
-      <c r="I2" s="176"/>
-      <c r="J2" s="176"/>
-      <c r="K2" s="176"/>
+      <c r="C2" s="265"/>
+      <c r="D2" s="265"/>
+      <c r="E2" s="265"/>
+      <c r="F2" s="265"/>
+      <c r="G2" s="265"/>
+      <c r="H2" s="265"/>
+      <c r="I2" s="265"/>
+      <c r="J2" s="265"/>
+      <c r="K2" s="265"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40699,11 +40501,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="183" t="s">
+      <c r="C11" s="263" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="183"/>
-      <c r="E11" s="183"/>
+      <c r="D11" s="263"/>
+      <c r="E11" s="263"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -40759,26 +40561,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="111.6" customHeight="1">
-      <c r="B1" s="185"/>
-      <c r="C1" s="185"/>
-      <c r="D1" s="185"/>
-      <c r="E1" s="185"/>
-      <c r="F1" s="185"/>
-      <c r="G1" s="185"/>
-      <c r="H1" s="185"/>
-      <c r="I1" s="185"/>
+      <c r="B1" s="266"/>
+      <c r="C1" s="266"/>
+      <c r="D1" s="266"/>
+      <c r="E1" s="266"/>
+      <c r="F1" s="266"/>
+      <c r="G1" s="266"/>
+      <c r="H1" s="266"/>
+      <c r="I1" s="266"/>
     </row>
     <row r="2" spans="2:9" ht="22.95" customHeight="1">
-      <c r="B2" s="184" t="s">
+      <c r="B2" s="264" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="176"/>
-      <c r="D2" s="176"/>
-      <c r="E2" s="176"/>
-      <c r="F2" s="176"/>
-      <c r="G2" s="176"/>
-      <c r="H2" s="176"/>
-      <c r="I2" s="176"/>
+      <c r="C2" s="265"/>
+      <c r="D2" s="265"/>
+      <c r="E2" s="265"/>
+      <c r="F2" s="265"/>
+      <c r="G2" s="265"/>
+      <c r="H2" s="265"/>
+      <c r="I2" s="265"/>
     </row>
     <row r="3" spans="2:9" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40888,12 +40690,12 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="183" t="s">
+      <c r="C11" s="263" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="183"/>
-      <c r="E11" s="183"/>
-      <c r="F11" s="183"/>
+      <c r="D11" s="263"/>
+      <c r="E11" s="263"/>
+      <c r="F11" s="263"/>
       <c r="G11" s="40" t="s">
         <v>29</v>
       </c>
@@ -40931,58 +40733,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="185"/>
-      <c r="C1" s="185"/>
-      <c r="D1" s="185"/>
-      <c r="E1" s="185"/>
-      <c r="F1" s="185"/>
+      <c r="B1" s="266"/>
+      <c r="C1" s="266"/>
+      <c r="D1" s="266"/>
+      <c r="E1" s="266"/>
+      <c r="F1" s="266"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="188" t="s">
+      <c r="B2" s="269" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="188"/>
-      <c r="D2" s="188"/>
-      <c r="E2" s="188"/>
-      <c r="F2" s="188"/>
+      <c r="C2" s="269"/>
+      <c r="D2" s="269"/>
+      <c r="E2" s="269"/>
+      <c r="F2" s="269"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="185"/>
-      <c r="C3" s="185"/>
-      <c r="D3" s="185"/>
-      <c r="E3" s="185"/>
-      <c r="F3" s="185"/>
+      <c r="B3" s="266"/>
+      <c r="C3" s="266"/>
+      <c r="D3" s="266"/>
+      <c r="E3" s="266"/>
+      <c r="F3" s="266"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="186" t="s">
+      <c r="B5" s="267" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="186" t="s">
+      <c r="C5" s="267" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="186" t="s">
+      <c r="D5" s="267" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="187" t="s">
+      <c r="E5" s="268" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="187" t="s">
+      <c r="F5" s="268" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="186"/>
-      <c r="C6" s="186"/>
-      <c r="D6" s="186"/>
-      <c r="E6" s="187"/>
-      <c r="F6" s="187"/>
+      <c r="B6" s="267"/>
+      <c r="C6" s="267"/>
+      <c r="D6" s="267"/>
+      <c r="E6" s="268"/>
+      <c r="F6" s="268"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="186"/>
-      <c r="C7" s="186"/>
-      <c r="D7" s="186"/>
-      <c r="E7" s="187"/>
-      <c r="F7" s="187"/>
+      <c r="B7" s="267"/>
+      <c r="C7" s="267"/>
+      <c r="D7" s="267"/>
+      <c r="E7" s="268"/>
+      <c r="F7" s="268"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -41103,45 +40905,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="240"/>
-      <c r="C1" s="241"/>
-      <c r="D1" s="241"/>
-      <c r="E1" s="241"/>
-      <c r="F1" s="241"/>
-      <c r="G1" s="241"/>
-      <c r="H1" s="241"/>
-      <c r="I1" s="241"/>
-      <c r="J1" s="241"/>
-      <c r="K1" s="241"/>
-      <c r="L1" s="242"/>
+      <c r="B1" s="179"/>
+      <c r="C1" s="180"/>
+      <c r="D1" s="180"/>
+      <c r="E1" s="180"/>
+      <c r="F1" s="180"/>
+      <c r="G1" s="180"/>
+      <c r="H1" s="180"/>
+      <c r="I1" s="180"/>
+      <c r="J1" s="180"/>
+      <c r="K1" s="180"/>
+      <c r="L1" s="181"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="243" t="s">
+      <c r="B2" s="182" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="244"/>
-      <c r="D2" s="244"/>
-      <c r="E2" s="244"/>
-      <c r="F2" s="244"/>
-      <c r="G2" s="244"/>
-      <c r="H2" s="244"/>
-      <c r="I2" s="245"/>
-      <c r="J2" s="249"/>
-      <c r="K2" s="250"/>
-      <c r="L2" s="251"/>
+      <c r="C2" s="183"/>
+      <c r="D2" s="183"/>
+      <c r="E2" s="183"/>
+      <c r="F2" s="183"/>
+      <c r="G2" s="183"/>
+      <c r="H2" s="183"/>
+      <c r="I2" s="184"/>
+      <c r="J2" s="188"/>
+      <c r="K2" s="189"/>
+      <c r="L2" s="190"/>
     </row>
     <row r="3" spans="1:13" ht="14.4" customHeight="1">
-      <c r="B3" s="246"/>
-      <c r="C3" s="247"/>
-      <c r="D3" s="247"/>
-      <c r="E3" s="247"/>
-      <c r="F3" s="247"/>
-      <c r="G3" s="247"/>
-      <c r="H3" s="247"/>
-      <c r="I3" s="248"/>
-      <c r="J3" s="252"/>
-      <c r="K3" s="253"/>
-      <c r="L3" s="254"/>
+      <c r="B3" s="185"/>
+      <c r="C3" s="186"/>
+      <c r="D3" s="186"/>
+      <c r="E3" s="186"/>
+      <c r="F3" s="186"/>
+      <c r="G3" s="186"/>
+      <c r="H3" s="186"/>
+      <c r="I3" s="187"/>
+      <c r="J3" s="191"/>
+      <c r="K3" s="192"/>
+      <c r="L3" s="193"/>
     </row>
     <row r="4" spans="1:13" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -41152,9 +40954,9 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="252"/>
-      <c r="K4" s="253"/>
-      <c r="L4" s="254"/>
+      <c r="J4" s="191"/>
+      <c r="K4" s="192"/>
+      <c r="L4" s="193"/>
     </row>
     <row r="5" spans="1:13" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -41169,9 +40971,9 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="252"/>
-      <c r="K5" s="253"/>
-      <c r="L5" s="254"/>
+      <c r="J5" s="191"/>
+      <c r="K5" s="192"/>
+      <c r="L5" s="193"/>
     </row>
     <row r="6" spans="1:13" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -41186,9 +40988,9 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="255"/>
-      <c r="K6" s="256"/>
-      <c r="L6" s="257"/>
+      <c r="J6" s="194"/>
+      <c r="K6" s="195"/>
+      <c r="L6" s="196"/>
     </row>
     <row r="7" spans="1:13" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -41244,38 +41046,38 @@
       <c r="L9" s="89"/>
     </row>
     <row r="10" spans="1:13" ht="15.6">
-      <c r="B10" s="291" t="s">
+      <c r="B10" s="197" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="292"/>
-      <c r="D10" s="292"/>
-      <c r="E10" s="292"/>
-      <c r="F10" s="293"/>
-      <c r="G10" s="292" t="s">
+      <c r="C10" s="198"/>
+      <c r="D10" s="198"/>
+      <c r="E10" s="198"/>
+      <c r="F10" s="199"/>
+      <c r="G10" s="198" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="292"/>
-      <c r="I10" s="292"/>
-      <c r="J10" s="293"/>
-      <c r="K10" s="292" t="s">
+      <c r="H10" s="198"/>
+      <c r="I10" s="198"/>
+      <c r="J10" s="199"/>
+      <c r="K10" s="198" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="294"/>
+      <c r="L10" s="200"/>
     </row>
     <row r="11" spans="1:13" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="220" t="s">
+      <c r="C11" s="219" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="235"/>
-      <c r="E11" s="235"/>
+      <c r="D11" s="220"/>
+      <c r="E11" s="220"/>
       <c r="F11" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="220" t="s">
+      <c r="G11" s="219" t="s">
         <v>57</v>
       </c>
       <c r="H11" s="221"/>
@@ -41481,56 +41283,56 @@
       <c r="L22" s="122"/>
     </row>
     <row r="23" spans="1:12" ht="16.2" thickBot="1">
-      <c r="B23" s="236"/>
-      <c r="C23" s="237"/>
-      <c r="D23" s="237"/>
-      <c r="E23" s="237"/>
+      <c r="B23" s="222"/>
+      <c r="C23" s="223"/>
+      <c r="D23" s="223"/>
+      <c r="E23" s="223"/>
       <c r="F23" s="123"/>
       <c r="G23" s="123"/>
       <c r="H23" s="124"/>
       <c r="I23" s="124"/>
-      <c r="J23" s="238"/>
-      <c r="K23" s="238"/>
-      <c r="L23" s="239"/>
+      <c r="J23" s="224"/>
+      <c r="K23" s="224"/>
+      <c r="L23" s="225"/>
     </row>
     <row r="24" spans="1:12" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="148" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="295" t="s">
+      <c r="B24" s="226" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="296" t="s">
+      <c r="C24" s="201" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="296"/>
-      <c r="E24" s="296"/>
-      <c r="F24" s="296"/>
-      <c r="G24" s="296"/>
-      <c r="H24" s="296"/>
-      <c r="I24" s="296"/>
-      <c r="J24" s="288" t="s">
+      <c r="D24" s="201"/>
+      <c r="E24" s="201"/>
+      <c r="F24" s="201"/>
+      <c r="G24" s="201"/>
+      <c r="H24" s="201"/>
+      <c r="I24" s="201"/>
+      <c r="J24" s="203" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="289"/>
-      <c r="L24" s="290"/>
+      <c r="K24" s="204"/>
+      <c r="L24" s="205"/>
     </row>
     <row r="25" spans="1:12" ht="31.2">
-      <c r="B25" s="297"/>
-      <c r="C25" s="298"/>
-      <c r="D25" s="298"/>
-      <c r="E25" s="298"/>
-      <c r="F25" s="298"/>
-      <c r="G25" s="298"/>
-      <c r="H25" s="298"/>
-      <c r="I25" s="298"/>
-      <c r="J25" s="299" t="s">
+      <c r="B25" s="227"/>
+      <c r="C25" s="202"/>
+      <c r="D25" s="202"/>
+      <c r="E25" s="202"/>
+      <c r="F25" s="202"/>
+      <c r="G25" s="202"/>
+      <c r="H25" s="202"/>
+      <c r="I25" s="202"/>
+      <c r="J25" s="176" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="300" t="s">
+      <c r="K25" s="177" t="s">
         <v>76</v>
       </c>
-      <c r="L25" s="301" t="s">
+      <c r="L25" s="178" t="s">
         <v>77</v>
       </c>
     </row>
@@ -42064,176 +41866,176 @@
       </c>
     </row>
     <row r="49" spans="2:12" ht="16.2" thickTop="1">
-      <c r="B49" s="202" t="s">
+      <c r="B49" s="241" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="203"/>
-      <c r="D49" s="203"/>
-      <c r="E49" s="203"/>
-      <c r="F49" s="203"/>
-      <c r="G49" s="203"/>
-      <c r="H49" s="203"/>
-      <c r="I49" s="203"/>
-      <c r="J49" s="204"/>
-      <c r="K49" s="233" t="s">
+      <c r="C49" s="242"/>
+      <c r="D49" s="242"/>
+      <c r="E49" s="242"/>
+      <c r="F49" s="242"/>
+      <c r="G49" s="242"/>
+      <c r="H49" s="242"/>
+      <c r="I49" s="242"/>
+      <c r="J49" s="243"/>
+      <c r="K49" s="217" t="s">
         <v>79</v>
       </c>
-      <c r="L49" s="234"/>
+      <c r="L49" s="218"/>
     </row>
     <row r="50" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B50" s="205"/>
-      <c r="C50" s="206"/>
-      <c r="D50" s="206"/>
-      <c r="E50" s="206"/>
-      <c r="F50" s="206"/>
-      <c r="G50" s="206"/>
-      <c r="H50" s="206"/>
-      <c r="I50" s="206"/>
-      <c r="J50" s="207"/>
-      <c r="K50" s="231" t="s">
+      <c r="B50" s="244"/>
+      <c r="C50" s="245"/>
+      <c r="D50" s="245"/>
+      <c r="E50" s="245"/>
+      <c r="F50" s="245"/>
+      <c r="G50" s="245"/>
+      <c r="H50" s="245"/>
+      <c r="I50" s="245"/>
+      <c r="J50" s="246"/>
+      <c r="K50" s="215" t="s">
         <v>103</v>
       </c>
-      <c r="L50" s="232"/>
+      <c r="L50" s="216"/>
     </row>
     <row r="51" spans="2:12" ht="15.6">
       <c r="B51" s="136"/>
-      <c r="C51" s="228"/>
-      <c r="D51" s="228"/>
-      <c r="E51" s="228"/>
-      <c r="F51" s="228"/>
-      <c r="G51" s="228"/>
-      <c r="H51" s="228"/>
-      <c r="I51" s="228"/>
+      <c r="C51" s="212"/>
+      <c r="D51" s="212"/>
+      <c r="E51" s="212"/>
+      <c r="F51" s="212"/>
+      <c r="G51" s="212"/>
+      <c r="H51" s="212"/>
+      <c r="I51" s="212"/>
       <c r="J51" s="137"/>
-      <c r="K51" s="226"/>
-      <c r="L51" s="227"/>
+      <c r="K51" s="210"/>
+      <c r="L51" s="211"/>
     </row>
     <row r="52" spans="2:12" ht="15.6">
       <c r="B52" s="138"/>
-      <c r="C52" s="229"/>
-      <c r="D52" s="229"/>
-      <c r="E52" s="229"/>
-      <c r="F52" s="229"/>
-      <c r="G52" s="229"/>
-      <c r="H52" s="229"/>
-      <c r="I52" s="229"/>
+      <c r="C52" s="213"/>
+      <c r="D52" s="213"/>
+      <c r="E52" s="213"/>
+      <c r="F52" s="213"/>
+      <c r="G52" s="213"/>
+      <c r="H52" s="213"/>
+      <c r="I52" s="213"/>
       <c r="J52" s="139"/>
       <c r="K52" s="154"/>
       <c r="L52" s="140"/>
     </row>
     <row r="53" spans="2:12" ht="15.6">
       <c r="B53" s="138"/>
-      <c r="C53" s="229"/>
-      <c r="D53" s="229"/>
-      <c r="E53" s="229"/>
-      <c r="F53" s="229"/>
-      <c r="G53" s="229"/>
-      <c r="H53" s="229"/>
-      <c r="I53" s="229"/>
+      <c r="C53" s="213"/>
+      <c r="D53" s="213"/>
+      <c r="E53" s="213"/>
+      <c r="F53" s="213"/>
+      <c r="G53" s="213"/>
+      <c r="H53" s="213"/>
+      <c r="I53" s="213"/>
       <c r="J53" s="139"/>
       <c r="K53" s="154"/>
       <c r="L53" s="140"/>
     </row>
     <row r="54" spans="2:12" ht="15.6">
       <c r="B54" s="138"/>
-      <c r="C54" s="229"/>
-      <c r="D54" s="229"/>
-      <c r="E54" s="229"/>
-      <c r="F54" s="229"/>
-      <c r="G54" s="229"/>
-      <c r="H54" s="229"/>
-      <c r="I54" s="229"/>
+      <c r="C54" s="213"/>
+      <c r="D54" s="213"/>
+      <c r="E54" s="213"/>
+      <c r="F54" s="213"/>
+      <c r="G54" s="213"/>
+      <c r="H54" s="213"/>
+      <c r="I54" s="213"/>
       <c r="J54" s="139"/>
       <c r="K54" s="154"/>
       <c r="L54" s="140"/>
     </row>
     <row r="55" spans="2:12" ht="15.6">
       <c r="B55" s="141"/>
-      <c r="C55" s="229"/>
-      <c r="D55" s="229"/>
-      <c r="E55" s="229"/>
-      <c r="F55" s="229"/>
-      <c r="G55" s="229"/>
-      <c r="H55" s="229"/>
-      <c r="I55" s="229"/>
+      <c r="C55" s="213"/>
+      <c r="D55" s="213"/>
+      <c r="E55" s="213"/>
+      <c r="F55" s="213"/>
+      <c r="G55" s="213"/>
+      <c r="H55" s="213"/>
+      <c r="I55" s="213"/>
       <c r="J55" s="142"/>
       <c r="K55" s="143"/>
       <c r="L55" s="144"/>
     </row>
     <row r="56" spans="2:12" ht="15.6">
       <c r="B56" s="141"/>
-      <c r="C56" s="229"/>
-      <c r="D56" s="229"/>
-      <c r="E56" s="229"/>
-      <c r="F56" s="229"/>
-      <c r="G56" s="229"/>
-      <c r="H56" s="229"/>
-      <c r="I56" s="229"/>
+      <c r="C56" s="213"/>
+      <c r="D56" s="213"/>
+      <c r="E56" s="213"/>
+      <c r="F56" s="213"/>
+      <c r="G56" s="213"/>
+      <c r="H56" s="213"/>
+      <c r="I56" s="213"/>
       <c r="J56" s="142"/>
       <c r="K56" s="143"/>
       <c r="L56" s="144"/>
     </row>
     <row r="57" spans="2:12" ht="15.6">
       <c r="B57" s="141"/>
-      <c r="C57" s="229"/>
-      <c r="D57" s="229"/>
-      <c r="E57" s="229"/>
-      <c r="F57" s="229"/>
-      <c r="G57" s="229"/>
-      <c r="H57" s="229"/>
-      <c r="I57" s="229"/>
+      <c r="C57" s="213"/>
+      <c r="D57" s="213"/>
+      <c r="E57" s="213"/>
+      <c r="F57" s="213"/>
+      <c r="G57" s="213"/>
+      <c r="H57" s="213"/>
+      <c r="I57" s="213"/>
       <c r="J57" s="142"/>
-      <c r="K57" s="222"/>
-      <c r="L57" s="223"/>
+      <c r="K57" s="206"/>
+      <c r="L57" s="207"/>
     </row>
     <row r="58" spans="2:12" ht="15.6">
       <c r="B58" s="141"/>
-      <c r="C58" s="229"/>
-      <c r="D58" s="229"/>
-      <c r="E58" s="229"/>
-      <c r="F58" s="229"/>
-      <c r="G58" s="229"/>
-      <c r="H58" s="229"/>
-      <c r="I58" s="229"/>
+      <c r="C58" s="213"/>
+      <c r="D58" s="213"/>
+      <c r="E58" s="213"/>
+      <c r="F58" s="213"/>
+      <c r="G58" s="213"/>
+      <c r="H58" s="213"/>
+      <c r="I58" s="213"/>
       <c r="J58" s="142"/>
-      <c r="K58" s="224"/>
-      <c r="L58" s="225"/>
+      <c r="K58" s="208"/>
+      <c r="L58" s="209"/>
     </row>
     <row r="59" spans="2:12" ht="15.6">
       <c r="B59" s="141"/>
-      <c r="C59" s="229"/>
-      <c r="D59" s="229"/>
-      <c r="E59" s="229"/>
-      <c r="F59" s="229"/>
-      <c r="G59" s="229"/>
-      <c r="H59" s="229"/>
-      <c r="I59" s="229"/>
+      <c r="C59" s="213"/>
+      <c r="D59" s="213"/>
+      <c r="E59" s="213"/>
+      <c r="F59" s="213"/>
+      <c r="G59" s="213"/>
+      <c r="H59" s="213"/>
+      <c r="I59" s="213"/>
       <c r="J59" s="142"/>
       <c r="K59" s="155"/>
       <c r="L59" s="76"/>
     </row>
     <row r="60" spans="2:12" ht="15.6">
       <c r="B60" s="141"/>
-      <c r="C60" s="229"/>
-      <c r="D60" s="229"/>
-      <c r="E60" s="229"/>
-      <c r="F60" s="229"/>
-      <c r="G60" s="229"/>
-      <c r="H60" s="229"/>
-      <c r="I60" s="229"/>
+      <c r="C60" s="213"/>
+      <c r="D60" s="213"/>
+      <c r="E60" s="213"/>
+      <c r="F60" s="213"/>
+      <c r="G60" s="213"/>
+      <c r="H60" s="213"/>
+      <c r="I60" s="213"/>
       <c r="J60" s="142"/>
       <c r="K60" s="155"/>
       <c r="L60" s="76"/>
     </row>
     <row r="61" spans="2:12" ht="15.6">
       <c r="B61" s="141"/>
-      <c r="C61" s="230"/>
-      <c r="D61" s="230"/>
-      <c r="E61" s="230"/>
-      <c r="F61" s="230"/>
-      <c r="G61" s="230"/>
-      <c r="H61" s="230"/>
-      <c r="I61" s="230"/>
+      <c r="C61" s="214"/>
+      <c r="D61" s="214"/>
+      <c r="E61" s="214"/>
+      <c r="F61" s="214"/>
+      <c r="G61" s="214"/>
+      <c r="H61" s="214"/>
+      <c r="I61" s="214"/>
       <c r="J61" s="142"/>
       <c r="K61" s="155"/>
       <c r="L61" s="76"/>
@@ -42252,125 +42054,125 @@
       <c r="L62" s="158"/>
     </row>
     <row r="63" spans="2:12" ht="15.6">
-      <c r="B63" s="189" t="s">
+      <c r="B63" s="228" t="s">
         <v>80</v>
       </c>
-      <c r="C63" s="190"/>
-      <c r="D63" s="190"/>
-      <c r="E63" s="191"/>
-      <c r="F63" s="192" t="s">
+      <c r="C63" s="229"/>
+      <c r="D63" s="229"/>
+      <c r="E63" s="230"/>
+      <c r="F63" s="231" t="s">
         <v>81</v>
       </c>
-      <c r="G63" s="191"/>
-      <c r="H63" s="192" t="s">
+      <c r="G63" s="230"/>
+      <c r="H63" s="231" t="s">
         <v>82</v>
       </c>
-      <c r="I63" s="190"/>
-      <c r="J63" s="191"/>
+      <c r="I63" s="229"/>
+      <c r="J63" s="230"/>
       <c r="K63" s="143"/>
       <c r="L63" s="144"/>
     </row>
     <row r="64" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B64" s="214"/>
-      <c r="C64" s="215"/>
-      <c r="D64" s="215"/>
-      <c r="E64" s="209"/>
-      <c r="F64" s="208"/>
-      <c r="G64" s="209"/>
-      <c r="H64" s="193"/>
-      <c r="I64" s="194"/>
-      <c r="J64" s="195"/>
+      <c r="B64" s="253"/>
+      <c r="C64" s="254"/>
+      <c r="D64" s="254"/>
+      <c r="E64" s="248"/>
+      <c r="F64" s="247"/>
+      <c r="G64" s="248"/>
+      <c r="H64" s="232"/>
+      <c r="I64" s="233"/>
+      <c r="J64" s="234"/>
       <c r="K64" s="143"/>
       <c r="L64" s="144"/>
     </row>
     <row r="65" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B65" s="216"/>
-      <c r="C65" s="217"/>
-      <c r="D65" s="217"/>
-      <c r="E65" s="211"/>
-      <c r="F65" s="210"/>
-      <c r="G65" s="211"/>
-      <c r="H65" s="196"/>
-      <c r="I65" s="197"/>
-      <c r="J65" s="198"/>
+      <c r="B65" s="255"/>
+      <c r="C65" s="256"/>
+      <c r="D65" s="256"/>
+      <c r="E65" s="250"/>
+      <c r="F65" s="249"/>
+      <c r="G65" s="250"/>
+      <c r="H65" s="235"/>
+      <c r="I65" s="236"/>
+      <c r="J65" s="237"/>
       <c r="K65" s="156"/>
       <c r="L65" s="144"/>
     </row>
     <row r="66" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B66" s="216"/>
-      <c r="C66" s="217"/>
-      <c r="D66" s="217"/>
-      <c r="E66" s="211"/>
-      <c r="F66" s="210"/>
-      <c r="G66" s="211"/>
-      <c r="H66" s="196"/>
-      <c r="I66" s="197"/>
-      <c r="J66" s="198"/>
+      <c r="B66" s="255"/>
+      <c r="C66" s="256"/>
+      <c r="D66" s="256"/>
+      <c r="E66" s="250"/>
+      <c r="F66" s="249"/>
+      <c r="G66" s="250"/>
+      <c r="H66" s="235"/>
+      <c r="I66" s="236"/>
+      <c r="J66" s="237"/>
       <c r="K66" s="143"/>
       <c r="L66" s="144"/>
     </row>
     <row r="67" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B67" s="216"/>
-      <c r="C67" s="217"/>
-      <c r="D67" s="217"/>
-      <c r="E67" s="211"/>
-      <c r="F67" s="210"/>
-      <c r="G67" s="211"/>
-      <c r="H67" s="196"/>
-      <c r="I67" s="197"/>
-      <c r="J67" s="198"/>
+      <c r="B67" s="255"/>
+      <c r="C67" s="256"/>
+      <c r="D67" s="256"/>
+      <c r="E67" s="250"/>
+      <c r="F67" s="249"/>
+      <c r="G67" s="250"/>
+      <c r="H67" s="235"/>
+      <c r="I67" s="236"/>
+      <c r="J67" s="237"/>
       <c r="K67" s="155"/>
       <c r="L67" s="76"/>
     </row>
     <row r="68" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B68" s="216"/>
-      <c r="C68" s="217"/>
-      <c r="D68" s="217"/>
-      <c r="E68" s="211"/>
-      <c r="F68" s="210"/>
-      <c r="G68" s="211"/>
-      <c r="H68" s="196"/>
-      <c r="I68" s="197"/>
-      <c r="J68" s="198"/>
+      <c r="B68" s="255"/>
+      <c r="C68" s="256"/>
+      <c r="D68" s="256"/>
+      <c r="E68" s="250"/>
+      <c r="F68" s="249"/>
+      <c r="G68" s="250"/>
+      <c r="H68" s="235"/>
+      <c r="I68" s="236"/>
+      <c r="J68" s="237"/>
       <c r="K68" s="155"/>
       <c r="L68" s="76"/>
     </row>
     <row r="69" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B69" s="216"/>
-      <c r="C69" s="217"/>
-      <c r="D69" s="217"/>
-      <c r="E69" s="211"/>
-      <c r="F69" s="210"/>
-      <c r="G69" s="211"/>
-      <c r="H69" s="196"/>
-      <c r="I69" s="197"/>
-      <c r="J69" s="198"/>
+      <c r="B69" s="255"/>
+      <c r="C69" s="256"/>
+      <c r="D69" s="256"/>
+      <c r="E69" s="250"/>
+      <c r="F69" s="249"/>
+      <c r="G69" s="250"/>
+      <c r="H69" s="235"/>
+      <c r="I69" s="236"/>
+      <c r="J69" s="237"/>
       <c r="K69" s="159"/>
       <c r="L69" s="160"/>
     </row>
     <row r="70" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B70" s="216"/>
-      <c r="C70" s="217"/>
-      <c r="D70" s="217"/>
-      <c r="E70" s="211"/>
-      <c r="F70" s="210"/>
-      <c r="G70" s="211"/>
-      <c r="H70" s="196"/>
-      <c r="I70" s="197"/>
-      <c r="J70" s="198"/>
+      <c r="B70" s="255"/>
+      <c r="C70" s="256"/>
+      <c r="D70" s="256"/>
+      <c r="E70" s="250"/>
+      <c r="F70" s="249"/>
+      <c r="G70" s="250"/>
+      <c r="H70" s="235"/>
+      <c r="I70" s="236"/>
+      <c r="J70" s="237"/>
       <c r="K70" s="159"/>
       <c r="L70" s="160"/>
     </row>
     <row r="71" spans="2:12" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B71" s="218"/>
-      <c r="C71" s="219"/>
-      <c r="D71" s="219"/>
-      <c r="E71" s="213"/>
-      <c r="F71" s="212"/>
-      <c r="G71" s="213"/>
-      <c r="H71" s="199"/>
-      <c r="I71" s="200"/>
-      <c r="J71" s="201"/>
+      <c r="B71" s="257"/>
+      <c r="C71" s="258"/>
+      <c r="D71" s="258"/>
+      <c r="E71" s="252"/>
+      <c r="F71" s="251"/>
+      <c r="G71" s="252"/>
+      <c r="H71" s="238"/>
+      <c r="I71" s="239"/>
+      <c r="J71" s="240"/>
       <c r="K71" s="146"/>
       <c r="L71" s="147"/>
     </row>
@@ -42381,12 +42183,18 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B1:L1"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="J2:L6"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="H63:J63"/>
+    <mergeCell ref="H64:J71"/>
+    <mergeCell ref="B49:J50"/>
+    <mergeCell ref="F64:G71"/>
+    <mergeCell ref="B64:E71"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="B24:B25"/>
     <mergeCell ref="C24:I25"/>
     <mergeCell ref="J24:L24"/>
     <mergeCell ref="K57:L57"/>
@@ -42395,18 +42203,12 @@
     <mergeCell ref="C51:I61"/>
     <mergeCell ref="K50:L50"/>
     <mergeCell ref="K49:L49"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="H63:J63"/>
-    <mergeCell ref="H64:J71"/>
-    <mergeCell ref="B49:J50"/>
-    <mergeCell ref="F64:G71"/>
-    <mergeCell ref="B64:E71"/>
+    <mergeCell ref="B1:L1"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="J2:L6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="K10:L10"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:I48">
     <cfRule type="expression" dxfId="3" priority="1">
@@ -42452,40 +42254,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="185"/>
-      <c r="C1" s="185"/>
-      <c r="D1" s="185"/>
-      <c r="E1" s="185"/>
-      <c r="F1" s="185"/>
-      <c r="G1" s="185"/>
-      <c r="H1" s="185"/>
-      <c r="I1" s="185"/>
-      <c r="J1" s="185"/>
-      <c r="K1" s="185"/>
-      <c r="L1" s="185"/>
-      <c r="M1" s="185"/>
-      <c r="N1" s="185"/>
-      <c r="O1" s="185"/>
-      <c r="P1" s="185"/>
+      <c r="B1" s="266"/>
+      <c r="C1" s="266"/>
+      <c r="D1" s="266"/>
+      <c r="E1" s="266"/>
+      <c r="F1" s="266"/>
+      <c r="G1" s="266"/>
+      <c r="H1" s="266"/>
+      <c r="I1" s="266"/>
+      <c r="J1" s="266"/>
+      <c r="K1" s="266"/>
+      <c r="L1" s="266"/>
+      <c r="M1" s="266"/>
+      <c r="N1" s="266"/>
+      <c r="O1" s="266"/>
+      <c r="P1" s="266"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="184" t="s">
+      <c r="B2" s="264" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="176"/>
-      <c r="D2" s="176"/>
-      <c r="E2" s="176"/>
-      <c r="F2" s="176"/>
-      <c r="G2" s="176"/>
-      <c r="H2" s="176"/>
-      <c r="I2" s="176"/>
-      <c r="J2" s="176"/>
-      <c r="K2" s="176"/>
-      <c r="L2" s="176"/>
-      <c r="M2" s="176"/>
-      <c r="N2" s="176"/>
-      <c r="O2" s="176"/>
-      <c r="P2" s="176"/>
+      <c r="C2" s="265"/>
+      <c r="D2" s="265"/>
+      <c r="E2" s="265"/>
+      <c r="F2" s="265"/>
+      <c r="G2" s="265"/>
+      <c r="H2" s="265"/>
+      <c r="I2" s="265"/>
+      <c r="J2" s="265"/>
+      <c r="K2" s="265"/>
+      <c r="L2" s="265"/>
+      <c r="M2" s="265"/>
+      <c r="N2" s="265"/>
+      <c r="O2" s="265"/>
+      <c r="P2" s="265"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -42512,16 +42314,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="260" t="s">
+      <c r="I4" s="272" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="260"/>
-      <c r="K4" s="260"/>
-      <c r="L4" s="260"/>
-      <c r="M4" s="260"/>
-      <c r="N4" s="260"/>
-      <c r="O4" s="260"/>
-      <c r="P4" s="260"/>
+      <c r="J4" s="272"/>
+      <c r="K4" s="272"/>
+      <c r="L4" s="272"/>
+      <c r="M4" s="272"/>
+      <c r="N4" s="272"/>
+      <c r="O4" s="272"/>
+      <c r="P4" s="272"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -42535,14 +42337,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="260"/>
-      <c r="J5" s="260"/>
-      <c r="K5" s="260"/>
-      <c r="L5" s="260"/>
-      <c r="M5" s="260"/>
-      <c r="N5" s="260"/>
-      <c r="O5" s="260"/>
-      <c r="P5" s="260"/>
+      <c r="I5" s="272"/>
+      <c r="J5" s="272"/>
+      <c r="K5" s="272"/>
+      <c r="L5" s="272"/>
+      <c r="M5" s="272"/>
+      <c r="N5" s="272"/>
+      <c r="O5" s="272"/>
+      <c r="P5" s="272"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -42677,70 +42479,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="183" t="s">
+      <c r="B12" s="263" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="183" t="s">
+      <c r="C12" s="263" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="183"/>
-      <c r="E12" s="183"/>
-      <c r="F12" s="183" t="s">
+      <c r="D12" s="263"/>
+      <c r="E12" s="263"/>
+      <c r="F12" s="263" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="183" t="s">
+      <c r="G12" s="263" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="183" t="s">
+      <c r="H12" s="263" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="183" t="s">
+      <c r="I12" s="263" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="183" t="s">
+      <c r="J12" s="263" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="183"/>
-      <c r="L12" s="183"/>
-      <c r="M12" s="183"/>
-      <c r="N12" s="183"/>
-      <c r="O12" s="183"/>
-      <c r="P12" s="259" t="s">
+      <c r="K12" s="263"/>
+      <c r="L12" s="263"/>
+      <c r="M12" s="263"/>
+      <c r="N12" s="263"/>
+      <c r="O12" s="263"/>
+      <c r="P12" s="271" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="183"/>
-      <c r="C13" s="183"/>
-      <c r="D13" s="183"/>
-      <c r="E13" s="183"/>
-      <c r="F13" s="183"/>
-      <c r="G13" s="183"/>
-      <c r="H13" s="183"/>
-      <c r="I13" s="183"/>
-      <c r="J13" s="258" t="s">
+      <c r="B13" s="263"/>
+      <c r="C13" s="263"/>
+      <c r="D13" s="263"/>
+      <c r="E13" s="263"/>
+      <c r="F13" s="263"/>
+      <c r="G13" s="263"/>
+      <c r="H13" s="263"/>
+      <c r="I13" s="263"/>
+      <c r="J13" s="270" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="258"/>
-      <c r="L13" s="258" t="s">
+      <c r="K13" s="270"/>
+      <c r="L13" s="270" t="s">
         <v>98</v>
       </c>
-      <c r="M13" s="258"/>
-      <c r="N13" s="258" t="s">
+      <c r="M13" s="270"/>
+      <c r="N13" s="270" t="s">
         <v>99</v>
       </c>
-      <c r="O13" s="258"/>
-      <c r="P13" s="259"/>
+      <c r="O13" s="270"/>
+      <c r="P13" s="271"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="183"/>
-      <c r="C14" s="183"/>
-      <c r="D14" s="183"/>
-      <c r="E14" s="183"/>
-      <c r="F14" s="183"/>
-      <c r="G14" s="183"/>
-      <c r="H14" s="183"/>
-      <c r="I14" s="183"/>
+      <c r="B14" s="263"/>
+      <c r="C14" s="263"/>
+      <c r="D14" s="263"/>
+      <c r="E14" s="263"/>
+      <c r="F14" s="263"/>
+      <c r="G14" s="263"/>
+      <c r="H14" s="263"/>
+      <c r="I14" s="263"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -42759,7 +42561,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="259"/>
+      <c r="P14" s="271"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>

</xml_diff>

<commit_message>
fix(progress): improve decimal input with comma support and prevent negative zero display
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504B2336-A84A-4373-AF1D-B46D2CDFD889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29426003-E918-4B30-8B09-2390F7A6E214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="132">
   <si>
     <t>HARGA SATUAN BAHAN, ALAT DAN UPAH</t>
   </si>
@@ -730,7 +730,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="112">
+  <borders count="116">
     <border>
       <left/>
       <right/>
@@ -2065,6 +2065,54 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2072,7 +2120,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="169" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="302">
+  <cellXfs count="306">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2365,24 +2413,8 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2399,24 +2431,8 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="169" fontId="24" fillId="0" borderId="36" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="170" fontId="24" fillId="0" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2433,36 +2449,8 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="38" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="33" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="41" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2481,36 +2469,8 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="49" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="24" fillId="0" borderId="53" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
     <xf numFmtId="2" fontId="24" fillId="0" borderId="54" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2560,20 +2520,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="15" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="24" fillId="0" borderId="52" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="24" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -3042,6 +2988,127 @@
     </xf>
     <xf numFmtId="0" fontId="32" fillId="4" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="112" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="114" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="112" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="114" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="39" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="115" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -4161,40 +4228,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="266"/>
-      <c r="C1" s="266"/>
-      <c r="D1" s="266"/>
-      <c r="E1" s="266"/>
-      <c r="F1" s="266"/>
-      <c r="G1" s="266"/>
-      <c r="H1" s="266"/>
-      <c r="I1" s="266"/>
-      <c r="J1" s="266"/>
-      <c r="K1" s="266"/>
-      <c r="L1" s="266"/>
-      <c r="M1" s="266"/>
-      <c r="N1" s="266"/>
-      <c r="O1" s="266"/>
-      <c r="P1" s="266"/>
+      <c r="B1" s="239"/>
+      <c r="C1" s="239"/>
+      <c r="D1" s="239"/>
+      <c r="E1" s="239"/>
+      <c r="F1" s="239"/>
+      <c r="G1" s="239"/>
+      <c r="H1" s="239"/>
+      <c r="I1" s="239"/>
+      <c r="J1" s="239"/>
+      <c r="K1" s="239"/>
+      <c r="L1" s="239"/>
+      <c r="M1" s="239"/>
+      <c r="N1" s="239"/>
+      <c r="O1" s="239"/>
+      <c r="P1" s="239"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="264" t="s">
+      <c r="B2" s="237" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="265"/>
-      <c r="D2" s="265"/>
-      <c r="E2" s="265"/>
-      <c r="F2" s="265"/>
-      <c r="G2" s="265"/>
-      <c r="H2" s="265"/>
-      <c r="I2" s="265"/>
-      <c r="J2" s="265"/>
-      <c r="K2" s="265"/>
-      <c r="L2" s="265"/>
-      <c r="M2" s="265"/>
-      <c r="N2" s="265"/>
-      <c r="O2" s="265"/>
-      <c r="P2" s="265"/>
+      <c r="C2" s="238"/>
+      <c r="D2" s="238"/>
+      <c r="E2" s="238"/>
+      <c r="F2" s="238"/>
+      <c r="G2" s="238"/>
+      <c r="H2" s="238"/>
+      <c r="I2" s="238"/>
+      <c r="J2" s="238"/>
+      <c r="K2" s="238"/>
+      <c r="L2" s="238"/>
+      <c r="M2" s="238"/>
+      <c r="N2" s="238"/>
+      <c r="O2" s="238"/>
+      <c r="P2" s="238"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4221,16 +4288,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="272" t="s">
+      <c r="I4" s="245" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="272"/>
-      <c r="K4" s="272"/>
-      <c r="L4" s="272"/>
-      <c r="M4" s="272"/>
-      <c r="N4" s="272"/>
-      <c r="O4" s="272"/>
-      <c r="P4" s="272"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
+      <c r="M4" s="245"/>
+      <c r="N4" s="245"/>
+      <c r="O4" s="245"/>
+      <c r="P4" s="245"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4244,14 +4311,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="272"/>
-      <c r="J5" s="272"/>
-      <c r="K5" s="272"/>
-      <c r="L5" s="272"/>
-      <c r="M5" s="272"/>
-      <c r="N5" s="272"/>
-      <c r="O5" s="272"/>
-      <c r="P5" s="272"/>
+      <c r="I5" s="245"/>
+      <c r="J5" s="245"/>
+      <c r="K5" s="245"/>
+      <c r="L5" s="245"/>
+      <c r="M5" s="245"/>
+      <c r="N5" s="245"/>
+      <c r="O5" s="245"/>
+      <c r="P5" s="245"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4386,70 +4453,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="263" t="s">
+      <c r="B12" s="236" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="263" t="s">
+      <c r="C12" s="236" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="263"/>
-      <c r="E12" s="263"/>
-      <c r="F12" s="263" t="s">
+      <c r="D12" s="236"/>
+      <c r="E12" s="236"/>
+      <c r="F12" s="236" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="263" t="s">
+      <c r="G12" s="236" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="263" t="s">
+      <c r="H12" s="236" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="263" t="s">
+      <c r="I12" s="236" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="263" t="s">
+      <c r="J12" s="236" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="263"/>
-      <c r="L12" s="263"/>
-      <c r="M12" s="263"/>
-      <c r="N12" s="263"/>
-      <c r="O12" s="263"/>
-      <c r="P12" s="271" t="s">
+      <c r="K12" s="236"/>
+      <c r="L12" s="236"/>
+      <c r="M12" s="236"/>
+      <c r="N12" s="236"/>
+      <c r="O12" s="236"/>
+      <c r="P12" s="244" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="263"/>
-      <c r="C13" s="263"/>
-      <c r="D13" s="263"/>
-      <c r="E13" s="263"/>
-      <c r="F13" s="263"/>
-      <c r="G13" s="263"/>
-      <c r="H13" s="263"/>
-      <c r="I13" s="263"/>
-      <c r="J13" s="270" t="s">
+      <c r="B13" s="236"/>
+      <c r="C13" s="236"/>
+      <c r="D13" s="236"/>
+      <c r="E13" s="236"/>
+      <c r="F13" s="236"/>
+      <c r="G13" s="236"/>
+      <c r="H13" s="236"/>
+      <c r="I13" s="236"/>
+      <c r="J13" s="243" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="270"/>
-      <c r="L13" s="270" t="s">
+      <c r="K13" s="243"/>
+      <c r="L13" s="243" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="270"/>
-      <c r="N13" s="270" t="s">
+      <c r="M13" s="243"/>
+      <c r="N13" s="243" t="s">
         <v>95</v>
       </c>
-      <c r="O13" s="270"/>
-      <c r="P13" s="271"/>
+      <c r="O13" s="243"/>
+      <c r="P13" s="244"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="263"/>
-      <c r="C14" s="263"/>
-      <c r="D14" s="263"/>
-      <c r="E14" s="263"/>
-      <c r="F14" s="263"/>
-      <c r="G14" s="263"/>
-      <c r="H14" s="263"/>
-      <c r="I14" s="263"/>
+      <c r="B14" s="236"/>
+      <c r="C14" s="236"/>
+      <c r="D14" s="236"/>
+      <c r="E14" s="236"/>
+      <c r="F14" s="236"/>
+      <c r="G14" s="236"/>
+      <c r="H14" s="236"/>
+      <c r="I14" s="236"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -4468,7 +4535,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="271"/>
+      <c r="P14" s="244"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -4891,38 +4958,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="103.2" customHeight="1">
-      <c r="B1" s="265"/>
-      <c r="C1" s="265"/>
-      <c r="D1" s="265"/>
-      <c r="E1" s="265"/>
-      <c r="F1" s="265"/>
-      <c r="G1" s="265"/>
-      <c r="H1" s="265"/>
-      <c r="I1" s="265"/>
-      <c r="J1" s="265"/>
-      <c r="K1" s="265"/>
-      <c r="L1" s="265"/>
-      <c r="M1" s="265"/>
-      <c r="N1" s="265"/>
-      <c r="O1" s="265"/>
+      <c r="B1" s="238"/>
+      <c r="C1" s="238"/>
+      <c r="D1" s="238"/>
+      <c r="E1" s="238"/>
+      <c r="F1" s="238"/>
+      <c r="G1" s="238"/>
+      <c r="H1" s="238"/>
+      <c r="I1" s="238"/>
+      <c r="J1" s="238"/>
+      <c r="K1" s="238"/>
+      <c r="L1" s="238"/>
+      <c r="M1" s="238"/>
+      <c r="N1" s="238"/>
+      <c r="O1" s="238"/>
     </row>
     <row r="2" spans="2:15" ht="22.95" customHeight="1">
-      <c r="B2" s="273" t="s">
+      <c r="B2" s="246" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="273"/>
-      <c r="D2" s="273"/>
-      <c r="E2" s="273"/>
-      <c r="F2" s="273"/>
-      <c r="G2" s="273"/>
-      <c r="H2" s="273"/>
-      <c r="I2" s="273"/>
-      <c r="J2" s="273"/>
-      <c r="K2" s="273"/>
-      <c r="L2" s="273"/>
-      <c r="M2" s="273"/>
-      <c r="N2" s="273"/>
-      <c r="O2" s="273"/>
+      <c r="C2" s="246"/>
+      <c r="D2" s="246"/>
+      <c r="E2" s="246"/>
+      <c r="F2" s="246"/>
+      <c r="G2" s="246"/>
+      <c r="H2" s="246"/>
+      <c r="I2" s="246"/>
+      <c r="J2" s="246"/>
+      <c r="K2" s="246"/>
+      <c r="L2" s="246"/>
+      <c r="M2" s="246"/>
+      <c r="N2" s="246"/>
+      <c r="O2" s="246"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" t="s">
@@ -4974,179 +5041,179 @@
     </row>
     <row r="9" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="11" spans="2:15" s="58" customFormat="1">
-      <c r="B11" s="274" t="s">
+      <c r="B11" s="247" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="274"/>
-      <c r="D11" s="274"/>
-      <c r="E11" s="274"/>
-      <c r="G11" s="274" t="s">
+      <c r="C11" s="247"/>
+      <c r="D11" s="247"/>
+      <c r="E11" s="247"/>
+      <c r="G11" s="247" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="274"/>
-      <c r="I11" s="274"/>
-      <c r="J11" s="274"/>
-      <c r="L11" s="274" t="s">
+      <c r="H11" s="247"/>
+      <c r="I11" s="247"/>
+      <c r="J11" s="247"/>
+      <c r="L11" s="247" t="s">
         <v>105</v>
       </c>
-      <c r="M11" s="274"/>
-      <c r="N11" s="274"/>
-      <c r="O11" s="274"/>
+      <c r="M11" s="247"/>
+      <c r="N11" s="247"/>
+      <c r="O11" s="247"/>
     </row>
     <row r="12" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="13" spans="2:15">
-      <c r="B13" s="265"/>
-      <c r="C13" s="265"/>
-      <c r="D13" s="265"/>
-      <c r="E13" s="265"/>
-      <c r="G13" s="265"/>
-      <c r="H13" s="265"/>
-      <c r="I13" s="265"/>
-      <c r="J13" s="265"/>
-      <c r="L13" s="265"/>
-      <c r="M13" s="265"/>
-      <c r="N13" s="265"/>
-      <c r="O13" s="265"/>
+      <c r="B13" s="238"/>
+      <c r="C13" s="238"/>
+      <c r="D13" s="238"/>
+      <c r="E13" s="238"/>
+      <c r="G13" s="238"/>
+      <c r="H13" s="238"/>
+      <c r="I13" s="238"/>
+      <c r="J13" s="238"/>
+      <c r="L13" s="238"/>
+      <c r="M13" s="238"/>
+      <c r="N13" s="238"/>
+      <c r="O13" s="238"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="265"/>
-      <c r="C14" s="265"/>
-      <c r="D14" s="265"/>
-      <c r="E14" s="265"/>
-      <c r="G14" s="265"/>
-      <c r="H14" s="265"/>
-      <c r="I14" s="265"/>
-      <c r="J14" s="265"/>
-      <c r="L14" s="265"/>
-      <c r="M14" s="265"/>
-      <c r="N14" s="265"/>
-      <c r="O14" s="265"/>
+      <c r="B14" s="238"/>
+      <c r="C14" s="238"/>
+      <c r="D14" s="238"/>
+      <c r="E14" s="238"/>
+      <c r="G14" s="238"/>
+      <c r="H14" s="238"/>
+      <c r="I14" s="238"/>
+      <c r="J14" s="238"/>
+      <c r="L14" s="238"/>
+      <c r="M14" s="238"/>
+      <c r="N14" s="238"/>
+      <c r="O14" s="238"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="265"/>
-      <c r="C15" s="265"/>
-      <c r="D15" s="265"/>
-      <c r="E15" s="265"/>
-      <c r="G15" s="265"/>
-      <c r="H15" s="265"/>
-      <c r="I15" s="265"/>
-      <c r="J15" s="265"/>
-      <c r="L15" s="265"/>
-      <c r="M15" s="265"/>
-      <c r="N15" s="265"/>
-      <c r="O15" s="265"/>
+      <c r="B15" s="238"/>
+      <c r="C15" s="238"/>
+      <c r="D15" s="238"/>
+      <c r="E15" s="238"/>
+      <c r="G15" s="238"/>
+      <c r="H15" s="238"/>
+      <c r="I15" s="238"/>
+      <c r="J15" s="238"/>
+      <c r="L15" s="238"/>
+      <c r="M15" s="238"/>
+      <c r="N15" s="238"/>
+      <c r="O15" s="238"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="265"/>
-      <c r="C16" s="265"/>
-      <c r="D16" s="265"/>
-      <c r="E16" s="265"/>
-      <c r="G16" s="265"/>
-      <c r="H16" s="265"/>
-      <c r="I16" s="265"/>
-      <c r="J16" s="265"/>
-      <c r="L16" s="265"/>
-      <c r="M16" s="265"/>
-      <c r="N16" s="265"/>
-      <c r="O16" s="265"/>
+      <c r="B16" s="238"/>
+      <c r="C16" s="238"/>
+      <c r="D16" s="238"/>
+      <c r="E16" s="238"/>
+      <c r="G16" s="238"/>
+      <c r="H16" s="238"/>
+      <c r="I16" s="238"/>
+      <c r="J16" s="238"/>
+      <c r="L16" s="238"/>
+      <c r="M16" s="238"/>
+      <c r="N16" s="238"/>
+      <c r="O16" s="238"/>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="265"/>
-      <c r="C17" s="265"/>
-      <c r="D17" s="265"/>
-      <c r="E17" s="265"/>
-      <c r="G17" s="265"/>
-      <c r="H17" s="265"/>
-      <c r="I17" s="265"/>
-      <c r="J17" s="265"/>
-      <c r="L17" s="265"/>
-      <c r="M17" s="265"/>
-      <c r="N17" s="265"/>
-      <c r="O17" s="265"/>
+      <c r="B17" s="238"/>
+      <c r="C17" s="238"/>
+      <c r="D17" s="238"/>
+      <c r="E17" s="238"/>
+      <c r="G17" s="238"/>
+      <c r="H17" s="238"/>
+      <c r="I17" s="238"/>
+      <c r="J17" s="238"/>
+      <c r="L17" s="238"/>
+      <c r="M17" s="238"/>
+      <c r="N17" s="238"/>
+      <c r="O17" s="238"/>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="265"/>
-      <c r="C18" s="265"/>
-      <c r="D18" s="265"/>
-      <c r="E18" s="265"/>
-      <c r="G18" s="265"/>
-      <c r="H18" s="265"/>
-      <c r="I18" s="265"/>
-      <c r="J18" s="265"/>
-      <c r="L18" s="265"/>
-      <c r="M18" s="265"/>
-      <c r="N18" s="265"/>
-      <c r="O18" s="265"/>
+      <c r="B18" s="238"/>
+      <c r="C18" s="238"/>
+      <c r="D18" s="238"/>
+      <c r="E18" s="238"/>
+      <c r="G18" s="238"/>
+      <c r="H18" s="238"/>
+      <c r="I18" s="238"/>
+      <c r="J18" s="238"/>
+      <c r="L18" s="238"/>
+      <c r="M18" s="238"/>
+      <c r="N18" s="238"/>
+      <c r="O18" s="238"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="B19" s="265"/>
-      <c r="C19" s="265"/>
-      <c r="D19" s="265"/>
-      <c r="E19" s="265"/>
-      <c r="G19" s="265"/>
-      <c r="H19" s="265"/>
-      <c r="I19" s="265"/>
-      <c r="J19" s="265"/>
-      <c r="L19" s="265"/>
-      <c r="M19" s="265"/>
-      <c r="N19" s="265"/>
-      <c r="O19" s="265"/>
+      <c r="B19" s="238"/>
+      <c r="C19" s="238"/>
+      <c r="D19" s="238"/>
+      <c r="E19" s="238"/>
+      <c r="G19" s="238"/>
+      <c r="H19" s="238"/>
+      <c r="I19" s="238"/>
+      <c r="J19" s="238"/>
+      <c r="L19" s="238"/>
+      <c r="M19" s="238"/>
+      <c r="N19" s="238"/>
+      <c r="O19" s="238"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="B20" s="265"/>
-      <c r="C20" s="265"/>
-      <c r="D20" s="265"/>
-      <c r="E20" s="265"/>
-      <c r="G20" s="265"/>
-      <c r="H20" s="265"/>
-      <c r="I20" s="265"/>
-      <c r="J20" s="265"/>
-      <c r="L20" s="265"/>
-      <c r="M20" s="265"/>
-      <c r="N20" s="265"/>
-      <c r="O20" s="265"/>
+      <c r="B20" s="238"/>
+      <c r="C20" s="238"/>
+      <c r="D20" s="238"/>
+      <c r="E20" s="238"/>
+      <c r="G20" s="238"/>
+      <c r="H20" s="238"/>
+      <c r="I20" s="238"/>
+      <c r="J20" s="238"/>
+      <c r="L20" s="238"/>
+      <c r="M20" s="238"/>
+      <c r="N20" s="238"/>
+      <c r="O20" s="238"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="B21" s="265"/>
-      <c r="C21" s="265"/>
-      <c r="D21" s="265"/>
-      <c r="E21" s="265"/>
-      <c r="G21" s="265"/>
-      <c r="H21" s="265"/>
-      <c r="I21" s="265"/>
-      <c r="J21" s="265"/>
-      <c r="L21" s="265"/>
-      <c r="M21" s="265"/>
-      <c r="N21" s="265"/>
-      <c r="O21" s="265"/>
+      <c r="B21" s="238"/>
+      <c r="C21" s="238"/>
+      <c r="D21" s="238"/>
+      <c r="E21" s="238"/>
+      <c r="G21" s="238"/>
+      <c r="H21" s="238"/>
+      <c r="I21" s="238"/>
+      <c r="J21" s="238"/>
+      <c r="L21" s="238"/>
+      <c r="M21" s="238"/>
+      <c r="N21" s="238"/>
+      <c r="O21" s="238"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="B22" s="265"/>
-      <c r="C22" s="265"/>
-      <c r="D22" s="265"/>
-      <c r="E22" s="265"/>
-      <c r="G22" s="265"/>
-      <c r="H22" s="265"/>
-      <c r="I22" s="265"/>
-      <c r="J22" s="265"/>
-      <c r="L22" s="265"/>
-      <c r="M22" s="265"/>
-      <c r="N22" s="265"/>
-      <c r="O22" s="265"/>
+      <c r="B22" s="238"/>
+      <c r="C22" s="238"/>
+      <c r="D22" s="238"/>
+      <c r="E22" s="238"/>
+      <c r="G22" s="238"/>
+      <c r="H22" s="238"/>
+      <c r="I22" s="238"/>
+      <c r="J22" s="238"/>
+      <c r="L22" s="238"/>
+      <c r="M22" s="238"/>
+      <c r="N22" s="238"/>
+      <c r="O22" s="238"/>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="265"/>
-      <c r="C23" s="265"/>
-      <c r="D23" s="265"/>
-      <c r="E23" s="265"/>
-      <c r="G23" s="265"/>
-      <c r="H23" s="265"/>
-      <c r="I23" s="265"/>
-      <c r="J23" s="265"/>
-      <c r="L23" s="265"/>
-      <c r="M23" s="265"/>
-      <c r="N23" s="265"/>
-      <c r="O23" s="265"/>
+      <c r="B23" s="238"/>
+      <c r="C23" s="238"/>
+      <c r="D23" s="238"/>
+      <c r="E23" s="238"/>
+      <c r="G23" s="238"/>
+      <c r="H23" s="238"/>
+      <c r="I23" s="238"/>
+      <c r="J23" s="238"/>
+      <c r="L23" s="238"/>
+      <c r="M23" s="238"/>
+      <c r="N23" s="238"/>
+      <c r="O23" s="238"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5180,330 +5247,330 @@
   <sheetData>
     <row r="1" spans="2:29" ht="4.8" customHeight="1" thickBot="1"/>
     <row r="2" spans="2:29" ht="19.95" customHeight="1" thickBot="1">
-      <c r="B2" s="275" t="s">
+      <c r="B2" s="248" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="276"/>
-      <c r="D2" s="276"/>
-      <c r="E2" s="276"/>
-      <c r="F2" s="276"/>
-      <c r="G2" s="276"/>
-      <c r="H2" s="276"/>
-      <c r="I2" s="276"/>
-      <c r="J2" s="276"/>
-      <c r="K2" s="276"/>
-      <c r="L2" s="276"/>
-      <c r="M2" s="276"/>
-      <c r="N2" s="276"/>
-      <c r="O2" s="276"/>
-      <c r="P2" s="276"/>
-      <c r="Q2" s="276"/>
-      <c r="R2" s="276"/>
-      <c r="S2" s="276"/>
-      <c r="T2" s="276"/>
-      <c r="U2" s="276"/>
-      <c r="V2" s="276"/>
-      <c r="W2" s="276"/>
-      <c r="X2" s="276"/>
-      <c r="Y2" s="276"/>
-      <c r="Z2" s="276"/>
-      <c r="AA2" s="276"/>
-      <c r="AB2" s="277"/>
-      <c r="AC2" s="168"/>
+      <c r="C2" s="249"/>
+      <c r="D2" s="249"/>
+      <c r="E2" s="249"/>
+      <c r="F2" s="249"/>
+      <c r="G2" s="249"/>
+      <c r="H2" s="249"/>
+      <c r="I2" s="249"/>
+      <c r="J2" s="249"/>
+      <c r="K2" s="249"/>
+      <c r="L2" s="249"/>
+      <c r="M2" s="249"/>
+      <c r="N2" s="249"/>
+      <c r="O2" s="249"/>
+      <c r="P2" s="249"/>
+      <c r="Q2" s="249"/>
+      <c r="R2" s="249"/>
+      <c r="S2" s="249"/>
+      <c r="T2" s="249"/>
+      <c r="U2" s="249"/>
+      <c r="V2" s="249"/>
+      <c r="W2" s="249"/>
+      <c r="X2" s="249"/>
+      <c r="Y2" s="249"/>
+      <c r="Z2" s="249"/>
+      <c r="AA2" s="249"/>
+      <c r="AB2" s="250"/>
+      <c r="AC2" s="141"/>
     </row>
     <row r="3" spans="2:29" ht="15" customHeight="1">
-      <c r="B3" s="167"/>
-      <c r="AB3" s="162"/>
+      <c r="B3" s="140"/>
+      <c r="AB3" s="135"/>
     </row>
     <row r="4" spans="2:29" ht="15" customHeight="1">
-      <c r="B4" s="161" t="s">
+      <c r="B4" s="134" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="163" t="s">
+      <c r="D4" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="AB4" s="162"/>
+      <c r="AB4" s="135"/>
     </row>
     <row r="5" spans="2:29" ht="15" customHeight="1">
-      <c r="B5" s="161" t="s">
+      <c r="B5" s="134" t="s">
         <v>108</v>
       </c>
-      <c r="D5" s="163" t="s">
+      <c r="D5" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="AB5" s="162"/>
+      <c r="AB5" s="135"/>
     </row>
     <row r="6" spans="2:29" ht="15" customHeight="1">
-      <c r="B6" s="161" t="s">
+      <c r="B6" s="134" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="163" t="s">
+      <c r="D6" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="AB6" s="162"/>
+      <c r="AB6" s="135"/>
     </row>
     <row r="7" spans="2:29" ht="15" customHeight="1">
-      <c r="B7" s="161" t="s">
+      <c r="B7" s="134" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="163" t="s">
+      <c r="D7" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="AB7" s="162"/>
+      <c r="AB7" s="135"/>
     </row>
     <row r="8" spans="2:29" ht="15" customHeight="1">
-      <c r="B8" s="161" t="s">
+      <c r="B8" s="134" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="163" t="s">
+      <c r="D8" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="AB8" s="162"/>
+      <c r="AB8" s="135"/>
     </row>
     <row r="9" spans="2:29" ht="15" customHeight="1">
-      <c r="B9" s="161" t="s">
+      <c r="B9" s="134" t="s">
         <v>110</v>
       </c>
-      <c r="D9" s="163" t="s">
+      <c r="D9" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="AB9" s="162"/>
+      <c r="AB9" s="135"/>
     </row>
     <row r="10" spans="2:29" ht="15" customHeight="1">
-      <c r="B10" s="161" t="s">
+      <c r="B10" s="134" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="163" t="s">
+      <c r="D10" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="AB10" s="162"/>
+      <c r="AB10" s="135"/>
     </row>
     <row r="11" spans="2:29" ht="15" customHeight="1" thickBot="1">
-      <c r="B11" s="164"/>
-      <c r="C11" s="165"/>
-      <c r="D11" s="165"/>
-      <c r="E11" s="165"/>
-      <c r="F11" s="165"/>
-      <c r="G11" s="165"/>
-      <c r="H11" s="165"/>
-      <c r="I11" s="165"/>
-      <c r="J11" s="165"/>
-      <c r="K11" s="165"/>
-      <c r="L11" s="165"/>
-      <c r="M11" s="165"/>
-      <c r="N11" s="165"/>
-      <c r="O11" s="165"/>
-      <c r="P11" s="165"/>
-      <c r="Q11" s="165"/>
-      <c r="R11" s="165"/>
-      <c r="S11" s="165"/>
-      <c r="T11" s="165"/>
-      <c r="U11" s="165"/>
-      <c r="V11" s="165"/>
-      <c r="W11" s="165"/>
-      <c r="X11" s="165"/>
-      <c r="Y11" s="165"/>
-      <c r="Z11" s="165"/>
-      <c r="AA11" s="165"/>
-      <c r="AB11" s="166"/>
+      <c r="B11" s="137"/>
+      <c r="C11" s="138"/>
+      <c r="D11" s="138"/>
+      <c r="E11" s="138"/>
+      <c r="F11" s="138"/>
+      <c r="G11" s="138"/>
+      <c r="H11" s="138"/>
+      <c r="I11" s="138"/>
+      <c r="J11" s="138"/>
+      <c r="K11" s="138"/>
+      <c r="L11" s="138"/>
+      <c r="M11" s="138"/>
+      <c r="N11" s="138"/>
+      <c r="O11" s="138"/>
+      <c r="P11" s="138"/>
+      <c r="Q11" s="138"/>
+      <c r="R11" s="138"/>
+      <c r="S11" s="138"/>
+      <c r="T11" s="138"/>
+      <c r="U11" s="138"/>
+      <c r="V11" s="138"/>
+      <c r="W11" s="138"/>
+      <c r="X11" s="138"/>
+      <c r="Y11" s="138"/>
+      <c r="Z11" s="138"/>
+      <c r="AA11" s="138"/>
+      <c r="AB11" s="139"/>
     </row>
     <row r="12" spans="2:29" ht="15" customHeight="1">
-      <c r="B12" s="287" t="s">
+      <c r="B12" s="260" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="289" t="s">
+      <c r="C12" s="262" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="290"/>
-      <c r="E12" s="290"/>
-      <c r="F12" s="290"/>
-      <c r="G12" s="290"/>
-      <c r="H12" s="290"/>
-      <c r="I12" s="290"/>
-      <c r="J12" s="290"/>
-      <c r="K12" s="290"/>
-      <c r="L12" s="291"/>
-      <c r="M12" s="295" t="s">
+      <c r="D12" s="263"/>
+      <c r="E12" s="263"/>
+      <c r="F12" s="263"/>
+      <c r="G12" s="263"/>
+      <c r="H12" s="263"/>
+      <c r="I12" s="263"/>
+      <c r="J12" s="263"/>
+      <c r="K12" s="263"/>
+      <c r="L12" s="264"/>
+      <c r="M12" s="268" t="s">
         <v>113</v>
       </c>
-      <c r="N12" s="295" t="s">
+      <c r="N12" s="268" t="s">
         <v>34</v>
       </c>
-      <c r="O12" s="300" t="s">
+      <c r="O12" s="273" t="s">
         <v>114</v>
       </c>
-      <c r="P12" s="300"/>
-      <c r="Q12" s="300"/>
-      <c r="R12" s="300"/>
-      <c r="S12" s="300"/>
-      <c r="T12" s="300"/>
-      <c r="U12" s="300"/>
-      <c r="V12" s="300"/>
-      <c r="W12" s="300"/>
-      <c r="X12" s="300"/>
-      <c r="Y12" s="300"/>
-      <c r="Z12" s="300"/>
-      <c r="AA12" s="300"/>
-      <c r="AB12" s="301"/>
+      <c r="P12" s="273"/>
+      <c r="Q12" s="273"/>
+      <c r="R12" s="273"/>
+      <c r="S12" s="273"/>
+      <c r="T12" s="273"/>
+      <c r="U12" s="273"/>
+      <c r="V12" s="273"/>
+      <c r="W12" s="273"/>
+      <c r="X12" s="273"/>
+      <c r="Y12" s="273"/>
+      <c r="Z12" s="273"/>
+      <c r="AA12" s="273"/>
+      <c r="AB12" s="274"/>
     </row>
     <row r="13" spans="2:29" ht="15" customHeight="1">
-      <c r="B13" s="288"/>
-      <c r="C13" s="292"/>
-      <c r="D13" s="293"/>
-      <c r="E13" s="293"/>
-      <c r="F13" s="293"/>
-      <c r="G13" s="293"/>
-      <c r="H13" s="293"/>
-      <c r="I13" s="293"/>
-      <c r="J13" s="293"/>
-      <c r="K13" s="293"/>
-      <c r="L13" s="294"/>
-      <c r="M13" s="296"/>
-      <c r="N13" s="296"/>
-      <c r="O13" s="297" t="s">
+      <c r="B13" s="261"/>
+      <c r="C13" s="265"/>
+      <c r="D13" s="266"/>
+      <c r="E13" s="266"/>
+      <c r="F13" s="266"/>
+      <c r="G13" s="266"/>
+      <c r="H13" s="266"/>
+      <c r="I13" s="266"/>
+      <c r="J13" s="266"/>
+      <c r="K13" s="266"/>
+      <c r="L13" s="267"/>
+      <c r="M13" s="269"/>
+      <c r="N13" s="269"/>
+      <c r="O13" s="270" t="s">
         <v>115</v>
       </c>
-      <c r="P13" s="298"/>
-      <c r="Q13" s="299"/>
-      <c r="R13" s="297" t="s">
+      <c r="P13" s="271"/>
+      <c r="Q13" s="272"/>
+      <c r="R13" s="270" t="s">
         <v>116</v>
       </c>
-      <c r="S13" s="298"/>
-      <c r="T13" s="299"/>
-      <c r="U13" s="297" t="s">
+      <c r="S13" s="271"/>
+      <c r="T13" s="272"/>
+      <c r="U13" s="270" t="s">
         <v>117</v>
       </c>
-      <c r="V13" s="298"/>
-      <c r="W13" s="299"/>
-      <c r="X13" s="278" t="s">
+      <c r="V13" s="271"/>
+      <c r="W13" s="272"/>
+      <c r="X13" s="251" t="s">
         <v>118</v>
       </c>
-      <c r="Y13" s="173" t="s">
+      <c r="Y13" s="146" t="s">
         <v>119</v>
       </c>
-      <c r="Z13" s="174" t="s">
+      <c r="Z13" s="147" t="s">
         <v>119</v>
       </c>
-      <c r="AA13" s="280" t="s">
+      <c r="AA13" s="253" t="s">
         <v>120</v>
       </c>
-      <c r="AB13" s="282" t="s">
+      <c r="AB13" s="255" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="14" spans="2:29" ht="15" customHeight="1">
-      <c r="B14" s="288"/>
-      <c r="C14" s="292"/>
-      <c r="D14" s="293"/>
-      <c r="E14" s="293"/>
-      <c r="F14" s="293"/>
-      <c r="G14" s="293"/>
-      <c r="H14" s="293"/>
-      <c r="I14" s="293"/>
-      <c r="J14" s="293"/>
-      <c r="K14" s="293"/>
-      <c r="L14" s="294"/>
-      <c r="M14" s="279"/>
-      <c r="N14" s="279"/>
-      <c r="O14" s="175" t="s">
+      <c r="B14" s="261"/>
+      <c r="C14" s="265"/>
+      <c r="D14" s="266"/>
+      <c r="E14" s="266"/>
+      <c r="F14" s="266"/>
+      <c r="G14" s="266"/>
+      <c r="H14" s="266"/>
+      <c r="I14" s="266"/>
+      <c r="J14" s="266"/>
+      <c r="K14" s="266"/>
+      <c r="L14" s="267"/>
+      <c r="M14" s="252"/>
+      <c r="N14" s="252"/>
+      <c r="O14" s="148" t="s">
         <v>122</v>
       </c>
-      <c r="P14" s="175" t="s">
+      <c r="P14" s="148" t="s">
         <v>123</v>
       </c>
-      <c r="Q14" s="175" t="s">
+      <c r="Q14" s="148" t="s">
         <v>124</v>
       </c>
-      <c r="R14" s="175" t="s">
+      <c r="R14" s="148" t="s">
         <v>125</v>
       </c>
-      <c r="S14" s="175" t="s">
+      <c r="S14" s="148" t="s">
         <v>126</v>
       </c>
-      <c r="T14" s="175" t="s">
+      <c r="T14" s="148" t="s">
         <v>124</v>
       </c>
-      <c r="U14" s="175" t="s">
+      <c r="U14" s="148" t="s">
         <v>127</v>
       </c>
-      <c r="V14" s="175" t="s">
+      <c r="V14" s="148" t="s">
         <v>128</v>
       </c>
-      <c r="W14" s="175" t="s">
+      <c r="W14" s="148" t="s">
         <v>129</v>
       </c>
-      <c r="X14" s="279"/>
-      <c r="Y14" s="173" t="s">
+      <c r="X14" s="252"/>
+      <c r="Y14" s="146" t="s">
         <v>130</v>
       </c>
-      <c r="Z14" s="175" t="s">
+      <c r="Z14" s="148" t="s">
         <v>131</v>
       </c>
-      <c r="AA14" s="281"/>
-      <c r="AB14" s="283"/>
+      <c r="AA14" s="254"/>
+      <c r="AB14" s="256"/>
     </row>
     <row r="15" spans="2:29" ht="15" customHeight="1" thickBot="1">
-      <c r="B15" s="169">
+      <c r="B15" s="142">
         <v>1</v>
       </c>
-      <c r="C15" s="284">
+      <c r="C15" s="257">
         <v>2</v>
       </c>
-      <c r="D15" s="285"/>
-      <c r="E15" s="285"/>
-      <c r="F15" s="285"/>
-      <c r="G15" s="285"/>
-      <c r="H15" s="285"/>
-      <c r="I15" s="285"/>
-      <c r="J15" s="285"/>
-      <c r="K15" s="285"/>
-      <c r="L15" s="286"/>
-      <c r="M15" s="170">
+      <c r="D15" s="258"/>
+      <c r="E15" s="258"/>
+      <c r="F15" s="258"/>
+      <c r="G15" s="258"/>
+      <c r="H15" s="258"/>
+      <c r="I15" s="258"/>
+      <c r="J15" s="258"/>
+      <c r="K15" s="258"/>
+      <c r="L15" s="259"/>
+      <c r="M15" s="143">
         <v>3</v>
       </c>
-      <c r="N15" s="170">
+      <c r="N15" s="143">
         <v>4</v>
       </c>
-      <c r="O15" s="171">
+      <c r="O15" s="144">
         <v>5</v>
       </c>
-      <c r="P15" s="171">
+      <c r="P15" s="144">
         <v>6</v>
       </c>
-      <c r="Q15" s="171">
+      <c r="Q15" s="144">
         <v>7</v>
       </c>
-      <c r="R15" s="171">
+      <c r="R15" s="144">
         <v>8</v>
       </c>
-      <c r="S15" s="171">
+      <c r="S15" s="144">
         <v>9</v>
       </c>
-      <c r="T15" s="171">
+      <c r="T15" s="144">
         <v>10</v>
       </c>
-      <c r="U15" s="171">
+      <c r="U15" s="144">
         <v>11</v>
       </c>
-      <c r="V15" s="171">
+      <c r="V15" s="144">
         <v>12</v>
       </c>
-      <c r="W15" s="171">
+      <c r="W15" s="144">
         <v>13</v>
       </c>
-      <c r="X15" s="171">
+      <c r="X15" s="144">
         <v>14</v>
       </c>
-      <c r="Y15" s="171">
+      <c r="Y15" s="144">
         <v>15</v>
       </c>
-      <c r="Z15" s="171">
+      <c r="Z15" s="144">
         <v>16</v>
       </c>
-      <c r="AA15" s="171">
+      <c r="AA15" s="144">
         <v>17</v>
       </c>
-      <c r="AB15" s="172">
+      <c r="AB15" s="145">
         <v>18</v>
       </c>
     </row>
@@ -5547,38 +5614,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="262"/>
-      <c r="C1" s="262"/>
-      <c r="D1" s="262"/>
-      <c r="E1" s="262"/>
-      <c r="F1" s="262"/>
-      <c r="G1" s="262"/>
-      <c r="H1" s="262"/>
-      <c r="I1" s="262"/>
+      <c r="B1" s="235"/>
+      <c r="C1" s="235"/>
+      <c r="D1" s="235"/>
+      <c r="E1" s="235"/>
+      <c r="F1" s="235"/>
+      <c r="G1" s="235"/>
+      <c r="H1" s="235"/>
+      <c r="I1" s="235"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="232" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="259"/>
-      <c r="D2" s="259"/>
-      <c r="E2" s="259"/>
-      <c r="F2" s="259"/>
-      <c r="G2" s="259"/>
-      <c r="H2" s="259"/>
-      <c r="I2" s="259"/>
+      <c r="C2" s="232"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
+      <c r="G2" s="232"/>
+      <c r="H2" s="232"/>
+      <c r="I2" s="232"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="260" t="s">
+      <c r="B3" s="233" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="260"/>
-      <c r="D3" s="260"/>
-      <c r="E3" s="260"/>
-      <c r="F3" s="260"/>
-      <c r="G3" s="260"/>
-      <c r="H3" s="260"/>
-      <c r="I3" s="260"/>
+      <c r="C3" s="233"/>
+      <c r="D3" s="233"/>
+      <c r="E3" s="233"/>
+      <c r="F3" s="233"/>
+      <c r="G3" s="233"/>
+      <c r="H3" s="233"/>
+      <c r="I3" s="233"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -5586,10 +5653,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="261" t="s">
+      <c r="C5" s="234" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="261"/>
+      <c r="D5" s="234"/>
       <c r="E5" s="11" t="s">
         <v>38</v>
       </c>
@@ -13976,63 +14043,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="262"/>
-      <c r="C1" s="262"/>
-      <c r="D1" s="262"/>
-      <c r="E1" s="262"/>
-      <c r="F1" s="262"/>
-      <c r="G1" s="262"/>
-      <c r="H1" s="262"/>
-      <c r="I1" s="262"/>
-      <c r="J1" s="262"/>
-      <c r="K1" s="262"/>
-      <c r="L1" s="262"/>
-      <c r="M1" s="262"/>
-      <c r="N1" s="262"/>
+      <c r="B1" s="235"/>
+      <c r="C1" s="235"/>
+      <c r="D1" s="235"/>
+      <c r="E1" s="235"/>
+      <c r="F1" s="235"/>
+      <c r="G1" s="235"/>
+      <c r="H1" s="235"/>
+      <c r="I1" s="235"/>
+      <c r="J1" s="235"/>
+      <c r="K1" s="235"/>
+      <c r="L1" s="235"/>
+      <c r="M1" s="235"/>
+      <c r="N1" s="235"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="232" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="259"/>
-      <c r="D2" s="259"/>
-      <c r="E2" s="259"/>
-      <c r="F2" s="259"/>
-      <c r="G2" s="259"/>
-      <c r="H2" s="259"/>
-      <c r="I2" s="259"/>
-      <c r="J2" s="259"/>
-      <c r="K2" s="259"/>
-      <c r="L2" s="259"/>
-      <c r="M2" s="259"/>
-      <c r="N2" s="259"/>
+      <c r="C2" s="232"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
+      <c r="G2" s="232"/>
+      <c r="H2" s="232"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
+      <c r="M2" s="232"/>
+      <c r="N2" s="232"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="260" t="s">
+      <c r="B3" s="233" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="260"/>
-      <c r="D3" s="260"/>
-      <c r="E3" s="260"/>
-      <c r="F3" s="260"/>
-      <c r="G3" s="260"/>
-      <c r="H3" s="260"/>
-      <c r="I3" s="260"/>
-      <c r="J3" s="260"/>
-      <c r="K3" s="260"/>
-      <c r="L3" s="260"/>
-      <c r="M3" s="260"/>
-      <c r="N3" s="260"/>
+      <c r="C3" s="233"/>
+      <c r="D3" s="233"/>
+      <c r="E3" s="233"/>
+      <c r="F3" s="233"/>
+      <c r="G3" s="233"/>
+      <c r="H3" s="233"/>
+      <c r="I3" s="233"/>
+      <c r="J3" s="233"/>
+      <c r="K3" s="233"/>
+      <c r="L3" s="233"/>
+      <c r="M3" s="233"/>
+      <c r="N3" s="233"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="263" t="s">
+      <c r="C5" s="236" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="263"/>
+      <c r="D5" s="236"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -16236,35 +16303,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="262"/>
-      <c r="C1" s="262"/>
-      <c r="D1" s="262"/>
-      <c r="E1" s="262"/>
-      <c r="F1" s="262"/>
-      <c r="G1" s="262"/>
-      <c r="H1" s="262"/>
+      <c r="B1" s="235"/>
+      <c r="C1" s="235"/>
+      <c r="D1" s="235"/>
+      <c r="E1" s="235"/>
+      <c r="F1" s="235"/>
+      <c r="G1" s="235"/>
+      <c r="H1" s="235"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="232" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="259"/>
-      <c r="D2" s="259"/>
-      <c r="E2" s="259"/>
-      <c r="F2" s="259"/>
-      <c r="G2" s="259"/>
-      <c r="H2" s="259"/>
+      <c r="C2" s="232"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
+      <c r="G2" s="232"/>
+      <c r="H2" s="232"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="260" t="s">
+      <c r="B3" s="233" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="260"/>
-      <c r="D3" s="260"/>
-      <c r="E3" s="260"/>
-      <c r="F3" s="260"/>
-      <c r="G3" s="260"/>
-      <c r="H3" s="260"/>
+      <c r="C3" s="233"/>
+      <c r="D3" s="233"/>
+      <c r="E3" s="233"/>
+      <c r="F3" s="233"/>
+      <c r="G3" s="233"/>
+      <c r="H3" s="233"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -40358,30 +40425,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="266"/>
-      <c r="C1" s="266"/>
-      <c r="D1" s="266"/>
-      <c r="E1" s="266"/>
-      <c r="F1" s="266"/>
-      <c r="G1" s="266"/>
-      <c r="H1" s="266"/>
-      <c r="I1" s="266"/>
-      <c r="J1" s="266"/>
-      <c r="K1" s="266"/>
+      <c r="B1" s="239"/>
+      <c r="C1" s="239"/>
+      <c r="D1" s="239"/>
+      <c r="E1" s="239"/>
+      <c r="F1" s="239"/>
+      <c r="G1" s="239"/>
+      <c r="H1" s="239"/>
+      <c r="I1" s="239"/>
+      <c r="J1" s="239"/>
+      <c r="K1" s="239"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="264" t="s">
+      <c r="B2" s="237" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="265"/>
-      <c r="D2" s="265"/>
-      <c r="E2" s="265"/>
-      <c r="F2" s="265"/>
-      <c r="G2" s="265"/>
-      <c r="H2" s="265"/>
-      <c r="I2" s="265"/>
-      <c r="J2" s="265"/>
-      <c r="K2" s="265"/>
+      <c r="C2" s="238"/>
+      <c r="D2" s="238"/>
+      <c r="E2" s="238"/>
+      <c r="F2" s="238"/>
+      <c r="G2" s="238"/>
+      <c r="H2" s="238"/>
+      <c r="I2" s="238"/>
+      <c r="J2" s="238"/>
+      <c r="K2" s="238"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40501,11 +40568,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="263" t="s">
+      <c r="C11" s="236" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="263"/>
-      <c r="E11" s="263"/>
+      <c r="D11" s="236"/>
+      <c r="E11" s="236"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -40561,26 +40628,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="111.6" customHeight="1">
-      <c r="B1" s="266"/>
-      <c r="C1" s="266"/>
-      <c r="D1" s="266"/>
-      <c r="E1" s="266"/>
-      <c r="F1" s="266"/>
-      <c r="G1" s="266"/>
-      <c r="H1" s="266"/>
-      <c r="I1" s="266"/>
+      <c r="B1" s="239"/>
+      <c r="C1" s="239"/>
+      <c r="D1" s="239"/>
+      <c r="E1" s="239"/>
+      <c r="F1" s="239"/>
+      <c r="G1" s="239"/>
+      <c r="H1" s="239"/>
+      <c r="I1" s="239"/>
     </row>
     <row r="2" spans="2:9" ht="22.95" customHeight="1">
-      <c r="B2" s="264" t="s">
+      <c r="B2" s="237" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="265"/>
-      <c r="D2" s="265"/>
-      <c r="E2" s="265"/>
-      <c r="F2" s="265"/>
-      <c r="G2" s="265"/>
-      <c r="H2" s="265"/>
-      <c r="I2" s="265"/>
+      <c r="C2" s="238"/>
+      <c r="D2" s="238"/>
+      <c r="E2" s="238"/>
+      <c r="F2" s="238"/>
+      <c r="G2" s="238"/>
+      <c r="H2" s="238"/>
+      <c r="I2" s="238"/>
     </row>
     <row r="3" spans="2:9" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40690,12 +40757,12 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="263" t="s">
+      <c r="C11" s="236" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="263"/>
-      <c r="E11" s="263"/>
-      <c r="F11" s="263"/>
+      <c r="D11" s="236"/>
+      <c r="E11" s="236"/>
+      <c r="F11" s="236"/>
       <c r="G11" s="40" t="s">
         <v>29</v>
       </c>
@@ -40733,58 +40800,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="266"/>
-      <c r="C1" s="266"/>
-      <c r="D1" s="266"/>
-      <c r="E1" s="266"/>
-      <c r="F1" s="266"/>
+      <c r="B1" s="239"/>
+      <c r="C1" s="239"/>
+      <c r="D1" s="239"/>
+      <c r="E1" s="239"/>
+      <c r="F1" s="239"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="269" t="s">
+      <c r="B2" s="242" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="269"/>
-      <c r="D2" s="269"/>
-      <c r="E2" s="269"/>
-      <c r="F2" s="269"/>
+      <c r="C2" s="242"/>
+      <c r="D2" s="242"/>
+      <c r="E2" s="242"/>
+      <c r="F2" s="242"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="266"/>
-      <c r="C3" s="266"/>
-      <c r="D3" s="266"/>
-      <c r="E3" s="266"/>
-      <c r="F3" s="266"/>
+      <c r="B3" s="239"/>
+      <c r="C3" s="239"/>
+      <c r="D3" s="239"/>
+      <c r="E3" s="239"/>
+      <c r="F3" s="239"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="267" t="s">
+      <c r="B5" s="240" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="267" t="s">
+      <c r="C5" s="240" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="267" t="s">
+      <c r="D5" s="240" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="268" t="s">
+      <c r="E5" s="241" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="268" t="s">
+      <c r="F5" s="241" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="267"/>
-      <c r="C6" s="267"/>
-      <c r="D6" s="267"/>
-      <c r="E6" s="268"/>
-      <c r="F6" s="268"/>
+      <c r="B6" s="240"/>
+      <c r="C6" s="240"/>
+      <c r="D6" s="240"/>
+      <c r="E6" s="241"/>
+      <c r="F6" s="241"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="267"/>
-      <c r="C7" s="267"/>
-      <c r="D7" s="267"/>
-      <c r="E7" s="268"/>
-      <c r="F7" s="268"/>
+      <c r="B7" s="240"/>
+      <c r="C7" s="240"/>
+      <c r="D7" s="240"/>
+      <c r="E7" s="241"/>
+      <c r="F7" s="241"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -40905,45 +40972,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="179"/>
-      <c r="C1" s="180"/>
-      <c r="D1" s="180"/>
-      <c r="E1" s="180"/>
-      <c r="F1" s="180"/>
-      <c r="G1" s="180"/>
-      <c r="H1" s="180"/>
-      <c r="I1" s="180"/>
-      <c r="J1" s="180"/>
-      <c r="K1" s="180"/>
-      <c r="L1" s="181"/>
+      <c r="B1" s="152"/>
+      <c r="C1" s="153"/>
+      <c r="D1" s="153"/>
+      <c r="E1" s="153"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="153"/>
+      <c r="H1" s="153"/>
+      <c r="I1" s="153"/>
+      <c r="J1" s="153"/>
+      <c r="K1" s="153"/>
+      <c r="L1" s="154"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="182" t="s">
+      <c r="B2" s="155" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="183"/>
-      <c r="D2" s="183"/>
-      <c r="E2" s="183"/>
-      <c r="F2" s="183"/>
-      <c r="G2" s="183"/>
-      <c r="H2" s="183"/>
-      <c r="I2" s="184"/>
-      <c r="J2" s="188"/>
-      <c r="K2" s="189"/>
-      <c r="L2" s="190"/>
+      <c r="C2" s="156"/>
+      <c r="D2" s="156"/>
+      <c r="E2" s="156"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="156"/>
+      <c r="H2" s="156"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="161"/>
+      <c r="K2" s="162"/>
+      <c r="L2" s="163"/>
     </row>
     <row r="3" spans="1:13" ht="14.4" customHeight="1">
-      <c r="B3" s="185"/>
-      <c r="C3" s="186"/>
-      <c r="D3" s="186"/>
-      <c r="E3" s="186"/>
-      <c r="F3" s="186"/>
-      <c r="G3" s="186"/>
-      <c r="H3" s="186"/>
-      <c r="I3" s="187"/>
-      <c r="J3" s="191"/>
-      <c r="K3" s="192"/>
-      <c r="L3" s="193"/>
+      <c r="B3" s="158"/>
+      <c r="C3" s="159"/>
+      <c r="D3" s="159"/>
+      <c r="E3" s="159"/>
+      <c r="F3" s="159"/>
+      <c r="G3" s="159"/>
+      <c r="H3" s="159"/>
+      <c r="I3" s="160"/>
+      <c r="J3" s="164"/>
+      <c r="K3" s="165"/>
+      <c r="L3" s="166"/>
     </row>
     <row r="4" spans="1:13" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -40954,9 +41021,9 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="191"/>
-      <c r="K4" s="192"/>
-      <c r="L4" s="193"/>
+      <c r="J4" s="164"/>
+      <c r="K4" s="165"/>
+      <c r="L4" s="166"/>
     </row>
     <row r="5" spans="1:13" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -40971,9 +41038,9 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="191"/>
-      <c r="K5" s="192"/>
-      <c r="L5" s="193"/>
+      <c r="J5" s="164"/>
+      <c r="K5" s="165"/>
+      <c r="L5" s="166"/>
     </row>
     <row r="6" spans="1:13" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -40988,9 +41055,9 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="194"/>
-      <c r="K6" s="195"/>
-      <c r="L6" s="196"/>
+      <c r="J6" s="167"/>
+      <c r="K6" s="168"/>
+      <c r="L6" s="169"/>
     </row>
     <row r="7" spans="1:13" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -41042,45 +41109,45 @@
       <c r="J9" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="K9" s="149"/>
+      <c r="K9" s="126"/>
       <c r="L9" s="89"/>
     </row>
     <row r="10" spans="1:13" ht="15.6">
-      <c r="B10" s="197" t="s">
+      <c r="B10" s="170" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="198"/>
-      <c r="D10" s="198"/>
-      <c r="E10" s="198"/>
-      <c r="F10" s="199"/>
-      <c r="G10" s="198" t="s">
+      <c r="C10" s="171"/>
+      <c r="D10" s="171"/>
+      <c r="E10" s="171"/>
+      <c r="F10" s="172"/>
+      <c r="G10" s="171" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="198"/>
-      <c r="I10" s="198"/>
-      <c r="J10" s="199"/>
-      <c r="K10" s="198" t="s">
+      <c r="H10" s="171"/>
+      <c r="I10" s="171"/>
+      <c r="J10" s="172"/>
+      <c r="K10" s="171" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="200"/>
+      <c r="L10" s="173"/>
     </row>
     <row r="11" spans="1:13" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="219" t="s">
+      <c r="C11" s="192" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="220"/>
-      <c r="E11" s="220"/>
+      <c r="D11" s="193"/>
+      <c r="E11" s="193"/>
       <c r="F11" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="219" t="s">
+      <c r="G11" s="192" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="221"/>
+      <c r="H11" s="194"/>
       <c r="I11" s="92" t="s">
         <v>27</v>
       </c>
@@ -41099,1082 +41166,1036 @@
       <c r="B12" s="94" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="95" t="s">
+      <c r="C12" s="294" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="96"/>
-      <c r="E12" s="96"/>
-      <c r="F12" s="97"/>
-      <c r="G12" s="98"/>
-      <c r="H12" s="99"/>
-      <c r="I12" s="100"/>
-      <c r="J12" s="100"/>
-      <c r="K12" s="101"/>
-      <c r="L12" s="102"/>
+      <c r="D12" s="295"/>
+      <c r="E12" s="296"/>
+      <c r="F12" s="95"/>
+      <c r="G12" s="275"/>
+      <c r="H12" s="276"/>
+      <c r="I12" s="96"/>
+      <c r="J12" s="96"/>
+      <c r="K12" s="97"/>
+      <c r="L12" s="98"/>
     </row>
     <row r="13" spans="1:13" ht="15.6">
-      <c r="B13" s="103">
+      <c r="B13" s="99">
         <v>1</v>
       </c>
-      <c r="C13" s="104" t="s">
+      <c r="C13" s="297" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="105"/>
-      <c r="E13" s="105"/>
-      <c r="F13" s="106"/>
-      <c r="G13" s="107"/>
-      <c r="H13" s="108"/>
-      <c r="I13" s="109"/>
-      <c r="J13" s="110"/>
-      <c r="K13" s="111"/>
-      <c r="L13" s="112"/>
+      <c r="D13" s="298"/>
+      <c r="E13" s="299"/>
+      <c r="F13" s="100"/>
+      <c r="G13" s="277"/>
+      <c r="H13" s="278"/>
+      <c r="I13" s="101"/>
+      <c r="J13" s="102"/>
+      <c r="K13" s="103"/>
+      <c r="L13" s="104"/>
     </row>
     <row r="14" spans="1:13" ht="15.6">
-      <c r="B14" s="103">
+      <c r="B14" s="99">
         <v>2</v>
       </c>
-      <c r="C14" s="104" t="s">
+      <c r="C14" s="297" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="105"/>
-      <c r="E14" s="105"/>
-      <c r="F14" s="106"/>
-      <c r="G14" s="107"/>
-      <c r="H14" s="108"/>
-      <c r="I14" s="109"/>
-      <c r="J14" s="110"/>
-      <c r="K14" s="111"/>
-      <c r="L14" s="112"/>
+      <c r="D14" s="298"/>
+      <c r="E14" s="299"/>
+      <c r="F14" s="100"/>
+      <c r="G14" s="277"/>
+      <c r="H14" s="278"/>
+      <c r="I14" s="101"/>
+      <c r="J14" s="102"/>
+      <c r="K14" s="103"/>
+      <c r="L14" s="104"/>
     </row>
     <row r="15" spans="1:13" ht="15.6">
-      <c r="B15" s="103">
+      <c r="B15" s="99">
         <v>3</v>
       </c>
-      <c r="C15" s="104" t="s">
+      <c r="C15" s="297" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="105"/>
-      <c r="E15" s="105"/>
-      <c r="F15" s="106"/>
-      <c r="G15" s="107"/>
-      <c r="H15" s="113"/>
-      <c r="I15" s="109"/>
-      <c r="J15" s="110"/>
-      <c r="K15" s="111"/>
-      <c r="L15" s="112"/>
+      <c r="D15" s="298"/>
+      <c r="E15" s="299"/>
+      <c r="F15" s="100"/>
+      <c r="G15" s="277"/>
+      <c r="H15" s="278"/>
+      <c r="I15" s="101"/>
+      <c r="J15" s="102"/>
+      <c r="K15" s="103"/>
+      <c r="L15" s="104"/>
     </row>
     <row r="16" spans="1:13" ht="15.6">
-      <c r="B16" s="103">
+      <c r="B16" s="99">
         <v>4</v>
       </c>
-      <c r="C16" s="104" t="s">
+      <c r="C16" s="297" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="105"/>
-      <c r="E16" s="105"/>
-      <c r="F16" s="106"/>
-      <c r="G16" s="107"/>
-      <c r="H16" s="108"/>
-      <c r="I16" s="109"/>
-      <c r="J16" s="110"/>
-      <c r="K16" s="111"/>
-      <c r="L16" s="112"/>
+      <c r="D16" s="298"/>
+      <c r="E16" s="299"/>
+      <c r="F16" s="100"/>
+      <c r="G16" s="277"/>
+      <c r="H16" s="278"/>
+      <c r="I16" s="101"/>
+      <c r="J16" s="102"/>
+      <c r="K16" s="103"/>
+      <c r="L16" s="104"/>
     </row>
     <row r="17" spans="1:12" ht="15.6">
-      <c r="B17" s="103">
+      <c r="B17" s="99">
         <v>5</v>
       </c>
-      <c r="C17" s="104" t="s">
+      <c r="C17" s="297" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="105"/>
-      <c r="E17" s="105"/>
-      <c r="F17" s="106"/>
-      <c r="G17" s="107"/>
-      <c r="H17" s="108"/>
-      <c r="I17" s="109"/>
-      <c r="J17" s="110"/>
-      <c r="K17" s="111"/>
-      <c r="L17" s="112"/>
+      <c r="D17" s="298"/>
+      <c r="E17" s="299"/>
+      <c r="F17" s="100"/>
+      <c r="G17" s="277"/>
+      <c r="H17" s="278"/>
+      <c r="I17" s="101"/>
+      <c r="J17" s="102"/>
+      <c r="K17" s="103"/>
+      <c r="L17" s="104"/>
     </row>
     <row r="18" spans="1:12" ht="15.6">
-      <c r="B18" s="103">
+      <c r="B18" s="99">
         <v>6</v>
       </c>
-      <c r="C18" s="104" t="s">
+      <c r="C18" s="297" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="105"/>
-      <c r="E18" s="105"/>
-      <c r="F18" s="106"/>
-      <c r="G18" s="107"/>
-      <c r="H18" s="114"/>
-      <c r="I18" s="109"/>
-      <c r="J18" s="110"/>
-      <c r="K18" s="111"/>
-      <c r="L18" s="112"/>
+      <c r="D18" s="298"/>
+      <c r="E18" s="299"/>
+      <c r="F18" s="100"/>
+      <c r="G18" s="277"/>
+      <c r="H18" s="278"/>
+      <c r="I18" s="101"/>
+      <c r="J18" s="102"/>
+      <c r="K18" s="103"/>
+      <c r="L18" s="104"/>
     </row>
     <row r="19" spans="1:12" ht="15.6">
-      <c r="B19" s="115" t="s">
+      <c r="B19" s="105" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="116" t="s">
+      <c r="C19" s="300" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="117"/>
-      <c r="E19" s="117"/>
-      <c r="F19" s="106"/>
-      <c r="G19" s="118"/>
-      <c r="H19" s="114"/>
-      <c r="I19" s="109"/>
-      <c r="J19" s="110"/>
-      <c r="K19" s="111"/>
-      <c r="L19" s="112"/>
+      <c r="D19" s="301"/>
+      <c r="E19" s="302"/>
+      <c r="F19" s="100"/>
+      <c r="G19" s="277"/>
+      <c r="H19" s="278"/>
+      <c r="I19" s="101"/>
+      <c r="J19" s="102"/>
+      <c r="K19" s="103"/>
+      <c r="L19" s="104"/>
     </row>
     <row r="20" spans="1:12" ht="15.6">
-      <c r="B20" s="103">
+      <c r="B20" s="99">
         <v>1</v>
       </c>
-      <c r="C20" s="104" t="s">
+      <c r="C20" s="297" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="105"/>
-      <c r="E20" s="105"/>
-      <c r="F20" s="106"/>
-      <c r="G20" s="118"/>
-      <c r="H20" s="114"/>
-      <c r="I20" s="109"/>
-      <c r="J20" s="110"/>
-      <c r="K20" s="111"/>
-      <c r="L20" s="112"/>
+      <c r="D20" s="298"/>
+      <c r="E20" s="299"/>
+      <c r="F20" s="100"/>
+      <c r="G20" s="277"/>
+      <c r="H20" s="278"/>
+      <c r="I20" s="101"/>
+      <c r="J20" s="102"/>
+      <c r="K20" s="103"/>
+      <c r="L20" s="104"/>
     </row>
     <row r="21" spans="1:12" ht="15.6">
-      <c r="B21" s="103">
+      <c r="B21" s="99">
         <v>2</v>
       </c>
-      <c r="C21" s="104" t="s">
+      <c r="C21" s="297" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="105"/>
-      <c r="E21" s="105"/>
-      <c r="F21" s="106"/>
-      <c r="G21" s="118"/>
-      <c r="H21" s="114"/>
-      <c r="I21" s="109"/>
-      <c r="J21" s="110"/>
-      <c r="K21" s="111"/>
-      <c r="L21" s="112"/>
+      <c r="D21" s="298"/>
+      <c r="E21" s="299"/>
+      <c r="F21" s="100"/>
+      <c r="G21" s="277"/>
+      <c r="H21" s="278"/>
+      <c r="I21" s="101"/>
+      <c r="J21" s="102"/>
+      <c r="K21" s="103"/>
+      <c r="L21" s="104"/>
     </row>
     <row r="22" spans="1:12" ht="15.6">
-      <c r="B22" s="103">
+      <c r="B22" s="99">
         <v>3</v>
       </c>
-      <c r="C22" s="104" t="s">
+      <c r="C22" s="303" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="105"/>
-      <c r="E22" s="105"/>
-      <c r="F22" s="106"/>
-      <c r="G22" s="119"/>
-      <c r="H22" s="120"/>
-      <c r="I22" s="109"/>
-      <c r="J22" s="110"/>
-      <c r="K22" s="121"/>
-      <c r="L22" s="122"/>
+      <c r="D22" s="304"/>
+      <c r="E22" s="305"/>
+      <c r="F22" s="100"/>
+      <c r="G22" s="279"/>
+      <c r="H22" s="280"/>
+      <c r="I22" s="101"/>
+      <c r="J22" s="102"/>
+      <c r="K22" s="106"/>
+      <c r="L22" s="107"/>
     </row>
     <row r="23" spans="1:12" ht="16.2" thickBot="1">
-      <c r="B23" s="222"/>
-      <c r="C23" s="223"/>
-      <c r="D23" s="223"/>
-      <c r="E23" s="223"/>
-      <c r="F23" s="123"/>
-      <c r="G23" s="123"/>
-      <c r="H23" s="124"/>
-      <c r="I23" s="124"/>
-      <c r="J23" s="224"/>
-      <c r="K23" s="224"/>
-      <c r="L23" s="225"/>
+      <c r="B23" s="195"/>
+      <c r="C23" s="196"/>
+      <c r="D23" s="196"/>
+      <c r="E23" s="196"/>
+      <c r="F23" s="108"/>
+      <c r="G23" s="108"/>
+      <c r="H23" s="109"/>
+      <c r="I23" s="109"/>
+      <c r="J23" s="197"/>
+      <c r="K23" s="197"/>
+      <c r="L23" s="198"/>
     </row>
     <row r="24" spans="1:12" ht="16.2" customHeight="1" thickTop="1">
-      <c r="A24" s="148" t="s">
+      <c r="A24" s="125" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="226" t="s">
+      <c r="B24" s="199" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="201" t="s">
+      <c r="C24" s="174" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="201"/>
-      <c r="E24" s="201"/>
-      <c r="F24" s="201"/>
-      <c r="G24" s="201"/>
-      <c r="H24" s="201"/>
-      <c r="I24" s="201"/>
-      <c r="J24" s="203" t="s">
+      <c r="D24" s="174"/>
+      <c r="E24" s="174"/>
+      <c r="F24" s="174"/>
+      <c r="G24" s="174"/>
+      <c r="H24" s="174"/>
+      <c r="I24" s="174"/>
+      <c r="J24" s="176" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="204"/>
-      <c r="L24" s="205"/>
+      <c r="K24" s="177"/>
+      <c r="L24" s="178"/>
     </row>
     <row r="25" spans="1:12" ht="31.2">
-      <c r="B25" s="227"/>
-      <c r="C25" s="202"/>
-      <c r="D25" s="202"/>
-      <c r="E25" s="202"/>
-      <c r="F25" s="202"/>
-      <c r="G25" s="202"/>
-      <c r="H25" s="202"/>
-      <c r="I25" s="202"/>
-      <c r="J25" s="176" t="s">
+      <c r="B25" s="200"/>
+      <c r="C25" s="175"/>
+      <c r="D25" s="175"/>
+      <c r="E25" s="175"/>
+      <c r="F25" s="175"/>
+      <c r="G25" s="175"/>
+      <c r="H25" s="175"/>
+      <c r="I25" s="175"/>
+      <c r="J25" s="149" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="177" t="s">
+      <c r="K25" s="150" t="s">
         <v>76</v>
       </c>
-      <c r="L25" s="178" t="s">
+      <c r="L25" s="151" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.6">
-      <c r="B26" s="125" t="s">
+      <c r="B26" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="126" t="s">
+      <c r="C26" s="281" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="150"/>
-      <c r="E26" s="127"/>
-      <c r="F26" s="127"/>
-      <c r="G26" s="127"/>
-      <c r="H26" s="127"/>
-      <c r="I26" s="128"/>
-      <c r="J26" s="129" t="s">
+      <c r="D26" s="282"/>
+      <c r="E26" s="282"/>
+      <c r="F26" s="282"/>
+      <c r="G26" s="282"/>
+      <c r="H26" s="282"/>
+      <c r="I26" s="283"/>
+      <c r="J26" s="281" t="s">
         <v>64</v>
       </c>
-      <c r="K26" s="152" t="s">
+      <c r="K26" s="283"/>
+      <c r="L26" s="111" t="s">
         <v>64</v>
       </c>
-      <c r="L26" s="130" t="s">
+    </row>
+    <row r="27" spans="1:12" ht="15.6">
+      <c r="B27" s="110" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" ht="15.6">
-      <c r="B27" s="125" t="s">
+      <c r="C27" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="C27" s="131" t="s">
+      <c r="D27" s="285"/>
+      <c r="E27" s="285"/>
+      <c r="F27" s="285"/>
+      <c r="G27" s="285"/>
+      <c r="H27" s="285"/>
+      <c r="I27" s="286"/>
+      <c r="J27" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="D27" s="151"/>
-      <c r="E27" s="132"/>
-      <c r="F27" s="132"/>
-      <c r="G27" s="132"/>
-      <c r="H27" s="132"/>
-      <c r="I27" s="133"/>
-      <c r="J27" s="134" t="s">
+      <c r="K27" s="291"/>
+      <c r="L27" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="K27" s="153" t="s">
+    </row>
+    <row r="28" spans="1:12" ht="15.6">
+      <c r="B28" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="L27" s="135" t="s">
+      <c r="C28" s="284" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" ht="15.6">
-      <c r="B28" s="125" t="s">
+      <c r="D28" s="285"/>
+      <c r="E28" s="285"/>
+      <c r="F28" s="285"/>
+      <c r="G28" s="285"/>
+      <c r="H28" s="285"/>
+      <c r="I28" s="286"/>
+      <c r="J28" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="131" t="s">
+      <c r="K28" s="291"/>
+      <c r="L28" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="D28" s="151"/>
-      <c r="E28" s="132"/>
-      <c r="F28" s="132"/>
-      <c r="G28" s="132"/>
-      <c r="H28" s="132"/>
-      <c r="I28" s="133"/>
-      <c r="J28" s="134" t="s">
+    </row>
+    <row r="29" spans="1:12" ht="15.6">
+      <c r="B29" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="K28" s="153" t="s">
+      <c r="C29" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="L28" s="135" t="s">
+      <c r="D29" s="285"/>
+      <c r="E29" s="285"/>
+      <c r="F29" s="285"/>
+      <c r="G29" s="285"/>
+      <c r="H29" s="285"/>
+      <c r="I29" s="286"/>
+      <c r="J29" s="290" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" ht="15.6">
-      <c r="B29" s="125" t="s">
+      <c r="K29" s="291"/>
+      <c r="L29" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="131" t="s">
+    </row>
+    <row r="30" spans="1:12" ht="15.6">
+      <c r="B30" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="151"/>
-      <c r="E29" s="132"/>
-      <c r="F29" s="132"/>
-      <c r="G29" s="132"/>
-      <c r="H29" s="132"/>
-      <c r="I29" s="133"/>
-      <c r="J29" s="134" t="s">
+      <c r="C30" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="K29" s="153" t="s">
+      <c r="D30" s="285"/>
+      <c r="E30" s="285"/>
+      <c r="F30" s="285"/>
+      <c r="G30" s="285"/>
+      <c r="H30" s="285"/>
+      <c r="I30" s="286"/>
+      <c r="J30" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="L29" s="135" t="s">
+      <c r="K30" s="291"/>
+      <c r="L30" s="112" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="15.6">
-      <c r="B30" s="125" t="s">
+    <row r="31" spans="1:12" ht="15.6">
+      <c r="B31" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="131" t="s">
+      <c r="C31" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="151"/>
-      <c r="E30" s="132"/>
-      <c r="F30" s="132"/>
-      <c r="G30" s="132"/>
-      <c r="H30" s="132"/>
-      <c r="I30" s="133"/>
-      <c r="J30" s="134" t="s">
+      <c r="D31" s="285"/>
+      <c r="E31" s="285"/>
+      <c r="F31" s="285"/>
+      <c r="G31" s="285"/>
+      <c r="H31" s="285"/>
+      <c r="I31" s="286"/>
+      <c r="J31" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="K30" s="153" t="s">
+      <c r="K31" s="291"/>
+      <c r="L31" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="L30" s="135" t="s">
+    </row>
+    <row r="32" spans="1:12" ht="15.6">
+      <c r="B32" s="110" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" ht="15.6">
-      <c r="B31" s="125" t="s">
+      <c r="C32" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="131" t="s">
+      <c r="D32" s="285"/>
+      <c r="E32" s="285"/>
+      <c r="F32" s="285"/>
+      <c r="G32" s="285"/>
+      <c r="H32" s="285"/>
+      <c r="I32" s="286"/>
+      <c r="J32" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="151"/>
-      <c r="E31" s="132"/>
-      <c r="F31" s="132"/>
-      <c r="G31" s="132"/>
-      <c r="H31" s="132"/>
-      <c r="I31" s="133"/>
-      <c r="J31" s="134" t="s">
+      <c r="K32" s="291"/>
+      <c r="L32" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="K31" s="153" t="s">
+    </row>
+    <row r="33" spans="2:12" ht="15.6">
+      <c r="B33" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="L31" s="135" t="s">
+      <c r="C33" s="284" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" ht="15.6">
-      <c r="B32" s="125" t="s">
+      <c r="D33" s="285"/>
+      <c r="E33" s="285"/>
+      <c r="F33" s="285"/>
+      <c r="G33" s="285"/>
+      <c r="H33" s="285"/>
+      <c r="I33" s="286"/>
+      <c r="J33" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="131" t="s">
+      <c r="K33" s="291"/>
+      <c r="L33" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="151"/>
-      <c r="E32" s="132"/>
-      <c r="F32" s="132"/>
-      <c r="G32" s="132"/>
-      <c r="H32" s="132"/>
-      <c r="I32" s="133"/>
-      <c r="J32" s="134" t="s">
+    </row>
+    <row r="34" spans="2:12" ht="15.6">
+      <c r="B34" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="K32" s="153" t="s">
+      <c r="C34" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="L32" s="135" t="s">
+      <c r="D34" s="285"/>
+      <c r="E34" s="285"/>
+      <c r="F34" s="285"/>
+      <c r="G34" s="285"/>
+      <c r="H34" s="285"/>
+      <c r="I34" s="286"/>
+      <c r="J34" s="290" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="33" spans="2:12" ht="15.6">
-      <c r="B33" s="125" t="s">
+      <c r="K34" s="291"/>
+      <c r="L34" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="131" t="s">
+    </row>
+    <row r="35" spans="2:12" ht="15.6">
+      <c r="B35" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="151"/>
-      <c r="E33" s="132"/>
-      <c r="F33" s="132"/>
-      <c r="G33" s="132"/>
-      <c r="H33" s="132"/>
-      <c r="I33" s="133"/>
-      <c r="J33" s="134" t="s">
+      <c r="C35" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="K33" s="153" t="s">
+      <c r="D35" s="285"/>
+      <c r="E35" s="285"/>
+      <c r="F35" s="285"/>
+      <c r="G35" s="285"/>
+      <c r="H35" s="285"/>
+      <c r="I35" s="286"/>
+      <c r="J35" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="L33" s="135" t="s">
+      <c r="K35" s="291"/>
+      <c r="L35" s="112" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="2:12" ht="15.6">
-      <c r="B34" s="125" t="s">
+    <row r="36" spans="2:12" ht="15.6">
+      <c r="B36" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="131" t="s">
+      <c r="C36" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="151"/>
-      <c r="E34" s="132"/>
-      <c r="F34" s="132"/>
-      <c r="G34" s="132"/>
-      <c r="H34" s="132"/>
-      <c r="I34" s="133"/>
-      <c r="J34" s="134" t="s">
+      <c r="D36" s="285"/>
+      <c r="E36" s="285"/>
+      <c r="F36" s="285"/>
+      <c r="G36" s="285"/>
+      <c r="H36" s="285"/>
+      <c r="I36" s="286"/>
+      <c r="J36" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="K34" s="153" t="s">
+      <c r="K36" s="291"/>
+      <c r="L36" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="L34" s="135" t="s">
+    </row>
+    <row r="37" spans="2:12" ht="15.6">
+      <c r="B37" s="110" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="35" spans="2:12" ht="15.6">
-      <c r="B35" s="125" t="s">
+      <c r="C37" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="131" t="s">
+      <c r="D37" s="285"/>
+      <c r="E37" s="285"/>
+      <c r="F37" s="285"/>
+      <c r="G37" s="285"/>
+      <c r="H37" s="285"/>
+      <c r="I37" s="286"/>
+      <c r="J37" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="151"/>
-      <c r="E35" s="132"/>
-      <c r="F35" s="132"/>
-      <c r="G35" s="132"/>
-      <c r="H35" s="132"/>
-      <c r="I35" s="133"/>
-      <c r="J35" s="134" t="s">
+      <c r="K37" s="291"/>
+      <c r="L37" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="K35" s="153" t="s">
+    </row>
+    <row r="38" spans="2:12" ht="15.6">
+      <c r="B38" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="L35" s="135" t="s">
+      <c r="C38" s="284" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="36" spans="2:12" ht="15.6">
-      <c r="B36" s="125" t="s">
+      <c r="D38" s="285"/>
+      <c r="E38" s="285"/>
+      <c r="F38" s="285"/>
+      <c r="G38" s="285"/>
+      <c r="H38" s="285"/>
+      <c r="I38" s="286"/>
+      <c r="J38" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="C36" s="131" t="s">
+      <c r="K38" s="291"/>
+      <c r="L38" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="151"/>
-      <c r="E36" s="132"/>
-      <c r="F36" s="132"/>
-      <c r="G36" s="132"/>
-      <c r="H36" s="132"/>
-      <c r="I36" s="133"/>
-      <c r="J36" s="134" t="s">
+    </row>
+    <row r="39" spans="2:12" ht="15.6">
+      <c r="B39" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="K36" s="153" t="s">
+      <c r="C39" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="L36" s="135" t="s">
+      <c r="D39" s="285"/>
+      <c r="E39" s="285"/>
+      <c r="F39" s="285"/>
+      <c r="G39" s="285"/>
+      <c r="H39" s="285"/>
+      <c r="I39" s="286"/>
+      <c r="J39" s="290" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="37" spans="2:12" ht="15.6">
-      <c r="B37" s="125" t="s">
+      <c r="K39" s="291"/>
+      <c r="L39" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="131" t="s">
+    </row>
+    <row r="40" spans="2:12" ht="15.6">
+      <c r="B40" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="151"/>
-      <c r="E37" s="132"/>
-      <c r="F37" s="132"/>
-      <c r="G37" s="132"/>
-      <c r="H37" s="132"/>
-      <c r="I37" s="133"/>
-      <c r="J37" s="134" t="s">
+      <c r="C40" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="K37" s="153" t="s">
+      <c r="D40" s="285"/>
+      <c r="E40" s="285"/>
+      <c r="F40" s="285"/>
+      <c r="G40" s="285"/>
+      <c r="H40" s="285"/>
+      <c r="I40" s="286"/>
+      <c r="J40" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="L37" s="135" t="s">
+      <c r="K40" s="291"/>
+      <c r="L40" s="112" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="2:12" ht="15.6">
-      <c r="B38" s="125" t="s">
+    <row r="41" spans="2:12" ht="15.6">
+      <c r="B41" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="131" t="s">
+      <c r="C41" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="151"/>
-      <c r="E38" s="132"/>
-      <c r="F38" s="132"/>
-      <c r="G38" s="132"/>
-      <c r="H38" s="132"/>
-      <c r="I38" s="133"/>
-      <c r="J38" s="134" t="s">
+      <c r="D41" s="285"/>
+      <c r="E41" s="285"/>
+      <c r="F41" s="285"/>
+      <c r="G41" s="285"/>
+      <c r="H41" s="285"/>
+      <c r="I41" s="286"/>
+      <c r="J41" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="K38" s="153" t="s">
+      <c r="K41" s="291"/>
+      <c r="L41" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="L38" s="135" t="s">
+    </row>
+    <row r="42" spans="2:12" ht="15.6">
+      <c r="B42" s="110" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="39" spans="2:12" ht="15.6">
-      <c r="B39" s="125" t="s">
+      <c r="C42" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="131" t="s">
+      <c r="D42" s="285"/>
+      <c r="E42" s="285"/>
+      <c r="F42" s="285"/>
+      <c r="G42" s="285"/>
+      <c r="H42" s="285"/>
+      <c r="I42" s="286"/>
+      <c r="J42" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="D39" s="151"/>
-      <c r="E39" s="132"/>
-      <c r="F39" s="132"/>
-      <c r="G39" s="132"/>
-      <c r="H39" s="132"/>
-      <c r="I39" s="133"/>
-      <c r="J39" s="134" t="s">
+      <c r="K42" s="291"/>
+      <c r="L42" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="K39" s="153" t="s">
+    </row>
+    <row r="43" spans="2:12" ht="15.6">
+      <c r="B43" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="L39" s="135" t="s">
+      <c r="C43" s="284" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="40" spans="2:12" ht="15.6">
-      <c r="B40" s="125" t="s">
+      <c r="D43" s="285"/>
+      <c r="E43" s="285"/>
+      <c r="F43" s="285"/>
+      <c r="G43" s="285"/>
+      <c r="H43" s="285"/>
+      <c r="I43" s="286"/>
+      <c r="J43" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="131" t="s">
+      <c r="K43" s="291"/>
+      <c r="L43" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="D40" s="151"/>
-      <c r="E40" s="132"/>
-      <c r="F40" s="132"/>
-      <c r="G40" s="132"/>
-      <c r="H40" s="132"/>
-      <c r="I40" s="133"/>
-      <c r="J40" s="134" t="s">
+    </row>
+    <row r="44" spans="2:12" ht="15.6">
+      <c r="B44" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="K40" s="153" t="s">
+      <c r="C44" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="L40" s="135" t="s">
+      <c r="D44" s="285"/>
+      <c r="E44" s="285"/>
+      <c r="F44" s="285"/>
+      <c r="G44" s="285"/>
+      <c r="H44" s="285"/>
+      <c r="I44" s="286"/>
+      <c r="J44" s="290" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="41" spans="2:12" ht="15.6">
-      <c r="B41" s="125" t="s">
+      <c r="K44" s="291"/>
+      <c r="L44" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="131" t="s">
+    </row>
+    <row r="45" spans="2:12" ht="15.6">
+      <c r="B45" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="D41" s="151"/>
-      <c r="E41" s="132"/>
-      <c r="F41" s="132"/>
-      <c r="G41" s="132"/>
-      <c r="H41" s="132"/>
-      <c r="I41" s="133"/>
-      <c r="J41" s="134" t="s">
+      <c r="C45" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="K41" s="153" t="s">
+      <c r="D45" s="285"/>
+      <c r="E45" s="285"/>
+      <c r="F45" s="285"/>
+      <c r="G45" s="285"/>
+      <c r="H45" s="285"/>
+      <c r="I45" s="286"/>
+      <c r="J45" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="L41" s="135" t="s">
+      <c r="K45" s="291"/>
+      <c r="L45" s="112" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="42" spans="2:12" ht="15.6">
-      <c r="B42" s="125" t="s">
+    <row r="46" spans="2:12" ht="15.6">
+      <c r="B46" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="131" t="s">
+      <c r="C46" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="151"/>
-      <c r="E42" s="132"/>
-      <c r="F42" s="132"/>
-      <c r="G42" s="132"/>
-      <c r="H42" s="132"/>
-      <c r="I42" s="133"/>
-      <c r="J42" s="134" t="s">
+      <c r="D46" s="285"/>
+      <c r="E46" s="285"/>
+      <c r="F46" s="285"/>
+      <c r="G46" s="285"/>
+      <c r="H46" s="285"/>
+      <c r="I46" s="286"/>
+      <c r="J46" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="K42" s="153" t="s">
+      <c r="K46" s="291"/>
+      <c r="L46" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="L42" s="135" t="s">
+    </row>
+    <row r="47" spans="2:12" ht="15.6">
+      <c r="B47" s="110" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="43" spans="2:12" ht="15.6">
-      <c r="B43" s="125" t="s">
+      <c r="C47" s="284" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="131" t="s">
+      <c r="D47" s="285"/>
+      <c r="E47" s="285"/>
+      <c r="F47" s="285"/>
+      <c r="G47" s="285"/>
+      <c r="H47" s="285"/>
+      <c r="I47" s="286"/>
+      <c r="J47" s="290" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="151"/>
-      <c r="E43" s="132"/>
-      <c r="F43" s="132"/>
-      <c r="G43" s="132"/>
-      <c r="H43" s="132"/>
-      <c r="I43" s="133"/>
-      <c r="J43" s="134" t="s">
+      <c r="K47" s="291"/>
+      <c r="L47" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="K43" s="153" t="s">
+    </row>
+    <row r="48" spans="2:12" ht="16.2" thickBot="1">
+      <c r="B48" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="L43" s="135" t="s">
+      <c r="C48" s="287" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="44" spans="2:12" ht="15.6">
-      <c r="B44" s="125" t="s">
+      <c r="D48" s="288"/>
+      <c r="E48" s="288"/>
+      <c r="F48" s="288"/>
+      <c r="G48" s="288"/>
+      <c r="H48" s="288"/>
+      <c r="I48" s="289"/>
+      <c r="J48" s="292" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="131" t="s">
+      <c r="K48" s="293"/>
+      <c r="L48" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="D44" s="151"/>
-      <c r="E44" s="132"/>
-      <c r="F44" s="132"/>
-      <c r="G44" s="132"/>
-      <c r="H44" s="132"/>
-      <c r="I44" s="133"/>
-      <c r="J44" s="134" t="s">
-        <v>64</v>
-      </c>
-      <c r="K44" s="153" t="s">
-        <v>64</v>
-      </c>
-      <c r="L44" s="135" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="45" spans="2:12" ht="15.6">
-      <c r="B45" s="125" t="s">
-        <v>64</v>
-      </c>
-      <c r="C45" s="131" t="s">
-        <v>64</v>
-      </c>
-      <c r="D45" s="151"/>
-      <c r="E45" s="132"/>
-      <c r="F45" s="132"/>
-      <c r="G45" s="132"/>
-      <c r="H45" s="132"/>
-      <c r="I45" s="133"/>
-      <c r="J45" s="134" t="s">
-        <v>64</v>
-      </c>
-      <c r="K45" s="153" t="s">
-        <v>64</v>
-      </c>
-      <c r="L45" s="135" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="46" spans="2:12" ht="15.6">
-      <c r="B46" s="125" t="s">
-        <v>64</v>
-      </c>
-      <c r="C46" s="131" t="s">
-        <v>64</v>
-      </c>
-      <c r="D46" s="151"/>
-      <c r="E46" s="132"/>
-      <c r="F46" s="132"/>
-      <c r="G46" s="132"/>
-      <c r="H46" s="132"/>
-      <c r="I46" s="133"/>
-      <c r="J46" s="134" t="s">
-        <v>64</v>
-      </c>
-      <c r="K46" s="153" t="s">
-        <v>64</v>
-      </c>
-      <c r="L46" s="135" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="47" spans="2:12" ht="15.6">
-      <c r="B47" s="125" t="s">
-        <v>64</v>
-      </c>
-      <c r="C47" s="131" t="s">
-        <v>64</v>
-      </c>
-      <c r="D47" s="151"/>
-      <c r="E47" s="132"/>
-      <c r="F47" s="132"/>
-      <c r="G47" s="132"/>
-      <c r="H47" s="132"/>
-      <c r="I47" s="133"/>
-      <c r="J47" s="134" t="s">
-        <v>64</v>
-      </c>
-      <c r="K47" s="153" t="s">
-        <v>64</v>
-      </c>
-      <c r="L47" s="135" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="48" spans="2:12" ht="16.2" thickBot="1">
-      <c r="B48" s="125" t="s">
-        <v>64</v>
-      </c>
-      <c r="C48" s="131" t="s">
-        <v>64</v>
-      </c>
-      <c r="D48" s="151"/>
-      <c r="E48" s="132"/>
-      <c r="F48" s="132"/>
-      <c r="G48" s="132"/>
-      <c r="H48" s="132"/>
-      <c r="I48" s="133"/>
-      <c r="J48" s="134" t="s">
-        <v>64</v>
-      </c>
-      <c r="K48" s="153" t="s">
-        <v>64</v>
-      </c>
-      <c r="L48" s="135" t="s">
-        <v>64</v>
-      </c>
     </row>
     <row r="49" spans="2:12" ht="16.2" thickTop="1">
-      <c r="B49" s="241" t="s">
+      <c r="B49" s="214" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="242"/>
-      <c r="D49" s="242"/>
-      <c r="E49" s="242"/>
-      <c r="F49" s="242"/>
-      <c r="G49" s="242"/>
-      <c r="H49" s="242"/>
-      <c r="I49" s="242"/>
-      <c r="J49" s="243"/>
-      <c r="K49" s="217" t="s">
+      <c r="C49" s="215"/>
+      <c r="D49" s="215"/>
+      <c r="E49" s="215"/>
+      <c r="F49" s="215"/>
+      <c r="G49" s="215"/>
+      <c r="H49" s="215"/>
+      <c r="I49" s="215"/>
+      <c r="J49" s="216"/>
+      <c r="K49" s="190" t="s">
         <v>79</v>
       </c>
-      <c r="L49" s="218"/>
+      <c r="L49" s="191"/>
     </row>
     <row r="50" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B50" s="244"/>
-      <c r="C50" s="245"/>
-      <c r="D50" s="245"/>
-      <c r="E50" s="245"/>
-      <c r="F50" s="245"/>
-      <c r="G50" s="245"/>
-      <c r="H50" s="245"/>
-      <c r="I50" s="245"/>
-      <c r="J50" s="246"/>
-      <c r="K50" s="215" t="s">
+      <c r="B50" s="217"/>
+      <c r="C50" s="218"/>
+      <c r="D50" s="218"/>
+      <c r="E50" s="218"/>
+      <c r="F50" s="218"/>
+      <c r="G50" s="218"/>
+      <c r="H50" s="218"/>
+      <c r="I50" s="218"/>
+      <c r="J50" s="219"/>
+      <c r="K50" s="188" t="s">
         <v>103</v>
       </c>
-      <c r="L50" s="216"/>
+      <c r="L50" s="189"/>
     </row>
     <row r="51" spans="2:12" ht="15.6">
-      <c r="B51" s="136"/>
-      <c r="C51" s="212"/>
-      <c r="D51" s="212"/>
-      <c r="E51" s="212"/>
-      <c r="F51" s="212"/>
-      <c r="G51" s="212"/>
-      <c r="H51" s="212"/>
-      <c r="I51" s="212"/>
-      <c r="J51" s="137"/>
-      <c r="K51" s="210"/>
-      <c r="L51" s="211"/>
+      <c r="B51" s="113"/>
+      <c r="C51" s="185"/>
+      <c r="D51" s="185"/>
+      <c r="E51" s="185"/>
+      <c r="F51" s="185"/>
+      <c r="G51" s="185"/>
+      <c r="H51" s="185"/>
+      <c r="I51" s="185"/>
+      <c r="J51" s="114"/>
+      <c r="K51" s="183"/>
+      <c r="L51" s="184"/>
     </row>
     <row r="52" spans="2:12" ht="15.6">
-      <c r="B52" s="138"/>
-      <c r="C52" s="213"/>
-      <c r="D52" s="213"/>
-      <c r="E52" s="213"/>
-      <c r="F52" s="213"/>
-      <c r="G52" s="213"/>
-      <c r="H52" s="213"/>
-      <c r="I52" s="213"/>
-      <c r="J52" s="139"/>
-      <c r="K52" s="154"/>
-      <c r="L52" s="140"/>
+      <c r="B52" s="115"/>
+      <c r="C52" s="186"/>
+      <c r="D52" s="186"/>
+      <c r="E52" s="186"/>
+      <c r="F52" s="186"/>
+      <c r="G52" s="186"/>
+      <c r="H52" s="186"/>
+      <c r="I52" s="186"/>
+      <c r="J52" s="116"/>
+      <c r="K52" s="127"/>
+      <c r="L52" s="117"/>
     </row>
     <row r="53" spans="2:12" ht="15.6">
-      <c r="B53" s="138"/>
-      <c r="C53" s="213"/>
-      <c r="D53" s="213"/>
-      <c r="E53" s="213"/>
-      <c r="F53" s="213"/>
-      <c r="G53" s="213"/>
-      <c r="H53" s="213"/>
-      <c r="I53" s="213"/>
-      <c r="J53" s="139"/>
-      <c r="K53" s="154"/>
-      <c r="L53" s="140"/>
+      <c r="B53" s="115"/>
+      <c r="C53" s="186"/>
+      <c r="D53" s="186"/>
+      <c r="E53" s="186"/>
+      <c r="F53" s="186"/>
+      <c r="G53" s="186"/>
+      <c r="H53" s="186"/>
+      <c r="I53" s="186"/>
+      <c r="J53" s="116"/>
+      <c r="K53" s="127"/>
+      <c r="L53" s="117"/>
     </row>
     <row r="54" spans="2:12" ht="15.6">
-      <c r="B54" s="138"/>
-      <c r="C54" s="213"/>
-      <c r="D54" s="213"/>
-      <c r="E54" s="213"/>
-      <c r="F54" s="213"/>
-      <c r="G54" s="213"/>
-      <c r="H54" s="213"/>
-      <c r="I54" s="213"/>
-      <c r="J54" s="139"/>
-      <c r="K54" s="154"/>
-      <c r="L54" s="140"/>
+      <c r="B54" s="115"/>
+      <c r="C54" s="186"/>
+      <c r="D54" s="186"/>
+      <c r="E54" s="186"/>
+      <c r="F54" s="186"/>
+      <c r="G54" s="186"/>
+      <c r="H54" s="186"/>
+      <c r="I54" s="186"/>
+      <c r="J54" s="116"/>
+      <c r="K54" s="127"/>
+      <c r="L54" s="117"/>
     </row>
     <row r="55" spans="2:12" ht="15.6">
-      <c r="B55" s="141"/>
-      <c r="C55" s="213"/>
-      <c r="D55" s="213"/>
-      <c r="E55" s="213"/>
-      <c r="F55" s="213"/>
-      <c r="G55" s="213"/>
-      <c r="H55" s="213"/>
-      <c r="I55" s="213"/>
-      <c r="J55" s="142"/>
-      <c r="K55" s="143"/>
-      <c r="L55" s="144"/>
+      <c r="B55" s="118"/>
+      <c r="C55" s="186"/>
+      <c r="D55" s="186"/>
+      <c r="E55" s="186"/>
+      <c r="F55" s="186"/>
+      <c r="G55" s="186"/>
+      <c r="H55" s="186"/>
+      <c r="I55" s="186"/>
+      <c r="J55" s="119"/>
+      <c r="K55" s="120"/>
+      <c r="L55" s="121"/>
     </row>
     <row r="56" spans="2:12" ht="15.6">
-      <c r="B56" s="141"/>
-      <c r="C56" s="213"/>
-      <c r="D56" s="213"/>
-      <c r="E56" s="213"/>
-      <c r="F56" s="213"/>
-      <c r="G56" s="213"/>
-      <c r="H56" s="213"/>
-      <c r="I56" s="213"/>
-      <c r="J56" s="142"/>
-      <c r="K56" s="143"/>
-      <c r="L56" s="144"/>
+      <c r="B56" s="118"/>
+      <c r="C56" s="186"/>
+      <c r="D56" s="186"/>
+      <c r="E56" s="186"/>
+      <c r="F56" s="186"/>
+      <c r="G56" s="186"/>
+      <c r="H56" s="186"/>
+      <c r="I56" s="186"/>
+      <c r="J56" s="119"/>
+      <c r="K56" s="120"/>
+      <c r="L56" s="121"/>
     </row>
     <row r="57" spans="2:12" ht="15.6">
-      <c r="B57" s="141"/>
-      <c r="C57" s="213"/>
-      <c r="D57" s="213"/>
-      <c r="E57" s="213"/>
-      <c r="F57" s="213"/>
-      <c r="G57" s="213"/>
-      <c r="H57" s="213"/>
-      <c r="I57" s="213"/>
-      <c r="J57" s="142"/>
-      <c r="K57" s="206"/>
-      <c r="L57" s="207"/>
+      <c r="B57" s="118"/>
+      <c r="C57" s="186"/>
+      <c r="D57" s="186"/>
+      <c r="E57" s="186"/>
+      <c r="F57" s="186"/>
+      <c r="G57" s="186"/>
+      <c r="H57" s="186"/>
+      <c r="I57" s="186"/>
+      <c r="J57" s="119"/>
+      <c r="K57" s="179"/>
+      <c r="L57" s="180"/>
     </row>
     <row r="58" spans="2:12" ht="15.6">
-      <c r="B58" s="141"/>
-      <c r="C58" s="213"/>
-      <c r="D58" s="213"/>
-      <c r="E58" s="213"/>
-      <c r="F58" s="213"/>
-      <c r="G58" s="213"/>
-      <c r="H58" s="213"/>
-      <c r="I58" s="213"/>
-      <c r="J58" s="142"/>
-      <c r="K58" s="208"/>
-      <c r="L58" s="209"/>
+      <c r="B58" s="118"/>
+      <c r="C58" s="186"/>
+      <c r="D58" s="186"/>
+      <c r="E58" s="186"/>
+      <c r="F58" s="186"/>
+      <c r="G58" s="186"/>
+      <c r="H58" s="186"/>
+      <c r="I58" s="186"/>
+      <c r="J58" s="119"/>
+      <c r="K58" s="181"/>
+      <c r="L58" s="182"/>
     </row>
     <row r="59" spans="2:12" ht="15.6">
-      <c r="B59" s="141"/>
-      <c r="C59" s="213"/>
-      <c r="D59" s="213"/>
-      <c r="E59" s="213"/>
-      <c r="F59" s="213"/>
-      <c r="G59" s="213"/>
-      <c r="H59" s="213"/>
-      <c r="I59" s="213"/>
-      <c r="J59" s="142"/>
-      <c r="K59" s="155"/>
+      <c r="B59" s="118"/>
+      <c r="C59" s="186"/>
+      <c r="D59" s="186"/>
+      <c r="E59" s="186"/>
+      <c r="F59" s="186"/>
+      <c r="G59" s="186"/>
+      <c r="H59" s="186"/>
+      <c r="I59" s="186"/>
+      <c r="J59" s="119"/>
+      <c r="K59" s="128"/>
       <c r="L59" s="76"/>
     </row>
     <row r="60" spans="2:12" ht="15.6">
-      <c r="B60" s="141"/>
-      <c r="C60" s="213"/>
-      <c r="D60" s="213"/>
-      <c r="E60" s="213"/>
-      <c r="F60" s="213"/>
-      <c r="G60" s="213"/>
-      <c r="H60" s="213"/>
-      <c r="I60" s="213"/>
-      <c r="J60" s="142"/>
-      <c r="K60" s="155"/>
+      <c r="B60" s="118"/>
+      <c r="C60" s="186"/>
+      <c r="D60" s="186"/>
+      <c r="E60" s="186"/>
+      <c r="F60" s="186"/>
+      <c r="G60" s="186"/>
+      <c r="H60" s="186"/>
+      <c r="I60" s="186"/>
+      <c r="J60" s="119"/>
+      <c r="K60" s="128"/>
       <c r="L60" s="76"/>
     </row>
     <row r="61" spans="2:12" ht="15.6">
-      <c r="B61" s="141"/>
-      <c r="C61" s="214"/>
-      <c r="D61" s="214"/>
-      <c r="E61" s="214"/>
-      <c r="F61" s="214"/>
-      <c r="G61" s="214"/>
-      <c r="H61" s="214"/>
-      <c r="I61" s="214"/>
-      <c r="J61" s="142"/>
-      <c r="K61" s="155"/>
+      <c r="B61" s="118"/>
+      <c r="C61" s="187"/>
+      <c r="D61" s="187"/>
+      <c r="E61" s="187"/>
+      <c r="F61" s="187"/>
+      <c r="G61" s="187"/>
+      <c r="H61" s="187"/>
+      <c r="I61" s="187"/>
+      <c r="J61" s="119"/>
+      <c r="K61" s="128"/>
       <c r="L61" s="76"/>
     </row>
     <row r="62" spans="2:12" ht="15.6">
-      <c r="B62" s="141"/>
-      <c r="C62" s="145"/>
-      <c r="D62" s="145"/>
-      <c r="E62" s="145"/>
-      <c r="F62" s="145"/>
-      <c r="G62" s="145"/>
-      <c r="H62" s="145"/>
-      <c r="I62" s="145"/>
-      <c r="J62" s="142"/>
-      <c r="K62" s="157"/>
-      <c r="L62" s="158"/>
+      <c r="B62" s="118"/>
+      <c r="C62" s="122"/>
+      <c r="D62" s="122"/>
+      <c r="E62" s="122"/>
+      <c r="F62" s="122"/>
+      <c r="G62" s="122"/>
+      <c r="H62" s="122"/>
+      <c r="I62" s="122"/>
+      <c r="J62" s="119"/>
+      <c r="K62" s="130"/>
+      <c r="L62" s="131"/>
     </row>
     <row r="63" spans="2:12" ht="15.6">
-      <c r="B63" s="228" t="s">
+      <c r="B63" s="201" t="s">
         <v>80</v>
       </c>
-      <c r="C63" s="229"/>
-      <c r="D63" s="229"/>
-      <c r="E63" s="230"/>
-      <c r="F63" s="231" t="s">
+      <c r="C63" s="202"/>
+      <c r="D63" s="202"/>
+      <c r="E63" s="203"/>
+      <c r="F63" s="204" t="s">
         <v>81</v>
       </c>
-      <c r="G63" s="230"/>
-      <c r="H63" s="231" t="s">
+      <c r="G63" s="203"/>
+      <c r="H63" s="204" t="s">
         <v>82</v>
       </c>
-      <c r="I63" s="229"/>
-      <c r="J63" s="230"/>
-      <c r="K63" s="143"/>
-      <c r="L63" s="144"/>
+      <c r="I63" s="202"/>
+      <c r="J63" s="203"/>
+      <c r="K63" s="120"/>
+      <c r="L63" s="121"/>
     </row>
     <row r="64" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B64" s="253"/>
-      <c r="C64" s="254"/>
-      <c r="D64" s="254"/>
-      <c r="E64" s="248"/>
-      <c r="F64" s="247"/>
-      <c r="G64" s="248"/>
-      <c r="H64" s="232"/>
-      <c r="I64" s="233"/>
-      <c r="J64" s="234"/>
-      <c r="K64" s="143"/>
-      <c r="L64" s="144"/>
+      <c r="B64" s="226"/>
+      <c r="C64" s="227"/>
+      <c r="D64" s="227"/>
+      <c r="E64" s="221"/>
+      <c r="F64" s="220"/>
+      <c r="G64" s="221"/>
+      <c r="H64" s="205"/>
+      <c r="I64" s="206"/>
+      <c r="J64" s="207"/>
+      <c r="K64" s="120"/>
+      <c r="L64" s="121"/>
     </row>
     <row r="65" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B65" s="255"/>
-      <c r="C65" s="256"/>
-      <c r="D65" s="256"/>
-      <c r="E65" s="250"/>
-      <c r="F65" s="249"/>
-      <c r="G65" s="250"/>
-      <c r="H65" s="235"/>
-      <c r="I65" s="236"/>
-      <c r="J65" s="237"/>
-      <c r="K65" s="156"/>
-      <c r="L65" s="144"/>
+      <c r="B65" s="228"/>
+      <c r="C65" s="229"/>
+      <c r="D65" s="229"/>
+      <c r="E65" s="223"/>
+      <c r="F65" s="222"/>
+      <c r="G65" s="223"/>
+      <c r="H65" s="208"/>
+      <c r="I65" s="209"/>
+      <c r="J65" s="210"/>
+      <c r="K65" s="129"/>
+      <c r="L65" s="121"/>
     </row>
     <row r="66" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B66" s="255"/>
-      <c r="C66" s="256"/>
-      <c r="D66" s="256"/>
-      <c r="E66" s="250"/>
-      <c r="F66" s="249"/>
-      <c r="G66" s="250"/>
-      <c r="H66" s="235"/>
-      <c r="I66" s="236"/>
-      <c r="J66" s="237"/>
-      <c r="K66" s="143"/>
-      <c r="L66" s="144"/>
+      <c r="B66" s="228"/>
+      <c r="C66" s="229"/>
+      <c r="D66" s="229"/>
+      <c r="E66" s="223"/>
+      <c r="F66" s="222"/>
+      <c r="G66" s="223"/>
+      <c r="H66" s="208"/>
+      <c r="I66" s="209"/>
+      <c r="J66" s="210"/>
+      <c r="K66" s="120"/>
+      <c r="L66" s="121"/>
     </row>
     <row r="67" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B67" s="255"/>
-      <c r="C67" s="256"/>
-      <c r="D67" s="256"/>
-      <c r="E67" s="250"/>
-      <c r="F67" s="249"/>
-      <c r="G67" s="250"/>
-      <c r="H67" s="235"/>
-      <c r="I67" s="236"/>
-      <c r="J67" s="237"/>
-      <c r="K67" s="155"/>
+      <c r="B67" s="228"/>
+      <c r="C67" s="229"/>
+      <c r="D67" s="229"/>
+      <c r="E67" s="223"/>
+      <c r="F67" s="222"/>
+      <c r="G67" s="223"/>
+      <c r="H67" s="208"/>
+      <c r="I67" s="209"/>
+      <c r="J67" s="210"/>
+      <c r="K67" s="128"/>
       <c r="L67" s="76"/>
     </row>
     <row r="68" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B68" s="255"/>
-      <c r="C68" s="256"/>
-      <c r="D68" s="256"/>
-      <c r="E68" s="250"/>
-      <c r="F68" s="249"/>
-      <c r="G68" s="250"/>
-      <c r="H68" s="235"/>
-      <c r="I68" s="236"/>
-      <c r="J68" s="237"/>
-      <c r="K68" s="155"/>
+      <c r="B68" s="228"/>
+      <c r="C68" s="229"/>
+      <c r="D68" s="229"/>
+      <c r="E68" s="223"/>
+      <c r="F68" s="222"/>
+      <c r="G68" s="223"/>
+      <c r="H68" s="208"/>
+      <c r="I68" s="209"/>
+      <c r="J68" s="210"/>
+      <c r="K68" s="128"/>
       <c r="L68" s="76"/>
     </row>
     <row r="69" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B69" s="255"/>
-      <c r="C69" s="256"/>
-      <c r="D69" s="256"/>
-      <c r="E69" s="250"/>
-      <c r="F69" s="249"/>
-      <c r="G69" s="250"/>
-      <c r="H69" s="235"/>
-      <c r="I69" s="236"/>
-      <c r="J69" s="237"/>
-      <c r="K69" s="159"/>
-      <c r="L69" s="160"/>
+      <c r="B69" s="228"/>
+      <c r="C69" s="229"/>
+      <c r="D69" s="229"/>
+      <c r="E69" s="223"/>
+      <c r="F69" s="222"/>
+      <c r="G69" s="223"/>
+      <c r="H69" s="208"/>
+      <c r="I69" s="209"/>
+      <c r="J69" s="210"/>
+      <c r="K69" s="132"/>
+      <c r="L69" s="133"/>
     </row>
     <row r="70" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B70" s="255"/>
-      <c r="C70" s="256"/>
-      <c r="D70" s="256"/>
-      <c r="E70" s="250"/>
-      <c r="F70" s="249"/>
-      <c r="G70" s="250"/>
-      <c r="H70" s="235"/>
-      <c r="I70" s="236"/>
-      <c r="J70" s="237"/>
-      <c r="K70" s="159"/>
-      <c r="L70" s="160"/>
+      <c r="B70" s="228"/>
+      <c r="C70" s="229"/>
+      <c r="D70" s="229"/>
+      <c r="E70" s="223"/>
+      <c r="F70" s="222"/>
+      <c r="G70" s="223"/>
+      <c r="H70" s="208"/>
+      <c r="I70" s="209"/>
+      <c r="J70" s="210"/>
+      <c r="K70" s="132"/>
+      <c r="L70" s="133"/>
     </row>
     <row r="71" spans="2:12" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B71" s="257"/>
-      <c r="C71" s="258"/>
-      <c r="D71" s="258"/>
-      <c r="E71" s="252"/>
-      <c r="F71" s="251"/>
-      <c r="G71" s="252"/>
-      <c r="H71" s="238"/>
-      <c r="I71" s="239"/>
-      <c r="J71" s="240"/>
-      <c r="K71" s="146"/>
-      <c r="L71" s="147"/>
+      <c r="B71" s="230"/>
+      <c r="C71" s="231"/>
+      <c r="D71" s="231"/>
+      <c r="E71" s="225"/>
+      <c r="F71" s="224"/>
+      <c r="G71" s="225"/>
+      <c r="H71" s="211"/>
+      <c r="I71" s="212"/>
+      <c r="J71" s="213"/>
+      <c r="K71" s="123"/>
+      <c r="L71" s="124"/>
     </row>
     <row r="72" spans="2:12" ht="15" thickTop="1">
       <c r="J72" s="61"/>
@@ -42182,7 +42203,56 @@
       <c r="L72" s="61"/>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="94">
+    <mergeCell ref="J46:K46"/>
+    <mergeCell ref="J47:K47"/>
+    <mergeCell ref="J48:K48"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="J41:K41"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="J44:K44"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="C44:I44"/>
+    <mergeCell ref="C45:I45"/>
+    <mergeCell ref="C46:I46"/>
+    <mergeCell ref="C47:I47"/>
+    <mergeCell ref="C48:I48"/>
+    <mergeCell ref="C39:I39"/>
+    <mergeCell ref="C40:I40"/>
+    <mergeCell ref="C41:I41"/>
+    <mergeCell ref="C42:I42"/>
+    <mergeCell ref="C43:I43"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="C36:I36"/>
+    <mergeCell ref="C37:I37"/>
+    <mergeCell ref="C38:I38"/>
     <mergeCell ref="B63:E63"/>
     <mergeCell ref="F63:G63"/>
     <mergeCell ref="H63:J63"/>
@@ -42195,6 +42265,17 @@
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="J23:L23"/>
     <mergeCell ref="B24:B25"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
     <mergeCell ref="C24:I25"/>
     <mergeCell ref="J24:L24"/>
     <mergeCell ref="K57:L57"/>
@@ -42203,6 +42284,14 @@
     <mergeCell ref="C51:I61"/>
     <mergeCell ref="K50:L50"/>
     <mergeCell ref="K49:L49"/>
+    <mergeCell ref="C26:I26"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="C28:I28"/>
+    <mergeCell ref="C29:I29"/>
+    <mergeCell ref="C30:I30"/>
+    <mergeCell ref="C31:I31"/>
+    <mergeCell ref="C32:I32"/>
+    <mergeCell ref="C33:I33"/>
     <mergeCell ref="B1:L1"/>
     <mergeCell ref="B2:I3"/>
     <mergeCell ref="J2:L6"/>
@@ -42210,12 +42299,12 @@
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="K10:L10"/>
   </mergeCells>
-  <conditionalFormatting sqref="B26:I48">
+  <conditionalFormatting sqref="B26:C48">
     <cfRule type="expression" dxfId="3" priority="1">
       <formula>ISTEXT($C26)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J27:L48">
+  <conditionalFormatting sqref="J27:J48 L27:L48">
     <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
@@ -42254,40 +42343,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="266"/>
-      <c r="C1" s="266"/>
-      <c r="D1" s="266"/>
-      <c r="E1" s="266"/>
-      <c r="F1" s="266"/>
-      <c r="G1" s="266"/>
-      <c r="H1" s="266"/>
-      <c r="I1" s="266"/>
-      <c r="J1" s="266"/>
-      <c r="K1" s="266"/>
-      <c r="L1" s="266"/>
-      <c r="M1" s="266"/>
-      <c r="N1" s="266"/>
-      <c r="O1" s="266"/>
-      <c r="P1" s="266"/>
+      <c r="B1" s="239"/>
+      <c r="C1" s="239"/>
+      <c r="D1" s="239"/>
+      <c r="E1" s="239"/>
+      <c r="F1" s="239"/>
+      <c r="G1" s="239"/>
+      <c r="H1" s="239"/>
+      <c r="I1" s="239"/>
+      <c r="J1" s="239"/>
+      <c r="K1" s="239"/>
+      <c r="L1" s="239"/>
+      <c r="M1" s="239"/>
+      <c r="N1" s="239"/>
+      <c r="O1" s="239"/>
+      <c r="P1" s="239"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="264" t="s">
+      <c r="B2" s="237" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="265"/>
-      <c r="D2" s="265"/>
-      <c r="E2" s="265"/>
-      <c r="F2" s="265"/>
-      <c r="G2" s="265"/>
-      <c r="H2" s="265"/>
-      <c r="I2" s="265"/>
-      <c r="J2" s="265"/>
-      <c r="K2" s="265"/>
-      <c r="L2" s="265"/>
-      <c r="M2" s="265"/>
-      <c r="N2" s="265"/>
-      <c r="O2" s="265"/>
-      <c r="P2" s="265"/>
+      <c r="C2" s="238"/>
+      <c r="D2" s="238"/>
+      <c r="E2" s="238"/>
+      <c r="F2" s="238"/>
+      <c r="G2" s="238"/>
+      <c r="H2" s="238"/>
+      <c r="I2" s="238"/>
+      <c r="J2" s="238"/>
+      <c r="K2" s="238"/>
+      <c r="L2" s="238"/>
+      <c r="M2" s="238"/>
+      <c r="N2" s="238"/>
+      <c r="O2" s="238"/>
+      <c r="P2" s="238"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -42314,16 +42403,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="272" t="s">
+      <c r="I4" s="245" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="272"/>
-      <c r="K4" s="272"/>
-      <c r="L4" s="272"/>
-      <c r="M4" s="272"/>
-      <c r="N4" s="272"/>
-      <c r="O4" s="272"/>
-      <c r="P4" s="272"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
+      <c r="M4" s="245"/>
+      <c r="N4" s="245"/>
+      <c r="O4" s="245"/>
+      <c r="P4" s="245"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -42337,14 +42426,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="272"/>
-      <c r="J5" s="272"/>
-      <c r="K5" s="272"/>
-      <c r="L5" s="272"/>
-      <c r="M5" s="272"/>
-      <c r="N5" s="272"/>
-      <c r="O5" s="272"/>
-      <c r="P5" s="272"/>
+      <c r="I5" s="245"/>
+      <c r="J5" s="245"/>
+      <c r="K5" s="245"/>
+      <c r="L5" s="245"/>
+      <c r="M5" s="245"/>
+      <c r="N5" s="245"/>
+      <c r="O5" s="245"/>
+      <c r="P5" s="245"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -42479,70 +42568,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="263" t="s">
+      <c r="B12" s="236" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="263" t="s">
+      <c r="C12" s="236" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="263"/>
-      <c r="E12" s="263"/>
-      <c r="F12" s="263" t="s">
+      <c r="D12" s="236"/>
+      <c r="E12" s="236"/>
+      <c r="F12" s="236" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="263" t="s">
+      <c r="G12" s="236" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="263" t="s">
+      <c r="H12" s="236" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="263" t="s">
+      <c r="I12" s="236" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="263" t="s">
+      <c r="J12" s="236" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="263"/>
-      <c r="L12" s="263"/>
-      <c r="M12" s="263"/>
-      <c r="N12" s="263"/>
-      <c r="O12" s="263"/>
-      <c r="P12" s="271" t="s">
+      <c r="K12" s="236"/>
+      <c r="L12" s="236"/>
+      <c r="M12" s="236"/>
+      <c r="N12" s="236"/>
+      <c r="O12" s="236"/>
+      <c r="P12" s="244" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="263"/>
-      <c r="C13" s="263"/>
-      <c r="D13" s="263"/>
-      <c r="E13" s="263"/>
-      <c r="F13" s="263"/>
-      <c r="G13" s="263"/>
-      <c r="H13" s="263"/>
-      <c r="I13" s="263"/>
-      <c r="J13" s="270" t="s">
+      <c r="B13" s="236"/>
+      <c r="C13" s="236"/>
+      <c r="D13" s="236"/>
+      <c r="E13" s="236"/>
+      <c r="F13" s="236"/>
+      <c r="G13" s="236"/>
+      <c r="H13" s="236"/>
+      <c r="I13" s="236"/>
+      <c r="J13" s="243" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="270"/>
-      <c r="L13" s="270" t="s">
+      <c r="K13" s="243"/>
+      <c r="L13" s="243" t="s">
         <v>98</v>
       </c>
-      <c r="M13" s="270"/>
-      <c r="N13" s="270" t="s">
+      <c r="M13" s="243"/>
+      <c r="N13" s="243" t="s">
         <v>99</v>
       </c>
-      <c r="O13" s="270"/>
-      <c r="P13" s="271"/>
+      <c r="O13" s="243"/>
+      <c r="P13" s="244"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="263"/>
-      <c r="C14" s="263"/>
-      <c r="D14" s="263"/>
-      <c r="E14" s="263"/>
-      <c r="F14" s="263"/>
-      <c r="G14" s="263"/>
-      <c r="H14" s="263"/>
-      <c r="I14" s="263"/>
+      <c r="B14" s="236"/>
+      <c r="C14" s="236"/>
+      <c r="D14" s="236"/>
+      <c r="E14" s="236"/>
+      <c r="F14" s="236"/>
+      <c r="G14" s="236"/>
+      <c r="H14" s="236"/>
+      <c r="I14" s="236"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -42561,7 +42650,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="271"/>
+      <c r="P14" s="244"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>

</xml_diff>

<commit_message>
style(excel): remove programmatic formatting in B26:L48 to allow template conditional formatting to prevail
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A7189F-EF8B-48D4-AAD5-529F69A8A1F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16A6567-9187-4859-A925-DC9A4EF0ABB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="136">
   <si>
     <t>HARGA SATUAN BAHAN, ALAT DAN UPAH</t>
   </si>
@@ -444,6 +444,18 @@
   </si>
   <si>
     <t>Unit</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>BAB 1</t>
+  </si>
+  <si>
+    <t>Pekerjaan 1</t>
+  </si>
+  <si>
+    <t>m2</t>
   </si>
 </sst>
 </file>
@@ -2150,7 +2162,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="169" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="308">
+  <cellXfs count="307">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2617,81 +2629,198 @@
     <xf numFmtId="2" fontId="33" fillId="4" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="67" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="60" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="39" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="115" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="112" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="114" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -2800,197 +2929,53 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="39" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="115" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="67" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="60" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3121,29 +3106,52 @@
     <xf numFmtId="0" fontId="32" fillId="4" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="112" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="114" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="116" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="117" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="114" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="116" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="36" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="117" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
   </cellXfs>
@@ -4264,40 +4272,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="265"/>
-      <c r="C1" s="265"/>
-      <c r="D1" s="265"/>
-      <c r="E1" s="265"/>
-      <c r="F1" s="265"/>
-      <c r="G1" s="265"/>
-      <c r="H1" s="265"/>
-      <c r="I1" s="265"/>
-      <c r="J1" s="265"/>
-      <c r="K1" s="265"/>
-      <c r="L1" s="265"/>
-      <c r="M1" s="265"/>
-      <c r="N1" s="265"/>
-      <c r="O1" s="265"/>
-      <c r="P1" s="265"/>
+      <c r="B1" s="258"/>
+      <c r="C1" s="258"/>
+      <c r="D1" s="258"/>
+      <c r="E1" s="258"/>
+      <c r="F1" s="258"/>
+      <c r="G1" s="258"/>
+      <c r="H1" s="258"/>
+      <c r="I1" s="258"/>
+      <c r="J1" s="258"/>
+      <c r="K1" s="258"/>
+      <c r="L1" s="258"/>
+      <c r="M1" s="258"/>
+      <c r="N1" s="258"/>
+      <c r="O1" s="258"/>
+      <c r="P1" s="258"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="263" t="s">
+      <c r="B2" s="256" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="264"/>
-      <c r="D2" s="264"/>
-      <c r="E2" s="264"/>
-      <c r="F2" s="264"/>
-      <c r="G2" s="264"/>
-      <c r="H2" s="264"/>
-      <c r="I2" s="264"/>
-      <c r="J2" s="264"/>
-      <c r="K2" s="264"/>
-      <c r="L2" s="264"/>
-      <c r="M2" s="264"/>
-      <c r="N2" s="264"/>
-      <c r="O2" s="264"/>
-      <c r="P2" s="264"/>
+      <c r="C2" s="257"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="257"/>
+      <c r="H2" s="257"/>
+      <c r="I2" s="257"/>
+      <c r="J2" s="257"/>
+      <c r="K2" s="257"/>
+      <c r="L2" s="257"/>
+      <c r="M2" s="257"/>
+      <c r="N2" s="257"/>
+      <c r="O2" s="257"/>
+      <c r="P2" s="257"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4324,16 +4332,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="271" t="s">
+      <c r="I4" s="264" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="271"/>
-      <c r="K4" s="271"/>
-      <c r="L4" s="271"/>
-      <c r="M4" s="271"/>
-      <c r="N4" s="271"/>
-      <c r="O4" s="271"/>
-      <c r="P4" s="271"/>
+      <c r="J4" s="264"/>
+      <c r="K4" s="264"/>
+      <c r="L4" s="264"/>
+      <c r="M4" s="264"/>
+      <c r="N4" s="264"/>
+      <c r="O4" s="264"/>
+      <c r="P4" s="264"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4347,14 +4355,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="271"/>
-      <c r="J5" s="271"/>
-      <c r="K5" s="271"/>
-      <c r="L5" s="271"/>
-      <c r="M5" s="271"/>
-      <c r="N5" s="271"/>
-      <c r="O5" s="271"/>
-      <c r="P5" s="271"/>
+      <c r="I5" s="264"/>
+      <c r="J5" s="264"/>
+      <c r="K5" s="264"/>
+      <c r="L5" s="264"/>
+      <c r="M5" s="264"/>
+      <c r="N5" s="264"/>
+      <c r="O5" s="264"/>
+      <c r="P5" s="264"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4489,70 +4497,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="262" t="s">
+      <c r="B12" s="255" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="262" t="s">
+      <c r="C12" s="255" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="262"/>
-      <c r="E12" s="262"/>
-      <c r="F12" s="262" t="s">
+      <c r="D12" s="255"/>
+      <c r="E12" s="255"/>
+      <c r="F12" s="255" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="262" t="s">
+      <c r="G12" s="255" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="262" t="s">
+      <c r="H12" s="255" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="262" t="s">
+      <c r="I12" s="255" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="262" t="s">
+      <c r="J12" s="255" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="262"/>
-      <c r="L12" s="262"/>
-      <c r="M12" s="262"/>
-      <c r="N12" s="262"/>
-      <c r="O12" s="262"/>
-      <c r="P12" s="270" t="s">
+      <c r="K12" s="255"/>
+      <c r="L12" s="255"/>
+      <c r="M12" s="255"/>
+      <c r="N12" s="255"/>
+      <c r="O12" s="255"/>
+      <c r="P12" s="263" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="262"/>
-      <c r="C13" s="262"/>
-      <c r="D13" s="262"/>
-      <c r="E13" s="262"/>
-      <c r="F13" s="262"/>
-      <c r="G13" s="262"/>
-      <c r="H13" s="262"/>
-      <c r="I13" s="262"/>
-      <c r="J13" s="269" t="s">
+      <c r="B13" s="255"/>
+      <c r="C13" s="255"/>
+      <c r="D13" s="255"/>
+      <c r="E13" s="255"/>
+      <c r="F13" s="255"/>
+      <c r="G13" s="255"/>
+      <c r="H13" s="255"/>
+      <c r="I13" s="255"/>
+      <c r="J13" s="262" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="269"/>
-      <c r="L13" s="269" t="s">
+      <c r="K13" s="262"/>
+      <c r="L13" s="262" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="269"/>
-      <c r="N13" s="269" t="s">
+      <c r="M13" s="262"/>
+      <c r="N13" s="262" t="s">
         <v>95</v>
       </c>
-      <c r="O13" s="269"/>
-      <c r="P13" s="270"/>
+      <c r="O13" s="262"/>
+      <c r="P13" s="263"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="262"/>
-      <c r="C14" s="262"/>
-      <c r="D14" s="262"/>
-      <c r="E14" s="262"/>
-      <c r="F14" s="262"/>
-      <c r="G14" s="262"/>
-      <c r="H14" s="262"/>
-      <c r="I14" s="262"/>
+      <c r="B14" s="255"/>
+      <c r="C14" s="255"/>
+      <c r="D14" s="255"/>
+      <c r="E14" s="255"/>
+      <c r="F14" s="255"/>
+      <c r="G14" s="255"/>
+      <c r="H14" s="255"/>
+      <c r="I14" s="255"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -4571,7 +4579,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="270"/>
+      <c r="P14" s="263"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -4994,38 +5002,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="103.2" customHeight="1">
-      <c r="B1" s="264"/>
-      <c r="C1" s="264"/>
-      <c r="D1" s="264"/>
-      <c r="E1" s="264"/>
-      <c r="F1" s="264"/>
-      <c r="G1" s="264"/>
-      <c r="H1" s="264"/>
-      <c r="I1" s="264"/>
-      <c r="J1" s="264"/>
-      <c r="K1" s="264"/>
-      <c r="L1" s="264"/>
-      <c r="M1" s="264"/>
-      <c r="N1" s="264"/>
-      <c r="O1" s="264"/>
+      <c r="B1" s="257"/>
+      <c r="C1" s="257"/>
+      <c r="D1" s="257"/>
+      <c r="E1" s="257"/>
+      <c r="F1" s="257"/>
+      <c r="G1" s="257"/>
+      <c r="H1" s="257"/>
+      <c r="I1" s="257"/>
+      <c r="J1" s="257"/>
+      <c r="K1" s="257"/>
+      <c r="L1" s="257"/>
+      <c r="M1" s="257"/>
+      <c r="N1" s="257"/>
+      <c r="O1" s="257"/>
     </row>
     <row r="2" spans="2:15" ht="22.95" customHeight="1">
-      <c r="B2" s="272" t="s">
+      <c r="B2" s="265" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="272"/>
-      <c r="D2" s="272"/>
-      <c r="E2" s="272"/>
-      <c r="F2" s="272"/>
-      <c r="G2" s="272"/>
-      <c r="H2" s="272"/>
-      <c r="I2" s="272"/>
-      <c r="J2" s="272"/>
-      <c r="K2" s="272"/>
-      <c r="L2" s="272"/>
-      <c r="M2" s="272"/>
-      <c r="N2" s="272"/>
-      <c r="O2" s="272"/>
+      <c r="C2" s="265"/>
+      <c r="D2" s="265"/>
+      <c r="E2" s="265"/>
+      <c r="F2" s="265"/>
+      <c r="G2" s="265"/>
+      <c r="H2" s="265"/>
+      <c r="I2" s="265"/>
+      <c r="J2" s="265"/>
+      <c r="K2" s="265"/>
+      <c r="L2" s="265"/>
+      <c r="M2" s="265"/>
+      <c r="N2" s="265"/>
+      <c r="O2" s="265"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" t="s">
@@ -5077,179 +5085,179 @@
     </row>
     <row r="9" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="11" spans="2:15" s="58" customFormat="1">
-      <c r="B11" s="273" t="s">
+      <c r="B11" s="266" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="273"/>
-      <c r="D11" s="273"/>
-      <c r="E11" s="273"/>
-      <c r="G11" s="273" t="s">
+      <c r="C11" s="266"/>
+      <c r="D11" s="266"/>
+      <c r="E11" s="266"/>
+      <c r="G11" s="266" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="273"/>
-      <c r="I11" s="273"/>
-      <c r="J11" s="273"/>
-      <c r="L11" s="273" t="s">
+      <c r="H11" s="266"/>
+      <c r="I11" s="266"/>
+      <c r="J11" s="266"/>
+      <c r="L11" s="266" t="s">
         <v>105</v>
       </c>
-      <c r="M11" s="273"/>
-      <c r="N11" s="273"/>
-      <c r="O11" s="273"/>
+      <c r="M11" s="266"/>
+      <c r="N11" s="266"/>
+      <c r="O11" s="266"/>
     </row>
     <row r="12" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="13" spans="2:15">
-      <c r="B13" s="264"/>
-      <c r="C13" s="264"/>
-      <c r="D13" s="264"/>
-      <c r="E13" s="264"/>
-      <c r="G13" s="264"/>
-      <c r="H13" s="264"/>
-      <c r="I13" s="264"/>
-      <c r="J13" s="264"/>
-      <c r="L13" s="264"/>
-      <c r="M13" s="264"/>
-      <c r="N13" s="264"/>
-      <c r="O13" s="264"/>
+      <c r="B13" s="257"/>
+      <c r="C13" s="257"/>
+      <c r="D13" s="257"/>
+      <c r="E13" s="257"/>
+      <c r="G13" s="257"/>
+      <c r="H13" s="257"/>
+      <c r="I13" s="257"/>
+      <c r="J13" s="257"/>
+      <c r="L13" s="257"/>
+      <c r="M13" s="257"/>
+      <c r="N13" s="257"/>
+      <c r="O13" s="257"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="264"/>
-      <c r="C14" s="264"/>
-      <c r="D14" s="264"/>
-      <c r="E14" s="264"/>
-      <c r="G14" s="264"/>
-      <c r="H14" s="264"/>
-      <c r="I14" s="264"/>
-      <c r="J14" s="264"/>
-      <c r="L14" s="264"/>
-      <c r="M14" s="264"/>
-      <c r="N14" s="264"/>
-      <c r="O14" s="264"/>
+      <c r="B14" s="257"/>
+      <c r="C14" s="257"/>
+      <c r="D14" s="257"/>
+      <c r="E14" s="257"/>
+      <c r="G14" s="257"/>
+      <c r="H14" s="257"/>
+      <c r="I14" s="257"/>
+      <c r="J14" s="257"/>
+      <c r="L14" s="257"/>
+      <c r="M14" s="257"/>
+      <c r="N14" s="257"/>
+      <c r="O14" s="257"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="264"/>
-      <c r="C15" s="264"/>
-      <c r="D15" s="264"/>
-      <c r="E15" s="264"/>
-      <c r="G15" s="264"/>
-      <c r="H15" s="264"/>
-      <c r="I15" s="264"/>
-      <c r="J15" s="264"/>
-      <c r="L15" s="264"/>
-      <c r="M15" s="264"/>
-      <c r="N15" s="264"/>
-      <c r="O15" s="264"/>
+      <c r="B15" s="257"/>
+      <c r="C15" s="257"/>
+      <c r="D15" s="257"/>
+      <c r="E15" s="257"/>
+      <c r="G15" s="257"/>
+      <c r="H15" s="257"/>
+      <c r="I15" s="257"/>
+      <c r="J15" s="257"/>
+      <c r="L15" s="257"/>
+      <c r="M15" s="257"/>
+      <c r="N15" s="257"/>
+      <c r="O15" s="257"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="264"/>
-      <c r="C16" s="264"/>
-      <c r="D16" s="264"/>
-      <c r="E16" s="264"/>
-      <c r="G16" s="264"/>
-      <c r="H16" s="264"/>
-      <c r="I16" s="264"/>
-      <c r="J16" s="264"/>
-      <c r="L16" s="264"/>
-      <c r="M16" s="264"/>
-      <c r="N16" s="264"/>
-      <c r="O16" s="264"/>
+      <c r="B16" s="257"/>
+      <c r="C16" s="257"/>
+      <c r="D16" s="257"/>
+      <c r="E16" s="257"/>
+      <c r="G16" s="257"/>
+      <c r="H16" s="257"/>
+      <c r="I16" s="257"/>
+      <c r="J16" s="257"/>
+      <c r="L16" s="257"/>
+      <c r="M16" s="257"/>
+      <c r="N16" s="257"/>
+      <c r="O16" s="257"/>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="264"/>
-      <c r="C17" s="264"/>
-      <c r="D17" s="264"/>
-      <c r="E17" s="264"/>
-      <c r="G17" s="264"/>
-      <c r="H17" s="264"/>
-      <c r="I17" s="264"/>
-      <c r="J17" s="264"/>
-      <c r="L17" s="264"/>
-      <c r="M17" s="264"/>
-      <c r="N17" s="264"/>
-      <c r="O17" s="264"/>
+      <c r="B17" s="257"/>
+      <c r="C17" s="257"/>
+      <c r="D17" s="257"/>
+      <c r="E17" s="257"/>
+      <c r="G17" s="257"/>
+      <c r="H17" s="257"/>
+      <c r="I17" s="257"/>
+      <c r="J17" s="257"/>
+      <c r="L17" s="257"/>
+      <c r="M17" s="257"/>
+      <c r="N17" s="257"/>
+      <c r="O17" s="257"/>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="264"/>
-      <c r="C18" s="264"/>
-      <c r="D18" s="264"/>
-      <c r="E18" s="264"/>
-      <c r="G18" s="264"/>
-      <c r="H18" s="264"/>
-      <c r="I18" s="264"/>
-      <c r="J18" s="264"/>
-      <c r="L18" s="264"/>
-      <c r="M18" s="264"/>
-      <c r="N18" s="264"/>
-      <c r="O18" s="264"/>
+      <c r="B18" s="257"/>
+      <c r="C18" s="257"/>
+      <c r="D18" s="257"/>
+      <c r="E18" s="257"/>
+      <c r="G18" s="257"/>
+      <c r="H18" s="257"/>
+      <c r="I18" s="257"/>
+      <c r="J18" s="257"/>
+      <c r="L18" s="257"/>
+      <c r="M18" s="257"/>
+      <c r="N18" s="257"/>
+      <c r="O18" s="257"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="B19" s="264"/>
-      <c r="C19" s="264"/>
-      <c r="D19" s="264"/>
-      <c r="E19" s="264"/>
-      <c r="G19" s="264"/>
-      <c r="H19" s="264"/>
-      <c r="I19" s="264"/>
-      <c r="J19" s="264"/>
-      <c r="L19" s="264"/>
-      <c r="M19" s="264"/>
-      <c r="N19" s="264"/>
-      <c r="O19" s="264"/>
+      <c r="B19" s="257"/>
+      <c r="C19" s="257"/>
+      <c r="D19" s="257"/>
+      <c r="E19" s="257"/>
+      <c r="G19" s="257"/>
+      <c r="H19" s="257"/>
+      <c r="I19" s="257"/>
+      <c r="J19" s="257"/>
+      <c r="L19" s="257"/>
+      <c r="M19" s="257"/>
+      <c r="N19" s="257"/>
+      <c r="O19" s="257"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="B20" s="264"/>
-      <c r="C20" s="264"/>
-      <c r="D20" s="264"/>
-      <c r="E20" s="264"/>
-      <c r="G20" s="264"/>
-      <c r="H20" s="264"/>
-      <c r="I20" s="264"/>
-      <c r="J20" s="264"/>
-      <c r="L20" s="264"/>
-      <c r="M20" s="264"/>
-      <c r="N20" s="264"/>
-      <c r="O20" s="264"/>
+      <c r="B20" s="257"/>
+      <c r="C20" s="257"/>
+      <c r="D20" s="257"/>
+      <c r="E20" s="257"/>
+      <c r="G20" s="257"/>
+      <c r="H20" s="257"/>
+      <c r="I20" s="257"/>
+      <c r="J20" s="257"/>
+      <c r="L20" s="257"/>
+      <c r="M20" s="257"/>
+      <c r="N20" s="257"/>
+      <c r="O20" s="257"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="B21" s="264"/>
-      <c r="C21" s="264"/>
-      <c r="D21" s="264"/>
-      <c r="E21" s="264"/>
-      <c r="G21" s="264"/>
-      <c r="H21" s="264"/>
-      <c r="I21" s="264"/>
-      <c r="J21" s="264"/>
-      <c r="L21" s="264"/>
-      <c r="M21" s="264"/>
-      <c r="N21" s="264"/>
-      <c r="O21" s="264"/>
+      <c r="B21" s="257"/>
+      <c r="C21" s="257"/>
+      <c r="D21" s="257"/>
+      <c r="E21" s="257"/>
+      <c r="G21" s="257"/>
+      <c r="H21" s="257"/>
+      <c r="I21" s="257"/>
+      <c r="J21" s="257"/>
+      <c r="L21" s="257"/>
+      <c r="M21" s="257"/>
+      <c r="N21" s="257"/>
+      <c r="O21" s="257"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="B22" s="264"/>
-      <c r="C22" s="264"/>
-      <c r="D22" s="264"/>
-      <c r="E22" s="264"/>
-      <c r="G22" s="264"/>
-      <c r="H22" s="264"/>
-      <c r="I22" s="264"/>
-      <c r="J22" s="264"/>
-      <c r="L22" s="264"/>
-      <c r="M22" s="264"/>
-      <c r="N22" s="264"/>
-      <c r="O22" s="264"/>
+      <c r="B22" s="257"/>
+      <c r="C22" s="257"/>
+      <c r="D22" s="257"/>
+      <c r="E22" s="257"/>
+      <c r="G22" s="257"/>
+      <c r="H22" s="257"/>
+      <c r="I22" s="257"/>
+      <c r="J22" s="257"/>
+      <c r="L22" s="257"/>
+      <c r="M22" s="257"/>
+      <c r="N22" s="257"/>
+      <c r="O22" s="257"/>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="264"/>
-      <c r="C23" s="264"/>
-      <c r="D23" s="264"/>
-      <c r="E23" s="264"/>
-      <c r="G23" s="264"/>
-      <c r="H23" s="264"/>
-      <c r="I23" s="264"/>
-      <c r="J23" s="264"/>
-      <c r="L23" s="264"/>
-      <c r="M23" s="264"/>
-      <c r="N23" s="264"/>
-      <c r="O23" s="264"/>
+      <c r="B23" s="257"/>
+      <c r="C23" s="257"/>
+      <c r="D23" s="257"/>
+      <c r="E23" s="257"/>
+      <c r="G23" s="257"/>
+      <c r="H23" s="257"/>
+      <c r="I23" s="257"/>
+      <c r="J23" s="257"/>
+      <c r="L23" s="257"/>
+      <c r="M23" s="257"/>
+      <c r="N23" s="257"/>
+      <c r="O23" s="257"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5283,35 +5291,35 @@
   <sheetData>
     <row r="1" spans="2:29" ht="4.8" customHeight="1" thickBot="1"/>
     <row r="2" spans="2:29" ht="19.95" customHeight="1" thickBot="1">
-      <c r="B2" s="274" t="s">
+      <c r="B2" s="267" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="275"/>
-      <c r="D2" s="275"/>
-      <c r="E2" s="275"/>
-      <c r="F2" s="275"/>
-      <c r="G2" s="275"/>
-      <c r="H2" s="275"/>
-      <c r="I2" s="275"/>
-      <c r="J2" s="275"/>
-      <c r="K2" s="275"/>
-      <c r="L2" s="275"/>
-      <c r="M2" s="275"/>
-      <c r="N2" s="275"/>
-      <c r="O2" s="275"/>
-      <c r="P2" s="275"/>
-      <c r="Q2" s="275"/>
-      <c r="R2" s="275"/>
-      <c r="S2" s="275"/>
-      <c r="T2" s="275"/>
-      <c r="U2" s="275"/>
-      <c r="V2" s="275"/>
-      <c r="W2" s="275"/>
-      <c r="X2" s="275"/>
-      <c r="Y2" s="275"/>
-      <c r="Z2" s="275"/>
-      <c r="AA2" s="275"/>
-      <c r="AB2" s="276"/>
+      <c r="C2" s="268"/>
+      <c r="D2" s="268"/>
+      <c r="E2" s="268"/>
+      <c r="F2" s="268"/>
+      <c r="G2" s="268"/>
+      <c r="H2" s="268"/>
+      <c r="I2" s="268"/>
+      <c r="J2" s="268"/>
+      <c r="K2" s="268"/>
+      <c r="L2" s="268"/>
+      <c r="M2" s="268"/>
+      <c r="N2" s="268"/>
+      <c r="O2" s="268"/>
+      <c r="P2" s="268"/>
+      <c r="Q2" s="268"/>
+      <c r="R2" s="268"/>
+      <c r="S2" s="268"/>
+      <c r="T2" s="268"/>
+      <c r="U2" s="268"/>
+      <c r="V2" s="268"/>
+      <c r="W2" s="268"/>
+      <c r="X2" s="268"/>
+      <c r="Y2" s="268"/>
+      <c r="Z2" s="268"/>
+      <c r="AA2" s="268"/>
+      <c r="AB2" s="269"/>
       <c r="AC2" s="141"/>
     </row>
     <row r="3" spans="2:29" ht="15" customHeight="1">
@@ -5411,74 +5419,74 @@
       <c r="AB11" s="139"/>
     </row>
     <row r="12" spans="2:29" ht="15" customHeight="1">
-      <c r="B12" s="286" t="s">
+      <c r="B12" s="279" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="288" t="s">
+      <c r="C12" s="281" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="289"/>
-      <c r="E12" s="289"/>
-      <c r="F12" s="289"/>
-      <c r="G12" s="289"/>
-      <c r="H12" s="289"/>
-      <c r="I12" s="289"/>
-      <c r="J12" s="289"/>
-      <c r="K12" s="289"/>
-      <c r="L12" s="290"/>
-      <c r="M12" s="294" t="s">
+      <c r="D12" s="282"/>
+      <c r="E12" s="282"/>
+      <c r="F12" s="282"/>
+      <c r="G12" s="282"/>
+      <c r="H12" s="282"/>
+      <c r="I12" s="282"/>
+      <c r="J12" s="282"/>
+      <c r="K12" s="282"/>
+      <c r="L12" s="283"/>
+      <c r="M12" s="287" t="s">
         <v>113</v>
       </c>
-      <c r="N12" s="294" t="s">
+      <c r="N12" s="287" t="s">
         <v>34</v>
       </c>
-      <c r="O12" s="299" t="s">
+      <c r="O12" s="292" t="s">
         <v>114</v>
       </c>
-      <c r="P12" s="299"/>
-      <c r="Q12" s="299"/>
-      <c r="R12" s="299"/>
-      <c r="S12" s="299"/>
-      <c r="T12" s="299"/>
-      <c r="U12" s="299"/>
-      <c r="V12" s="299"/>
-      <c r="W12" s="299"/>
-      <c r="X12" s="299"/>
-      <c r="Y12" s="299"/>
-      <c r="Z12" s="299"/>
-      <c r="AA12" s="299"/>
-      <c r="AB12" s="300"/>
+      <c r="P12" s="292"/>
+      <c r="Q12" s="292"/>
+      <c r="R12" s="292"/>
+      <c r="S12" s="292"/>
+      <c r="T12" s="292"/>
+      <c r="U12" s="292"/>
+      <c r="V12" s="292"/>
+      <c r="W12" s="292"/>
+      <c r="X12" s="292"/>
+      <c r="Y12" s="292"/>
+      <c r="Z12" s="292"/>
+      <c r="AA12" s="292"/>
+      <c r="AB12" s="293"/>
     </row>
     <row r="13" spans="2:29" ht="15" customHeight="1">
-      <c r="B13" s="287"/>
-      <c r="C13" s="291"/>
-      <c r="D13" s="292"/>
-      <c r="E13" s="292"/>
-      <c r="F13" s="292"/>
-      <c r="G13" s="292"/>
-      <c r="H13" s="292"/>
-      <c r="I13" s="292"/>
-      <c r="J13" s="292"/>
-      <c r="K13" s="292"/>
-      <c r="L13" s="293"/>
-      <c r="M13" s="295"/>
-      <c r="N13" s="295"/>
-      <c r="O13" s="296" t="s">
+      <c r="B13" s="280"/>
+      <c r="C13" s="284"/>
+      <c r="D13" s="285"/>
+      <c r="E13" s="285"/>
+      <c r="F13" s="285"/>
+      <c r="G13" s="285"/>
+      <c r="H13" s="285"/>
+      <c r="I13" s="285"/>
+      <c r="J13" s="285"/>
+      <c r="K13" s="285"/>
+      <c r="L13" s="286"/>
+      <c r="M13" s="288"/>
+      <c r="N13" s="288"/>
+      <c r="O13" s="289" t="s">
         <v>115</v>
       </c>
-      <c r="P13" s="297"/>
-      <c r="Q13" s="298"/>
-      <c r="R13" s="296" t="s">
+      <c r="P13" s="290"/>
+      <c r="Q13" s="291"/>
+      <c r="R13" s="289" t="s">
         <v>116</v>
       </c>
-      <c r="S13" s="297"/>
-      <c r="T13" s="298"/>
-      <c r="U13" s="296" t="s">
+      <c r="S13" s="290"/>
+      <c r="T13" s="291"/>
+      <c r="U13" s="289" t="s">
         <v>117</v>
       </c>
-      <c r="V13" s="297"/>
-      <c r="W13" s="298"/>
-      <c r="X13" s="277" t="s">
+      <c r="V13" s="290"/>
+      <c r="W13" s="291"/>
+      <c r="X13" s="270" t="s">
         <v>118</v>
       </c>
       <c r="Y13" s="146" t="s">
@@ -5487,27 +5495,27 @@
       <c r="Z13" s="147" t="s">
         <v>119</v>
       </c>
-      <c r="AA13" s="279" t="s">
+      <c r="AA13" s="272" t="s">
         <v>120</v>
       </c>
-      <c r="AB13" s="281" t="s">
+      <c r="AB13" s="274" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="14" spans="2:29" ht="15" customHeight="1">
-      <c r="B14" s="287"/>
-      <c r="C14" s="291"/>
-      <c r="D14" s="292"/>
-      <c r="E14" s="292"/>
-      <c r="F14" s="292"/>
-      <c r="G14" s="292"/>
-      <c r="H14" s="292"/>
-      <c r="I14" s="292"/>
-      <c r="J14" s="292"/>
-      <c r="K14" s="292"/>
-      <c r="L14" s="293"/>
-      <c r="M14" s="278"/>
-      <c r="N14" s="278"/>
+      <c r="B14" s="280"/>
+      <c r="C14" s="284"/>
+      <c r="D14" s="285"/>
+      <c r="E14" s="285"/>
+      <c r="F14" s="285"/>
+      <c r="G14" s="285"/>
+      <c r="H14" s="285"/>
+      <c r="I14" s="285"/>
+      <c r="J14" s="285"/>
+      <c r="K14" s="285"/>
+      <c r="L14" s="286"/>
+      <c r="M14" s="271"/>
+      <c r="N14" s="271"/>
       <c r="O14" s="148" t="s">
         <v>122</v>
       </c>
@@ -5535,32 +5543,32 @@
       <c r="W14" s="148" t="s">
         <v>129</v>
       </c>
-      <c r="X14" s="278"/>
+      <c r="X14" s="271"/>
       <c r="Y14" s="146" t="s">
         <v>130</v>
       </c>
       <c r="Z14" s="148" t="s">
         <v>131</v>
       </c>
-      <c r="AA14" s="280"/>
-      <c r="AB14" s="282"/>
+      <c r="AA14" s="273"/>
+      <c r="AB14" s="275"/>
     </row>
     <row r="15" spans="2:29" ht="15" customHeight="1" thickBot="1">
       <c r="B15" s="142">
         <v>1</v>
       </c>
-      <c r="C15" s="283">
+      <c r="C15" s="276">
         <v>2</v>
       </c>
-      <c r="D15" s="284"/>
-      <c r="E15" s="284"/>
-      <c r="F15" s="284"/>
-      <c r="G15" s="284"/>
-      <c r="H15" s="284"/>
-      <c r="I15" s="284"/>
-      <c r="J15" s="284"/>
-      <c r="K15" s="284"/>
-      <c r="L15" s="285"/>
+      <c r="D15" s="277"/>
+      <c r="E15" s="277"/>
+      <c r="F15" s="277"/>
+      <c r="G15" s="277"/>
+      <c r="H15" s="277"/>
+      <c r="I15" s="277"/>
+      <c r="J15" s="277"/>
+      <c r="K15" s="277"/>
+      <c r="L15" s="278"/>
       <c r="M15" s="143">
         <v>3</v>
       </c>
@@ -5650,38 +5658,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="261"/>
-      <c r="C1" s="261"/>
-      <c r="D1" s="261"/>
-      <c r="E1" s="261"/>
-      <c r="F1" s="261"/>
-      <c r="G1" s="261"/>
-      <c r="H1" s="261"/>
-      <c r="I1" s="261"/>
+      <c r="B1" s="254"/>
+      <c r="C1" s="254"/>
+      <c r="D1" s="254"/>
+      <c r="E1" s="254"/>
+      <c r="F1" s="254"/>
+      <c r="G1" s="254"/>
+      <c r="H1" s="254"/>
+      <c r="I1" s="254"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="258" t="s">
+      <c r="B2" s="251" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="258"/>
-      <c r="D2" s="258"/>
-      <c r="E2" s="258"/>
-      <c r="F2" s="258"/>
-      <c r="G2" s="258"/>
-      <c r="H2" s="258"/>
-      <c r="I2" s="258"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="251"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="251"/>
+      <c r="I2" s="251"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="259" t="s">
+      <c r="B3" s="252" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="259"/>
-      <c r="D3" s="259"/>
-      <c r="E3" s="259"/>
-      <c r="F3" s="259"/>
-      <c r="G3" s="259"/>
-      <c r="H3" s="259"/>
-      <c r="I3" s="259"/>
+      <c r="C3" s="252"/>
+      <c r="D3" s="252"/>
+      <c r="E3" s="252"/>
+      <c r="F3" s="252"/>
+      <c r="G3" s="252"/>
+      <c r="H3" s="252"/>
+      <c r="I3" s="252"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -5689,10 +5697,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="260" t="s">
+      <c r="C5" s="253" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="260"/>
+      <c r="D5" s="253"/>
       <c r="E5" s="11" t="s">
         <v>38</v>
       </c>
@@ -14079,63 +14087,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="261"/>
-      <c r="C1" s="261"/>
-      <c r="D1" s="261"/>
-      <c r="E1" s="261"/>
-      <c r="F1" s="261"/>
-      <c r="G1" s="261"/>
-      <c r="H1" s="261"/>
-      <c r="I1" s="261"/>
-      <c r="J1" s="261"/>
-      <c r="K1" s="261"/>
-      <c r="L1" s="261"/>
-      <c r="M1" s="261"/>
-      <c r="N1" s="261"/>
+      <c r="B1" s="254"/>
+      <c r="C1" s="254"/>
+      <c r="D1" s="254"/>
+      <c r="E1" s="254"/>
+      <c r="F1" s="254"/>
+      <c r="G1" s="254"/>
+      <c r="H1" s="254"/>
+      <c r="I1" s="254"/>
+      <c r="J1" s="254"/>
+      <c r="K1" s="254"/>
+      <c r="L1" s="254"/>
+      <c r="M1" s="254"/>
+      <c r="N1" s="254"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="258" t="s">
+      <c r="B2" s="251" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="258"/>
-      <c r="D2" s="258"/>
-      <c r="E2" s="258"/>
-      <c r="F2" s="258"/>
-      <c r="G2" s="258"/>
-      <c r="H2" s="258"/>
-      <c r="I2" s="258"/>
-      <c r="J2" s="258"/>
-      <c r="K2" s="258"/>
-      <c r="L2" s="258"/>
-      <c r="M2" s="258"/>
-      <c r="N2" s="258"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="251"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="251"/>
+      <c r="I2" s="251"/>
+      <c r="J2" s="251"/>
+      <c r="K2" s="251"/>
+      <c r="L2" s="251"/>
+      <c r="M2" s="251"/>
+      <c r="N2" s="251"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="259" t="s">
+      <c r="B3" s="252" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="259"/>
-      <c r="D3" s="259"/>
-      <c r="E3" s="259"/>
-      <c r="F3" s="259"/>
-      <c r="G3" s="259"/>
-      <c r="H3" s="259"/>
-      <c r="I3" s="259"/>
-      <c r="J3" s="259"/>
-      <c r="K3" s="259"/>
-      <c r="L3" s="259"/>
-      <c r="M3" s="259"/>
-      <c r="N3" s="259"/>
+      <c r="C3" s="252"/>
+      <c r="D3" s="252"/>
+      <c r="E3" s="252"/>
+      <c r="F3" s="252"/>
+      <c r="G3" s="252"/>
+      <c r="H3" s="252"/>
+      <c r="I3" s="252"/>
+      <c r="J3" s="252"/>
+      <c r="K3" s="252"/>
+      <c r="L3" s="252"/>
+      <c r="M3" s="252"/>
+      <c r="N3" s="252"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="262" t="s">
+      <c r="C5" s="255" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="262"/>
+      <c r="D5" s="255"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -16339,35 +16347,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="261"/>
-      <c r="C1" s="261"/>
-      <c r="D1" s="261"/>
-      <c r="E1" s="261"/>
-      <c r="F1" s="261"/>
-      <c r="G1" s="261"/>
-      <c r="H1" s="261"/>
+      <c r="B1" s="254"/>
+      <c r="C1" s="254"/>
+      <c r="D1" s="254"/>
+      <c r="E1" s="254"/>
+      <c r="F1" s="254"/>
+      <c r="G1" s="254"/>
+      <c r="H1" s="254"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="258" t="s">
+      <c r="B2" s="251" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="258"/>
-      <c r="D2" s="258"/>
-      <c r="E2" s="258"/>
-      <c r="F2" s="258"/>
-      <c r="G2" s="258"/>
-      <c r="H2" s="258"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="251"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="251"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="259" t="s">
+      <c r="B3" s="252" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="259"/>
-      <c r="D3" s="259"/>
-      <c r="E3" s="259"/>
-      <c r="F3" s="259"/>
-      <c r="G3" s="259"/>
-      <c r="H3" s="259"/>
+      <c r="C3" s="252"/>
+      <c r="D3" s="252"/>
+      <c r="E3" s="252"/>
+      <c r="F3" s="252"/>
+      <c r="G3" s="252"/>
+      <c r="H3" s="252"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -40461,30 +40469,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="265"/>
-      <c r="C1" s="265"/>
-      <c r="D1" s="265"/>
-      <c r="E1" s="265"/>
-      <c r="F1" s="265"/>
-      <c r="G1" s="265"/>
-      <c r="H1" s="265"/>
-      <c r="I1" s="265"/>
-      <c r="J1" s="265"/>
-      <c r="K1" s="265"/>
+      <c r="B1" s="258"/>
+      <c r="C1" s="258"/>
+      <c r="D1" s="258"/>
+      <c r="E1" s="258"/>
+      <c r="F1" s="258"/>
+      <c r="G1" s="258"/>
+      <c r="H1" s="258"/>
+      <c r="I1" s="258"/>
+      <c r="J1" s="258"/>
+      <c r="K1" s="258"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="263" t="s">
+      <c r="B2" s="256" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="264"/>
-      <c r="D2" s="264"/>
-      <c r="E2" s="264"/>
-      <c r="F2" s="264"/>
-      <c r="G2" s="264"/>
-      <c r="H2" s="264"/>
-      <c r="I2" s="264"/>
-      <c r="J2" s="264"/>
-      <c r="K2" s="264"/>
+      <c r="C2" s="257"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="257"/>
+      <c r="H2" s="257"/>
+      <c r="I2" s="257"/>
+      <c r="J2" s="257"/>
+      <c r="K2" s="257"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40604,11 +40612,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="262" t="s">
+      <c r="C11" s="255" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="262"/>
-      <c r="E11" s="262"/>
+      <c r="D11" s="255"/>
+      <c r="E11" s="255"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -40664,26 +40672,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="111.6" customHeight="1">
-      <c r="B1" s="265"/>
-      <c r="C1" s="265"/>
-      <c r="D1" s="265"/>
-      <c r="E1" s="265"/>
-      <c r="F1" s="265"/>
-      <c r="G1" s="265"/>
-      <c r="H1" s="265"/>
-      <c r="I1" s="265"/>
+      <c r="B1" s="258"/>
+      <c r="C1" s="258"/>
+      <c r="D1" s="258"/>
+      <c r="E1" s="258"/>
+      <c r="F1" s="258"/>
+      <c r="G1" s="258"/>
+      <c r="H1" s="258"/>
+      <c r="I1" s="258"/>
     </row>
     <row r="2" spans="2:9" ht="22.95" customHeight="1">
-      <c r="B2" s="263" t="s">
+      <c r="B2" s="256" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="264"/>
-      <c r="D2" s="264"/>
-      <c r="E2" s="264"/>
-      <c r="F2" s="264"/>
-      <c r="G2" s="264"/>
-      <c r="H2" s="264"/>
-      <c r="I2" s="264"/>
+      <c r="C2" s="257"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="257"/>
+      <c r="H2" s="257"/>
+      <c r="I2" s="257"/>
     </row>
     <row r="3" spans="2:9" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40793,12 +40801,12 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="262" t="s">
+      <c r="C11" s="255" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="262"/>
-      <c r="E11" s="262"/>
-      <c r="F11" s="262"/>
+      <c r="D11" s="255"/>
+      <c r="E11" s="255"/>
+      <c r="F11" s="255"/>
       <c r="G11" s="40" t="s">
         <v>29</v>
       </c>
@@ -40836,58 +40844,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="265"/>
-      <c r="C1" s="265"/>
-      <c r="D1" s="265"/>
-      <c r="E1" s="265"/>
-      <c r="F1" s="265"/>
+      <c r="B1" s="258"/>
+      <c r="C1" s="258"/>
+      <c r="D1" s="258"/>
+      <c r="E1" s="258"/>
+      <c r="F1" s="258"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="268" t="s">
+      <c r="B2" s="261" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="268"/>
-      <c r="D2" s="268"/>
-      <c r="E2" s="268"/>
-      <c r="F2" s="268"/>
+      <c r="C2" s="261"/>
+      <c r="D2" s="261"/>
+      <c r="E2" s="261"/>
+      <c r="F2" s="261"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="265"/>
-      <c r="C3" s="265"/>
-      <c r="D3" s="265"/>
-      <c r="E3" s="265"/>
-      <c r="F3" s="265"/>
+      <c r="B3" s="258"/>
+      <c r="C3" s="258"/>
+      <c r="D3" s="258"/>
+      <c r="E3" s="258"/>
+      <c r="F3" s="258"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="266" t="s">
+      <c r="B5" s="259" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="266" t="s">
+      <c r="C5" s="259" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="266" t="s">
+      <c r="D5" s="259" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="267" t="s">
+      <c r="E5" s="260" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="267" t="s">
+      <c r="F5" s="260" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="266"/>
-      <c r="C6" s="266"/>
-      <c r="D6" s="266"/>
-      <c r="E6" s="267"/>
-      <c r="F6" s="267"/>
+      <c r="B6" s="259"/>
+      <c r="C6" s="259"/>
+      <c r="D6" s="259"/>
+      <c r="E6" s="260"/>
+      <c r="F6" s="260"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="266"/>
-      <c r="C7" s="266"/>
-      <c r="D7" s="266"/>
-      <c r="E7" s="267"/>
-      <c r="F7" s="267"/>
+      <c r="B7" s="259"/>
+      <c r="C7" s="259"/>
+      <c r="D7" s="259"/>
+      <c r="E7" s="260"/>
+      <c r="F7" s="260"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -41008,45 +41016,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="236"/>
-      <c r="C1" s="237"/>
-      <c r="D1" s="237"/>
-      <c r="E1" s="237"/>
-      <c r="F1" s="237"/>
-      <c r="G1" s="237"/>
-      <c r="H1" s="237"/>
-      <c r="I1" s="237"/>
-      <c r="J1" s="237"/>
-      <c r="K1" s="237"/>
-      <c r="L1" s="238"/>
+      <c r="B1" s="153"/>
+      <c r="C1" s="154"/>
+      <c r="D1" s="154"/>
+      <c r="E1" s="154"/>
+      <c r="F1" s="154"/>
+      <c r="G1" s="154"/>
+      <c r="H1" s="154"/>
+      <c r="I1" s="154"/>
+      <c r="J1" s="154"/>
+      <c r="K1" s="154"/>
+      <c r="L1" s="155"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="239" t="s">
+      <c r="B2" s="156" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="240"/>
-      <c r="D2" s="240"/>
-      <c r="E2" s="240"/>
-      <c r="F2" s="240"/>
-      <c r="G2" s="240"/>
-      <c r="H2" s="240"/>
-      <c r="I2" s="241"/>
-      <c r="J2" s="245"/>
-      <c r="K2" s="246"/>
-      <c r="L2" s="247"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="157"/>
+      <c r="F2" s="157"/>
+      <c r="G2" s="157"/>
+      <c r="H2" s="157"/>
+      <c r="I2" s="158"/>
+      <c r="J2" s="162"/>
+      <c r="K2" s="163"/>
+      <c r="L2" s="164"/>
     </row>
     <row r="3" spans="1:13" ht="14.4" customHeight="1">
-      <c r="B3" s="242"/>
-      <c r="C3" s="243"/>
-      <c r="D3" s="243"/>
-      <c r="E3" s="243"/>
-      <c r="F3" s="243"/>
-      <c r="G3" s="243"/>
-      <c r="H3" s="243"/>
-      <c r="I3" s="244"/>
-      <c r="J3" s="248"/>
-      <c r="K3" s="249"/>
-      <c r="L3" s="250"/>
+      <c r="B3" s="159"/>
+      <c r="C3" s="160"/>
+      <c r="D3" s="160"/>
+      <c r="E3" s="160"/>
+      <c r="F3" s="160"/>
+      <c r="G3" s="160"/>
+      <c r="H3" s="160"/>
+      <c r="I3" s="161"/>
+      <c r="J3" s="165"/>
+      <c r="K3" s="166"/>
+      <c r="L3" s="167"/>
     </row>
     <row r="4" spans="1:13" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -41057,9 +41065,9 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="248"/>
-      <c r="K4" s="249"/>
-      <c r="L4" s="250"/>
+      <c r="J4" s="165"/>
+      <c r="K4" s="166"/>
+      <c r="L4" s="167"/>
     </row>
     <row r="5" spans="1:13" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -41074,9 +41082,9 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="248"/>
-      <c r="K5" s="249"/>
-      <c r="L5" s="250"/>
+      <c r="J5" s="165"/>
+      <c r="K5" s="166"/>
+      <c r="L5" s="167"/>
     </row>
     <row r="6" spans="1:13" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -41091,9 +41099,9 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="251"/>
-      <c r="K6" s="252"/>
-      <c r="L6" s="253"/>
+      <c r="J6" s="168"/>
+      <c r="K6" s="169"/>
+      <c r="L6" s="170"/>
     </row>
     <row r="7" spans="1:13" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -41149,41 +41157,41 @@
       <c r="L9" s="89"/>
     </row>
     <row r="10" spans="1:13" ht="15.6">
-      <c r="B10" s="254" t="s">
+      <c r="B10" s="171" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="255"/>
-      <c r="D10" s="255"/>
-      <c r="E10" s="255"/>
-      <c r="F10" s="256"/>
-      <c r="G10" s="255" t="s">
+      <c r="C10" s="172"/>
+      <c r="D10" s="172"/>
+      <c r="E10" s="172"/>
+      <c r="F10" s="173"/>
+      <c r="G10" s="172" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="255"/>
-      <c r="I10" s="255"/>
-      <c r="J10" s="256"/>
-      <c r="K10" s="255" t="s">
+      <c r="H10" s="172"/>
+      <c r="I10" s="172"/>
+      <c r="J10" s="173"/>
+      <c r="K10" s="172" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="257"/>
+      <c r="L10" s="174"/>
     </row>
     <row r="11" spans="1:13" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="202" t="s">
+      <c r="C11" s="193" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="203"/>
-      <c r="E11" s="203"/>
+      <c r="D11" s="194"/>
+      <c r="E11" s="194"/>
       <c r="F11" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="202" t="s">
+      <c r="G11" s="193" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="204"/>
+      <c r="H11" s="195"/>
       <c r="I11" s="92" t="s">
         <v>27</v>
       </c>
@@ -41202,14 +41210,14 @@
       <c r="B12" s="94" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="151" t="s">
+      <c r="C12" s="239" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="152"/>
-      <c r="E12" s="153"/>
+      <c r="D12" s="240"/>
+      <c r="E12" s="241"/>
       <c r="F12" s="95"/>
-      <c r="G12" s="211"/>
-      <c r="H12" s="212"/>
+      <c r="G12" s="202"/>
+      <c r="H12" s="203"/>
       <c r="I12" s="96"/>
       <c r="J12" s="96"/>
       <c r="K12" s="97"/>
@@ -41219,14 +41227,14 @@
       <c r="B13" s="99">
         <v>1</v>
       </c>
-      <c r="C13" s="154" t="s">
+      <c r="C13" s="242" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="155"/>
-      <c r="E13" s="156"/>
+      <c r="D13" s="243"/>
+      <c r="E13" s="244"/>
       <c r="F13" s="100"/>
-      <c r="G13" s="213"/>
-      <c r="H13" s="214"/>
+      <c r="G13" s="204"/>
+      <c r="H13" s="205"/>
       <c r="I13" s="101"/>
       <c r="J13" s="102"/>
       <c r="K13" s="103"/>
@@ -41236,14 +41244,14 @@
       <c r="B14" s="99">
         <v>2</v>
       </c>
-      <c r="C14" s="154" t="s">
+      <c r="C14" s="242" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="155"/>
-      <c r="E14" s="156"/>
+      <c r="D14" s="243"/>
+      <c r="E14" s="244"/>
       <c r="F14" s="100"/>
-      <c r="G14" s="213"/>
-      <c r="H14" s="214"/>
+      <c r="G14" s="204"/>
+      <c r="H14" s="205"/>
       <c r="I14" s="101"/>
       <c r="J14" s="102"/>
       <c r="K14" s="103"/>
@@ -41253,14 +41261,14 @@
       <c r="B15" s="99">
         <v>3</v>
       </c>
-      <c r="C15" s="154" t="s">
+      <c r="C15" s="242" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="155"/>
-      <c r="E15" s="156"/>
+      <c r="D15" s="243"/>
+      <c r="E15" s="244"/>
       <c r="F15" s="100"/>
-      <c r="G15" s="213"/>
-      <c r="H15" s="214"/>
+      <c r="G15" s="204"/>
+      <c r="H15" s="205"/>
       <c r="I15" s="101"/>
       <c r="J15" s="102"/>
       <c r="K15" s="103"/>
@@ -41270,14 +41278,14 @@
       <c r="B16" s="99">
         <v>4</v>
       </c>
-      <c r="C16" s="154" t="s">
+      <c r="C16" s="242" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="155"/>
-      <c r="E16" s="156"/>
+      <c r="D16" s="243"/>
+      <c r="E16" s="244"/>
       <c r="F16" s="100"/>
-      <c r="G16" s="213"/>
-      <c r="H16" s="214"/>
+      <c r="G16" s="204"/>
+      <c r="H16" s="205"/>
       <c r="I16" s="101"/>
       <c r="J16" s="102"/>
       <c r="K16" s="103"/>
@@ -41287,14 +41295,14 @@
       <c r="B17" s="99">
         <v>5</v>
       </c>
-      <c r="C17" s="154" t="s">
+      <c r="C17" s="242" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="155"/>
-      <c r="E17" s="156"/>
+      <c r="D17" s="243"/>
+      <c r="E17" s="244"/>
       <c r="F17" s="100"/>
-      <c r="G17" s="213"/>
-      <c r="H17" s="214"/>
+      <c r="G17" s="204"/>
+      <c r="H17" s="205"/>
       <c r="I17" s="101"/>
       <c r="J17" s="102"/>
       <c r="K17" s="103"/>
@@ -41304,14 +41312,14 @@
       <c r="B18" s="99">
         <v>6</v>
       </c>
-      <c r="C18" s="154" t="s">
+      <c r="C18" s="242" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="155"/>
-      <c r="E18" s="156"/>
+      <c r="D18" s="243"/>
+      <c r="E18" s="244"/>
       <c r="F18" s="100"/>
-      <c r="G18" s="213"/>
-      <c r="H18" s="214"/>
+      <c r="G18" s="204"/>
+      <c r="H18" s="205"/>
       <c r="I18" s="101"/>
       <c r="J18" s="102"/>
       <c r="K18" s="103"/>
@@ -41321,14 +41329,14 @@
       <c r="B19" s="105" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="157" t="s">
+      <c r="C19" s="245" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="158"/>
-      <c r="E19" s="159"/>
+      <c r="D19" s="246"/>
+      <c r="E19" s="247"/>
       <c r="F19" s="100"/>
-      <c r="G19" s="213"/>
-      <c r="H19" s="214"/>
+      <c r="G19" s="204"/>
+      <c r="H19" s="205"/>
       <c r="I19" s="101"/>
       <c r="J19" s="102"/>
       <c r="K19" s="103"/>
@@ -41338,14 +41346,14 @@
       <c r="B20" s="99">
         <v>1</v>
       </c>
-      <c r="C20" s="154" t="s">
+      <c r="C20" s="242" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="155"/>
-      <c r="E20" s="156"/>
+      <c r="D20" s="243"/>
+      <c r="E20" s="244"/>
       <c r="F20" s="100"/>
-      <c r="G20" s="213"/>
-      <c r="H20" s="214"/>
+      <c r="G20" s="204"/>
+      <c r="H20" s="205"/>
       <c r="I20" s="101"/>
       <c r="J20" s="102"/>
       <c r="K20" s="103"/>
@@ -41355,14 +41363,14 @@
       <c r="B21" s="99">
         <v>2</v>
       </c>
-      <c r="C21" s="154" t="s">
+      <c r="C21" s="242" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="155"/>
-      <c r="E21" s="156"/>
+      <c r="D21" s="243"/>
+      <c r="E21" s="244"/>
       <c r="F21" s="100"/>
-      <c r="G21" s="213"/>
-      <c r="H21" s="214"/>
+      <c r="G21" s="204"/>
+      <c r="H21" s="205"/>
       <c r="I21" s="101"/>
       <c r="J21" s="102"/>
       <c r="K21" s="103"/>
@@ -41372,64 +41380,64 @@
       <c r="B22" s="99">
         <v>3</v>
       </c>
-      <c r="C22" s="160" t="s">
+      <c r="C22" s="248" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="161"/>
-      <c r="E22" s="162"/>
+      <c r="D22" s="249"/>
+      <c r="E22" s="250"/>
       <c r="F22" s="100"/>
-      <c r="G22" s="215"/>
-      <c r="H22" s="216"/>
+      <c r="G22" s="206"/>
+      <c r="H22" s="207"/>
       <c r="I22" s="101"/>
       <c r="J22" s="102"/>
       <c r="K22" s="106"/>
       <c r="L22" s="107"/>
     </row>
     <row r="23" spans="1:12" ht="16.2" thickBot="1">
-      <c r="B23" s="205"/>
-      <c r="C23" s="206"/>
-      <c r="D23" s="206"/>
-      <c r="E23" s="206"/>
+      <c r="B23" s="196"/>
+      <c r="C23" s="197"/>
+      <c r="D23" s="197"/>
+      <c r="E23" s="197"/>
       <c r="F23" s="108"/>
       <c r="G23" s="108"/>
       <c r="H23" s="109"/>
       <c r="I23" s="109"/>
-      <c r="J23" s="207"/>
-      <c r="K23" s="207"/>
-      <c r="L23" s="208"/>
+      <c r="J23" s="198"/>
+      <c r="K23" s="198"/>
+      <c r="L23" s="199"/>
     </row>
     <row r="24" spans="1:12" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="125" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="209" t="s">
+      <c r="B24" s="200" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="217" t="s">
+      <c r="C24" s="175" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="217"/>
-      <c r="E24" s="217"/>
-      <c r="F24" s="217"/>
-      <c r="G24" s="217"/>
-      <c r="H24" s="217"/>
-      <c r="I24" s="217"/>
-      <c r="J24" s="219" t="s">
+      <c r="D24" s="175"/>
+      <c r="E24" s="175"/>
+      <c r="F24" s="175"/>
+      <c r="G24" s="175"/>
+      <c r="H24" s="175"/>
+      <c r="I24" s="175"/>
+      <c r="J24" s="177" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="220"/>
-      <c r="L24" s="221"/>
+      <c r="K24" s="178"/>
+      <c r="L24" s="179"/>
     </row>
     <row r="25" spans="1:12" ht="31.2">
-      <c r="B25" s="210"/>
-      <c r="C25" s="218"/>
-      <c r="D25" s="218"/>
-      <c r="E25" s="218"/>
-      <c r="F25" s="218"/>
-      <c r="G25" s="218"/>
-      <c r="H25" s="218"/>
-      <c r="I25" s="218"/>
-      <c r="J25" s="304" t="s">
+      <c r="B25" s="201"/>
+      <c r="C25" s="176"/>
+      <c r="D25" s="176"/>
+      <c r="E25" s="176"/>
+      <c r="F25" s="176"/>
+      <c r="G25" s="176"/>
+      <c r="H25" s="176"/>
+      <c r="I25" s="176"/>
+      <c r="J25" s="152" t="s">
         <v>9</v>
       </c>
       <c r="K25" s="149" t="s">
@@ -41441,63 +41449,63 @@
     </row>
     <row r="26" spans="1:12" ht="15.6">
       <c r="B26" s="110" t="s">
+        <v>132</v>
+      </c>
+      <c r="C26" s="294" t="s">
+        <v>133</v>
+      </c>
+      <c r="D26" s="295"/>
+      <c r="E26" s="295"/>
+      <c r="F26" s="295"/>
+      <c r="G26" s="295"/>
+      <c r="H26" s="295"/>
+      <c r="I26" s="296"/>
+      <c r="J26" s="303" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="163" t="s">
-        <v>64</v>
-      </c>
-      <c r="D26" s="235"/>
-      <c r="E26" s="235"/>
-      <c r="F26" s="235"/>
-      <c r="G26" s="235"/>
-      <c r="H26" s="235"/>
-      <c r="I26" s="164"/>
-      <c r="J26" s="305" t="s">
-        <v>64</v>
-      </c>
-      <c r="K26" s="301"/>
+      <c r="K26" s="151"/>
       <c r="L26" s="111" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="15.6">
-      <c r="B27" s="110" t="s">
-        <v>64</v>
+      <c r="B27" s="110">
+        <v>1</v>
       </c>
-      <c r="C27" s="165" t="s">
-        <v>64</v>
+      <c r="C27" s="297" t="s">
+        <v>134</v>
       </c>
-      <c r="D27" s="166"/>
-      <c r="E27" s="166"/>
-      <c r="F27" s="166"/>
-      <c r="G27" s="166"/>
-      <c r="H27" s="166"/>
-      <c r="I27" s="167"/>
-      <c r="J27" s="306" t="s">
-        <v>64</v>
+      <c r="D27" s="298"/>
+      <c r="E27" s="298"/>
+      <c r="F27" s="298"/>
+      <c r="G27" s="298"/>
+      <c r="H27" s="298"/>
+      <c r="I27" s="299"/>
+      <c r="J27" s="102" t="s">
+        <v>135</v>
       </c>
-      <c r="K27" s="302"/>
+      <c r="K27" s="305"/>
       <c r="L27" s="112" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="15.6">
-      <c r="B28" s="110" t="s">
+      <c r="B28" s="110">
+        <v>2</v>
+      </c>
+      <c r="C28" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="165" t="s">
+      <c r="D28" s="298"/>
+      <c r="E28" s="298"/>
+      <c r="F28" s="298"/>
+      <c r="G28" s="298"/>
+      <c r="H28" s="298"/>
+      <c r="I28" s="299"/>
+      <c r="J28" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="D28" s="166"/>
-      <c r="E28" s="166"/>
-      <c r="F28" s="166"/>
-      <c r="G28" s="166"/>
-      <c r="H28" s="166"/>
-      <c r="I28" s="167"/>
-      <c r="J28" s="306" t="s">
-        <v>64</v>
-      </c>
-      <c r="K28" s="302"/>
+      <c r="K28" s="305"/>
       <c r="L28" s="112" t="s">
         <v>64</v>
       </c>
@@ -41506,19 +41514,19 @@
       <c r="B29" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="165" t="s">
+      <c r="C29" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="166"/>
-      <c r="E29" s="166"/>
-      <c r="F29" s="166"/>
-      <c r="G29" s="166"/>
-      <c r="H29" s="166"/>
-      <c r="I29" s="167"/>
-      <c r="J29" s="306" t="s">
+      <c r="D29" s="298"/>
+      <c r="E29" s="298"/>
+      <c r="F29" s="298"/>
+      <c r="G29" s="298"/>
+      <c r="H29" s="298"/>
+      <c r="I29" s="299"/>
+      <c r="J29" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K29" s="302"/>
+      <c r="K29" s="305"/>
       <c r="L29" s="112" t="s">
         <v>64</v>
       </c>
@@ -41527,19 +41535,19 @@
       <c r="B30" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="165" t="s">
+      <c r="C30" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="166"/>
-      <c r="E30" s="166"/>
-      <c r="F30" s="166"/>
-      <c r="G30" s="166"/>
-      <c r="H30" s="166"/>
-      <c r="I30" s="167"/>
-      <c r="J30" s="306" t="s">
+      <c r="D30" s="298"/>
+      <c r="E30" s="298"/>
+      <c r="F30" s="298"/>
+      <c r="G30" s="298"/>
+      <c r="H30" s="298"/>
+      <c r="I30" s="299"/>
+      <c r="J30" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K30" s="302"/>
+      <c r="K30" s="305"/>
       <c r="L30" s="112" t="s">
         <v>64</v>
       </c>
@@ -41548,19 +41556,19 @@
       <c r="B31" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="165" t="s">
+      <c r="C31" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="166"/>
-      <c r="E31" s="166"/>
-      <c r="F31" s="166"/>
-      <c r="G31" s="166"/>
-      <c r="H31" s="166"/>
-      <c r="I31" s="167"/>
-      <c r="J31" s="306" t="s">
+      <c r="D31" s="298"/>
+      <c r="E31" s="298"/>
+      <c r="F31" s="298"/>
+      <c r="G31" s="298"/>
+      <c r="H31" s="298"/>
+      <c r="I31" s="299"/>
+      <c r="J31" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K31" s="302"/>
+      <c r="K31" s="305"/>
       <c r="L31" s="112" t="s">
         <v>64</v>
       </c>
@@ -41569,19 +41577,19 @@
       <c r="B32" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="165" t="s">
+      <c r="C32" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="166"/>
-      <c r="E32" s="166"/>
-      <c r="F32" s="166"/>
-      <c r="G32" s="166"/>
-      <c r="H32" s="166"/>
-      <c r="I32" s="167"/>
-      <c r="J32" s="306" t="s">
+      <c r="D32" s="298"/>
+      <c r="E32" s="298"/>
+      <c r="F32" s="298"/>
+      <c r="G32" s="298"/>
+      <c r="H32" s="298"/>
+      <c r="I32" s="299"/>
+      <c r="J32" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K32" s="302"/>
+      <c r="K32" s="305"/>
       <c r="L32" s="112" t="s">
         <v>64</v>
       </c>
@@ -41590,19 +41598,19 @@
       <c r="B33" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="165" t="s">
+      <c r="C33" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="166"/>
-      <c r="E33" s="166"/>
-      <c r="F33" s="166"/>
-      <c r="G33" s="166"/>
-      <c r="H33" s="166"/>
-      <c r="I33" s="167"/>
-      <c r="J33" s="306" t="s">
+      <c r="D33" s="298"/>
+      <c r="E33" s="298"/>
+      <c r="F33" s="298"/>
+      <c r="G33" s="298"/>
+      <c r="H33" s="298"/>
+      <c r="I33" s="299"/>
+      <c r="J33" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K33" s="302"/>
+      <c r="K33" s="305"/>
       <c r="L33" s="112" t="s">
         <v>64</v>
       </c>
@@ -41611,19 +41619,19 @@
       <c r="B34" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="165" t="s">
+      <c r="C34" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="166"/>
-      <c r="E34" s="166"/>
-      <c r="F34" s="166"/>
-      <c r="G34" s="166"/>
-      <c r="H34" s="166"/>
-      <c r="I34" s="167"/>
-      <c r="J34" s="306" t="s">
+      <c r="D34" s="298"/>
+      <c r="E34" s="298"/>
+      <c r="F34" s="298"/>
+      <c r="G34" s="298"/>
+      <c r="H34" s="298"/>
+      <c r="I34" s="299"/>
+      <c r="J34" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K34" s="302"/>
+      <c r="K34" s="305"/>
       <c r="L34" s="112" t="s">
         <v>64</v>
       </c>
@@ -41632,19 +41640,19 @@
       <c r="B35" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="165" t="s">
+      <c r="C35" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="166"/>
-      <c r="E35" s="166"/>
-      <c r="F35" s="166"/>
-      <c r="G35" s="166"/>
-      <c r="H35" s="166"/>
-      <c r="I35" s="167"/>
-      <c r="J35" s="306" t="s">
+      <c r="D35" s="298"/>
+      <c r="E35" s="298"/>
+      <c r="F35" s="298"/>
+      <c r="G35" s="298"/>
+      <c r="H35" s="298"/>
+      <c r="I35" s="299"/>
+      <c r="J35" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K35" s="302"/>
+      <c r="K35" s="305"/>
       <c r="L35" s="112" t="s">
         <v>64</v>
       </c>
@@ -41653,19 +41661,19 @@
       <c r="B36" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C36" s="165" t="s">
+      <c r="C36" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="166"/>
-      <c r="E36" s="166"/>
-      <c r="F36" s="166"/>
-      <c r="G36" s="166"/>
-      <c r="H36" s="166"/>
-      <c r="I36" s="167"/>
-      <c r="J36" s="306" t="s">
+      <c r="D36" s="298"/>
+      <c r="E36" s="298"/>
+      <c r="F36" s="298"/>
+      <c r="G36" s="298"/>
+      <c r="H36" s="298"/>
+      <c r="I36" s="299"/>
+      <c r="J36" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K36" s="302"/>
+      <c r="K36" s="305"/>
       <c r="L36" s="112" t="s">
         <v>64</v>
       </c>
@@ -41674,19 +41682,19 @@
       <c r="B37" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="165" t="s">
+      <c r="C37" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="166"/>
-      <c r="E37" s="166"/>
-      <c r="F37" s="166"/>
-      <c r="G37" s="166"/>
-      <c r="H37" s="166"/>
-      <c r="I37" s="167"/>
-      <c r="J37" s="306" t="s">
+      <c r="D37" s="298"/>
+      <c r="E37" s="298"/>
+      <c r="F37" s="298"/>
+      <c r="G37" s="298"/>
+      <c r="H37" s="298"/>
+      <c r="I37" s="299"/>
+      <c r="J37" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K37" s="302"/>
+      <c r="K37" s="305"/>
       <c r="L37" s="112" t="s">
         <v>64</v>
       </c>
@@ -41695,19 +41703,19 @@
       <c r="B38" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="165" t="s">
+      <c r="C38" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="166"/>
-      <c r="E38" s="166"/>
-      <c r="F38" s="166"/>
-      <c r="G38" s="166"/>
-      <c r="H38" s="166"/>
-      <c r="I38" s="167"/>
-      <c r="J38" s="306" t="s">
+      <c r="D38" s="298"/>
+      <c r="E38" s="298"/>
+      <c r="F38" s="298"/>
+      <c r="G38" s="298"/>
+      <c r="H38" s="298"/>
+      <c r="I38" s="299"/>
+      <c r="J38" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K38" s="302"/>
+      <c r="K38" s="305"/>
       <c r="L38" s="112" t="s">
         <v>64</v>
       </c>
@@ -41716,19 +41724,19 @@
       <c r="B39" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="165" t="s">
+      <c r="C39" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D39" s="166"/>
-      <c r="E39" s="166"/>
-      <c r="F39" s="166"/>
-      <c r="G39" s="166"/>
-      <c r="H39" s="166"/>
-      <c r="I39" s="167"/>
-      <c r="J39" s="306" t="s">
+      <c r="D39" s="298"/>
+      <c r="E39" s="298"/>
+      <c r="F39" s="298"/>
+      <c r="G39" s="298"/>
+      <c r="H39" s="298"/>
+      <c r="I39" s="299"/>
+      <c r="J39" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K39" s="302"/>
+      <c r="K39" s="305"/>
       <c r="L39" s="112" t="s">
         <v>64</v>
       </c>
@@ -41737,19 +41745,19 @@
       <c r="B40" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="165" t="s">
+      <c r="C40" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D40" s="166"/>
-      <c r="E40" s="166"/>
-      <c r="F40" s="166"/>
-      <c r="G40" s="166"/>
-      <c r="H40" s="166"/>
-      <c r="I40" s="167"/>
-      <c r="J40" s="306" t="s">
+      <c r="D40" s="298"/>
+      <c r="E40" s="298"/>
+      <c r="F40" s="298"/>
+      <c r="G40" s="298"/>
+      <c r="H40" s="298"/>
+      <c r="I40" s="299"/>
+      <c r="J40" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K40" s="302"/>
+      <c r="K40" s="305"/>
       <c r="L40" s="112" t="s">
         <v>64</v>
       </c>
@@ -41758,19 +41766,19 @@
       <c r="B41" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="165" t="s">
+      <c r="C41" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D41" s="166"/>
-      <c r="E41" s="166"/>
-      <c r="F41" s="166"/>
-      <c r="G41" s="166"/>
-      <c r="H41" s="166"/>
-      <c r="I41" s="167"/>
-      <c r="J41" s="306" t="s">
+      <c r="D41" s="298"/>
+      <c r="E41" s="298"/>
+      <c r="F41" s="298"/>
+      <c r="G41" s="298"/>
+      <c r="H41" s="298"/>
+      <c r="I41" s="299"/>
+      <c r="J41" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K41" s="302"/>
+      <c r="K41" s="305"/>
       <c r="L41" s="112" t="s">
         <v>64</v>
       </c>
@@ -41779,19 +41787,19 @@
       <c r="B42" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="165" t="s">
+      <c r="C42" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="166"/>
-      <c r="E42" s="166"/>
-      <c r="F42" s="166"/>
-      <c r="G42" s="166"/>
-      <c r="H42" s="166"/>
-      <c r="I42" s="167"/>
-      <c r="J42" s="306" t="s">
+      <c r="D42" s="298"/>
+      <c r="E42" s="298"/>
+      <c r="F42" s="298"/>
+      <c r="G42" s="298"/>
+      <c r="H42" s="298"/>
+      <c r="I42" s="299"/>
+      <c r="J42" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K42" s="302"/>
+      <c r="K42" s="305"/>
       <c r="L42" s="112" t="s">
         <v>64</v>
       </c>
@@ -41800,19 +41808,19 @@
       <c r="B43" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="165" t="s">
+      <c r="C43" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="166"/>
-      <c r="E43" s="166"/>
-      <c r="F43" s="166"/>
-      <c r="G43" s="166"/>
-      <c r="H43" s="166"/>
-      <c r="I43" s="167"/>
-      <c r="J43" s="306" t="s">
+      <c r="D43" s="298"/>
+      <c r="E43" s="298"/>
+      <c r="F43" s="298"/>
+      <c r="G43" s="298"/>
+      <c r="H43" s="298"/>
+      <c r="I43" s="299"/>
+      <c r="J43" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K43" s="302"/>
+      <c r="K43" s="305"/>
       <c r="L43" s="112" t="s">
         <v>64</v>
       </c>
@@ -41821,19 +41829,19 @@
       <c r="B44" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="165" t="s">
+      <c r="C44" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D44" s="166"/>
-      <c r="E44" s="166"/>
-      <c r="F44" s="166"/>
-      <c r="G44" s="166"/>
-      <c r="H44" s="166"/>
-      <c r="I44" s="167"/>
-      <c r="J44" s="306" t="s">
+      <c r="D44" s="298"/>
+      <c r="E44" s="298"/>
+      <c r="F44" s="298"/>
+      <c r="G44" s="298"/>
+      <c r="H44" s="298"/>
+      <c r="I44" s="299"/>
+      <c r="J44" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K44" s="302"/>
+      <c r="K44" s="305"/>
       <c r="L44" s="112" t="s">
         <v>64</v>
       </c>
@@ -41842,19 +41850,19 @@
       <c r="B45" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C45" s="165" t="s">
+      <c r="C45" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D45" s="166"/>
-      <c r="E45" s="166"/>
-      <c r="F45" s="166"/>
-      <c r="G45" s="166"/>
-      <c r="H45" s="166"/>
-      <c r="I45" s="167"/>
-      <c r="J45" s="306" t="s">
+      <c r="D45" s="298"/>
+      <c r="E45" s="298"/>
+      <c r="F45" s="298"/>
+      <c r="G45" s="298"/>
+      <c r="H45" s="298"/>
+      <c r="I45" s="299"/>
+      <c r="J45" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K45" s="302"/>
+      <c r="K45" s="305"/>
       <c r="L45" s="112" t="s">
         <v>64</v>
       </c>
@@ -41863,19 +41871,19 @@
       <c r="B46" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C46" s="165" t="s">
+      <c r="C46" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="166"/>
-      <c r="E46" s="166"/>
-      <c r="F46" s="166"/>
-      <c r="G46" s="166"/>
-      <c r="H46" s="166"/>
-      <c r="I46" s="167"/>
-      <c r="J46" s="306" t="s">
+      <c r="D46" s="298"/>
+      <c r="E46" s="298"/>
+      <c r="F46" s="298"/>
+      <c r="G46" s="298"/>
+      <c r="H46" s="298"/>
+      <c r="I46" s="299"/>
+      <c r="J46" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K46" s="302"/>
+      <c r="K46" s="305"/>
       <c r="L46" s="112" t="s">
         <v>64</v>
       </c>
@@ -41884,19 +41892,19 @@
       <c r="B47" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="165" t="s">
+      <c r="C47" s="297" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="166"/>
-      <c r="E47" s="166"/>
-      <c r="F47" s="166"/>
-      <c r="G47" s="166"/>
-      <c r="H47" s="166"/>
-      <c r="I47" s="167"/>
-      <c r="J47" s="306" t="s">
+      <c r="D47" s="298"/>
+      <c r="E47" s="298"/>
+      <c r="F47" s="298"/>
+      <c r="G47" s="298"/>
+      <c r="H47" s="298"/>
+      <c r="I47" s="299"/>
+      <c r="J47" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K47" s="302"/>
+      <c r="K47" s="305"/>
       <c r="L47" s="112" t="s">
         <v>64</v>
       </c>
@@ -41905,194 +41913,194 @@
       <c r="B48" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C48" s="168" t="s">
+      <c r="C48" s="300" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="169"/>
-      <c r="E48" s="169"/>
-      <c r="F48" s="169"/>
-      <c r="G48" s="169"/>
-      <c r="H48" s="169"/>
-      <c r="I48" s="170"/>
-      <c r="J48" s="307" t="s">
+      <c r="D48" s="301"/>
+      <c r="E48" s="301"/>
+      <c r="F48" s="301"/>
+      <c r="G48" s="301"/>
+      <c r="H48" s="301"/>
+      <c r="I48" s="302"/>
+      <c r="J48" s="304" t="s">
         <v>64</v>
       </c>
-      <c r="K48" s="303"/>
+      <c r="K48" s="306"/>
       <c r="L48" s="112" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="49" spans="2:12" ht="16.2" thickTop="1">
-      <c r="B49" s="184" t="s">
+      <c r="B49" s="221" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="185"/>
-      <c r="D49" s="185"/>
-      <c r="E49" s="185"/>
-      <c r="F49" s="185"/>
-      <c r="G49" s="185"/>
-      <c r="H49" s="185"/>
-      <c r="I49" s="185"/>
-      <c r="J49" s="186"/>
-      <c r="K49" s="233" t="s">
+      <c r="C49" s="222"/>
+      <c r="D49" s="222"/>
+      <c r="E49" s="222"/>
+      <c r="F49" s="222"/>
+      <c r="G49" s="222"/>
+      <c r="H49" s="222"/>
+      <c r="I49" s="222"/>
+      <c r="J49" s="223"/>
+      <c r="K49" s="191" t="s">
         <v>79</v>
       </c>
-      <c r="L49" s="234"/>
+      <c r="L49" s="192"/>
     </row>
     <row r="50" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B50" s="187"/>
-      <c r="C50" s="188"/>
-      <c r="D50" s="188"/>
-      <c r="E50" s="188"/>
-      <c r="F50" s="188"/>
-      <c r="G50" s="188"/>
-      <c r="H50" s="188"/>
-      <c r="I50" s="188"/>
-      <c r="J50" s="189"/>
-      <c r="K50" s="231" t="s">
+      <c r="B50" s="224"/>
+      <c r="C50" s="225"/>
+      <c r="D50" s="225"/>
+      <c r="E50" s="225"/>
+      <c r="F50" s="225"/>
+      <c r="G50" s="225"/>
+      <c r="H50" s="225"/>
+      <c r="I50" s="225"/>
+      <c r="J50" s="226"/>
+      <c r="K50" s="189" t="s">
         <v>103</v>
       </c>
-      <c r="L50" s="232"/>
+      <c r="L50" s="190"/>
     </row>
     <row r="51" spans="2:12" ht="15.6">
       <c r="B51" s="113"/>
-      <c r="C51" s="228"/>
-      <c r="D51" s="228"/>
-      <c r="E51" s="228"/>
-      <c r="F51" s="228"/>
-      <c r="G51" s="228"/>
-      <c r="H51" s="228"/>
-      <c r="I51" s="228"/>
+      <c r="C51" s="186"/>
+      <c r="D51" s="186"/>
+      <c r="E51" s="186"/>
+      <c r="F51" s="186"/>
+      <c r="G51" s="186"/>
+      <c r="H51" s="186"/>
+      <c r="I51" s="186"/>
       <c r="J51" s="114"/>
-      <c r="K51" s="226"/>
-      <c r="L51" s="227"/>
+      <c r="K51" s="184"/>
+      <c r="L51" s="185"/>
     </row>
     <row r="52" spans="2:12" ht="15.6">
       <c r="B52" s="115"/>
-      <c r="C52" s="229"/>
-      <c r="D52" s="229"/>
-      <c r="E52" s="229"/>
-      <c r="F52" s="229"/>
-      <c r="G52" s="229"/>
-      <c r="H52" s="229"/>
-      <c r="I52" s="229"/>
+      <c r="C52" s="187"/>
+      <c r="D52" s="187"/>
+      <c r="E52" s="187"/>
+      <c r="F52" s="187"/>
+      <c r="G52" s="187"/>
+      <c r="H52" s="187"/>
+      <c r="I52" s="187"/>
       <c r="J52" s="116"/>
       <c r="K52" s="127"/>
       <c r="L52" s="117"/>
     </row>
     <row r="53" spans="2:12" ht="15.6">
       <c r="B53" s="115"/>
-      <c r="C53" s="229"/>
-      <c r="D53" s="229"/>
-      <c r="E53" s="229"/>
-      <c r="F53" s="229"/>
-      <c r="G53" s="229"/>
-      <c r="H53" s="229"/>
-      <c r="I53" s="229"/>
+      <c r="C53" s="187"/>
+      <c r="D53" s="187"/>
+      <c r="E53" s="187"/>
+      <c r="F53" s="187"/>
+      <c r="G53" s="187"/>
+      <c r="H53" s="187"/>
+      <c r="I53" s="187"/>
       <c r="J53" s="116"/>
       <c r="K53" s="127"/>
       <c r="L53" s="117"/>
     </row>
     <row r="54" spans="2:12" ht="15.6">
       <c r="B54" s="115"/>
-      <c r="C54" s="229"/>
-      <c r="D54" s="229"/>
-      <c r="E54" s="229"/>
-      <c r="F54" s="229"/>
-      <c r="G54" s="229"/>
-      <c r="H54" s="229"/>
-      <c r="I54" s="229"/>
+      <c r="C54" s="187"/>
+      <c r="D54" s="187"/>
+      <c r="E54" s="187"/>
+      <c r="F54" s="187"/>
+      <c r="G54" s="187"/>
+      <c r="H54" s="187"/>
+      <c r="I54" s="187"/>
       <c r="J54" s="116"/>
       <c r="K54" s="127"/>
       <c r="L54" s="117"/>
     </row>
     <row r="55" spans="2:12" ht="15.6">
       <c r="B55" s="118"/>
-      <c r="C55" s="229"/>
-      <c r="D55" s="229"/>
-      <c r="E55" s="229"/>
-      <c r="F55" s="229"/>
-      <c r="G55" s="229"/>
-      <c r="H55" s="229"/>
-      <c r="I55" s="229"/>
+      <c r="C55" s="187"/>
+      <c r="D55" s="187"/>
+      <c r="E55" s="187"/>
+      <c r="F55" s="187"/>
+      <c r="G55" s="187"/>
+      <c r="H55" s="187"/>
+      <c r="I55" s="187"/>
       <c r="J55" s="119"/>
       <c r="K55" s="120"/>
       <c r="L55" s="121"/>
     </row>
     <row r="56" spans="2:12" ht="15.6">
       <c r="B56" s="118"/>
-      <c r="C56" s="229"/>
-      <c r="D56" s="229"/>
-      <c r="E56" s="229"/>
-      <c r="F56" s="229"/>
-      <c r="G56" s="229"/>
-      <c r="H56" s="229"/>
-      <c r="I56" s="229"/>
+      <c r="C56" s="187"/>
+      <c r="D56" s="187"/>
+      <c r="E56" s="187"/>
+      <c r="F56" s="187"/>
+      <c r="G56" s="187"/>
+      <c r="H56" s="187"/>
+      <c r="I56" s="187"/>
       <c r="J56" s="119"/>
       <c r="K56" s="120"/>
       <c r="L56" s="121"/>
     </row>
     <row r="57" spans="2:12" ht="15.6">
       <c r="B57" s="118"/>
-      <c r="C57" s="229"/>
-      <c r="D57" s="229"/>
-      <c r="E57" s="229"/>
-      <c r="F57" s="229"/>
-      <c r="G57" s="229"/>
-      <c r="H57" s="229"/>
-      <c r="I57" s="229"/>
+      <c r="C57" s="187"/>
+      <c r="D57" s="187"/>
+      <c r="E57" s="187"/>
+      <c r="F57" s="187"/>
+      <c r="G57" s="187"/>
+      <c r="H57" s="187"/>
+      <c r="I57" s="187"/>
       <c r="J57" s="119"/>
-      <c r="K57" s="222"/>
-      <c r="L57" s="223"/>
+      <c r="K57" s="180"/>
+      <c r="L57" s="181"/>
     </row>
     <row r="58" spans="2:12" ht="15.6">
       <c r="B58" s="118"/>
-      <c r="C58" s="229"/>
-      <c r="D58" s="229"/>
-      <c r="E58" s="229"/>
-      <c r="F58" s="229"/>
-      <c r="G58" s="229"/>
-      <c r="H58" s="229"/>
-      <c r="I58" s="229"/>
+      <c r="C58" s="187"/>
+      <c r="D58" s="187"/>
+      <c r="E58" s="187"/>
+      <c r="F58" s="187"/>
+      <c r="G58" s="187"/>
+      <c r="H58" s="187"/>
+      <c r="I58" s="187"/>
       <c r="J58" s="119"/>
-      <c r="K58" s="224"/>
-      <c r="L58" s="225"/>
+      <c r="K58" s="182"/>
+      <c r="L58" s="183"/>
     </row>
     <row r="59" spans="2:12" ht="15.6">
       <c r="B59" s="118"/>
-      <c r="C59" s="229"/>
-      <c r="D59" s="229"/>
-      <c r="E59" s="229"/>
-      <c r="F59" s="229"/>
-      <c r="G59" s="229"/>
-      <c r="H59" s="229"/>
-      <c r="I59" s="229"/>
+      <c r="C59" s="187"/>
+      <c r="D59" s="187"/>
+      <c r="E59" s="187"/>
+      <c r="F59" s="187"/>
+      <c r="G59" s="187"/>
+      <c r="H59" s="187"/>
+      <c r="I59" s="187"/>
       <c r="J59" s="119"/>
       <c r="K59" s="128"/>
       <c r="L59" s="76"/>
     </row>
     <row r="60" spans="2:12" ht="15.6">
       <c r="B60" s="118"/>
-      <c r="C60" s="229"/>
-      <c r="D60" s="229"/>
-      <c r="E60" s="229"/>
-      <c r="F60" s="229"/>
-      <c r="G60" s="229"/>
-      <c r="H60" s="229"/>
-      <c r="I60" s="229"/>
+      <c r="C60" s="187"/>
+      <c r="D60" s="187"/>
+      <c r="E60" s="187"/>
+      <c r="F60" s="187"/>
+      <c r="G60" s="187"/>
+      <c r="H60" s="187"/>
+      <c r="I60" s="187"/>
       <c r="J60" s="119"/>
       <c r="K60" s="128"/>
       <c r="L60" s="76"/>
     </row>
     <row r="61" spans="2:12" ht="15.6">
       <c r="B61" s="118"/>
-      <c r="C61" s="230"/>
-      <c r="D61" s="230"/>
-      <c r="E61" s="230"/>
-      <c r="F61" s="230"/>
-      <c r="G61" s="230"/>
-      <c r="H61" s="230"/>
-      <c r="I61" s="230"/>
+      <c r="C61" s="188"/>
+      <c r="D61" s="188"/>
+      <c r="E61" s="188"/>
+      <c r="F61" s="188"/>
+      <c r="G61" s="188"/>
+      <c r="H61" s="188"/>
+      <c r="I61" s="188"/>
       <c r="J61" s="119"/>
       <c r="K61" s="128"/>
       <c r="L61" s="76"/>
@@ -42111,125 +42119,125 @@
       <c r="L62" s="131"/>
     </row>
     <row r="63" spans="2:12" ht="15.6">
-      <c r="B63" s="171" t="s">
+      <c r="B63" s="208" t="s">
         <v>80</v>
       </c>
-      <c r="C63" s="172"/>
-      <c r="D63" s="172"/>
-      <c r="E63" s="173"/>
-      <c r="F63" s="174" t="s">
+      <c r="C63" s="209"/>
+      <c r="D63" s="209"/>
+      <c r="E63" s="210"/>
+      <c r="F63" s="211" t="s">
         <v>81</v>
       </c>
-      <c r="G63" s="173"/>
-      <c r="H63" s="174" t="s">
+      <c r="G63" s="210"/>
+      <c r="H63" s="211" t="s">
         <v>82</v>
       </c>
-      <c r="I63" s="172"/>
-      <c r="J63" s="173"/>
+      <c r="I63" s="209"/>
+      <c r="J63" s="210"/>
       <c r="K63" s="120"/>
       <c r="L63" s="121"/>
     </row>
     <row r="64" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B64" s="196"/>
-      <c r="C64" s="197"/>
-      <c r="D64" s="197"/>
-      <c r="E64" s="191"/>
-      <c r="F64" s="190"/>
-      <c r="G64" s="191"/>
-      <c r="H64" s="175"/>
-      <c r="I64" s="176"/>
-      <c r="J64" s="177"/>
+      <c r="B64" s="233"/>
+      <c r="C64" s="234"/>
+      <c r="D64" s="234"/>
+      <c r="E64" s="228"/>
+      <c r="F64" s="227"/>
+      <c r="G64" s="228"/>
+      <c r="H64" s="212"/>
+      <c r="I64" s="213"/>
+      <c r="J64" s="214"/>
       <c r="K64" s="120"/>
       <c r="L64" s="121"/>
     </row>
     <row r="65" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B65" s="198"/>
-      <c r="C65" s="199"/>
-      <c r="D65" s="199"/>
-      <c r="E65" s="193"/>
-      <c r="F65" s="192"/>
-      <c r="G65" s="193"/>
-      <c r="H65" s="178"/>
-      <c r="I65" s="179"/>
-      <c r="J65" s="180"/>
+      <c r="B65" s="235"/>
+      <c r="C65" s="236"/>
+      <c r="D65" s="236"/>
+      <c r="E65" s="230"/>
+      <c r="F65" s="229"/>
+      <c r="G65" s="230"/>
+      <c r="H65" s="215"/>
+      <c r="I65" s="216"/>
+      <c r="J65" s="217"/>
       <c r="K65" s="129"/>
       <c r="L65" s="121"/>
     </row>
     <row r="66" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B66" s="198"/>
-      <c r="C66" s="199"/>
-      <c r="D66" s="199"/>
-      <c r="E66" s="193"/>
-      <c r="F66" s="192"/>
-      <c r="G66" s="193"/>
-      <c r="H66" s="178"/>
-      <c r="I66" s="179"/>
-      <c r="J66" s="180"/>
+      <c r="B66" s="235"/>
+      <c r="C66" s="236"/>
+      <c r="D66" s="236"/>
+      <c r="E66" s="230"/>
+      <c r="F66" s="229"/>
+      <c r="G66" s="230"/>
+      <c r="H66" s="215"/>
+      <c r="I66" s="216"/>
+      <c r="J66" s="217"/>
       <c r="K66" s="120"/>
       <c r="L66" s="121"/>
     </row>
     <row r="67" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B67" s="198"/>
-      <c r="C67" s="199"/>
-      <c r="D67" s="199"/>
-      <c r="E67" s="193"/>
-      <c r="F67" s="192"/>
-      <c r="G67" s="193"/>
-      <c r="H67" s="178"/>
-      <c r="I67" s="179"/>
-      <c r="J67" s="180"/>
+      <c r="B67" s="235"/>
+      <c r="C67" s="236"/>
+      <c r="D67" s="236"/>
+      <c r="E67" s="230"/>
+      <c r="F67" s="229"/>
+      <c r="G67" s="230"/>
+      <c r="H67" s="215"/>
+      <c r="I67" s="216"/>
+      <c r="J67" s="217"/>
       <c r="K67" s="128"/>
       <c r="L67" s="76"/>
     </row>
     <row r="68" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B68" s="198"/>
-      <c r="C68" s="199"/>
-      <c r="D68" s="199"/>
-      <c r="E68" s="193"/>
-      <c r="F68" s="192"/>
-      <c r="G68" s="193"/>
-      <c r="H68" s="178"/>
-      <c r="I68" s="179"/>
-      <c r="J68" s="180"/>
+      <c r="B68" s="235"/>
+      <c r="C68" s="236"/>
+      <c r="D68" s="236"/>
+      <c r="E68" s="230"/>
+      <c r="F68" s="229"/>
+      <c r="G68" s="230"/>
+      <c r="H68" s="215"/>
+      <c r="I68" s="216"/>
+      <c r="J68" s="217"/>
       <c r="K68" s="128"/>
       <c r="L68" s="76"/>
     </row>
     <row r="69" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B69" s="198"/>
-      <c r="C69" s="199"/>
-      <c r="D69" s="199"/>
-      <c r="E69" s="193"/>
-      <c r="F69" s="192"/>
-      <c r="G69" s="193"/>
-      <c r="H69" s="178"/>
-      <c r="I69" s="179"/>
-      <c r="J69" s="180"/>
+      <c r="B69" s="235"/>
+      <c r="C69" s="236"/>
+      <c r="D69" s="236"/>
+      <c r="E69" s="230"/>
+      <c r="F69" s="229"/>
+      <c r="G69" s="230"/>
+      <c r="H69" s="215"/>
+      <c r="I69" s="216"/>
+      <c r="J69" s="217"/>
       <c r="K69" s="132"/>
       <c r="L69" s="133"/>
     </row>
     <row r="70" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B70" s="198"/>
-      <c r="C70" s="199"/>
-      <c r="D70" s="199"/>
-      <c r="E70" s="193"/>
-      <c r="F70" s="192"/>
-      <c r="G70" s="193"/>
-      <c r="H70" s="178"/>
-      <c r="I70" s="179"/>
-      <c r="J70" s="180"/>
+      <c r="B70" s="235"/>
+      <c r="C70" s="236"/>
+      <c r="D70" s="236"/>
+      <c r="E70" s="230"/>
+      <c r="F70" s="229"/>
+      <c r="G70" s="230"/>
+      <c r="H70" s="215"/>
+      <c r="I70" s="216"/>
+      <c r="J70" s="217"/>
       <c r="K70" s="132"/>
       <c r="L70" s="133"/>
     </row>
     <row r="71" spans="2:12" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B71" s="200"/>
-      <c r="C71" s="201"/>
-      <c r="D71" s="201"/>
-      <c r="E71" s="195"/>
-      <c r="F71" s="194"/>
-      <c r="G71" s="195"/>
-      <c r="H71" s="181"/>
-      <c r="I71" s="182"/>
-      <c r="J71" s="183"/>
+      <c r="B71" s="237"/>
+      <c r="C71" s="238"/>
+      <c r="D71" s="238"/>
+      <c r="E71" s="232"/>
+      <c r="F71" s="231"/>
+      <c r="G71" s="232"/>
+      <c r="H71" s="218"/>
+      <c r="I71" s="219"/>
+      <c r="J71" s="220"/>
       <c r="K71" s="123"/>
       <c r="L71" s="124"/>
     </row>
@@ -42240,12 +42248,55 @@
     </row>
   </sheetData>
   <mergeCells count="71">
-    <mergeCell ref="B1:L1"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="J2:L6"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C44:I44"/>
+    <mergeCell ref="C45:I45"/>
+    <mergeCell ref="C46:I46"/>
+    <mergeCell ref="C47:I47"/>
+    <mergeCell ref="C48:I48"/>
+    <mergeCell ref="C39:I39"/>
+    <mergeCell ref="C40:I40"/>
+    <mergeCell ref="C41:I41"/>
+    <mergeCell ref="C42:I42"/>
+    <mergeCell ref="C43:I43"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="C36:I36"/>
+    <mergeCell ref="C37:I37"/>
+    <mergeCell ref="C38:I38"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="H63:J63"/>
+    <mergeCell ref="H64:J71"/>
+    <mergeCell ref="B49:J50"/>
+    <mergeCell ref="F64:G71"/>
+    <mergeCell ref="B64:E71"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
     <mergeCell ref="C24:I25"/>
     <mergeCell ref="J24:L24"/>
     <mergeCell ref="K57:L57"/>
@@ -42262,55 +42313,12 @@
     <mergeCell ref="C31:I31"/>
     <mergeCell ref="C32:I32"/>
     <mergeCell ref="C33:I33"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="H63:J63"/>
-    <mergeCell ref="H64:J71"/>
-    <mergeCell ref="B49:J50"/>
-    <mergeCell ref="F64:G71"/>
-    <mergeCell ref="B64:E71"/>
-    <mergeCell ref="C34:I34"/>
-    <mergeCell ref="C35:I35"/>
-    <mergeCell ref="C36:I36"/>
-    <mergeCell ref="C37:I37"/>
-    <mergeCell ref="C38:I38"/>
-    <mergeCell ref="C39:I39"/>
-    <mergeCell ref="C40:I40"/>
-    <mergeCell ref="C41:I41"/>
-    <mergeCell ref="C42:I42"/>
-    <mergeCell ref="C43:I43"/>
-    <mergeCell ref="C44:I44"/>
-    <mergeCell ref="C45:I45"/>
-    <mergeCell ref="C46:I46"/>
-    <mergeCell ref="C47:I47"/>
-    <mergeCell ref="C48:I48"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="B1:L1"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="J2:L6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="K10:L10"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:C48">
     <cfRule type="expression" dxfId="3" priority="1">
@@ -42356,40 +42364,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="265"/>
-      <c r="C1" s="265"/>
-      <c r="D1" s="265"/>
-      <c r="E1" s="265"/>
-      <c r="F1" s="265"/>
-      <c r="G1" s="265"/>
-      <c r="H1" s="265"/>
-      <c r="I1" s="265"/>
-      <c r="J1" s="265"/>
-      <c r="K1" s="265"/>
-      <c r="L1" s="265"/>
-      <c r="M1" s="265"/>
-      <c r="N1" s="265"/>
-      <c r="O1" s="265"/>
-      <c r="P1" s="265"/>
+      <c r="B1" s="258"/>
+      <c r="C1" s="258"/>
+      <c r="D1" s="258"/>
+      <c r="E1" s="258"/>
+      <c r="F1" s="258"/>
+      <c r="G1" s="258"/>
+      <c r="H1" s="258"/>
+      <c r="I1" s="258"/>
+      <c r="J1" s="258"/>
+      <c r="K1" s="258"/>
+      <c r="L1" s="258"/>
+      <c r="M1" s="258"/>
+      <c r="N1" s="258"/>
+      <c r="O1" s="258"/>
+      <c r="P1" s="258"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="263" t="s">
+      <c r="B2" s="256" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="264"/>
-      <c r="D2" s="264"/>
-      <c r="E2" s="264"/>
-      <c r="F2" s="264"/>
-      <c r="G2" s="264"/>
-      <c r="H2" s="264"/>
-      <c r="I2" s="264"/>
-      <c r="J2" s="264"/>
-      <c r="K2" s="264"/>
-      <c r="L2" s="264"/>
-      <c r="M2" s="264"/>
-      <c r="N2" s="264"/>
-      <c r="O2" s="264"/>
-      <c r="P2" s="264"/>
+      <c r="C2" s="257"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="257"/>
+      <c r="H2" s="257"/>
+      <c r="I2" s="257"/>
+      <c r="J2" s="257"/>
+      <c r="K2" s="257"/>
+      <c r="L2" s="257"/>
+      <c r="M2" s="257"/>
+      <c r="N2" s="257"/>
+      <c r="O2" s="257"/>
+      <c r="P2" s="257"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -42416,16 +42424,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="271" t="s">
+      <c r="I4" s="264" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="271"/>
-      <c r="K4" s="271"/>
-      <c r="L4" s="271"/>
-      <c r="M4" s="271"/>
-      <c r="N4" s="271"/>
-      <c r="O4" s="271"/>
-      <c r="P4" s="271"/>
+      <c r="J4" s="264"/>
+      <c r="K4" s="264"/>
+      <c r="L4" s="264"/>
+      <c r="M4" s="264"/>
+      <c r="N4" s="264"/>
+      <c r="O4" s="264"/>
+      <c r="P4" s="264"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -42439,14 +42447,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="271"/>
-      <c r="J5" s="271"/>
-      <c r="K5" s="271"/>
-      <c r="L5" s="271"/>
-      <c r="M5" s="271"/>
-      <c r="N5" s="271"/>
-      <c r="O5" s="271"/>
-      <c r="P5" s="271"/>
+      <c r="I5" s="264"/>
+      <c r="J5" s="264"/>
+      <c r="K5" s="264"/>
+      <c r="L5" s="264"/>
+      <c r="M5" s="264"/>
+      <c r="N5" s="264"/>
+      <c r="O5" s="264"/>
+      <c r="P5" s="264"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -42581,70 +42589,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="262" t="s">
+      <c r="B12" s="255" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="262" t="s">
+      <c r="C12" s="255" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="262"/>
-      <c r="E12" s="262"/>
-      <c r="F12" s="262" t="s">
+      <c r="D12" s="255"/>
+      <c r="E12" s="255"/>
+      <c r="F12" s="255" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="262" t="s">
+      <c r="G12" s="255" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="262" t="s">
+      <c r="H12" s="255" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="262" t="s">
+      <c r="I12" s="255" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="262" t="s">
+      <c r="J12" s="255" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="262"/>
-      <c r="L12" s="262"/>
-      <c r="M12" s="262"/>
-      <c r="N12" s="262"/>
-      <c r="O12" s="262"/>
-      <c r="P12" s="270" t="s">
+      <c r="K12" s="255"/>
+      <c r="L12" s="255"/>
+      <c r="M12" s="255"/>
+      <c r="N12" s="255"/>
+      <c r="O12" s="255"/>
+      <c r="P12" s="263" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="262"/>
-      <c r="C13" s="262"/>
-      <c r="D13" s="262"/>
-      <c r="E13" s="262"/>
-      <c r="F13" s="262"/>
-      <c r="G13" s="262"/>
-      <c r="H13" s="262"/>
-      <c r="I13" s="262"/>
-      <c r="J13" s="269" t="s">
+      <c r="B13" s="255"/>
+      <c r="C13" s="255"/>
+      <c r="D13" s="255"/>
+      <c r="E13" s="255"/>
+      <c r="F13" s="255"/>
+      <c r="G13" s="255"/>
+      <c r="H13" s="255"/>
+      <c r="I13" s="255"/>
+      <c r="J13" s="262" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="269"/>
-      <c r="L13" s="269" t="s">
+      <c r="K13" s="262"/>
+      <c r="L13" s="262" t="s">
         <v>98</v>
       </c>
-      <c r="M13" s="269"/>
-      <c r="N13" s="269" t="s">
+      <c r="M13" s="262"/>
+      <c r="N13" s="262" t="s">
         <v>99</v>
       </c>
-      <c r="O13" s="269"/>
-      <c r="P13" s="270"/>
+      <c r="O13" s="262"/>
+      <c r="P13" s="263"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="262"/>
-      <c r="C14" s="262"/>
-      <c r="D14" s="262"/>
-      <c r="E14" s="262"/>
-      <c r="F14" s="262"/>
-      <c r="G14" s="262"/>
-      <c r="H14" s="262"/>
-      <c r="I14" s="262"/>
+      <c r="B14" s="255"/>
+      <c r="C14" s="255"/>
+      <c r="D14" s="255"/>
+      <c r="E14" s="255"/>
+      <c r="F14" s="255"/>
+      <c r="G14" s="255"/>
+      <c r="H14" s="255"/>
+      <c r="I14" s="255"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -42663,7 +42671,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="270"/>
+      <c r="P14" s="263"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>

</xml_diff>

<commit_message>
chore(template): update master template with new conditional formatting and layout
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16A6567-9187-4859-A925-DC9A4EF0ABB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2BBF9A4-DD3F-4B10-A4C7-C49C5E69D421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="132">
   <si>
     <t>HARGA SATUAN BAHAN, ALAT DAN UPAH</t>
   </si>
@@ -445,18 +445,6 @@
   <si>
     <t>Unit</t>
   </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>BAB 1</t>
-  </si>
-  <si>
-    <t>Pekerjaan 1</t>
-  </si>
-  <si>
-    <t>m2</t>
-  </si>
 </sst>
 </file>
 
@@ -742,7 +730,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="118">
+  <borders count="117">
     <border>
       <left/>
       <right/>
@@ -1382,19 +1370,6 @@
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="double">
         <color indexed="64"/>
       </right>
       <top style="thin">
@@ -2511,30 +2486,27 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="49" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="53" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="54" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="53" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="61" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="63" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="64" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="63" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="65" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="64" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="66" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="65" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2551,11 +2523,11 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="75" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -2590,37 +2562,37 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="90" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="85" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="106" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="110" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="109" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="98" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="98" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="171" fontId="33" fillId="4" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2635,13 +2607,13 @@
     <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="75" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="78" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2746,16 +2718,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="62" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="61" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="67" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="66" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="60" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="59" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
@@ -2763,11 +2735,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="54" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -2836,13 +2808,13 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2854,13 +2826,13 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2872,20 +2844,20 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="59" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -2897,19 +2869,19 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="73" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="74" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="67" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="68" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="69" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -2921,11 +2893,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="70" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="72" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="71" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -2969,7 +2941,7 @@
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="115" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="114" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -3025,20 +2997,26 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="92" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="31" fillId="4" borderId="93" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="4" borderId="94" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="110" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="4" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3046,11 +3024,8 @@
     <xf numFmtId="0" fontId="32" fillId="4" borderId="105" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="106" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="108" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3058,14 +3033,14 @@
     <xf numFmtId="0" fontId="14" fillId="6" borderId="109" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="110" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="95" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3076,20 +3051,20 @@
     <xf numFmtId="0" fontId="32" fillId="4" borderId="82" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="4" borderId="83" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="105" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="4" borderId="100" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3097,13 +3072,10 @@
     <xf numFmtId="0" fontId="32" fillId="4" borderId="101" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="88" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3127,6 +3099,10 @@
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="111" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="169" fontId="24" fillId="0" borderId="112" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
@@ -3135,14 +3111,10 @@
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="114" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="116" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="115" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="117" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="116" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -3150,8 +3122,12 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="114" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="113" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="24" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
   </cellXfs>
@@ -3161,7 +3137,7 @@
     <cellStyle name="Normal 2 2 3" xfId="2" xr:uid="{25DAB206-4C06-437D-BFFA-FD21FFA5A242}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="27">
     <dxf>
       <font>
         <b/>
@@ -3194,6 +3170,28 @@
         <b/>
         <i val="0"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -4272,40 +4270,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="258"/>
-      <c r="C1" s="258"/>
-      <c r="D1" s="258"/>
-      <c r="E1" s="258"/>
-      <c r="F1" s="258"/>
-      <c r="G1" s="258"/>
-      <c r="H1" s="258"/>
-      <c r="I1" s="258"/>
-      <c r="J1" s="258"/>
-      <c r="K1" s="258"/>
-      <c r="L1" s="258"/>
-      <c r="M1" s="258"/>
-      <c r="N1" s="258"/>
-      <c r="O1" s="258"/>
-      <c r="P1" s="258"/>
+      <c r="B1" s="257"/>
+      <c r="C1" s="257"/>
+      <c r="D1" s="257"/>
+      <c r="E1" s="257"/>
+      <c r="F1" s="257"/>
+      <c r="G1" s="257"/>
+      <c r="H1" s="257"/>
+      <c r="I1" s="257"/>
+      <c r="J1" s="257"/>
+      <c r="K1" s="257"/>
+      <c r="L1" s="257"/>
+      <c r="M1" s="257"/>
+      <c r="N1" s="257"/>
+      <c r="O1" s="257"/>
+      <c r="P1" s="257"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="256" t="s">
+      <c r="B2" s="255" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="257"/>
-      <c r="F2" s="257"/>
-      <c r="G2" s="257"/>
-      <c r="H2" s="257"/>
-      <c r="I2" s="257"/>
-      <c r="J2" s="257"/>
-      <c r="K2" s="257"/>
-      <c r="L2" s="257"/>
-      <c r="M2" s="257"/>
-      <c r="N2" s="257"/>
-      <c r="O2" s="257"/>
-      <c r="P2" s="257"/>
+      <c r="C2" s="256"/>
+      <c r="D2" s="256"/>
+      <c r="E2" s="256"/>
+      <c r="F2" s="256"/>
+      <c r="G2" s="256"/>
+      <c r="H2" s="256"/>
+      <c r="I2" s="256"/>
+      <c r="J2" s="256"/>
+      <c r="K2" s="256"/>
+      <c r="L2" s="256"/>
+      <c r="M2" s="256"/>
+      <c r="N2" s="256"/>
+      <c r="O2" s="256"/>
+      <c r="P2" s="256"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4332,16 +4330,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="264" t="s">
+      <c r="I4" s="263" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="264"/>
-      <c r="K4" s="264"/>
-      <c r="L4" s="264"/>
-      <c r="M4" s="264"/>
-      <c r="N4" s="264"/>
-      <c r="O4" s="264"/>
-      <c r="P4" s="264"/>
+      <c r="J4" s="263"/>
+      <c r="K4" s="263"/>
+      <c r="L4" s="263"/>
+      <c r="M4" s="263"/>
+      <c r="N4" s="263"/>
+      <c r="O4" s="263"/>
+      <c r="P4" s="263"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4355,14 +4353,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="264"/>
-      <c r="J5" s="264"/>
-      <c r="K5" s="264"/>
-      <c r="L5" s="264"/>
-      <c r="M5" s="264"/>
-      <c r="N5" s="264"/>
-      <c r="O5" s="264"/>
-      <c r="P5" s="264"/>
+      <c r="I5" s="263"/>
+      <c r="J5" s="263"/>
+      <c r="K5" s="263"/>
+      <c r="L5" s="263"/>
+      <c r="M5" s="263"/>
+      <c r="N5" s="263"/>
+      <c r="O5" s="263"/>
+      <c r="P5" s="263"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4497,70 +4495,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="255" t="s">
+      <c r="B12" s="254" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="255" t="s">
+      <c r="C12" s="254" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="255"/>
-      <c r="E12" s="255"/>
-      <c r="F12" s="255" t="s">
+      <c r="D12" s="254"/>
+      <c r="E12" s="254"/>
+      <c r="F12" s="254" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="255" t="s">
+      <c r="G12" s="254" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="255" t="s">
+      <c r="H12" s="254" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="255" t="s">
+      <c r="I12" s="254" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="255" t="s">
+      <c r="J12" s="254" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="255"/>
-      <c r="L12" s="255"/>
-      <c r="M12" s="255"/>
-      <c r="N12" s="255"/>
-      <c r="O12" s="255"/>
-      <c r="P12" s="263" t="s">
+      <c r="K12" s="254"/>
+      <c r="L12" s="254"/>
+      <c r="M12" s="254"/>
+      <c r="N12" s="254"/>
+      <c r="O12" s="254"/>
+      <c r="P12" s="262" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="255"/>
-      <c r="C13" s="255"/>
-      <c r="D13" s="255"/>
-      <c r="E13" s="255"/>
-      <c r="F13" s="255"/>
-      <c r="G13" s="255"/>
-      <c r="H13" s="255"/>
-      <c r="I13" s="255"/>
-      <c r="J13" s="262" t="s">
+      <c r="B13" s="254"/>
+      <c r="C13" s="254"/>
+      <c r="D13" s="254"/>
+      <c r="E13" s="254"/>
+      <c r="F13" s="254"/>
+      <c r="G13" s="254"/>
+      <c r="H13" s="254"/>
+      <c r="I13" s="254"/>
+      <c r="J13" s="261" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="262"/>
-      <c r="L13" s="262" t="s">
+      <c r="K13" s="261"/>
+      <c r="L13" s="261" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="262"/>
-      <c r="N13" s="262" t="s">
+      <c r="M13" s="261"/>
+      <c r="N13" s="261" t="s">
         <v>95</v>
       </c>
-      <c r="O13" s="262"/>
-      <c r="P13" s="263"/>
+      <c r="O13" s="261"/>
+      <c r="P13" s="262"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="255"/>
-      <c r="C14" s="255"/>
-      <c r="D14" s="255"/>
-      <c r="E14" s="255"/>
-      <c r="F14" s="255"/>
-      <c r="G14" s="255"/>
-      <c r="H14" s="255"/>
-      <c r="I14" s="255"/>
+      <c r="B14" s="254"/>
+      <c r="C14" s="254"/>
+      <c r="D14" s="254"/>
+      <c r="E14" s="254"/>
+      <c r="F14" s="254"/>
+      <c r="G14" s="254"/>
+      <c r="H14" s="254"/>
+      <c r="I14" s="254"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -4579,7 +4577,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="263"/>
+      <c r="P14" s="262"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -4975,7 +4973,7 @@
     <mergeCell ref="G12:G14"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P51">
-    <cfRule type="expression" dxfId="0" priority="14">
+    <cfRule type="expression" dxfId="4" priority="14">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5002,38 +5000,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="103.2" customHeight="1">
-      <c r="B1" s="257"/>
-      <c r="C1" s="257"/>
-      <c r="D1" s="257"/>
-      <c r="E1" s="257"/>
-      <c r="F1" s="257"/>
-      <c r="G1" s="257"/>
-      <c r="H1" s="257"/>
-      <c r="I1" s="257"/>
-      <c r="J1" s="257"/>
-      <c r="K1" s="257"/>
-      <c r="L1" s="257"/>
-      <c r="M1" s="257"/>
-      <c r="N1" s="257"/>
-      <c r="O1" s="257"/>
+      <c r="B1" s="256"/>
+      <c r="C1" s="256"/>
+      <c r="D1" s="256"/>
+      <c r="E1" s="256"/>
+      <c r="F1" s="256"/>
+      <c r="G1" s="256"/>
+      <c r="H1" s="256"/>
+      <c r="I1" s="256"/>
+      <c r="J1" s="256"/>
+      <c r="K1" s="256"/>
+      <c r="L1" s="256"/>
+      <c r="M1" s="256"/>
+      <c r="N1" s="256"/>
+      <c r="O1" s="256"/>
     </row>
     <row r="2" spans="2:15" ht="22.95" customHeight="1">
-      <c r="B2" s="265" t="s">
+      <c r="B2" s="264" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="265"/>
-      <c r="D2" s="265"/>
-      <c r="E2" s="265"/>
-      <c r="F2" s="265"/>
-      <c r="G2" s="265"/>
-      <c r="H2" s="265"/>
-      <c r="I2" s="265"/>
-      <c r="J2" s="265"/>
-      <c r="K2" s="265"/>
-      <c r="L2" s="265"/>
-      <c r="M2" s="265"/>
-      <c r="N2" s="265"/>
-      <c r="O2" s="265"/>
+      <c r="C2" s="264"/>
+      <c r="D2" s="264"/>
+      <c r="E2" s="264"/>
+      <c r="F2" s="264"/>
+      <c r="G2" s="264"/>
+      <c r="H2" s="264"/>
+      <c r="I2" s="264"/>
+      <c r="J2" s="264"/>
+      <c r="K2" s="264"/>
+      <c r="L2" s="264"/>
+      <c r="M2" s="264"/>
+      <c r="N2" s="264"/>
+      <c r="O2" s="264"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" t="s">
@@ -5085,179 +5083,179 @@
     </row>
     <row r="9" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="11" spans="2:15" s="58" customFormat="1">
-      <c r="B11" s="266" t="s">
+      <c r="B11" s="265" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="266"/>
-      <c r="D11" s="266"/>
-      <c r="E11" s="266"/>
-      <c r="G11" s="266" t="s">
+      <c r="C11" s="265"/>
+      <c r="D11" s="265"/>
+      <c r="E11" s="265"/>
+      <c r="G11" s="265" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="266"/>
-      <c r="I11" s="266"/>
-      <c r="J11" s="266"/>
-      <c r="L11" s="266" t="s">
+      <c r="H11" s="265"/>
+      <c r="I11" s="265"/>
+      <c r="J11" s="265"/>
+      <c r="L11" s="265" t="s">
         <v>105</v>
       </c>
-      <c r="M11" s="266"/>
-      <c r="N11" s="266"/>
-      <c r="O11" s="266"/>
+      <c r="M11" s="265"/>
+      <c r="N11" s="265"/>
+      <c r="O11" s="265"/>
     </row>
     <row r="12" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="13" spans="2:15">
-      <c r="B13" s="257"/>
-      <c r="C13" s="257"/>
-      <c r="D13" s="257"/>
-      <c r="E13" s="257"/>
-      <c r="G13" s="257"/>
-      <c r="H13" s="257"/>
-      <c r="I13" s="257"/>
-      <c r="J13" s="257"/>
-      <c r="L13" s="257"/>
-      <c r="M13" s="257"/>
-      <c r="N13" s="257"/>
-      <c r="O13" s="257"/>
+      <c r="B13" s="256"/>
+      <c r="C13" s="256"/>
+      <c r="D13" s="256"/>
+      <c r="E13" s="256"/>
+      <c r="G13" s="256"/>
+      <c r="H13" s="256"/>
+      <c r="I13" s="256"/>
+      <c r="J13" s="256"/>
+      <c r="L13" s="256"/>
+      <c r="M13" s="256"/>
+      <c r="N13" s="256"/>
+      <c r="O13" s="256"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="257"/>
-      <c r="C14" s="257"/>
-      <c r="D14" s="257"/>
-      <c r="E14" s="257"/>
-      <c r="G14" s="257"/>
-      <c r="H14" s="257"/>
-      <c r="I14" s="257"/>
-      <c r="J14" s="257"/>
-      <c r="L14" s="257"/>
-      <c r="M14" s="257"/>
-      <c r="N14" s="257"/>
-      <c r="O14" s="257"/>
+      <c r="B14" s="256"/>
+      <c r="C14" s="256"/>
+      <c r="D14" s="256"/>
+      <c r="E14" s="256"/>
+      <c r="G14" s="256"/>
+      <c r="H14" s="256"/>
+      <c r="I14" s="256"/>
+      <c r="J14" s="256"/>
+      <c r="L14" s="256"/>
+      <c r="M14" s="256"/>
+      <c r="N14" s="256"/>
+      <c r="O14" s="256"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="257"/>
-      <c r="C15" s="257"/>
-      <c r="D15" s="257"/>
-      <c r="E15" s="257"/>
-      <c r="G15" s="257"/>
-      <c r="H15" s="257"/>
-      <c r="I15" s="257"/>
-      <c r="J15" s="257"/>
-      <c r="L15" s="257"/>
-      <c r="M15" s="257"/>
-      <c r="N15" s="257"/>
-      <c r="O15" s="257"/>
+      <c r="B15" s="256"/>
+      <c r="C15" s="256"/>
+      <c r="D15" s="256"/>
+      <c r="E15" s="256"/>
+      <c r="G15" s="256"/>
+      <c r="H15" s="256"/>
+      <c r="I15" s="256"/>
+      <c r="J15" s="256"/>
+      <c r="L15" s="256"/>
+      <c r="M15" s="256"/>
+      <c r="N15" s="256"/>
+      <c r="O15" s="256"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="257"/>
-      <c r="C16" s="257"/>
-      <c r="D16" s="257"/>
-      <c r="E16" s="257"/>
-      <c r="G16" s="257"/>
-      <c r="H16" s="257"/>
-      <c r="I16" s="257"/>
-      <c r="J16" s="257"/>
-      <c r="L16" s="257"/>
-      <c r="M16" s="257"/>
-      <c r="N16" s="257"/>
-      <c r="O16" s="257"/>
+      <c r="B16" s="256"/>
+      <c r="C16" s="256"/>
+      <c r="D16" s="256"/>
+      <c r="E16" s="256"/>
+      <c r="G16" s="256"/>
+      <c r="H16" s="256"/>
+      <c r="I16" s="256"/>
+      <c r="J16" s="256"/>
+      <c r="L16" s="256"/>
+      <c r="M16" s="256"/>
+      <c r="N16" s="256"/>
+      <c r="O16" s="256"/>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="257"/>
-      <c r="C17" s="257"/>
-      <c r="D17" s="257"/>
-      <c r="E17" s="257"/>
-      <c r="G17" s="257"/>
-      <c r="H17" s="257"/>
-      <c r="I17" s="257"/>
-      <c r="J17" s="257"/>
-      <c r="L17" s="257"/>
-      <c r="M17" s="257"/>
-      <c r="N17" s="257"/>
-      <c r="O17" s="257"/>
+      <c r="B17" s="256"/>
+      <c r="C17" s="256"/>
+      <c r="D17" s="256"/>
+      <c r="E17" s="256"/>
+      <c r="G17" s="256"/>
+      <c r="H17" s="256"/>
+      <c r="I17" s="256"/>
+      <c r="J17" s="256"/>
+      <c r="L17" s="256"/>
+      <c r="M17" s="256"/>
+      <c r="N17" s="256"/>
+      <c r="O17" s="256"/>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="257"/>
-      <c r="C18" s="257"/>
-      <c r="D18" s="257"/>
-      <c r="E18" s="257"/>
-      <c r="G18" s="257"/>
-      <c r="H18" s="257"/>
-      <c r="I18" s="257"/>
-      <c r="J18" s="257"/>
-      <c r="L18" s="257"/>
-      <c r="M18" s="257"/>
-      <c r="N18" s="257"/>
-      <c r="O18" s="257"/>
+      <c r="B18" s="256"/>
+      <c r="C18" s="256"/>
+      <c r="D18" s="256"/>
+      <c r="E18" s="256"/>
+      <c r="G18" s="256"/>
+      <c r="H18" s="256"/>
+      <c r="I18" s="256"/>
+      <c r="J18" s="256"/>
+      <c r="L18" s="256"/>
+      <c r="M18" s="256"/>
+      <c r="N18" s="256"/>
+      <c r="O18" s="256"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="B19" s="257"/>
-      <c r="C19" s="257"/>
-      <c r="D19" s="257"/>
-      <c r="E19" s="257"/>
-      <c r="G19" s="257"/>
-      <c r="H19" s="257"/>
-      <c r="I19" s="257"/>
-      <c r="J19" s="257"/>
-      <c r="L19" s="257"/>
-      <c r="M19" s="257"/>
-      <c r="N19" s="257"/>
-      <c r="O19" s="257"/>
+      <c r="B19" s="256"/>
+      <c r="C19" s="256"/>
+      <c r="D19" s="256"/>
+      <c r="E19" s="256"/>
+      <c r="G19" s="256"/>
+      <c r="H19" s="256"/>
+      <c r="I19" s="256"/>
+      <c r="J19" s="256"/>
+      <c r="L19" s="256"/>
+      <c r="M19" s="256"/>
+      <c r="N19" s="256"/>
+      <c r="O19" s="256"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="B20" s="257"/>
-      <c r="C20" s="257"/>
-      <c r="D20" s="257"/>
-      <c r="E20" s="257"/>
-      <c r="G20" s="257"/>
-      <c r="H20" s="257"/>
-      <c r="I20" s="257"/>
-      <c r="J20" s="257"/>
-      <c r="L20" s="257"/>
-      <c r="M20" s="257"/>
-      <c r="N20" s="257"/>
-      <c r="O20" s="257"/>
+      <c r="B20" s="256"/>
+      <c r="C20" s="256"/>
+      <c r="D20" s="256"/>
+      <c r="E20" s="256"/>
+      <c r="G20" s="256"/>
+      <c r="H20" s="256"/>
+      <c r="I20" s="256"/>
+      <c r="J20" s="256"/>
+      <c r="L20" s="256"/>
+      <c r="M20" s="256"/>
+      <c r="N20" s="256"/>
+      <c r="O20" s="256"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="B21" s="257"/>
-      <c r="C21" s="257"/>
-      <c r="D21" s="257"/>
-      <c r="E21" s="257"/>
-      <c r="G21" s="257"/>
-      <c r="H21" s="257"/>
-      <c r="I21" s="257"/>
-      <c r="J21" s="257"/>
-      <c r="L21" s="257"/>
-      <c r="M21" s="257"/>
-      <c r="N21" s="257"/>
-      <c r="O21" s="257"/>
+      <c r="B21" s="256"/>
+      <c r="C21" s="256"/>
+      <c r="D21" s="256"/>
+      <c r="E21" s="256"/>
+      <c r="G21" s="256"/>
+      <c r="H21" s="256"/>
+      <c r="I21" s="256"/>
+      <c r="J21" s="256"/>
+      <c r="L21" s="256"/>
+      <c r="M21" s="256"/>
+      <c r="N21" s="256"/>
+      <c r="O21" s="256"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="B22" s="257"/>
-      <c r="C22" s="257"/>
-      <c r="D22" s="257"/>
-      <c r="E22" s="257"/>
-      <c r="G22" s="257"/>
-      <c r="H22" s="257"/>
-      <c r="I22" s="257"/>
-      <c r="J22" s="257"/>
-      <c r="L22" s="257"/>
-      <c r="M22" s="257"/>
-      <c r="N22" s="257"/>
-      <c r="O22" s="257"/>
+      <c r="B22" s="256"/>
+      <c r="C22" s="256"/>
+      <c r="D22" s="256"/>
+      <c r="E22" s="256"/>
+      <c r="G22" s="256"/>
+      <c r="H22" s="256"/>
+      <c r="I22" s="256"/>
+      <c r="J22" s="256"/>
+      <c r="L22" s="256"/>
+      <c r="M22" s="256"/>
+      <c r="N22" s="256"/>
+      <c r="O22" s="256"/>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="257"/>
-      <c r="C23" s="257"/>
-      <c r="D23" s="257"/>
-      <c r="E23" s="257"/>
-      <c r="G23" s="257"/>
-      <c r="H23" s="257"/>
-      <c r="I23" s="257"/>
-      <c r="J23" s="257"/>
-      <c r="L23" s="257"/>
-      <c r="M23" s="257"/>
-      <c r="N23" s="257"/>
-      <c r="O23" s="257"/>
+      <c r="B23" s="256"/>
+      <c r="C23" s="256"/>
+      <c r="D23" s="256"/>
+      <c r="E23" s="256"/>
+      <c r="G23" s="256"/>
+      <c r="H23" s="256"/>
+      <c r="I23" s="256"/>
+      <c r="J23" s="256"/>
+      <c r="L23" s="256"/>
+      <c r="M23" s="256"/>
+      <c r="N23" s="256"/>
+      <c r="O23" s="256"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5291,330 +5289,330 @@
   <sheetData>
     <row r="1" spans="2:29" ht="4.8" customHeight="1" thickBot="1"/>
     <row r="2" spans="2:29" ht="19.95" customHeight="1" thickBot="1">
-      <c r="B2" s="267" t="s">
+      <c r="B2" s="266" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="268"/>
-      <c r="D2" s="268"/>
-      <c r="E2" s="268"/>
-      <c r="F2" s="268"/>
-      <c r="G2" s="268"/>
-      <c r="H2" s="268"/>
-      <c r="I2" s="268"/>
-      <c r="J2" s="268"/>
-      <c r="K2" s="268"/>
-      <c r="L2" s="268"/>
-      <c r="M2" s="268"/>
-      <c r="N2" s="268"/>
-      <c r="O2" s="268"/>
-      <c r="P2" s="268"/>
-      <c r="Q2" s="268"/>
-      <c r="R2" s="268"/>
-      <c r="S2" s="268"/>
-      <c r="T2" s="268"/>
-      <c r="U2" s="268"/>
-      <c r="V2" s="268"/>
-      <c r="W2" s="268"/>
-      <c r="X2" s="268"/>
-      <c r="Y2" s="268"/>
-      <c r="Z2" s="268"/>
-      <c r="AA2" s="268"/>
-      <c r="AB2" s="269"/>
-      <c r="AC2" s="141"/>
+      <c r="C2" s="267"/>
+      <c r="D2" s="267"/>
+      <c r="E2" s="267"/>
+      <c r="F2" s="267"/>
+      <c r="G2" s="267"/>
+      <c r="H2" s="267"/>
+      <c r="I2" s="267"/>
+      <c r="J2" s="267"/>
+      <c r="K2" s="267"/>
+      <c r="L2" s="267"/>
+      <c r="M2" s="267"/>
+      <c r="N2" s="267"/>
+      <c r="O2" s="267"/>
+      <c r="P2" s="267"/>
+      <c r="Q2" s="267"/>
+      <c r="R2" s="267"/>
+      <c r="S2" s="267"/>
+      <c r="T2" s="267"/>
+      <c r="U2" s="267"/>
+      <c r="V2" s="267"/>
+      <c r="W2" s="267"/>
+      <c r="X2" s="267"/>
+      <c r="Y2" s="267"/>
+      <c r="Z2" s="267"/>
+      <c r="AA2" s="267"/>
+      <c r="AB2" s="268"/>
+      <c r="AC2" s="140"/>
     </row>
     <row r="3" spans="2:29" ht="15" customHeight="1">
-      <c r="B3" s="140"/>
-      <c r="AB3" s="135"/>
+      <c r="B3" s="139"/>
+      <c r="AB3" s="134"/>
     </row>
     <row r="4" spans="2:29" ht="15" customHeight="1">
-      <c r="B4" s="134" t="s">
+      <c r="B4" s="133" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="136" t="s">
+      <c r="D4" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="AB4" s="135"/>
+      <c r="AB4" s="134"/>
     </row>
     <row r="5" spans="2:29" ht="15" customHeight="1">
-      <c r="B5" s="134" t="s">
+      <c r="B5" s="133" t="s">
         <v>108</v>
       </c>
-      <c r="D5" s="136" t="s">
+      <c r="D5" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="AB5" s="135"/>
+      <c r="AB5" s="134"/>
     </row>
     <row r="6" spans="2:29" ht="15" customHeight="1">
-      <c r="B6" s="134" t="s">
+      <c r="B6" s="133" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="136" t="s">
+      <c r="D6" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="AB6" s="135"/>
+      <c r="AB6" s="134"/>
     </row>
     <row r="7" spans="2:29" ht="15" customHeight="1">
-      <c r="B7" s="134" t="s">
+      <c r="B7" s="133" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="136" t="s">
+      <c r="D7" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="AB7" s="135"/>
+      <c r="AB7" s="134"/>
     </row>
     <row r="8" spans="2:29" ht="15" customHeight="1">
-      <c r="B8" s="134" t="s">
+      <c r="B8" s="133" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="136" t="s">
+      <c r="D8" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="AB8" s="135"/>
+      <c r="AB8" s="134"/>
     </row>
     <row r="9" spans="2:29" ht="15" customHeight="1">
-      <c r="B9" s="134" t="s">
+      <c r="B9" s="133" t="s">
         <v>110</v>
       </c>
-      <c r="D9" s="136" t="s">
+      <c r="D9" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="AB9" s="135"/>
+      <c r="AB9" s="134"/>
     </row>
     <row r="10" spans="2:29" ht="15" customHeight="1">
-      <c r="B10" s="134" t="s">
+      <c r="B10" s="133" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="136" t="s">
+      <c r="D10" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="AB10" s="135"/>
+      <c r="AB10" s="134"/>
     </row>
     <row r="11" spans="2:29" ht="15" customHeight="1" thickBot="1">
-      <c r="B11" s="137"/>
-      <c r="C11" s="138"/>
-      <c r="D11" s="138"/>
-      <c r="E11" s="138"/>
-      <c r="F11" s="138"/>
-      <c r="G11" s="138"/>
-      <c r="H11" s="138"/>
-      <c r="I11" s="138"/>
-      <c r="J11" s="138"/>
-      <c r="K11" s="138"/>
-      <c r="L11" s="138"/>
-      <c r="M11" s="138"/>
-      <c r="N11" s="138"/>
-      <c r="O11" s="138"/>
-      <c r="P11" s="138"/>
-      <c r="Q11" s="138"/>
-      <c r="R11" s="138"/>
-      <c r="S11" s="138"/>
-      <c r="T11" s="138"/>
-      <c r="U11" s="138"/>
-      <c r="V11" s="138"/>
-      <c r="W11" s="138"/>
-      <c r="X11" s="138"/>
-      <c r="Y11" s="138"/>
-      <c r="Z11" s="138"/>
-      <c r="AA11" s="138"/>
-      <c r="AB11" s="139"/>
+      <c r="B11" s="136"/>
+      <c r="C11" s="137"/>
+      <c r="D11" s="137"/>
+      <c r="E11" s="137"/>
+      <c r="F11" s="137"/>
+      <c r="G11" s="137"/>
+      <c r="H11" s="137"/>
+      <c r="I11" s="137"/>
+      <c r="J11" s="137"/>
+      <c r="K11" s="137"/>
+      <c r="L11" s="137"/>
+      <c r="M11" s="137"/>
+      <c r="N11" s="137"/>
+      <c r="O11" s="137"/>
+      <c r="P11" s="137"/>
+      <c r="Q11" s="137"/>
+      <c r="R11" s="137"/>
+      <c r="S11" s="137"/>
+      <c r="T11" s="137"/>
+      <c r="U11" s="137"/>
+      <c r="V11" s="137"/>
+      <c r="W11" s="137"/>
+      <c r="X11" s="137"/>
+      <c r="Y11" s="137"/>
+      <c r="Z11" s="137"/>
+      <c r="AA11" s="137"/>
+      <c r="AB11" s="138"/>
     </row>
     <row r="12" spans="2:29" ht="15" customHeight="1">
-      <c r="B12" s="279" t="s">
+      <c r="B12" s="278" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="281" t="s">
+      <c r="C12" s="280" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="282"/>
-      <c r="E12" s="282"/>
-      <c r="F12" s="282"/>
-      <c r="G12" s="282"/>
-      <c r="H12" s="282"/>
-      <c r="I12" s="282"/>
-      <c r="J12" s="282"/>
-      <c r="K12" s="282"/>
-      <c r="L12" s="283"/>
-      <c r="M12" s="287" t="s">
+      <c r="D12" s="281"/>
+      <c r="E12" s="281"/>
+      <c r="F12" s="281"/>
+      <c r="G12" s="281"/>
+      <c r="H12" s="281"/>
+      <c r="I12" s="281"/>
+      <c r="J12" s="281"/>
+      <c r="K12" s="281"/>
+      <c r="L12" s="282"/>
+      <c r="M12" s="286" t="s">
         <v>113</v>
       </c>
-      <c r="N12" s="287" t="s">
+      <c r="N12" s="286" t="s">
         <v>34</v>
       </c>
-      <c r="O12" s="292" t="s">
+      <c r="O12" s="291" t="s">
         <v>114</v>
       </c>
-      <c r="P12" s="292"/>
-      <c r="Q12" s="292"/>
-      <c r="R12" s="292"/>
-      <c r="S12" s="292"/>
-      <c r="T12" s="292"/>
-      <c r="U12" s="292"/>
-      <c r="V12" s="292"/>
-      <c r="W12" s="292"/>
-      <c r="X12" s="292"/>
-      <c r="Y12" s="292"/>
-      <c r="Z12" s="292"/>
-      <c r="AA12" s="292"/>
-      <c r="AB12" s="293"/>
+      <c r="P12" s="291"/>
+      <c r="Q12" s="291"/>
+      <c r="R12" s="291"/>
+      <c r="S12" s="291"/>
+      <c r="T12" s="291"/>
+      <c r="U12" s="291"/>
+      <c r="V12" s="291"/>
+      <c r="W12" s="291"/>
+      <c r="X12" s="291"/>
+      <c r="Y12" s="291"/>
+      <c r="Z12" s="291"/>
+      <c r="AA12" s="291"/>
+      <c r="AB12" s="292"/>
     </row>
     <row r="13" spans="2:29" ht="15" customHeight="1">
-      <c r="B13" s="280"/>
-      <c r="C13" s="284"/>
-      <c r="D13" s="285"/>
-      <c r="E13" s="285"/>
-      <c r="F13" s="285"/>
-      <c r="G13" s="285"/>
-      <c r="H13" s="285"/>
-      <c r="I13" s="285"/>
-      <c r="J13" s="285"/>
-      <c r="K13" s="285"/>
-      <c r="L13" s="286"/>
-      <c r="M13" s="288"/>
-      <c r="N13" s="288"/>
-      <c r="O13" s="289" t="s">
+      <c r="B13" s="279"/>
+      <c r="C13" s="283"/>
+      <c r="D13" s="284"/>
+      <c r="E13" s="284"/>
+      <c r="F13" s="284"/>
+      <c r="G13" s="284"/>
+      <c r="H13" s="284"/>
+      <c r="I13" s="284"/>
+      <c r="J13" s="284"/>
+      <c r="K13" s="284"/>
+      <c r="L13" s="285"/>
+      <c r="M13" s="287"/>
+      <c r="N13" s="287"/>
+      <c r="O13" s="288" t="s">
         <v>115</v>
       </c>
-      <c r="P13" s="290"/>
-      <c r="Q13" s="291"/>
-      <c r="R13" s="289" t="s">
+      <c r="P13" s="289"/>
+      <c r="Q13" s="290"/>
+      <c r="R13" s="288" t="s">
         <v>116</v>
       </c>
-      <c r="S13" s="290"/>
-      <c r="T13" s="291"/>
-      <c r="U13" s="289" t="s">
+      <c r="S13" s="289"/>
+      <c r="T13" s="290"/>
+      <c r="U13" s="288" t="s">
         <v>117</v>
       </c>
-      <c r="V13" s="290"/>
-      <c r="W13" s="291"/>
-      <c r="X13" s="270" t="s">
+      <c r="V13" s="289"/>
+      <c r="W13" s="290"/>
+      <c r="X13" s="269" t="s">
         <v>118</v>
       </c>
-      <c r="Y13" s="146" t="s">
+      <c r="Y13" s="145" t="s">
         <v>119</v>
       </c>
-      <c r="Z13" s="147" t="s">
+      <c r="Z13" s="146" t="s">
         <v>119</v>
       </c>
-      <c r="AA13" s="272" t="s">
+      <c r="AA13" s="271" t="s">
         <v>120</v>
       </c>
-      <c r="AB13" s="274" t="s">
+      <c r="AB13" s="273" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="14" spans="2:29" ht="15" customHeight="1">
-      <c r="B14" s="280"/>
-      <c r="C14" s="284"/>
-      <c r="D14" s="285"/>
-      <c r="E14" s="285"/>
-      <c r="F14" s="285"/>
-      <c r="G14" s="285"/>
-      <c r="H14" s="285"/>
-      <c r="I14" s="285"/>
-      <c r="J14" s="285"/>
-      <c r="K14" s="285"/>
-      <c r="L14" s="286"/>
-      <c r="M14" s="271"/>
-      <c r="N14" s="271"/>
-      <c r="O14" s="148" t="s">
+      <c r="B14" s="279"/>
+      <c r="C14" s="283"/>
+      <c r="D14" s="284"/>
+      <c r="E14" s="284"/>
+      <c r="F14" s="284"/>
+      <c r="G14" s="284"/>
+      <c r="H14" s="284"/>
+      <c r="I14" s="284"/>
+      <c r="J14" s="284"/>
+      <c r="K14" s="284"/>
+      <c r="L14" s="285"/>
+      <c r="M14" s="270"/>
+      <c r="N14" s="270"/>
+      <c r="O14" s="147" t="s">
         <v>122</v>
       </c>
-      <c r="P14" s="148" t="s">
+      <c r="P14" s="147" t="s">
         <v>123</v>
       </c>
-      <c r="Q14" s="148" t="s">
+      <c r="Q14" s="147" t="s">
         <v>124</v>
       </c>
-      <c r="R14" s="148" t="s">
+      <c r="R14" s="147" t="s">
         <v>125</v>
       </c>
-      <c r="S14" s="148" t="s">
+      <c r="S14" s="147" t="s">
         <v>126</v>
       </c>
-      <c r="T14" s="148" t="s">
+      <c r="T14" s="147" t="s">
         <v>124</v>
       </c>
-      <c r="U14" s="148" t="s">
+      <c r="U14" s="147" t="s">
         <v>127</v>
       </c>
-      <c r="V14" s="148" t="s">
+      <c r="V14" s="147" t="s">
         <v>128</v>
       </c>
-      <c r="W14" s="148" t="s">
+      <c r="W14" s="147" t="s">
         <v>129</v>
       </c>
-      <c r="X14" s="271"/>
-      <c r="Y14" s="146" t="s">
+      <c r="X14" s="270"/>
+      <c r="Y14" s="145" t="s">
         <v>130</v>
       </c>
-      <c r="Z14" s="148" t="s">
+      <c r="Z14" s="147" t="s">
         <v>131</v>
       </c>
-      <c r="AA14" s="273"/>
-      <c r="AB14" s="275"/>
+      <c r="AA14" s="272"/>
+      <c r="AB14" s="274"/>
     </row>
     <row r="15" spans="2:29" ht="15" customHeight="1" thickBot="1">
-      <c r="B15" s="142">
+      <c r="B15" s="141">
         <v>1</v>
       </c>
-      <c r="C15" s="276">
+      <c r="C15" s="275">
         <v>2</v>
       </c>
-      <c r="D15" s="277"/>
-      <c r="E15" s="277"/>
-      <c r="F15" s="277"/>
-      <c r="G15" s="277"/>
-      <c r="H15" s="277"/>
-      <c r="I15" s="277"/>
-      <c r="J15" s="277"/>
-      <c r="K15" s="277"/>
-      <c r="L15" s="278"/>
-      <c r="M15" s="143">
+      <c r="D15" s="276"/>
+      <c r="E15" s="276"/>
+      <c r="F15" s="276"/>
+      <c r="G15" s="276"/>
+      <c r="H15" s="276"/>
+      <c r="I15" s="276"/>
+      <c r="J15" s="276"/>
+      <c r="K15" s="276"/>
+      <c r="L15" s="277"/>
+      <c r="M15" s="142">
         <v>3</v>
       </c>
-      <c r="N15" s="143">
+      <c r="N15" s="142">
         <v>4</v>
       </c>
-      <c r="O15" s="144">
+      <c r="O15" s="143">
         <v>5</v>
       </c>
-      <c r="P15" s="144">
+      <c r="P15" s="143">
         <v>6</v>
       </c>
-      <c r="Q15" s="144">
+      <c r="Q15" s="143">
         <v>7</v>
       </c>
-      <c r="R15" s="144">
+      <c r="R15" s="143">
         <v>8</v>
       </c>
-      <c r="S15" s="144">
+      <c r="S15" s="143">
         <v>9</v>
       </c>
-      <c r="T15" s="144">
+      <c r="T15" s="143">
         <v>10</v>
       </c>
-      <c r="U15" s="144">
+      <c r="U15" s="143">
         <v>11</v>
       </c>
-      <c r="V15" s="144">
+      <c r="V15" s="143">
         <v>12</v>
       </c>
-      <c r="W15" s="144">
+      <c r="W15" s="143">
         <v>13</v>
       </c>
-      <c r="X15" s="144">
+      <c r="X15" s="143">
         <v>14</v>
       </c>
-      <c r="Y15" s="144">
+      <c r="Y15" s="143">
         <v>15</v>
       </c>
-      <c r="Z15" s="144">
+      <c r="Z15" s="143">
         <v>16</v>
       </c>
-      <c r="AA15" s="144">
+      <c r="AA15" s="143">
         <v>17</v>
       </c>
-      <c r="AB15" s="145">
+      <c r="AB15" s="144">
         <v>18</v>
       </c>
     </row>
@@ -5658,38 +5656,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="254"/>
-      <c r="C1" s="254"/>
-      <c r="D1" s="254"/>
-      <c r="E1" s="254"/>
-      <c r="F1" s="254"/>
-      <c r="G1" s="254"/>
-      <c r="H1" s="254"/>
-      <c r="I1" s="254"/>
+      <c r="B1" s="253"/>
+      <c r="C1" s="253"/>
+      <c r="D1" s="253"/>
+      <c r="E1" s="253"/>
+      <c r="F1" s="253"/>
+      <c r="G1" s="253"/>
+      <c r="H1" s="253"/>
+      <c r="I1" s="253"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="251" t="s">
+      <c r="B2" s="250" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="251"/>
-      <c r="D2" s="251"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="251"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="251"/>
-      <c r="I2" s="251"/>
+      <c r="C2" s="250"/>
+      <c r="D2" s="250"/>
+      <c r="E2" s="250"/>
+      <c r="F2" s="250"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="250"/>
+      <c r="I2" s="250"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="252" t="s">
+      <c r="B3" s="251" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="252"/>
-      <c r="D3" s="252"/>
-      <c r="E3" s="252"/>
-      <c r="F3" s="252"/>
-      <c r="G3" s="252"/>
-      <c r="H3" s="252"/>
-      <c r="I3" s="252"/>
+      <c r="C3" s="251"/>
+      <c r="D3" s="251"/>
+      <c r="E3" s="251"/>
+      <c r="F3" s="251"/>
+      <c r="G3" s="251"/>
+      <c r="H3" s="251"/>
+      <c r="I3" s="251"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -5697,10 +5695,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="253" t="s">
+      <c r="C5" s="252" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="253"/>
+      <c r="D5" s="252"/>
       <c r="E5" s="11" t="s">
         <v>38</v>
       </c>
@@ -14054,7 +14052,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="24" priority="2">
+    <cfRule type="expression" dxfId="26" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14087,63 +14085,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="254"/>
-      <c r="C1" s="254"/>
-      <c r="D1" s="254"/>
-      <c r="E1" s="254"/>
-      <c r="F1" s="254"/>
-      <c r="G1" s="254"/>
-      <c r="H1" s="254"/>
-      <c r="I1" s="254"/>
-      <c r="J1" s="254"/>
-      <c r="K1" s="254"/>
-      <c r="L1" s="254"/>
-      <c r="M1" s="254"/>
-      <c r="N1" s="254"/>
+      <c r="B1" s="253"/>
+      <c r="C1" s="253"/>
+      <c r="D1" s="253"/>
+      <c r="E1" s="253"/>
+      <c r="F1" s="253"/>
+      <c r="G1" s="253"/>
+      <c r="H1" s="253"/>
+      <c r="I1" s="253"/>
+      <c r="J1" s="253"/>
+      <c r="K1" s="253"/>
+      <c r="L1" s="253"/>
+      <c r="M1" s="253"/>
+      <c r="N1" s="253"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="251" t="s">
+      <c r="B2" s="250" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="251"/>
-      <c r="D2" s="251"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="251"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="251"/>
-      <c r="I2" s="251"/>
-      <c r="J2" s="251"/>
-      <c r="K2" s="251"/>
-      <c r="L2" s="251"/>
-      <c r="M2" s="251"/>
-      <c r="N2" s="251"/>
+      <c r="C2" s="250"/>
+      <c r="D2" s="250"/>
+      <c r="E2" s="250"/>
+      <c r="F2" s="250"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="250"/>
+      <c r="I2" s="250"/>
+      <c r="J2" s="250"/>
+      <c r="K2" s="250"/>
+      <c r="L2" s="250"/>
+      <c r="M2" s="250"/>
+      <c r="N2" s="250"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="252" t="s">
+      <c r="B3" s="251" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="252"/>
-      <c r="D3" s="252"/>
-      <c r="E3" s="252"/>
-      <c r="F3" s="252"/>
-      <c r="G3" s="252"/>
-      <c r="H3" s="252"/>
-      <c r="I3" s="252"/>
-      <c r="J3" s="252"/>
-      <c r="K3" s="252"/>
-      <c r="L3" s="252"/>
-      <c r="M3" s="252"/>
-      <c r="N3" s="252"/>
+      <c r="C3" s="251"/>
+      <c r="D3" s="251"/>
+      <c r="E3" s="251"/>
+      <c r="F3" s="251"/>
+      <c r="G3" s="251"/>
+      <c r="H3" s="251"/>
+      <c r="I3" s="251"/>
+      <c r="J3" s="251"/>
+      <c r="K3" s="251"/>
+      <c r="L3" s="251"/>
+      <c r="M3" s="251"/>
+      <c r="N3" s="251"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="255" t="s">
+      <c r="C5" s="254" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="255"/>
+      <c r="D5" s="254"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -16304,23 +16302,23 @@
     <mergeCell ref="B1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:N16997">
-    <cfRule type="expression" dxfId="23" priority="1">
+    <cfRule type="expression" dxfId="25" priority="1">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="2">
+    <cfRule type="expression" dxfId="24" priority="2">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="5">
+    <cfRule type="expression" dxfId="23" priority="5">
       <formula>AND($B6="",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H16997">
-    <cfRule type="expression" dxfId="20" priority="9">
+    <cfRule type="expression" dxfId="22" priority="9">
       <formula>IF(G6&lt;&gt;"", NOT(AND(OR(LEFT($E6,2)="L.", LEFT($E6,2)="A.", LEFT($E6,2)="B.", LEFT($E6,2)="M."), $H6&lt;&gt;"", $E6&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:K16997">
-    <cfRule type="notContainsBlanks" dxfId="19" priority="8">
+    <cfRule type="notContainsBlanks" dxfId="21" priority="8">
       <formula>LEN(TRIM(H6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16347,35 +16345,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="254"/>
-      <c r="C1" s="254"/>
-      <c r="D1" s="254"/>
-      <c r="E1" s="254"/>
-      <c r="F1" s="254"/>
-      <c r="G1" s="254"/>
-      <c r="H1" s="254"/>
+      <c r="B1" s="253"/>
+      <c r="C1" s="253"/>
+      <c r="D1" s="253"/>
+      <c r="E1" s="253"/>
+      <c r="F1" s="253"/>
+      <c r="G1" s="253"/>
+      <c r="H1" s="253"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="251" t="s">
+      <c r="B2" s="250" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="251"/>
-      <c r="D2" s="251"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="251"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="251"/>
+      <c r="C2" s="250"/>
+      <c r="D2" s="250"/>
+      <c r="E2" s="250"/>
+      <c r="F2" s="250"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="250"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="252" t="s">
+      <c r="B3" s="251" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="252"/>
-      <c r="D3" s="252"/>
-      <c r="E3" s="252"/>
-      <c r="F3" s="252"/>
-      <c r="G3" s="252"/>
-      <c r="H3" s="252"/>
+      <c r="C3" s="251"/>
+      <c r="D3" s="251"/>
+      <c r="E3" s="251"/>
+      <c r="F3" s="251"/>
+      <c r="G3" s="251"/>
+      <c r="H3" s="251"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -40423,18 +40421,18 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B995 E6:H995">
-    <cfRule type="expression" dxfId="18" priority="7">
+    <cfRule type="expression" dxfId="20" priority="7">
       <formula>$J6=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:H995">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="19" priority="1">
       <formula>AND(LEN($B6)=1,$C6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="2">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>AND($C6="",$B6&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="17" priority="3">
       <formula>AND($B6&lt;&gt;"",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -40469,30 +40467,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="258"/>
-      <c r="C1" s="258"/>
-      <c r="D1" s="258"/>
-      <c r="E1" s="258"/>
-      <c r="F1" s="258"/>
-      <c r="G1" s="258"/>
-      <c r="H1" s="258"/>
-      <c r="I1" s="258"/>
-      <c r="J1" s="258"/>
-      <c r="K1" s="258"/>
+      <c r="B1" s="257"/>
+      <c r="C1" s="257"/>
+      <c r="D1" s="257"/>
+      <c r="E1" s="257"/>
+      <c r="F1" s="257"/>
+      <c r="G1" s="257"/>
+      <c r="H1" s="257"/>
+      <c r="I1" s="257"/>
+      <c r="J1" s="257"/>
+      <c r="K1" s="257"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="256" t="s">
+      <c r="B2" s="255" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="257"/>
-      <c r="F2" s="257"/>
-      <c r="G2" s="257"/>
-      <c r="H2" s="257"/>
-      <c r="I2" s="257"/>
-      <c r="J2" s="257"/>
-      <c r="K2" s="257"/>
+      <c r="C2" s="256"/>
+      <c r="D2" s="256"/>
+      <c r="E2" s="256"/>
+      <c r="F2" s="256"/>
+      <c r="G2" s="256"/>
+      <c r="H2" s="256"/>
+      <c r="I2" s="256"/>
+      <c r="J2" s="256"/>
+      <c r="K2" s="256"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40612,11 +40610,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="255" t="s">
+      <c r="C11" s="254" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="255"/>
-      <c r="E11" s="255"/>
+      <c r="D11" s="254"/>
+      <c r="E11" s="254"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -40672,26 +40670,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="111.6" customHeight="1">
-      <c r="B1" s="258"/>
-      <c r="C1" s="258"/>
-      <c r="D1" s="258"/>
-      <c r="E1" s="258"/>
-      <c r="F1" s="258"/>
-      <c r="G1" s="258"/>
-      <c r="H1" s="258"/>
-      <c r="I1" s="258"/>
+      <c r="B1" s="257"/>
+      <c r="C1" s="257"/>
+      <c r="D1" s="257"/>
+      <c r="E1" s="257"/>
+      <c r="F1" s="257"/>
+      <c r="G1" s="257"/>
+      <c r="H1" s="257"/>
+      <c r="I1" s="257"/>
     </row>
     <row r="2" spans="2:9" ht="22.95" customHeight="1">
-      <c r="B2" s="256" t="s">
+      <c r="B2" s="255" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="257"/>
-      <c r="F2" s="257"/>
-      <c r="G2" s="257"/>
-      <c r="H2" s="257"/>
-      <c r="I2" s="257"/>
+      <c r="C2" s="256"/>
+      <c r="D2" s="256"/>
+      <c r="E2" s="256"/>
+      <c r="F2" s="256"/>
+      <c r="G2" s="256"/>
+      <c r="H2" s="256"/>
+      <c r="I2" s="256"/>
     </row>
     <row r="3" spans="2:9" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40801,12 +40799,12 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="255" t="s">
+      <c r="C11" s="254" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="255"/>
-      <c r="E11" s="255"/>
-      <c r="F11" s="255"/>
+      <c r="D11" s="254"/>
+      <c r="E11" s="254"/>
+      <c r="F11" s="254"/>
       <c r="G11" s="40" t="s">
         <v>29</v>
       </c>
@@ -40844,58 +40842,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="258"/>
-      <c r="C1" s="258"/>
-      <c r="D1" s="258"/>
-      <c r="E1" s="258"/>
-      <c r="F1" s="258"/>
+      <c r="B1" s="257"/>
+      <c r="C1" s="257"/>
+      <c r="D1" s="257"/>
+      <c r="E1" s="257"/>
+      <c r="F1" s="257"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="261" t="s">
+      <c r="B2" s="260" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="261"/>
-      <c r="D2" s="261"/>
-      <c r="E2" s="261"/>
-      <c r="F2" s="261"/>
+      <c r="C2" s="260"/>
+      <c r="D2" s="260"/>
+      <c r="E2" s="260"/>
+      <c r="F2" s="260"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="258"/>
-      <c r="C3" s="258"/>
-      <c r="D3" s="258"/>
-      <c r="E3" s="258"/>
-      <c r="F3" s="258"/>
+      <c r="B3" s="257"/>
+      <c r="C3" s="257"/>
+      <c r="D3" s="257"/>
+      <c r="E3" s="257"/>
+      <c r="F3" s="257"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="259" t="s">
+      <c r="B5" s="258" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="259" t="s">
+      <c r="C5" s="258" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="259" t="s">
+      <c r="D5" s="258" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="260" t="s">
+      <c r="E5" s="259" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="260" t="s">
+      <c r="F5" s="259" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="259"/>
-      <c r="C6" s="259"/>
-      <c r="D6" s="259"/>
-      <c r="E6" s="260"/>
-      <c r="F6" s="260"/>
+      <c r="B6" s="258"/>
+      <c r="C6" s="258"/>
+      <c r="D6" s="258"/>
+      <c r="E6" s="259"/>
+      <c r="F6" s="259"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="259"/>
-      <c r="C7" s="259"/>
-      <c r="D7" s="259"/>
-      <c r="E7" s="260"/>
-      <c r="F7" s="260"/>
+      <c r="B7" s="258"/>
+      <c r="C7" s="258"/>
+      <c r="D7" s="258"/>
+      <c r="E7" s="259"/>
+      <c r="F7" s="259"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -40943,39 +40941,39 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:CE7">
-    <cfRule type="expression" dxfId="14" priority="12">
+    <cfRule type="expression" dxfId="16" priority="12">
       <formula>B5&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:CE201">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="15" priority="1">
       <formula>AND(G8&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>AND(G$7&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="3">
+    <cfRule type="expression" dxfId="13" priority="3">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="4">
+    <cfRule type="expression" dxfId="12" priority="4">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="11" priority="5">
       <formula>AND(G8&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="10" priority="6">
       <formula>AND(G$7&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="7">
+    <cfRule type="expression" dxfId="9" priority="7">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="8">
+    <cfRule type="expression" dxfId="8" priority="8">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="10">
+    <cfRule type="expression" dxfId="6" priority="10">
       <formula>AND(G$7&lt;&gt;"",$B8="DEVIASI")</formula>
     </cfRule>
     <cfRule type="colorScale" priority="11">
@@ -41016,45 +41014,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="153"/>
-      <c r="C1" s="154"/>
-      <c r="D1" s="154"/>
-      <c r="E1" s="154"/>
-      <c r="F1" s="154"/>
-      <c r="G1" s="154"/>
-      <c r="H1" s="154"/>
-      <c r="I1" s="154"/>
-      <c r="J1" s="154"/>
-      <c r="K1" s="154"/>
-      <c r="L1" s="155"/>
+      <c r="B1" s="152"/>
+      <c r="C1" s="153"/>
+      <c r="D1" s="153"/>
+      <c r="E1" s="153"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="153"/>
+      <c r="H1" s="153"/>
+      <c r="I1" s="153"/>
+      <c r="J1" s="153"/>
+      <c r="K1" s="153"/>
+      <c r="L1" s="154"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="156" t="s">
+      <c r="B2" s="155" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="157"/>
-      <c r="D2" s="157"/>
-      <c r="E2" s="157"/>
-      <c r="F2" s="157"/>
-      <c r="G2" s="157"/>
-      <c r="H2" s="157"/>
-      <c r="I2" s="158"/>
-      <c r="J2" s="162"/>
-      <c r="K2" s="163"/>
-      <c r="L2" s="164"/>
+      <c r="C2" s="156"/>
+      <c r="D2" s="156"/>
+      <c r="E2" s="156"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="156"/>
+      <c r="H2" s="156"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="161"/>
+      <c r="K2" s="162"/>
+      <c r="L2" s="163"/>
     </row>
     <row r="3" spans="1:13" ht="14.4" customHeight="1">
-      <c r="B3" s="159"/>
-      <c r="C3" s="160"/>
-      <c r="D3" s="160"/>
-      <c r="E3" s="160"/>
-      <c r="F3" s="160"/>
-      <c r="G3" s="160"/>
-      <c r="H3" s="160"/>
-      <c r="I3" s="161"/>
-      <c r="J3" s="165"/>
-      <c r="K3" s="166"/>
-      <c r="L3" s="167"/>
+      <c r="B3" s="158"/>
+      <c r="C3" s="159"/>
+      <c r="D3" s="159"/>
+      <c r="E3" s="159"/>
+      <c r="F3" s="159"/>
+      <c r="G3" s="159"/>
+      <c r="H3" s="159"/>
+      <c r="I3" s="160"/>
+      <c r="J3" s="164"/>
+      <c r="K3" s="165"/>
+      <c r="L3" s="166"/>
     </row>
     <row r="4" spans="1:13" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -41065,9 +41063,9 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="165"/>
-      <c r="K4" s="166"/>
-      <c r="L4" s="167"/>
+      <c r="J4" s="164"/>
+      <c r="K4" s="165"/>
+      <c r="L4" s="166"/>
     </row>
     <row r="5" spans="1:13" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -41082,9 +41080,9 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="165"/>
-      <c r="K5" s="166"/>
-      <c r="L5" s="167"/>
+      <c r="J5" s="164"/>
+      <c r="K5" s="165"/>
+      <c r="L5" s="166"/>
     </row>
     <row r="6" spans="1:13" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -41099,9 +41097,9 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="168"/>
-      <c r="K6" s="169"/>
-      <c r="L6" s="170"/>
+      <c r="J6" s="167"/>
+      <c r="K6" s="168"/>
+      <c r="L6" s="169"/>
     </row>
     <row r="7" spans="1:13" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -41153,45 +41151,45 @@
       <c r="J9" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="K9" s="126"/>
+      <c r="K9" s="125"/>
       <c r="L9" s="89"/>
     </row>
     <row r="10" spans="1:13" ht="15.6">
-      <c r="B10" s="171" t="s">
+      <c r="B10" s="170" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="172"/>
-      <c r="D10" s="172"/>
-      <c r="E10" s="172"/>
-      <c r="F10" s="173"/>
-      <c r="G10" s="172" t="s">
+      <c r="C10" s="171"/>
+      <c r="D10" s="171"/>
+      <c r="E10" s="171"/>
+      <c r="F10" s="172"/>
+      <c r="G10" s="171" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="172"/>
-      <c r="I10" s="172"/>
-      <c r="J10" s="173"/>
-      <c r="K10" s="172" t="s">
+      <c r="H10" s="171"/>
+      <c r="I10" s="171"/>
+      <c r="J10" s="172"/>
+      <c r="K10" s="171" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="174"/>
+      <c r="L10" s="173"/>
     </row>
     <row r="11" spans="1:13" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="193" t="s">
+      <c r="C11" s="192" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="194"/>
-      <c r="E11" s="194"/>
+      <c r="D11" s="193"/>
+      <c r="E11" s="193"/>
       <c r="F11" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="193" t="s">
+      <c r="G11" s="192" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="195"/>
+      <c r="H11" s="194"/>
       <c r="I11" s="92" t="s">
         <v>27</v>
       </c>
@@ -41210,14 +41208,14 @@
       <c r="B12" s="94" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="239" t="s">
+      <c r="C12" s="238" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="240"/>
-      <c r="E12" s="241"/>
+      <c r="D12" s="239"/>
+      <c r="E12" s="240"/>
       <c r="F12" s="95"/>
-      <c r="G12" s="202"/>
-      <c r="H12" s="203"/>
+      <c r="G12" s="201"/>
+      <c r="H12" s="202"/>
       <c r="I12" s="96"/>
       <c r="J12" s="96"/>
       <c r="K12" s="97"/>
@@ -41227,14 +41225,14 @@
       <c r="B13" s="99">
         <v>1</v>
       </c>
-      <c r="C13" s="242" t="s">
+      <c r="C13" s="241" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="243"/>
-      <c r="E13" s="244"/>
+      <c r="D13" s="242"/>
+      <c r="E13" s="243"/>
       <c r="F13" s="100"/>
-      <c r="G13" s="204"/>
-      <c r="H13" s="205"/>
+      <c r="G13" s="203"/>
+      <c r="H13" s="204"/>
       <c r="I13" s="101"/>
       <c r="J13" s="102"/>
       <c r="K13" s="103"/>
@@ -41244,14 +41242,14 @@
       <c r="B14" s="99">
         <v>2</v>
       </c>
-      <c r="C14" s="242" t="s">
+      <c r="C14" s="241" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="243"/>
-      <c r="E14" s="244"/>
+      <c r="D14" s="242"/>
+      <c r="E14" s="243"/>
       <c r="F14" s="100"/>
-      <c r="G14" s="204"/>
-      <c r="H14" s="205"/>
+      <c r="G14" s="203"/>
+      <c r="H14" s="204"/>
       <c r="I14" s="101"/>
       <c r="J14" s="102"/>
       <c r="K14" s="103"/>
@@ -41261,14 +41259,14 @@
       <c r="B15" s="99">
         <v>3</v>
       </c>
-      <c r="C15" s="242" t="s">
+      <c r="C15" s="241" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="243"/>
-      <c r="E15" s="244"/>
+      <c r="D15" s="242"/>
+      <c r="E15" s="243"/>
       <c r="F15" s="100"/>
-      <c r="G15" s="204"/>
-      <c r="H15" s="205"/>
+      <c r="G15" s="203"/>
+      <c r="H15" s="204"/>
       <c r="I15" s="101"/>
       <c r="J15" s="102"/>
       <c r="K15" s="103"/>
@@ -41278,14 +41276,14 @@
       <c r="B16" s="99">
         <v>4</v>
       </c>
-      <c r="C16" s="242" t="s">
+      <c r="C16" s="241" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="243"/>
-      <c r="E16" s="244"/>
+      <c r="D16" s="242"/>
+      <c r="E16" s="243"/>
       <c r="F16" s="100"/>
-      <c r="G16" s="204"/>
-      <c r="H16" s="205"/>
+      <c r="G16" s="203"/>
+      <c r="H16" s="204"/>
       <c r="I16" s="101"/>
       <c r="J16" s="102"/>
       <c r="K16" s="103"/>
@@ -41295,14 +41293,14 @@
       <c r="B17" s="99">
         <v>5</v>
       </c>
-      <c r="C17" s="242" t="s">
+      <c r="C17" s="241" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="243"/>
-      <c r="E17" s="244"/>
+      <c r="D17" s="242"/>
+      <c r="E17" s="243"/>
       <c r="F17" s="100"/>
-      <c r="G17" s="204"/>
-      <c r="H17" s="205"/>
+      <c r="G17" s="203"/>
+      <c r="H17" s="204"/>
       <c r="I17" s="101"/>
       <c r="J17" s="102"/>
       <c r="K17" s="103"/>
@@ -41312,14 +41310,14 @@
       <c r="B18" s="99">
         <v>6</v>
       </c>
-      <c r="C18" s="242" t="s">
+      <c r="C18" s="241" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="243"/>
-      <c r="E18" s="244"/>
+      <c r="D18" s="242"/>
+      <c r="E18" s="243"/>
       <c r="F18" s="100"/>
-      <c r="G18" s="204"/>
-      <c r="H18" s="205"/>
+      <c r="G18" s="203"/>
+      <c r="H18" s="204"/>
       <c r="I18" s="101"/>
       <c r="J18" s="102"/>
       <c r="K18" s="103"/>
@@ -41329,14 +41327,14 @@
       <c r="B19" s="105" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="245" t="s">
+      <c r="C19" s="244" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="246"/>
-      <c r="E19" s="247"/>
+      <c r="D19" s="245"/>
+      <c r="E19" s="246"/>
       <c r="F19" s="100"/>
-      <c r="G19" s="204"/>
-      <c r="H19" s="205"/>
+      <c r="G19" s="203"/>
+      <c r="H19" s="204"/>
       <c r="I19" s="101"/>
       <c r="J19" s="102"/>
       <c r="K19" s="103"/>
@@ -41346,14 +41344,14 @@
       <c r="B20" s="99">
         <v>1</v>
       </c>
-      <c r="C20" s="242" t="s">
+      <c r="C20" s="241" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="243"/>
-      <c r="E20" s="244"/>
+      <c r="D20" s="242"/>
+      <c r="E20" s="243"/>
       <c r="F20" s="100"/>
-      <c r="G20" s="204"/>
-      <c r="H20" s="205"/>
+      <c r="G20" s="203"/>
+      <c r="H20" s="204"/>
       <c r="I20" s="101"/>
       <c r="J20" s="102"/>
       <c r="K20" s="103"/>
@@ -41363,14 +41361,14 @@
       <c r="B21" s="99">
         <v>2</v>
       </c>
-      <c r="C21" s="242" t="s">
+      <c r="C21" s="241" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="243"/>
-      <c r="E21" s="244"/>
+      <c r="D21" s="242"/>
+      <c r="E21" s="243"/>
       <c r="F21" s="100"/>
-      <c r="G21" s="204"/>
-      <c r="H21" s="205"/>
+      <c r="G21" s="203"/>
+      <c r="H21" s="204"/>
       <c r="I21" s="101"/>
       <c r="J21" s="102"/>
       <c r="K21" s="103"/>
@@ -41380,175 +41378,143 @@
       <c r="B22" s="99">
         <v>3</v>
       </c>
-      <c r="C22" s="248" t="s">
+      <c r="C22" s="247" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="249"/>
-      <c r="E22" s="250"/>
+      <c r="D22" s="248"/>
+      <c r="E22" s="249"/>
       <c r="F22" s="100"/>
-      <c r="G22" s="206"/>
-      <c r="H22" s="207"/>
+      <c r="G22" s="205"/>
+      <c r="H22" s="206"/>
       <c r="I22" s="101"/>
       <c r="J22" s="102"/>
       <c r="K22" s="106"/>
       <c r="L22" s="107"/>
     </row>
     <row r="23" spans="1:12" ht="16.2" thickBot="1">
-      <c r="B23" s="196"/>
-      <c r="C23" s="197"/>
-      <c r="D23" s="197"/>
-      <c r="E23" s="197"/>
+      <c r="B23" s="195"/>
+      <c r="C23" s="196"/>
+      <c r="D23" s="196"/>
+      <c r="E23" s="196"/>
       <c r="F23" s="108"/>
       <c r="G23" s="108"/>
       <c r="H23" s="109"/>
       <c r="I23" s="109"/>
-      <c r="J23" s="198"/>
-      <c r="K23" s="198"/>
-      <c r="L23" s="199"/>
+      <c r="J23" s="197"/>
+      <c r="K23" s="197"/>
+      <c r="L23" s="198"/>
     </row>
     <row r="24" spans="1:12" ht="16.2" customHeight="1" thickTop="1">
-      <c r="A24" s="125" t="s">
+      <c r="A24" s="124" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="200" t="s">
+      <c r="B24" s="199" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="175" t="s">
+      <c r="C24" s="174" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="175"/>
-      <c r="E24" s="175"/>
-      <c r="F24" s="175"/>
-      <c r="G24" s="175"/>
-      <c r="H24" s="175"/>
-      <c r="I24" s="175"/>
-      <c r="J24" s="177" t="s">
+      <c r="D24" s="174"/>
+      <c r="E24" s="174"/>
+      <c r="F24" s="174"/>
+      <c r="G24" s="174"/>
+      <c r="H24" s="174"/>
+      <c r="I24" s="174"/>
+      <c r="J24" s="176" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="178"/>
-      <c r="L24" s="179"/>
+      <c r="K24" s="177"/>
+      <c r="L24" s="178"/>
     </row>
     <row r="25" spans="1:12" ht="31.2">
-      <c r="B25" s="201"/>
-      <c r="C25" s="176"/>
-      <c r="D25" s="176"/>
-      <c r="E25" s="176"/>
-      <c r="F25" s="176"/>
-      <c r="G25" s="176"/>
-      <c r="H25" s="176"/>
-      <c r="I25" s="176"/>
-      <c r="J25" s="152" t="s">
+      <c r="B25" s="200"/>
+      <c r="C25" s="175"/>
+      <c r="D25" s="175"/>
+      <c r="E25" s="175"/>
+      <c r="F25" s="175"/>
+      <c r="G25" s="175"/>
+      <c r="H25" s="175"/>
+      <c r="I25" s="175"/>
+      <c r="J25" s="151" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="149" t="s">
+      <c r="K25" s="148" t="s">
         <v>76</v>
       </c>
-      <c r="L25" s="150" t="s">
+      <c r="L25" s="149" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.6">
-      <c r="B26" s="110" t="s">
-        <v>132</v>
-      </c>
-      <c r="C26" s="294" t="s">
-        <v>133</v>
-      </c>
-      <c r="D26" s="295"/>
-      <c r="E26" s="295"/>
-      <c r="F26" s="295"/>
-      <c r="G26" s="295"/>
-      <c r="H26" s="295"/>
-      <c r="I26" s="296"/>
-      <c r="J26" s="303" t="s">
-        <v>64</v>
-      </c>
-      <c r="K26" s="151"/>
-      <c r="L26" s="111" t="s">
-        <v>64</v>
-      </c>
+      <c r="B26" s="110"/>
+      <c r="C26" s="293"/>
+      <c r="D26" s="294"/>
+      <c r="E26" s="294"/>
+      <c r="F26" s="294"/>
+      <c r="G26" s="294"/>
+      <c r="H26" s="294"/>
+      <c r="I26" s="295"/>
+      <c r="J26" s="302"/>
+      <c r="K26" s="150"/>
+      <c r="L26" s="306"/>
     </row>
     <row r="27" spans="1:12" ht="15.6">
-      <c r="B27" s="110">
-        <v>1</v>
-      </c>
-      <c r="C27" s="297" t="s">
-        <v>134</v>
-      </c>
-      <c r="D27" s="298"/>
-      <c r="E27" s="298"/>
-      <c r="F27" s="298"/>
-      <c r="G27" s="298"/>
-      <c r="H27" s="298"/>
-      <c r="I27" s="299"/>
-      <c r="J27" s="102" t="s">
-        <v>135</v>
-      </c>
-      <c r="K27" s="305"/>
-      <c r="L27" s="112" t="s">
-        <v>64</v>
-      </c>
+      <c r="B27" s="110"/>
+      <c r="C27" s="296"/>
+      <c r="D27" s="297"/>
+      <c r="E27" s="297"/>
+      <c r="F27" s="297"/>
+      <c r="G27" s="297"/>
+      <c r="H27" s="297"/>
+      <c r="I27" s="298"/>
+      <c r="J27" s="102"/>
+      <c r="K27" s="304"/>
+      <c r="L27" s="306"/>
     </row>
     <row r="28" spans="1:12" ht="15.6">
-      <c r="B28" s="110">
-        <v>2</v>
-      </c>
-      <c r="C28" s="297" t="s">
-        <v>64</v>
-      </c>
-      <c r="D28" s="298"/>
-      <c r="E28" s="298"/>
-      <c r="F28" s="298"/>
-      <c r="G28" s="298"/>
-      <c r="H28" s="298"/>
-      <c r="I28" s="299"/>
-      <c r="J28" s="102" t="s">
-        <v>64</v>
-      </c>
-      <c r="K28" s="305"/>
-      <c r="L28" s="112" t="s">
-        <v>64</v>
-      </c>
+      <c r="B28" s="110"/>
+      <c r="C28" s="296"/>
+      <c r="D28" s="297"/>
+      <c r="E28" s="297"/>
+      <c r="F28" s="297"/>
+      <c r="G28" s="297"/>
+      <c r="H28" s="297"/>
+      <c r="I28" s="298"/>
+      <c r="J28" s="102"/>
+      <c r="K28" s="304"/>
+      <c r="L28" s="111"/>
     </row>
     <row r="29" spans="1:12" ht="15.6">
-      <c r="B29" s="110" t="s">
-        <v>64</v>
-      </c>
-      <c r="C29" s="297" t="s">
-        <v>64</v>
-      </c>
-      <c r="D29" s="298"/>
-      <c r="E29" s="298"/>
-      <c r="F29" s="298"/>
-      <c r="G29" s="298"/>
-      <c r="H29" s="298"/>
-      <c r="I29" s="299"/>
-      <c r="J29" s="102" t="s">
-        <v>64</v>
-      </c>
-      <c r="K29" s="305"/>
-      <c r="L29" s="112" t="s">
-        <v>64</v>
-      </c>
+      <c r="B29" s="110"/>
+      <c r="C29" s="296"/>
+      <c r="D29" s="297"/>
+      <c r="E29" s="297"/>
+      <c r="F29" s="297"/>
+      <c r="G29" s="297"/>
+      <c r="H29" s="297"/>
+      <c r="I29" s="298"/>
+      <c r="J29" s="102"/>
+      <c r="K29" s="304"/>
+      <c r="L29" s="111"/>
     </row>
     <row r="30" spans="1:12" ht="15.6">
       <c r="B30" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="297" t="s">
+      <c r="C30" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="298"/>
-      <c r="E30" s="298"/>
-      <c r="F30" s="298"/>
-      <c r="G30" s="298"/>
-      <c r="H30" s="298"/>
-      <c r="I30" s="299"/>
+      <c r="D30" s="297"/>
+      <c r="E30" s="297"/>
+      <c r="F30" s="297"/>
+      <c r="G30" s="297"/>
+      <c r="H30" s="297"/>
+      <c r="I30" s="298"/>
       <c r="J30" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K30" s="305"/>
-      <c r="L30" s="112" t="s">
+      <c r="K30" s="304"/>
+      <c r="L30" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41556,20 +41522,20 @@
       <c r="B31" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="297" t="s">
+      <c r="C31" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="298"/>
-      <c r="E31" s="298"/>
-      <c r="F31" s="298"/>
-      <c r="G31" s="298"/>
-      <c r="H31" s="298"/>
-      <c r="I31" s="299"/>
+      <c r="D31" s="297"/>
+      <c r="E31" s="297"/>
+      <c r="F31" s="297"/>
+      <c r="G31" s="297"/>
+      <c r="H31" s="297"/>
+      <c r="I31" s="298"/>
       <c r="J31" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K31" s="305"/>
-      <c r="L31" s="112" t="s">
+      <c r="K31" s="304"/>
+      <c r="L31" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41577,20 +41543,20 @@
       <c r="B32" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="297" t="s">
+      <c r="C32" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="298"/>
-      <c r="E32" s="298"/>
-      <c r="F32" s="298"/>
-      <c r="G32" s="298"/>
-      <c r="H32" s="298"/>
-      <c r="I32" s="299"/>
+      <c r="D32" s="297"/>
+      <c r="E32" s="297"/>
+      <c r="F32" s="297"/>
+      <c r="G32" s="297"/>
+      <c r="H32" s="297"/>
+      <c r="I32" s="298"/>
       <c r="J32" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K32" s="305"/>
-      <c r="L32" s="112" t="s">
+      <c r="K32" s="304"/>
+      <c r="L32" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41598,20 +41564,20 @@
       <c r="B33" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="297" t="s">
+      <c r="C33" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="298"/>
-      <c r="E33" s="298"/>
-      <c r="F33" s="298"/>
-      <c r="G33" s="298"/>
-      <c r="H33" s="298"/>
-      <c r="I33" s="299"/>
+      <c r="D33" s="297"/>
+      <c r="E33" s="297"/>
+      <c r="F33" s="297"/>
+      <c r="G33" s="297"/>
+      <c r="H33" s="297"/>
+      <c r="I33" s="298"/>
       <c r="J33" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K33" s="305"/>
-      <c r="L33" s="112" t="s">
+      <c r="K33" s="304"/>
+      <c r="L33" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41619,20 +41585,20 @@
       <c r="B34" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="297" t="s">
+      <c r="C34" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="298"/>
-      <c r="E34" s="298"/>
-      <c r="F34" s="298"/>
-      <c r="G34" s="298"/>
-      <c r="H34" s="298"/>
-      <c r="I34" s="299"/>
+      <c r="D34" s="297"/>
+      <c r="E34" s="297"/>
+      <c r="F34" s="297"/>
+      <c r="G34" s="297"/>
+      <c r="H34" s="297"/>
+      <c r="I34" s="298"/>
       <c r="J34" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K34" s="305"/>
-      <c r="L34" s="112" t="s">
+      <c r="K34" s="304"/>
+      <c r="L34" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41640,20 +41606,20 @@
       <c r="B35" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="297" t="s">
+      <c r="C35" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="298"/>
-      <c r="E35" s="298"/>
-      <c r="F35" s="298"/>
-      <c r="G35" s="298"/>
-      <c r="H35" s="298"/>
-      <c r="I35" s="299"/>
+      <c r="D35" s="297"/>
+      <c r="E35" s="297"/>
+      <c r="F35" s="297"/>
+      <c r="G35" s="297"/>
+      <c r="H35" s="297"/>
+      <c r="I35" s="298"/>
       <c r="J35" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K35" s="305"/>
-      <c r="L35" s="112" t="s">
+      <c r="K35" s="304"/>
+      <c r="L35" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41661,20 +41627,20 @@
       <c r="B36" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C36" s="297" t="s">
+      <c r="C36" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="298"/>
-      <c r="E36" s="298"/>
-      <c r="F36" s="298"/>
-      <c r="G36" s="298"/>
-      <c r="H36" s="298"/>
-      <c r="I36" s="299"/>
+      <c r="D36" s="297"/>
+      <c r="E36" s="297"/>
+      <c r="F36" s="297"/>
+      <c r="G36" s="297"/>
+      <c r="H36" s="297"/>
+      <c r="I36" s="298"/>
       <c r="J36" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K36" s="305"/>
-      <c r="L36" s="112" t="s">
+      <c r="K36" s="304"/>
+      <c r="L36" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41682,20 +41648,20 @@
       <c r="B37" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="297" t="s">
+      <c r="C37" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="298"/>
-      <c r="E37" s="298"/>
-      <c r="F37" s="298"/>
-      <c r="G37" s="298"/>
-      <c r="H37" s="298"/>
-      <c r="I37" s="299"/>
+      <c r="D37" s="297"/>
+      <c r="E37" s="297"/>
+      <c r="F37" s="297"/>
+      <c r="G37" s="297"/>
+      <c r="H37" s="297"/>
+      <c r="I37" s="298"/>
       <c r="J37" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K37" s="305"/>
-      <c r="L37" s="112" t="s">
+      <c r="K37" s="304"/>
+      <c r="L37" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41703,20 +41669,20 @@
       <c r="B38" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="297" t="s">
+      <c r="C38" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="298"/>
-      <c r="E38" s="298"/>
-      <c r="F38" s="298"/>
-      <c r="G38" s="298"/>
-      <c r="H38" s="298"/>
-      <c r="I38" s="299"/>
+      <c r="D38" s="297"/>
+      <c r="E38" s="297"/>
+      <c r="F38" s="297"/>
+      <c r="G38" s="297"/>
+      <c r="H38" s="297"/>
+      <c r="I38" s="298"/>
       <c r="J38" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K38" s="305"/>
-      <c r="L38" s="112" t="s">
+      <c r="K38" s="304"/>
+      <c r="L38" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41724,20 +41690,20 @@
       <c r="B39" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="297" t="s">
+      <c r="C39" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D39" s="298"/>
-      <c r="E39" s="298"/>
-      <c r="F39" s="298"/>
-      <c r="G39" s="298"/>
-      <c r="H39" s="298"/>
-      <c r="I39" s="299"/>
+      <c r="D39" s="297"/>
+      <c r="E39" s="297"/>
+      <c r="F39" s="297"/>
+      <c r="G39" s="297"/>
+      <c r="H39" s="297"/>
+      <c r="I39" s="298"/>
       <c r="J39" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K39" s="305"/>
-      <c r="L39" s="112" t="s">
+      <c r="K39" s="304"/>
+      <c r="L39" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41745,20 +41711,20 @@
       <c r="B40" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="297" t="s">
+      <c r="C40" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D40" s="298"/>
-      <c r="E40" s="298"/>
-      <c r="F40" s="298"/>
-      <c r="G40" s="298"/>
-      <c r="H40" s="298"/>
-      <c r="I40" s="299"/>
+      <c r="D40" s="297"/>
+      <c r="E40" s="297"/>
+      <c r="F40" s="297"/>
+      <c r="G40" s="297"/>
+      <c r="H40" s="297"/>
+      <c r="I40" s="298"/>
       <c r="J40" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K40" s="305"/>
-      <c r="L40" s="112" t="s">
+      <c r="K40" s="304"/>
+      <c r="L40" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41766,20 +41732,20 @@
       <c r="B41" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="297" t="s">
+      <c r="C41" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D41" s="298"/>
-      <c r="E41" s="298"/>
-      <c r="F41" s="298"/>
-      <c r="G41" s="298"/>
-      <c r="H41" s="298"/>
-      <c r="I41" s="299"/>
+      <c r="D41" s="297"/>
+      <c r="E41" s="297"/>
+      <c r="F41" s="297"/>
+      <c r="G41" s="297"/>
+      <c r="H41" s="297"/>
+      <c r="I41" s="298"/>
       <c r="J41" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K41" s="305"/>
-      <c r="L41" s="112" t="s">
+      <c r="K41" s="304"/>
+      <c r="L41" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41787,20 +41753,20 @@
       <c r="B42" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="297" t="s">
+      <c r="C42" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="298"/>
-      <c r="E42" s="298"/>
-      <c r="F42" s="298"/>
-      <c r="G42" s="298"/>
-      <c r="H42" s="298"/>
-      <c r="I42" s="299"/>
+      <c r="D42" s="297"/>
+      <c r="E42" s="297"/>
+      <c r="F42" s="297"/>
+      <c r="G42" s="297"/>
+      <c r="H42" s="297"/>
+      <c r="I42" s="298"/>
       <c r="J42" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K42" s="305"/>
-      <c r="L42" s="112" t="s">
+      <c r="K42" s="304"/>
+      <c r="L42" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41808,20 +41774,20 @@
       <c r="B43" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="297" t="s">
+      <c r="C43" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="298"/>
-      <c r="E43" s="298"/>
-      <c r="F43" s="298"/>
-      <c r="G43" s="298"/>
-      <c r="H43" s="298"/>
-      <c r="I43" s="299"/>
+      <c r="D43" s="297"/>
+      <c r="E43" s="297"/>
+      <c r="F43" s="297"/>
+      <c r="G43" s="297"/>
+      <c r="H43" s="297"/>
+      <c r="I43" s="298"/>
       <c r="J43" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K43" s="305"/>
-      <c r="L43" s="112" t="s">
+      <c r="K43" s="304"/>
+      <c r="L43" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41829,20 +41795,20 @@
       <c r="B44" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="297" t="s">
+      <c r="C44" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D44" s="298"/>
-      <c r="E44" s="298"/>
-      <c r="F44" s="298"/>
-      <c r="G44" s="298"/>
-      <c r="H44" s="298"/>
-      <c r="I44" s="299"/>
+      <c r="D44" s="297"/>
+      <c r="E44" s="297"/>
+      <c r="F44" s="297"/>
+      <c r="G44" s="297"/>
+      <c r="H44" s="297"/>
+      <c r="I44" s="298"/>
       <c r="J44" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K44" s="305"/>
-      <c r="L44" s="112" t="s">
+      <c r="K44" s="304"/>
+      <c r="L44" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41850,20 +41816,20 @@
       <c r="B45" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C45" s="297" t="s">
+      <c r="C45" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D45" s="298"/>
-      <c r="E45" s="298"/>
-      <c r="F45" s="298"/>
-      <c r="G45" s="298"/>
-      <c r="H45" s="298"/>
-      <c r="I45" s="299"/>
+      <c r="D45" s="297"/>
+      <c r="E45" s="297"/>
+      <c r="F45" s="297"/>
+      <c r="G45" s="297"/>
+      <c r="H45" s="297"/>
+      <c r="I45" s="298"/>
       <c r="J45" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K45" s="305"/>
-      <c r="L45" s="112" t="s">
+      <c r="K45" s="304"/>
+      <c r="L45" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41871,20 +41837,20 @@
       <c r="B46" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C46" s="297" t="s">
+      <c r="C46" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="298"/>
-      <c r="E46" s="298"/>
-      <c r="F46" s="298"/>
-      <c r="G46" s="298"/>
-      <c r="H46" s="298"/>
-      <c r="I46" s="299"/>
+      <c r="D46" s="297"/>
+      <c r="E46" s="297"/>
+      <c r="F46" s="297"/>
+      <c r="G46" s="297"/>
+      <c r="H46" s="297"/>
+      <c r="I46" s="298"/>
       <c r="J46" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K46" s="305"/>
-      <c r="L46" s="112" t="s">
+      <c r="K46" s="304"/>
+      <c r="L46" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41892,20 +41858,20 @@
       <c r="B47" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="297" t="s">
+      <c r="C47" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="298"/>
-      <c r="E47" s="298"/>
-      <c r="F47" s="298"/>
-      <c r="G47" s="298"/>
-      <c r="H47" s="298"/>
-      <c r="I47" s="299"/>
+      <c r="D47" s="297"/>
+      <c r="E47" s="297"/>
+      <c r="F47" s="297"/>
+      <c r="G47" s="297"/>
+      <c r="H47" s="297"/>
+      <c r="I47" s="298"/>
       <c r="J47" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K47" s="305"/>
-      <c r="L47" s="112" t="s">
+      <c r="K47" s="304"/>
+      <c r="L47" s="111" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41913,333 +41879,333 @@
       <c r="B48" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C48" s="300" t="s">
+      <c r="C48" s="299" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="301"/>
-      <c r="E48" s="301"/>
-      <c r="F48" s="301"/>
-      <c r="G48" s="301"/>
-      <c r="H48" s="301"/>
-      <c r="I48" s="302"/>
-      <c r="J48" s="304" t="s">
+      <c r="D48" s="300"/>
+      <c r="E48" s="300"/>
+      <c r="F48" s="300"/>
+      <c r="G48" s="300"/>
+      <c r="H48" s="300"/>
+      <c r="I48" s="301"/>
+      <c r="J48" s="303" t="s">
         <v>64</v>
       </c>
-      <c r="K48" s="306"/>
-      <c r="L48" s="112" t="s">
+      <c r="K48" s="305"/>
+      <c r="L48" s="111" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="49" spans="2:12" ht="16.2" thickTop="1">
-      <c r="B49" s="221" t="s">
+      <c r="B49" s="220" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="222"/>
-      <c r="D49" s="222"/>
-      <c r="E49" s="222"/>
-      <c r="F49" s="222"/>
-      <c r="G49" s="222"/>
-      <c r="H49" s="222"/>
-      <c r="I49" s="222"/>
-      <c r="J49" s="223"/>
-      <c r="K49" s="191" t="s">
+      <c r="C49" s="221"/>
+      <c r="D49" s="221"/>
+      <c r="E49" s="221"/>
+      <c r="F49" s="221"/>
+      <c r="G49" s="221"/>
+      <c r="H49" s="221"/>
+      <c r="I49" s="221"/>
+      <c r="J49" s="222"/>
+      <c r="K49" s="190" t="s">
         <v>79</v>
       </c>
-      <c r="L49" s="192"/>
+      <c r="L49" s="191"/>
     </row>
     <row r="50" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B50" s="224"/>
-      <c r="C50" s="225"/>
-      <c r="D50" s="225"/>
-      <c r="E50" s="225"/>
-      <c r="F50" s="225"/>
-      <c r="G50" s="225"/>
-      <c r="H50" s="225"/>
-      <c r="I50" s="225"/>
-      <c r="J50" s="226"/>
-      <c r="K50" s="189" t="s">
+      <c r="B50" s="223"/>
+      <c r="C50" s="224"/>
+      <c r="D50" s="224"/>
+      <c r="E50" s="224"/>
+      <c r="F50" s="224"/>
+      <c r="G50" s="224"/>
+      <c r="H50" s="224"/>
+      <c r="I50" s="224"/>
+      <c r="J50" s="225"/>
+      <c r="K50" s="188" t="s">
         <v>103</v>
       </c>
-      <c r="L50" s="190"/>
+      <c r="L50" s="189"/>
     </row>
     <row r="51" spans="2:12" ht="15.6">
-      <c r="B51" s="113"/>
-      <c r="C51" s="186"/>
-      <c r="D51" s="186"/>
-      <c r="E51" s="186"/>
-      <c r="F51" s="186"/>
-      <c r="G51" s="186"/>
-      <c r="H51" s="186"/>
-      <c r="I51" s="186"/>
-      <c r="J51" s="114"/>
-      <c r="K51" s="184"/>
-      <c r="L51" s="185"/>
+      <c r="B51" s="112"/>
+      <c r="C51" s="185"/>
+      <c r="D51" s="185"/>
+      <c r="E51" s="185"/>
+      <c r="F51" s="185"/>
+      <c r="G51" s="185"/>
+      <c r="H51" s="185"/>
+      <c r="I51" s="185"/>
+      <c r="J51" s="113"/>
+      <c r="K51" s="183"/>
+      <c r="L51" s="184"/>
     </row>
     <row r="52" spans="2:12" ht="15.6">
-      <c r="B52" s="115"/>
-      <c r="C52" s="187"/>
-      <c r="D52" s="187"/>
-      <c r="E52" s="187"/>
-      <c r="F52" s="187"/>
-      <c r="G52" s="187"/>
-      <c r="H52" s="187"/>
-      <c r="I52" s="187"/>
-      <c r="J52" s="116"/>
-      <c r="K52" s="127"/>
-      <c r="L52" s="117"/>
+      <c r="B52" s="114"/>
+      <c r="C52" s="186"/>
+      <c r="D52" s="186"/>
+      <c r="E52" s="186"/>
+      <c r="F52" s="186"/>
+      <c r="G52" s="186"/>
+      <c r="H52" s="186"/>
+      <c r="I52" s="186"/>
+      <c r="J52" s="115"/>
+      <c r="K52" s="126"/>
+      <c r="L52" s="116"/>
     </row>
     <row r="53" spans="2:12" ht="15.6">
-      <c r="B53" s="115"/>
-      <c r="C53" s="187"/>
-      <c r="D53" s="187"/>
-      <c r="E53" s="187"/>
-      <c r="F53" s="187"/>
-      <c r="G53" s="187"/>
-      <c r="H53" s="187"/>
-      <c r="I53" s="187"/>
-      <c r="J53" s="116"/>
-      <c r="K53" s="127"/>
-      <c r="L53" s="117"/>
+      <c r="B53" s="114"/>
+      <c r="C53" s="186"/>
+      <c r="D53" s="186"/>
+      <c r="E53" s="186"/>
+      <c r="F53" s="186"/>
+      <c r="G53" s="186"/>
+      <c r="H53" s="186"/>
+      <c r="I53" s="186"/>
+      <c r="J53" s="115"/>
+      <c r="K53" s="126"/>
+      <c r="L53" s="116"/>
     </row>
     <row r="54" spans="2:12" ht="15.6">
-      <c r="B54" s="115"/>
-      <c r="C54" s="187"/>
-      <c r="D54" s="187"/>
-      <c r="E54" s="187"/>
-      <c r="F54" s="187"/>
-      <c r="G54" s="187"/>
-      <c r="H54" s="187"/>
-      <c r="I54" s="187"/>
-      <c r="J54" s="116"/>
-      <c r="K54" s="127"/>
-      <c r="L54" s="117"/>
+      <c r="B54" s="114"/>
+      <c r="C54" s="186"/>
+      <c r="D54" s="186"/>
+      <c r="E54" s="186"/>
+      <c r="F54" s="186"/>
+      <c r="G54" s="186"/>
+      <c r="H54" s="186"/>
+      <c r="I54" s="186"/>
+      <c r="J54" s="115"/>
+      <c r="K54" s="126"/>
+      <c r="L54" s="116"/>
     </row>
     <row r="55" spans="2:12" ht="15.6">
-      <c r="B55" s="118"/>
-      <c r="C55" s="187"/>
-      <c r="D55" s="187"/>
-      <c r="E55" s="187"/>
-      <c r="F55" s="187"/>
-      <c r="G55" s="187"/>
-      <c r="H55" s="187"/>
-      <c r="I55" s="187"/>
-      <c r="J55" s="119"/>
-      <c r="K55" s="120"/>
-      <c r="L55" s="121"/>
+      <c r="B55" s="117"/>
+      <c r="C55" s="186"/>
+      <c r="D55" s="186"/>
+      <c r="E55" s="186"/>
+      <c r="F55" s="186"/>
+      <c r="G55" s="186"/>
+      <c r="H55" s="186"/>
+      <c r="I55" s="186"/>
+      <c r="J55" s="118"/>
+      <c r="K55" s="119"/>
+      <c r="L55" s="120"/>
     </row>
     <row r="56" spans="2:12" ht="15.6">
-      <c r="B56" s="118"/>
-      <c r="C56" s="187"/>
-      <c r="D56" s="187"/>
-      <c r="E56" s="187"/>
-      <c r="F56" s="187"/>
-      <c r="G56" s="187"/>
-      <c r="H56" s="187"/>
-      <c r="I56" s="187"/>
-      <c r="J56" s="119"/>
-      <c r="K56" s="120"/>
-      <c r="L56" s="121"/>
+      <c r="B56" s="117"/>
+      <c r="C56" s="186"/>
+      <c r="D56" s="186"/>
+      <c r="E56" s="186"/>
+      <c r="F56" s="186"/>
+      <c r="G56" s="186"/>
+      <c r="H56" s="186"/>
+      <c r="I56" s="186"/>
+      <c r="J56" s="118"/>
+      <c r="K56" s="119"/>
+      <c r="L56" s="120"/>
     </row>
     <row r="57" spans="2:12" ht="15.6">
-      <c r="B57" s="118"/>
-      <c r="C57" s="187"/>
-      <c r="D57" s="187"/>
-      <c r="E57" s="187"/>
-      <c r="F57" s="187"/>
-      <c r="G57" s="187"/>
-      <c r="H57" s="187"/>
-      <c r="I57" s="187"/>
-      <c r="J57" s="119"/>
-      <c r="K57" s="180"/>
-      <c r="L57" s="181"/>
+      <c r="B57" s="117"/>
+      <c r="C57" s="186"/>
+      <c r="D57" s="186"/>
+      <c r="E57" s="186"/>
+      <c r="F57" s="186"/>
+      <c r="G57" s="186"/>
+      <c r="H57" s="186"/>
+      <c r="I57" s="186"/>
+      <c r="J57" s="118"/>
+      <c r="K57" s="179"/>
+      <c r="L57" s="180"/>
     </row>
     <row r="58" spans="2:12" ht="15.6">
-      <c r="B58" s="118"/>
-      <c r="C58" s="187"/>
-      <c r="D58" s="187"/>
-      <c r="E58" s="187"/>
-      <c r="F58" s="187"/>
-      <c r="G58" s="187"/>
-      <c r="H58" s="187"/>
-      <c r="I58" s="187"/>
-      <c r="J58" s="119"/>
-      <c r="K58" s="182"/>
-      <c r="L58" s="183"/>
+      <c r="B58" s="117"/>
+      <c r="C58" s="186"/>
+      <c r="D58" s="186"/>
+      <c r="E58" s="186"/>
+      <c r="F58" s="186"/>
+      <c r="G58" s="186"/>
+      <c r="H58" s="186"/>
+      <c r="I58" s="186"/>
+      <c r="J58" s="118"/>
+      <c r="K58" s="181"/>
+      <c r="L58" s="182"/>
     </row>
     <row r="59" spans="2:12" ht="15.6">
-      <c r="B59" s="118"/>
-      <c r="C59" s="187"/>
-      <c r="D59" s="187"/>
-      <c r="E59" s="187"/>
-      <c r="F59" s="187"/>
-      <c r="G59" s="187"/>
-      <c r="H59" s="187"/>
-      <c r="I59" s="187"/>
-      <c r="J59" s="119"/>
-      <c r="K59" s="128"/>
+      <c r="B59" s="117"/>
+      <c r="C59" s="186"/>
+      <c r="D59" s="186"/>
+      <c r="E59" s="186"/>
+      <c r="F59" s="186"/>
+      <c r="G59" s="186"/>
+      <c r="H59" s="186"/>
+      <c r="I59" s="186"/>
+      <c r="J59" s="118"/>
+      <c r="K59" s="127"/>
       <c r="L59" s="76"/>
     </row>
     <row r="60" spans="2:12" ht="15.6">
-      <c r="B60" s="118"/>
-      <c r="C60" s="187"/>
-      <c r="D60" s="187"/>
-      <c r="E60" s="187"/>
-      <c r="F60" s="187"/>
-      <c r="G60" s="187"/>
-      <c r="H60" s="187"/>
-      <c r="I60" s="187"/>
-      <c r="J60" s="119"/>
-      <c r="K60" s="128"/>
+      <c r="B60" s="117"/>
+      <c r="C60" s="186"/>
+      <c r="D60" s="186"/>
+      <c r="E60" s="186"/>
+      <c r="F60" s="186"/>
+      <c r="G60" s="186"/>
+      <c r="H60" s="186"/>
+      <c r="I60" s="186"/>
+      <c r="J60" s="118"/>
+      <c r="K60" s="127"/>
       <c r="L60" s="76"/>
     </row>
     <row r="61" spans="2:12" ht="15.6">
-      <c r="B61" s="118"/>
-      <c r="C61" s="188"/>
-      <c r="D61" s="188"/>
-      <c r="E61" s="188"/>
-      <c r="F61" s="188"/>
-      <c r="G61" s="188"/>
-      <c r="H61" s="188"/>
-      <c r="I61" s="188"/>
-      <c r="J61" s="119"/>
-      <c r="K61" s="128"/>
+      <c r="B61" s="117"/>
+      <c r="C61" s="187"/>
+      <c r="D61" s="187"/>
+      <c r="E61" s="187"/>
+      <c r="F61" s="187"/>
+      <c r="G61" s="187"/>
+      <c r="H61" s="187"/>
+      <c r="I61" s="187"/>
+      <c r="J61" s="118"/>
+      <c r="K61" s="127"/>
       <c r="L61" s="76"/>
     </row>
     <row r="62" spans="2:12" ht="15.6">
-      <c r="B62" s="118"/>
-      <c r="C62" s="122"/>
-      <c r="D62" s="122"/>
-      <c r="E62" s="122"/>
-      <c r="F62" s="122"/>
-      <c r="G62" s="122"/>
-      <c r="H62" s="122"/>
-      <c r="I62" s="122"/>
-      <c r="J62" s="119"/>
-      <c r="K62" s="130"/>
-      <c r="L62" s="131"/>
+      <c r="B62" s="117"/>
+      <c r="C62" s="121"/>
+      <c r="D62" s="121"/>
+      <c r="E62" s="121"/>
+      <c r="F62" s="121"/>
+      <c r="G62" s="121"/>
+      <c r="H62" s="121"/>
+      <c r="I62" s="121"/>
+      <c r="J62" s="118"/>
+      <c r="K62" s="129"/>
+      <c r="L62" s="130"/>
     </row>
     <row r="63" spans="2:12" ht="15.6">
-      <c r="B63" s="208" t="s">
+      <c r="B63" s="207" t="s">
         <v>80</v>
       </c>
-      <c r="C63" s="209"/>
-      <c r="D63" s="209"/>
-      <c r="E63" s="210"/>
-      <c r="F63" s="211" t="s">
+      <c r="C63" s="208"/>
+      <c r="D63" s="208"/>
+      <c r="E63" s="209"/>
+      <c r="F63" s="210" t="s">
         <v>81</v>
       </c>
-      <c r="G63" s="210"/>
-      <c r="H63" s="211" t="s">
+      <c r="G63" s="209"/>
+      <c r="H63" s="210" t="s">
         <v>82</v>
       </c>
-      <c r="I63" s="209"/>
-      <c r="J63" s="210"/>
-      <c r="K63" s="120"/>
-      <c r="L63" s="121"/>
+      <c r="I63" s="208"/>
+      <c r="J63" s="209"/>
+      <c r="K63" s="119"/>
+      <c r="L63" s="120"/>
     </row>
     <row r="64" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B64" s="233"/>
-      <c r="C64" s="234"/>
-      <c r="D64" s="234"/>
-      <c r="E64" s="228"/>
-      <c r="F64" s="227"/>
-      <c r="G64" s="228"/>
-      <c r="H64" s="212"/>
-      <c r="I64" s="213"/>
-      <c r="J64" s="214"/>
-      <c r="K64" s="120"/>
-      <c r="L64" s="121"/>
+      <c r="B64" s="232"/>
+      <c r="C64" s="233"/>
+      <c r="D64" s="233"/>
+      <c r="E64" s="227"/>
+      <c r="F64" s="226"/>
+      <c r="G64" s="227"/>
+      <c r="H64" s="211"/>
+      <c r="I64" s="212"/>
+      <c r="J64" s="213"/>
+      <c r="K64" s="119"/>
+      <c r="L64" s="120"/>
     </row>
     <row r="65" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B65" s="235"/>
-      <c r="C65" s="236"/>
-      <c r="D65" s="236"/>
-      <c r="E65" s="230"/>
-      <c r="F65" s="229"/>
-      <c r="G65" s="230"/>
-      <c r="H65" s="215"/>
-      <c r="I65" s="216"/>
-      <c r="J65" s="217"/>
-      <c r="K65" s="129"/>
-      <c r="L65" s="121"/>
+      <c r="B65" s="234"/>
+      <c r="C65" s="235"/>
+      <c r="D65" s="235"/>
+      <c r="E65" s="229"/>
+      <c r="F65" s="228"/>
+      <c r="G65" s="229"/>
+      <c r="H65" s="214"/>
+      <c r="I65" s="215"/>
+      <c r="J65" s="216"/>
+      <c r="K65" s="128"/>
+      <c r="L65" s="120"/>
     </row>
     <row r="66" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B66" s="235"/>
-      <c r="C66" s="236"/>
-      <c r="D66" s="236"/>
-      <c r="E66" s="230"/>
-      <c r="F66" s="229"/>
-      <c r="G66" s="230"/>
-      <c r="H66" s="215"/>
-      <c r="I66" s="216"/>
-      <c r="J66" s="217"/>
-      <c r="K66" s="120"/>
-      <c r="L66" s="121"/>
+      <c r="B66" s="234"/>
+      <c r="C66" s="235"/>
+      <c r="D66" s="235"/>
+      <c r="E66" s="229"/>
+      <c r="F66" s="228"/>
+      <c r="G66" s="229"/>
+      <c r="H66" s="214"/>
+      <c r="I66" s="215"/>
+      <c r="J66" s="216"/>
+      <c r="K66" s="119"/>
+      <c r="L66" s="120"/>
     </row>
     <row r="67" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B67" s="235"/>
-      <c r="C67" s="236"/>
-      <c r="D67" s="236"/>
-      <c r="E67" s="230"/>
-      <c r="F67" s="229"/>
-      <c r="G67" s="230"/>
-      <c r="H67" s="215"/>
-      <c r="I67" s="216"/>
-      <c r="J67" s="217"/>
-      <c r="K67" s="128"/>
+      <c r="B67" s="234"/>
+      <c r="C67" s="235"/>
+      <c r="D67" s="235"/>
+      <c r="E67" s="229"/>
+      <c r="F67" s="228"/>
+      <c r="G67" s="229"/>
+      <c r="H67" s="214"/>
+      <c r="I67" s="215"/>
+      <c r="J67" s="216"/>
+      <c r="K67" s="127"/>
       <c r="L67" s="76"/>
     </row>
     <row r="68" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B68" s="235"/>
-      <c r="C68" s="236"/>
-      <c r="D68" s="236"/>
-      <c r="E68" s="230"/>
-      <c r="F68" s="229"/>
-      <c r="G68" s="230"/>
-      <c r="H68" s="215"/>
-      <c r="I68" s="216"/>
-      <c r="J68" s="217"/>
-      <c r="K68" s="128"/>
+      <c r="B68" s="234"/>
+      <c r="C68" s="235"/>
+      <c r="D68" s="235"/>
+      <c r="E68" s="229"/>
+      <c r="F68" s="228"/>
+      <c r="G68" s="229"/>
+      <c r="H68" s="214"/>
+      <c r="I68" s="215"/>
+      <c r="J68" s="216"/>
+      <c r="K68" s="127"/>
       <c r="L68" s="76"/>
     </row>
     <row r="69" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B69" s="235"/>
-      <c r="C69" s="236"/>
-      <c r="D69" s="236"/>
-      <c r="E69" s="230"/>
-      <c r="F69" s="229"/>
-      <c r="G69" s="230"/>
-      <c r="H69" s="215"/>
-      <c r="I69" s="216"/>
-      <c r="J69" s="217"/>
-      <c r="K69" s="132"/>
-      <c r="L69" s="133"/>
+      <c r="B69" s="234"/>
+      <c r="C69" s="235"/>
+      <c r="D69" s="235"/>
+      <c r="E69" s="229"/>
+      <c r="F69" s="228"/>
+      <c r="G69" s="229"/>
+      <c r="H69" s="214"/>
+      <c r="I69" s="215"/>
+      <c r="J69" s="216"/>
+      <c r="K69" s="131"/>
+      <c r="L69" s="132"/>
     </row>
     <row r="70" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B70" s="235"/>
-      <c r="C70" s="236"/>
-      <c r="D70" s="236"/>
-      <c r="E70" s="230"/>
-      <c r="F70" s="229"/>
-      <c r="G70" s="230"/>
-      <c r="H70" s="215"/>
-      <c r="I70" s="216"/>
-      <c r="J70" s="217"/>
-      <c r="K70" s="132"/>
-      <c r="L70" s="133"/>
+      <c r="B70" s="234"/>
+      <c r="C70" s="235"/>
+      <c r="D70" s="235"/>
+      <c r="E70" s="229"/>
+      <c r="F70" s="228"/>
+      <c r="G70" s="229"/>
+      <c r="H70" s="214"/>
+      <c r="I70" s="215"/>
+      <c r="J70" s="216"/>
+      <c r="K70" s="131"/>
+      <c r="L70" s="132"/>
     </row>
     <row r="71" spans="2:12" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B71" s="237"/>
-      <c r="C71" s="238"/>
-      <c r="D71" s="238"/>
-      <c r="E71" s="232"/>
-      <c r="F71" s="231"/>
-      <c r="G71" s="232"/>
-      <c r="H71" s="218"/>
-      <c r="I71" s="219"/>
-      <c r="J71" s="220"/>
-      <c r="K71" s="123"/>
-      <c r="L71" s="124"/>
+      <c r="B71" s="236"/>
+      <c r="C71" s="237"/>
+      <c r="D71" s="237"/>
+      <c r="E71" s="231"/>
+      <c r="F71" s="230"/>
+      <c r="G71" s="231"/>
+      <c r="H71" s="217"/>
+      <c r="I71" s="218"/>
+      <c r="J71" s="219"/>
+      <c r="K71" s="122"/>
+      <c r="L71" s="123"/>
     </row>
     <row r="72" spans="2:12" ht="15" thickTop="1">
       <c r="J72" s="61"/>
@@ -42320,14 +42286,9 @@
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="K10:L10"/>
   </mergeCells>
-  <conditionalFormatting sqref="B26:C48">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>ISTEXT($C26)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J27:J48 L27:L48">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
-      <formula>0</formula>
+  <conditionalFormatting sqref="B26:L48">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>AND($B26&lt;&gt;"",$J26="",$L26&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -42364,40 +42325,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="258"/>
-      <c r="C1" s="258"/>
-      <c r="D1" s="258"/>
-      <c r="E1" s="258"/>
-      <c r="F1" s="258"/>
-      <c r="G1" s="258"/>
-      <c r="H1" s="258"/>
-      <c r="I1" s="258"/>
-      <c r="J1" s="258"/>
-      <c r="K1" s="258"/>
-      <c r="L1" s="258"/>
-      <c r="M1" s="258"/>
-      <c r="N1" s="258"/>
-      <c r="O1" s="258"/>
-      <c r="P1" s="258"/>
+      <c r="B1" s="257"/>
+      <c r="C1" s="257"/>
+      <c r="D1" s="257"/>
+      <c r="E1" s="257"/>
+      <c r="F1" s="257"/>
+      <c r="G1" s="257"/>
+      <c r="H1" s="257"/>
+      <c r="I1" s="257"/>
+      <c r="J1" s="257"/>
+      <c r="K1" s="257"/>
+      <c r="L1" s="257"/>
+      <c r="M1" s="257"/>
+      <c r="N1" s="257"/>
+      <c r="O1" s="257"/>
+      <c r="P1" s="257"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="256" t="s">
+      <c r="B2" s="255" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="257"/>
-      <c r="F2" s="257"/>
-      <c r="G2" s="257"/>
-      <c r="H2" s="257"/>
-      <c r="I2" s="257"/>
-      <c r="J2" s="257"/>
-      <c r="K2" s="257"/>
-      <c r="L2" s="257"/>
-      <c r="M2" s="257"/>
-      <c r="N2" s="257"/>
-      <c r="O2" s="257"/>
-      <c r="P2" s="257"/>
+      <c r="C2" s="256"/>
+      <c r="D2" s="256"/>
+      <c r="E2" s="256"/>
+      <c r="F2" s="256"/>
+      <c r="G2" s="256"/>
+      <c r="H2" s="256"/>
+      <c r="I2" s="256"/>
+      <c r="J2" s="256"/>
+      <c r="K2" s="256"/>
+      <c r="L2" s="256"/>
+      <c r="M2" s="256"/>
+      <c r="N2" s="256"/>
+      <c r="O2" s="256"/>
+      <c r="P2" s="256"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -42424,16 +42385,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="264" t="s">
+      <c r="I4" s="263" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="264"/>
-      <c r="K4" s="264"/>
-      <c r="L4" s="264"/>
-      <c r="M4" s="264"/>
-      <c r="N4" s="264"/>
-      <c r="O4" s="264"/>
-      <c r="P4" s="264"/>
+      <c r="J4" s="263"/>
+      <c r="K4" s="263"/>
+      <c r="L4" s="263"/>
+      <c r="M4" s="263"/>
+      <c r="N4" s="263"/>
+      <c r="O4" s="263"/>
+      <c r="P4" s="263"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -42447,14 +42408,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="264"/>
-      <c r="J5" s="264"/>
-      <c r="K5" s="264"/>
-      <c r="L5" s="264"/>
-      <c r="M5" s="264"/>
-      <c r="N5" s="264"/>
-      <c r="O5" s="264"/>
-      <c r="P5" s="264"/>
+      <c r="I5" s="263"/>
+      <c r="J5" s="263"/>
+      <c r="K5" s="263"/>
+      <c r="L5" s="263"/>
+      <c r="M5" s="263"/>
+      <c r="N5" s="263"/>
+      <c r="O5" s="263"/>
+      <c r="P5" s="263"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -42589,70 +42550,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="255" t="s">
+      <c r="B12" s="254" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="255" t="s">
+      <c r="C12" s="254" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="255"/>
-      <c r="E12" s="255"/>
-      <c r="F12" s="255" t="s">
+      <c r="D12" s="254"/>
+      <c r="E12" s="254"/>
+      <c r="F12" s="254" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="255" t="s">
+      <c r="G12" s="254" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="255" t="s">
+      <c r="H12" s="254" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="255" t="s">
+      <c r="I12" s="254" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="255" t="s">
+      <c r="J12" s="254" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="255"/>
-      <c r="L12" s="255"/>
-      <c r="M12" s="255"/>
-      <c r="N12" s="255"/>
-      <c r="O12" s="255"/>
-      <c r="P12" s="263" t="s">
+      <c r="K12" s="254"/>
+      <c r="L12" s="254"/>
+      <c r="M12" s="254"/>
+      <c r="N12" s="254"/>
+      <c r="O12" s="254"/>
+      <c r="P12" s="262" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="255"/>
-      <c r="C13" s="255"/>
-      <c r="D13" s="255"/>
-      <c r="E13" s="255"/>
-      <c r="F13" s="255"/>
-      <c r="G13" s="255"/>
-      <c r="H13" s="255"/>
-      <c r="I13" s="255"/>
-      <c r="J13" s="262" t="s">
+      <c r="B13" s="254"/>
+      <c r="C13" s="254"/>
+      <c r="D13" s="254"/>
+      <c r="E13" s="254"/>
+      <c r="F13" s="254"/>
+      <c r="G13" s="254"/>
+      <c r="H13" s="254"/>
+      <c r="I13" s="254"/>
+      <c r="J13" s="261" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="262"/>
-      <c r="L13" s="262" t="s">
+      <c r="K13" s="261"/>
+      <c r="L13" s="261" t="s">
         <v>98</v>
       </c>
-      <c r="M13" s="262"/>
-      <c r="N13" s="262" t="s">
+      <c r="M13" s="261"/>
+      <c r="N13" s="261" t="s">
         <v>99</v>
       </c>
-      <c r="O13" s="262"/>
-      <c r="P13" s="263"/>
+      <c r="O13" s="261"/>
+      <c r="P13" s="262"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="255"/>
-      <c r="C14" s="255"/>
-      <c r="D14" s="255"/>
-      <c r="E14" s="255"/>
-      <c r="F14" s="255"/>
-      <c r="G14" s="255"/>
-      <c r="H14" s="255"/>
-      <c r="I14" s="255"/>
+      <c r="B14" s="254"/>
+      <c r="C14" s="254"/>
+      <c r="D14" s="254"/>
+      <c r="E14" s="254"/>
+      <c r="F14" s="254"/>
+      <c r="G14" s="254"/>
+      <c r="H14" s="254"/>
+      <c r="I14" s="254"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -42671,7 +42632,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="263"/>
+      <c r="P14" s="262"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -43021,7 +42982,7 @@
     <mergeCell ref="I4:P5"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P49">
-    <cfRule type="expression" dxfId="1" priority="13">
+    <cfRule type="expression" dxfId="5" priority="13">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
feat(reporting): add consultant and contractor titles to identity and excel signatures
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2BBF9A4-DD3F-4B10-A4C7-C49C5E69D421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148673E3-5DC4-4721-9482-E7DD71BE303A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2137,7 +2137,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="169" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="307">
+  <cellXfs count="309">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2548,14 +2548,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2694,19 +2686,7 @@
     <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="166" fontId="26" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -3130,6 +3110,22 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma [0] 2" xfId="3" xr:uid="{5950E916-03C9-42B5-8F65-57AD3DC32531}"/>
@@ -3137,7 +3133,7 @@
     <cellStyle name="Normal 2 2 3" xfId="2" xr:uid="{25DAB206-4C06-437D-BFFA-FD21FFA5A242}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="24">
     <dxf>
       <font>
         <b/>
@@ -3148,28 +3144,6 @@
           <bgColor theme="0" tint="-0.14996795556505021"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -4270,40 +4244,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="257"/>
-      <c r="C1" s="257"/>
-      <c r="D1" s="257"/>
-      <c r="E1" s="257"/>
-      <c r="F1" s="257"/>
-      <c r="G1" s="257"/>
-      <c r="H1" s="257"/>
-      <c r="I1" s="257"/>
-      <c r="J1" s="257"/>
-      <c r="K1" s="257"/>
-      <c r="L1" s="257"/>
-      <c r="M1" s="257"/>
-      <c r="N1" s="257"/>
-      <c r="O1" s="257"/>
-      <c r="P1" s="257"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+      <c r="H1" s="252"/>
+      <c r="I1" s="252"/>
+      <c r="J1" s="252"/>
+      <c r="K1" s="252"/>
+      <c r="L1" s="252"/>
+      <c r="M1" s="252"/>
+      <c r="N1" s="252"/>
+      <c r="O1" s="252"/>
+      <c r="P1" s="252"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="255" t="s">
+      <c r="B2" s="250" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="256"/>
-      <c r="D2" s="256"/>
-      <c r="E2" s="256"/>
-      <c r="F2" s="256"/>
-      <c r="G2" s="256"/>
-      <c r="H2" s="256"/>
-      <c r="I2" s="256"/>
-      <c r="J2" s="256"/>
-      <c r="K2" s="256"/>
-      <c r="L2" s="256"/>
-      <c r="M2" s="256"/>
-      <c r="N2" s="256"/>
-      <c r="O2" s="256"/>
-      <c r="P2" s="256"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="251"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="251"/>
+      <c r="I2" s="251"/>
+      <c r="J2" s="251"/>
+      <c r="K2" s="251"/>
+      <c r="L2" s="251"/>
+      <c r="M2" s="251"/>
+      <c r="N2" s="251"/>
+      <c r="O2" s="251"/>
+      <c r="P2" s="251"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4330,16 +4304,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="263" t="s">
+      <c r="I4" s="258" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="263"/>
-      <c r="K4" s="263"/>
-      <c r="L4" s="263"/>
-      <c r="M4" s="263"/>
-      <c r="N4" s="263"/>
-      <c r="O4" s="263"/>
-      <c r="P4" s="263"/>
+      <c r="J4" s="258"/>
+      <c r="K4" s="258"/>
+      <c r="L4" s="258"/>
+      <c r="M4" s="258"/>
+      <c r="N4" s="258"/>
+      <c r="O4" s="258"/>
+      <c r="P4" s="258"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4353,14 +4327,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="263"/>
-      <c r="J5" s="263"/>
-      <c r="K5" s="263"/>
-      <c r="L5" s="263"/>
-      <c r="M5" s="263"/>
-      <c r="N5" s="263"/>
-      <c r="O5" s="263"/>
-      <c r="P5" s="263"/>
+      <c r="I5" s="258"/>
+      <c r="J5" s="258"/>
+      <c r="K5" s="258"/>
+      <c r="L5" s="258"/>
+      <c r="M5" s="258"/>
+      <c r="N5" s="258"/>
+      <c r="O5" s="258"/>
+      <c r="P5" s="258"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4495,70 +4469,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="254" t="s">
+      <c r="B12" s="249" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="254" t="s">
+      <c r="C12" s="249" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="254"/>
-      <c r="E12" s="254"/>
-      <c r="F12" s="254" t="s">
+      <c r="D12" s="249"/>
+      <c r="E12" s="249"/>
+      <c r="F12" s="249" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="254" t="s">
+      <c r="G12" s="249" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="254" t="s">
+      <c r="H12" s="249" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="254" t="s">
+      <c r="I12" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="254" t="s">
+      <c r="J12" s="249" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="254"/>
-      <c r="L12" s="254"/>
-      <c r="M12" s="254"/>
-      <c r="N12" s="254"/>
-      <c r="O12" s="254"/>
-      <c r="P12" s="262" t="s">
+      <c r="K12" s="249"/>
+      <c r="L12" s="249"/>
+      <c r="M12" s="249"/>
+      <c r="N12" s="249"/>
+      <c r="O12" s="249"/>
+      <c r="P12" s="257" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="254"/>
-      <c r="C13" s="254"/>
-      <c r="D13" s="254"/>
-      <c r="E13" s="254"/>
-      <c r="F13" s="254"/>
-      <c r="G13" s="254"/>
-      <c r="H13" s="254"/>
-      <c r="I13" s="254"/>
-      <c r="J13" s="261" t="s">
+      <c r="B13" s="249"/>
+      <c r="C13" s="249"/>
+      <c r="D13" s="249"/>
+      <c r="E13" s="249"/>
+      <c r="F13" s="249"/>
+      <c r="G13" s="249"/>
+      <c r="H13" s="249"/>
+      <c r="I13" s="249"/>
+      <c r="J13" s="256" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="261"/>
-      <c r="L13" s="261" t="s">
+      <c r="K13" s="256"/>
+      <c r="L13" s="256" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="261"/>
-      <c r="N13" s="261" t="s">
+      <c r="M13" s="256"/>
+      <c r="N13" s="256" t="s">
         <v>95</v>
       </c>
-      <c r="O13" s="261"/>
-      <c r="P13" s="262"/>
+      <c r="O13" s="256"/>
+      <c r="P13" s="257"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="254"/>
-      <c r="C14" s="254"/>
-      <c r="D14" s="254"/>
-      <c r="E14" s="254"/>
-      <c r="F14" s="254"/>
-      <c r="G14" s="254"/>
-      <c r="H14" s="254"/>
-      <c r="I14" s="254"/>
+      <c r="B14" s="249"/>
+      <c r="C14" s="249"/>
+      <c r="D14" s="249"/>
+      <c r="E14" s="249"/>
+      <c r="F14" s="249"/>
+      <c r="G14" s="249"/>
+      <c r="H14" s="249"/>
+      <c r="I14" s="249"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -4577,7 +4551,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="262"/>
+      <c r="P14" s="257"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -4973,7 +4947,7 @@
     <mergeCell ref="G12:G14"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P51">
-    <cfRule type="expression" dxfId="4" priority="14">
+    <cfRule type="expression" dxfId="0" priority="14">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5000,38 +4974,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="103.2" customHeight="1">
-      <c r="B1" s="256"/>
-      <c r="C1" s="256"/>
-      <c r="D1" s="256"/>
-      <c r="E1" s="256"/>
-      <c r="F1" s="256"/>
-      <c r="G1" s="256"/>
-      <c r="H1" s="256"/>
-      <c r="I1" s="256"/>
-      <c r="J1" s="256"/>
-      <c r="K1" s="256"/>
-      <c r="L1" s="256"/>
-      <c r="M1" s="256"/>
-      <c r="N1" s="256"/>
-      <c r="O1" s="256"/>
+      <c r="B1" s="251"/>
+      <c r="C1" s="251"/>
+      <c r="D1" s="251"/>
+      <c r="E1" s="251"/>
+      <c r="F1" s="251"/>
+      <c r="G1" s="251"/>
+      <c r="H1" s="251"/>
+      <c r="I1" s="251"/>
+      <c r="J1" s="251"/>
+      <c r="K1" s="251"/>
+      <c r="L1" s="251"/>
+      <c r="M1" s="251"/>
+      <c r="N1" s="251"/>
+      <c r="O1" s="251"/>
     </row>
     <row r="2" spans="2:15" ht="22.95" customHeight="1">
-      <c r="B2" s="264" t="s">
+      <c r="B2" s="259" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="264"/>
-      <c r="D2" s="264"/>
-      <c r="E2" s="264"/>
-      <c r="F2" s="264"/>
-      <c r="G2" s="264"/>
-      <c r="H2" s="264"/>
-      <c r="I2" s="264"/>
-      <c r="J2" s="264"/>
-      <c r="K2" s="264"/>
-      <c r="L2" s="264"/>
-      <c r="M2" s="264"/>
-      <c r="N2" s="264"/>
-      <c r="O2" s="264"/>
+      <c r="C2" s="259"/>
+      <c r="D2" s="259"/>
+      <c r="E2" s="259"/>
+      <c r="F2" s="259"/>
+      <c r="G2" s="259"/>
+      <c r="H2" s="259"/>
+      <c r="I2" s="259"/>
+      <c r="J2" s="259"/>
+      <c r="K2" s="259"/>
+      <c r="L2" s="259"/>
+      <c r="M2" s="259"/>
+      <c r="N2" s="259"/>
+      <c r="O2" s="259"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" t="s">
@@ -5083,179 +5057,179 @@
     </row>
     <row r="9" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="11" spans="2:15" s="58" customFormat="1">
-      <c r="B11" s="265" t="s">
+      <c r="B11" s="260" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="265"/>
-      <c r="D11" s="265"/>
-      <c r="E11" s="265"/>
-      <c r="G11" s="265" t="s">
+      <c r="C11" s="260"/>
+      <c r="D11" s="260"/>
+      <c r="E11" s="260"/>
+      <c r="G11" s="260" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="265"/>
-      <c r="I11" s="265"/>
-      <c r="J11" s="265"/>
-      <c r="L11" s="265" t="s">
+      <c r="H11" s="260"/>
+      <c r="I11" s="260"/>
+      <c r="J11" s="260"/>
+      <c r="L11" s="260" t="s">
         <v>105</v>
       </c>
-      <c r="M11" s="265"/>
-      <c r="N11" s="265"/>
-      <c r="O11" s="265"/>
+      <c r="M11" s="260"/>
+      <c r="N11" s="260"/>
+      <c r="O11" s="260"/>
     </row>
     <row r="12" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="13" spans="2:15">
-      <c r="B13" s="256"/>
-      <c r="C13" s="256"/>
-      <c r="D13" s="256"/>
-      <c r="E13" s="256"/>
-      <c r="G13" s="256"/>
-      <c r="H13" s="256"/>
-      <c r="I13" s="256"/>
-      <c r="J13" s="256"/>
-      <c r="L13" s="256"/>
-      <c r="M13" s="256"/>
-      <c r="N13" s="256"/>
-      <c r="O13" s="256"/>
+      <c r="B13" s="251"/>
+      <c r="C13" s="251"/>
+      <c r="D13" s="251"/>
+      <c r="E13" s="251"/>
+      <c r="G13" s="251"/>
+      <c r="H13" s="251"/>
+      <c r="I13" s="251"/>
+      <c r="J13" s="251"/>
+      <c r="L13" s="251"/>
+      <c r="M13" s="251"/>
+      <c r="N13" s="251"/>
+      <c r="O13" s="251"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="256"/>
-      <c r="C14" s="256"/>
-      <c r="D14" s="256"/>
-      <c r="E14" s="256"/>
-      <c r="G14" s="256"/>
-      <c r="H14" s="256"/>
-      <c r="I14" s="256"/>
-      <c r="J14" s="256"/>
-      <c r="L14" s="256"/>
-      <c r="M14" s="256"/>
-      <c r="N14" s="256"/>
-      <c r="O14" s="256"/>
+      <c r="B14" s="251"/>
+      <c r="C14" s="251"/>
+      <c r="D14" s="251"/>
+      <c r="E14" s="251"/>
+      <c r="G14" s="251"/>
+      <c r="H14" s="251"/>
+      <c r="I14" s="251"/>
+      <c r="J14" s="251"/>
+      <c r="L14" s="251"/>
+      <c r="M14" s="251"/>
+      <c r="N14" s="251"/>
+      <c r="O14" s="251"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="256"/>
-      <c r="C15" s="256"/>
-      <c r="D15" s="256"/>
-      <c r="E15" s="256"/>
-      <c r="G15" s="256"/>
-      <c r="H15" s="256"/>
-      <c r="I15" s="256"/>
-      <c r="J15" s="256"/>
-      <c r="L15" s="256"/>
-      <c r="M15" s="256"/>
-      <c r="N15" s="256"/>
-      <c r="O15" s="256"/>
+      <c r="B15" s="251"/>
+      <c r="C15" s="251"/>
+      <c r="D15" s="251"/>
+      <c r="E15" s="251"/>
+      <c r="G15" s="251"/>
+      <c r="H15" s="251"/>
+      <c r="I15" s="251"/>
+      <c r="J15" s="251"/>
+      <c r="L15" s="251"/>
+      <c r="M15" s="251"/>
+      <c r="N15" s="251"/>
+      <c r="O15" s="251"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="256"/>
-      <c r="C16" s="256"/>
-      <c r="D16" s="256"/>
-      <c r="E16" s="256"/>
-      <c r="G16" s="256"/>
-      <c r="H16" s="256"/>
-      <c r="I16" s="256"/>
-      <c r="J16" s="256"/>
-      <c r="L16" s="256"/>
-      <c r="M16" s="256"/>
-      <c r="N16" s="256"/>
-      <c r="O16" s="256"/>
+      <c r="B16" s="251"/>
+      <c r="C16" s="251"/>
+      <c r="D16" s="251"/>
+      <c r="E16" s="251"/>
+      <c r="G16" s="251"/>
+      <c r="H16" s="251"/>
+      <c r="I16" s="251"/>
+      <c r="J16" s="251"/>
+      <c r="L16" s="251"/>
+      <c r="M16" s="251"/>
+      <c r="N16" s="251"/>
+      <c r="O16" s="251"/>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="256"/>
-      <c r="C17" s="256"/>
-      <c r="D17" s="256"/>
-      <c r="E17" s="256"/>
-      <c r="G17" s="256"/>
-      <c r="H17" s="256"/>
-      <c r="I17" s="256"/>
-      <c r="J17" s="256"/>
-      <c r="L17" s="256"/>
-      <c r="M17" s="256"/>
-      <c r="N17" s="256"/>
-      <c r="O17" s="256"/>
+      <c r="B17" s="251"/>
+      <c r="C17" s="251"/>
+      <c r="D17" s="251"/>
+      <c r="E17" s="251"/>
+      <c r="G17" s="251"/>
+      <c r="H17" s="251"/>
+      <c r="I17" s="251"/>
+      <c r="J17" s="251"/>
+      <c r="L17" s="251"/>
+      <c r="M17" s="251"/>
+      <c r="N17" s="251"/>
+      <c r="O17" s="251"/>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="256"/>
-      <c r="C18" s="256"/>
-      <c r="D18" s="256"/>
-      <c r="E18" s="256"/>
-      <c r="G18" s="256"/>
-      <c r="H18" s="256"/>
-      <c r="I18" s="256"/>
-      <c r="J18" s="256"/>
-      <c r="L18" s="256"/>
-      <c r="M18" s="256"/>
-      <c r="N18" s="256"/>
-      <c r="O18" s="256"/>
+      <c r="B18" s="251"/>
+      <c r="C18" s="251"/>
+      <c r="D18" s="251"/>
+      <c r="E18" s="251"/>
+      <c r="G18" s="251"/>
+      <c r="H18" s="251"/>
+      <c r="I18" s="251"/>
+      <c r="J18" s="251"/>
+      <c r="L18" s="251"/>
+      <c r="M18" s="251"/>
+      <c r="N18" s="251"/>
+      <c r="O18" s="251"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="B19" s="256"/>
-      <c r="C19" s="256"/>
-      <c r="D19" s="256"/>
-      <c r="E19" s="256"/>
-      <c r="G19" s="256"/>
-      <c r="H19" s="256"/>
-      <c r="I19" s="256"/>
-      <c r="J19" s="256"/>
-      <c r="L19" s="256"/>
-      <c r="M19" s="256"/>
-      <c r="N19" s="256"/>
-      <c r="O19" s="256"/>
+      <c r="B19" s="251"/>
+      <c r="C19" s="251"/>
+      <c r="D19" s="251"/>
+      <c r="E19" s="251"/>
+      <c r="G19" s="251"/>
+      <c r="H19" s="251"/>
+      <c r="I19" s="251"/>
+      <c r="J19" s="251"/>
+      <c r="L19" s="251"/>
+      <c r="M19" s="251"/>
+      <c r="N19" s="251"/>
+      <c r="O19" s="251"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="B20" s="256"/>
-      <c r="C20" s="256"/>
-      <c r="D20" s="256"/>
-      <c r="E20" s="256"/>
-      <c r="G20" s="256"/>
-      <c r="H20" s="256"/>
-      <c r="I20" s="256"/>
-      <c r="J20" s="256"/>
-      <c r="L20" s="256"/>
-      <c r="M20" s="256"/>
-      <c r="N20" s="256"/>
-      <c r="O20" s="256"/>
+      <c r="B20" s="251"/>
+      <c r="C20" s="251"/>
+      <c r="D20" s="251"/>
+      <c r="E20" s="251"/>
+      <c r="G20" s="251"/>
+      <c r="H20" s="251"/>
+      <c r="I20" s="251"/>
+      <c r="J20" s="251"/>
+      <c r="L20" s="251"/>
+      <c r="M20" s="251"/>
+      <c r="N20" s="251"/>
+      <c r="O20" s="251"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="B21" s="256"/>
-      <c r="C21" s="256"/>
-      <c r="D21" s="256"/>
-      <c r="E21" s="256"/>
-      <c r="G21" s="256"/>
-      <c r="H21" s="256"/>
-      <c r="I21" s="256"/>
-      <c r="J21" s="256"/>
-      <c r="L21" s="256"/>
-      <c r="M21" s="256"/>
-      <c r="N21" s="256"/>
-      <c r="O21" s="256"/>
+      <c r="B21" s="251"/>
+      <c r="C21" s="251"/>
+      <c r="D21" s="251"/>
+      <c r="E21" s="251"/>
+      <c r="G21" s="251"/>
+      <c r="H21" s="251"/>
+      <c r="I21" s="251"/>
+      <c r="J21" s="251"/>
+      <c r="L21" s="251"/>
+      <c r="M21" s="251"/>
+      <c r="N21" s="251"/>
+      <c r="O21" s="251"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="B22" s="256"/>
-      <c r="C22" s="256"/>
-      <c r="D22" s="256"/>
-      <c r="E22" s="256"/>
-      <c r="G22" s="256"/>
-      <c r="H22" s="256"/>
-      <c r="I22" s="256"/>
-      <c r="J22" s="256"/>
-      <c r="L22" s="256"/>
-      <c r="M22" s="256"/>
-      <c r="N22" s="256"/>
-      <c r="O22" s="256"/>
+      <c r="B22" s="251"/>
+      <c r="C22" s="251"/>
+      <c r="D22" s="251"/>
+      <c r="E22" s="251"/>
+      <c r="G22" s="251"/>
+      <c r="H22" s="251"/>
+      <c r="I22" s="251"/>
+      <c r="J22" s="251"/>
+      <c r="L22" s="251"/>
+      <c r="M22" s="251"/>
+      <c r="N22" s="251"/>
+      <c r="O22" s="251"/>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="256"/>
-      <c r="C23" s="256"/>
-      <c r="D23" s="256"/>
-      <c r="E23" s="256"/>
-      <c r="G23" s="256"/>
-      <c r="H23" s="256"/>
-      <c r="I23" s="256"/>
-      <c r="J23" s="256"/>
-      <c r="L23" s="256"/>
-      <c r="M23" s="256"/>
-      <c r="N23" s="256"/>
-      <c r="O23" s="256"/>
+      <c r="B23" s="251"/>
+      <c r="C23" s="251"/>
+      <c r="D23" s="251"/>
+      <c r="E23" s="251"/>
+      <c r="G23" s="251"/>
+      <c r="H23" s="251"/>
+      <c r="I23" s="251"/>
+      <c r="J23" s="251"/>
+      <c r="L23" s="251"/>
+      <c r="M23" s="251"/>
+      <c r="N23" s="251"/>
+      <c r="O23" s="251"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5289,330 +5263,330 @@
   <sheetData>
     <row r="1" spans="2:29" ht="4.8" customHeight="1" thickBot="1"/>
     <row r="2" spans="2:29" ht="19.95" customHeight="1" thickBot="1">
-      <c r="B2" s="266" t="s">
+      <c r="B2" s="261" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="267"/>
-      <c r="D2" s="267"/>
-      <c r="E2" s="267"/>
-      <c r="F2" s="267"/>
-      <c r="G2" s="267"/>
-      <c r="H2" s="267"/>
-      <c r="I2" s="267"/>
-      <c r="J2" s="267"/>
-      <c r="K2" s="267"/>
-      <c r="L2" s="267"/>
-      <c r="M2" s="267"/>
-      <c r="N2" s="267"/>
-      <c r="O2" s="267"/>
-      <c r="P2" s="267"/>
-      <c r="Q2" s="267"/>
-      <c r="R2" s="267"/>
-      <c r="S2" s="267"/>
-      <c r="T2" s="267"/>
-      <c r="U2" s="267"/>
-      <c r="V2" s="267"/>
-      <c r="W2" s="267"/>
-      <c r="X2" s="267"/>
-      <c r="Y2" s="267"/>
-      <c r="Z2" s="267"/>
-      <c r="AA2" s="267"/>
-      <c r="AB2" s="268"/>
-      <c r="AC2" s="140"/>
+      <c r="C2" s="262"/>
+      <c r="D2" s="262"/>
+      <c r="E2" s="262"/>
+      <c r="F2" s="262"/>
+      <c r="G2" s="262"/>
+      <c r="H2" s="262"/>
+      <c r="I2" s="262"/>
+      <c r="J2" s="262"/>
+      <c r="K2" s="262"/>
+      <c r="L2" s="262"/>
+      <c r="M2" s="262"/>
+      <c r="N2" s="262"/>
+      <c r="O2" s="262"/>
+      <c r="P2" s="262"/>
+      <c r="Q2" s="262"/>
+      <c r="R2" s="262"/>
+      <c r="S2" s="262"/>
+      <c r="T2" s="262"/>
+      <c r="U2" s="262"/>
+      <c r="V2" s="262"/>
+      <c r="W2" s="262"/>
+      <c r="X2" s="262"/>
+      <c r="Y2" s="262"/>
+      <c r="Z2" s="262"/>
+      <c r="AA2" s="262"/>
+      <c r="AB2" s="263"/>
+      <c r="AC2" s="138"/>
     </row>
     <row r="3" spans="2:29" ht="15" customHeight="1">
-      <c r="B3" s="139"/>
-      <c r="AB3" s="134"/>
+      <c r="B3" s="137"/>
+      <c r="AB3" s="132"/>
     </row>
     <row r="4" spans="2:29" ht="15" customHeight="1">
-      <c r="B4" s="133" t="s">
+      <c r="B4" s="131" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="135" t="s">
+      <c r="D4" s="133" t="s">
         <v>20</v>
       </c>
-      <c r="AB4" s="134"/>
+      <c r="AB4" s="132"/>
     </row>
     <row r="5" spans="2:29" ht="15" customHeight="1">
-      <c r="B5" s="133" t="s">
+      <c r="B5" s="131" t="s">
         <v>108</v>
       </c>
-      <c r="D5" s="135" t="s">
+      <c r="D5" s="133" t="s">
         <v>20</v>
       </c>
-      <c r="AB5" s="134"/>
+      <c r="AB5" s="132"/>
     </row>
     <row r="6" spans="2:29" ht="15" customHeight="1">
-      <c r="B6" s="133" t="s">
+      <c r="B6" s="131" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="135" t="s">
+      <c r="D6" s="133" t="s">
         <v>20</v>
       </c>
-      <c r="AB6" s="134"/>
+      <c r="AB6" s="132"/>
     </row>
     <row r="7" spans="2:29" ht="15" customHeight="1">
-      <c r="B7" s="133" t="s">
+      <c r="B7" s="131" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="135" t="s">
+      <c r="D7" s="133" t="s">
         <v>20</v>
       </c>
-      <c r="AB7" s="134"/>
+      <c r="AB7" s="132"/>
     </row>
     <row r="8" spans="2:29" ht="15" customHeight="1">
-      <c r="B8" s="133" t="s">
+      <c r="B8" s="131" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="135" t="s">
+      <c r="D8" s="133" t="s">
         <v>20</v>
       </c>
-      <c r="AB8" s="134"/>
+      <c r="AB8" s="132"/>
     </row>
     <row r="9" spans="2:29" ht="15" customHeight="1">
-      <c r="B9" s="133" t="s">
+      <c r="B9" s="131" t="s">
         <v>110</v>
       </c>
-      <c r="D9" s="135" t="s">
+      <c r="D9" s="133" t="s">
         <v>20</v>
       </c>
-      <c r="AB9" s="134"/>
+      <c r="AB9" s="132"/>
     </row>
     <row r="10" spans="2:29" ht="15" customHeight="1">
-      <c r="B10" s="133" t="s">
+      <c r="B10" s="131" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="135" t="s">
+      <c r="D10" s="133" t="s">
         <v>20</v>
       </c>
-      <c r="AB10" s="134"/>
+      <c r="AB10" s="132"/>
     </row>
     <row r="11" spans="2:29" ht="15" customHeight="1" thickBot="1">
-      <c r="B11" s="136"/>
-      <c r="C11" s="137"/>
-      <c r="D11" s="137"/>
-      <c r="E11" s="137"/>
-      <c r="F11" s="137"/>
-      <c r="G11" s="137"/>
-      <c r="H11" s="137"/>
-      <c r="I11" s="137"/>
-      <c r="J11" s="137"/>
-      <c r="K11" s="137"/>
-      <c r="L11" s="137"/>
-      <c r="M11" s="137"/>
-      <c r="N11" s="137"/>
-      <c r="O11" s="137"/>
-      <c r="P11" s="137"/>
-      <c r="Q11" s="137"/>
-      <c r="R11" s="137"/>
-      <c r="S11" s="137"/>
-      <c r="T11" s="137"/>
-      <c r="U11" s="137"/>
-      <c r="V11" s="137"/>
-      <c r="W11" s="137"/>
-      <c r="X11" s="137"/>
-      <c r="Y11" s="137"/>
-      <c r="Z11" s="137"/>
-      <c r="AA11" s="137"/>
-      <c r="AB11" s="138"/>
+      <c r="B11" s="134"/>
+      <c r="C11" s="135"/>
+      <c r="D11" s="135"/>
+      <c r="E11" s="135"/>
+      <c r="F11" s="135"/>
+      <c r="G11" s="135"/>
+      <c r="H11" s="135"/>
+      <c r="I11" s="135"/>
+      <c r="J11" s="135"/>
+      <c r="K11" s="135"/>
+      <c r="L11" s="135"/>
+      <c r="M11" s="135"/>
+      <c r="N11" s="135"/>
+      <c r="O11" s="135"/>
+      <c r="P11" s="135"/>
+      <c r="Q11" s="135"/>
+      <c r="R11" s="135"/>
+      <c r="S11" s="135"/>
+      <c r="T11" s="135"/>
+      <c r="U11" s="135"/>
+      <c r="V11" s="135"/>
+      <c r="W11" s="135"/>
+      <c r="X11" s="135"/>
+      <c r="Y11" s="135"/>
+      <c r="Z11" s="135"/>
+      <c r="AA11" s="135"/>
+      <c r="AB11" s="136"/>
     </row>
     <row r="12" spans="2:29" ht="15" customHeight="1">
-      <c r="B12" s="278" t="s">
+      <c r="B12" s="273" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="280" t="s">
+      <c r="C12" s="275" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="281"/>
-      <c r="E12" s="281"/>
-      <c r="F12" s="281"/>
-      <c r="G12" s="281"/>
-      <c r="H12" s="281"/>
-      <c r="I12" s="281"/>
-      <c r="J12" s="281"/>
-      <c r="K12" s="281"/>
-      <c r="L12" s="282"/>
-      <c r="M12" s="286" t="s">
+      <c r="D12" s="276"/>
+      <c r="E12" s="276"/>
+      <c r="F12" s="276"/>
+      <c r="G12" s="276"/>
+      <c r="H12" s="276"/>
+      <c r="I12" s="276"/>
+      <c r="J12" s="276"/>
+      <c r="K12" s="276"/>
+      <c r="L12" s="277"/>
+      <c r="M12" s="281" t="s">
         <v>113</v>
       </c>
-      <c r="N12" s="286" t="s">
+      <c r="N12" s="281" t="s">
         <v>34</v>
       </c>
-      <c r="O12" s="291" t="s">
+      <c r="O12" s="286" t="s">
         <v>114</v>
       </c>
-      <c r="P12" s="291"/>
-      <c r="Q12" s="291"/>
-      <c r="R12" s="291"/>
-      <c r="S12" s="291"/>
-      <c r="T12" s="291"/>
-      <c r="U12" s="291"/>
-      <c r="V12" s="291"/>
-      <c r="W12" s="291"/>
-      <c r="X12" s="291"/>
-      <c r="Y12" s="291"/>
-      <c r="Z12" s="291"/>
-      <c r="AA12" s="291"/>
-      <c r="AB12" s="292"/>
+      <c r="P12" s="286"/>
+      <c r="Q12" s="286"/>
+      <c r="R12" s="286"/>
+      <c r="S12" s="286"/>
+      <c r="T12" s="286"/>
+      <c r="U12" s="286"/>
+      <c r="V12" s="286"/>
+      <c r="W12" s="286"/>
+      <c r="X12" s="286"/>
+      <c r="Y12" s="286"/>
+      <c r="Z12" s="286"/>
+      <c r="AA12" s="286"/>
+      <c r="AB12" s="287"/>
     </row>
     <row r="13" spans="2:29" ht="15" customHeight="1">
-      <c r="B13" s="279"/>
-      <c r="C13" s="283"/>
-      <c r="D13" s="284"/>
-      <c r="E13" s="284"/>
-      <c r="F13" s="284"/>
-      <c r="G13" s="284"/>
-      <c r="H13" s="284"/>
-      <c r="I13" s="284"/>
-      <c r="J13" s="284"/>
-      <c r="K13" s="284"/>
-      <c r="L13" s="285"/>
-      <c r="M13" s="287"/>
-      <c r="N13" s="287"/>
-      <c r="O13" s="288" t="s">
+      <c r="B13" s="274"/>
+      <c r="C13" s="278"/>
+      <c r="D13" s="279"/>
+      <c r="E13" s="279"/>
+      <c r="F13" s="279"/>
+      <c r="G13" s="279"/>
+      <c r="H13" s="279"/>
+      <c r="I13" s="279"/>
+      <c r="J13" s="279"/>
+      <c r="K13" s="279"/>
+      <c r="L13" s="280"/>
+      <c r="M13" s="282"/>
+      <c r="N13" s="282"/>
+      <c r="O13" s="283" t="s">
         <v>115</v>
       </c>
-      <c r="P13" s="289"/>
-      <c r="Q13" s="290"/>
-      <c r="R13" s="288" t="s">
+      <c r="P13" s="284"/>
+      <c r="Q13" s="285"/>
+      <c r="R13" s="283" t="s">
         <v>116</v>
       </c>
-      <c r="S13" s="289"/>
-      <c r="T13" s="290"/>
-      <c r="U13" s="288" t="s">
+      <c r="S13" s="284"/>
+      <c r="T13" s="285"/>
+      <c r="U13" s="283" t="s">
         <v>117</v>
       </c>
-      <c r="V13" s="289"/>
-      <c r="W13" s="290"/>
-      <c r="X13" s="269" t="s">
+      <c r="V13" s="284"/>
+      <c r="W13" s="285"/>
+      <c r="X13" s="264" t="s">
         <v>118</v>
       </c>
-      <c r="Y13" s="145" t="s">
+      <c r="Y13" s="143" t="s">
         <v>119</v>
       </c>
-      <c r="Z13" s="146" t="s">
+      <c r="Z13" s="144" t="s">
         <v>119</v>
       </c>
-      <c r="AA13" s="271" t="s">
+      <c r="AA13" s="266" t="s">
         <v>120</v>
       </c>
-      <c r="AB13" s="273" t="s">
+      <c r="AB13" s="268" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="14" spans="2:29" ht="15" customHeight="1">
-      <c r="B14" s="279"/>
-      <c r="C14" s="283"/>
-      <c r="D14" s="284"/>
-      <c r="E14" s="284"/>
-      <c r="F14" s="284"/>
-      <c r="G14" s="284"/>
-      <c r="H14" s="284"/>
-      <c r="I14" s="284"/>
-      <c r="J14" s="284"/>
-      <c r="K14" s="284"/>
-      <c r="L14" s="285"/>
-      <c r="M14" s="270"/>
-      <c r="N14" s="270"/>
-      <c r="O14" s="147" t="s">
+      <c r="B14" s="274"/>
+      <c r="C14" s="278"/>
+      <c r="D14" s="279"/>
+      <c r="E14" s="279"/>
+      <c r="F14" s="279"/>
+      <c r="G14" s="279"/>
+      <c r="H14" s="279"/>
+      <c r="I14" s="279"/>
+      <c r="J14" s="279"/>
+      <c r="K14" s="279"/>
+      <c r="L14" s="280"/>
+      <c r="M14" s="265"/>
+      <c r="N14" s="265"/>
+      <c r="O14" s="145" t="s">
         <v>122</v>
       </c>
-      <c r="P14" s="147" t="s">
+      <c r="P14" s="145" t="s">
         <v>123</v>
       </c>
-      <c r="Q14" s="147" t="s">
+      <c r="Q14" s="145" t="s">
         <v>124</v>
       </c>
-      <c r="R14" s="147" t="s">
+      <c r="R14" s="145" t="s">
         <v>125</v>
       </c>
-      <c r="S14" s="147" t="s">
+      <c r="S14" s="145" t="s">
         <v>126</v>
       </c>
-      <c r="T14" s="147" t="s">
+      <c r="T14" s="145" t="s">
         <v>124</v>
       </c>
-      <c r="U14" s="147" t="s">
+      <c r="U14" s="145" t="s">
         <v>127</v>
       </c>
-      <c r="V14" s="147" t="s">
+      <c r="V14" s="145" t="s">
         <v>128</v>
       </c>
-      <c r="W14" s="147" t="s">
+      <c r="W14" s="145" t="s">
         <v>129</v>
       </c>
-      <c r="X14" s="270"/>
-      <c r="Y14" s="145" t="s">
+      <c r="X14" s="265"/>
+      <c r="Y14" s="143" t="s">
         <v>130</v>
       </c>
-      <c r="Z14" s="147" t="s">
+      <c r="Z14" s="145" t="s">
         <v>131</v>
       </c>
-      <c r="AA14" s="272"/>
-      <c r="AB14" s="274"/>
+      <c r="AA14" s="267"/>
+      <c r="AB14" s="269"/>
     </row>
     <row r="15" spans="2:29" ht="15" customHeight="1" thickBot="1">
-      <c r="B15" s="141">
+      <c r="B15" s="139">
         <v>1</v>
       </c>
-      <c r="C15" s="275">
+      <c r="C15" s="270">
         <v>2</v>
       </c>
-      <c r="D15" s="276"/>
-      <c r="E15" s="276"/>
-      <c r="F15" s="276"/>
-      <c r="G15" s="276"/>
-      <c r="H15" s="276"/>
-      <c r="I15" s="276"/>
-      <c r="J15" s="276"/>
-      <c r="K15" s="276"/>
-      <c r="L15" s="277"/>
-      <c r="M15" s="142">
+      <c r="D15" s="271"/>
+      <c r="E15" s="271"/>
+      <c r="F15" s="271"/>
+      <c r="G15" s="271"/>
+      <c r="H15" s="271"/>
+      <c r="I15" s="271"/>
+      <c r="J15" s="271"/>
+      <c r="K15" s="271"/>
+      <c r="L15" s="272"/>
+      <c r="M15" s="140">
         <v>3</v>
       </c>
-      <c r="N15" s="142">
+      <c r="N15" s="140">
         <v>4</v>
       </c>
-      <c r="O15" s="143">
+      <c r="O15" s="141">
         <v>5</v>
       </c>
-      <c r="P15" s="143">
+      <c r="P15" s="141">
         <v>6</v>
       </c>
-      <c r="Q15" s="143">
+      <c r="Q15" s="141">
         <v>7</v>
       </c>
-      <c r="R15" s="143">
+      <c r="R15" s="141">
         <v>8</v>
       </c>
-      <c r="S15" s="143">
+      <c r="S15" s="141">
         <v>9</v>
       </c>
-      <c r="T15" s="143">
+      <c r="T15" s="141">
         <v>10</v>
       </c>
-      <c r="U15" s="143">
+      <c r="U15" s="141">
         <v>11</v>
       </c>
-      <c r="V15" s="143">
+      <c r="V15" s="141">
         <v>12</v>
       </c>
-      <c r="W15" s="143">
+      <c r="W15" s="141">
         <v>13</v>
       </c>
-      <c r="X15" s="143">
+      <c r="X15" s="141">
         <v>14</v>
       </c>
-      <c r="Y15" s="143">
+      <c r="Y15" s="141">
         <v>15</v>
       </c>
-      <c r="Z15" s="143">
+      <c r="Z15" s="141">
         <v>16</v>
       </c>
-      <c r="AA15" s="143">
+      <c r="AA15" s="141">
         <v>17</v>
       </c>
-      <c r="AB15" s="144">
+      <c r="AB15" s="142">
         <v>18</v>
       </c>
     </row>
@@ -5656,38 +5630,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="253"/>
-      <c r="C1" s="253"/>
-      <c r="D1" s="253"/>
-      <c r="E1" s="253"/>
-      <c r="F1" s="253"/>
-      <c r="G1" s="253"/>
-      <c r="H1" s="253"/>
-      <c r="I1" s="253"/>
+      <c r="B1" s="248"/>
+      <c r="C1" s="248"/>
+      <c r="D1" s="248"/>
+      <c r="E1" s="248"/>
+      <c r="F1" s="248"/>
+      <c r="G1" s="248"/>
+      <c r="H1" s="248"/>
+      <c r="I1" s="248"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="250" t="s">
+      <c r="B2" s="245" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="250"/>
-      <c r="D2" s="250"/>
-      <c r="E2" s="250"/>
-      <c r="F2" s="250"/>
-      <c r="G2" s="250"/>
-      <c r="H2" s="250"/>
-      <c r="I2" s="250"/>
+      <c r="C2" s="245"/>
+      <c r="D2" s="245"/>
+      <c r="E2" s="245"/>
+      <c r="F2" s="245"/>
+      <c r="G2" s="245"/>
+      <c r="H2" s="245"/>
+      <c r="I2" s="245"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="251" t="s">
+      <c r="B3" s="246" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="251"/>
-      <c r="D3" s="251"/>
-      <c r="E3" s="251"/>
-      <c r="F3" s="251"/>
-      <c r="G3" s="251"/>
-      <c r="H3" s="251"/>
-      <c r="I3" s="251"/>
+      <c r="C3" s="246"/>
+      <c r="D3" s="246"/>
+      <c r="E3" s="246"/>
+      <c r="F3" s="246"/>
+      <c r="G3" s="246"/>
+      <c r="H3" s="246"/>
+      <c r="I3" s="246"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -5695,10 +5669,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="252" t="s">
+      <c r="C5" s="247" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="252"/>
+      <c r="D5" s="247"/>
       <c r="E5" s="11" t="s">
         <v>38</v>
       </c>
@@ -14052,7 +14026,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="26" priority="2">
+    <cfRule type="expression" dxfId="23" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14085,63 +14059,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="253"/>
-      <c r="C1" s="253"/>
-      <c r="D1" s="253"/>
-      <c r="E1" s="253"/>
-      <c r="F1" s="253"/>
-      <c r="G1" s="253"/>
-      <c r="H1" s="253"/>
-      <c r="I1" s="253"/>
-      <c r="J1" s="253"/>
-      <c r="K1" s="253"/>
-      <c r="L1" s="253"/>
-      <c r="M1" s="253"/>
-      <c r="N1" s="253"/>
+      <c r="B1" s="248"/>
+      <c r="C1" s="248"/>
+      <c r="D1" s="248"/>
+      <c r="E1" s="248"/>
+      <c r="F1" s="248"/>
+      <c r="G1" s="248"/>
+      <c r="H1" s="248"/>
+      <c r="I1" s="248"/>
+      <c r="J1" s="248"/>
+      <c r="K1" s="248"/>
+      <c r="L1" s="248"/>
+      <c r="M1" s="248"/>
+      <c r="N1" s="248"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="250" t="s">
+      <c r="B2" s="245" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="250"/>
-      <c r="D2" s="250"/>
-      <c r="E2" s="250"/>
-      <c r="F2" s="250"/>
-      <c r="G2" s="250"/>
-      <c r="H2" s="250"/>
-      <c r="I2" s="250"/>
-      <c r="J2" s="250"/>
-      <c r="K2" s="250"/>
-      <c r="L2" s="250"/>
-      <c r="M2" s="250"/>
-      <c r="N2" s="250"/>
+      <c r="C2" s="245"/>
+      <c r="D2" s="245"/>
+      <c r="E2" s="245"/>
+      <c r="F2" s="245"/>
+      <c r="G2" s="245"/>
+      <c r="H2" s="245"/>
+      <c r="I2" s="245"/>
+      <c r="J2" s="245"/>
+      <c r="K2" s="245"/>
+      <c r="L2" s="245"/>
+      <c r="M2" s="245"/>
+      <c r="N2" s="245"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="251" t="s">
+      <c r="B3" s="246" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="251"/>
-      <c r="D3" s="251"/>
-      <c r="E3" s="251"/>
-      <c r="F3" s="251"/>
-      <c r="G3" s="251"/>
-      <c r="H3" s="251"/>
-      <c r="I3" s="251"/>
-      <c r="J3" s="251"/>
-      <c r="K3" s="251"/>
-      <c r="L3" s="251"/>
-      <c r="M3" s="251"/>
-      <c r="N3" s="251"/>
+      <c r="C3" s="246"/>
+      <c r="D3" s="246"/>
+      <c r="E3" s="246"/>
+      <c r="F3" s="246"/>
+      <c r="G3" s="246"/>
+      <c r="H3" s="246"/>
+      <c r="I3" s="246"/>
+      <c r="J3" s="246"/>
+      <c r="K3" s="246"/>
+      <c r="L3" s="246"/>
+      <c r="M3" s="246"/>
+      <c r="N3" s="246"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="254" t="s">
+      <c r="C5" s="249" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="254"/>
+      <c r="D5" s="249"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -16302,23 +16276,23 @@
     <mergeCell ref="B1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:N16997">
-    <cfRule type="expression" dxfId="25" priority="1">
+    <cfRule type="expression" dxfId="22" priority="1">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="2">
+    <cfRule type="expression" dxfId="21" priority="2">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="5">
+    <cfRule type="expression" dxfId="20" priority="5">
       <formula>AND($B6="",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H16997">
-    <cfRule type="expression" dxfId="22" priority="9">
+    <cfRule type="expression" dxfId="19" priority="9">
       <formula>IF(G6&lt;&gt;"", NOT(AND(OR(LEFT($E6,2)="L.", LEFT($E6,2)="A.", LEFT($E6,2)="B.", LEFT($E6,2)="M."), $H6&lt;&gt;"", $E6&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:K16997">
-    <cfRule type="notContainsBlanks" dxfId="21" priority="8">
+    <cfRule type="notContainsBlanks" dxfId="18" priority="8">
       <formula>LEN(TRIM(H6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16345,35 +16319,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="253"/>
-      <c r="C1" s="253"/>
-      <c r="D1" s="253"/>
-      <c r="E1" s="253"/>
-      <c r="F1" s="253"/>
-      <c r="G1" s="253"/>
-      <c r="H1" s="253"/>
+      <c r="B1" s="248"/>
+      <c r="C1" s="248"/>
+      <c r="D1" s="248"/>
+      <c r="E1" s="248"/>
+      <c r="F1" s="248"/>
+      <c r="G1" s="248"/>
+      <c r="H1" s="248"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="250" t="s">
+      <c r="B2" s="245" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="250"/>
-      <c r="D2" s="250"/>
-      <c r="E2" s="250"/>
-      <c r="F2" s="250"/>
-      <c r="G2" s="250"/>
-      <c r="H2" s="250"/>
+      <c r="C2" s="245"/>
+      <c r="D2" s="245"/>
+      <c r="E2" s="245"/>
+      <c r="F2" s="245"/>
+      <c r="G2" s="245"/>
+      <c r="H2" s="245"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="251" t="s">
+      <c r="B3" s="246" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="251"/>
-      <c r="D3" s="251"/>
-      <c r="E3" s="251"/>
-      <c r="F3" s="251"/>
-      <c r="G3" s="251"/>
-      <c r="H3" s="251"/>
+      <c r="C3" s="246"/>
+      <c r="D3" s="246"/>
+      <c r="E3" s="246"/>
+      <c r="F3" s="246"/>
+      <c r="G3" s="246"/>
+      <c r="H3" s="246"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -40421,18 +40395,18 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B995 E6:H995">
-    <cfRule type="expression" dxfId="20" priority="7">
+    <cfRule type="expression" dxfId="17" priority="7">
       <formula>$J6=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:H995">
-    <cfRule type="expression" dxfId="19" priority="1">
+    <cfRule type="expression" dxfId="16" priority="1">
       <formula>AND(LEN($B6)=1,$C6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="15" priority="2">
       <formula>AND($C6="",$B6&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="3">
+    <cfRule type="expression" dxfId="14" priority="3">
       <formula>AND($B6&lt;&gt;"",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -40467,30 +40441,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="257"/>
-      <c r="C1" s="257"/>
-      <c r="D1" s="257"/>
-      <c r="E1" s="257"/>
-      <c r="F1" s="257"/>
-      <c r="G1" s="257"/>
-      <c r="H1" s="257"/>
-      <c r="I1" s="257"/>
-      <c r="J1" s="257"/>
-      <c r="K1" s="257"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+      <c r="H1" s="252"/>
+      <c r="I1" s="252"/>
+      <c r="J1" s="252"/>
+      <c r="K1" s="252"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="255" t="s">
+      <c r="B2" s="250" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="256"/>
-      <c r="D2" s="256"/>
-      <c r="E2" s="256"/>
-      <c r="F2" s="256"/>
-      <c r="G2" s="256"/>
-      <c r="H2" s="256"/>
-      <c r="I2" s="256"/>
-      <c r="J2" s="256"/>
-      <c r="K2" s="256"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="251"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="251"/>
+      <c r="I2" s="251"/>
+      <c r="J2" s="251"/>
+      <c r="K2" s="251"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40610,11 +40584,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="254" t="s">
+      <c r="C11" s="249" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="254"/>
-      <c r="E11" s="254"/>
+      <c r="D11" s="249"/>
+      <c r="E11" s="249"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -40670,26 +40644,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="111.6" customHeight="1">
-      <c r="B1" s="257"/>
-      <c r="C1" s="257"/>
-      <c r="D1" s="257"/>
-      <c r="E1" s="257"/>
-      <c r="F1" s="257"/>
-      <c r="G1" s="257"/>
-      <c r="H1" s="257"/>
-      <c r="I1" s="257"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+      <c r="H1" s="252"/>
+      <c r="I1" s="252"/>
     </row>
     <row r="2" spans="2:9" ht="22.95" customHeight="1">
-      <c r="B2" s="255" t="s">
+      <c r="B2" s="250" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="256"/>
-      <c r="D2" s="256"/>
-      <c r="E2" s="256"/>
-      <c r="F2" s="256"/>
-      <c r="G2" s="256"/>
-      <c r="H2" s="256"/>
-      <c r="I2" s="256"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="251"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="251"/>
+      <c r="I2" s="251"/>
     </row>
     <row r="3" spans="2:9" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40799,12 +40773,12 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="254" t="s">
+      <c r="C11" s="249" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="254"/>
-      <c r="E11" s="254"/>
-      <c r="F11" s="254"/>
+      <c r="D11" s="249"/>
+      <c r="E11" s="249"/>
+      <c r="F11" s="249"/>
       <c r="G11" s="40" t="s">
         <v>29</v>
       </c>
@@ -40842,58 +40816,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="257"/>
-      <c r="C1" s="257"/>
-      <c r="D1" s="257"/>
-      <c r="E1" s="257"/>
-      <c r="F1" s="257"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="260" t="s">
+      <c r="B2" s="255" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="260"/>
-      <c r="D2" s="260"/>
-      <c r="E2" s="260"/>
-      <c r="F2" s="260"/>
+      <c r="C2" s="255"/>
+      <c r="D2" s="255"/>
+      <c r="E2" s="255"/>
+      <c r="F2" s="255"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="257"/>
-      <c r="C3" s="257"/>
-      <c r="D3" s="257"/>
-      <c r="E3" s="257"/>
-      <c r="F3" s="257"/>
+      <c r="B3" s="252"/>
+      <c r="C3" s="252"/>
+      <c r="D3" s="252"/>
+      <c r="E3" s="252"/>
+      <c r="F3" s="252"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="258" t="s">
+      <c r="B5" s="253" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="258" t="s">
+      <c r="C5" s="253" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="258" t="s">
+      <c r="D5" s="253" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="259" t="s">
+      <c r="E5" s="254" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="259" t="s">
+      <c r="F5" s="254" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="258"/>
-      <c r="C6" s="258"/>
-      <c r="D6" s="258"/>
-      <c r="E6" s="259"/>
-      <c r="F6" s="259"/>
+      <c r="B6" s="253"/>
+      <c r="C6" s="253"/>
+      <c r="D6" s="253"/>
+      <c r="E6" s="254"/>
+      <c r="F6" s="254"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="258"/>
-      <c r="C7" s="258"/>
-      <c r="D7" s="258"/>
-      <c r="E7" s="259"/>
-      <c r="F7" s="259"/>
+      <c r="B7" s="253"/>
+      <c r="C7" s="253"/>
+      <c r="D7" s="253"/>
+      <c r="E7" s="254"/>
+      <c r="F7" s="254"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -40941,39 +40915,39 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:CE7">
-    <cfRule type="expression" dxfId="16" priority="12">
+    <cfRule type="expression" dxfId="13" priority="12">
       <formula>B5&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:CE201">
-    <cfRule type="expression" dxfId="15" priority="1">
+    <cfRule type="expression" dxfId="12" priority="1">
       <formula>AND(G8&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="2">
+    <cfRule type="expression" dxfId="11" priority="2">
       <formula>AND(G$7&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="3">
+    <cfRule type="expression" dxfId="10" priority="3">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="4">
+    <cfRule type="expression" dxfId="9" priority="4">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="5">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>AND(G8&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="6">
+    <cfRule type="expression" dxfId="7" priority="6">
       <formula>AND(G$7&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="7">
+    <cfRule type="expression" dxfId="6" priority="7">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="8">
+    <cfRule type="expression" dxfId="5" priority="8">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="10">
+    <cfRule type="expression" dxfId="3" priority="10">
       <formula>AND(G$7&lt;&gt;"",$B8="DEVIASI")</formula>
     </cfRule>
     <cfRule type="colorScale" priority="11">
@@ -40998,7 +40972,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88F31D85-A709-474B-AD17-FD7EE521F5B5}">
-  <dimension ref="A1:M72"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="1.21875" customWidth="1"/>
@@ -41014,45 +40988,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="152"/>
-      <c r="C1" s="153"/>
-      <c r="D1" s="153"/>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="153"/>
-      <c r="H1" s="153"/>
-      <c r="I1" s="153"/>
-      <c r="J1" s="153"/>
-      <c r="K1" s="153"/>
-      <c r="L1" s="154"/>
+      <c r="B1" s="150"/>
+      <c r="C1" s="151"/>
+      <c r="D1" s="151"/>
+      <c r="E1" s="151"/>
+      <c r="F1" s="151"/>
+      <c r="G1" s="151"/>
+      <c r="H1" s="151"/>
+      <c r="I1" s="151"/>
+      <c r="J1" s="151"/>
+      <c r="K1" s="151"/>
+      <c r="L1" s="152"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="155" t="s">
+      <c r="B2" s="153" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="156"/>
-      <c r="D2" s="156"/>
-      <c r="E2" s="156"/>
-      <c r="F2" s="156"/>
-      <c r="G2" s="156"/>
-      <c r="H2" s="156"/>
-      <c r="I2" s="157"/>
-      <c r="J2" s="161"/>
-      <c r="K2" s="162"/>
-      <c r="L2" s="163"/>
+      <c r="C2" s="154"/>
+      <c r="D2" s="154"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="154"/>
+      <c r="G2" s="154"/>
+      <c r="H2" s="154"/>
+      <c r="I2" s="155"/>
+      <c r="J2" s="159"/>
+      <c r="K2" s="160"/>
+      <c r="L2" s="161"/>
     </row>
     <row r="3" spans="1:13" ht="14.4" customHeight="1">
-      <c r="B3" s="158"/>
-      <c r="C3" s="159"/>
-      <c r="D3" s="159"/>
-      <c r="E3" s="159"/>
-      <c r="F3" s="159"/>
-      <c r="G3" s="159"/>
-      <c r="H3" s="159"/>
-      <c r="I3" s="160"/>
-      <c r="J3" s="164"/>
-      <c r="K3" s="165"/>
-      <c r="L3" s="166"/>
+      <c r="B3" s="156"/>
+      <c r="C3" s="157"/>
+      <c r="D3" s="157"/>
+      <c r="E3" s="157"/>
+      <c r="F3" s="157"/>
+      <c r="G3" s="157"/>
+      <c r="H3" s="157"/>
+      <c r="I3" s="158"/>
+      <c r="J3" s="162"/>
+      <c r="K3" s="163"/>
+      <c r="L3" s="164"/>
     </row>
     <row r="4" spans="1:13" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -41063,9 +41037,9 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="164"/>
-      <c r="K4" s="165"/>
-      <c r="L4" s="166"/>
+      <c r="J4" s="162"/>
+      <c r="K4" s="163"/>
+      <c r="L4" s="164"/>
     </row>
     <row r="5" spans="1:13" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -41080,9 +41054,9 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="164"/>
-      <c r="K5" s="165"/>
-      <c r="L5" s="166"/>
+      <c r="J5" s="162"/>
+      <c r="K5" s="163"/>
+      <c r="L5" s="164"/>
     </row>
     <row r="6" spans="1:13" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -41097,9 +41071,9 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="167"/>
-      <c r="K6" s="168"/>
-      <c r="L6" s="169"/>
+      <c r="J6" s="165"/>
+      <c r="K6" s="166"/>
+      <c r="L6" s="167"/>
     </row>
     <row r="7" spans="1:13" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -41155,41 +41129,41 @@
       <c r="L9" s="89"/>
     </row>
     <row r="10" spans="1:13" ht="15.6">
-      <c r="B10" s="170" t="s">
+      <c r="B10" s="168" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="171"/>
-      <c r="D10" s="171"/>
-      <c r="E10" s="171"/>
-      <c r="F10" s="172"/>
-      <c r="G10" s="171" t="s">
+      <c r="C10" s="169"/>
+      <c r="D10" s="169"/>
+      <c r="E10" s="169"/>
+      <c r="F10" s="170"/>
+      <c r="G10" s="169" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="171"/>
-      <c r="I10" s="171"/>
-      <c r="J10" s="172"/>
-      <c r="K10" s="171" t="s">
+      <c r="H10" s="169"/>
+      <c r="I10" s="169"/>
+      <c r="J10" s="170"/>
+      <c r="K10" s="169" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="173"/>
+      <c r="L10" s="171"/>
     </row>
     <row r="11" spans="1:13" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="192" t="s">
+      <c r="C11" s="187" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="193"/>
-      <c r="E11" s="193"/>
+      <c r="D11" s="188"/>
+      <c r="E11" s="188"/>
       <c r="F11" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="192" t="s">
+      <c r="G11" s="187" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="194"/>
+      <c r="H11" s="189"/>
       <c r="I11" s="92" t="s">
         <v>27</v>
       </c>
@@ -41208,14 +41182,14 @@
       <c r="B12" s="94" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="238" t="s">
+      <c r="C12" s="233" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="239"/>
-      <c r="E12" s="240"/>
+      <c r="D12" s="234"/>
+      <c r="E12" s="235"/>
       <c r="F12" s="95"/>
-      <c r="G12" s="201"/>
-      <c r="H12" s="202"/>
+      <c r="G12" s="196"/>
+      <c r="H12" s="197"/>
       <c r="I12" s="96"/>
       <c r="J12" s="96"/>
       <c r="K12" s="97"/>
@@ -41225,14 +41199,14 @@
       <c r="B13" s="99">
         <v>1</v>
       </c>
-      <c r="C13" s="241" t="s">
+      <c r="C13" s="236" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="242"/>
-      <c r="E13" s="243"/>
+      <c r="D13" s="237"/>
+      <c r="E13" s="238"/>
       <c r="F13" s="100"/>
-      <c r="G13" s="203"/>
-      <c r="H13" s="204"/>
+      <c r="G13" s="198"/>
+      <c r="H13" s="199"/>
       <c r="I13" s="101"/>
       <c r="J13" s="102"/>
       <c r="K13" s="103"/>
@@ -41242,14 +41216,14 @@
       <c r="B14" s="99">
         <v>2</v>
       </c>
-      <c r="C14" s="241" t="s">
+      <c r="C14" s="236" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="242"/>
-      <c r="E14" s="243"/>
+      <c r="D14" s="237"/>
+      <c r="E14" s="238"/>
       <c r="F14" s="100"/>
-      <c r="G14" s="203"/>
-      <c r="H14" s="204"/>
+      <c r="G14" s="198"/>
+      <c r="H14" s="199"/>
       <c r="I14" s="101"/>
       <c r="J14" s="102"/>
       <c r="K14" s="103"/>
@@ -41259,14 +41233,14 @@
       <c r="B15" s="99">
         <v>3</v>
       </c>
-      <c r="C15" s="241" t="s">
+      <c r="C15" s="236" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="242"/>
-      <c r="E15" s="243"/>
+      <c r="D15" s="237"/>
+      <c r="E15" s="238"/>
       <c r="F15" s="100"/>
-      <c r="G15" s="203"/>
-      <c r="H15" s="204"/>
+      <c r="G15" s="198"/>
+      <c r="H15" s="199"/>
       <c r="I15" s="101"/>
       <c r="J15" s="102"/>
       <c r="K15" s="103"/>
@@ -41276,14 +41250,14 @@
       <c r="B16" s="99">
         <v>4</v>
       </c>
-      <c r="C16" s="241" t="s">
+      <c r="C16" s="236" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="242"/>
-      <c r="E16" s="243"/>
+      <c r="D16" s="237"/>
+      <c r="E16" s="238"/>
       <c r="F16" s="100"/>
-      <c r="G16" s="203"/>
-      <c r="H16" s="204"/>
+      <c r="G16" s="198"/>
+      <c r="H16" s="199"/>
       <c r="I16" s="101"/>
       <c r="J16" s="102"/>
       <c r="K16" s="103"/>
@@ -41293,14 +41267,14 @@
       <c r="B17" s="99">
         <v>5</v>
       </c>
-      <c r="C17" s="241" t="s">
+      <c r="C17" s="236" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="242"/>
-      <c r="E17" s="243"/>
+      <c r="D17" s="237"/>
+      <c r="E17" s="238"/>
       <c r="F17" s="100"/>
-      <c r="G17" s="203"/>
-      <c r="H17" s="204"/>
+      <c r="G17" s="198"/>
+      <c r="H17" s="199"/>
       <c r="I17" s="101"/>
       <c r="J17" s="102"/>
       <c r="K17" s="103"/>
@@ -41310,14 +41284,14 @@
       <c r="B18" s="99">
         <v>6</v>
       </c>
-      <c r="C18" s="241" t="s">
+      <c r="C18" s="236" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="242"/>
-      <c r="E18" s="243"/>
+      <c r="D18" s="237"/>
+      <c r="E18" s="238"/>
       <c r="F18" s="100"/>
-      <c r="G18" s="203"/>
-      <c r="H18" s="204"/>
+      <c r="G18" s="198"/>
+      <c r="H18" s="199"/>
       <c r="I18" s="101"/>
       <c r="J18" s="102"/>
       <c r="K18" s="103"/>
@@ -41327,14 +41301,14 @@
       <c r="B19" s="105" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="244" t="s">
+      <c r="C19" s="239" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="245"/>
-      <c r="E19" s="246"/>
+      <c r="D19" s="240"/>
+      <c r="E19" s="241"/>
       <c r="F19" s="100"/>
-      <c r="G19" s="203"/>
-      <c r="H19" s="204"/>
+      <c r="G19" s="198"/>
+      <c r="H19" s="199"/>
       <c r="I19" s="101"/>
       <c r="J19" s="102"/>
       <c r="K19" s="103"/>
@@ -41344,14 +41318,14 @@
       <c r="B20" s="99">
         <v>1</v>
       </c>
-      <c r="C20" s="241" t="s">
+      <c r="C20" s="236" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="242"/>
-      <c r="E20" s="243"/>
+      <c r="D20" s="237"/>
+      <c r="E20" s="238"/>
       <c r="F20" s="100"/>
-      <c r="G20" s="203"/>
-      <c r="H20" s="204"/>
+      <c r="G20" s="198"/>
+      <c r="H20" s="199"/>
       <c r="I20" s="101"/>
       <c r="J20" s="102"/>
       <c r="K20" s="103"/>
@@ -41361,14 +41335,14 @@
       <c r="B21" s="99">
         <v>2</v>
       </c>
-      <c r="C21" s="241" t="s">
+      <c r="C21" s="236" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="242"/>
-      <c r="E21" s="243"/>
+      <c r="D21" s="237"/>
+      <c r="E21" s="238"/>
       <c r="F21" s="100"/>
-      <c r="G21" s="203"/>
-      <c r="H21" s="204"/>
+      <c r="G21" s="198"/>
+      <c r="H21" s="199"/>
       <c r="I21" s="101"/>
       <c r="J21" s="102"/>
       <c r="K21" s="103"/>
@@ -41378,142 +41352,142 @@
       <c r="B22" s="99">
         <v>3</v>
       </c>
-      <c r="C22" s="247" t="s">
+      <c r="C22" s="242" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="248"/>
-      <c r="E22" s="249"/>
+      <c r="D22" s="243"/>
+      <c r="E22" s="244"/>
       <c r="F22" s="100"/>
-      <c r="G22" s="205"/>
-      <c r="H22" s="206"/>
+      <c r="G22" s="200"/>
+      <c r="H22" s="201"/>
       <c r="I22" s="101"/>
       <c r="J22" s="102"/>
       <c r="K22" s="106"/>
       <c r="L22" s="107"/>
     </row>
     <row r="23" spans="1:12" ht="16.2" thickBot="1">
-      <c r="B23" s="195"/>
-      <c r="C23" s="196"/>
-      <c r="D23" s="196"/>
-      <c r="E23" s="196"/>
+      <c r="B23" s="190"/>
+      <c r="C23" s="191"/>
+      <c r="D23" s="191"/>
+      <c r="E23" s="191"/>
       <c r="F23" s="108"/>
       <c r="G23" s="108"/>
       <c r="H23" s="109"/>
       <c r="I23" s="109"/>
-      <c r="J23" s="197"/>
-      <c r="K23" s="197"/>
-      <c r="L23" s="198"/>
+      <c r="J23" s="192"/>
+      <c r="K23" s="192"/>
+      <c r="L23" s="193"/>
     </row>
     <row r="24" spans="1:12" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="124" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="199" t="s">
+      <c r="B24" s="194" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="174" t="s">
+      <c r="C24" s="172" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="174"/>
-      <c r="E24" s="174"/>
-      <c r="F24" s="174"/>
-      <c r="G24" s="174"/>
-      <c r="H24" s="174"/>
-      <c r="I24" s="174"/>
-      <c r="J24" s="176" t="s">
+      <c r="D24" s="172"/>
+      <c r="E24" s="172"/>
+      <c r="F24" s="172"/>
+      <c r="G24" s="172"/>
+      <c r="H24" s="172"/>
+      <c r="I24" s="172"/>
+      <c r="J24" s="174" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="177"/>
-      <c r="L24" s="178"/>
+      <c r="K24" s="175"/>
+      <c r="L24" s="176"/>
     </row>
     <row r="25" spans="1:12" ht="31.2">
-      <c r="B25" s="200"/>
-      <c r="C25" s="175"/>
-      <c r="D25" s="175"/>
-      <c r="E25" s="175"/>
-      <c r="F25" s="175"/>
-      <c r="G25" s="175"/>
-      <c r="H25" s="175"/>
-      <c r="I25" s="175"/>
-      <c r="J25" s="151" t="s">
+      <c r="B25" s="195"/>
+      <c r="C25" s="173"/>
+      <c r="D25" s="173"/>
+      <c r="E25" s="173"/>
+      <c r="F25" s="173"/>
+      <c r="G25" s="173"/>
+      <c r="H25" s="173"/>
+      <c r="I25" s="173"/>
+      <c r="J25" s="149" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="148" t="s">
+      <c r="K25" s="146" t="s">
         <v>76</v>
       </c>
-      <c r="L25" s="149" t="s">
+      <c r="L25" s="147" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.6">
       <c r="B26" s="110"/>
-      <c r="C26" s="293"/>
-      <c r="D26" s="294"/>
-      <c r="E26" s="294"/>
-      <c r="F26" s="294"/>
-      <c r="G26" s="294"/>
-      <c r="H26" s="294"/>
-      <c r="I26" s="295"/>
-      <c r="J26" s="302"/>
-      <c r="K26" s="150"/>
-      <c r="L26" s="306"/>
+      <c r="C26" s="288"/>
+      <c r="D26" s="289"/>
+      <c r="E26" s="289"/>
+      <c r="F26" s="289"/>
+      <c r="G26" s="289"/>
+      <c r="H26" s="289"/>
+      <c r="I26" s="290"/>
+      <c r="J26" s="297"/>
+      <c r="K26" s="148"/>
+      <c r="L26" s="301"/>
     </row>
     <row r="27" spans="1:12" ht="15.6">
       <c r="B27" s="110"/>
-      <c r="C27" s="296"/>
-      <c r="D27" s="297"/>
-      <c r="E27" s="297"/>
-      <c r="F27" s="297"/>
-      <c r="G27" s="297"/>
-      <c r="H27" s="297"/>
-      <c r="I27" s="298"/>
+      <c r="C27" s="291"/>
+      <c r="D27" s="292"/>
+      <c r="E27" s="292"/>
+      <c r="F27" s="292"/>
+      <c r="G27" s="292"/>
+      <c r="H27" s="292"/>
+      <c r="I27" s="293"/>
       <c r="J27" s="102"/>
-      <c r="K27" s="304"/>
-      <c r="L27" s="306"/>
+      <c r="K27" s="299"/>
+      <c r="L27" s="301"/>
     </row>
     <row r="28" spans="1:12" ht="15.6">
       <c r="B28" s="110"/>
-      <c r="C28" s="296"/>
-      <c r="D28" s="297"/>
-      <c r="E28" s="297"/>
-      <c r="F28" s="297"/>
-      <c r="G28" s="297"/>
-      <c r="H28" s="297"/>
-      <c r="I28" s="298"/>
+      <c r="C28" s="291"/>
+      <c r="D28" s="292"/>
+      <c r="E28" s="292"/>
+      <c r="F28" s="292"/>
+      <c r="G28" s="292"/>
+      <c r="H28" s="292"/>
+      <c r="I28" s="293"/>
       <c r="J28" s="102"/>
-      <c r="K28" s="304"/>
+      <c r="K28" s="299"/>
       <c r="L28" s="111"/>
     </row>
     <row r="29" spans="1:12" ht="15.6">
       <c r="B29" s="110"/>
-      <c r="C29" s="296"/>
-      <c r="D29" s="297"/>
-      <c r="E29" s="297"/>
-      <c r="F29" s="297"/>
-      <c r="G29" s="297"/>
-      <c r="H29" s="297"/>
-      <c r="I29" s="298"/>
+      <c r="C29" s="291"/>
+      <c r="D29" s="292"/>
+      <c r="E29" s="292"/>
+      <c r="F29" s="292"/>
+      <c r="G29" s="292"/>
+      <c r="H29" s="292"/>
+      <c r="I29" s="293"/>
       <c r="J29" s="102"/>
-      <c r="K29" s="304"/>
+      <c r="K29" s="299"/>
       <c r="L29" s="111"/>
     </row>
     <row r="30" spans="1:12" ht="15.6">
       <c r="B30" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="296" t="s">
+      <c r="C30" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="297"/>
-      <c r="E30" s="297"/>
-      <c r="F30" s="297"/>
-      <c r="G30" s="297"/>
-      <c r="H30" s="297"/>
-      <c r="I30" s="298"/>
+      <c r="D30" s="292"/>
+      <c r="E30" s="292"/>
+      <c r="F30" s="292"/>
+      <c r="G30" s="292"/>
+      <c r="H30" s="292"/>
+      <c r="I30" s="293"/>
       <c r="J30" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K30" s="304"/>
+      <c r="K30" s="299"/>
       <c r="L30" s="111" t="s">
         <v>64</v>
       </c>
@@ -41522,19 +41496,19 @@
       <c r="B31" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="296" t="s">
+      <c r="C31" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="297"/>
-      <c r="E31" s="297"/>
-      <c r="F31" s="297"/>
-      <c r="G31" s="297"/>
-      <c r="H31" s="297"/>
-      <c r="I31" s="298"/>
+      <c r="D31" s="292"/>
+      <c r="E31" s="292"/>
+      <c r="F31" s="292"/>
+      <c r="G31" s="292"/>
+      <c r="H31" s="292"/>
+      <c r="I31" s="293"/>
       <c r="J31" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K31" s="304"/>
+      <c r="K31" s="299"/>
       <c r="L31" s="111" t="s">
         <v>64</v>
       </c>
@@ -41543,19 +41517,19 @@
       <c r="B32" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="296" t="s">
+      <c r="C32" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="297"/>
-      <c r="E32" s="297"/>
-      <c r="F32" s="297"/>
-      <c r="G32" s="297"/>
-      <c r="H32" s="297"/>
-      <c r="I32" s="298"/>
+      <c r="D32" s="292"/>
+      <c r="E32" s="292"/>
+      <c r="F32" s="292"/>
+      <c r="G32" s="292"/>
+      <c r="H32" s="292"/>
+      <c r="I32" s="293"/>
       <c r="J32" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K32" s="304"/>
+      <c r="K32" s="299"/>
       <c r="L32" s="111" t="s">
         <v>64</v>
       </c>
@@ -41564,19 +41538,19 @@
       <c r="B33" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="296" t="s">
+      <c r="C33" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="297"/>
-      <c r="E33" s="297"/>
-      <c r="F33" s="297"/>
-      <c r="G33" s="297"/>
-      <c r="H33" s="297"/>
-      <c r="I33" s="298"/>
+      <c r="D33" s="292"/>
+      <c r="E33" s="292"/>
+      <c r="F33" s="292"/>
+      <c r="G33" s="292"/>
+      <c r="H33" s="292"/>
+      <c r="I33" s="293"/>
       <c r="J33" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K33" s="304"/>
+      <c r="K33" s="299"/>
       <c r="L33" s="111" t="s">
         <v>64</v>
       </c>
@@ -41585,19 +41559,19 @@
       <c r="B34" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="296" t="s">
+      <c r="C34" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="297"/>
-      <c r="E34" s="297"/>
-      <c r="F34" s="297"/>
-      <c r="G34" s="297"/>
-      <c r="H34" s="297"/>
-      <c r="I34" s="298"/>
+      <c r="D34" s="292"/>
+      <c r="E34" s="292"/>
+      <c r="F34" s="292"/>
+      <c r="G34" s="292"/>
+      <c r="H34" s="292"/>
+      <c r="I34" s="293"/>
       <c r="J34" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K34" s="304"/>
+      <c r="K34" s="299"/>
       <c r="L34" s="111" t="s">
         <v>64</v>
       </c>
@@ -41606,19 +41580,19 @@
       <c r="B35" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="296" t="s">
+      <c r="C35" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="297"/>
-      <c r="E35" s="297"/>
-      <c r="F35" s="297"/>
-      <c r="G35" s="297"/>
-      <c r="H35" s="297"/>
-      <c r="I35" s="298"/>
+      <c r="D35" s="292"/>
+      <c r="E35" s="292"/>
+      <c r="F35" s="292"/>
+      <c r="G35" s="292"/>
+      <c r="H35" s="292"/>
+      <c r="I35" s="293"/>
       <c r="J35" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K35" s="304"/>
+      <c r="K35" s="299"/>
       <c r="L35" s="111" t="s">
         <v>64</v>
       </c>
@@ -41627,19 +41601,19 @@
       <c r="B36" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C36" s="296" t="s">
+      <c r="C36" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="297"/>
-      <c r="E36" s="297"/>
-      <c r="F36" s="297"/>
-      <c r="G36" s="297"/>
-      <c r="H36" s="297"/>
-      <c r="I36" s="298"/>
+      <c r="D36" s="292"/>
+      <c r="E36" s="292"/>
+      <c r="F36" s="292"/>
+      <c r="G36" s="292"/>
+      <c r="H36" s="292"/>
+      <c r="I36" s="293"/>
       <c r="J36" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K36" s="304"/>
+      <c r="K36" s="299"/>
       <c r="L36" s="111" t="s">
         <v>64</v>
       </c>
@@ -41648,19 +41622,19 @@
       <c r="B37" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="296" t="s">
+      <c r="C37" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="297"/>
-      <c r="E37" s="297"/>
-      <c r="F37" s="297"/>
-      <c r="G37" s="297"/>
-      <c r="H37" s="297"/>
-      <c r="I37" s="298"/>
+      <c r="D37" s="292"/>
+      <c r="E37" s="292"/>
+      <c r="F37" s="292"/>
+      <c r="G37" s="292"/>
+      <c r="H37" s="292"/>
+      <c r="I37" s="293"/>
       <c r="J37" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K37" s="304"/>
+      <c r="K37" s="299"/>
       <c r="L37" s="111" t="s">
         <v>64</v>
       </c>
@@ -41669,19 +41643,19 @@
       <c r="B38" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="296" t="s">
+      <c r="C38" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="297"/>
-      <c r="E38" s="297"/>
-      <c r="F38" s="297"/>
-      <c r="G38" s="297"/>
-      <c r="H38" s="297"/>
-      <c r="I38" s="298"/>
+      <c r="D38" s="292"/>
+      <c r="E38" s="292"/>
+      <c r="F38" s="292"/>
+      <c r="G38" s="292"/>
+      <c r="H38" s="292"/>
+      <c r="I38" s="293"/>
       <c r="J38" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K38" s="304"/>
+      <c r="K38" s="299"/>
       <c r="L38" s="111" t="s">
         <v>64</v>
       </c>
@@ -41690,19 +41664,19 @@
       <c r="B39" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="296" t="s">
+      <c r="C39" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D39" s="297"/>
-      <c r="E39" s="297"/>
-      <c r="F39" s="297"/>
-      <c r="G39" s="297"/>
-      <c r="H39" s="297"/>
-      <c r="I39" s="298"/>
+      <c r="D39" s="292"/>
+      <c r="E39" s="292"/>
+      <c r="F39" s="292"/>
+      <c r="G39" s="292"/>
+      <c r="H39" s="292"/>
+      <c r="I39" s="293"/>
       <c r="J39" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K39" s="304"/>
+      <c r="K39" s="299"/>
       <c r="L39" s="111" t="s">
         <v>64</v>
       </c>
@@ -41711,19 +41685,19 @@
       <c r="B40" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="296" t="s">
+      <c r="C40" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D40" s="297"/>
-      <c r="E40" s="297"/>
-      <c r="F40" s="297"/>
-      <c r="G40" s="297"/>
-      <c r="H40" s="297"/>
-      <c r="I40" s="298"/>
+      <c r="D40" s="292"/>
+      <c r="E40" s="292"/>
+      <c r="F40" s="292"/>
+      <c r="G40" s="292"/>
+      <c r="H40" s="292"/>
+      <c r="I40" s="293"/>
       <c r="J40" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K40" s="304"/>
+      <c r="K40" s="299"/>
       <c r="L40" s="111" t="s">
         <v>64</v>
       </c>
@@ -41732,19 +41706,19 @@
       <c r="B41" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="296" t="s">
+      <c r="C41" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D41" s="297"/>
-      <c r="E41" s="297"/>
-      <c r="F41" s="297"/>
-      <c r="G41" s="297"/>
-      <c r="H41" s="297"/>
-      <c r="I41" s="298"/>
+      <c r="D41" s="292"/>
+      <c r="E41" s="292"/>
+      <c r="F41" s="292"/>
+      <c r="G41" s="292"/>
+      <c r="H41" s="292"/>
+      <c r="I41" s="293"/>
       <c r="J41" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K41" s="304"/>
+      <c r="K41" s="299"/>
       <c r="L41" s="111" t="s">
         <v>64</v>
       </c>
@@ -41753,19 +41727,19 @@
       <c r="B42" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="296" t="s">
+      <c r="C42" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="297"/>
-      <c r="E42" s="297"/>
-      <c r="F42" s="297"/>
-      <c r="G42" s="297"/>
-      <c r="H42" s="297"/>
-      <c r="I42" s="298"/>
+      <c r="D42" s="292"/>
+      <c r="E42" s="292"/>
+      <c r="F42" s="292"/>
+      <c r="G42" s="292"/>
+      <c r="H42" s="292"/>
+      <c r="I42" s="293"/>
       <c r="J42" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K42" s="304"/>
+      <c r="K42" s="299"/>
       <c r="L42" s="111" t="s">
         <v>64</v>
       </c>
@@ -41774,19 +41748,19 @@
       <c r="B43" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="296" t="s">
+      <c r="C43" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="297"/>
-      <c r="E43" s="297"/>
-      <c r="F43" s="297"/>
-      <c r="G43" s="297"/>
-      <c r="H43" s="297"/>
-      <c r="I43" s="298"/>
+      <c r="D43" s="292"/>
+      <c r="E43" s="292"/>
+      <c r="F43" s="292"/>
+      <c r="G43" s="292"/>
+      <c r="H43" s="292"/>
+      <c r="I43" s="293"/>
       <c r="J43" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K43" s="304"/>
+      <c r="K43" s="299"/>
       <c r="L43" s="111" t="s">
         <v>64</v>
       </c>
@@ -41795,19 +41769,19 @@
       <c r="B44" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="296" t="s">
+      <c r="C44" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D44" s="297"/>
-      <c r="E44" s="297"/>
-      <c r="F44" s="297"/>
-      <c r="G44" s="297"/>
-      <c r="H44" s="297"/>
-      <c r="I44" s="298"/>
+      <c r="D44" s="292"/>
+      <c r="E44" s="292"/>
+      <c r="F44" s="292"/>
+      <c r="G44" s="292"/>
+      <c r="H44" s="292"/>
+      <c r="I44" s="293"/>
       <c r="J44" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K44" s="304"/>
+      <c r="K44" s="299"/>
       <c r="L44" s="111" t="s">
         <v>64</v>
       </c>
@@ -41816,19 +41790,19 @@
       <c r="B45" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C45" s="296" t="s">
+      <c r="C45" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D45" s="297"/>
-      <c r="E45" s="297"/>
-      <c r="F45" s="297"/>
-      <c r="G45" s="297"/>
-      <c r="H45" s="297"/>
-      <c r="I45" s="298"/>
+      <c r="D45" s="292"/>
+      <c r="E45" s="292"/>
+      <c r="F45" s="292"/>
+      <c r="G45" s="292"/>
+      <c r="H45" s="292"/>
+      <c r="I45" s="293"/>
       <c r="J45" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K45" s="304"/>
+      <c r="K45" s="299"/>
       <c r="L45" s="111" t="s">
         <v>64</v>
       </c>
@@ -41837,19 +41811,19 @@
       <c r="B46" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C46" s="296" t="s">
+      <c r="C46" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="297"/>
-      <c r="E46" s="297"/>
-      <c r="F46" s="297"/>
-      <c r="G46" s="297"/>
-      <c r="H46" s="297"/>
-      <c r="I46" s="298"/>
+      <c r="D46" s="292"/>
+      <c r="E46" s="292"/>
+      <c r="F46" s="292"/>
+      <c r="G46" s="292"/>
+      <c r="H46" s="292"/>
+      <c r="I46" s="293"/>
       <c r="J46" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K46" s="304"/>
+      <c r="K46" s="299"/>
       <c r="L46" s="111" t="s">
         <v>64</v>
       </c>
@@ -41858,19 +41832,19 @@
       <c r="B47" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="296" t="s">
+      <c r="C47" s="291" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="297"/>
-      <c r="E47" s="297"/>
-      <c r="F47" s="297"/>
-      <c r="G47" s="297"/>
-      <c r="H47" s="297"/>
-      <c r="I47" s="298"/>
+      <c r="D47" s="292"/>
+      <c r="E47" s="292"/>
+      <c r="F47" s="292"/>
+      <c r="G47" s="292"/>
+      <c r="H47" s="292"/>
+      <c r="I47" s="293"/>
       <c r="J47" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K47" s="304"/>
+      <c r="K47" s="299"/>
       <c r="L47" s="111" t="s">
         <v>64</v>
       </c>
@@ -41879,342 +41853,278 @@
       <c r="B48" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C48" s="299" t="s">
+      <c r="C48" s="294" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="300"/>
-      <c r="E48" s="300"/>
-      <c r="F48" s="300"/>
-      <c r="G48" s="300"/>
-      <c r="H48" s="300"/>
-      <c r="I48" s="301"/>
-      <c r="J48" s="303" t="s">
+      <c r="D48" s="295"/>
+      <c r="E48" s="295"/>
+      <c r="F48" s="295"/>
+      <c r="G48" s="295"/>
+      <c r="H48" s="295"/>
+      <c r="I48" s="296"/>
+      <c r="J48" s="298" t="s">
         <v>64</v>
       </c>
-      <c r="K48" s="305"/>
+      <c r="K48" s="300"/>
       <c r="L48" s="111" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="49" spans="2:12" ht="16.2" thickTop="1">
-      <c r="B49" s="220" t="s">
+      <c r="B49" s="215" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="221"/>
-      <c r="D49" s="221"/>
-      <c r="E49" s="221"/>
-      <c r="F49" s="221"/>
-      <c r="G49" s="221"/>
-      <c r="H49" s="221"/>
-      <c r="I49" s="221"/>
-      <c r="J49" s="222"/>
-      <c r="K49" s="190" t="s">
+      <c r="C49" s="216"/>
+      <c r="D49" s="216"/>
+      <c r="E49" s="216"/>
+      <c r="F49" s="216"/>
+      <c r="G49" s="216"/>
+      <c r="H49" s="216"/>
+      <c r="I49" s="216"/>
+      <c r="J49" s="217"/>
+      <c r="K49" s="185" t="s">
         <v>79</v>
       </c>
-      <c r="L49" s="191"/>
+      <c r="L49" s="186"/>
     </row>
     <row r="50" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B50" s="223"/>
-      <c r="C50" s="224"/>
-      <c r="D50" s="224"/>
-      <c r="E50" s="224"/>
-      <c r="F50" s="224"/>
-      <c r="G50" s="224"/>
-      <c r="H50" s="224"/>
-      <c r="I50" s="224"/>
-      <c r="J50" s="225"/>
-      <c r="K50" s="188" t="s">
+      <c r="B50" s="218"/>
+      <c r="C50" s="219"/>
+      <c r="D50" s="219"/>
+      <c r="E50" s="219"/>
+      <c r="F50" s="219"/>
+      <c r="G50" s="219"/>
+      <c r="H50" s="219"/>
+      <c r="I50" s="219"/>
+      <c r="J50" s="220"/>
+      <c r="K50" s="183" t="s">
         <v>103</v>
       </c>
-      <c r="L50" s="189"/>
+      <c r="L50" s="184"/>
     </row>
     <row r="51" spans="2:12" ht="15.6">
       <c r="B51" s="112"/>
-      <c r="C51" s="185"/>
-      <c r="D51" s="185"/>
-      <c r="E51" s="185"/>
-      <c r="F51" s="185"/>
-      <c r="G51" s="185"/>
-      <c r="H51" s="185"/>
-      <c r="I51" s="185"/>
+      <c r="C51" s="180"/>
+      <c r="D51" s="180"/>
+      <c r="E51" s="180"/>
+      <c r="F51" s="180"/>
+      <c r="G51" s="180"/>
+      <c r="H51" s="180"/>
+      <c r="I51" s="180"/>
       <c r="J51" s="113"/>
-      <c r="K51" s="183"/>
-      <c r="L51" s="184"/>
+      <c r="K51" s="178"/>
+      <c r="L51" s="179"/>
     </row>
     <row r="52" spans="2:12" ht="15.6">
       <c r="B52" s="114"/>
-      <c r="C52" s="186"/>
-      <c r="D52" s="186"/>
-      <c r="E52" s="186"/>
-      <c r="F52" s="186"/>
-      <c r="G52" s="186"/>
-      <c r="H52" s="186"/>
-      <c r="I52" s="186"/>
+      <c r="C52" s="181"/>
+      <c r="D52" s="181"/>
+      <c r="E52" s="181"/>
+      <c r="F52" s="181"/>
+      <c r="G52" s="181"/>
+      <c r="H52" s="181"/>
+      <c r="I52" s="181"/>
       <c r="J52" s="115"/>
       <c r="K52" s="126"/>
       <c r="L52" s="116"/>
     </row>
     <row r="53" spans="2:12" ht="15.6">
-      <c r="B53" s="114"/>
-      <c r="C53" s="186"/>
-      <c r="D53" s="186"/>
-      <c r="E53" s="186"/>
-      <c r="F53" s="186"/>
-      <c r="G53" s="186"/>
-      <c r="H53" s="186"/>
-      <c r="I53" s="186"/>
-      <c r="J53" s="115"/>
-      <c r="K53" s="126"/>
-      <c r="L53" s="116"/>
+      <c r="B53" s="117"/>
+      <c r="C53" s="181"/>
+      <c r="D53" s="181"/>
+      <c r="E53" s="181"/>
+      <c r="F53" s="181"/>
+      <c r="G53" s="181"/>
+      <c r="H53" s="181"/>
+      <c r="I53" s="181"/>
+      <c r="J53" s="118"/>
+      <c r="K53" s="119"/>
+      <c r="L53" s="120"/>
     </row>
     <row r="54" spans="2:12" ht="15.6">
-      <c r="B54" s="114"/>
-      <c r="C54" s="186"/>
-      <c r="D54" s="186"/>
-      <c r="E54" s="186"/>
-      <c r="F54" s="186"/>
-      <c r="G54" s="186"/>
-      <c r="H54" s="186"/>
-      <c r="I54" s="186"/>
-      <c r="J54" s="115"/>
-      <c r="K54" s="126"/>
-      <c r="L54" s="116"/>
+      <c r="B54" s="117"/>
+      <c r="C54" s="181"/>
+      <c r="D54" s="181"/>
+      <c r="E54" s="181"/>
+      <c r="F54" s="181"/>
+      <c r="G54" s="181"/>
+      <c r="H54" s="181"/>
+      <c r="I54" s="181"/>
+      <c r="J54" s="118"/>
+      <c r="K54" s="302"/>
+      <c r="L54" s="303"/>
     </row>
     <row r="55" spans="2:12" ht="15.6">
       <c r="B55" s="117"/>
-      <c r="C55" s="186"/>
-      <c r="D55" s="186"/>
-      <c r="E55" s="186"/>
-      <c r="F55" s="186"/>
-      <c r="G55" s="186"/>
-      <c r="H55" s="186"/>
-      <c r="I55" s="186"/>
+      <c r="C55" s="181"/>
+      <c r="D55" s="181"/>
+      <c r="E55" s="181"/>
+      <c r="F55" s="181"/>
+      <c r="G55" s="181"/>
+      <c r="H55" s="181"/>
+      <c r="I55" s="181"/>
       <c r="J55" s="118"/>
-      <c r="K55" s="119"/>
-      <c r="L55" s="120"/>
+      <c r="K55" s="305"/>
+      <c r="L55" s="306"/>
     </row>
     <row r="56" spans="2:12" ht="15.6">
       <c r="B56" s="117"/>
-      <c r="C56" s="186"/>
-      <c r="D56" s="186"/>
-      <c r="E56" s="186"/>
-      <c r="F56" s="186"/>
-      <c r="G56" s="186"/>
-      <c r="H56" s="186"/>
-      <c r="I56" s="186"/>
+      <c r="C56" s="181"/>
+      <c r="D56" s="181"/>
+      <c r="E56" s="181"/>
+      <c r="F56" s="181"/>
+      <c r="G56" s="181"/>
+      <c r="H56" s="181"/>
+      <c r="I56" s="181"/>
       <c r="J56" s="118"/>
-      <c r="K56" s="119"/>
-      <c r="L56" s="120"/>
+      <c r="K56" s="307"/>
+      <c r="L56" s="308"/>
     </row>
     <row r="57" spans="2:12" ht="15.6">
       <c r="B57" s="117"/>
-      <c r="C57" s="186"/>
-      <c r="D57" s="186"/>
-      <c r="E57" s="186"/>
-      <c r="F57" s="186"/>
-      <c r="G57" s="186"/>
-      <c r="H57" s="186"/>
-      <c r="I57" s="186"/>
+      <c r="C57" s="181"/>
+      <c r="D57" s="181"/>
+      <c r="E57" s="181"/>
+      <c r="F57" s="181"/>
+      <c r="G57" s="181"/>
+      <c r="H57" s="181"/>
+      <c r="I57" s="181"/>
       <c r="J57" s="118"/>
-      <c r="K57" s="179"/>
-      <c r="L57" s="180"/>
+      <c r="K57" s="305"/>
+      <c r="L57" s="306"/>
     </row>
     <row r="58" spans="2:12" ht="15.6">
       <c r="B58" s="117"/>
-      <c r="C58" s="186"/>
-      <c r="D58" s="186"/>
-      <c r="E58" s="186"/>
-      <c r="F58" s="186"/>
-      <c r="G58" s="186"/>
-      <c r="H58" s="186"/>
-      <c r="I58" s="186"/>
+      <c r="C58" s="182"/>
+      <c r="D58" s="182"/>
+      <c r="E58" s="182"/>
+      <c r="F58" s="182"/>
+      <c r="G58" s="182"/>
+      <c r="H58" s="182"/>
+      <c r="I58" s="182"/>
       <c r="J58" s="118"/>
-      <c r="K58" s="181"/>
-      <c r="L58" s="182"/>
+      <c r="K58" s="304"/>
+      <c r="L58" s="177"/>
     </row>
     <row r="59" spans="2:12" ht="15.6">
       <c r="B59" s="117"/>
-      <c r="C59" s="186"/>
-      <c r="D59" s="186"/>
-      <c r="E59" s="186"/>
-      <c r="F59" s="186"/>
-      <c r="G59" s="186"/>
-      <c r="H59" s="186"/>
-      <c r="I59" s="186"/>
+      <c r="C59" s="121"/>
+      <c r="D59" s="121"/>
+      <c r="E59" s="121"/>
+      <c r="F59" s="121"/>
+      <c r="G59" s="121"/>
+      <c r="H59" s="121"/>
+      <c r="I59" s="121"/>
       <c r="J59" s="118"/>
-      <c r="K59" s="127"/>
-      <c r="L59" s="76"/>
+      <c r="K59" s="304"/>
+      <c r="L59" s="177"/>
     </row>
     <row r="60" spans="2:12" ht="15.6">
-      <c r="B60" s="117"/>
-      <c r="C60" s="186"/>
-      <c r="D60" s="186"/>
-      <c r="E60" s="186"/>
-      <c r="F60" s="186"/>
-      <c r="G60" s="186"/>
-      <c r="H60" s="186"/>
-      <c r="I60" s="186"/>
-      <c r="J60" s="118"/>
-      <c r="K60" s="127"/>
-      <c r="L60" s="76"/>
-    </row>
-    <row r="61" spans="2:12" ht="15.6">
-      <c r="B61" s="117"/>
-      <c r="C61" s="187"/>
-      <c r="D61" s="187"/>
-      <c r="E61" s="187"/>
-      <c r="F61" s="187"/>
-      <c r="G61" s="187"/>
-      <c r="H61" s="187"/>
-      <c r="I61" s="187"/>
-      <c r="J61" s="118"/>
-      <c r="K61" s="127"/>
-      <c r="L61" s="76"/>
-    </row>
-    <row r="62" spans="2:12" ht="15.6">
-      <c r="B62" s="117"/>
-      <c r="C62" s="121"/>
-      <c r="D62" s="121"/>
-      <c r="E62" s="121"/>
-      <c r="F62" s="121"/>
-      <c r="G62" s="121"/>
-      <c r="H62" s="121"/>
-      <c r="I62" s="121"/>
-      <c r="J62" s="118"/>
-      <c r="K62" s="129"/>
-      <c r="L62" s="130"/>
-    </row>
-    <row r="63" spans="2:12" ht="15.6">
-      <c r="B63" s="207" t="s">
+      <c r="B60" s="202" t="s">
         <v>80</v>
       </c>
-      <c r="C63" s="208"/>
-      <c r="D63" s="208"/>
-      <c r="E63" s="209"/>
-      <c r="F63" s="210" t="s">
+      <c r="C60" s="203"/>
+      <c r="D60" s="203"/>
+      <c r="E60" s="204"/>
+      <c r="F60" s="205" t="s">
         <v>81</v>
       </c>
-      <c r="G63" s="209"/>
-      <c r="H63" s="210" t="s">
+      <c r="G60" s="204"/>
+      <c r="H60" s="205" t="s">
         <v>82</v>
       </c>
-      <c r="I63" s="208"/>
-      <c r="J63" s="209"/>
-      <c r="K63" s="119"/>
-      <c r="L63" s="120"/>
+      <c r="I60" s="203"/>
+      <c r="J60" s="204"/>
+      <c r="K60" s="119"/>
+      <c r="L60" s="120"/>
+    </row>
+    <row r="61" spans="2:12" ht="15.6" customHeight="1">
+      <c r="B61" s="227"/>
+      <c r="C61" s="228"/>
+      <c r="D61" s="228"/>
+      <c r="E61" s="222"/>
+      <c r="F61" s="221"/>
+      <c r="G61" s="222"/>
+      <c r="H61" s="206"/>
+      <c r="I61" s="207"/>
+      <c r="J61" s="208"/>
+      <c r="K61" s="119"/>
+      <c r="L61" s="120"/>
+    </row>
+    <row r="62" spans="2:12" ht="15.6" customHeight="1">
+      <c r="B62" s="229"/>
+      <c r="C62" s="230"/>
+      <c r="D62" s="230"/>
+      <c r="E62" s="224"/>
+      <c r="F62" s="223"/>
+      <c r="G62" s="224"/>
+      <c r="H62" s="209"/>
+      <c r="I62" s="210"/>
+      <c r="J62" s="211"/>
+      <c r="K62" s="128"/>
+      <c r="L62" s="120"/>
+    </row>
+    <row r="63" spans="2:12" ht="15.6" customHeight="1">
+      <c r="B63" s="229"/>
+      <c r="C63" s="230"/>
+      <c r="D63" s="230"/>
+      <c r="E63" s="224"/>
+      <c r="F63" s="223"/>
+      <c r="G63" s="224"/>
+      <c r="H63" s="209"/>
+      <c r="I63" s="210"/>
+      <c r="J63" s="211"/>
+      <c r="K63" s="127"/>
+      <c r="L63" s="76"/>
     </row>
     <row r="64" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B64" s="232"/>
-      <c r="C64" s="233"/>
-      <c r="D64" s="233"/>
-      <c r="E64" s="227"/>
-      <c r="F64" s="226"/>
-      <c r="G64" s="227"/>
-      <c r="H64" s="211"/>
-      <c r="I64" s="212"/>
-      <c r="J64" s="213"/>
-      <c r="K64" s="119"/>
-      <c r="L64" s="120"/>
+      <c r="B64" s="229"/>
+      <c r="C64" s="230"/>
+      <c r="D64" s="230"/>
+      <c r="E64" s="224"/>
+      <c r="F64" s="223"/>
+      <c r="G64" s="224"/>
+      <c r="H64" s="209"/>
+      <c r="I64" s="210"/>
+      <c r="J64" s="211"/>
+      <c r="K64" s="129"/>
+      <c r="L64" s="130"/>
     </row>
     <row r="65" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B65" s="234"/>
-      <c r="C65" s="235"/>
-      <c r="D65" s="235"/>
-      <c r="E65" s="229"/>
-      <c r="F65" s="228"/>
-      <c r="G65" s="229"/>
-      <c r="H65" s="214"/>
-      <c r="I65" s="215"/>
-      <c r="J65" s="216"/>
-      <c r="K65" s="128"/>
-      <c r="L65" s="120"/>
-    </row>
-    <row r="66" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B66" s="234"/>
-      <c r="C66" s="235"/>
-      <c r="D66" s="235"/>
-      <c r="E66" s="229"/>
-      <c r="F66" s="228"/>
-      <c r="G66" s="229"/>
-      <c r="H66" s="214"/>
-      <c r="I66" s="215"/>
-      <c r="J66" s="216"/>
-      <c r="K66" s="119"/>
-      <c r="L66" s="120"/>
-    </row>
-    <row r="67" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B67" s="234"/>
-      <c r="C67" s="235"/>
-      <c r="D67" s="235"/>
-      <c r="E67" s="229"/>
-      <c r="F67" s="228"/>
-      <c r="G67" s="229"/>
-      <c r="H67" s="214"/>
-      <c r="I67" s="215"/>
-      <c r="J67" s="216"/>
-      <c r="K67" s="127"/>
-      <c r="L67" s="76"/>
-    </row>
-    <row r="68" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B68" s="234"/>
-      <c r="C68" s="235"/>
-      <c r="D68" s="235"/>
-      <c r="E68" s="229"/>
-      <c r="F68" s="228"/>
-      <c r="G68" s="229"/>
-      <c r="H68" s="214"/>
-      <c r="I68" s="215"/>
-      <c r="J68" s="216"/>
-      <c r="K68" s="127"/>
-      <c r="L68" s="76"/>
-    </row>
-    <row r="69" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B69" s="234"/>
-      <c r="C69" s="235"/>
-      <c r="D69" s="235"/>
-      <c r="E69" s="229"/>
-      <c r="F69" s="228"/>
-      <c r="G69" s="229"/>
-      <c r="H69" s="214"/>
-      <c r="I69" s="215"/>
-      <c r="J69" s="216"/>
-      <c r="K69" s="131"/>
-      <c r="L69" s="132"/>
-    </row>
-    <row r="70" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B70" s="234"/>
-      <c r="C70" s="235"/>
-      <c r="D70" s="235"/>
-      <c r="E70" s="229"/>
-      <c r="F70" s="228"/>
-      <c r="G70" s="229"/>
-      <c r="H70" s="214"/>
-      <c r="I70" s="215"/>
-      <c r="J70" s="216"/>
-      <c r="K70" s="131"/>
-      <c r="L70" s="132"/>
-    </row>
-    <row r="71" spans="2:12" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B71" s="236"/>
-      <c r="C71" s="237"/>
-      <c r="D71" s="237"/>
-      <c r="E71" s="231"/>
-      <c r="F71" s="230"/>
-      <c r="G71" s="231"/>
-      <c r="H71" s="217"/>
-      <c r="I71" s="218"/>
-      <c r="J71" s="219"/>
-      <c r="K71" s="122"/>
-      <c r="L71" s="123"/>
-    </row>
-    <row r="72" spans="2:12" ht="15" thickTop="1">
-      <c r="J72" s="61"/>
-      <c r="K72" s="61"/>
-      <c r="L72" s="61"/>
+      <c r="B65" s="229"/>
+      <c r="C65" s="230"/>
+      <c r="D65" s="230"/>
+      <c r="E65" s="224"/>
+      <c r="F65" s="223"/>
+      <c r="G65" s="224"/>
+      <c r="H65" s="209"/>
+      <c r="I65" s="210"/>
+      <c r="J65" s="211"/>
+      <c r="K65" s="129"/>
+      <c r="L65" s="130"/>
+    </row>
+    <row r="66" spans="2:12" ht="16.2" customHeight="1" thickBot="1">
+      <c r="B66" s="231"/>
+      <c r="C66" s="232"/>
+      <c r="D66" s="232"/>
+      <c r="E66" s="226"/>
+      <c r="F66" s="225"/>
+      <c r="G66" s="226"/>
+      <c r="H66" s="212"/>
+      <c r="I66" s="213"/>
+      <c r="J66" s="214"/>
+      <c r="K66" s="122"/>
+      <c r="L66" s="123"/>
+    </row>
+    <row r="67" spans="2:12" ht="15" thickTop="1">
+      <c r="J67" s="61"/>
+      <c r="K67" s="61"/>
+      <c r="L67" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="71">
     <mergeCell ref="C22:E22"/>
+    <mergeCell ref="K59:L59"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="C19:E19"/>
@@ -42240,13 +42150,13 @@
     <mergeCell ref="C36:I36"/>
     <mergeCell ref="C37:I37"/>
     <mergeCell ref="C38:I38"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="H63:J63"/>
-    <mergeCell ref="H64:J71"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="H60:J60"/>
+    <mergeCell ref="H61:J66"/>
     <mergeCell ref="B49:J50"/>
-    <mergeCell ref="F64:G71"/>
-    <mergeCell ref="B64:E71"/>
+    <mergeCell ref="F61:G66"/>
+    <mergeCell ref="B61:E66"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="B23:E23"/>
@@ -42265,10 +42175,9 @@
     <mergeCell ref="G22:H22"/>
     <mergeCell ref="C24:I25"/>
     <mergeCell ref="J24:L24"/>
-    <mergeCell ref="K57:L57"/>
     <mergeCell ref="K58:L58"/>
     <mergeCell ref="K51:L51"/>
-    <mergeCell ref="C51:I61"/>
+    <mergeCell ref="C51:I58"/>
     <mergeCell ref="K50:L50"/>
     <mergeCell ref="K49:L49"/>
     <mergeCell ref="C26:I26"/>
@@ -42287,7 +42196,7 @@
     <mergeCell ref="K10:L10"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:L48">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>AND($B26&lt;&gt;"",$J26="",$L26&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -42325,40 +42234,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="257"/>
-      <c r="C1" s="257"/>
-      <c r="D1" s="257"/>
-      <c r="E1" s="257"/>
-      <c r="F1" s="257"/>
-      <c r="G1" s="257"/>
-      <c r="H1" s="257"/>
-      <c r="I1" s="257"/>
-      <c r="J1" s="257"/>
-      <c r="K1" s="257"/>
-      <c r="L1" s="257"/>
-      <c r="M1" s="257"/>
-      <c r="N1" s="257"/>
-      <c r="O1" s="257"/>
-      <c r="P1" s="257"/>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+      <c r="H1" s="252"/>
+      <c r="I1" s="252"/>
+      <c r="J1" s="252"/>
+      <c r="K1" s="252"/>
+      <c r="L1" s="252"/>
+      <c r="M1" s="252"/>
+      <c r="N1" s="252"/>
+      <c r="O1" s="252"/>
+      <c r="P1" s="252"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="255" t="s">
+      <c r="B2" s="250" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="256"/>
-      <c r="D2" s="256"/>
-      <c r="E2" s="256"/>
-      <c r="F2" s="256"/>
-      <c r="G2" s="256"/>
-      <c r="H2" s="256"/>
-      <c r="I2" s="256"/>
-      <c r="J2" s="256"/>
-      <c r="K2" s="256"/>
-      <c r="L2" s="256"/>
-      <c r="M2" s="256"/>
-      <c r="N2" s="256"/>
-      <c r="O2" s="256"/>
-      <c r="P2" s="256"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="251"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="251"/>
+      <c r="I2" s="251"/>
+      <c r="J2" s="251"/>
+      <c r="K2" s="251"/>
+      <c r="L2" s="251"/>
+      <c r="M2" s="251"/>
+      <c r="N2" s="251"/>
+      <c r="O2" s="251"/>
+      <c r="P2" s="251"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -42385,16 +42294,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="263" t="s">
+      <c r="I4" s="258" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="263"/>
-      <c r="K4" s="263"/>
-      <c r="L4" s="263"/>
-      <c r="M4" s="263"/>
-      <c r="N4" s="263"/>
-      <c r="O4" s="263"/>
-      <c r="P4" s="263"/>
+      <c r="J4" s="258"/>
+      <c r="K4" s="258"/>
+      <c r="L4" s="258"/>
+      <c r="M4" s="258"/>
+      <c r="N4" s="258"/>
+      <c r="O4" s="258"/>
+      <c r="P4" s="258"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -42408,14 +42317,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="263"/>
-      <c r="J5" s="263"/>
-      <c r="K5" s="263"/>
-      <c r="L5" s="263"/>
-      <c r="M5" s="263"/>
-      <c r="N5" s="263"/>
-      <c r="O5" s="263"/>
-      <c r="P5" s="263"/>
+      <c r="I5" s="258"/>
+      <c r="J5" s="258"/>
+      <c r="K5" s="258"/>
+      <c r="L5" s="258"/>
+      <c r="M5" s="258"/>
+      <c r="N5" s="258"/>
+      <c r="O5" s="258"/>
+      <c r="P5" s="258"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -42550,70 +42459,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="254" t="s">
+      <c r="B12" s="249" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="254" t="s">
+      <c r="C12" s="249" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="254"/>
-      <c r="E12" s="254"/>
-      <c r="F12" s="254" t="s">
+      <c r="D12" s="249"/>
+      <c r="E12" s="249"/>
+      <c r="F12" s="249" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="254" t="s">
+      <c r="G12" s="249" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="254" t="s">
+      <c r="H12" s="249" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="254" t="s">
+      <c r="I12" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="254" t="s">
+      <c r="J12" s="249" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="254"/>
-      <c r="L12" s="254"/>
-      <c r="M12" s="254"/>
-      <c r="N12" s="254"/>
-      <c r="O12" s="254"/>
-      <c r="P12" s="262" t="s">
+      <c r="K12" s="249"/>
+      <c r="L12" s="249"/>
+      <c r="M12" s="249"/>
+      <c r="N12" s="249"/>
+      <c r="O12" s="249"/>
+      <c r="P12" s="257" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="254"/>
-      <c r="C13" s="254"/>
-      <c r="D13" s="254"/>
-      <c r="E13" s="254"/>
-      <c r="F13" s="254"/>
-      <c r="G13" s="254"/>
-      <c r="H13" s="254"/>
-      <c r="I13" s="254"/>
-      <c r="J13" s="261" t="s">
+      <c r="B13" s="249"/>
+      <c r="C13" s="249"/>
+      <c r="D13" s="249"/>
+      <c r="E13" s="249"/>
+      <c r="F13" s="249"/>
+      <c r="G13" s="249"/>
+      <c r="H13" s="249"/>
+      <c r="I13" s="249"/>
+      <c r="J13" s="256" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="261"/>
-      <c r="L13" s="261" t="s">
+      <c r="K13" s="256"/>
+      <c r="L13" s="256" t="s">
         <v>98</v>
       </c>
-      <c r="M13" s="261"/>
-      <c r="N13" s="261" t="s">
+      <c r="M13" s="256"/>
+      <c r="N13" s="256" t="s">
         <v>99</v>
       </c>
-      <c r="O13" s="261"/>
-      <c r="P13" s="262"/>
+      <c r="O13" s="256"/>
+      <c r="P13" s="257"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="254"/>
-      <c r="C14" s="254"/>
-      <c r="D14" s="254"/>
-      <c r="E14" s="254"/>
-      <c r="F14" s="254"/>
-      <c r="G14" s="254"/>
-      <c r="H14" s="254"/>
-      <c r="I14" s="254"/>
+      <c r="B14" s="249"/>
+      <c r="C14" s="249"/>
+      <c r="D14" s="249"/>
+      <c r="E14" s="249"/>
+      <c r="F14" s="249"/>
+      <c r="G14" s="249"/>
+      <c r="H14" s="249"/>
+      <c r="I14" s="249"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -42632,7 +42541,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="262"/>
+      <c r="P14" s="257"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -42982,7 +42891,7 @@
     <mergeCell ref="I4:P5"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P49">
-    <cfRule type="expression" dxfId="5" priority="13">
+    <cfRule type="expression" dxfId="1" priority="13">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
fix(excel): show work items with cumulative progress and use Roman numerals for headers
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148673E3-5DC4-4721-9482-E7DD71BE303A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA686C7-84B9-4A3A-BBE7-F2415C45845B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2486,10 +2486,6 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="49" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="53" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="60" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2592,9 +2588,6 @@
     </xf>
     <xf numFmtId="2" fontId="33" fillId="4" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3098,18 +3091,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="113" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="24" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -3124,6 +3105,25 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="0" borderId="53" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="0" borderId="53" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="52" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
   </cellXfs>
@@ -4244,40 +4244,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
-      <c r="H1" s="252"/>
-      <c r="I1" s="252"/>
-      <c r="J1" s="252"/>
-      <c r="K1" s="252"/>
-      <c r="L1" s="252"/>
-      <c r="M1" s="252"/>
-      <c r="N1" s="252"/>
-      <c r="O1" s="252"/>
-      <c r="P1" s="252"/>
+      <c r="B1" s="250"/>
+      <c r="C1" s="250"/>
+      <c r="D1" s="250"/>
+      <c r="E1" s="250"/>
+      <c r="F1" s="250"/>
+      <c r="G1" s="250"/>
+      <c r="H1" s="250"/>
+      <c r="I1" s="250"/>
+      <c r="J1" s="250"/>
+      <c r="K1" s="250"/>
+      <c r="L1" s="250"/>
+      <c r="M1" s="250"/>
+      <c r="N1" s="250"/>
+      <c r="O1" s="250"/>
+      <c r="P1" s="250"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="250" t="s">
+      <c r="B2" s="248" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="251"/>
-      <c r="D2" s="251"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="251"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="251"/>
-      <c r="I2" s="251"/>
-      <c r="J2" s="251"/>
-      <c r="K2" s="251"/>
-      <c r="L2" s="251"/>
-      <c r="M2" s="251"/>
-      <c r="N2" s="251"/>
-      <c r="O2" s="251"/>
-      <c r="P2" s="251"/>
+      <c r="C2" s="249"/>
+      <c r="D2" s="249"/>
+      <c r="E2" s="249"/>
+      <c r="F2" s="249"/>
+      <c r="G2" s="249"/>
+      <c r="H2" s="249"/>
+      <c r="I2" s="249"/>
+      <c r="J2" s="249"/>
+      <c r="K2" s="249"/>
+      <c r="L2" s="249"/>
+      <c r="M2" s="249"/>
+      <c r="N2" s="249"/>
+      <c r="O2" s="249"/>
+      <c r="P2" s="249"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4304,16 +4304,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="258" t="s">
+      <c r="I4" s="256" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="258"/>
-      <c r="K4" s="258"/>
-      <c r="L4" s="258"/>
-      <c r="M4" s="258"/>
-      <c r="N4" s="258"/>
-      <c r="O4" s="258"/>
-      <c r="P4" s="258"/>
+      <c r="J4" s="256"/>
+      <c r="K4" s="256"/>
+      <c r="L4" s="256"/>
+      <c r="M4" s="256"/>
+      <c r="N4" s="256"/>
+      <c r="O4" s="256"/>
+      <c r="P4" s="256"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4327,14 +4327,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="258"/>
-      <c r="J5" s="258"/>
-      <c r="K5" s="258"/>
-      <c r="L5" s="258"/>
-      <c r="M5" s="258"/>
-      <c r="N5" s="258"/>
-      <c r="O5" s="258"/>
-      <c r="P5" s="258"/>
+      <c r="I5" s="256"/>
+      <c r="J5" s="256"/>
+      <c r="K5" s="256"/>
+      <c r="L5" s="256"/>
+      <c r="M5" s="256"/>
+      <c r="N5" s="256"/>
+      <c r="O5" s="256"/>
+      <c r="P5" s="256"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4469,70 +4469,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="249" t="s">
+      <c r="B12" s="247" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="249" t="s">
+      <c r="C12" s="247" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="249"/>
-      <c r="E12" s="249"/>
-      <c r="F12" s="249" t="s">
+      <c r="D12" s="247"/>
+      <c r="E12" s="247"/>
+      <c r="F12" s="247" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="249" t="s">
+      <c r="G12" s="247" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="249" t="s">
+      <c r="H12" s="247" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="249" t="s">
+      <c r="I12" s="247" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="249" t="s">
+      <c r="J12" s="247" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="249"/>
-      <c r="L12" s="249"/>
-      <c r="M12" s="249"/>
-      <c r="N12" s="249"/>
-      <c r="O12" s="249"/>
-      <c r="P12" s="257" t="s">
+      <c r="K12" s="247"/>
+      <c r="L12" s="247"/>
+      <c r="M12" s="247"/>
+      <c r="N12" s="247"/>
+      <c r="O12" s="247"/>
+      <c r="P12" s="255" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="249"/>
-      <c r="C13" s="249"/>
-      <c r="D13" s="249"/>
-      <c r="E13" s="249"/>
-      <c r="F13" s="249"/>
-      <c r="G13" s="249"/>
-      <c r="H13" s="249"/>
-      <c r="I13" s="249"/>
-      <c r="J13" s="256" t="s">
+      <c r="B13" s="247"/>
+      <c r="C13" s="247"/>
+      <c r="D13" s="247"/>
+      <c r="E13" s="247"/>
+      <c r="F13" s="247"/>
+      <c r="G13" s="247"/>
+      <c r="H13" s="247"/>
+      <c r="I13" s="247"/>
+      <c r="J13" s="254" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="256"/>
-      <c r="L13" s="256" t="s">
+      <c r="K13" s="254"/>
+      <c r="L13" s="254" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="256"/>
-      <c r="N13" s="256" t="s">
+      <c r="M13" s="254"/>
+      <c r="N13" s="254" t="s">
         <v>95</v>
       </c>
-      <c r="O13" s="256"/>
-      <c r="P13" s="257"/>
+      <c r="O13" s="254"/>
+      <c r="P13" s="255"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="249"/>
-      <c r="C14" s="249"/>
-      <c r="D14" s="249"/>
-      <c r="E14" s="249"/>
-      <c r="F14" s="249"/>
-      <c r="G14" s="249"/>
-      <c r="H14" s="249"/>
-      <c r="I14" s="249"/>
+      <c r="B14" s="247"/>
+      <c r="C14" s="247"/>
+      <c r="D14" s="247"/>
+      <c r="E14" s="247"/>
+      <c r="F14" s="247"/>
+      <c r="G14" s="247"/>
+      <c r="H14" s="247"/>
+      <c r="I14" s="247"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -4551,7 +4551,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="257"/>
+      <c r="P14" s="255"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -4974,38 +4974,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="103.2" customHeight="1">
-      <c r="B1" s="251"/>
-      <c r="C1" s="251"/>
-      <c r="D1" s="251"/>
-      <c r="E1" s="251"/>
-      <c r="F1" s="251"/>
-      <c r="G1" s="251"/>
-      <c r="H1" s="251"/>
-      <c r="I1" s="251"/>
-      <c r="J1" s="251"/>
-      <c r="K1" s="251"/>
-      <c r="L1" s="251"/>
-      <c r="M1" s="251"/>
-      <c r="N1" s="251"/>
-      <c r="O1" s="251"/>
+      <c r="B1" s="249"/>
+      <c r="C1" s="249"/>
+      <c r="D1" s="249"/>
+      <c r="E1" s="249"/>
+      <c r="F1" s="249"/>
+      <c r="G1" s="249"/>
+      <c r="H1" s="249"/>
+      <c r="I1" s="249"/>
+      <c r="J1" s="249"/>
+      <c r="K1" s="249"/>
+      <c r="L1" s="249"/>
+      <c r="M1" s="249"/>
+      <c r="N1" s="249"/>
+      <c r="O1" s="249"/>
     </row>
     <row r="2" spans="2:15" ht="22.95" customHeight="1">
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="257" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="259"/>
-      <c r="D2" s="259"/>
-      <c r="E2" s="259"/>
-      <c r="F2" s="259"/>
-      <c r="G2" s="259"/>
-      <c r="H2" s="259"/>
-      <c r="I2" s="259"/>
-      <c r="J2" s="259"/>
-      <c r="K2" s="259"/>
-      <c r="L2" s="259"/>
-      <c r="M2" s="259"/>
-      <c r="N2" s="259"/>
-      <c r="O2" s="259"/>
+      <c r="C2" s="257"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="257"/>
+      <c r="H2" s="257"/>
+      <c r="I2" s="257"/>
+      <c r="J2" s="257"/>
+      <c r="K2" s="257"/>
+      <c r="L2" s="257"/>
+      <c r="M2" s="257"/>
+      <c r="N2" s="257"/>
+      <c r="O2" s="257"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" t="s">
@@ -5057,179 +5057,179 @@
     </row>
     <row r="9" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="11" spans="2:15" s="58" customFormat="1">
-      <c r="B11" s="260" t="s">
+      <c r="B11" s="258" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="260"/>
-      <c r="D11" s="260"/>
-      <c r="E11" s="260"/>
-      <c r="G11" s="260" t="s">
+      <c r="C11" s="258"/>
+      <c r="D11" s="258"/>
+      <c r="E11" s="258"/>
+      <c r="G11" s="258" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="260"/>
-      <c r="I11" s="260"/>
-      <c r="J11" s="260"/>
-      <c r="L11" s="260" t="s">
+      <c r="H11" s="258"/>
+      <c r="I11" s="258"/>
+      <c r="J11" s="258"/>
+      <c r="L11" s="258" t="s">
         <v>105</v>
       </c>
-      <c r="M11" s="260"/>
-      <c r="N11" s="260"/>
-      <c r="O11" s="260"/>
+      <c r="M11" s="258"/>
+      <c r="N11" s="258"/>
+      <c r="O11" s="258"/>
     </row>
     <row r="12" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="13" spans="2:15">
-      <c r="B13" s="251"/>
-      <c r="C13" s="251"/>
-      <c r="D13" s="251"/>
-      <c r="E13" s="251"/>
-      <c r="G13" s="251"/>
-      <c r="H13" s="251"/>
-      <c r="I13" s="251"/>
-      <c r="J13" s="251"/>
-      <c r="L13" s="251"/>
-      <c r="M13" s="251"/>
-      <c r="N13" s="251"/>
-      <c r="O13" s="251"/>
+      <c r="B13" s="249"/>
+      <c r="C13" s="249"/>
+      <c r="D13" s="249"/>
+      <c r="E13" s="249"/>
+      <c r="G13" s="249"/>
+      <c r="H13" s="249"/>
+      <c r="I13" s="249"/>
+      <c r="J13" s="249"/>
+      <c r="L13" s="249"/>
+      <c r="M13" s="249"/>
+      <c r="N13" s="249"/>
+      <c r="O13" s="249"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="251"/>
-      <c r="C14" s="251"/>
-      <c r="D14" s="251"/>
-      <c r="E14" s="251"/>
-      <c r="G14" s="251"/>
-      <c r="H14" s="251"/>
-      <c r="I14" s="251"/>
-      <c r="J14" s="251"/>
-      <c r="L14" s="251"/>
-      <c r="M14" s="251"/>
-      <c r="N14" s="251"/>
-      <c r="O14" s="251"/>
+      <c r="B14" s="249"/>
+      <c r="C14" s="249"/>
+      <c r="D14" s="249"/>
+      <c r="E14" s="249"/>
+      <c r="G14" s="249"/>
+      <c r="H14" s="249"/>
+      <c r="I14" s="249"/>
+      <c r="J14" s="249"/>
+      <c r="L14" s="249"/>
+      <c r="M14" s="249"/>
+      <c r="N14" s="249"/>
+      <c r="O14" s="249"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="251"/>
-      <c r="C15" s="251"/>
-      <c r="D15" s="251"/>
-      <c r="E15" s="251"/>
-      <c r="G15" s="251"/>
-      <c r="H15" s="251"/>
-      <c r="I15" s="251"/>
-      <c r="J15" s="251"/>
-      <c r="L15" s="251"/>
-      <c r="M15" s="251"/>
-      <c r="N15" s="251"/>
-      <c r="O15" s="251"/>
+      <c r="B15" s="249"/>
+      <c r="C15" s="249"/>
+      <c r="D15" s="249"/>
+      <c r="E15" s="249"/>
+      <c r="G15" s="249"/>
+      <c r="H15" s="249"/>
+      <c r="I15" s="249"/>
+      <c r="J15" s="249"/>
+      <c r="L15" s="249"/>
+      <c r="M15" s="249"/>
+      <c r="N15" s="249"/>
+      <c r="O15" s="249"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="251"/>
-      <c r="C16" s="251"/>
-      <c r="D16" s="251"/>
-      <c r="E16" s="251"/>
-      <c r="G16" s="251"/>
-      <c r="H16" s="251"/>
-      <c r="I16" s="251"/>
-      <c r="J16" s="251"/>
-      <c r="L16" s="251"/>
-      <c r="M16" s="251"/>
-      <c r="N16" s="251"/>
-      <c r="O16" s="251"/>
+      <c r="B16" s="249"/>
+      <c r="C16" s="249"/>
+      <c r="D16" s="249"/>
+      <c r="E16" s="249"/>
+      <c r="G16" s="249"/>
+      <c r="H16" s="249"/>
+      <c r="I16" s="249"/>
+      <c r="J16" s="249"/>
+      <c r="L16" s="249"/>
+      <c r="M16" s="249"/>
+      <c r="N16" s="249"/>
+      <c r="O16" s="249"/>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="251"/>
-      <c r="C17" s="251"/>
-      <c r="D17" s="251"/>
-      <c r="E17" s="251"/>
-      <c r="G17" s="251"/>
-      <c r="H17" s="251"/>
-      <c r="I17" s="251"/>
-      <c r="J17" s="251"/>
-      <c r="L17" s="251"/>
-      <c r="M17" s="251"/>
-      <c r="N17" s="251"/>
-      <c r="O17" s="251"/>
+      <c r="B17" s="249"/>
+      <c r="C17" s="249"/>
+      <c r="D17" s="249"/>
+      <c r="E17" s="249"/>
+      <c r="G17" s="249"/>
+      <c r="H17" s="249"/>
+      <c r="I17" s="249"/>
+      <c r="J17" s="249"/>
+      <c r="L17" s="249"/>
+      <c r="M17" s="249"/>
+      <c r="N17" s="249"/>
+      <c r="O17" s="249"/>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="251"/>
-      <c r="C18" s="251"/>
-      <c r="D18" s="251"/>
-      <c r="E18" s="251"/>
-      <c r="G18" s="251"/>
-      <c r="H18" s="251"/>
-      <c r="I18" s="251"/>
-      <c r="J18" s="251"/>
-      <c r="L18" s="251"/>
-      <c r="M18" s="251"/>
-      <c r="N18" s="251"/>
-      <c r="O18" s="251"/>
+      <c r="B18" s="249"/>
+      <c r="C18" s="249"/>
+      <c r="D18" s="249"/>
+      <c r="E18" s="249"/>
+      <c r="G18" s="249"/>
+      <c r="H18" s="249"/>
+      <c r="I18" s="249"/>
+      <c r="J18" s="249"/>
+      <c r="L18" s="249"/>
+      <c r="M18" s="249"/>
+      <c r="N18" s="249"/>
+      <c r="O18" s="249"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="B19" s="251"/>
-      <c r="C19" s="251"/>
-      <c r="D19" s="251"/>
-      <c r="E19" s="251"/>
-      <c r="G19" s="251"/>
-      <c r="H19" s="251"/>
-      <c r="I19" s="251"/>
-      <c r="J19" s="251"/>
-      <c r="L19" s="251"/>
-      <c r="M19" s="251"/>
-      <c r="N19" s="251"/>
-      <c r="O19" s="251"/>
+      <c r="B19" s="249"/>
+      <c r="C19" s="249"/>
+      <c r="D19" s="249"/>
+      <c r="E19" s="249"/>
+      <c r="G19" s="249"/>
+      <c r="H19" s="249"/>
+      <c r="I19" s="249"/>
+      <c r="J19" s="249"/>
+      <c r="L19" s="249"/>
+      <c r="M19" s="249"/>
+      <c r="N19" s="249"/>
+      <c r="O19" s="249"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="B20" s="251"/>
-      <c r="C20" s="251"/>
-      <c r="D20" s="251"/>
-      <c r="E20" s="251"/>
-      <c r="G20" s="251"/>
-      <c r="H20" s="251"/>
-      <c r="I20" s="251"/>
-      <c r="J20" s="251"/>
-      <c r="L20" s="251"/>
-      <c r="M20" s="251"/>
-      <c r="N20" s="251"/>
-      <c r="O20" s="251"/>
+      <c r="B20" s="249"/>
+      <c r="C20" s="249"/>
+      <c r="D20" s="249"/>
+      <c r="E20" s="249"/>
+      <c r="G20" s="249"/>
+      <c r="H20" s="249"/>
+      <c r="I20" s="249"/>
+      <c r="J20" s="249"/>
+      <c r="L20" s="249"/>
+      <c r="M20" s="249"/>
+      <c r="N20" s="249"/>
+      <c r="O20" s="249"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="B21" s="251"/>
-      <c r="C21" s="251"/>
-      <c r="D21" s="251"/>
-      <c r="E21" s="251"/>
-      <c r="G21" s="251"/>
-      <c r="H21" s="251"/>
-      <c r="I21" s="251"/>
-      <c r="J21" s="251"/>
-      <c r="L21" s="251"/>
-      <c r="M21" s="251"/>
-      <c r="N21" s="251"/>
-      <c r="O21" s="251"/>
+      <c r="B21" s="249"/>
+      <c r="C21" s="249"/>
+      <c r="D21" s="249"/>
+      <c r="E21" s="249"/>
+      <c r="G21" s="249"/>
+      <c r="H21" s="249"/>
+      <c r="I21" s="249"/>
+      <c r="J21" s="249"/>
+      <c r="L21" s="249"/>
+      <c r="M21" s="249"/>
+      <c r="N21" s="249"/>
+      <c r="O21" s="249"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="B22" s="251"/>
-      <c r="C22" s="251"/>
-      <c r="D22" s="251"/>
-      <c r="E22" s="251"/>
-      <c r="G22" s="251"/>
-      <c r="H22" s="251"/>
-      <c r="I22" s="251"/>
-      <c r="J22" s="251"/>
-      <c r="L22" s="251"/>
-      <c r="M22" s="251"/>
-      <c r="N22" s="251"/>
-      <c r="O22" s="251"/>
+      <c r="B22" s="249"/>
+      <c r="C22" s="249"/>
+      <c r="D22" s="249"/>
+      <c r="E22" s="249"/>
+      <c r="G22" s="249"/>
+      <c r="H22" s="249"/>
+      <c r="I22" s="249"/>
+      <c r="J22" s="249"/>
+      <c r="L22" s="249"/>
+      <c r="M22" s="249"/>
+      <c r="N22" s="249"/>
+      <c r="O22" s="249"/>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="251"/>
-      <c r="C23" s="251"/>
-      <c r="D23" s="251"/>
-      <c r="E23" s="251"/>
-      <c r="G23" s="251"/>
-      <c r="H23" s="251"/>
-      <c r="I23" s="251"/>
-      <c r="J23" s="251"/>
-      <c r="L23" s="251"/>
-      <c r="M23" s="251"/>
-      <c r="N23" s="251"/>
-      <c r="O23" s="251"/>
+      <c r="B23" s="249"/>
+      <c r="C23" s="249"/>
+      <c r="D23" s="249"/>
+      <c r="E23" s="249"/>
+      <c r="G23" s="249"/>
+      <c r="H23" s="249"/>
+      <c r="I23" s="249"/>
+      <c r="J23" s="249"/>
+      <c r="L23" s="249"/>
+      <c r="M23" s="249"/>
+      <c r="N23" s="249"/>
+      <c r="O23" s="249"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5263,330 +5263,330 @@
   <sheetData>
     <row r="1" spans="2:29" ht="4.8" customHeight="1" thickBot="1"/>
     <row r="2" spans="2:29" ht="19.95" customHeight="1" thickBot="1">
-      <c r="B2" s="261" t="s">
+      <c r="B2" s="259" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="262"/>
-      <c r="D2" s="262"/>
-      <c r="E2" s="262"/>
-      <c r="F2" s="262"/>
-      <c r="G2" s="262"/>
-      <c r="H2" s="262"/>
-      <c r="I2" s="262"/>
-      <c r="J2" s="262"/>
-      <c r="K2" s="262"/>
-      <c r="L2" s="262"/>
-      <c r="M2" s="262"/>
-      <c r="N2" s="262"/>
-      <c r="O2" s="262"/>
-      <c r="P2" s="262"/>
-      <c r="Q2" s="262"/>
-      <c r="R2" s="262"/>
-      <c r="S2" s="262"/>
-      <c r="T2" s="262"/>
-      <c r="U2" s="262"/>
-      <c r="V2" s="262"/>
-      <c r="W2" s="262"/>
-      <c r="X2" s="262"/>
-      <c r="Y2" s="262"/>
-      <c r="Z2" s="262"/>
-      <c r="AA2" s="262"/>
-      <c r="AB2" s="263"/>
-      <c r="AC2" s="138"/>
+      <c r="C2" s="260"/>
+      <c r="D2" s="260"/>
+      <c r="E2" s="260"/>
+      <c r="F2" s="260"/>
+      <c r="G2" s="260"/>
+      <c r="H2" s="260"/>
+      <c r="I2" s="260"/>
+      <c r="J2" s="260"/>
+      <c r="K2" s="260"/>
+      <c r="L2" s="260"/>
+      <c r="M2" s="260"/>
+      <c r="N2" s="260"/>
+      <c r="O2" s="260"/>
+      <c r="P2" s="260"/>
+      <c r="Q2" s="260"/>
+      <c r="R2" s="260"/>
+      <c r="S2" s="260"/>
+      <c r="T2" s="260"/>
+      <c r="U2" s="260"/>
+      <c r="V2" s="260"/>
+      <c r="W2" s="260"/>
+      <c r="X2" s="260"/>
+      <c r="Y2" s="260"/>
+      <c r="Z2" s="260"/>
+      <c r="AA2" s="260"/>
+      <c r="AB2" s="261"/>
+      <c r="AC2" s="137"/>
     </row>
     <row r="3" spans="2:29" ht="15" customHeight="1">
-      <c r="B3" s="137"/>
-      <c r="AB3" s="132"/>
+      <c r="B3" s="136"/>
+      <c r="AB3" s="131"/>
     </row>
     <row r="4" spans="2:29" ht="15" customHeight="1">
-      <c r="B4" s="131" t="s">
+      <c r="B4" s="130" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="133" t="s">
+      <c r="D4" s="132" t="s">
         <v>20</v>
       </c>
-      <c r="AB4" s="132"/>
+      <c r="AB4" s="131"/>
     </row>
     <row r="5" spans="2:29" ht="15" customHeight="1">
-      <c r="B5" s="131" t="s">
+      <c r="B5" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="D5" s="133" t="s">
+      <c r="D5" s="132" t="s">
         <v>20</v>
       </c>
-      <c r="AB5" s="132"/>
+      <c r="AB5" s="131"/>
     </row>
     <row r="6" spans="2:29" ht="15" customHeight="1">
-      <c r="B6" s="131" t="s">
+      <c r="B6" s="130" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="133" t="s">
+      <c r="D6" s="132" t="s">
         <v>20</v>
       </c>
-      <c r="AB6" s="132"/>
+      <c r="AB6" s="131"/>
     </row>
     <row r="7" spans="2:29" ht="15" customHeight="1">
-      <c r="B7" s="131" t="s">
+      <c r="B7" s="130" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="133" t="s">
+      <c r="D7" s="132" t="s">
         <v>20</v>
       </c>
-      <c r="AB7" s="132"/>
+      <c r="AB7" s="131"/>
     </row>
     <row r="8" spans="2:29" ht="15" customHeight="1">
-      <c r="B8" s="131" t="s">
+      <c r="B8" s="130" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="133" t="s">
+      <c r="D8" s="132" t="s">
         <v>20</v>
       </c>
-      <c r="AB8" s="132"/>
+      <c r="AB8" s="131"/>
     </row>
     <row r="9" spans="2:29" ht="15" customHeight="1">
-      <c r="B9" s="131" t="s">
+      <c r="B9" s="130" t="s">
         <v>110</v>
       </c>
-      <c r="D9" s="133" t="s">
+      <c r="D9" s="132" t="s">
         <v>20</v>
       </c>
-      <c r="AB9" s="132"/>
+      <c r="AB9" s="131"/>
     </row>
     <row r="10" spans="2:29" ht="15" customHeight="1">
-      <c r="B10" s="131" t="s">
+      <c r="B10" s="130" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="133" t="s">
+      <c r="D10" s="132" t="s">
         <v>20</v>
       </c>
-      <c r="AB10" s="132"/>
+      <c r="AB10" s="131"/>
     </row>
     <row r="11" spans="2:29" ht="15" customHeight="1" thickBot="1">
-      <c r="B11" s="134"/>
-      <c r="C11" s="135"/>
-      <c r="D11" s="135"/>
-      <c r="E11" s="135"/>
-      <c r="F11" s="135"/>
-      <c r="G11" s="135"/>
-      <c r="H11" s="135"/>
-      <c r="I11" s="135"/>
-      <c r="J11" s="135"/>
-      <c r="K11" s="135"/>
-      <c r="L11" s="135"/>
-      <c r="M11" s="135"/>
-      <c r="N11" s="135"/>
-      <c r="O11" s="135"/>
-      <c r="P11" s="135"/>
-      <c r="Q11" s="135"/>
-      <c r="R11" s="135"/>
-      <c r="S11" s="135"/>
-      <c r="T11" s="135"/>
-      <c r="U11" s="135"/>
-      <c r="V11" s="135"/>
-      <c r="W11" s="135"/>
-      <c r="X11" s="135"/>
-      <c r="Y11" s="135"/>
-      <c r="Z11" s="135"/>
-      <c r="AA11" s="135"/>
-      <c r="AB11" s="136"/>
+      <c r="B11" s="133"/>
+      <c r="C11" s="134"/>
+      <c r="D11" s="134"/>
+      <c r="E11" s="134"/>
+      <c r="F11" s="134"/>
+      <c r="G11" s="134"/>
+      <c r="H11" s="134"/>
+      <c r="I11" s="134"/>
+      <c r="J11" s="134"/>
+      <c r="K11" s="134"/>
+      <c r="L11" s="134"/>
+      <c r="M11" s="134"/>
+      <c r="N11" s="134"/>
+      <c r="O11" s="134"/>
+      <c r="P11" s="134"/>
+      <c r="Q11" s="134"/>
+      <c r="R11" s="134"/>
+      <c r="S11" s="134"/>
+      <c r="T11" s="134"/>
+      <c r="U11" s="134"/>
+      <c r="V11" s="134"/>
+      <c r="W11" s="134"/>
+      <c r="X11" s="134"/>
+      <c r="Y11" s="134"/>
+      <c r="Z11" s="134"/>
+      <c r="AA11" s="134"/>
+      <c r="AB11" s="135"/>
     </row>
     <row r="12" spans="2:29" ht="15" customHeight="1">
-      <c r="B12" s="273" t="s">
+      <c r="B12" s="271" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="275" t="s">
+      <c r="C12" s="273" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="276"/>
-      <c r="E12" s="276"/>
-      <c r="F12" s="276"/>
-      <c r="G12" s="276"/>
-      <c r="H12" s="276"/>
-      <c r="I12" s="276"/>
-      <c r="J12" s="276"/>
-      <c r="K12" s="276"/>
-      <c r="L12" s="277"/>
-      <c r="M12" s="281" t="s">
+      <c r="D12" s="274"/>
+      <c r="E12" s="274"/>
+      <c r="F12" s="274"/>
+      <c r="G12" s="274"/>
+      <c r="H12" s="274"/>
+      <c r="I12" s="274"/>
+      <c r="J12" s="274"/>
+      <c r="K12" s="274"/>
+      <c r="L12" s="275"/>
+      <c r="M12" s="279" t="s">
         <v>113</v>
       </c>
-      <c r="N12" s="281" t="s">
+      <c r="N12" s="279" t="s">
         <v>34</v>
       </c>
-      <c r="O12" s="286" t="s">
+      <c r="O12" s="284" t="s">
         <v>114</v>
       </c>
-      <c r="P12" s="286"/>
-      <c r="Q12" s="286"/>
-      <c r="R12" s="286"/>
-      <c r="S12" s="286"/>
-      <c r="T12" s="286"/>
-      <c r="U12" s="286"/>
-      <c r="V12" s="286"/>
-      <c r="W12" s="286"/>
-      <c r="X12" s="286"/>
-      <c r="Y12" s="286"/>
-      <c r="Z12" s="286"/>
-      <c r="AA12" s="286"/>
-      <c r="AB12" s="287"/>
+      <c r="P12" s="284"/>
+      <c r="Q12" s="284"/>
+      <c r="R12" s="284"/>
+      <c r="S12" s="284"/>
+      <c r="T12" s="284"/>
+      <c r="U12" s="284"/>
+      <c r="V12" s="284"/>
+      <c r="W12" s="284"/>
+      <c r="X12" s="284"/>
+      <c r="Y12" s="284"/>
+      <c r="Z12" s="284"/>
+      <c r="AA12" s="284"/>
+      <c r="AB12" s="285"/>
     </row>
     <row r="13" spans="2:29" ht="15" customHeight="1">
-      <c r="B13" s="274"/>
-      <c r="C13" s="278"/>
-      <c r="D13" s="279"/>
-      <c r="E13" s="279"/>
-      <c r="F13" s="279"/>
-      <c r="G13" s="279"/>
-      <c r="H13" s="279"/>
-      <c r="I13" s="279"/>
-      <c r="J13" s="279"/>
-      <c r="K13" s="279"/>
-      <c r="L13" s="280"/>
-      <c r="M13" s="282"/>
-      <c r="N13" s="282"/>
-      <c r="O13" s="283" t="s">
+      <c r="B13" s="272"/>
+      <c r="C13" s="276"/>
+      <c r="D13" s="277"/>
+      <c r="E13" s="277"/>
+      <c r="F13" s="277"/>
+      <c r="G13" s="277"/>
+      <c r="H13" s="277"/>
+      <c r="I13" s="277"/>
+      <c r="J13" s="277"/>
+      <c r="K13" s="277"/>
+      <c r="L13" s="278"/>
+      <c r="M13" s="280"/>
+      <c r="N13" s="280"/>
+      <c r="O13" s="281" t="s">
         <v>115</v>
       </c>
-      <c r="P13" s="284"/>
-      <c r="Q13" s="285"/>
-      <c r="R13" s="283" t="s">
+      <c r="P13" s="282"/>
+      <c r="Q13" s="283"/>
+      <c r="R13" s="281" t="s">
         <v>116</v>
       </c>
-      <c r="S13" s="284"/>
-      <c r="T13" s="285"/>
-      <c r="U13" s="283" t="s">
+      <c r="S13" s="282"/>
+      <c r="T13" s="283"/>
+      <c r="U13" s="281" t="s">
         <v>117</v>
       </c>
-      <c r="V13" s="284"/>
-      <c r="W13" s="285"/>
-      <c r="X13" s="264" t="s">
+      <c r="V13" s="282"/>
+      <c r="W13" s="283"/>
+      <c r="X13" s="262" t="s">
         <v>118</v>
       </c>
-      <c r="Y13" s="143" t="s">
+      <c r="Y13" s="142" t="s">
         <v>119</v>
       </c>
-      <c r="Z13" s="144" t="s">
+      <c r="Z13" s="143" t="s">
         <v>119</v>
       </c>
-      <c r="AA13" s="266" t="s">
+      <c r="AA13" s="264" t="s">
         <v>120</v>
       </c>
-      <c r="AB13" s="268" t="s">
+      <c r="AB13" s="266" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="14" spans="2:29" ht="15" customHeight="1">
-      <c r="B14" s="274"/>
-      <c r="C14" s="278"/>
-      <c r="D14" s="279"/>
-      <c r="E14" s="279"/>
-      <c r="F14" s="279"/>
-      <c r="G14" s="279"/>
-      <c r="H14" s="279"/>
-      <c r="I14" s="279"/>
-      <c r="J14" s="279"/>
-      <c r="K14" s="279"/>
-      <c r="L14" s="280"/>
-      <c r="M14" s="265"/>
-      <c r="N14" s="265"/>
-      <c r="O14" s="145" t="s">
+      <c r="B14" s="272"/>
+      <c r="C14" s="276"/>
+      <c r="D14" s="277"/>
+      <c r="E14" s="277"/>
+      <c r="F14" s="277"/>
+      <c r="G14" s="277"/>
+      <c r="H14" s="277"/>
+      <c r="I14" s="277"/>
+      <c r="J14" s="277"/>
+      <c r="K14" s="277"/>
+      <c r="L14" s="278"/>
+      <c r="M14" s="263"/>
+      <c r="N14" s="263"/>
+      <c r="O14" s="144" t="s">
         <v>122</v>
       </c>
-      <c r="P14" s="145" t="s">
+      <c r="P14" s="144" t="s">
         <v>123</v>
       </c>
-      <c r="Q14" s="145" t="s">
+      <c r="Q14" s="144" t="s">
         <v>124</v>
       </c>
-      <c r="R14" s="145" t="s">
+      <c r="R14" s="144" t="s">
         <v>125</v>
       </c>
-      <c r="S14" s="145" t="s">
+      <c r="S14" s="144" t="s">
         <v>126</v>
       </c>
-      <c r="T14" s="145" t="s">
+      <c r="T14" s="144" t="s">
         <v>124</v>
       </c>
-      <c r="U14" s="145" t="s">
+      <c r="U14" s="144" t="s">
         <v>127</v>
       </c>
-      <c r="V14" s="145" t="s">
+      <c r="V14" s="144" t="s">
         <v>128</v>
       </c>
-      <c r="W14" s="145" t="s">
+      <c r="W14" s="144" t="s">
         <v>129</v>
       </c>
-      <c r="X14" s="265"/>
-      <c r="Y14" s="143" t="s">
+      <c r="X14" s="263"/>
+      <c r="Y14" s="142" t="s">
         <v>130</v>
       </c>
-      <c r="Z14" s="145" t="s">
+      <c r="Z14" s="144" t="s">
         <v>131</v>
       </c>
-      <c r="AA14" s="267"/>
-      <c r="AB14" s="269"/>
+      <c r="AA14" s="265"/>
+      <c r="AB14" s="267"/>
     </row>
     <row r="15" spans="2:29" ht="15" customHeight="1" thickBot="1">
-      <c r="B15" s="139">
+      <c r="B15" s="138">
         <v>1</v>
       </c>
-      <c r="C15" s="270">
+      <c r="C15" s="268">
         <v>2</v>
       </c>
-      <c r="D15" s="271"/>
-      <c r="E15" s="271"/>
-      <c r="F15" s="271"/>
-      <c r="G15" s="271"/>
-      <c r="H15" s="271"/>
-      <c r="I15" s="271"/>
-      <c r="J15" s="271"/>
-      <c r="K15" s="271"/>
-      <c r="L15" s="272"/>
-      <c r="M15" s="140">
+      <c r="D15" s="269"/>
+      <c r="E15" s="269"/>
+      <c r="F15" s="269"/>
+      <c r="G15" s="269"/>
+      <c r="H15" s="269"/>
+      <c r="I15" s="269"/>
+      <c r="J15" s="269"/>
+      <c r="K15" s="269"/>
+      <c r="L15" s="270"/>
+      <c r="M15" s="139">
         <v>3</v>
       </c>
-      <c r="N15" s="140">
+      <c r="N15" s="139">
         <v>4</v>
       </c>
-      <c r="O15" s="141">
+      <c r="O15" s="140">
         <v>5</v>
       </c>
-      <c r="P15" s="141">
+      <c r="P15" s="140">
         <v>6</v>
       </c>
-      <c r="Q15" s="141">
+      <c r="Q15" s="140">
         <v>7</v>
       </c>
-      <c r="R15" s="141">
+      <c r="R15" s="140">
         <v>8</v>
       </c>
-      <c r="S15" s="141">
+      <c r="S15" s="140">
         <v>9</v>
       </c>
-      <c r="T15" s="141">
+      <c r="T15" s="140">
         <v>10</v>
       </c>
-      <c r="U15" s="141">
+      <c r="U15" s="140">
         <v>11</v>
       </c>
-      <c r="V15" s="141">
+      <c r="V15" s="140">
         <v>12</v>
       </c>
-      <c r="W15" s="141">
+      <c r="W15" s="140">
         <v>13</v>
       </c>
-      <c r="X15" s="141">
+      <c r="X15" s="140">
         <v>14</v>
       </c>
-      <c r="Y15" s="141">
+      <c r="Y15" s="140">
         <v>15</v>
       </c>
-      <c r="Z15" s="141">
+      <c r="Z15" s="140">
         <v>16</v>
       </c>
-      <c r="AA15" s="141">
+      <c r="AA15" s="140">
         <v>17</v>
       </c>
-      <c r="AB15" s="142">
+      <c r="AB15" s="141">
         <v>18</v>
       </c>
     </row>
@@ -5630,38 +5630,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="248"/>
-      <c r="C1" s="248"/>
-      <c r="D1" s="248"/>
-      <c r="E1" s="248"/>
-      <c r="F1" s="248"/>
-      <c r="G1" s="248"/>
-      <c r="H1" s="248"/>
-      <c r="I1" s="248"/>
+      <c r="B1" s="246"/>
+      <c r="C1" s="246"/>
+      <c r="D1" s="246"/>
+      <c r="E1" s="246"/>
+      <c r="F1" s="246"/>
+      <c r="G1" s="246"/>
+      <c r="H1" s="246"/>
+      <c r="I1" s="246"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="245" t="s">
+      <c r="B2" s="243" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="245"/>
-      <c r="D2" s="245"/>
-      <c r="E2" s="245"/>
-      <c r="F2" s="245"/>
-      <c r="G2" s="245"/>
-      <c r="H2" s="245"/>
-      <c r="I2" s="245"/>
+      <c r="C2" s="243"/>
+      <c r="D2" s="243"/>
+      <c r="E2" s="243"/>
+      <c r="F2" s="243"/>
+      <c r="G2" s="243"/>
+      <c r="H2" s="243"/>
+      <c r="I2" s="243"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="246" t="s">
+      <c r="B3" s="244" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="246"/>
-      <c r="D3" s="246"/>
-      <c r="E3" s="246"/>
-      <c r="F3" s="246"/>
-      <c r="G3" s="246"/>
-      <c r="H3" s="246"/>
-      <c r="I3" s="246"/>
+      <c r="C3" s="244"/>
+      <c r="D3" s="244"/>
+      <c r="E3" s="244"/>
+      <c r="F3" s="244"/>
+      <c r="G3" s="244"/>
+      <c r="H3" s="244"/>
+      <c r="I3" s="244"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -5669,10 +5669,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="247" t="s">
+      <c r="C5" s="245" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="247"/>
+      <c r="D5" s="245"/>
       <c r="E5" s="11" t="s">
         <v>38</v>
       </c>
@@ -14059,63 +14059,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="248"/>
-      <c r="C1" s="248"/>
-      <c r="D1" s="248"/>
-      <c r="E1" s="248"/>
-      <c r="F1" s="248"/>
-      <c r="G1" s="248"/>
-      <c r="H1" s="248"/>
-      <c r="I1" s="248"/>
-      <c r="J1" s="248"/>
-      <c r="K1" s="248"/>
-      <c r="L1" s="248"/>
-      <c r="M1" s="248"/>
-      <c r="N1" s="248"/>
+      <c r="B1" s="246"/>
+      <c r="C1" s="246"/>
+      <c r="D1" s="246"/>
+      <c r="E1" s="246"/>
+      <c r="F1" s="246"/>
+      <c r="G1" s="246"/>
+      <c r="H1" s="246"/>
+      <c r="I1" s="246"/>
+      <c r="J1" s="246"/>
+      <c r="K1" s="246"/>
+      <c r="L1" s="246"/>
+      <c r="M1" s="246"/>
+      <c r="N1" s="246"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="245" t="s">
+      <c r="B2" s="243" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="245"/>
-      <c r="D2" s="245"/>
-      <c r="E2" s="245"/>
-      <c r="F2" s="245"/>
-      <c r="G2" s="245"/>
-      <c r="H2" s="245"/>
-      <c r="I2" s="245"/>
-      <c r="J2" s="245"/>
-      <c r="K2" s="245"/>
-      <c r="L2" s="245"/>
-      <c r="M2" s="245"/>
-      <c r="N2" s="245"/>
+      <c r="C2" s="243"/>
+      <c r="D2" s="243"/>
+      <c r="E2" s="243"/>
+      <c r="F2" s="243"/>
+      <c r="G2" s="243"/>
+      <c r="H2" s="243"/>
+      <c r="I2" s="243"/>
+      <c r="J2" s="243"/>
+      <c r="K2" s="243"/>
+      <c r="L2" s="243"/>
+      <c r="M2" s="243"/>
+      <c r="N2" s="243"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="246" t="s">
+      <c r="B3" s="244" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="246"/>
-      <c r="D3" s="246"/>
-      <c r="E3" s="246"/>
-      <c r="F3" s="246"/>
-      <c r="G3" s="246"/>
-      <c r="H3" s="246"/>
-      <c r="I3" s="246"/>
-      <c r="J3" s="246"/>
-      <c r="K3" s="246"/>
-      <c r="L3" s="246"/>
-      <c r="M3" s="246"/>
-      <c r="N3" s="246"/>
+      <c r="C3" s="244"/>
+      <c r="D3" s="244"/>
+      <c r="E3" s="244"/>
+      <c r="F3" s="244"/>
+      <c r="G3" s="244"/>
+      <c r="H3" s="244"/>
+      <c r="I3" s="244"/>
+      <c r="J3" s="244"/>
+      <c r="K3" s="244"/>
+      <c r="L3" s="244"/>
+      <c r="M3" s="244"/>
+      <c r="N3" s="244"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="249" t="s">
+      <c r="C5" s="247" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="249"/>
+      <c r="D5" s="247"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -16319,35 +16319,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="248"/>
-      <c r="C1" s="248"/>
-      <c r="D1" s="248"/>
-      <c r="E1" s="248"/>
-      <c r="F1" s="248"/>
-      <c r="G1" s="248"/>
-      <c r="H1" s="248"/>
+      <c r="B1" s="246"/>
+      <c r="C1" s="246"/>
+      <c r="D1" s="246"/>
+      <c r="E1" s="246"/>
+      <c r="F1" s="246"/>
+      <c r="G1" s="246"/>
+      <c r="H1" s="246"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="245" t="s">
+      <c r="B2" s="243" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="245"/>
-      <c r="D2" s="245"/>
-      <c r="E2" s="245"/>
-      <c r="F2" s="245"/>
-      <c r="G2" s="245"/>
-      <c r="H2" s="245"/>
+      <c r="C2" s="243"/>
+      <c r="D2" s="243"/>
+      <c r="E2" s="243"/>
+      <c r="F2" s="243"/>
+      <c r="G2" s="243"/>
+      <c r="H2" s="243"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="246" t="s">
+      <c r="B3" s="244" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="246"/>
-      <c r="D3" s="246"/>
-      <c r="E3" s="246"/>
-      <c r="F3" s="246"/>
-      <c r="G3" s="246"/>
-      <c r="H3" s="246"/>
+      <c r="C3" s="244"/>
+      <c r="D3" s="244"/>
+      <c r="E3" s="244"/>
+      <c r="F3" s="244"/>
+      <c r="G3" s="244"/>
+      <c r="H3" s="244"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -40441,30 +40441,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
-      <c r="H1" s="252"/>
-      <c r="I1" s="252"/>
-      <c r="J1" s="252"/>
-      <c r="K1" s="252"/>
+      <c r="B1" s="250"/>
+      <c r="C1" s="250"/>
+      <c r="D1" s="250"/>
+      <c r="E1" s="250"/>
+      <c r="F1" s="250"/>
+      <c r="G1" s="250"/>
+      <c r="H1" s="250"/>
+      <c r="I1" s="250"/>
+      <c r="J1" s="250"/>
+      <c r="K1" s="250"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="250" t="s">
+      <c r="B2" s="248" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="251"/>
-      <c r="D2" s="251"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="251"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="251"/>
-      <c r="I2" s="251"/>
-      <c r="J2" s="251"/>
-      <c r="K2" s="251"/>
+      <c r="C2" s="249"/>
+      <c r="D2" s="249"/>
+      <c r="E2" s="249"/>
+      <c r="F2" s="249"/>
+      <c r="G2" s="249"/>
+      <c r="H2" s="249"/>
+      <c r="I2" s="249"/>
+      <c r="J2" s="249"/>
+      <c r="K2" s="249"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40584,11 +40584,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="249" t="s">
+      <c r="C11" s="247" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="249"/>
-      <c r="E11" s="249"/>
+      <c r="D11" s="247"/>
+      <c r="E11" s="247"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -40644,26 +40644,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="111.6" customHeight="1">
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
-      <c r="H1" s="252"/>
-      <c r="I1" s="252"/>
+      <c r="B1" s="250"/>
+      <c r="C1" s="250"/>
+      <c r="D1" s="250"/>
+      <c r="E1" s="250"/>
+      <c r="F1" s="250"/>
+      <c r="G1" s="250"/>
+      <c r="H1" s="250"/>
+      <c r="I1" s="250"/>
     </row>
     <row r="2" spans="2:9" ht="22.95" customHeight="1">
-      <c r="B2" s="250" t="s">
+      <c r="B2" s="248" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="251"/>
-      <c r="D2" s="251"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="251"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="251"/>
-      <c r="I2" s="251"/>
+      <c r="C2" s="249"/>
+      <c r="D2" s="249"/>
+      <c r="E2" s="249"/>
+      <c r="F2" s="249"/>
+      <c r="G2" s="249"/>
+      <c r="H2" s="249"/>
+      <c r="I2" s="249"/>
     </row>
     <row r="3" spans="2:9" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40773,12 +40773,12 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="249" t="s">
+      <c r="C11" s="247" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="249"/>
-      <c r="E11" s="249"/>
-      <c r="F11" s="249"/>
+      <c r="D11" s="247"/>
+      <c r="E11" s="247"/>
+      <c r="F11" s="247"/>
       <c r="G11" s="40" t="s">
         <v>29</v>
       </c>
@@ -40816,58 +40816,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
+      <c r="B1" s="250"/>
+      <c r="C1" s="250"/>
+      <c r="D1" s="250"/>
+      <c r="E1" s="250"/>
+      <c r="F1" s="250"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="255" t="s">
+      <c r="B2" s="253" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="255"/>
-      <c r="D2" s="255"/>
-      <c r="E2" s="255"/>
-      <c r="F2" s="255"/>
+      <c r="C2" s="253"/>
+      <c r="D2" s="253"/>
+      <c r="E2" s="253"/>
+      <c r="F2" s="253"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="252"/>
-      <c r="C3" s="252"/>
-      <c r="D3" s="252"/>
-      <c r="E3" s="252"/>
-      <c r="F3" s="252"/>
+      <c r="B3" s="250"/>
+      <c r="C3" s="250"/>
+      <c r="D3" s="250"/>
+      <c r="E3" s="250"/>
+      <c r="F3" s="250"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="253" t="s">
+      <c r="B5" s="251" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="253" t="s">
+      <c r="C5" s="251" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="253" t="s">
+      <c r="D5" s="251" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="254" t="s">
+      <c r="E5" s="252" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="254" t="s">
+      <c r="F5" s="252" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="253"/>
-      <c r="C6" s="253"/>
-      <c r="D6" s="253"/>
-      <c r="E6" s="254"/>
-      <c r="F6" s="254"/>
+      <c r="B6" s="251"/>
+      <c r="C6" s="251"/>
+      <c r="D6" s="251"/>
+      <c r="E6" s="252"/>
+      <c r="F6" s="252"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="253"/>
-      <c r="C7" s="253"/>
-      <c r="D7" s="253"/>
-      <c r="E7" s="254"/>
-      <c r="F7" s="254"/>
+      <c r="B7" s="251"/>
+      <c r="C7" s="251"/>
+      <c r="D7" s="251"/>
+      <c r="E7" s="252"/>
+      <c r="F7" s="252"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -40988,45 +40988,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="150"/>
-      <c r="C1" s="151"/>
-      <c r="D1" s="151"/>
-      <c r="E1" s="151"/>
-      <c r="F1" s="151"/>
-      <c r="G1" s="151"/>
-      <c r="H1" s="151"/>
-      <c r="I1" s="151"/>
-      <c r="J1" s="151"/>
-      <c r="K1" s="151"/>
-      <c r="L1" s="152"/>
+      <c r="B1" s="148"/>
+      <c r="C1" s="149"/>
+      <c r="D1" s="149"/>
+      <c r="E1" s="149"/>
+      <c r="F1" s="149"/>
+      <c r="G1" s="149"/>
+      <c r="H1" s="149"/>
+      <c r="I1" s="149"/>
+      <c r="J1" s="149"/>
+      <c r="K1" s="149"/>
+      <c r="L1" s="150"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="153" t="s">
+      <c r="B2" s="151" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="154"/>
-      <c r="D2" s="154"/>
-      <c r="E2" s="154"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="154"/>
-      <c r="H2" s="154"/>
-      <c r="I2" s="155"/>
-      <c r="J2" s="159"/>
-      <c r="K2" s="160"/>
-      <c r="L2" s="161"/>
+      <c r="C2" s="152"/>
+      <c r="D2" s="152"/>
+      <c r="E2" s="152"/>
+      <c r="F2" s="152"/>
+      <c r="G2" s="152"/>
+      <c r="H2" s="152"/>
+      <c r="I2" s="153"/>
+      <c r="J2" s="157"/>
+      <c r="K2" s="158"/>
+      <c r="L2" s="159"/>
     </row>
     <row r="3" spans="1:13" ht="14.4" customHeight="1">
-      <c r="B3" s="156"/>
-      <c r="C3" s="157"/>
-      <c r="D3" s="157"/>
-      <c r="E3" s="157"/>
-      <c r="F3" s="157"/>
-      <c r="G3" s="157"/>
-      <c r="H3" s="157"/>
-      <c r="I3" s="158"/>
-      <c r="J3" s="162"/>
-      <c r="K3" s="163"/>
-      <c r="L3" s="164"/>
+      <c r="B3" s="154"/>
+      <c r="C3" s="155"/>
+      <c r="D3" s="155"/>
+      <c r="E3" s="155"/>
+      <c r="F3" s="155"/>
+      <c r="G3" s="155"/>
+      <c r="H3" s="155"/>
+      <c r="I3" s="156"/>
+      <c r="J3" s="160"/>
+      <c r="K3" s="161"/>
+      <c r="L3" s="162"/>
     </row>
     <row r="4" spans="1:13" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -41037,9 +41037,9 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="162"/>
-      <c r="K4" s="163"/>
-      <c r="L4" s="164"/>
+      <c r="J4" s="160"/>
+      <c r="K4" s="161"/>
+      <c r="L4" s="162"/>
     </row>
     <row r="5" spans="1:13" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -41054,9 +41054,9 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="162"/>
-      <c r="K5" s="163"/>
-      <c r="L5" s="164"/>
+      <c r="J5" s="160"/>
+      <c r="K5" s="161"/>
+      <c r="L5" s="162"/>
     </row>
     <row r="6" spans="1:13" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -41071,9 +41071,9 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="165"/>
-      <c r="K6" s="166"/>
-      <c r="L6" s="167"/>
+      <c r="J6" s="163"/>
+      <c r="K6" s="164"/>
+      <c r="L6" s="165"/>
     </row>
     <row r="7" spans="1:13" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -41125,45 +41125,45 @@
       <c r="J9" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="K9" s="125"/>
+      <c r="K9" s="124"/>
       <c r="L9" s="89"/>
     </row>
     <row r="10" spans="1:13" ht="15.6">
-      <c r="B10" s="168" t="s">
+      <c r="B10" s="166" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="169"/>
-      <c r="D10" s="169"/>
-      <c r="E10" s="169"/>
-      <c r="F10" s="170"/>
-      <c r="G10" s="169" t="s">
+      <c r="C10" s="167"/>
+      <c r="D10" s="167"/>
+      <c r="E10" s="167"/>
+      <c r="F10" s="168"/>
+      <c r="G10" s="167" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="169"/>
-      <c r="I10" s="169"/>
-      <c r="J10" s="170"/>
-      <c r="K10" s="169" t="s">
+      <c r="H10" s="167"/>
+      <c r="I10" s="167"/>
+      <c r="J10" s="168"/>
+      <c r="K10" s="167" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="171"/>
+      <c r="L10" s="169"/>
     </row>
     <row r="11" spans="1:13" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="187" t="s">
+      <c r="C11" s="185" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="188"/>
-      <c r="E11" s="188"/>
+      <c r="D11" s="186"/>
+      <c r="E11" s="186"/>
       <c r="F11" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="187" t="s">
+      <c r="G11" s="185" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="189"/>
+      <c r="H11" s="187"/>
       <c r="I11" s="92" t="s">
         <v>27</v>
       </c>
@@ -41182,14 +41182,14 @@
       <c r="B12" s="94" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="233" t="s">
+      <c r="C12" s="231" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="234"/>
-      <c r="E12" s="235"/>
+      <c r="D12" s="232"/>
+      <c r="E12" s="233"/>
       <c r="F12" s="95"/>
-      <c r="G12" s="196"/>
-      <c r="H12" s="197"/>
+      <c r="G12" s="194"/>
+      <c r="H12" s="195"/>
       <c r="I12" s="96"/>
       <c r="J12" s="96"/>
       <c r="K12" s="97"/>
@@ -41199,14 +41199,14 @@
       <c r="B13" s="99">
         <v>1</v>
       </c>
-      <c r="C13" s="236" t="s">
+      <c r="C13" s="234" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="237"/>
-      <c r="E13" s="238"/>
+      <c r="D13" s="235"/>
+      <c r="E13" s="236"/>
       <c r="F13" s="100"/>
-      <c r="G13" s="198"/>
-      <c r="H13" s="199"/>
+      <c r="G13" s="196"/>
+      <c r="H13" s="197"/>
       <c r="I13" s="101"/>
       <c r="J13" s="102"/>
       <c r="K13" s="103"/>
@@ -41216,14 +41216,14 @@
       <c r="B14" s="99">
         <v>2</v>
       </c>
-      <c r="C14" s="236" t="s">
+      <c r="C14" s="234" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="237"/>
-      <c r="E14" s="238"/>
+      <c r="D14" s="235"/>
+      <c r="E14" s="236"/>
       <c r="F14" s="100"/>
-      <c r="G14" s="198"/>
-      <c r="H14" s="199"/>
+      <c r="G14" s="196"/>
+      <c r="H14" s="197"/>
       <c r="I14" s="101"/>
       <c r="J14" s="102"/>
       <c r="K14" s="103"/>
@@ -41233,14 +41233,14 @@
       <c r="B15" s="99">
         <v>3</v>
       </c>
-      <c r="C15" s="236" t="s">
+      <c r="C15" s="234" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="237"/>
-      <c r="E15" s="238"/>
+      <c r="D15" s="235"/>
+      <c r="E15" s="236"/>
       <c r="F15" s="100"/>
-      <c r="G15" s="198"/>
-      <c r="H15" s="199"/>
+      <c r="G15" s="196"/>
+      <c r="H15" s="197"/>
       <c r="I15" s="101"/>
       <c r="J15" s="102"/>
       <c r="K15" s="103"/>
@@ -41250,14 +41250,14 @@
       <c r="B16" s="99">
         <v>4</v>
       </c>
-      <c r="C16" s="236" t="s">
+      <c r="C16" s="234" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="237"/>
-      <c r="E16" s="238"/>
+      <c r="D16" s="235"/>
+      <c r="E16" s="236"/>
       <c r="F16" s="100"/>
-      <c r="G16" s="198"/>
-      <c r="H16" s="199"/>
+      <c r="G16" s="196"/>
+      <c r="H16" s="197"/>
       <c r="I16" s="101"/>
       <c r="J16" s="102"/>
       <c r="K16" s="103"/>
@@ -41267,14 +41267,14 @@
       <c r="B17" s="99">
         <v>5</v>
       </c>
-      <c r="C17" s="236" t="s">
+      <c r="C17" s="234" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="237"/>
-      <c r="E17" s="238"/>
+      <c r="D17" s="235"/>
+      <c r="E17" s="236"/>
       <c r="F17" s="100"/>
-      <c r="G17" s="198"/>
-      <c r="H17" s="199"/>
+      <c r="G17" s="196"/>
+      <c r="H17" s="197"/>
       <c r="I17" s="101"/>
       <c r="J17" s="102"/>
       <c r="K17" s="103"/>
@@ -41284,14 +41284,14 @@
       <c r="B18" s="99">
         <v>6</v>
       </c>
-      <c r="C18" s="236" t="s">
+      <c r="C18" s="234" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="237"/>
-      <c r="E18" s="238"/>
+      <c r="D18" s="235"/>
+      <c r="E18" s="236"/>
       <c r="F18" s="100"/>
-      <c r="G18" s="198"/>
-      <c r="H18" s="199"/>
+      <c r="G18" s="196"/>
+      <c r="H18" s="197"/>
       <c r="I18" s="101"/>
       <c r="J18" s="102"/>
       <c r="K18" s="103"/>
@@ -41301,14 +41301,14 @@
       <c r="B19" s="105" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="239" t="s">
+      <c r="C19" s="237" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="240"/>
-      <c r="E19" s="241"/>
+      <c r="D19" s="238"/>
+      <c r="E19" s="239"/>
       <c r="F19" s="100"/>
-      <c r="G19" s="198"/>
-      <c r="H19" s="199"/>
+      <c r="G19" s="196"/>
+      <c r="H19" s="197"/>
       <c r="I19" s="101"/>
       <c r="J19" s="102"/>
       <c r="K19" s="103"/>
@@ -41318,14 +41318,14 @@
       <c r="B20" s="99">
         <v>1</v>
       </c>
-      <c r="C20" s="236" t="s">
+      <c r="C20" s="234" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="237"/>
-      <c r="E20" s="238"/>
+      <c r="D20" s="235"/>
+      <c r="E20" s="236"/>
       <c r="F20" s="100"/>
-      <c r="G20" s="198"/>
-      <c r="H20" s="199"/>
+      <c r="G20" s="196"/>
+      <c r="H20" s="197"/>
       <c r="I20" s="101"/>
       <c r="J20" s="102"/>
       <c r="K20" s="103"/>
@@ -41335,14 +41335,14 @@
       <c r="B21" s="99">
         <v>2</v>
       </c>
-      <c r="C21" s="236" t="s">
+      <c r="C21" s="234" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="237"/>
-      <c r="E21" s="238"/>
+      <c r="D21" s="235"/>
+      <c r="E21" s="236"/>
       <c r="F21" s="100"/>
-      <c r="G21" s="198"/>
-      <c r="H21" s="199"/>
+      <c r="G21" s="196"/>
+      <c r="H21" s="197"/>
       <c r="I21" s="101"/>
       <c r="J21" s="102"/>
       <c r="K21" s="103"/>
@@ -41352,143 +41352,143 @@
       <c r="B22" s="99">
         <v>3</v>
       </c>
-      <c r="C22" s="242" t="s">
+      <c r="C22" s="240" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="243"/>
-      <c r="E22" s="244"/>
+      <c r="D22" s="241"/>
+      <c r="E22" s="242"/>
       <c r="F22" s="100"/>
-      <c r="G22" s="200"/>
-      <c r="H22" s="201"/>
+      <c r="G22" s="198"/>
+      <c r="H22" s="199"/>
       <c r="I22" s="101"/>
       <c r="J22" s="102"/>
       <c r="K22" s="106"/>
       <c r="L22" s="107"/>
     </row>
     <row r="23" spans="1:12" ht="16.2" thickBot="1">
-      <c r="B23" s="190"/>
-      <c r="C23" s="191"/>
-      <c r="D23" s="191"/>
-      <c r="E23" s="191"/>
+      <c r="B23" s="188"/>
+      <c r="C23" s="189"/>
+      <c r="D23" s="189"/>
+      <c r="E23" s="189"/>
       <c r="F23" s="108"/>
       <c r="G23" s="108"/>
       <c r="H23" s="109"/>
       <c r="I23" s="109"/>
-      <c r="J23" s="192"/>
-      <c r="K23" s="192"/>
-      <c r="L23" s="193"/>
+      <c r="J23" s="190"/>
+      <c r="K23" s="190"/>
+      <c r="L23" s="191"/>
     </row>
     <row r="24" spans="1:12" ht="16.2" customHeight="1" thickTop="1">
-      <c r="A24" s="124" t="s">
+      <c r="A24" s="123" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="194" t="s">
+      <c r="B24" s="192" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="172" t="s">
+      <c r="C24" s="170" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="172"/>
-      <c r="E24" s="172"/>
-      <c r="F24" s="172"/>
-      <c r="G24" s="172"/>
-      <c r="H24" s="172"/>
-      <c r="I24" s="172"/>
-      <c r="J24" s="174" t="s">
+      <c r="D24" s="170"/>
+      <c r="E24" s="170"/>
+      <c r="F24" s="170"/>
+      <c r="G24" s="170"/>
+      <c r="H24" s="170"/>
+      <c r="I24" s="170"/>
+      <c r="J24" s="172" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="175"/>
-      <c r="L24" s="176"/>
+      <c r="K24" s="173"/>
+      <c r="L24" s="174"/>
     </row>
     <row r="25" spans="1:12" ht="31.2">
-      <c r="B25" s="195"/>
-      <c r="C25" s="173"/>
-      <c r="D25" s="173"/>
-      <c r="E25" s="173"/>
-      <c r="F25" s="173"/>
-      <c r="G25" s="173"/>
-      <c r="H25" s="173"/>
-      <c r="I25" s="173"/>
-      <c r="J25" s="149" t="s">
+      <c r="B25" s="193"/>
+      <c r="C25" s="171"/>
+      <c r="D25" s="171"/>
+      <c r="E25" s="171"/>
+      <c r="F25" s="171"/>
+      <c r="G25" s="171"/>
+      <c r="H25" s="171"/>
+      <c r="I25" s="171"/>
+      <c r="J25" s="147" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="146" t="s">
+      <c r="K25" s="145" t="s">
         <v>76</v>
       </c>
-      <c r="L25" s="147" t="s">
+      <c r="L25" s="146" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.6">
       <c r="B26" s="110"/>
-      <c r="C26" s="288"/>
-      <c r="D26" s="289"/>
-      <c r="E26" s="289"/>
-      <c r="F26" s="289"/>
-      <c r="G26" s="289"/>
-      <c r="H26" s="289"/>
-      <c r="I26" s="290"/>
-      <c r="J26" s="297"/>
-      <c r="K26" s="148"/>
-      <c r="L26" s="301"/>
+      <c r="C26" s="286"/>
+      <c r="D26" s="287"/>
+      <c r="E26" s="287"/>
+      <c r="F26" s="287"/>
+      <c r="G26" s="287"/>
+      <c r="H26" s="287"/>
+      <c r="I26" s="288"/>
+      <c r="J26" s="295"/>
+      <c r="K26" s="306"/>
+      <c r="L26" s="304"/>
     </row>
     <row r="27" spans="1:12" ht="15.6">
       <c r="B27" s="110"/>
-      <c r="C27" s="291"/>
-      <c r="D27" s="292"/>
-      <c r="E27" s="292"/>
-      <c r="F27" s="292"/>
-      <c r="G27" s="292"/>
-      <c r="H27" s="292"/>
-      <c r="I27" s="293"/>
+      <c r="C27" s="289"/>
+      <c r="D27" s="290"/>
+      <c r="E27" s="290"/>
+      <c r="F27" s="290"/>
+      <c r="G27" s="290"/>
+      <c r="H27" s="290"/>
+      <c r="I27" s="291"/>
       <c r="J27" s="102"/>
-      <c r="K27" s="299"/>
-      <c r="L27" s="301"/>
+      <c r="K27" s="307"/>
+      <c r="L27" s="304"/>
     </row>
     <row r="28" spans="1:12" ht="15.6">
       <c r="B28" s="110"/>
-      <c r="C28" s="291"/>
-      <c r="D28" s="292"/>
-      <c r="E28" s="292"/>
-      <c r="F28" s="292"/>
-      <c r="G28" s="292"/>
-      <c r="H28" s="292"/>
-      <c r="I28" s="293"/>
+      <c r="C28" s="289"/>
+      <c r="D28" s="290"/>
+      <c r="E28" s="290"/>
+      <c r="F28" s="290"/>
+      <c r="G28" s="290"/>
+      <c r="H28" s="290"/>
+      <c r="I28" s="291"/>
       <c r="J28" s="102"/>
-      <c r="K28" s="299"/>
-      <c r="L28" s="111"/>
+      <c r="K28" s="307"/>
+      <c r="L28" s="305"/>
     </row>
     <row r="29" spans="1:12" ht="15.6">
       <c r="B29" s="110"/>
-      <c r="C29" s="291"/>
-      <c r="D29" s="292"/>
-      <c r="E29" s="292"/>
-      <c r="F29" s="292"/>
-      <c r="G29" s="292"/>
-      <c r="H29" s="292"/>
-      <c r="I29" s="293"/>
+      <c r="C29" s="289"/>
+      <c r="D29" s="290"/>
+      <c r="E29" s="290"/>
+      <c r="F29" s="290"/>
+      <c r="G29" s="290"/>
+      <c r="H29" s="290"/>
+      <c r="I29" s="291"/>
       <c r="J29" s="102"/>
-      <c r="K29" s="299"/>
-      <c r="L29" s="111"/>
+      <c r="K29" s="307"/>
+      <c r="L29" s="305"/>
     </row>
     <row r="30" spans="1:12" ht="15.6">
       <c r="B30" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="291" t="s">
+      <c r="C30" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="292"/>
-      <c r="E30" s="292"/>
-      <c r="F30" s="292"/>
-      <c r="G30" s="292"/>
-      <c r="H30" s="292"/>
-      <c r="I30" s="293"/>
+      <c r="D30" s="290"/>
+      <c r="E30" s="290"/>
+      <c r="F30" s="290"/>
+      <c r="G30" s="290"/>
+      <c r="H30" s="290"/>
+      <c r="I30" s="291"/>
       <c r="J30" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K30" s="299"/>
-      <c r="L30" s="111" t="s">
+      <c r="K30" s="307"/>
+      <c r="L30" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41496,20 +41496,20 @@
       <c r="B31" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="291" t="s">
+      <c r="C31" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="292"/>
-      <c r="E31" s="292"/>
-      <c r="F31" s="292"/>
-      <c r="G31" s="292"/>
-      <c r="H31" s="292"/>
-      <c r="I31" s="293"/>
+      <c r="D31" s="290"/>
+      <c r="E31" s="290"/>
+      <c r="F31" s="290"/>
+      <c r="G31" s="290"/>
+      <c r="H31" s="290"/>
+      <c r="I31" s="291"/>
       <c r="J31" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K31" s="299"/>
-      <c r="L31" s="111" t="s">
+      <c r="K31" s="307"/>
+      <c r="L31" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41517,20 +41517,20 @@
       <c r="B32" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="291" t="s">
+      <c r="C32" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="292"/>
-      <c r="E32" s="292"/>
-      <c r="F32" s="292"/>
-      <c r="G32" s="292"/>
-      <c r="H32" s="292"/>
-      <c r="I32" s="293"/>
+      <c r="D32" s="290"/>
+      <c r="E32" s="290"/>
+      <c r="F32" s="290"/>
+      <c r="G32" s="290"/>
+      <c r="H32" s="290"/>
+      <c r="I32" s="291"/>
       <c r="J32" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K32" s="299"/>
-      <c r="L32" s="111" t="s">
+      <c r="K32" s="307"/>
+      <c r="L32" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41538,20 +41538,20 @@
       <c r="B33" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="291" t="s">
+      <c r="C33" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="292"/>
-      <c r="E33" s="292"/>
-      <c r="F33" s="292"/>
-      <c r="G33" s="292"/>
-      <c r="H33" s="292"/>
-      <c r="I33" s="293"/>
+      <c r="D33" s="290"/>
+      <c r="E33" s="290"/>
+      <c r="F33" s="290"/>
+      <c r="G33" s="290"/>
+      <c r="H33" s="290"/>
+      <c r="I33" s="291"/>
       <c r="J33" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K33" s="299"/>
-      <c r="L33" s="111" t="s">
+      <c r="K33" s="307"/>
+      <c r="L33" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41559,20 +41559,20 @@
       <c r="B34" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="291" t="s">
+      <c r="C34" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="292"/>
-      <c r="E34" s="292"/>
-      <c r="F34" s="292"/>
-      <c r="G34" s="292"/>
-      <c r="H34" s="292"/>
-      <c r="I34" s="293"/>
+      <c r="D34" s="290"/>
+      <c r="E34" s="290"/>
+      <c r="F34" s="290"/>
+      <c r="G34" s="290"/>
+      <c r="H34" s="290"/>
+      <c r="I34" s="291"/>
       <c r="J34" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K34" s="299"/>
-      <c r="L34" s="111" t="s">
+      <c r="K34" s="307"/>
+      <c r="L34" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41580,20 +41580,20 @@
       <c r="B35" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="291" t="s">
+      <c r="C35" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="292"/>
-      <c r="E35" s="292"/>
-      <c r="F35" s="292"/>
-      <c r="G35" s="292"/>
-      <c r="H35" s="292"/>
-      <c r="I35" s="293"/>
+      <c r="D35" s="290"/>
+      <c r="E35" s="290"/>
+      <c r="F35" s="290"/>
+      <c r="G35" s="290"/>
+      <c r="H35" s="290"/>
+      <c r="I35" s="291"/>
       <c r="J35" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K35" s="299"/>
-      <c r="L35" s="111" t="s">
+      <c r="K35" s="307"/>
+      <c r="L35" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41601,20 +41601,20 @@
       <c r="B36" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C36" s="291" t="s">
+      <c r="C36" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="292"/>
-      <c r="E36" s="292"/>
-      <c r="F36" s="292"/>
-      <c r="G36" s="292"/>
-      <c r="H36" s="292"/>
-      <c r="I36" s="293"/>
+      <c r="D36" s="290"/>
+      <c r="E36" s="290"/>
+      <c r="F36" s="290"/>
+      <c r="G36" s="290"/>
+      <c r="H36" s="290"/>
+      <c r="I36" s="291"/>
       <c r="J36" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K36" s="299"/>
-      <c r="L36" s="111" t="s">
+      <c r="K36" s="307"/>
+      <c r="L36" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41622,20 +41622,20 @@
       <c r="B37" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="291" t="s">
+      <c r="C37" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="292"/>
-      <c r="E37" s="292"/>
-      <c r="F37" s="292"/>
-      <c r="G37" s="292"/>
-      <c r="H37" s="292"/>
-      <c r="I37" s="293"/>
+      <c r="D37" s="290"/>
+      <c r="E37" s="290"/>
+      <c r="F37" s="290"/>
+      <c r="G37" s="290"/>
+      <c r="H37" s="290"/>
+      <c r="I37" s="291"/>
       <c r="J37" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K37" s="299"/>
-      <c r="L37" s="111" t="s">
+      <c r="K37" s="307"/>
+      <c r="L37" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41643,20 +41643,20 @@
       <c r="B38" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="291" t="s">
+      <c r="C38" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="292"/>
-      <c r="E38" s="292"/>
-      <c r="F38" s="292"/>
-      <c r="G38" s="292"/>
-      <c r="H38" s="292"/>
-      <c r="I38" s="293"/>
+      <c r="D38" s="290"/>
+      <c r="E38" s="290"/>
+      <c r="F38" s="290"/>
+      <c r="G38" s="290"/>
+      <c r="H38" s="290"/>
+      <c r="I38" s="291"/>
       <c r="J38" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K38" s="299"/>
-      <c r="L38" s="111" t="s">
+      <c r="K38" s="307"/>
+      <c r="L38" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41664,20 +41664,20 @@
       <c r="B39" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="291" t="s">
+      <c r="C39" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D39" s="292"/>
-      <c r="E39" s="292"/>
-      <c r="F39" s="292"/>
-      <c r="G39" s="292"/>
-      <c r="H39" s="292"/>
-      <c r="I39" s="293"/>
+      <c r="D39" s="290"/>
+      <c r="E39" s="290"/>
+      <c r="F39" s="290"/>
+      <c r="G39" s="290"/>
+      <c r="H39" s="290"/>
+      <c r="I39" s="291"/>
       <c r="J39" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K39" s="299"/>
-      <c r="L39" s="111" t="s">
+      <c r="K39" s="307"/>
+      <c r="L39" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41685,20 +41685,20 @@
       <c r="B40" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="291" t="s">
+      <c r="C40" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D40" s="292"/>
-      <c r="E40" s="292"/>
-      <c r="F40" s="292"/>
-      <c r="G40" s="292"/>
-      <c r="H40" s="292"/>
-      <c r="I40" s="293"/>
+      <c r="D40" s="290"/>
+      <c r="E40" s="290"/>
+      <c r="F40" s="290"/>
+      <c r="G40" s="290"/>
+      <c r="H40" s="290"/>
+      <c r="I40" s="291"/>
       <c r="J40" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K40" s="299"/>
-      <c r="L40" s="111" t="s">
+      <c r="K40" s="307"/>
+      <c r="L40" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41706,20 +41706,20 @@
       <c r="B41" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="291" t="s">
+      <c r="C41" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D41" s="292"/>
-      <c r="E41" s="292"/>
-      <c r="F41" s="292"/>
-      <c r="G41" s="292"/>
-      <c r="H41" s="292"/>
-      <c r="I41" s="293"/>
+      <c r="D41" s="290"/>
+      <c r="E41" s="290"/>
+      <c r="F41" s="290"/>
+      <c r="G41" s="290"/>
+      <c r="H41" s="290"/>
+      <c r="I41" s="291"/>
       <c r="J41" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K41" s="299"/>
-      <c r="L41" s="111" t="s">
+      <c r="K41" s="307"/>
+      <c r="L41" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41727,20 +41727,20 @@
       <c r="B42" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="291" t="s">
+      <c r="C42" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="292"/>
-      <c r="E42" s="292"/>
-      <c r="F42" s="292"/>
-      <c r="G42" s="292"/>
-      <c r="H42" s="292"/>
-      <c r="I42" s="293"/>
+      <c r="D42" s="290"/>
+      <c r="E42" s="290"/>
+      <c r="F42" s="290"/>
+      <c r="G42" s="290"/>
+      <c r="H42" s="290"/>
+      <c r="I42" s="291"/>
       <c r="J42" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K42" s="299"/>
-      <c r="L42" s="111" t="s">
+      <c r="K42" s="307"/>
+      <c r="L42" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41748,20 +41748,20 @@
       <c r="B43" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="291" t="s">
+      <c r="C43" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="292"/>
-      <c r="E43" s="292"/>
-      <c r="F43" s="292"/>
-      <c r="G43" s="292"/>
-      <c r="H43" s="292"/>
-      <c r="I43" s="293"/>
+      <c r="D43" s="290"/>
+      <c r="E43" s="290"/>
+      <c r="F43" s="290"/>
+      <c r="G43" s="290"/>
+      <c r="H43" s="290"/>
+      <c r="I43" s="291"/>
       <c r="J43" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K43" s="299"/>
-      <c r="L43" s="111" t="s">
+      <c r="K43" s="307"/>
+      <c r="L43" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41769,20 +41769,20 @@
       <c r="B44" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="291" t="s">
+      <c r="C44" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D44" s="292"/>
-      <c r="E44" s="292"/>
-      <c r="F44" s="292"/>
-      <c r="G44" s="292"/>
-      <c r="H44" s="292"/>
-      <c r="I44" s="293"/>
+      <c r="D44" s="290"/>
+      <c r="E44" s="290"/>
+      <c r="F44" s="290"/>
+      <c r="G44" s="290"/>
+      <c r="H44" s="290"/>
+      <c r="I44" s="291"/>
       <c r="J44" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K44" s="299"/>
-      <c r="L44" s="111" t="s">
+      <c r="K44" s="307"/>
+      <c r="L44" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41790,20 +41790,20 @@
       <c r="B45" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C45" s="291" t="s">
+      <c r="C45" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D45" s="292"/>
-      <c r="E45" s="292"/>
-      <c r="F45" s="292"/>
-      <c r="G45" s="292"/>
-      <c r="H45" s="292"/>
-      <c r="I45" s="293"/>
+      <c r="D45" s="290"/>
+      <c r="E45" s="290"/>
+      <c r="F45" s="290"/>
+      <c r="G45" s="290"/>
+      <c r="H45" s="290"/>
+      <c r="I45" s="291"/>
       <c r="J45" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K45" s="299"/>
-      <c r="L45" s="111" t="s">
+      <c r="K45" s="307"/>
+      <c r="L45" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41811,20 +41811,20 @@
       <c r="B46" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C46" s="291" t="s">
+      <c r="C46" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="292"/>
-      <c r="E46" s="292"/>
-      <c r="F46" s="292"/>
-      <c r="G46" s="292"/>
-      <c r="H46" s="292"/>
-      <c r="I46" s="293"/>
+      <c r="D46" s="290"/>
+      <c r="E46" s="290"/>
+      <c r="F46" s="290"/>
+      <c r="G46" s="290"/>
+      <c r="H46" s="290"/>
+      <c r="I46" s="291"/>
       <c r="J46" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K46" s="299"/>
-      <c r="L46" s="111" t="s">
+      <c r="K46" s="307"/>
+      <c r="L46" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41832,20 +41832,20 @@
       <c r="B47" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="291" t="s">
+      <c r="C47" s="289" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="292"/>
-      <c r="E47" s="292"/>
-      <c r="F47" s="292"/>
-      <c r="G47" s="292"/>
-      <c r="H47" s="292"/>
-      <c r="I47" s="293"/>
+      <c r="D47" s="290"/>
+      <c r="E47" s="290"/>
+      <c r="F47" s="290"/>
+      <c r="G47" s="290"/>
+      <c r="H47" s="290"/>
+      <c r="I47" s="291"/>
       <c r="J47" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="K47" s="299"/>
-      <c r="L47" s="111" t="s">
+      <c r="K47" s="307"/>
+      <c r="L47" s="305" t="s">
         <v>64</v>
       </c>
     </row>
@@ -41853,268 +41853,268 @@
       <c r="B48" s="110" t="s">
         <v>64</v>
       </c>
-      <c r="C48" s="294" t="s">
+      <c r="C48" s="292" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="295"/>
-      <c r="E48" s="295"/>
-      <c r="F48" s="295"/>
-      <c r="G48" s="295"/>
-      <c r="H48" s="295"/>
-      <c r="I48" s="296"/>
-      <c r="J48" s="298" t="s">
+      <c r="D48" s="293"/>
+      <c r="E48" s="293"/>
+      <c r="F48" s="293"/>
+      <c r="G48" s="293"/>
+      <c r="H48" s="293"/>
+      <c r="I48" s="294"/>
+      <c r="J48" s="296" t="s">
         <v>64</v>
       </c>
-      <c r="K48" s="300"/>
-      <c r="L48" s="111" t="s">
+      <c r="K48" s="308"/>
+      <c r="L48" s="305" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="49" spans="2:12" ht="16.2" thickTop="1">
-      <c r="B49" s="215" t="s">
+      <c r="B49" s="213" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="216"/>
-      <c r="D49" s="216"/>
-      <c r="E49" s="216"/>
-      <c r="F49" s="216"/>
-      <c r="G49" s="216"/>
-      <c r="H49" s="216"/>
-      <c r="I49" s="216"/>
-      <c r="J49" s="217"/>
-      <c r="K49" s="185" t="s">
+      <c r="C49" s="214"/>
+      <c r="D49" s="214"/>
+      <c r="E49" s="214"/>
+      <c r="F49" s="214"/>
+      <c r="G49" s="214"/>
+      <c r="H49" s="214"/>
+      <c r="I49" s="214"/>
+      <c r="J49" s="215"/>
+      <c r="K49" s="183" t="s">
         <v>79</v>
       </c>
-      <c r="L49" s="186"/>
+      <c r="L49" s="184"/>
     </row>
     <row r="50" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B50" s="218"/>
-      <c r="C50" s="219"/>
-      <c r="D50" s="219"/>
-      <c r="E50" s="219"/>
-      <c r="F50" s="219"/>
-      <c r="G50" s="219"/>
-      <c r="H50" s="219"/>
-      <c r="I50" s="219"/>
-      <c r="J50" s="220"/>
-      <c r="K50" s="183" t="s">
+      <c r="B50" s="216"/>
+      <c r="C50" s="217"/>
+      <c r="D50" s="217"/>
+      <c r="E50" s="217"/>
+      <c r="F50" s="217"/>
+      <c r="G50" s="217"/>
+      <c r="H50" s="217"/>
+      <c r="I50" s="217"/>
+      <c r="J50" s="218"/>
+      <c r="K50" s="181" t="s">
         <v>103</v>
       </c>
-      <c r="L50" s="184"/>
+      <c r="L50" s="182"/>
     </row>
     <row r="51" spans="2:12" ht="15.6">
-      <c r="B51" s="112"/>
-      <c r="C51" s="180"/>
-      <c r="D51" s="180"/>
-      <c r="E51" s="180"/>
-      <c r="F51" s="180"/>
-      <c r="G51" s="180"/>
-      <c r="H51" s="180"/>
-      <c r="I51" s="180"/>
-      <c r="J51" s="113"/>
-      <c r="K51" s="178"/>
-      <c r="L51" s="179"/>
+      <c r="B51" s="111"/>
+      <c r="C51" s="178"/>
+      <c r="D51" s="178"/>
+      <c r="E51" s="178"/>
+      <c r="F51" s="178"/>
+      <c r="G51" s="178"/>
+      <c r="H51" s="178"/>
+      <c r="I51" s="178"/>
+      <c r="J51" s="112"/>
+      <c r="K51" s="176"/>
+      <c r="L51" s="177"/>
     </row>
     <row r="52" spans="2:12" ht="15.6">
-      <c r="B52" s="114"/>
-      <c r="C52" s="181"/>
-      <c r="D52" s="181"/>
-      <c r="E52" s="181"/>
-      <c r="F52" s="181"/>
-      <c r="G52" s="181"/>
-      <c r="H52" s="181"/>
-      <c r="I52" s="181"/>
-      <c r="J52" s="115"/>
-      <c r="K52" s="126"/>
-      <c r="L52" s="116"/>
+      <c r="B52" s="113"/>
+      <c r="C52" s="179"/>
+      <c r="D52" s="179"/>
+      <c r="E52" s="179"/>
+      <c r="F52" s="179"/>
+      <c r="G52" s="179"/>
+      <c r="H52" s="179"/>
+      <c r="I52" s="179"/>
+      <c r="J52" s="114"/>
+      <c r="K52" s="125"/>
+      <c r="L52" s="115"/>
     </row>
     <row r="53" spans="2:12" ht="15.6">
-      <c r="B53" s="117"/>
-      <c r="C53" s="181"/>
-      <c r="D53" s="181"/>
-      <c r="E53" s="181"/>
-      <c r="F53" s="181"/>
-      <c r="G53" s="181"/>
-      <c r="H53" s="181"/>
-      <c r="I53" s="181"/>
-      <c r="J53" s="118"/>
-      <c r="K53" s="119"/>
-      <c r="L53" s="120"/>
+      <c r="B53" s="116"/>
+      <c r="C53" s="179"/>
+      <c r="D53" s="179"/>
+      <c r="E53" s="179"/>
+      <c r="F53" s="179"/>
+      <c r="G53" s="179"/>
+      <c r="H53" s="179"/>
+      <c r="I53" s="179"/>
+      <c r="J53" s="117"/>
+      <c r="K53" s="118"/>
+      <c r="L53" s="119"/>
     </row>
     <row r="54" spans="2:12" ht="15.6">
-      <c r="B54" s="117"/>
-      <c r="C54" s="181"/>
-      <c r="D54" s="181"/>
-      <c r="E54" s="181"/>
-      <c r="F54" s="181"/>
-      <c r="G54" s="181"/>
-      <c r="H54" s="181"/>
-      <c r="I54" s="181"/>
-      <c r="J54" s="118"/>
-      <c r="K54" s="302"/>
-      <c r="L54" s="303"/>
+      <c r="B54" s="116"/>
+      <c r="C54" s="179"/>
+      <c r="D54" s="179"/>
+      <c r="E54" s="179"/>
+      <c r="F54" s="179"/>
+      <c r="G54" s="179"/>
+      <c r="H54" s="179"/>
+      <c r="I54" s="179"/>
+      <c r="J54" s="117"/>
+      <c r="K54" s="297"/>
+      <c r="L54" s="298"/>
     </row>
     <row r="55" spans="2:12" ht="15.6">
-      <c r="B55" s="117"/>
-      <c r="C55" s="181"/>
-      <c r="D55" s="181"/>
-      <c r="E55" s="181"/>
-      <c r="F55" s="181"/>
-      <c r="G55" s="181"/>
-      <c r="H55" s="181"/>
-      <c r="I55" s="181"/>
-      <c r="J55" s="118"/>
-      <c r="K55" s="305"/>
-      <c r="L55" s="306"/>
+      <c r="B55" s="116"/>
+      <c r="C55" s="179"/>
+      <c r="D55" s="179"/>
+      <c r="E55" s="179"/>
+      <c r="F55" s="179"/>
+      <c r="G55" s="179"/>
+      <c r="H55" s="179"/>
+      <c r="I55" s="179"/>
+      <c r="J55" s="117"/>
+      <c r="K55" s="300"/>
+      <c r="L55" s="301"/>
     </row>
     <row r="56" spans="2:12" ht="15.6">
-      <c r="B56" s="117"/>
-      <c r="C56" s="181"/>
-      <c r="D56" s="181"/>
-      <c r="E56" s="181"/>
-      <c r="F56" s="181"/>
-      <c r="G56" s="181"/>
-      <c r="H56" s="181"/>
-      <c r="I56" s="181"/>
-      <c r="J56" s="118"/>
-      <c r="K56" s="307"/>
-      <c r="L56" s="308"/>
+      <c r="B56" s="116"/>
+      <c r="C56" s="179"/>
+      <c r="D56" s="179"/>
+      <c r="E56" s="179"/>
+      <c r="F56" s="179"/>
+      <c r="G56" s="179"/>
+      <c r="H56" s="179"/>
+      <c r="I56" s="179"/>
+      <c r="J56" s="117"/>
+      <c r="K56" s="302"/>
+      <c r="L56" s="303"/>
     </row>
     <row r="57" spans="2:12" ht="15.6">
-      <c r="B57" s="117"/>
-      <c r="C57" s="181"/>
-      <c r="D57" s="181"/>
-      <c r="E57" s="181"/>
-      <c r="F57" s="181"/>
-      <c r="G57" s="181"/>
-      <c r="H57" s="181"/>
-      <c r="I57" s="181"/>
-      <c r="J57" s="118"/>
-      <c r="K57" s="305"/>
-      <c r="L57" s="306"/>
+      <c r="B57" s="116"/>
+      <c r="C57" s="179"/>
+      <c r="D57" s="179"/>
+      <c r="E57" s="179"/>
+      <c r="F57" s="179"/>
+      <c r="G57" s="179"/>
+      <c r="H57" s="179"/>
+      <c r="I57" s="179"/>
+      <c r="J57" s="117"/>
+      <c r="K57" s="300"/>
+      <c r="L57" s="301"/>
     </row>
     <row r="58" spans="2:12" ht="15.6">
-      <c r="B58" s="117"/>
-      <c r="C58" s="182"/>
-      <c r="D58" s="182"/>
-      <c r="E58" s="182"/>
-      <c r="F58" s="182"/>
-      <c r="G58" s="182"/>
-      <c r="H58" s="182"/>
-      <c r="I58" s="182"/>
-      <c r="J58" s="118"/>
-      <c r="K58" s="304"/>
-      <c r="L58" s="177"/>
+      <c r="B58" s="116"/>
+      <c r="C58" s="180"/>
+      <c r="D58" s="180"/>
+      <c r="E58" s="180"/>
+      <c r="F58" s="180"/>
+      <c r="G58" s="180"/>
+      <c r="H58" s="180"/>
+      <c r="I58" s="180"/>
+      <c r="J58" s="117"/>
+      <c r="K58" s="299"/>
+      <c r="L58" s="175"/>
     </row>
     <row r="59" spans="2:12" ht="15.6">
-      <c r="B59" s="117"/>
-      <c r="C59" s="121"/>
-      <c r="D59" s="121"/>
-      <c r="E59" s="121"/>
-      <c r="F59" s="121"/>
-      <c r="G59" s="121"/>
-      <c r="H59" s="121"/>
-      <c r="I59" s="121"/>
-      <c r="J59" s="118"/>
-      <c r="K59" s="304"/>
-      <c r="L59" s="177"/>
+      <c r="B59" s="116"/>
+      <c r="C59" s="120"/>
+      <c r="D59" s="120"/>
+      <c r="E59" s="120"/>
+      <c r="F59" s="120"/>
+      <c r="G59" s="120"/>
+      <c r="H59" s="120"/>
+      <c r="I59" s="120"/>
+      <c r="J59" s="117"/>
+      <c r="K59" s="299"/>
+      <c r="L59" s="175"/>
     </row>
     <row r="60" spans="2:12" ht="15.6">
-      <c r="B60" s="202" t="s">
+      <c r="B60" s="200" t="s">
         <v>80</v>
       </c>
-      <c r="C60" s="203"/>
-      <c r="D60" s="203"/>
-      <c r="E60" s="204"/>
-      <c r="F60" s="205" t="s">
+      <c r="C60" s="201"/>
+      <c r="D60" s="201"/>
+      <c r="E60" s="202"/>
+      <c r="F60" s="203" t="s">
         <v>81</v>
       </c>
-      <c r="G60" s="204"/>
-      <c r="H60" s="205" t="s">
+      <c r="G60" s="202"/>
+      <c r="H60" s="203" t="s">
         <v>82</v>
       </c>
-      <c r="I60" s="203"/>
-      <c r="J60" s="204"/>
-      <c r="K60" s="119"/>
-      <c r="L60" s="120"/>
+      <c r="I60" s="201"/>
+      <c r="J60" s="202"/>
+      <c r="K60" s="118"/>
+      <c r="L60" s="119"/>
     </row>
     <row r="61" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B61" s="227"/>
-      <c r="C61" s="228"/>
-      <c r="D61" s="228"/>
-      <c r="E61" s="222"/>
-      <c r="F61" s="221"/>
-      <c r="G61" s="222"/>
-      <c r="H61" s="206"/>
-      <c r="I61" s="207"/>
-      <c r="J61" s="208"/>
-      <c r="K61" s="119"/>
-      <c r="L61" s="120"/>
+      <c r="B61" s="225"/>
+      <c r="C61" s="226"/>
+      <c r="D61" s="226"/>
+      <c r="E61" s="220"/>
+      <c r="F61" s="219"/>
+      <c r="G61" s="220"/>
+      <c r="H61" s="204"/>
+      <c r="I61" s="205"/>
+      <c r="J61" s="206"/>
+      <c r="K61" s="118"/>
+      <c r="L61" s="119"/>
     </row>
     <row r="62" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B62" s="229"/>
-      <c r="C62" s="230"/>
-      <c r="D62" s="230"/>
-      <c r="E62" s="224"/>
-      <c r="F62" s="223"/>
-      <c r="G62" s="224"/>
-      <c r="H62" s="209"/>
-      <c r="I62" s="210"/>
-      <c r="J62" s="211"/>
-      <c r="K62" s="128"/>
-      <c r="L62" s="120"/>
+      <c r="B62" s="227"/>
+      <c r="C62" s="228"/>
+      <c r="D62" s="228"/>
+      <c r="E62" s="222"/>
+      <c r="F62" s="221"/>
+      <c r="G62" s="222"/>
+      <c r="H62" s="207"/>
+      <c r="I62" s="208"/>
+      <c r="J62" s="209"/>
+      <c r="K62" s="127"/>
+      <c r="L62" s="119"/>
     </row>
     <row r="63" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B63" s="229"/>
-      <c r="C63" s="230"/>
-      <c r="D63" s="230"/>
-      <c r="E63" s="224"/>
-      <c r="F63" s="223"/>
-      <c r="G63" s="224"/>
-      <c r="H63" s="209"/>
-      <c r="I63" s="210"/>
-      <c r="J63" s="211"/>
-      <c r="K63" s="127"/>
+      <c r="B63" s="227"/>
+      <c r="C63" s="228"/>
+      <c r="D63" s="228"/>
+      <c r="E63" s="222"/>
+      <c r="F63" s="221"/>
+      <c r="G63" s="222"/>
+      <c r="H63" s="207"/>
+      <c r="I63" s="208"/>
+      <c r="J63" s="209"/>
+      <c r="K63" s="126"/>
       <c r="L63" s="76"/>
     </row>
     <row r="64" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B64" s="229"/>
-      <c r="C64" s="230"/>
-      <c r="D64" s="230"/>
-      <c r="E64" s="224"/>
-      <c r="F64" s="223"/>
-      <c r="G64" s="224"/>
-      <c r="H64" s="209"/>
-      <c r="I64" s="210"/>
-      <c r="J64" s="211"/>
-      <c r="K64" s="129"/>
-      <c r="L64" s="130"/>
+      <c r="B64" s="227"/>
+      <c r="C64" s="228"/>
+      <c r="D64" s="228"/>
+      <c r="E64" s="222"/>
+      <c r="F64" s="221"/>
+      <c r="G64" s="222"/>
+      <c r="H64" s="207"/>
+      <c r="I64" s="208"/>
+      <c r="J64" s="209"/>
+      <c r="K64" s="128"/>
+      <c r="L64" s="129"/>
     </row>
     <row r="65" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B65" s="229"/>
-      <c r="C65" s="230"/>
-      <c r="D65" s="230"/>
-      <c r="E65" s="224"/>
-      <c r="F65" s="223"/>
-      <c r="G65" s="224"/>
-      <c r="H65" s="209"/>
-      <c r="I65" s="210"/>
-      <c r="J65" s="211"/>
-      <c r="K65" s="129"/>
-      <c r="L65" s="130"/>
+      <c r="B65" s="227"/>
+      <c r="C65" s="228"/>
+      <c r="D65" s="228"/>
+      <c r="E65" s="222"/>
+      <c r="F65" s="221"/>
+      <c r="G65" s="222"/>
+      <c r="H65" s="207"/>
+      <c r="I65" s="208"/>
+      <c r="J65" s="209"/>
+      <c r="K65" s="128"/>
+      <c r="L65" s="129"/>
     </row>
     <row r="66" spans="2:12" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B66" s="231"/>
-      <c r="C66" s="232"/>
-      <c r="D66" s="232"/>
-      <c r="E66" s="226"/>
-      <c r="F66" s="225"/>
-      <c r="G66" s="226"/>
-      <c r="H66" s="212"/>
-      <c r="I66" s="213"/>
-      <c r="J66" s="214"/>
-      <c r="K66" s="122"/>
-      <c r="L66" s="123"/>
+      <c r="B66" s="229"/>
+      <c r="C66" s="230"/>
+      <c r="D66" s="230"/>
+      <c r="E66" s="224"/>
+      <c r="F66" s="223"/>
+      <c r="G66" s="224"/>
+      <c r="H66" s="210"/>
+      <c r="I66" s="211"/>
+      <c r="J66" s="212"/>
+      <c r="K66" s="121"/>
+      <c r="L66" s="122"/>
     </row>
     <row r="67" spans="2:12" ht="15" thickTop="1">
       <c r="J67" s="61"/>
@@ -42234,40 +42234,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="252"/>
-      <c r="C1" s="252"/>
-      <c r="D1" s="252"/>
-      <c r="E1" s="252"/>
-      <c r="F1" s="252"/>
-      <c r="G1" s="252"/>
-      <c r="H1" s="252"/>
-      <c r="I1" s="252"/>
-      <c r="J1" s="252"/>
-      <c r="K1" s="252"/>
-      <c r="L1" s="252"/>
-      <c r="M1" s="252"/>
-      <c r="N1" s="252"/>
-      <c r="O1" s="252"/>
-      <c r="P1" s="252"/>
+      <c r="B1" s="250"/>
+      <c r="C1" s="250"/>
+      <c r="D1" s="250"/>
+      <c r="E1" s="250"/>
+      <c r="F1" s="250"/>
+      <c r="G1" s="250"/>
+      <c r="H1" s="250"/>
+      <c r="I1" s="250"/>
+      <c r="J1" s="250"/>
+      <c r="K1" s="250"/>
+      <c r="L1" s="250"/>
+      <c r="M1" s="250"/>
+      <c r="N1" s="250"/>
+      <c r="O1" s="250"/>
+      <c r="P1" s="250"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="250" t="s">
+      <c r="B2" s="248" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="251"/>
-      <c r="D2" s="251"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="251"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="251"/>
-      <c r="I2" s="251"/>
-      <c r="J2" s="251"/>
-      <c r="K2" s="251"/>
-      <c r="L2" s="251"/>
-      <c r="M2" s="251"/>
-      <c r="N2" s="251"/>
-      <c r="O2" s="251"/>
-      <c r="P2" s="251"/>
+      <c r="C2" s="249"/>
+      <c r="D2" s="249"/>
+      <c r="E2" s="249"/>
+      <c r="F2" s="249"/>
+      <c r="G2" s="249"/>
+      <c r="H2" s="249"/>
+      <c r="I2" s="249"/>
+      <c r="J2" s="249"/>
+      <c r="K2" s="249"/>
+      <c r="L2" s="249"/>
+      <c r="M2" s="249"/>
+      <c r="N2" s="249"/>
+      <c r="O2" s="249"/>
+      <c r="P2" s="249"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -42294,16 +42294,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="258" t="s">
+      <c r="I4" s="256" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="258"/>
-      <c r="K4" s="258"/>
-      <c r="L4" s="258"/>
-      <c r="M4" s="258"/>
-      <c r="N4" s="258"/>
-      <c r="O4" s="258"/>
-      <c r="P4" s="258"/>
+      <c r="J4" s="256"/>
+      <c r="K4" s="256"/>
+      <c r="L4" s="256"/>
+      <c r="M4" s="256"/>
+      <c r="N4" s="256"/>
+      <c r="O4" s="256"/>
+      <c r="P4" s="256"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -42317,14 +42317,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="258"/>
-      <c r="J5" s="258"/>
-      <c r="K5" s="258"/>
-      <c r="L5" s="258"/>
-      <c r="M5" s="258"/>
-      <c r="N5" s="258"/>
-      <c r="O5" s="258"/>
-      <c r="P5" s="258"/>
+      <c r="I5" s="256"/>
+      <c r="J5" s="256"/>
+      <c r="K5" s="256"/>
+      <c r="L5" s="256"/>
+      <c r="M5" s="256"/>
+      <c r="N5" s="256"/>
+      <c r="O5" s="256"/>
+      <c r="P5" s="256"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -42459,70 +42459,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="249" t="s">
+      <c r="B12" s="247" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="249" t="s">
+      <c r="C12" s="247" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="249"/>
-      <c r="E12" s="249"/>
-      <c r="F12" s="249" t="s">
+      <c r="D12" s="247"/>
+      <c r="E12" s="247"/>
+      <c r="F12" s="247" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="249" t="s">
+      <c r="G12" s="247" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="249" t="s">
+      <c r="H12" s="247" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="249" t="s">
+      <c r="I12" s="247" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="249" t="s">
+      <c r="J12" s="247" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="249"/>
-      <c r="L12" s="249"/>
-      <c r="M12" s="249"/>
-      <c r="N12" s="249"/>
-      <c r="O12" s="249"/>
-      <c r="P12" s="257" t="s">
+      <c r="K12" s="247"/>
+      <c r="L12" s="247"/>
+      <c r="M12" s="247"/>
+      <c r="N12" s="247"/>
+      <c r="O12" s="247"/>
+      <c r="P12" s="255" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="249"/>
-      <c r="C13" s="249"/>
-      <c r="D13" s="249"/>
-      <c r="E13" s="249"/>
-      <c r="F13" s="249"/>
-      <c r="G13" s="249"/>
-      <c r="H13" s="249"/>
-      <c r="I13" s="249"/>
-      <c r="J13" s="256" t="s">
+      <c r="B13" s="247"/>
+      <c r="C13" s="247"/>
+      <c r="D13" s="247"/>
+      <c r="E13" s="247"/>
+      <c r="F13" s="247"/>
+      <c r="G13" s="247"/>
+      <c r="H13" s="247"/>
+      <c r="I13" s="247"/>
+      <c r="J13" s="254" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="256"/>
-      <c r="L13" s="256" t="s">
+      <c r="K13" s="254"/>
+      <c r="L13" s="254" t="s">
         <v>98</v>
       </c>
-      <c r="M13" s="256"/>
-      <c r="N13" s="256" t="s">
+      <c r="M13" s="254"/>
+      <c r="N13" s="254" t="s">
         <v>99</v>
       </c>
-      <c r="O13" s="256"/>
-      <c r="P13" s="257"/>
+      <c r="O13" s="254"/>
+      <c r="P13" s="255"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="249"/>
-      <c r="C14" s="249"/>
-      <c r="D14" s="249"/>
-      <c r="E14" s="249"/>
-      <c r="F14" s="249"/>
-      <c r="G14" s="249"/>
-      <c r="H14" s="249"/>
-      <c r="I14" s="249"/>
+      <c r="B14" s="247"/>
+      <c r="C14" s="247"/>
+      <c r="D14" s="247"/>
+      <c r="E14" s="247"/>
+      <c r="F14" s="247"/>
+      <c r="G14" s="247"/>
+      <c r="H14" s="247"/>
+      <c r="I14" s="247"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -42541,7 +42541,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="257"/>
+      <c r="P14" s="255"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>

</xml_diff>

<commit_message>
fix(schema): allow manual_duration to be saved and update excel report stability
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA686C7-84B9-4A3A-BBE7-F2415C45845B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02DF717D-E059-4EAC-9B08-848151C5FD45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -450,14 +450,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="8">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0.00;\-#,##0.00;;@"/>
     <numFmt numFmtId="165" formatCode="_(&quot;Rp&quot;* #,##0.00_);_(&quot;Rp&quot;* \(#,##0.00\);_(&quot;Rp&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="[$-421]dddd"/>
     <numFmt numFmtId="168" formatCode="[$-421]dd\ mmm\ yyyy;@"/>
     <numFmt numFmtId="169" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="170" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="171" formatCode="0.000"/>
   </numFmts>
   <fonts count="34">
@@ -2430,29 +2429,7 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="32" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="33" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="36" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="24" fillId="0" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -2460,21 +2437,9 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="38" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="33" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="41" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="42" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2592,181 +2557,120 @@
     <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="75" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="115" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="116" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="0" borderId="53" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="0" borderId="53" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="52" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="39" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="114" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="26" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="61" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="66" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="59" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="54" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="111" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="112" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2874,53 +2778,187 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="39" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="61" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="66" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="59" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="114" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="54" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="75" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3051,80 +3089,47 @@
     <xf numFmtId="0" fontId="32" fillId="4" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="111" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="112" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="115" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="116" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="10" fontId="24" fillId="0" borderId="53" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="24" fillId="0" borderId="53" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="52" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="38" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="42" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="41" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -4244,40 +4249,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="250"/>
-      <c r="C1" s="250"/>
-      <c r="D1" s="250"/>
-      <c r="E1" s="250"/>
-      <c r="F1" s="250"/>
-      <c r="G1" s="250"/>
-      <c r="H1" s="250"/>
-      <c r="I1" s="250"/>
-      <c r="J1" s="250"/>
-      <c r="K1" s="250"/>
-      <c r="L1" s="250"/>
-      <c r="M1" s="250"/>
-      <c r="N1" s="250"/>
-      <c r="O1" s="250"/>
-      <c r="P1" s="250"/>
+      <c r="B1" s="261"/>
+      <c r="C1" s="261"/>
+      <c r="D1" s="261"/>
+      <c r="E1" s="261"/>
+      <c r="F1" s="261"/>
+      <c r="G1" s="261"/>
+      <c r="H1" s="261"/>
+      <c r="I1" s="261"/>
+      <c r="J1" s="261"/>
+      <c r="K1" s="261"/>
+      <c r="L1" s="261"/>
+      <c r="M1" s="261"/>
+      <c r="N1" s="261"/>
+      <c r="O1" s="261"/>
+      <c r="P1" s="261"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="248" t="s">
+      <c r="B2" s="259" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="249"/>
-      <c r="D2" s="249"/>
-      <c r="E2" s="249"/>
-      <c r="F2" s="249"/>
-      <c r="G2" s="249"/>
-      <c r="H2" s="249"/>
-      <c r="I2" s="249"/>
-      <c r="J2" s="249"/>
-      <c r="K2" s="249"/>
-      <c r="L2" s="249"/>
-      <c r="M2" s="249"/>
-      <c r="N2" s="249"/>
-      <c r="O2" s="249"/>
-      <c r="P2" s="249"/>
+      <c r="C2" s="260"/>
+      <c r="D2" s="260"/>
+      <c r="E2" s="260"/>
+      <c r="F2" s="260"/>
+      <c r="G2" s="260"/>
+      <c r="H2" s="260"/>
+      <c r="I2" s="260"/>
+      <c r="J2" s="260"/>
+      <c r="K2" s="260"/>
+      <c r="L2" s="260"/>
+      <c r="M2" s="260"/>
+      <c r="N2" s="260"/>
+      <c r="O2" s="260"/>
+      <c r="P2" s="260"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4304,16 +4309,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="256" t="s">
+      <c r="I4" s="267" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="256"/>
-      <c r="K4" s="256"/>
-      <c r="L4" s="256"/>
-      <c r="M4" s="256"/>
-      <c r="N4" s="256"/>
-      <c r="O4" s="256"/>
-      <c r="P4" s="256"/>
+      <c r="J4" s="267"/>
+      <c r="K4" s="267"/>
+      <c r="L4" s="267"/>
+      <c r="M4" s="267"/>
+      <c r="N4" s="267"/>
+      <c r="O4" s="267"/>
+      <c r="P4" s="267"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4327,14 +4332,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="256"/>
-      <c r="J5" s="256"/>
-      <c r="K5" s="256"/>
-      <c r="L5" s="256"/>
-      <c r="M5" s="256"/>
-      <c r="N5" s="256"/>
-      <c r="O5" s="256"/>
-      <c r="P5" s="256"/>
+      <c r="I5" s="267"/>
+      <c r="J5" s="267"/>
+      <c r="K5" s="267"/>
+      <c r="L5" s="267"/>
+      <c r="M5" s="267"/>
+      <c r="N5" s="267"/>
+      <c r="O5" s="267"/>
+      <c r="P5" s="267"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4469,70 +4474,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="247" t="s">
+      <c r="B12" s="258" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="247" t="s">
+      <c r="C12" s="258" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="247"/>
-      <c r="E12" s="247"/>
-      <c r="F12" s="247" t="s">
+      <c r="D12" s="258"/>
+      <c r="E12" s="258"/>
+      <c r="F12" s="258" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="247" t="s">
+      <c r="G12" s="258" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="247" t="s">
+      <c r="H12" s="258" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="247" t="s">
+      <c r="I12" s="258" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="247" t="s">
+      <c r="J12" s="258" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="247"/>
-      <c r="L12" s="247"/>
-      <c r="M12" s="247"/>
-      <c r="N12" s="247"/>
-      <c r="O12" s="247"/>
-      <c r="P12" s="255" t="s">
+      <c r="K12" s="258"/>
+      <c r="L12" s="258"/>
+      <c r="M12" s="258"/>
+      <c r="N12" s="258"/>
+      <c r="O12" s="258"/>
+      <c r="P12" s="266" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="247"/>
-      <c r="C13" s="247"/>
-      <c r="D13" s="247"/>
-      <c r="E13" s="247"/>
-      <c r="F13" s="247"/>
-      <c r="G13" s="247"/>
-      <c r="H13" s="247"/>
-      <c r="I13" s="247"/>
-      <c r="J13" s="254" t="s">
+      <c r="B13" s="258"/>
+      <c r="C13" s="258"/>
+      <c r="D13" s="258"/>
+      <c r="E13" s="258"/>
+      <c r="F13" s="258"/>
+      <c r="G13" s="258"/>
+      <c r="H13" s="258"/>
+      <c r="I13" s="258"/>
+      <c r="J13" s="265" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="254"/>
-      <c r="L13" s="254" t="s">
+      <c r="K13" s="265"/>
+      <c r="L13" s="265" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="254"/>
-      <c r="N13" s="254" t="s">
+      <c r="M13" s="265"/>
+      <c r="N13" s="265" t="s">
         <v>95</v>
       </c>
-      <c r="O13" s="254"/>
-      <c r="P13" s="255"/>
+      <c r="O13" s="265"/>
+      <c r="P13" s="266"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="247"/>
-      <c r="C14" s="247"/>
-      <c r="D14" s="247"/>
-      <c r="E14" s="247"/>
-      <c r="F14" s="247"/>
-      <c r="G14" s="247"/>
-      <c r="H14" s="247"/>
-      <c r="I14" s="247"/>
+      <c r="B14" s="258"/>
+      <c r="C14" s="258"/>
+      <c r="D14" s="258"/>
+      <c r="E14" s="258"/>
+      <c r="F14" s="258"/>
+      <c r="G14" s="258"/>
+      <c r="H14" s="258"/>
+      <c r="I14" s="258"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -4551,7 +4556,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="255"/>
+      <c r="P14" s="266"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -4974,38 +4979,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="103.2" customHeight="1">
-      <c r="B1" s="249"/>
-      <c r="C1" s="249"/>
-      <c r="D1" s="249"/>
-      <c r="E1" s="249"/>
-      <c r="F1" s="249"/>
-      <c r="G1" s="249"/>
-      <c r="H1" s="249"/>
-      <c r="I1" s="249"/>
-      <c r="J1" s="249"/>
-      <c r="K1" s="249"/>
-      <c r="L1" s="249"/>
-      <c r="M1" s="249"/>
-      <c r="N1" s="249"/>
-      <c r="O1" s="249"/>
+      <c r="B1" s="260"/>
+      <c r="C1" s="260"/>
+      <c r="D1" s="260"/>
+      <c r="E1" s="260"/>
+      <c r="F1" s="260"/>
+      <c r="G1" s="260"/>
+      <c r="H1" s="260"/>
+      <c r="I1" s="260"/>
+      <c r="J1" s="260"/>
+      <c r="K1" s="260"/>
+      <c r="L1" s="260"/>
+      <c r="M1" s="260"/>
+      <c r="N1" s="260"/>
+      <c r="O1" s="260"/>
     </row>
     <row r="2" spans="2:15" ht="22.95" customHeight="1">
-      <c r="B2" s="257" t="s">
+      <c r="B2" s="268" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="257"/>
-      <c r="F2" s="257"/>
-      <c r="G2" s="257"/>
-      <c r="H2" s="257"/>
-      <c r="I2" s="257"/>
-      <c r="J2" s="257"/>
-      <c r="K2" s="257"/>
-      <c r="L2" s="257"/>
-      <c r="M2" s="257"/>
-      <c r="N2" s="257"/>
-      <c r="O2" s="257"/>
+      <c r="C2" s="268"/>
+      <c r="D2" s="268"/>
+      <c r="E2" s="268"/>
+      <c r="F2" s="268"/>
+      <c r="G2" s="268"/>
+      <c r="H2" s="268"/>
+      <c r="I2" s="268"/>
+      <c r="J2" s="268"/>
+      <c r="K2" s="268"/>
+      <c r="L2" s="268"/>
+      <c r="M2" s="268"/>
+      <c r="N2" s="268"/>
+      <c r="O2" s="268"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" t="s">
@@ -5057,179 +5062,179 @@
     </row>
     <row r="9" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="11" spans="2:15" s="58" customFormat="1">
-      <c r="B11" s="258" t="s">
+      <c r="B11" s="269" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="258"/>
-      <c r="D11" s="258"/>
-      <c r="E11" s="258"/>
-      <c r="G11" s="258" t="s">
+      <c r="C11" s="269"/>
+      <c r="D11" s="269"/>
+      <c r="E11" s="269"/>
+      <c r="G11" s="269" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="258"/>
-      <c r="I11" s="258"/>
-      <c r="J11" s="258"/>
-      <c r="L11" s="258" t="s">
+      <c r="H11" s="269"/>
+      <c r="I11" s="269"/>
+      <c r="J11" s="269"/>
+      <c r="L11" s="269" t="s">
         <v>105</v>
       </c>
-      <c r="M11" s="258"/>
-      <c r="N11" s="258"/>
-      <c r="O11" s="258"/>
+      <c r="M11" s="269"/>
+      <c r="N11" s="269"/>
+      <c r="O11" s="269"/>
     </row>
     <row r="12" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="13" spans="2:15">
-      <c r="B13" s="249"/>
-      <c r="C13" s="249"/>
-      <c r="D13" s="249"/>
-      <c r="E13" s="249"/>
-      <c r="G13" s="249"/>
-      <c r="H13" s="249"/>
-      <c r="I13" s="249"/>
-      <c r="J13" s="249"/>
-      <c r="L13" s="249"/>
-      <c r="M13" s="249"/>
-      <c r="N13" s="249"/>
-      <c r="O13" s="249"/>
+      <c r="B13" s="260"/>
+      <c r="C13" s="260"/>
+      <c r="D13" s="260"/>
+      <c r="E13" s="260"/>
+      <c r="G13" s="260"/>
+      <c r="H13" s="260"/>
+      <c r="I13" s="260"/>
+      <c r="J13" s="260"/>
+      <c r="L13" s="260"/>
+      <c r="M13" s="260"/>
+      <c r="N13" s="260"/>
+      <c r="O13" s="260"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="249"/>
-      <c r="C14" s="249"/>
-      <c r="D14" s="249"/>
-      <c r="E14" s="249"/>
-      <c r="G14" s="249"/>
-      <c r="H14" s="249"/>
-      <c r="I14" s="249"/>
-      <c r="J14" s="249"/>
-      <c r="L14" s="249"/>
-      <c r="M14" s="249"/>
-      <c r="N14" s="249"/>
-      <c r="O14" s="249"/>
+      <c r="B14" s="260"/>
+      <c r="C14" s="260"/>
+      <c r="D14" s="260"/>
+      <c r="E14" s="260"/>
+      <c r="G14" s="260"/>
+      <c r="H14" s="260"/>
+      <c r="I14" s="260"/>
+      <c r="J14" s="260"/>
+      <c r="L14" s="260"/>
+      <c r="M14" s="260"/>
+      <c r="N14" s="260"/>
+      <c r="O14" s="260"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="249"/>
-      <c r="C15" s="249"/>
-      <c r="D15" s="249"/>
-      <c r="E15" s="249"/>
-      <c r="G15" s="249"/>
-      <c r="H15" s="249"/>
-      <c r="I15" s="249"/>
-      <c r="J15" s="249"/>
-      <c r="L15" s="249"/>
-      <c r="M15" s="249"/>
-      <c r="N15" s="249"/>
-      <c r="O15" s="249"/>
+      <c r="B15" s="260"/>
+      <c r="C15" s="260"/>
+      <c r="D15" s="260"/>
+      <c r="E15" s="260"/>
+      <c r="G15" s="260"/>
+      <c r="H15" s="260"/>
+      <c r="I15" s="260"/>
+      <c r="J15" s="260"/>
+      <c r="L15" s="260"/>
+      <c r="M15" s="260"/>
+      <c r="N15" s="260"/>
+      <c r="O15" s="260"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="249"/>
-      <c r="C16" s="249"/>
-      <c r="D16" s="249"/>
-      <c r="E16" s="249"/>
-      <c r="G16" s="249"/>
-      <c r="H16" s="249"/>
-      <c r="I16" s="249"/>
-      <c r="J16" s="249"/>
-      <c r="L16" s="249"/>
-      <c r="M16" s="249"/>
-      <c r="N16" s="249"/>
-      <c r="O16" s="249"/>
+      <c r="B16" s="260"/>
+      <c r="C16" s="260"/>
+      <c r="D16" s="260"/>
+      <c r="E16" s="260"/>
+      <c r="G16" s="260"/>
+      <c r="H16" s="260"/>
+      <c r="I16" s="260"/>
+      <c r="J16" s="260"/>
+      <c r="L16" s="260"/>
+      <c r="M16" s="260"/>
+      <c r="N16" s="260"/>
+      <c r="O16" s="260"/>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="249"/>
-      <c r="C17" s="249"/>
-      <c r="D17" s="249"/>
-      <c r="E17" s="249"/>
-      <c r="G17" s="249"/>
-      <c r="H17" s="249"/>
-      <c r="I17" s="249"/>
-      <c r="J17" s="249"/>
-      <c r="L17" s="249"/>
-      <c r="M17" s="249"/>
-      <c r="N17" s="249"/>
-      <c r="O17" s="249"/>
+      <c r="B17" s="260"/>
+      <c r="C17" s="260"/>
+      <c r="D17" s="260"/>
+      <c r="E17" s="260"/>
+      <c r="G17" s="260"/>
+      <c r="H17" s="260"/>
+      <c r="I17" s="260"/>
+      <c r="J17" s="260"/>
+      <c r="L17" s="260"/>
+      <c r="M17" s="260"/>
+      <c r="N17" s="260"/>
+      <c r="O17" s="260"/>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="249"/>
-      <c r="C18" s="249"/>
-      <c r="D18" s="249"/>
-      <c r="E18" s="249"/>
-      <c r="G18" s="249"/>
-      <c r="H18" s="249"/>
-      <c r="I18" s="249"/>
-      <c r="J18" s="249"/>
-      <c r="L18" s="249"/>
-      <c r="M18" s="249"/>
-      <c r="N18" s="249"/>
-      <c r="O18" s="249"/>
+      <c r="B18" s="260"/>
+      <c r="C18" s="260"/>
+      <c r="D18" s="260"/>
+      <c r="E18" s="260"/>
+      <c r="G18" s="260"/>
+      <c r="H18" s="260"/>
+      <c r="I18" s="260"/>
+      <c r="J18" s="260"/>
+      <c r="L18" s="260"/>
+      <c r="M18" s="260"/>
+      <c r="N18" s="260"/>
+      <c r="O18" s="260"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="B19" s="249"/>
-      <c r="C19" s="249"/>
-      <c r="D19" s="249"/>
-      <c r="E19" s="249"/>
-      <c r="G19" s="249"/>
-      <c r="H19" s="249"/>
-      <c r="I19" s="249"/>
-      <c r="J19" s="249"/>
-      <c r="L19" s="249"/>
-      <c r="M19" s="249"/>
-      <c r="N19" s="249"/>
-      <c r="O19" s="249"/>
+      <c r="B19" s="260"/>
+      <c r="C19" s="260"/>
+      <c r="D19" s="260"/>
+      <c r="E19" s="260"/>
+      <c r="G19" s="260"/>
+      <c r="H19" s="260"/>
+      <c r="I19" s="260"/>
+      <c r="J19" s="260"/>
+      <c r="L19" s="260"/>
+      <c r="M19" s="260"/>
+      <c r="N19" s="260"/>
+      <c r="O19" s="260"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="B20" s="249"/>
-      <c r="C20" s="249"/>
-      <c r="D20" s="249"/>
-      <c r="E20" s="249"/>
-      <c r="G20" s="249"/>
-      <c r="H20" s="249"/>
-      <c r="I20" s="249"/>
-      <c r="J20" s="249"/>
-      <c r="L20" s="249"/>
-      <c r="M20" s="249"/>
-      <c r="N20" s="249"/>
-      <c r="O20" s="249"/>
+      <c r="B20" s="260"/>
+      <c r="C20" s="260"/>
+      <c r="D20" s="260"/>
+      <c r="E20" s="260"/>
+      <c r="G20" s="260"/>
+      <c r="H20" s="260"/>
+      <c r="I20" s="260"/>
+      <c r="J20" s="260"/>
+      <c r="L20" s="260"/>
+      <c r="M20" s="260"/>
+      <c r="N20" s="260"/>
+      <c r="O20" s="260"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="B21" s="249"/>
-      <c r="C21" s="249"/>
-      <c r="D21" s="249"/>
-      <c r="E21" s="249"/>
-      <c r="G21" s="249"/>
-      <c r="H21" s="249"/>
-      <c r="I21" s="249"/>
-      <c r="J21" s="249"/>
-      <c r="L21" s="249"/>
-      <c r="M21" s="249"/>
-      <c r="N21" s="249"/>
-      <c r="O21" s="249"/>
+      <c r="B21" s="260"/>
+      <c r="C21" s="260"/>
+      <c r="D21" s="260"/>
+      <c r="E21" s="260"/>
+      <c r="G21" s="260"/>
+      <c r="H21" s="260"/>
+      <c r="I21" s="260"/>
+      <c r="J21" s="260"/>
+      <c r="L21" s="260"/>
+      <c r="M21" s="260"/>
+      <c r="N21" s="260"/>
+      <c r="O21" s="260"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="B22" s="249"/>
-      <c r="C22" s="249"/>
-      <c r="D22" s="249"/>
-      <c r="E22" s="249"/>
-      <c r="G22" s="249"/>
-      <c r="H22" s="249"/>
-      <c r="I22" s="249"/>
-      <c r="J22" s="249"/>
-      <c r="L22" s="249"/>
-      <c r="M22" s="249"/>
-      <c r="N22" s="249"/>
-      <c r="O22" s="249"/>
+      <c r="B22" s="260"/>
+      <c r="C22" s="260"/>
+      <c r="D22" s="260"/>
+      <c r="E22" s="260"/>
+      <c r="G22" s="260"/>
+      <c r="H22" s="260"/>
+      <c r="I22" s="260"/>
+      <c r="J22" s="260"/>
+      <c r="L22" s="260"/>
+      <c r="M22" s="260"/>
+      <c r="N22" s="260"/>
+      <c r="O22" s="260"/>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="249"/>
-      <c r="C23" s="249"/>
-      <c r="D23" s="249"/>
-      <c r="E23" s="249"/>
-      <c r="G23" s="249"/>
-      <c r="H23" s="249"/>
-      <c r="I23" s="249"/>
-      <c r="J23" s="249"/>
-      <c r="L23" s="249"/>
-      <c r="M23" s="249"/>
-      <c r="N23" s="249"/>
-      <c r="O23" s="249"/>
+      <c r="B23" s="260"/>
+      <c r="C23" s="260"/>
+      <c r="D23" s="260"/>
+      <c r="E23" s="260"/>
+      <c r="G23" s="260"/>
+      <c r="H23" s="260"/>
+      <c r="I23" s="260"/>
+      <c r="J23" s="260"/>
+      <c r="L23" s="260"/>
+      <c r="M23" s="260"/>
+      <c r="N23" s="260"/>
+      <c r="O23" s="260"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5263,330 +5268,330 @@
   <sheetData>
     <row r="1" spans="2:29" ht="4.8" customHeight="1" thickBot="1"/>
     <row r="2" spans="2:29" ht="19.95" customHeight="1" thickBot="1">
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="270" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="260"/>
-      <c r="D2" s="260"/>
-      <c r="E2" s="260"/>
-      <c r="F2" s="260"/>
-      <c r="G2" s="260"/>
-      <c r="H2" s="260"/>
-      <c r="I2" s="260"/>
-      <c r="J2" s="260"/>
-      <c r="K2" s="260"/>
-      <c r="L2" s="260"/>
-      <c r="M2" s="260"/>
-      <c r="N2" s="260"/>
-      <c r="O2" s="260"/>
-      <c r="P2" s="260"/>
-      <c r="Q2" s="260"/>
-      <c r="R2" s="260"/>
-      <c r="S2" s="260"/>
-      <c r="T2" s="260"/>
-      <c r="U2" s="260"/>
-      <c r="V2" s="260"/>
-      <c r="W2" s="260"/>
-      <c r="X2" s="260"/>
-      <c r="Y2" s="260"/>
-      <c r="Z2" s="260"/>
-      <c r="AA2" s="260"/>
-      <c r="AB2" s="261"/>
-      <c r="AC2" s="137"/>
+      <c r="C2" s="271"/>
+      <c r="D2" s="271"/>
+      <c r="E2" s="271"/>
+      <c r="F2" s="271"/>
+      <c r="G2" s="271"/>
+      <c r="H2" s="271"/>
+      <c r="I2" s="271"/>
+      <c r="J2" s="271"/>
+      <c r="K2" s="271"/>
+      <c r="L2" s="271"/>
+      <c r="M2" s="271"/>
+      <c r="N2" s="271"/>
+      <c r="O2" s="271"/>
+      <c r="P2" s="271"/>
+      <c r="Q2" s="271"/>
+      <c r="R2" s="271"/>
+      <c r="S2" s="271"/>
+      <c r="T2" s="271"/>
+      <c r="U2" s="271"/>
+      <c r="V2" s="271"/>
+      <c r="W2" s="271"/>
+      <c r="X2" s="271"/>
+      <c r="Y2" s="271"/>
+      <c r="Z2" s="271"/>
+      <c r="AA2" s="271"/>
+      <c r="AB2" s="272"/>
+      <c r="AC2" s="127"/>
     </row>
     <row r="3" spans="2:29" ht="15" customHeight="1">
-      <c r="B3" s="136"/>
-      <c r="AB3" s="131"/>
+      <c r="B3" s="126"/>
+      <c r="AB3" s="121"/>
     </row>
     <row r="4" spans="2:29" ht="15" customHeight="1">
-      <c r="B4" s="130" t="s">
+      <c r="B4" s="120" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="132" t="s">
+      <c r="D4" s="122" t="s">
         <v>20</v>
       </c>
-      <c r="AB4" s="131"/>
+      <c r="AB4" s="121"/>
     </row>
     <row r="5" spans="2:29" ht="15" customHeight="1">
-      <c r="B5" s="130" t="s">
+      <c r="B5" s="120" t="s">
         <v>108</v>
       </c>
-      <c r="D5" s="132" t="s">
+      <c r="D5" s="122" t="s">
         <v>20</v>
       </c>
-      <c r="AB5" s="131"/>
+      <c r="AB5" s="121"/>
     </row>
     <row r="6" spans="2:29" ht="15" customHeight="1">
-      <c r="B6" s="130" t="s">
+      <c r="B6" s="120" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="132" t="s">
+      <c r="D6" s="122" t="s">
         <v>20</v>
       </c>
-      <c r="AB6" s="131"/>
+      <c r="AB6" s="121"/>
     </row>
     <row r="7" spans="2:29" ht="15" customHeight="1">
-      <c r="B7" s="130" t="s">
+      <c r="B7" s="120" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="132" t="s">
+      <c r="D7" s="122" t="s">
         <v>20</v>
       </c>
-      <c r="AB7" s="131"/>
+      <c r="AB7" s="121"/>
     </row>
     <row r="8" spans="2:29" ht="15" customHeight="1">
-      <c r="B8" s="130" t="s">
+      <c r="B8" s="120" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="132" t="s">
+      <c r="D8" s="122" t="s">
         <v>20</v>
       </c>
-      <c r="AB8" s="131"/>
+      <c r="AB8" s="121"/>
     </row>
     <row r="9" spans="2:29" ht="15" customHeight="1">
-      <c r="B9" s="130" t="s">
+      <c r="B9" s="120" t="s">
         <v>110</v>
       </c>
-      <c r="D9" s="132" t="s">
+      <c r="D9" s="122" t="s">
         <v>20</v>
       </c>
-      <c r="AB9" s="131"/>
+      <c r="AB9" s="121"/>
     </row>
     <row r="10" spans="2:29" ht="15" customHeight="1">
-      <c r="B10" s="130" t="s">
+      <c r="B10" s="120" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="132" t="s">
+      <c r="D10" s="122" t="s">
         <v>20</v>
       </c>
-      <c r="AB10" s="131"/>
+      <c r="AB10" s="121"/>
     </row>
     <row r="11" spans="2:29" ht="15" customHeight="1" thickBot="1">
-      <c r="B11" s="133"/>
-      <c r="C11" s="134"/>
-      <c r="D11" s="134"/>
-      <c r="E11" s="134"/>
-      <c r="F11" s="134"/>
-      <c r="G11" s="134"/>
-      <c r="H11" s="134"/>
-      <c r="I11" s="134"/>
-      <c r="J11" s="134"/>
-      <c r="K11" s="134"/>
-      <c r="L11" s="134"/>
-      <c r="M11" s="134"/>
-      <c r="N11" s="134"/>
-      <c r="O11" s="134"/>
-      <c r="P11" s="134"/>
-      <c r="Q11" s="134"/>
-      <c r="R11" s="134"/>
-      <c r="S11" s="134"/>
-      <c r="T11" s="134"/>
-      <c r="U11" s="134"/>
-      <c r="V11" s="134"/>
-      <c r="W11" s="134"/>
-      <c r="X11" s="134"/>
-      <c r="Y11" s="134"/>
-      <c r="Z11" s="134"/>
-      <c r="AA11" s="134"/>
-      <c r="AB11" s="135"/>
+      <c r="B11" s="123"/>
+      <c r="C11" s="124"/>
+      <c r="D11" s="124"/>
+      <c r="E11" s="124"/>
+      <c r="F11" s="124"/>
+      <c r="G11" s="124"/>
+      <c r="H11" s="124"/>
+      <c r="I11" s="124"/>
+      <c r="J11" s="124"/>
+      <c r="K11" s="124"/>
+      <c r="L11" s="124"/>
+      <c r="M11" s="124"/>
+      <c r="N11" s="124"/>
+      <c r="O11" s="124"/>
+      <c r="P11" s="124"/>
+      <c r="Q11" s="124"/>
+      <c r="R11" s="124"/>
+      <c r="S11" s="124"/>
+      <c r="T11" s="124"/>
+      <c r="U11" s="124"/>
+      <c r="V11" s="124"/>
+      <c r="W11" s="124"/>
+      <c r="X11" s="124"/>
+      <c r="Y11" s="124"/>
+      <c r="Z11" s="124"/>
+      <c r="AA11" s="124"/>
+      <c r="AB11" s="125"/>
     </row>
     <row r="12" spans="2:29" ht="15" customHeight="1">
-      <c r="B12" s="271" t="s">
+      <c r="B12" s="282" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="273" t="s">
+      <c r="C12" s="284" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="274"/>
-      <c r="E12" s="274"/>
-      <c r="F12" s="274"/>
-      <c r="G12" s="274"/>
-      <c r="H12" s="274"/>
-      <c r="I12" s="274"/>
-      <c r="J12" s="274"/>
-      <c r="K12" s="274"/>
-      <c r="L12" s="275"/>
-      <c r="M12" s="279" t="s">
+      <c r="D12" s="285"/>
+      <c r="E12" s="285"/>
+      <c r="F12" s="285"/>
+      <c r="G12" s="285"/>
+      <c r="H12" s="285"/>
+      <c r="I12" s="285"/>
+      <c r="J12" s="285"/>
+      <c r="K12" s="285"/>
+      <c r="L12" s="286"/>
+      <c r="M12" s="290" t="s">
         <v>113</v>
       </c>
-      <c r="N12" s="279" t="s">
+      <c r="N12" s="290" t="s">
         <v>34</v>
       </c>
-      <c r="O12" s="284" t="s">
+      <c r="O12" s="295" t="s">
         <v>114</v>
       </c>
-      <c r="P12" s="284"/>
-      <c r="Q12" s="284"/>
-      <c r="R12" s="284"/>
-      <c r="S12" s="284"/>
-      <c r="T12" s="284"/>
-      <c r="U12" s="284"/>
-      <c r="V12" s="284"/>
-      <c r="W12" s="284"/>
-      <c r="X12" s="284"/>
-      <c r="Y12" s="284"/>
-      <c r="Z12" s="284"/>
-      <c r="AA12" s="284"/>
-      <c r="AB12" s="285"/>
+      <c r="P12" s="295"/>
+      <c r="Q12" s="295"/>
+      <c r="R12" s="295"/>
+      <c r="S12" s="295"/>
+      <c r="T12" s="295"/>
+      <c r="U12" s="295"/>
+      <c r="V12" s="295"/>
+      <c r="W12" s="295"/>
+      <c r="X12" s="295"/>
+      <c r="Y12" s="295"/>
+      <c r="Z12" s="295"/>
+      <c r="AA12" s="295"/>
+      <c r="AB12" s="296"/>
     </row>
     <row r="13" spans="2:29" ht="15" customHeight="1">
-      <c r="B13" s="272"/>
-      <c r="C13" s="276"/>
-      <c r="D13" s="277"/>
-      <c r="E13" s="277"/>
-      <c r="F13" s="277"/>
-      <c r="G13" s="277"/>
-      <c r="H13" s="277"/>
-      <c r="I13" s="277"/>
-      <c r="J13" s="277"/>
-      <c r="K13" s="277"/>
-      <c r="L13" s="278"/>
-      <c r="M13" s="280"/>
-      <c r="N13" s="280"/>
-      <c r="O13" s="281" t="s">
+      <c r="B13" s="283"/>
+      <c r="C13" s="287"/>
+      <c r="D13" s="288"/>
+      <c r="E13" s="288"/>
+      <c r="F13" s="288"/>
+      <c r="G13" s="288"/>
+      <c r="H13" s="288"/>
+      <c r="I13" s="288"/>
+      <c r="J13" s="288"/>
+      <c r="K13" s="288"/>
+      <c r="L13" s="289"/>
+      <c r="M13" s="291"/>
+      <c r="N13" s="291"/>
+      <c r="O13" s="292" t="s">
         <v>115</v>
       </c>
-      <c r="P13" s="282"/>
-      <c r="Q13" s="283"/>
-      <c r="R13" s="281" t="s">
+      <c r="P13" s="293"/>
+      <c r="Q13" s="294"/>
+      <c r="R13" s="292" t="s">
         <v>116</v>
       </c>
-      <c r="S13" s="282"/>
-      <c r="T13" s="283"/>
-      <c r="U13" s="281" t="s">
+      <c r="S13" s="293"/>
+      <c r="T13" s="294"/>
+      <c r="U13" s="292" t="s">
         <v>117</v>
       </c>
-      <c r="V13" s="282"/>
-      <c r="W13" s="283"/>
-      <c r="X13" s="262" t="s">
+      <c r="V13" s="293"/>
+      <c r="W13" s="294"/>
+      <c r="X13" s="273" t="s">
         <v>118</v>
       </c>
-      <c r="Y13" s="142" t="s">
+      <c r="Y13" s="132" t="s">
         <v>119</v>
       </c>
-      <c r="Z13" s="143" t="s">
+      <c r="Z13" s="133" t="s">
         <v>119</v>
       </c>
-      <c r="AA13" s="264" t="s">
+      <c r="AA13" s="275" t="s">
         <v>120</v>
       </c>
-      <c r="AB13" s="266" t="s">
+      <c r="AB13" s="277" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="14" spans="2:29" ht="15" customHeight="1">
-      <c r="B14" s="272"/>
-      <c r="C14" s="276"/>
-      <c r="D14" s="277"/>
-      <c r="E14" s="277"/>
-      <c r="F14" s="277"/>
-      <c r="G14" s="277"/>
-      <c r="H14" s="277"/>
-      <c r="I14" s="277"/>
-      <c r="J14" s="277"/>
-      <c r="K14" s="277"/>
-      <c r="L14" s="278"/>
-      <c r="M14" s="263"/>
-      <c r="N14" s="263"/>
-      <c r="O14" s="144" t="s">
+      <c r="B14" s="283"/>
+      <c r="C14" s="287"/>
+      <c r="D14" s="288"/>
+      <c r="E14" s="288"/>
+      <c r="F14" s="288"/>
+      <c r="G14" s="288"/>
+      <c r="H14" s="288"/>
+      <c r="I14" s="288"/>
+      <c r="J14" s="288"/>
+      <c r="K14" s="288"/>
+      <c r="L14" s="289"/>
+      <c r="M14" s="274"/>
+      <c r="N14" s="274"/>
+      <c r="O14" s="134" t="s">
         <v>122</v>
       </c>
-      <c r="P14" s="144" t="s">
+      <c r="P14" s="134" t="s">
         <v>123</v>
       </c>
-      <c r="Q14" s="144" t="s">
+      <c r="Q14" s="134" t="s">
         <v>124</v>
       </c>
-      <c r="R14" s="144" t="s">
+      <c r="R14" s="134" t="s">
         <v>125</v>
       </c>
-      <c r="S14" s="144" t="s">
+      <c r="S14" s="134" t="s">
         <v>126</v>
       </c>
-      <c r="T14" s="144" t="s">
+      <c r="T14" s="134" t="s">
         <v>124</v>
       </c>
-      <c r="U14" s="144" t="s">
+      <c r="U14" s="134" t="s">
         <v>127</v>
       </c>
-      <c r="V14" s="144" t="s">
+      <c r="V14" s="134" t="s">
         <v>128</v>
       </c>
-      <c r="W14" s="144" t="s">
+      <c r="W14" s="134" t="s">
         <v>129</v>
       </c>
-      <c r="X14" s="263"/>
-      <c r="Y14" s="142" t="s">
+      <c r="X14" s="274"/>
+      <c r="Y14" s="132" t="s">
         <v>130</v>
       </c>
-      <c r="Z14" s="144" t="s">
+      <c r="Z14" s="134" t="s">
         <v>131</v>
       </c>
-      <c r="AA14" s="265"/>
-      <c r="AB14" s="267"/>
+      <c r="AA14" s="276"/>
+      <c r="AB14" s="278"/>
     </row>
     <row r="15" spans="2:29" ht="15" customHeight="1" thickBot="1">
-      <c r="B15" s="138">
+      <c r="B15" s="128">
         <v>1</v>
       </c>
-      <c r="C15" s="268">
+      <c r="C15" s="279">
         <v>2</v>
       </c>
-      <c r="D15" s="269"/>
-      <c r="E15" s="269"/>
-      <c r="F15" s="269"/>
-      <c r="G15" s="269"/>
-      <c r="H15" s="269"/>
-      <c r="I15" s="269"/>
-      <c r="J15" s="269"/>
-      <c r="K15" s="269"/>
-      <c r="L15" s="270"/>
-      <c r="M15" s="139">
+      <c r="D15" s="280"/>
+      <c r="E15" s="280"/>
+      <c r="F15" s="280"/>
+      <c r="G15" s="280"/>
+      <c r="H15" s="280"/>
+      <c r="I15" s="280"/>
+      <c r="J15" s="280"/>
+      <c r="K15" s="280"/>
+      <c r="L15" s="281"/>
+      <c r="M15" s="129">
         <v>3</v>
       </c>
-      <c r="N15" s="139">
+      <c r="N15" s="129">
         <v>4</v>
       </c>
-      <c r="O15" s="140">
+      <c r="O15" s="130">
         <v>5</v>
       </c>
-      <c r="P15" s="140">
+      <c r="P15" s="130">
         <v>6</v>
       </c>
-      <c r="Q15" s="140">
+      <c r="Q15" s="130">
         <v>7</v>
       </c>
-      <c r="R15" s="140">
+      <c r="R15" s="130">
         <v>8</v>
       </c>
-      <c r="S15" s="140">
+      <c r="S15" s="130">
         <v>9</v>
       </c>
-      <c r="T15" s="140">
+      <c r="T15" s="130">
         <v>10</v>
       </c>
-      <c r="U15" s="140">
+      <c r="U15" s="130">
         <v>11</v>
       </c>
-      <c r="V15" s="140">
+      <c r="V15" s="130">
         <v>12</v>
       </c>
-      <c r="W15" s="140">
+      <c r="W15" s="130">
         <v>13</v>
       </c>
-      <c r="X15" s="140">
+      <c r="X15" s="130">
         <v>14</v>
       </c>
-      <c r="Y15" s="140">
+      <c r="Y15" s="130">
         <v>15</v>
       </c>
-      <c r="Z15" s="140">
+      <c r="Z15" s="130">
         <v>16</v>
       </c>
-      <c r="AA15" s="140">
+      <c r="AA15" s="130">
         <v>17</v>
       </c>
-      <c r="AB15" s="141">
+      <c r="AB15" s="131">
         <v>18</v>
       </c>
     </row>
@@ -5630,38 +5635,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="246"/>
-      <c r="C1" s="246"/>
-      <c r="D1" s="246"/>
-      <c r="E1" s="246"/>
-      <c r="F1" s="246"/>
-      <c r="G1" s="246"/>
-      <c r="H1" s="246"/>
-      <c r="I1" s="246"/>
+      <c r="B1" s="257"/>
+      <c r="C1" s="257"/>
+      <c r="D1" s="257"/>
+      <c r="E1" s="257"/>
+      <c r="F1" s="257"/>
+      <c r="G1" s="257"/>
+      <c r="H1" s="257"/>
+      <c r="I1" s="257"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="243" t="s">
+      <c r="B2" s="254" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="243"/>
-      <c r="D2" s="243"/>
-      <c r="E2" s="243"/>
-      <c r="F2" s="243"/>
-      <c r="G2" s="243"/>
-      <c r="H2" s="243"/>
-      <c r="I2" s="243"/>
+      <c r="C2" s="254"/>
+      <c r="D2" s="254"/>
+      <c r="E2" s="254"/>
+      <c r="F2" s="254"/>
+      <c r="G2" s="254"/>
+      <c r="H2" s="254"/>
+      <c r="I2" s="254"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="244" t="s">
+      <c r="B3" s="255" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="244"/>
-      <c r="D3" s="244"/>
-      <c r="E3" s="244"/>
-      <c r="F3" s="244"/>
-      <c r="G3" s="244"/>
-      <c r="H3" s="244"/>
-      <c r="I3" s="244"/>
+      <c r="C3" s="255"/>
+      <c r="D3" s="255"/>
+      <c r="E3" s="255"/>
+      <c r="F3" s="255"/>
+      <c r="G3" s="255"/>
+      <c r="H3" s="255"/>
+      <c r="I3" s="255"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -5669,10 +5674,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="245" t="s">
+      <c r="C5" s="256" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="245"/>
+      <c r="D5" s="256"/>
       <c r="E5" s="11" t="s">
         <v>38</v>
       </c>
@@ -14059,63 +14064,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="246"/>
-      <c r="C1" s="246"/>
-      <c r="D1" s="246"/>
-      <c r="E1" s="246"/>
-      <c r="F1" s="246"/>
-      <c r="G1" s="246"/>
-      <c r="H1" s="246"/>
-      <c r="I1" s="246"/>
-      <c r="J1" s="246"/>
-      <c r="K1" s="246"/>
-      <c r="L1" s="246"/>
-      <c r="M1" s="246"/>
-      <c r="N1" s="246"/>
+      <c r="B1" s="257"/>
+      <c r="C1" s="257"/>
+      <c r="D1" s="257"/>
+      <c r="E1" s="257"/>
+      <c r="F1" s="257"/>
+      <c r="G1" s="257"/>
+      <c r="H1" s="257"/>
+      <c r="I1" s="257"/>
+      <c r="J1" s="257"/>
+      <c r="K1" s="257"/>
+      <c r="L1" s="257"/>
+      <c r="M1" s="257"/>
+      <c r="N1" s="257"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="243" t="s">
+      <c r="B2" s="254" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="243"/>
-      <c r="D2" s="243"/>
-      <c r="E2" s="243"/>
-      <c r="F2" s="243"/>
-      <c r="G2" s="243"/>
-      <c r="H2" s="243"/>
-      <c r="I2" s="243"/>
-      <c r="J2" s="243"/>
-      <c r="K2" s="243"/>
-      <c r="L2" s="243"/>
-      <c r="M2" s="243"/>
-      <c r="N2" s="243"/>
+      <c r="C2" s="254"/>
+      <c r="D2" s="254"/>
+      <c r="E2" s="254"/>
+      <c r="F2" s="254"/>
+      <c r="G2" s="254"/>
+      <c r="H2" s="254"/>
+      <c r="I2" s="254"/>
+      <c r="J2" s="254"/>
+      <c r="K2" s="254"/>
+      <c r="L2" s="254"/>
+      <c r="M2" s="254"/>
+      <c r="N2" s="254"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="244" t="s">
+      <c r="B3" s="255" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="244"/>
-      <c r="D3" s="244"/>
-      <c r="E3" s="244"/>
-      <c r="F3" s="244"/>
-      <c r="G3" s="244"/>
-      <c r="H3" s="244"/>
-      <c r="I3" s="244"/>
-      <c r="J3" s="244"/>
-      <c r="K3" s="244"/>
-      <c r="L3" s="244"/>
-      <c r="M3" s="244"/>
-      <c r="N3" s="244"/>
+      <c r="C3" s="255"/>
+      <c r="D3" s="255"/>
+      <c r="E3" s="255"/>
+      <c r="F3" s="255"/>
+      <c r="G3" s="255"/>
+      <c r="H3" s="255"/>
+      <c r="I3" s="255"/>
+      <c r="J3" s="255"/>
+      <c r="K3" s="255"/>
+      <c r="L3" s="255"/>
+      <c r="M3" s="255"/>
+      <c r="N3" s="255"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="247" t="s">
+      <c r="C5" s="258" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="247"/>
+      <c r="D5" s="258"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -16319,35 +16324,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="246"/>
-      <c r="C1" s="246"/>
-      <c r="D1" s="246"/>
-      <c r="E1" s="246"/>
-      <c r="F1" s="246"/>
-      <c r="G1" s="246"/>
-      <c r="H1" s="246"/>
+      <c r="B1" s="257"/>
+      <c r="C1" s="257"/>
+      <c r="D1" s="257"/>
+      <c r="E1" s="257"/>
+      <c r="F1" s="257"/>
+      <c r="G1" s="257"/>
+      <c r="H1" s="257"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="243" t="s">
+      <c r="B2" s="254" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="243"/>
-      <c r="D2" s="243"/>
-      <c r="E2" s="243"/>
-      <c r="F2" s="243"/>
-      <c r="G2" s="243"/>
-      <c r="H2" s="243"/>
+      <c r="C2" s="254"/>
+      <c r="D2" s="254"/>
+      <c r="E2" s="254"/>
+      <c r="F2" s="254"/>
+      <c r="G2" s="254"/>
+      <c r="H2" s="254"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="244" t="s">
+      <c r="B3" s="255" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="244"/>
-      <c r="D3" s="244"/>
-      <c r="E3" s="244"/>
-      <c r="F3" s="244"/>
-      <c r="G3" s="244"/>
-      <c r="H3" s="244"/>
+      <c r="C3" s="255"/>
+      <c r="D3" s="255"/>
+      <c r="E3" s="255"/>
+      <c r="F3" s="255"/>
+      <c r="G3" s="255"/>
+      <c r="H3" s="255"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -40441,30 +40446,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="250"/>
-      <c r="C1" s="250"/>
-      <c r="D1" s="250"/>
-      <c r="E1" s="250"/>
-      <c r="F1" s="250"/>
-      <c r="G1" s="250"/>
-      <c r="H1" s="250"/>
-      <c r="I1" s="250"/>
-      <c r="J1" s="250"/>
-      <c r="K1" s="250"/>
+      <c r="B1" s="261"/>
+      <c r="C1" s="261"/>
+      <c r="D1" s="261"/>
+      <c r="E1" s="261"/>
+      <c r="F1" s="261"/>
+      <c r="G1" s="261"/>
+      <c r="H1" s="261"/>
+      <c r="I1" s="261"/>
+      <c r="J1" s="261"/>
+      <c r="K1" s="261"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="248" t="s">
+      <c r="B2" s="259" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="249"/>
-      <c r="D2" s="249"/>
-      <c r="E2" s="249"/>
-      <c r="F2" s="249"/>
-      <c r="G2" s="249"/>
-      <c r="H2" s="249"/>
-      <c r="I2" s="249"/>
-      <c r="J2" s="249"/>
-      <c r="K2" s="249"/>
+      <c r="C2" s="260"/>
+      <c r="D2" s="260"/>
+      <c r="E2" s="260"/>
+      <c r="F2" s="260"/>
+      <c r="G2" s="260"/>
+      <c r="H2" s="260"/>
+      <c r="I2" s="260"/>
+      <c r="J2" s="260"/>
+      <c r="K2" s="260"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40584,11 +40589,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="247" t="s">
+      <c r="C11" s="258" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="247"/>
-      <c r="E11" s="247"/>
+      <c r="D11" s="258"/>
+      <c r="E11" s="258"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -40644,26 +40649,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="111.6" customHeight="1">
-      <c r="B1" s="250"/>
-      <c r="C1" s="250"/>
-      <c r="D1" s="250"/>
-      <c r="E1" s="250"/>
-      <c r="F1" s="250"/>
-      <c r="G1" s="250"/>
-      <c r="H1" s="250"/>
-      <c r="I1" s="250"/>
+      <c r="B1" s="261"/>
+      <c r="C1" s="261"/>
+      <c r="D1" s="261"/>
+      <c r="E1" s="261"/>
+      <c r="F1" s="261"/>
+      <c r="G1" s="261"/>
+      <c r="H1" s="261"/>
+      <c r="I1" s="261"/>
     </row>
     <row r="2" spans="2:9" ht="22.95" customHeight="1">
-      <c r="B2" s="248" t="s">
+      <c r="B2" s="259" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="249"/>
-      <c r="D2" s="249"/>
-      <c r="E2" s="249"/>
-      <c r="F2" s="249"/>
-      <c r="G2" s="249"/>
-      <c r="H2" s="249"/>
-      <c r="I2" s="249"/>
+      <c r="C2" s="260"/>
+      <c r="D2" s="260"/>
+      <c r="E2" s="260"/>
+      <c r="F2" s="260"/>
+      <c r="G2" s="260"/>
+      <c r="H2" s="260"/>
+      <c r="I2" s="260"/>
     </row>
     <row r="3" spans="2:9" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40773,12 +40778,12 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="247" t="s">
+      <c r="C11" s="258" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="247"/>
-      <c r="E11" s="247"/>
-      <c r="F11" s="247"/>
+      <c r="D11" s="258"/>
+      <c r="E11" s="258"/>
+      <c r="F11" s="258"/>
       <c r="G11" s="40" t="s">
         <v>29</v>
       </c>
@@ -40816,58 +40821,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="250"/>
-      <c r="C1" s="250"/>
-      <c r="D1" s="250"/>
-      <c r="E1" s="250"/>
-      <c r="F1" s="250"/>
+      <c r="B1" s="261"/>
+      <c r="C1" s="261"/>
+      <c r="D1" s="261"/>
+      <c r="E1" s="261"/>
+      <c r="F1" s="261"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="253" t="s">
+      <c r="B2" s="264" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="253"/>
-      <c r="D2" s="253"/>
-      <c r="E2" s="253"/>
-      <c r="F2" s="253"/>
+      <c r="C2" s="264"/>
+      <c r="D2" s="264"/>
+      <c r="E2" s="264"/>
+      <c r="F2" s="264"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="250"/>
-      <c r="C3" s="250"/>
-      <c r="D3" s="250"/>
-      <c r="E3" s="250"/>
-      <c r="F3" s="250"/>
+      <c r="B3" s="261"/>
+      <c r="C3" s="261"/>
+      <c r="D3" s="261"/>
+      <c r="E3" s="261"/>
+      <c r="F3" s="261"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="251" t="s">
+      <c r="B5" s="262" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="251" t="s">
+      <c r="C5" s="262" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="251" t="s">
+      <c r="D5" s="262" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="252" t="s">
+      <c r="E5" s="263" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="252" t="s">
+      <c r="F5" s="263" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="251"/>
-      <c r="C6" s="251"/>
-      <c r="D6" s="251"/>
-      <c r="E6" s="252"/>
-      <c r="F6" s="252"/>
+      <c r="B6" s="262"/>
+      <c r="C6" s="262"/>
+      <c r="D6" s="262"/>
+      <c r="E6" s="263"/>
+      <c r="F6" s="263"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="251"/>
-      <c r="C7" s="251"/>
-      <c r="D7" s="251"/>
-      <c r="E7" s="252"/>
-      <c r="F7" s="252"/>
+      <c r="B7" s="262"/>
+      <c r="C7" s="262"/>
+      <c r="D7" s="262"/>
+      <c r="E7" s="263"/>
+      <c r="F7" s="263"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -40988,45 +40993,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="148"/>
-      <c r="C1" s="149"/>
-      <c r="D1" s="149"/>
-      <c r="E1" s="149"/>
-      <c r="F1" s="149"/>
-      <c r="G1" s="149"/>
-      <c r="H1" s="149"/>
-      <c r="I1" s="149"/>
-      <c r="J1" s="149"/>
-      <c r="K1" s="149"/>
-      <c r="L1" s="150"/>
+      <c r="B1" s="232"/>
+      <c r="C1" s="233"/>
+      <c r="D1" s="233"/>
+      <c r="E1" s="233"/>
+      <c r="F1" s="233"/>
+      <c r="G1" s="233"/>
+      <c r="H1" s="233"/>
+      <c r="I1" s="233"/>
+      <c r="J1" s="233"/>
+      <c r="K1" s="233"/>
+      <c r="L1" s="234"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="151" t="s">
+      <c r="B2" s="235" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
-      <c r="E2" s="152"/>
-      <c r="F2" s="152"/>
-      <c r="G2" s="152"/>
-      <c r="H2" s="152"/>
-      <c r="I2" s="153"/>
-      <c r="J2" s="157"/>
-      <c r="K2" s="158"/>
-      <c r="L2" s="159"/>
+      <c r="C2" s="236"/>
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
+      <c r="F2" s="236"/>
+      <c r="G2" s="236"/>
+      <c r="H2" s="236"/>
+      <c r="I2" s="237"/>
+      <c r="J2" s="241"/>
+      <c r="K2" s="242"/>
+      <c r="L2" s="243"/>
     </row>
     <row r="3" spans="1:13" ht="14.4" customHeight="1">
-      <c r="B3" s="154"/>
-      <c r="C3" s="155"/>
-      <c r="D3" s="155"/>
-      <c r="E3" s="155"/>
-      <c r="F3" s="155"/>
-      <c r="G3" s="155"/>
-      <c r="H3" s="155"/>
-      <c r="I3" s="156"/>
-      <c r="J3" s="160"/>
-      <c r="K3" s="161"/>
-      <c r="L3" s="162"/>
+      <c r="B3" s="238"/>
+      <c r="C3" s="239"/>
+      <c r="D3" s="239"/>
+      <c r="E3" s="239"/>
+      <c r="F3" s="239"/>
+      <c r="G3" s="239"/>
+      <c r="H3" s="239"/>
+      <c r="I3" s="240"/>
+      <c r="J3" s="244"/>
+      <c r="K3" s="245"/>
+      <c r="L3" s="246"/>
     </row>
     <row r="4" spans="1:13" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -41037,9 +41042,9 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="160"/>
-      <c r="K4" s="161"/>
-      <c r="L4" s="162"/>
+      <c r="J4" s="244"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="246"/>
     </row>
     <row r="5" spans="1:13" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -41054,9 +41059,9 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="160"/>
-      <c r="K5" s="161"/>
-      <c r="L5" s="162"/>
+      <c r="J5" s="244"/>
+      <c r="K5" s="245"/>
+      <c r="L5" s="246"/>
     </row>
     <row r="6" spans="1:13" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -41071,9 +41076,9 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="163"/>
-      <c r="K6" s="164"/>
-      <c r="L6" s="165"/>
+      <c r="J6" s="247"/>
+      <c r="K6" s="248"/>
+      <c r="L6" s="249"/>
     </row>
     <row r="7" spans="1:13" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -41125,45 +41130,45 @@
       <c r="J9" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="K9" s="124"/>
+      <c r="K9" s="114"/>
       <c r="L9" s="89"/>
     </row>
     <row r="10" spans="1:13" ht="15.6">
-      <c r="B10" s="166" t="s">
+      <c r="B10" s="250" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="167"/>
-      <c r="D10" s="167"/>
-      <c r="E10" s="167"/>
-      <c r="F10" s="168"/>
-      <c r="G10" s="167" t="s">
+      <c r="C10" s="251"/>
+      <c r="D10" s="251"/>
+      <c r="E10" s="251"/>
+      <c r="F10" s="252"/>
+      <c r="G10" s="251" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="167"/>
-      <c r="I10" s="167"/>
-      <c r="J10" s="168"/>
-      <c r="K10" s="167" t="s">
+      <c r="H10" s="251"/>
+      <c r="I10" s="251"/>
+      <c r="J10" s="252"/>
+      <c r="K10" s="251" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="169"/>
+      <c r="L10" s="253"/>
     </row>
     <row r="11" spans="1:13" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="185" t="s">
+      <c r="C11" s="200" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="186"/>
-      <c r="E11" s="186"/>
+      <c r="D11" s="201"/>
+      <c r="E11" s="201"/>
       <c r="F11" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="185" t="s">
+      <c r="G11" s="200" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="187"/>
+      <c r="H11" s="202"/>
       <c r="I11" s="92" t="s">
         <v>27</v>
       </c>
@@ -41182,939 +41187,939 @@
       <c r="B12" s="94" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="231" t="s">
+      <c r="C12" s="160" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="232"/>
-      <c r="E12" s="233"/>
-      <c r="F12" s="95"/>
-      <c r="G12" s="194"/>
-      <c r="H12" s="195"/>
-      <c r="I12" s="96"/>
-      <c r="J12" s="96"/>
-      <c r="K12" s="97"/>
-      <c r="L12" s="98"/>
+      <c r="D12" s="161"/>
+      <c r="E12" s="162"/>
+      <c r="F12" s="299"/>
+      <c r="G12" s="209"/>
+      <c r="H12" s="210"/>
+      <c r="I12" s="297"/>
+      <c r="J12" s="304"/>
+      <c r="K12" s="305"/>
+      <c r="L12" s="301"/>
     </row>
     <row r="13" spans="1:13" ht="15.6">
-      <c r="B13" s="99">
+      <c r="B13" s="95">
         <v>1</v>
       </c>
-      <c r="C13" s="234" t="s">
+      <c r="C13" s="154" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="235"/>
-      <c r="E13" s="236"/>
-      <c r="F13" s="100"/>
-      <c r="G13" s="196"/>
-      <c r="H13" s="197"/>
-      <c r="I13" s="101"/>
-      <c r="J13" s="102"/>
-      <c r="K13" s="103"/>
-      <c r="L13" s="104"/>
+      <c r="D13" s="155"/>
+      <c r="E13" s="156"/>
+      <c r="F13" s="300"/>
+      <c r="G13" s="211"/>
+      <c r="H13" s="212"/>
+      <c r="I13" s="298"/>
+      <c r="J13" s="306"/>
+      <c r="K13" s="307"/>
+      <c r="L13" s="302"/>
     </row>
     <row r="14" spans="1:13" ht="15.6">
-      <c r="B14" s="99">
+      <c r="B14" s="95">
         <v>2</v>
       </c>
-      <c r="C14" s="234" t="s">
+      <c r="C14" s="154" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="235"/>
-      <c r="E14" s="236"/>
-      <c r="F14" s="100"/>
-      <c r="G14" s="196"/>
-      <c r="H14" s="197"/>
-      <c r="I14" s="101"/>
-      <c r="J14" s="102"/>
-      <c r="K14" s="103"/>
-      <c r="L14" s="104"/>
+      <c r="D14" s="155"/>
+      <c r="E14" s="156"/>
+      <c r="F14" s="300"/>
+      <c r="G14" s="211"/>
+      <c r="H14" s="212"/>
+      <c r="I14" s="298"/>
+      <c r="J14" s="306"/>
+      <c r="K14" s="307"/>
+      <c r="L14" s="302"/>
     </row>
     <row r="15" spans="1:13" ht="15.6">
-      <c r="B15" s="99">
+      <c r="B15" s="95">
         <v>3</v>
       </c>
-      <c r="C15" s="234" t="s">
+      <c r="C15" s="154" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="235"/>
-      <c r="E15" s="236"/>
-      <c r="F15" s="100"/>
-      <c r="G15" s="196"/>
-      <c r="H15" s="197"/>
-      <c r="I15" s="101"/>
-      <c r="J15" s="102"/>
-      <c r="K15" s="103"/>
-      <c r="L15" s="104"/>
+      <c r="D15" s="155"/>
+      <c r="E15" s="156"/>
+      <c r="F15" s="300"/>
+      <c r="G15" s="211"/>
+      <c r="H15" s="212"/>
+      <c r="I15" s="298"/>
+      <c r="J15" s="306"/>
+      <c r="K15" s="307"/>
+      <c r="L15" s="302"/>
     </row>
     <row r="16" spans="1:13" ht="15.6">
-      <c r="B16" s="99">
+      <c r="B16" s="95">
         <v>4</v>
       </c>
-      <c r="C16" s="234" t="s">
+      <c r="C16" s="154" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="235"/>
-      <c r="E16" s="236"/>
-      <c r="F16" s="100"/>
-      <c r="G16" s="196"/>
-      <c r="H16" s="197"/>
-      <c r="I16" s="101"/>
-      <c r="J16" s="102"/>
-      <c r="K16" s="103"/>
-      <c r="L16" s="104"/>
+      <c r="D16" s="155"/>
+      <c r="E16" s="156"/>
+      <c r="F16" s="300"/>
+      <c r="G16" s="211"/>
+      <c r="H16" s="212"/>
+      <c r="I16" s="298"/>
+      <c r="J16" s="306"/>
+      <c r="K16" s="307"/>
+      <c r="L16" s="302"/>
     </row>
     <row r="17" spans="1:12" ht="15.6">
-      <c r="B17" s="99">
+      <c r="B17" s="95">
         <v>5</v>
       </c>
-      <c r="C17" s="234" t="s">
+      <c r="C17" s="154" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="235"/>
-      <c r="E17" s="236"/>
-      <c r="F17" s="100"/>
-      <c r="G17" s="196"/>
-      <c r="H17" s="197"/>
-      <c r="I17" s="101"/>
-      <c r="J17" s="102"/>
-      <c r="K17" s="103"/>
-      <c r="L17" s="104"/>
+      <c r="D17" s="155"/>
+      <c r="E17" s="156"/>
+      <c r="F17" s="300"/>
+      <c r="G17" s="211"/>
+      <c r="H17" s="212"/>
+      <c r="I17" s="298"/>
+      <c r="J17" s="306"/>
+      <c r="K17" s="307"/>
+      <c r="L17" s="302"/>
     </row>
     <row r="18" spans="1:12" ht="15.6">
-      <c r="B18" s="99">
+      <c r="B18" s="95">
         <v>6</v>
       </c>
-      <c r="C18" s="234" t="s">
+      <c r="C18" s="154" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="235"/>
-      <c r="E18" s="236"/>
-      <c r="F18" s="100"/>
-      <c r="G18" s="196"/>
-      <c r="H18" s="197"/>
-      <c r="I18" s="101"/>
-      <c r="J18" s="102"/>
-      <c r="K18" s="103"/>
-      <c r="L18" s="104"/>
+      <c r="D18" s="155"/>
+      <c r="E18" s="156"/>
+      <c r="F18" s="300"/>
+      <c r="G18" s="211"/>
+      <c r="H18" s="212"/>
+      <c r="I18" s="298"/>
+      <c r="J18" s="306"/>
+      <c r="K18" s="307"/>
+      <c r="L18" s="302"/>
     </row>
     <row r="19" spans="1:12" ht="15.6">
-      <c r="B19" s="105" t="s">
+      <c r="B19" s="97" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="237" t="s">
+      <c r="C19" s="157" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="238"/>
-      <c r="E19" s="239"/>
-      <c r="F19" s="100"/>
-      <c r="G19" s="196"/>
-      <c r="H19" s="197"/>
-      <c r="I19" s="101"/>
-      <c r="J19" s="102"/>
-      <c r="K19" s="103"/>
-      <c r="L19" s="104"/>
+      <c r="D19" s="158"/>
+      <c r="E19" s="159"/>
+      <c r="F19" s="300"/>
+      <c r="G19" s="211"/>
+      <c r="H19" s="212"/>
+      <c r="I19" s="298"/>
+      <c r="J19" s="306"/>
+      <c r="K19" s="307"/>
+      <c r="L19" s="302"/>
     </row>
     <row r="20" spans="1:12" ht="15.6">
-      <c r="B20" s="99">
+      <c r="B20" s="95">
         <v>1</v>
       </c>
-      <c r="C20" s="234" t="s">
+      <c r="C20" s="154" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="235"/>
-      <c r="E20" s="236"/>
-      <c r="F20" s="100"/>
-      <c r="G20" s="196"/>
-      <c r="H20" s="197"/>
-      <c r="I20" s="101"/>
-      <c r="J20" s="102"/>
-      <c r="K20" s="103"/>
-      <c r="L20" s="104"/>
+      <c r="D20" s="155"/>
+      <c r="E20" s="156"/>
+      <c r="F20" s="300"/>
+      <c r="G20" s="211"/>
+      <c r="H20" s="212"/>
+      <c r="I20" s="298"/>
+      <c r="J20" s="306"/>
+      <c r="K20" s="307"/>
+      <c r="L20" s="302"/>
     </row>
     <row r="21" spans="1:12" ht="15.6">
-      <c r="B21" s="99">
+      <c r="B21" s="95">
         <v>2</v>
       </c>
-      <c r="C21" s="234" t="s">
+      <c r="C21" s="154" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="235"/>
-      <c r="E21" s="236"/>
-      <c r="F21" s="100"/>
-      <c r="G21" s="196"/>
-      <c r="H21" s="197"/>
-      <c r="I21" s="101"/>
-      <c r="J21" s="102"/>
-      <c r="K21" s="103"/>
-      <c r="L21" s="104"/>
+      <c r="D21" s="155"/>
+      <c r="E21" s="156"/>
+      <c r="F21" s="300"/>
+      <c r="G21" s="211"/>
+      <c r="H21" s="212"/>
+      <c r="I21" s="298"/>
+      <c r="J21" s="306"/>
+      <c r="K21" s="307"/>
+      <c r="L21" s="302"/>
     </row>
     <row r="22" spans="1:12" ht="15.6">
-      <c r="B22" s="99">
+      <c r="B22" s="95">
         <v>3</v>
       </c>
-      <c r="C22" s="240" t="s">
+      <c r="C22" s="149" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="241"/>
-      <c r="E22" s="242"/>
-      <c r="F22" s="100"/>
-      <c r="G22" s="198"/>
-      <c r="H22" s="199"/>
-      <c r="I22" s="101"/>
-      <c r="J22" s="102"/>
-      <c r="K22" s="106"/>
-      <c r="L22" s="107"/>
+      <c r="D22" s="150"/>
+      <c r="E22" s="151"/>
+      <c r="F22" s="300"/>
+      <c r="G22" s="213"/>
+      <c r="H22" s="214"/>
+      <c r="I22" s="298"/>
+      <c r="J22" s="306"/>
+      <c r="K22" s="308"/>
+      <c r="L22" s="303"/>
     </row>
     <row r="23" spans="1:12" ht="16.2" thickBot="1">
-      <c r="B23" s="188"/>
-      <c r="C23" s="189"/>
-      <c r="D23" s="189"/>
-      <c r="E23" s="189"/>
-      <c r="F23" s="108"/>
-      <c r="G23" s="108"/>
-      <c r="H23" s="109"/>
-      <c r="I23" s="109"/>
-      <c r="J23" s="190"/>
-      <c r="K23" s="190"/>
-      <c r="L23" s="191"/>
+      <c r="B23" s="203"/>
+      <c r="C23" s="204"/>
+      <c r="D23" s="204"/>
+      <c r="E23" s="204"/>
+      <c r="F23" s="98"/>
+      <c r="G23" s="98"/>
+      <c r="H23" s="99"/>
+      <c r="I23" s="99"/>
+      <c r="J23" s="205"/>
+      <c r="K23" s="205"/>
+      <c r="L23" s="206"/>
     </row>
     <row r="24" spans="1:12" ht="16.2" customHeight="1" thickTop="1">
-      <c r="A24" s="123" t="s">
+      <c r="A24" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="192" t="s">
+      <c r="B24" s="207" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="170" t="s">
+      <c r="C24" s="215" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="170"/>
-      <c r="E24" s="170"/>
-      <c r="F24" s="170"/>
-      <c r="G24" s="170"/>
-      <c r="H24" s="170"/>
-      <c r="I24" s="170"/>
-      <c r="J24" s="172" t="s">
+      <c r="D24" s="215"/>
+      <c r="E24" s="215"/>
+      <c r="F24" s="215"/>
+      <c r="G24" s="215"/>
+      <c r="H24" s="215"/>
+      <c r="I24" s="215"/>
+      <c r="J24" s="217" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="173"/>
-      <c r="L24" s="174"/>
+      <c r="K24" s="218"/>
+      <c r="L24" s="219"/>
     </row>
     <row r="25" spans="1:12" ht="31.2">
-      <c r="B25" s="193"/>
-      <c r="C25" s="171"/>
-      <c r="D25" s="171"/>
-      <c r="E25" s="171"/>
-      <c r="F25" s="171"/>
-      <c r="G25" s="171"/>
-      <c r="H25" s="171"/>
-      <c r="I25" s="171"/>
-      <c r="J25" s="147" t="s">
+      <c r="B25" s="208"/>
+      <c r="C25" s="216"/>
+      <c r="D25" s="216"/>
+      <c r="E25" s="216"/>
+      <c r="F25" s="216"/>
+      <c r="G25" s="216"/>
+      <c r="H25" s="216"/>
+      <c r="I25" s="216"/>
+      <c r="J25" s="137" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="145" t="s">
+      <c r="K25" s="135" t="s">
         <v>76</v>
       </c>
-      <c r="L25" s="146" t="s">
+      <c r="L25" s="136" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.6">
-      <c r="B26" s="110"/>
-      <c r="C26" s="286"/>
-      <c r="D26" s="287"/>
-      <c r="E26" s="287"/>
-      <c r="F26" s="287"/>
-      <c r="G26" s="287"/>
-      <c r="H26" s="287"/>
-      <c r="I26" s="288"/>
-      <c r="J26" s="295"/>
-      <c r="K26" s="306"/>
-      <c r="L26" s="304"/>
+      <c r="B26" s="100"/>
+      <c r="C26" s="229"/>
+      <c r="D26" s="230"/>
+      <c r="E26" s="230"/>
+      <c r="F26" s="230"/>
+      <c r="G26" s="230"/>
+      <c r="H26" s="230"/>
+      <c r="I26" s="231"/>
+      <c r="J26" s="138"/>
+      <c r="K26" s="146"/>
+      <c r="L26" s="144"/>
     </row>
     <row r="27" spans="1:12" ht="15.6">
-      <c r="B27" s="110"/>
-      <c r="C27" s="289"/>
-      <c r="D27" s="290"/>
-      <c r="E27" s="290"/>
-      <c r="F27" s="290"/>
-      <c r="G27" s="290"/>
-      <c r="H27" s="290"/>
-      <c r="I27" s="291"/>
-      <c r="J27" s="102"/>
-      <c r="K27" s="307"/>
-      <c r="L27" s="304"/>
+      <c r="B27" s="100"/>
+      <c r="C27" s="163"/>
+      <c r="D27" s="164"/>
+      <c r="E27" s="164"/>
+      <c r="F27" s="164"/>
+      <c r="G27" s="164"/>
+      <c r="H27" s="164"/>
+      <c r="I27" s="165"/>
+      <c r="J27" s="96"/>
+      <c r="K27" s="147"/>
+      <c r="L27" s="144"/>
     </row>
     <row r="28" spans="1:12" ht="15.6">
-      <c r="B28" s="110"/>
-      <c r="C28" s="289"/>
-      <c r="D28" s="290"/>
-      <c r="E28" s="290"/>
-      <c r="F28" s="290"/>
-      <c r="G28" s="290"/>
-      <c r="H28" s="290"/>
-      <c r="I28" s="291"/>
-      <c r="J28" s="102"/>
-      <c r="K28" s="307"/>
-      <c r="L28" s="305"/>
+      <c r="B28" s="100"/>
+      <c r="C28" s="163"/>
+      <c r="D28" s="164"/>
+      <c r="E28" s="164"/>
+      <c r="F28" s="164"/>
+      <c r="G28" s="164"/>
+      <c r="H28" s="164"/>
+      <c r="I28" s="165"/>
+      <c r="J28" s="96"/>
+      <c r="K28" s="147"/>
+      <c r="L28" s="145"/>
     </row>
     <row r="29" spans="1:12" ht="15.6">
-      <c r="B29" s="110"/>
-      <c r="C29" s="289"/>
-      <c r="D29" s="290"/>
-      <c r="E29" s="290"/>
-      <c r="F29" s="290"/>
-      <c r="G29" s="290"/>
-      <c r="H29" s="290"/>
-      <c r="I29" s="291"/>
-      <c r="J29" s="102"/>
-      <c r="K29" s="307"/>
-      <c r="L29" s="305"/>
+      <c r="B29" s="100"/>
+      <c r="C29" s="163"/>
+      <c r="D29" s="164"/>
+      <c r="E29" s="164"/>
+      <c r="F29" s="164"/>
+      <c r="G29" s="164"/>
+      <c r="H29" s="164"/>
+      <c r="I29" s="165"/>
+      <c r="J29" s="96"/>
+      <c r="K29" s="147"/>
+      <c r="L29" s="145"/>
     </row>
     <row r="30" spans="1:12" ht="15.6">
-      <c r="B30" s="110" t="s">
+      <c r="B30" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="289" t="s">
+      <c r="C30" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="290"/>
-      <c r="E30" s="290"/>
-      <c r="F30" s="290"/>
-      <c r="G30" s="290"/>
-      <c r="H30" s="290"/>
-      <c r="I30" s="291"/>
-      <c r="J30" s="102" t="s">
+      <c r="D30" s="164"/>
+      <c r="E30" s="164"/>
+      <c r="F30" s="164"/>
+      <c r="G30" s="164"/>
+      <c r="H30" s="164"/>
+      <c r="I30" s="165"/>
+      <c r="J30" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K30" s="307"/>
-      <c r="L30" s="305" t="s">
+      <c r="K30" s="147"/>
+      <c r="L30" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="15.6">
-      <c r="B31" s="110" t="s">
+      <c r="B31" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="289" t="s">
+      <c r="C31" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="290"/>
-      <c r="E31" s="290"/>
-      <c r="F31" s="290"/>
-      <c r="G31" s="290"/>
-      <c r="H31" s="290"/>
-      <c r="I31" s="291"/>
-      <c r="J31" s="102" t="s">
+      <c r="D31" s="164"/>
+      <c r="E31" s="164"/>
+      <c r="F31" s="164"/>
+      <c r="G31" s="164"/>
+      <c r="H31" s="164"/>
+      <c r="I31" s="165"/>
+      <c r="J31" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K31" s="307"/>
-      <c r="L31" s="305" t="s">
+      <c r="K31" s="147"/>
+      <c r="L31" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="15.6">
-      <c r="B32" s="110" t="s">
+      <c r="B32" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="289" t="s">
+      <c r="C32" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="290"/>
-      <c r="E32" s="290"/>
-      <c r="F32" s="290"/>
-      <c r="G32" s="290"/>
-      <c r="H32" s="290"/>
-      <c r="I32" s="291"/>
-      <c r="J32" s="102" t="s">
+      <c r="D32" s="164"/>
+      <c r="E32" s="164"/>
+      <c r="F32" s="164"/>
+      <c r="G32" s="164"/>
+      <c r="H32" s="164"/>
+      <c r="I32" s="165"/>
+      <c r="J32" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K32" s="307"/>
-      <c r="L32" s="305" t="s">
+      <c r="K32" s="147"/>
+      <c r="L32" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="33" spans="2:12" ht="15.6">
-      <c r="B33" s="110" t="s">
+      <c r="B33" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="289" t="s">
+      <c r="C33" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="290"/>
-      <c r="E33" s="290"/>
-      <c r="F33" s="290"/>
-      <c r="G33" s="290"/>
-      <c r="H33" s="290"/>
-      <c r="I33" s="291"/>
-      <c r="J33" s="102" t="s">
+      <c r="D33" s="164"/>
+      <c r="E33" s="164"/>
+      <c r="F33" s="164"/>
+      <c r="G33" s="164"/>
+      <c r="H33" s="164"/>
+      <c r="I33" s="165"/>
+      <c r="J33" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K33" s="307"/>
-      <c r="L33" s="305" t="s">
+      <c r="K33" s="147"/>
+      <c r="L33" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="34" spans="2:12" ht="15.6">
-      <c r="B34" s="110" t="s">
+      <c r="B34" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="289" t="s">
+      <c r="C34" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="290"/>
-      <c r="E34" s="290"/>
-      <c r="F34" s="290"/>
-      <c r="G34" s="290"/>
-      <c r="H34" s="290"/>
-      <c r="I34" s="291"/>
-      <c r="J34" s="102" t="s">
+      <c r="D34" s="164"/>
+      <c r="E34" s="164"/>
+      <c r="F34" s="164"/>
+      <c r="G34" s="164"/>
+      <c r="H34" s="164"/>
+      <c r="I34" s="165"/>
+      <c r="J34" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K34" s="307"/>
-      <c r="L34" s="305" t="s">
+      <c r="K34" s="147"/>
+      <c r="L34" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="35" spans="2:12" ht="15.6">
-      <c r="B35" s="110" t="s">
+      <c r="B35" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="289" t="s">
+      <c r="C35" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="290"/>
-      <c r="E35" s="290"/>
-      <c r="F35" s="290"/>
-      <c r="G35" s="290"/>
-      <c r="H35" s="290"/>
-      <c r="I35" s="291"/>
-      <c r="J35" s="102" t="s">
+      <c r="D35" s="164"/>
+      <c r="E35" s="164"/>
+      <c r="F35" s="164"/>
+      <c r="G35" s="164"/>
+      <c r="H35" s="164"/>
+      <c r="I35" s="165"/>
+      <c r="J35" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K35" s="307"/>
-      <c r="L35" s="305" t="s">
+      <c r="K35" s="147"/>
+      <c r="L35" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="36" spans="2:12" ht="15.6">
-      <c r="B36" s="110" t="s">
+      <c r="B36" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C36" s="289" t="s">
+      <c r="C36" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="290"/>
-      <c r="E36" s="290"/>
-      <c r="F36" s="290"/>
-      <c r="G36" s="290"/>
-      <c r="H36" s="290"/>
-      <c r="I36" s="291"/>
-      <c r="J36" s="102" t="s">
+      <c r="D36" s="164"/>
+      <c r="E36" s="164"/>
+      <c r="F36" s="164"/>
+      <c r="G36" s="164"/>
+      <c r="H36" s="164"/>
+      <c r="I36" s="165"/>
+      <c r="J36" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K36" s="307"/>
-      <c r="L36" s="305" t="s">
+      <c r="K36" s="147"/>
+      <c r="L36" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="37" spans="2:12" ht="15.6">
-      <c r="B37" s="110" t="s">
+      <c r="B37" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="289" t="s">
+      <c r="C37" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="290"/>
-      <c r="E37" s="290"/>
-      <c r="F37" s="290"/>
-      <c r="G37" s="290"/>
-      <c r="H37" s="290"/>
-      <c r="I37" s="291"/>
-      <c r="J37" s="102" t="s">
+      <c r="D37" s="164"/>
+      <c r="E37" s="164"/>
+      <c r="F37" s="164"/>
+      <c r="G37" s="164"/>
+      <c r="H37" s="164"/>
+      <c r="I37" s="165"/>
+      <c r="J37" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K37" s="307"/>
-      <c r="L37" s="305" t="s">
+      <c r="K37" s="147"/>
+      <c r="L37" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="38" spans="2:12" ht="15.6">
-      <c r="B38" s="110" t="s">
+      <c r="B38" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="289" t="s">
+      <c r="C38" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="290"/>
-      <c r="E38" s="290"/>
-      <c r="F38" s="290"/>
-      <c r="G38" s="290"/>
-      <c r="H38" s="290"/>
-      <c r="I38" s="291"/>
-      <c r="J38" s="102" t="s">
+      <c r="D38" s="164"/>
+      <c r="E38" s="164"/>
+      <c r="F38" s="164"/>
+      <c r="G38" s="164"/>
+      <c r="H38" s="164"/>
+      <c r="I38" s="165"/>
+      <c r="J38" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K38" s="307"/>
-      <c r="L38" s="305" t="s">
+      <c r="K38" s="147"/>
+      <c r="L38" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="39" spans="2:12" ht="15.6">
-      <c r="B39" s="110" t="s">
+      <c r="B39" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="289" t="s">
+      <c r="C39" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D39" s="290"/>
-      <c r="E39" s="290"/>
-      <c r="F39" s="290"/>
-      <c r="G39" s="290"/>
-      <c r="H39" s="290"/>
-      <c r="I39" s="291"/>
-      <c r="J39" s="102" t="s">
+      <c r="D39" s="164"/>
+      <c r="E39" s="164"/>
+      <c r="F39" s="164"/>
+      <c r="G39" s="164"/>
+      <c r="H39" s="164"/>
+      <c r="I39" s="165"/>
+      <c r="J39" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K39" s="307"/>
-      <c r="L39" s="305" t="s">
+      <c r="K39" s="147"/>
+      <c r="L39" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="40" spans="2:12" ht="15.6">
-      <c r="B40" s="110" t="s">
+      <c r="B40" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="289" t="s">
+      <c r="C40" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D40" s="290"/>
-      <c r="E40" s="290"/>
-      <c r="F40" s="290"/>
-      <c r="G40" s="290"/>
-      <c r="H40" s="290"/>
-      <c r="I40" s="291"/>
-      <c r="J40" s="102" t="s">
+      <c r="D40" s="164"/>
+      <c r="E40" s="164"/>
+      <c r="F40" s="164"/>
+      <c r="G40" s="164"/>
+      <c r="H40" s="164"/>
+      <c r="I40" s="165"/>
+      <c r="J40" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K40" s="307"/>
-      <c r="L40" s="305" t="s">
+      <c r="K40" s="147"/>
+      <c r="L40" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="41" spans="2:12" ht="15.6">
-      <c r="B41" s="110" t="s">
+      <c r="B41" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="289" t="s">
+      <c r="C41" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D41" s="290"/>
-      <c r="E41" s="290"/>
-      <c r="F41" s="290"/>
-      <c r="G41" s="290"/>
-      <c r="H41" s="290"/>
-      <c r="I41" s="291"/>
-      <c r="J41" s="102" t="s">
+      <c r="D41" s="164"/>
+      <c r="E41" s="164"/>
+      <c r="F41" s="164"/>
+      <c r="G41" s="164"/>
+      <c r="H41" s="164"/>
+      <c r="I41" s="165"/>
+      <c r="J41" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K41" s="307"/>
-      <c r="L41" s="305" t="s">
+      <c r="K41" s="147"/>
+      <c r="L41" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="42" spans="2:12" ht="15.6">
-      <c r="B42" s="110" t="s">
+      <c r="B42" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="289" t="s">
+      <c r="C42" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="290"/>
-      <c r="E42" s="290"/>
-      <c r="F42" s="290"/>
-      <c r="G42" s="290"/>
-      <c r="H42" s="290"/>
-      <c r="I42" s="291"/>
-      <c r="J42" s="102" t="s">
+      <c r="D42" s="164"/>
+      <c r="E42" s="164"/>
+      <c r="F42" s="164"/>
+      <c r="G42" s="164"/>
+      <c r="H42" s="164"/>
+      <c r="I42" s="165"/>
+      <c r="J42" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K42" s="307"/>
-      <c r="L42" s="305" t="s">
+      <c r="K42" s="147"/>
+      <c r="L42" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="43" spans="2:12" ht="15.6">
-      <c r="B43" s="110" t="s">
+      <c r="B43" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="289" t="s">
+      <c r="C43" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="290"/>
-      <c r="E43" s="290"/>
-      <c r="F43" s="290"/>
-      <c r="G43" s="290"/>
-      <c r="H43" s="290"/>
-      <c r="I43" s="291"/>
-      <c r="J43" s="102" t="s">
+      <c r="D43" s="164"/>
+      <c r="E43" s="164"/>
+      <c r="F43" s="164"/>
+      <c r="G43" s="164"/>
+      <c r="H43" s="164"/>
+      <c r="I43" s="165"/>
+      <c r="J43" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K43" s="307"/>
-      <c r="L43" s="305" t="s">
+      <c r="K43" s="147"/>
+      <c r="L43" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="44" spans="2:12" ht="15.6">
-      <c r="B44" s="110" t="s">
+      <c r="B44" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="289" t="s">
+      <c r="C44" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D44" s="290"/>
-      <c r="E44" s="290"/>
-      <c r="F44" s="290"/>
-      <c r="G44" s="290"/>
-      <c r="H44" s="290"/>
-      <c r="I44" s="291"/>
-      <c r="J44" s="102" t="s">
+      <c r="D44" s="164"/>
+      <c r="E44" s="164"/>
+      <c r="F44" s="164"/>
+      <c r="G44" s="164"/>
+      <c r="H44" s="164"/>
+      <c r="I44" s="165"/>
+      <c r="J44" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K44" s="307"/>
-      <c r="L44" s="305" t="s">
+      <c r="K44" s="147"/>
+      <c r="L44" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="45" spans="2:12" ht="15.6">
-      <c r="B45" s="110" t="s">
+      <c r="B45" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C45" s="289" t="s">
+      <c r="C45" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D45" s="290"/>
-      <c r="E45" s="290"/>
-      <c r="F45" s="290"/>
-      <c r="G45" s="290"/>
-      <c r="H45" s="290"/>
-      <c r="I45" s="291"/>
-      <c r="J45" s="102" t="s">
+      <c r="D45" s="164"/>
+      <c r="E45" s="164"/>
+      <c r="F45" s="164"/>
+      <c r="G45" s="164"/>
+      <c r="H45" s="164"/>
+      <c r="I45" s="165"/>
+      <c r="J45" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K45" s="307"/>
-      <c r="L45" s="305" t="s">
+      <c r="K45" s="147"/>
+      <c r="L45" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="46" spans="2:12" ht="15.6">
-      <c r="B46" s="110" t="s">
+      <c r="B46" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C46" s="289" t="s">
+      <c r="C46" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="290"/>
-      <c r="E46" s="290"/>
-      <c r="F46" s="290"/>
-      <c r="G46" s="290"/>
-      <c r="H46" s="290"/>
-      <c r="I46" s="291"/>
-      <c r="J46" s="102" t="s">
+      <c r="D46" s="164"/>
+      <c r="E46" s="164"/>
+      <c r="F46" s="164"/>
+      <c r="G46" s="164"/>
+      <c r="H46" s="164"/>
+      <c r="I46" s="165"/>
+      <c r="J46" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K46" s="307"/>
-      <c r="L46" s="305" t="s">
+      <c r="K46" s="147"/>
+      <c r="L46" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="47" spans="2:12" ht="15.6">
-      <c r="B47" s="110" t="s">
+      <c r="B47" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="289" t="s">
+      <c r="C47" s="163" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="290"/>
-      <c r="E47" s="290"/>
-      <c r="F47" s="290"/>
-      <c r="G47" s="290"/>
-      <c r="H47" s="290"/>
-      <c r="I47" s="291"/>
-      <c r="J47" s="102" t="s">
+      <c r="D47" s="164"/>
+      <c r="E47" s="164"/>
+      <c r="F47" s="164"/>
+      <c r="G47" s="164"/>
+      <c r="H47" s="164"/>
+      <c r="I47" s="165"/>
+      <c r="J47" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="K47" s="307"/>
-      <c r="L47" s="305" t="s">
+      <c r="K47" s="147"/>
+      <c r="L47" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="48" spans="2:12" ht="16.2" thickBot="1">
-      <c r="B48" s="110" t="s">
+      <c r="B48" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C48" s="292" t="s">
+      <c r="C48" s="166" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="293"/>
-      <c r="E48" s="293"/>
-      <c r="F48" s="293"/>
-      <c r="G48" s="293"/>
-      <c r="H48" s="293"/>
-      <c r="I48" s="294"/>
-      <c r="J48" s="296" t="s">
+      <c r="D48" s="167"/>
+      <c r="E48" s="167"/>
+      <c r="F48" s="167"/>
+      <c r="G48" s="167"/>
+      <c r="H48" s="167"/>
+      <c r="I48" s="168"/>
+      <c r="J48" s="139" t="s">
         <v>64</v>
       </c>
-      <c r="K48" s="308"/>
-      <c r="L48" s="305" t="s">
+      <c r="K48" s="148"/>
+      <c r="L48" s="145" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="49" spans="2:12" ht="16.2" thickTop="1">
-      <c r="B49" s="213" t="s">
+      <c r="B49" s="182" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="214"/>
-      <c r="D49" s="214"/>
-      <c r="E49" s="214"/>
-      <c r="F49" s="214"/>
-      <c r="G49" s="214"/>
-      <c r="H49" s="214"/>
-      <c r="I49" s="214"/>
-      <c r="J49" s="215"/>
-      <c r="K49" s="183" t="s">
+      <c r="C49" s="183"/>
+      <c r="D49" s="183"/>
+      <c r="E49" s="183"/>
+      <c r="F49" s="183"/>
+      <c r="G49" s="183"/>
+      <c r="H49" s="183"/>
+      <c r="I49" s="183"/>
+      <c r="J49" s="184"/>
+      <c r="K49" s="227" t="s">
         <v>79</v>
       </c>
-      <c r="L49" s="184"/>
+      <c r="L49" s="228"/>
     </row>
     <row r="50" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B50" s="216"/>
-      <c r="C50" s="217"/>
-      <c r="D50" s="217"/>
-      <c r="E50" s="217"/>
-      <c r="F50" s="217"/>
-      <c r="G50" s="217"/>
-      <c r="H50" s="217"/>
-      <c r="I50" s="217"/>
-      <c r="J50" s="218"/>
-      <c r="K50" s="181" t="s">
+      <c r="B50" s="185"/>
+      <c r="C50" s="186"/>
+      <c r="D50" s="186"/>
+      <c r="E50" s="186"/>
+      <c r="F50" s="186"/>
+      <c r="G50" s="186"/>
+      <c r="H50" s="186"/>
+      <c r="I50" s="186"/>
+      <c r="J50" s="187"/>
+      <c r="K50" s="225" t="s">
         <v>103</v>
       </c>
-      <c r="L50" s="182"/>
+      <c r="L50" s="226"/>
     </row>
     <row r="51" spans="2:12" ht="15.6">
-      <c r="B51" s="111"/>
-      <c r="C51" s="178"/>
-      <c r="D51" s="178"/>
-      <c r="E51" s="178"/>
-      <c r="F51" s="178"/>
-      <c r="G51" s="178"/>
-      <c r="H51" s="178"/>
-      <c r="I51" s="178"/>
-      <c r="J51" s="112"/>
-      <c r="K51" s="176"/>
-      <c r="L51" s="177"/>
+      <c r="B51" s="101"/>
+      <c r="C51" s="222"/>
+      <c r="D51" s="222"/>
+      <c r="E51" s="222"/>
+      <c r="F51" s="222"/>
+      <c r="G51" s="222"/>
+      <c r="H51" s="222"/>
+      <c r="I51" s="222"/>
+      <c r="J51" s="102"/>
+      <c r="K51" s="220"/>
+      <c r="L51" s="221"/>
     </row>
     <row r="52" spans="2:12" ht="15.6">
-      <c r="B52" s="113"/>
-      <c r="C52" s="179"/>
-      <c r="D52" s="179"/>
-      <c r="E52" s="179"/>
-      <c r="F52" s="179"/>
-      <c r="G52" s="179"/>
-      <c r="H52" s="179"/>
-      <c r="I52" s="179"/>
-      <c r="J52" s="114"/>
-      <c r="K52" s="125"/>
-      <c r="L52" s="115"/>
+      <c r="B52" s="103"/>
+      <c r="C52" s="223"/>
+      <c r="D52" s="223"/>
+      <c r="E52" s="223"/>
+      <c r="F52" s="223"/>
+      <c r="G52" s="223"/>
+      <c r="H52" s="223"/>
+      <c r="I52" s="223"/>
+      <c r="J52" s="104"/>
+      <c r="K52" s="115"/>
+      <c r="L52" s="105"/>
     </row>
     <row r="53" spans="2:12" ht="15.6">
-      <c r="B53" s="116"/>
-      <c r="C53" s="179"/>
-      <c r="D53" s="179"/>
-      <c r="E53" s="179"/>
-      <c r="F53" s="179"/>
-      <c r="G53" s="179"/>
-      <c r="H53" s="179"/>
-      <c r="I53" s="179"/>
-      <c r="J53" s="117"/>
-      <c r="K53" s="118"/>
-      <c r="L53" s="119"/>
+      <c r="B53" s="106"/>
+      <c r="C53" s="223"/>
+      <c r="D53" s="223"/>
+      <c r="E53" s="223"/>
+      <c r="F53" s="223"/>
+      <c r="G53" s="223"/>
+      <c r="H53" s="223"/>
+      <c r="I53" s="223"/>
+      <c r="J53" s="107"/>
+      <c r="K53" s="108"/>
+      <c r="L53" s="109"/>
     </row>
     <row r="54" spans="2:12" ht="15.6">
-      <c r="B54" s="116"/>
-      <c r="C54" s="179"/>
-      <c r="D54" s="179"/>
-      <c r="E54" s="179"/>
-      <c r="F54" s="179"/>
-      <c r="G54" s="179"/>
-      <c r="H54" s="179"/>
-      <c r="I54" s="179"/>
-      <c r="J54" s="117"/>
-      <c r="K54" s="297"/>
-      <c r="L54" s="298"/>
+      <c r="B54" s="106"/>
+      <c r="C54" s="223"/>
+      <c r="D54" s="223"/>
+      <c r="E54" s="223"/>
+      <c r="F54" s="223"/>
+      <c r="G54" s="223"/>
+      <c r="H54" s="223"/>
+      <c r="I54" s="223"/>
+      <c r="J54" s="107"/>
+      <c r="K54" s="140"/>
+      <c r="L54" s="141"/>
     </row>
     <row r="55" spans="2:12" ht="15.6">
-      <c r="B55" s="116"/>
-      <c r="C55" s="179"/>
-      <c r="D55" s="179"/>
-      <c r="E55" s="179"/>
-      <c r="F55" s="179"/>
-      <c r="G55" s="179"/>
-      <c r="H55" s="179"/>
-      <c r="I55" s="179"/>
-      <c r="J55" s="117"/>
-      <c r="K55" s="300"/>
-      <c r="L55" s="301"/>
+      <c r="B55" s="106"/>
+      <c r="C55" s="223"/>
+      <c r="D55" s="223"/>
+      <c r="E55" s="223"/>
+      <c r="F55" s="223"/>
+      <c r="G55" s="223"/>
+      <c r="H55" s="223"/>
+      <c r="I55" s="223"/>
+      <c r="J55" s="107"/>
+      <c r="K55" s="140"/>
+      <c r="L55" s="141"/>
     </row>
     <row r="56" spans="2:12" ht="15.6">
-      <c r="B56" s="116"/>
-      <c r="C56" s="179"/>
-      <c r="D56" s="179"/>
-      <c r="E56" s="179"/>
-      <c r="F56" s="179"/>
-      <c r="G56" s="179"/>
-      <c r="H56" s="179"/>
-      <c r="I56" s="179"/>
-      <c r="J56" s="117"/>
-      <c r="K56" s="302"/>
-      <c r="L56" s="303"/>
+      <c r="B56" s="106"/>
+      <c r="C56" s="223"/>
+      <c r="D56" s="223"/>
+      <c r="E56" s="223"/>
+      <c r="F56" s="223"/>
+      <c r="G56" s="223"/>
+      <c r="H56" s="223"/>
+      <c r="I56" s="223"/>
+      <c r="J56" s="107"/>
+      <c r="K56" s="142"/>
+      <c r="L56" s="143"/>
     </row>
     <row r="57" spans="2:12" ht="15.6">
-      <c r="B57" s="116"/>
-      <c r="C57" s="179"/>
-      <c r="D57" s="179"/>
-      <c r="E57" s="179"/>
-      <c r="F57" s="179"/>
-      <c r="G57" s="179"/>
-      <c r="H57" s="179"/>
-      <c r="I57" s="179"/>
-      <c r="J57" s="117"/>
-      <c r="K57" s="300"/>
-      <c r="L57" s="301"/>
+      <c r="B57" s="106"/>
+      <c r="C57" s="223"/>
+      <c r="D57" s="223"/>
+      <c r="E57" s="223"/>
+      <c r="F57" s="223"/>
+      <c r="G57" s="223"/>
+      <c r="H57" s="223"/>
+      <c r="I57" s="223"/>
+      <c r="J57" s="107"/>
+      <c r="K57" s="140"/>
+      <c r="L57" s="141"/>
     </row>
     <row r="58" spans="2:12" ht="15.6">
-      <c r="B58" s="116"/>
-      <c r="C58" s="180"/>
-      <c r="D58" s="180"/>
-      <c r="E58" s="180"/>
-      <c r="F58" s="180"/>
-      <c r="G58" s="180"/>
-      <c r="H58" s="180"/>
-      <c r="I58" s="180"/>
-      <c r="J58" s="117"/>
-      <c r="K58" s="299"/>
-      <c r="L58" s="175"/>
+      <c r="B58" s="106"/>
+      <c r="C58" s="224"/>
+      <c r="D58" s="224"/>
+      <c r="E58" s="224"/>
+      <c r="F58" s="224"/>
+      <c r="G58" s="224"/>
+      <c r="H58" s="224"/>
+      <c r="I58" s="224"/>
+      <c r="J58" s="107"/>
+      <c r="K58" s="152"/>
+      <c r="L58" s="153"/>
     </row>
     <row r="59" spans="2:12" ht="15.6">
-      <c r="B59" s="116"/>
-      <c r="C59" s="120"/>
-      <c r="D59" s="120"/>
-      <c r="E59" s="120"/>
-      <c r="F59" s="120"/>
-      <c r="G59" s="120"/>
-      <c r="H59" s="120"/>
-      <c r="I59" s="120"/>
-      <c r="J59" s="117"/>
-      <c r="K59" s="299"/>
-      <c r="L59" s="175"/>
+      <c r="B59" s="106"/>
+      <c r="C59" s="110"/>
+      <c r="D59" s="110"/>
+      <c r="E59" s="110"/>
+      <c r="F59" s="110"/>
+      <c r="G59" s="110"/>
+      <c r="H59" s="110"/>
+      <c r="I59" s="110"/>
+      <c r="J59" s="107"/>
+      <c r="K59" s="152"/>
+      <c r="L59" s="153"/>
     </row>
     <row r="60" spans="2:12" ht="15.6">
-      <c r="B60" s="200" t="s">
+      <c r="B60" s="169" t="s">
         <v>80</v>
       </c>
-      <c r="C60" s="201"/>
-      <c r="D60" s="201"/>
-      <c r="E60" s="202"/>
-      <c r="F60" s="203" t="s">
+      <c r="C60" s="170"/>
+      <c r="D60" s="170"/>
+      <c r="E60" s="171"/>
+      <c r="F60" s="172" t="s">
         <v>81</v>
       </c>
-      <c r="G60" s="202"/>
-      <c r="H60" s="203" t="s">
+      <c r="G60" s="171"/>
+      <c r="H60" s="172" t="s">
         <v>82</v>
       </c>
-      <c r="I60" s="201"/>
-      <c r="J60" s="202"/>
-      <c r="K60" s="118"/>
-      <c r="L60" s="119"/>
+      <c r="I60" s="170"/>
+      <c r="J60" s="171"/>
+      <c r="K60" s="108"/>
+      <c r="L60" s="109"/>
     </row>
     <row r="61" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B61" s="225"/>
-      <c r="C61" s="226"/>
-      <c r="D61" s="226"/>
-      <c r="E61" s="220"/>
-      <c r="F61" s="219"/>
-      <c r="G61" s="220"/>
-      <c r="H61" s="204"/>
-      <c r="I61" s="205"/>
-      <c r="J61" s="206"/>
-      <c r="K61" s="118"/>
-      <c r="L61" s="119"/>
+      <c r="B61" s="194"/>
+      <c r="C61" s="195"/>
+      <c r="D61" s="195"/>
+      <c r="E61" s="189"/>
+      <c r="F61" s="188"/>
+      <c r="G61" s="189"/>
+      <c r="H61" s="173"/>
+      <c r="I61" s="174"/>
+      <c r="J61" s="175"/>
+      <c r="K61" s="108"/>
+      <c r="L61" s="109"/>
     </row>
     <row r="62" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B62" s="227"/>
-      <c r="C62" s="228"/>
-      <c r="D62" s="228"/>
-      <c r="E62" s="222"/>
-      <c r="F62" s="221"/>
-      <c r="G62" s="222"/>
-      <c r="H62" s="207"/>
-      <c r="I62" s="208"/>
-      <c r="J62" s="209"/>
-      <c r="K62" s="127"/>
-      <c r="L62" s="119"/>
+      <c r="B62" s="196"/>
+      <c r="C62" s="197"/>
+      <c r="D62" s="197"/>
+      <c r="E62" s="191"/>
+      <c r="F62" s="190"/>
+      <c r="G62" s="191"/>
+      <c r="H62" s="176"/>
+      <c r="I62" s="177"/>
+      <c r="J62" s="178"/>
+      <c r="K62" s="117"/>
+      <c r="L62" s="109"/>
     </row>
     <row r="63" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B63" s="227"/>
-      <c r="C63" s="228"/>
-      <c r="D63" s="228"/>
-      <c r="E63" s="222"/>
-      <c r="F63" s="221"/>
-      <c r="G63" s="222"/>
-      <c r="H63" s="207"/>
-      <c r="I63" s="208"/>
-      <c r="J63" s="209"/>
-      <c r="K63" s="126"/>
+      <c r="B63" s="196"/>
+      <c r="C63" s="197"/>
+      <c r="D63" s="197"/>
+      <c r="E63" s="191"/>
+      <c r="F63" s="190"/>
+      <c r="G63" s="191"/>
+      <c r="H63" s="176"/>
+      <c r="I63" s="177"/>
+      <c r="J63" s="178"/>
+      <c r="K63" s="116"/>
       <c r="L63" s="76"/>
     </row>
     <row r="64" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B64" s="227"/>
-      <c r="C64" s="228"/>
-      <c r="D64" s="228"/>
-      <c r="E64" s="222"/>
-      <c r="F64" s="221"/>
-      <c r="G64" s="222"/>
-      <c r="H64" s="207"/>
-      <c r="I64" s="208"/>
-      <c r="J64" s="209"/>
-      <c r="K64" s="128"/>
-      <c r="L64" s="129"/>
+      <c r="B64" s="196"/>
+      <c r="C64" s="197"/>
+      <c r="D64" s="197"/>
+      <c r="E64" s="191"/>
+      <c r="F64" s="190"/>
+      <c r="G64" s="191"/>
+      <c r="H64" s="176"/>
+      <c r="I64" s="177"/>
+      <c r="J64" s="178"/>
+      <c r="K64" s="118"/>
+      <c r="L64" s="119"/>
     </row>
     <row r="65" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B65" s="227"/>
-      <c r="C65" s="228"/>
-      <c r="D65" s="228"/>
-      <c r="E65" s="222"/>
-      <c r="F65" s="221"/>
-      <c r="G65" s="222"/>
-      <c r="H65" s="207"/>
-      <c r="I65" s="208"/>
-      <c r="J65" s="209"/>
-      <c r="K65" s="128"/>
-      <c r="L65" s="129"/>
+      <c r="B65" s="196"/>
+      <c r="C65" s="197"/>
+      <c r="D65" s="197"/>
+      <c r="E65" s="191"/>
+      <c r="F65" s="190"/>
+      <c r="G65" s="191"/>
+      <c r="H65" s="176"/>
+      <c r="I65" s="177"/>
+      <c r="J65" s="178"/>
+      <c r="K65" s="118"/>
+      <c r="L65" s="119"/>
     </row>
     <row r="66" spans="2:12" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B66" s="229"/>
-      <c r="C66" s="230"/>
-      <c r="D66" s="230"/>
-      <c r="E66" s="224"/>
-      <c r="F66" s="223"/>
-      <c r="G66" s="224"/>
-      <c r="H66" s="210"/>
-      <c r="I66" s="211"/>
-      <c r="J66" s="212"/>
-      <c r="K66" s="121"/>
-      <c r="L66" s="122"/>
+      <c r="B66" s="198"/>
+      <c r="C66" s="199"/>
+      <c r="D66" s="199"/>
+      <c r="E66" s="193"/>
+      <c r="F66" s="192"/>
+      <c r="G66" s="193"/>
+      <c r="H66" s="179"/>
+      <c r="I66" s="180"/>
+      <c r="J66" s="181"/>
+      <c r="K66" s="111"/>
+      <c r="L66" s="112"/>
     </row>
     <row r="67" spans="2:12" ht="15" thickTop="1">
       <c r="J67" s="61"/>
@@ -42123,40 +42128,27 @@
     </row>
   </sheetData>
   <mergeCells count="71">
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="K59:L59"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C44:I44"/>
-    <mergeCell ref="C45:I45"/>
-    <mergeCell ref="C46:I46"/>
-    <mergeCell ref="C47:I47"/>
-    <mergeCell ref="C48:I48"/>
-    <mergeCell ref="C39:I39"/>
-    <mergeCell ref="C40:I40"/>
-    <mergeCell ref="C41:I41"/>
-    <mergeCell ref="C42:I42"/>
-    <mergeCell ref="C43:I43"/>
-    <mergeCell ref="C34:I34"/>
-    <mergeCell ref="C35:I35"/>
-    <mergeCell ref="C36:I36"/>
-    <mergeCell ref="C37:I37"/>
-    <mergeCell ref="C38:I38"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="H60:J60"/>
-    <mergeCell ref="H61:J66"/>
-    <mergeCell ref="B49:J50"/>
-    <mergeCell ref="F61:G66"/>
-    <mergeCell ref="B61:E66"/>
+    <mergeCell ref="B1:L1"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="J2:L6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="C24:I25"/>
+    <mergeCell ref="J24:L24"/>
+    <mergeCell ref="K58:L58"/>
+    <mergeCell ref="K51:L51"/>
+    <mergeCell ref="C51:I58"/>
+    <mergeCell ref="K50:L50"/>
+    <mergeCell ref="K49:L49"/>
+    <mergeCell ref="C26:I26"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="C28:I28"/>
+    <mergeCell ref="C29:I29"/>
+    <mergeCell ref="C30:I30"/>
+    <mergeCell ref="C31:I31"/>
+    <mergeCell ref="C32:I32"/>
+    <mergeCell ref="C33:I33"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="B23:E23"/>
@@ -42173,27 +42165,40 @@
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="G22:H22"/>
-    <mergeCell ref="C24:I25"/>
-    <mergeCell ref="J24:L24"/>
-    <mergeCell ref="K58:L58"/>
-    <mergeCell ref="K51:L51"/>
-    <mergeCell ref="C51:I58"/>
-    <mergeCell ref="K50:L50"/>
-    <mergeCell ref="K49:L49"/>
-    <mergeCell ref="C26:I26"/>
-    <mergeCell ref="C27:I27"/>
-    <mergeCell ref="C28:I28"/>
-    <mergeCell ref="C29:I29"/>
-    <mergeCell ref="C30:I30"/>
-    <mergeCell ref="C31:I31"/>
-    <mergeCell ref="C32:I32"/>
-    <mergeCell ref="C33:I33"/>
-    <mergeCell ref="B1:L1"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="J2:L6"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="H60:J60"/>
+    <mergeCell ref="H61:J66"/>
+    <mergeCell ref="B49:J50"/>
+    <mergeCell ref="F61:G66"/>
+    <mergeCell ref="B61:E66"/>
+    <mergeCell ref="C43:I43"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="C36:I36"/>
+    <mergeCell ref="C37:I37"/>
+    <mergeCell ref="C38:I38"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="K59:L59"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C44:I44"/>
+    <mergeCell ref="C45:I45"/>
+    <mergeCell ref="C46:I46"/>
+    <mergeCell ref="C47:I47"/>
+    <mergeCell ref="C48:I48"/>
+    <mergeCell ref="C39:I39"/>
+    <mergeCell ref="C40:I40"/>
+    <mergeCell ref="C41:I41"/>
+    <mergeCell ref="C42:I42"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:L48">
     <cfRule type="expression" dxfId="2" priority="1">
@@ -42234,40 +42239,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="250"/>
-      <c r="C1" s="250"/>
-      <c r="D1" s="250"/>
-      <c r="E1" s="250"/>
-      <c r="F1" s="250"/>
-      <c r="G1" s="250"/>
-      <c r="H1" s="250"/>
-      <c r="I1" s="250"/>
-      <c r="J1" s="250"/>
-      <c r="K1" s="250"/>
-      <c r="L1" s="250"/>
-      <c r="M1" s="250"/>
-      <c r="N1" s="250"/>
-      <c r="O1" s="250"/>
-      <c r="P1" s="250"/>
+      <c r="B1" s="261"/>
+      <c r="C1" s="261"/>
+      <c r="D1" s="261"/>
+      <c r="E1" s="261"/>
+      <c r="F1" s="261"/>
+      <c r="G1" s="261"/>
+      <c r="H1" s="261"/>
+      <c r="I1" s="261"/>
+      <c r="J1" s="261"/>
+      <c r="K1" s="261"/>
+      <c r="L1" s="261"/>
+      <c r="M1" s="261"/>
+      <c r="N1" s="261"/>
+      <c r="O1" s="261"/>
+      <c r="P1" s="261"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="248" t="s">
+      <c r="B2" s="259" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="249"/>
-      <c r="D2" s="249"/>
-      <c r="E2" s="249"/>
-      <c r="F2" s="249"/>
-      <c r="G2" s="249"/>
-      <c r="H2" s="249"/>
-      <c r="I2" s="249"/>
-      <c r="J2" s="249"/>
-      <c r="K2" s="249"/>
-      <c r="L2" s="249"/>
-      <c r="M2" s="249"/>
-      <c r="N2" s="249"/>
-      <c r="O2" s="249"/>
-      <c r="P2" s="249"/>
+      <c r="C2" s="260"/>
+      <c r="D2" s="260"/>
+      <c r="E2" s="260"/>
+      <c r="F2" s="260"/>
+      <c r="G2" s="260"/>
+      <c r="H2" s="260"/>
+      <c r="I2" s="260"/>
+      <c r="J2" s="260"/>
+      <c r="K2" s="260"/>
+      <c r="L2" s="260"/>
+      <c r="M2" s="260"/>
+      <c r="N2" s="260"/>
+      <c r="O2" s="260"/>
+      <c r="P2" s="260"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -42294,16 +42299,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="256" t="s">
+      <c r="I4" s="267" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="256"/>
-      <c r="K4" s="256"/>
-      <c r="L4" s="256"/>
-      <c r="M4" s="256"/>
-      <c r="N4" s="256"/>
-      <c r="O4" s="256"/>
-      <c r="P4" s="256"/>
+      <c r="J4" s="267"/>
+      <c r="K4" s="267"/>
+      <c r="L4" s="267"/>
+      <c r="M4" s="267"/>
+      <c r="N4" s="267"/>
+      <c r="O4" s="267"/>
+      <c r="P4" s="267"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -42317,14 +42322,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="256"/>
-      <c r="J5" s="256"/>
-      <c r="K5" s="256"/>
-      <c r="L5" s="256"/>
-      <c r="M5" s="256"/>
-      <c r="N5" s="256"/>
-      <c r="O5" s="256"/>
-      <c r="P5" s="256"/>
+      <c r="I5" s="267"/>
+      <c r="J5" s="267"/>
+      <c r="K5" s="267"/>
+      <c r="L5" s="267"/>
+      <c r="M5" s="267"/>
+      <c r="N5" s="267"/>
+      <c r="O5" s="267"/>
+      <c r="P5" s="267"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -42459,70 +42464,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="247" t="s">
+      <c r="B12" s="258" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="247" t="s">
+      <c r="C12" s="258" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="247"/>
-      <c r="E12" s="247"/>
-      <c r="F12" s="247" t="s">
+      <c r="D12" s="258"/>
+      <c r="E12" s="258"/>
+      <c r="F12" s="258" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="247" t="s">
+      <c r="G12" s="258" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="247" t="s">
+      <c r="H12" s="258" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="247" t="s">
+      <c r="I12" s="258" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="247" t="s">
+      <c r="J12" s="258" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="247"/>
-      <c r="L12" s="247"/>
-      <c r="M12" s="247"/>
-      <c r="N12" s="247"/>
-      <c r="O12" s="247"/>
-      <c r="P12" s="255" t="s">
+      <c r="K12" s="258"/>
+      <c r="L12" s="258"/>
+      <c r="M12" s="258"/>
+      <c r="N12" s="258"/>
+      <c r="O12" s="258"/>
+      <c r="P12" s="266" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="247"/>
-      <c r="C13" s="247"/>
-      <c r="D13" s="247"/>
-      <c r="E13" s="247"/>
-      <c r="F13" s="247"/>
-      <c r="G13" s="247"/>
-      <c r="H13" s="247"/>
-      <c r="I13" s="247"/>
-      <c r="J13" s="254" t="s">
+      <c r="B13" s="258"/>
+      <c r="C13" s="258"/>
+      <c r="D13" s="258"/>
+      <c r="E13" s="258"/>
+      <c r="F13" s="258"/>
+      <c r="G13" s="258"/>
+      <c r="H13" s="258"/>
+      <c r="I13" s="258"/>
+      <c r="J13" s="265" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="254"/>
-      <c r="L13" s="254" t="s">
+      <c r="K13" s="265"/>
+      <c r="L13" s="265" t="s">
         <v>98</v>
       </c>
-      <c r="M13" s="254"/>
-      <c r="N13" s="254" t="s">
+      <c r="M13" s="265"/>
+      <c r="N13" s="265" t="s">
         <v>99</v>
       </c>
-      <c r="O13" s="254"/>
-      <c r="P13" s="255"/>
+      <c r="O13" s="265"/>
+      <c r="P13" s="266"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="247"/>
-      <c r="C14" s="247"/>
-      <c r="D14" s="247"/>
-      <c r="E14" s="247"/>
-      <c r="F14" s="247"/>
-      <c r="G14" s="247"/>
-      <c r="H14" s="247"/>
-      <c r="I14" s="247"/>
+      <c r="B14" s="258"/>
+      <c r="C14" s="258"/>
+      <c r="D14" s="258"/>
+      <c r="E14" s="258"/>
+      <c r="F14" s="258"/>
+      <c r="G14" s="258"/>
+      <c r="H14" s="258"/>
+      <c r="I14" s="258"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -42541,7 +42546,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="255"/>
+      <c r="P14" s="266"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>

</xml_diff>

<commit_message>
chore(template): update master excel template
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02DF717D-E059-4EAC-9B08-848151C5FD45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34BB051A-374A-45A1-A127-34253AA92841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cover" sheetId="21" r:id="rId1"/>
@@ -457,7 +457,7 @@
     <numFmt numFmtId="167" formatCode="[$-421]dddd"/>
     <numFmt numFmtId="168" formatCode="[$-421]dd\ mmm\ yyyy;@"/>
     <numFmt numFmtId="169" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="171" formatCode="0.000"/>
+    <numFmt numFmtId="170" formatCode="0.000"/>
   </numFmts>
   <fonts count="34">
     <font>
@@ -2136,7 +2136,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="169" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="309">
+  <cellXfs count="308">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2548,7 +2548,7 @@
     <xf numFmtId="0" fontId="32" fillId="4" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="33" fillId="4" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="33" fillId="4" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="33" fillId="4" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2593,17 +2593,130 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="39" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="114" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="38" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="0" borderId="42" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="41" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="75" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2613,41 +2726,47 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="61" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="66" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="59" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="54" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
     <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2661,16 +2780,57 @@
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="111" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="112" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2778,187 +2938,65 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="39" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="114" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="61" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="66" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="59" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="54" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="111" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="112" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="75" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3089,48 +3127,6 @@
     <xf numFmtId="0" fontId="32" fillId="4" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="38" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="24" fillId="0" borderId="42" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="41" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma [0] 2" xfId="3" xr:uid="{5950E916-03C9-42B5-8F65-57AD3DC32531}"/>
@@ -3138,7 +3134,119 @@
     <cellStyle name="Normal 2 2 3" xfId="2" xr:uid="{25DAB206-4C06-437D-BFFA-FD21FFA5A242}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="27">
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color rgb="FFFFC000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor theme="7" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color rgb="FFFFC000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor theme="7" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -3291,68 +3399,6 @@
           <bgColor rgb="FF002060"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color rgb="FFFFC000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor theme="7" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <fill>
@@ -4249,40 +4295,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="261"/>
-      <c r="C1" s="261"/>
-      <c r="D1" s="261"/>
-      <c r="E1" s="261"/>
-      <c r="F1" s="261"/>
-      <c r="G1" s="261"/>
-      <c r="H1" s="261"/>
-      <c r="I1" s="261"/>
-      <c r="J1" s="261"/>
-      <c r="K1" s="261"/>
-      <c r="L1" s="261"/>
-      <c r="M1" s="261"/>
-      <c r="N1" s="261"/>
-      <c r="O1" s="261"/>
-      <c r="P1" s="261"/>
+      <c r="B1" s="272"/>
+      <c r="C1" s="272"/>
+      <c r="D1" s="272"/>
+      <c r="E1" s="272"/>
+      <c r="F1" s="272"/>
+      <c r="G1" s="272"/>
+      <c r="H1" s="272"/>
+      <c r="I1" s="272"/>
+      <c r="J1" s="272"/>
+      <c r="K1" s="272"/>
+      <c r="L1" s="272"/>
+      <c r="M1" s="272"/>
+      <c r="N1" s="272"/>
+      <c r="O1" s="272"/>
+      <c r="P1" s="272"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="270" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="260"/>
-      <c r="D2" s="260"/>
-      <c r="E2" s="260"/>
-      <c r="F2" s="260"/>
-      <c r="G2" s="260"/>
-      <c r="H2" s="260"/>
-      <c r="I2" s="260"/>
-      <c r="J2" s="260"/>
-      <c r="K2" s="260"/>
-      <c r="L2" s="260"/>
-      <c r="M2" s="260"/>
-      <c r="N2" s="260"/>
-      <c r="O2" s="260"/>
-      <c r="P2" s="260"/>
+      <c r="C2" s="271"/>
+      <c r="D2" s="271"/>
+      <c r="E2" s="271"/>
+      <c r="F2" s="271"/>
+      <c r="G2" s="271"/>
+      <c r="H2" s="271"/>
+      <c r="I2" s="271"/>
+      <c r="J2" s="271"/>
+      <c r="K2" s="271"/>
+      <c r="L2" s="271"/>
+      <c r="M2" s="271"/>
+      <c r="N2" s="271"/>
+      <c r="O2" s="271"/>
+      <c r="P2" s="271"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -4309,16 +4355,16 @@
       <c r="F4" s="61"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="267" t="s">
+      <c r="I4" s="278" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="267"/>
-      <c r="K4" s="267"/>
-      <c r="L4" s="267"/>
-      <c r="M4" s="267"/>
-      <c r="N4" s="267"/>
-      <c r="O4" s="267"/>
-      <c r="P4" s="267"/>
+      <c r="J4" s="278"/>
+      <c r="K4" s="278"/>
+      <c r="L4" s="278"/>
+      <c r="M4" s="278"/>
+      <c r="N4" s="278"/>
+      <c r="O4" s="278"/>
+      <c r="P4" s="278"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -4332,14 +4378,14 @@
       <c r="F5" s="58"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="267"/>
-      <c r="J5" s="267"/>
-      <c r="K5" s="267"/>
-      <c r="L5" s="267"/>
-      <c r="M5" s="267"/>
-      <c r="N5" s="267"/>
-      <c r="O5" s="267"/>
-      <c r="P5" s="267"/>
+      <c r="I5" s="278"/>
+      <c r="J5" s="278"/>
+      <c r="K5" s="278"/>
+      <c r="L5" s="278"/>
+      <c r="M5" s="278"/>
+      <c r="N5" s="278"/>
+      <c r="O5" s="278"/>
+      <c r="P5" s="278"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -4474,70 +4520,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="258" t="s">
+      <c r="B12" s="269" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="258" t="s">
+      <c r="C12" s="269" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="258"/>
-      <c r="E12" s="258"/>
-      <c r="F12" s="258" t="s">
+      <c r="D12" s="269"/>
+      <c r="E12" s="269"/>
+      <c r="F12" s="269" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="258" t="s">
+      <c r="G12" s="269" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="258" t="s">
+      <c r="H12" s="269" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="258" t="s">
+      <c r="I12" s="269" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="258" t="s">
+      <c r="J12" s="269" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="258"/>
-      <c r="L12" s="258"/>
-      <c r="M12" s="258"/>
-      <c r="N12" s="258"/>
-      <c r="O12" s="258"/>
-      <c r="P12" s="266" t="s">
+      <c r="K12" s="269"/>
+      <c r="L12" s="269"/>
+      <c r="M12" s="269"/>
+      <c r="N12" s="269"/>
+      <c r="O12" s="269"/>
+      <c r="P12" s="277" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="258"/>
-      <c r="C13" s="258"/>
-      <c r="D13" s="258"/>
-      <c r="E13" s="258"/>
-      <c r="F13" s="258"/>
-      <c r="G13" s="258"/>
-      <c r="H13" s="258"/>
-      <c r="I13" s="258"/>
-      <c r="J13" s="265" t="s">
+      <c r="B13" s="269"/>
+      <c r="C13" s="269"/>
+      <c r="D13" s="269"/>
+      <c r="E13" s="269"/>
+      <c r="F13" s="269"/>
+      <c r="G13" s="269"/>
+      <c r="H13" s="269"/>
+      <c r="I13" s="269"/>
+      <c r="J13" s="276" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="265"/>
-      <c r="L13" s="265" t="s">
+      <c r="K13" s="276"/>
+      <c r="L13" s="276" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="265"/>
-      <c r="N13" s="265" t="s">
+      <c r="M13" s="276"/>
+      <c r="N13" s="276" t="s">
         <v>95</v>
       </c>
-      <c r="O13" s="265"/>
-      <c r="P13" s="266"/>
+      <c r="O13" s="276"/>
+      <c r="P13" s="277"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="258"/>
-      <c r="C14" s="258"/>
-      <c r="D14" s="258"/>
-      <c r="E14" s="258"/>
-      <c r="F14" s="258"/>
-      <c r="G14" s="258"/>
-      <c r="H14" s="258"/>
-      <c r="I14" s="258"/>
+      <c r="B14" s="269"/>
+      <c r="C14" s="269"/>
+      <c r="D14" s="269"/>
+      <c r="E14" s="269"/>
+      <c r="F14" s="269"/>
+      <c r="G14" s="269"/>
+      <c r="H14" s="269"/>
+      <c r="I14" s="269"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -4556,7 +4602,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="266"/>
+      <c r="P14" s="277"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -4952,7 +4998,7 @@
     <mergeCell ref="G12:G14"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P51">
-    <cfRule type="expression" dxfId="0" priority="14">
+    <cfRule type="expression" dxfId="7" priority="14">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4979,38 +5025,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="103.2" customHeight="1">
-      <c r="B1" s="260"/>
-      <c r="C1" s="260"/>
-      <c r="D1" s="260"/>
-      <c r="E1" s="260"/>
-      <c r="F1" s="260"/>
-      <c r="G1" s="260"/>
-      <c r="H1" s="260"/>
-      <c r="I1" s="260"/>
-      <c r="J1" s="260"/>
-      <c r="K1" s="260"/>
-      <c r="L1" s="260"/>
-      <c r="M1" s="260"/>
-      <c r="N1" s="260"/>
-      <c r="O1" s="260"/>
+      <c r="B1" s="271"/>
+      <c r="C1" s="271"/>
+      <c r="D1" s="271"/>
+      <c r="E1" s="271"/>
+      <c r="F1" s="271"/>
+      <c r="G1" s="271"/>
+      <c r="H1" s="271"/>
+      <c r="I1" s="271"/>
+      <c r="J1" s="271"/>
+      <c r="K1" s="271"/>
+      <c r="L1" s="271"/>
+      <c r="M1" s="271"/>
+      <c r="N1" s="271"/>
+      <c r="O1" s="271"/>
     </row>
     <row r="2" spans="2:15" ht="22.95" customHeight="1">
-      <c r="B2" s="268" t="s">
+      <c r="B2" s="279" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="268"/>
-      <c r="D2" s="268"/>
-      <c r="E2" s="268"/>
-      <c r="F2" s="268"/>
-      <c r="G2" s="268"/>
-      <c r="H2" s="268"/>
-      <c r="I2" s="268"/>
-      <c r="J2" s="268"/>
-      <c r="K2" s="268"/>
-      <c r="L2" s="268"/>
-      <c r="M2" s="268"/>
-      <c r="N2" s="268"/>
-      <c r="O2" s="268"/>
+      <c r="C2" s="279"/>
+      <c r="D2" s="279"/>
+      <c r="E2" s="279"/>
+      <c r="F2" s="279"/>
+      <c r="G2" s="279"/>
+      <c r="H2" s="279"/>
+      <c r="I2" s="279"/>
+      <c r="J2" s="279"/>
+      <c r="K2" s="279"/>
+      <c r="L2" s="279"/>
+      <c r="M2" s="279"/>
+      <c r="N2" s="279"/>
+      <c r="O2" s="279"/>
     </row>
     <row r="3" spans="2:15">
       <c r="B3" t="s">
@@ -5062,179 +5108,179 @@
     </row>
     <row r="9" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="11" spans="2:15" s="58" customFormat="1">
-      <c r="B11" s="269" t="s">
+      <c r="B11" s="280" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="269"/>
-      <c r="D11" s="269"/>
-      <c r="E11" s="269"/>
-      <c r="G11" s="269" t="s">
+      <c r="C11" s="280"/>
+      <c r="D11" s="280"/>
+      <c r="E11" s="280"/>
+      <c r="G11" s="280" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="269"/>
-      <c r="I11" s="269"/>
-      <c r="J11" s="269"/>
-      <c r="L11" s="269" t="s">
+      <c r="H11" s="280"/>
+      <c r="I11" s="280"/>
+      <c r="J11" s="280"/>
+      <c r="L11" s="280" t="s">
         <v>105</v>
       </c>
-      <c r="M11" s="269"/>
-      <c r="N11" s="269"/>
-      <c r="O11" s="269"/>
+      <c r="M11" s="280"/>
+      <c r="N11" s="280"/>
+      <c r="O11" s="280"/>
     </row>
     <row r="12" spans="2:15" ht="4.95" customHeight="1"/>
     <row r="13" spans="2:15">
-      <c r="B13" s="260"/>
-      <c r="C13" s="260"/>
-      <c r="D13" s="260"/>
-      <c r="E13" s="260"/>
-      <c r="G13" s="260"/>
-      <c r="H13" s="260"/>
-      <c r="I13" s="260"/>
-      <c r="J13" s="260"/>
-      <c r="L13" s="260"/>
-      <c r="M13" s="260"/>
-      <c r="N13" s="260"/>
-      <c r="O13" s="260"/>
+      <c r="B13" s="271"/>
+      <c r="C13" s="271"/>
+      <c r="D13" s="271"/>
+      <c r="E13" s="271"/>
+      <c r="G13" s="271"/>
+      <c r="H13" s="271"/>
+      <c r="I13" s="271"/>
+      <c r="J13" s="271"/>
+      <c r="L13" s="271"/>
+      <c r="M13" s="271"/>
+      <c r="N13" s="271"/>
+      <c r="O13" s="271"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="260"/>
-      <c r="C14" s="260"/>
-      <c r="D14" s="260"/>
-      <c r="E14" s="260"/>
-      <c r="G14" s="260"/>
-      <c r="H14" s="260"/>
-      <c r="I14" s="260"/>
-      <c r="J14" s="260"/>
-      <c r="L14" s="260"/>
-      <c r="M14" s="260"/>
-      <c r="N14" s="260"/>
-      <c r="O14" s="260"/>
+      <c r="B14" s="271"/>
+      <c r="C14" s="271"/>
+      <c r="D14" s="271"/>
+      <c r="E14" s="271"/>
+      <c r="G14" s="271"/>
+      <c r="H14" s="271"/>
+      <c r="I14" s="271"/>
+      <c r="J14" s="271"/>
+      <c r="L14" s="271"/>
+      <c r="M14" s="271"/>
+      <c r="N14" s="271"/>
+      <c r="O14" s="271"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="260"/>
-      <c r="C15" s="260"/>
-      <c r="D15" s="260"/>
-      <c r="E15" s="260"/>
-      <c r="G15" s="260"/>
-      <c r="H15" s="260"/>
-      <c r="I15" s="260"/>
-      <c r="J15" s="260"/>
-      <c r="L15" s="260"/>
-      <c r="M15" s="260"/>
-      <c r="N15" s="260"/>
-      <c r="O15" s="260"/>
+      <c r="B15" s="271"/>
+      <c r="C15" s="271"/>
+      <c r="D15" s="271"/>
+      <c r="E15" s="271"/>
+      <c r="G15" s="271"/>
+      <c r="H15" s="271"/>
+      <c r="I15" s="271"/>
+      <c r="J15" s="271"/>
+      <c r="L15" s="271"/>
+      <c r="M15" s="271"/>
+      <c r="N15" s="271"/>
+      <c r="O15" s="271"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="260"/>
-      <c r="C16" s="260"/>
-      <c r="D16" s="260"/>
-      <c r="E16" s="260"/>
-      <c r="G16" s="260"/>
-      <c r="H16" s="260"/>
-      <c r="I16" s="260"/>
-      <c r="J16" s="260"/>
-      <c r="L16" s="260"/>
-      <c r="M16" s="260"/>
-      <c r="N16" s="260"/>
-      <c r="O16" s="260"/>
+      <c r="B16" s="271"/>
+      <c r="C16" s="271"/>
+      <c r="D16" s="271"/>
+      <c r="E16" s="271"/>
+      <c r="G16" s="271"/>
+      <c r="H16" s="271"/>
+      <c r="I16" s="271"/>
+      <c r="J16" s="271"/>
+      <c r="L16" s="271"/>
+      <c r="M16" s="271"/>
+      <c r="N16" s="271"/>
+      <c r="O16" s="271"/>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="260"/>
-      <c r="C17" s="260"/>
-      <c r="D17" s="260"/>
-      <c r="E17" s="260"/>
-      <c r="G17" s="260"/>
-      <c r="H17" s="260"/>
-      <c r="I17" s="260"/>
-      <c r="J17" s="260"/>
-      <c r="L17" s="260"/>
-      <c r="M17" s="260"/>
-      <c r="N17" s="260"/>
-      <c r="O17" s="260"/>
+      <c r="B17" s="271"/>
+      <c r="C17" s="271"/>
+      <c r="D17" s="271"/>
+      <c r="E17" s="271"/>
+      <c r="G17" s="271"/>
+      <c r="H17" s="271"/>
+      <c r="I17" s="271"/>
+      <c r="J17" s="271"/>
+      <c r="L17" s="271"/>
+      <c r="M17" s="271"/>
+      <c r="N17" s="271"/>
+      <c r="O17" s="271"/>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="260"/>
-      <c r="C18" s="260"/>
-      <c r="D18" s="260"/>
-      <c r="E18" s="260"/>
-      <c r="G18" s="260"/>
-      <c r="H18" s="260"/>
-      <c r="I18" s="260"/>
-      <c r="J18" s="260"/>
-      <c r="L18" s="260"/>
-      <c r="M18" s="260"/>
-      <c r="N18" s="260"/>
-      <c r="O18" s="260"/>
+      <c r="B18" s="271"/>
+      <c r="C18" s="271"/>
+      <c r="D18" s="271"/>
+      <c r="E18" s="271"/>
+      <c r="G18" s="271"/>
+      <c r="H18" s="271"/>
+      <c r="I18" s="271"/>
+      <c r="J18" s="271"/>
+      <c r="L18" s="271"/>
+      <c r="M18" s="271"/>
+      <c r="N18" s="271"/>
+      <c r="O18" s="271"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="B19" s="260"/>
-      <c r="C19" s="260"/>
-      <c r="D19" s="260"/>
-      <c r="E19" s="260"/>
-      <c r="G19" s="260"/>
-      <c r="H19" s="260"/>
-      <c r="I19" s="260"/>
-      <c r="J19" s="260"/>
-      <c r="L19" s="260"/>
-      <c r="M19" s="260"/>
-      <c r="N19" s="260"/>
-      <c r="O19" s="260"/>
+      <c r="B19" s="271"/>
+      <c r="C19" s="271"/>
+      <c r="D19" s="271"/>
+      <c r="E19" s="271"/>
+      <c r="G19" s="271"/>
+      <c r="H19" s="271"/>
+      <c r="I19" s="271"/>
+      <c r="J19" s="271"/>
+      <c r="L19" s="271"/>
+      <c r="M19" s="271"/>
+      <c r="N19" s="271"/>
+      <c r="O19" s="271"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="B20" s="260"/>
-      <c r="C20" s="260"/>
-      <c r="D20" s="260"/>
-      <c r="E20" s="260"/>
-      <c r="G20" s="260"/>
-      <c r="H20" s="260"/>
-      <c r="I20" s="260"/>
-      <c r="J20" s="260"/>
-      <c r="L20" s="260"/>
-      <c r="M20" s="260"/>
-      <c r="N20" s="260"/>
-      <c r="O20" s="260"/>
+      <c r="B20" s="271"/>
+      <c r="C20" s="271"/>
+      <c r="D20" s="271"/>
+      <c r="E20" s="271"/>
+      <c r="G20" s="271"/>
+      <c r="H20" s="271"/>
+      <c r="I20" s="271"/>
+      <c r="J20" s="271"/>
+      <c r="L20" s="271"/>
+      <c r="M20" s="271"/>
+      <c r="N20" s="271"/>
+      <c r="O20" s="271"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="B21" s="260"/>
-      <c r="C21" s="260"/>
-      <c r="D21" s="260"/>
-      <c r="E21" s="260"/>
-      <c r="G21" s="260"/>
-      <c r="H21" s="260"/>
-      <c r="I21" s="260"/>
-      <c r="J21" s="260"/>
-      <c r="L21" s="260"/>
-      <c r="M21" s="260"/>
-      <c r="N21" s="260"/>
-      <c r="O21" s="260"/>
+      <c r="B21" s="271"/>
+      <c r="C21" s="271"/>
+      <c r="D21" s="271"/>
+      <c r="E21" s="271"/>
+      <c r="G21" s="271"/>
+      <c r="H21" s="271"/>
+      <c r="I21" s="271"/>
+      <c r="J21" s="271"/>
+      <c r="L21" s="271"/>
+      <c r="M21" s="271"/>
+      <c r="N21" s="271"/>
+      <c r="O21" s="271"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="B22" s="260"/>
-      <c r="C22" s="260"/>
-      <c r="D22" s="260"/>
-      <c r="E22" s="260"/>
-      <c r="G22" s="260"/>
-      <c r="H22" s="260"/>
-      <c r="I22" s="260"/>
-      <c r="J22" s="260"/>
-      <c r="L22" s="260"/>
-      <c r="M22" s="260"/>
-      <c r="N22" s="260"/>
-      <c r="O22" s="260"/>
+      <c r="B22" s="271"/>
+      <c r="C22" s="271"/>
+      <c r="D22" s="271"/>
+      <c r="E22" s="271"/>
+      <c r="G22" s="271"/>
+      <c r="H22" s="271"/>
+      <c r="I22" s="271"/>
+      <c r="J22" s="271"/>
+      <c r="L22" s="271"/>
+      <c r="M22" s="271"/>
+      <c r="N22" s="271"/>
+      <c r="O22" s="271"/>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="260"/>
-      <c r="C23" s="260"/>
-      <c r="D23" s="260"/>
-      <c r="E23" s="260"/>
-      <c r="G23" s="260"/>
-      <c r="H23" s="260"/>
-      <c r="I23" s="260"/>
-      <c r="J23" s="260"/>
-      <c r="L23" s="260"/>
-      <c r="M23" s="260"/>
-      <c r="N23" s="260"/>
-      <c r="O23" s="260"/>
+      <c r="B23" s="271"/>
+      <c r="C23" s="271"/>
+      <c r="D23" s="271"/>
+      <c r="E23" s="271"/>
+      <c r="G23" s="271"/>
+      <c r="H23" s="271"/>
+      <c r="I23" s="271"/>
+      <c r="J23" s="271"/>
+      <c r="L23" s="271"/>
+      <c r="M23" s="271"/>
+      <c r="N23" s="271"/>
+      <c r="O23" s="271"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5268,35 +5314,35 @@
   <sheetData>
     <row r="1" spans="2:29" ht="4.8" customHeight="1" thickBot="1"/>
     <row r="2" spans="2:29" ht="19.95" customHeight="1" thickBot="1">
-      <c r="B2" s="270" t="s">
+      <c r="B2" s="281" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="271"/>
-      <c r="D2" s="271"/>
-      <c r="E2" s="271"/>
-      <c r="F2" s="271"/>
-      <c r="G2" s="271"/>
-      <c r="H2" s="271"/>
-      <c r="I2" s="271"/>
-      <c r="J2" s="271"/>
-      <c r="K2" s="271"/>
-      <c r="L2" s="271"/>
-      <c r="M2" s="271"/>
-      <c r="N2" s="271"/>
-      <c r="O2" s="271"/>
-      <c r="P2" s="271"/>
-      <c r="Q2" s="271"/>
-      <c r="R2" s="271"/>
-      <c r="S2" s="271"/>
-      <c r="T2" s="271"/>
-      <c r="U2" s="271"/>
-      <c r="V2" s="271"/>
-      <c r="W2" s="271"/>
-      <c r="X2" s="271"/>
-      <c r="Y2" s="271"/>
-      <c r="Z2" s="271"/>
-      <c r="AA2" s="271"/>
-      <c r="AB2" s="272"/>
+      <c r="C2" s="282"/>
+      <c r="D2" s="282"/>
+      <c r="E2" s="282"/>
+      <c r="F2" s="282"/>
+      <c r="G2" s="282"/>
+      <c r="H2" s="282"/>
+      <c r="I2" s="282"/>
+      <c r="J2" s="282"/>
+      <c r="K2" s="282"/>
+      <c r="L2" s="282"/>
+      <c r="M2" s="282"/>
+      <c r="N2" s="282"/>
+      <c r="O2" s="282"/>
+      <c r="P2" s="282"/>
+      <c r="Q2" s="282"/>
+      <c r="R2" s="282"/>
+      <c r="S2" s="282"/>
+      <c r="T2" s="282"/>
+      <c r="U2" s="282"/>
+      <c r="V2" s="282"/>
+      <c r="W2" s="282"/>
+      <c r="X2" s="282"/>
+      <c r="Y2" s="282"/>
+      <c r="Z2" s="282"/>
+      <c r="AA2" s="282"/>
+      <c r="AB2" s="283"/>
       <c r="AC2" s="127"/>
     </row>
     <row r="3" spans="2:29" ht="15" customHeight="1">
@@ -5396,74 +5442,74 @@
       <c r="AB11" s="125"/>
     </row>
     <row r="12" spans="2:29" ht="15" customHeight="1">
-      <c r="B12" s="282" t="s">
+      <c r="B12" s="293" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="284" t="s">
+      <c r="C12" s="295" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="285"/>
-      <c r="E12" s="285"/>
-      <c r="F12" s="285"/>
-      <c r="G12" s="285"/>
-      <c r="H12" s="285"/>
-      <c r="I12" s="285"/>
-      <c r="J12" s="285"/>
-      <c r="K12" s="285"/>
-      <c r="L12" s="286"/>
-      <c r="M12" s="290" t="s">
+      <c r="D12" s="296"/>
+      <c r="E12" s="296"/>
+      <c r="F12" s="296"/>
+      <c r="G12" s="296"/>
+      <c r="H12" s="296"/>
+      <c r="I12" s="296"/>
+      <c r="J12" s="296"/>
+      <c r="K12" s="296"/>
+      <c r="L12" s="297"/>
+      <c r="M12" s="301" t="s">
         <v>113</v>
       </c>
-      <c r="N12" s="290" t="s">
+      <c r="N12" s="301" t="s">
         <v>34</v>
       </c>
-      <c r="O12" s="295" t="s">
+      <c r="O12" s="306" t="s">
         <v>114</v>
       </c>
-      <c r="P12" s="295"/>
-      <c r="Q12" s="295"/>
-      <c r="R12" s="295"/>
-      <c r="S12" s="295"/>
-      <c r="T12" s="295"/>
-      <c r="U12" s="295"/>
-      <c r="V12" s="295"/>
-      <c r="W12" s="295"/>
-      <c r="X12" s="295"/>
-      <c r="Y12" s="295"/>
-      <c r="Z12" s="295"/>
-      <c r="AA12" s="295"/>
-      <c r="AB12" s="296"/>
+      <c r="P12" s="306"/>
+      <c r="Q12" s="306"/>
+      <c r="R12" s="306"/>
+      <c r="S12" s="306"/>
+      <c r="T12" s="306"/>
+      <c r="U12" s="306"/>
+      <c r="V12" s="306"/>
+      <c r="W12" s="306"/>
+      <c r="X12" s="306"/>
+      <c r="Y12" s="306"/>
+      <c r="Z12" s="306"/>
+      <c r="AA12" s="306"/>
+      <c r="AB12" s="307"/>
     </row>
     <row r="13" spans="2:29" ht="15" customHeight="1">
-      <c r="B13" s="283"/>
-      <c r="C13" s="287"/>
-      <c r="D13" s="288"/>
-      <c r="E13" s="288"/>
-      <c r="F13" s="288"/>
-      <c r="G13" s="288"/>
-      <c r="H13" s="288"/>
-      <c r="I13" s="288"/>
-      <c r="J13" s="288"/>
-      <c r="K13" s="288"/>
-      <c r="L13" s="289"/>
-      <c r="M13" s="291"/>
-      <c r="N13" s="291"/>
-      <c r="O13" s="292" t="s">
+      <c r="B13" s="294"/>
+      <c r="C13" s="298"/>
+      <c r="D13" s="299"/>
+      <c r="E13" s="299"/>
+      <c r="F13" s="299"/>
+      <c r="G13" s="299"/>
+      <c r="H13" s="299"/>
+      <c r="I13" s="299"/>
+      <c r="J13" s="299"/>
+      <c r="K13" s="299"/>
+      <c r="L13" s="300"/>
+      <c r="M13" s="302"/>
+      <c r="N13" s="302"/>
+      <c r="O13" s="303" t="s">
         <v>115</v>
       </c>
-      <c r="P13" s="293"/>
-      <c r="Q13" s="294"/>
-      <c r="R13" s="292" t="s">
+      <c r="P13" s="304"/>
+      <c r="Q13" s="305"/>
+      <c r="R13" s="303" t="s">
         <v>116</v>
       </c>
-      <c r="S13" s="293"/>
-      <c r="T13" s="294"/>
-      <c r="U13" s="292" t="s">
+      <c r="S13" s="304"/>
+      <c r="T13" s="305"/>
+      <c r="U13" s="303" t="s">
         <v>117</v>
       </c>
-      <c r="V13" s="293"/>
-      <c r="W13" s="294"/>
-      <c r="X13" s="273" t="s">
+      <c r="V13" s="304"/>
+      <c r="W13" s="305"/>
+      <c r="X13" s="284" t="s">
         <v>118</v>
       </c>
       <c r="Y13" s="132" t="s">
@@ -5472,27 +5518,27 @@
       <c r="Z13" s="133" t="s">
         <v>119</v>
       </c>
-      <c r="AA13" s="275" t="s">
+      <c r="AA13" s="286" t="s">
         <v>120</v>
       </c>
-      <c r="AB13" s="277" t="s">
+      <c r="AB13" s="288" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="14" spans="2:29" ht="15" customHeight="1">
-      <c r="B14" s="283"/>
-      <c r="C14" s="287"/>
-      <c r="D14" s="288"/>
-      <c r="E14" s="288"/>
-      <c r="F14" s="288"/>
-      <c r="G14" s="288"/>
-      <c r="H14" s="288"/>
-      <c r="I14" s="288"/>
-      <c r="J14" s="288"/>
-      <c r="K14" s="288"/>
-      <c r="L14" s="289"/>
-      <c r="M14" s="274"/>
-      <c r="N14" s="274"/>
+      <c r="B14" s="294"/>
+      <c r="C14" s="298"/>
+      <c r="D14" s="299"/>
+      <c r="E14" s="299"/>
+      <c r="F14" s="299"/>
+      <c r="G14" s="299"/>
+      <c r="H14" s="299"/>
+      <c r="I14" s="299"/>
+      <c r="J14" s="299"/>
+      <c r="K14" s="299"/>
+      <c r="L14" s="300"/>
+      <c r="M14" s="285"/>
+      <c r="N14" s="285"/>
       <c r="O14" s="134" t="s">
         <v>122</v>
       </c>
@@ -5520,32 +5566,32 @@
       <c r="W14" s="134" t="s">
         <v>129</v>
       </c>
-      <c r="X14" s="274"/>
+      <c r="X14" s="285"/>
       <c r="Y14" s="132" t="s">
         <v>130</v>
       </c>
       <c r="Z14" s="134" t="s">
         <v>131</v>
       </c>
-      <c r="AA14" s="276"/>
-      <c r="AB14" s="278"/>
+      <c r="AA14" s="287"/>
+      <c r="AB14" s="289"/>
     </row>
     <row r="15" spans="2:29" ht="15" customHeight="1" thickBot="1">
       <c r="B15" s="128">
         <v>1</v>
       </c>
-      <c r="C15" s="279">
+      <c r="C15" s="290">
         <v>2</v>
       </c>
-      <c r="D15" s="280"/>
-      <c r="E15" s="280"/>
-      <c r="F15" s="280"/>
-      <c r="G15" s="280"/>
-      <c r="H15" s="280"/>
-      <c r="I15" s="280"/>
-      <c r="J15" s="280"/>
-      <c r="K15" s="280"/>
-      <c r="L15" s="281"/>
+      <c r="D15" s="291"/>
+      <c r="E15" s="291"/>
+      <c r="F15" s="291"/>
+      <c r="G15" s="291"/>
+      <c r="H15" s="291"/>
+      <c r="I15" s="291"/>
+      <c r="J15" s="291"/>
+      <c r="K15" s="291"/>
+      <c r="L15" s="292"/>
       <c r="M15" s="129">
         <v>3</v>
       </c>
@@ -5635,38 +5681,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="120" customHeight="1">
-      <c r="B1" s="257"/>
-      <c r="C1" s="257"/>
-      <c r="D1" s="257"/>
-      <c r="E1" s="257"/>
-      <c r="F1" s="257"/>
-      <c r="G1" s="257"/>
-      <c r="H1" s="257"/>
-      <c r="I1" s="257"/>
+      <c r="B1" s="268"/>
+      <c r="C1" s="268"/>
+      <c r="D1" s="268"/>
+      <c r="E1" s="268"/>
+      <c r="F1" s="268"/>
+      <c r="G1" s="268"/>
+      <c r="H1" s="268"/>
+      <c r="I1" s="268"/>
     </row>
     <row r="2" spans="1:9" ht="28.8" customHeight="1">
-      <c r="B2" s="254" t="s">
+      <c r="B2" s="265" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="254"/>
-      <c r="D2" s="254"/>
-      <c r="E2" s="254"/>
-      <c r="F2" s="254"/>
-      <c r="G2" s="254"/>
-      <c r="H2" s="254"/>
-      <c r="I2" s="254"/>
+      <c r="C2" s="265"/>
+      <c r="D2" s="265"/>
+      <c r="E2" s="265"/>
+      <c r="F2" s="265"/>
+      <c r="G2" s="265"/>
+      <c r="H2" s="265"/>
+      <c r="I2" s="265"/>
     </row>
     <row r="3" spans="1:9" ht="19.8" customHeight="1">
-      <c r="B3" s="255" t="s">
+      <c r="B3" s="266" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="255"/>
-      <c r="D3" s="255"/>
-      <c r="E3" s="255"/>
-      <c r="F3" s="255"/>
-      <c r="G3" s="255"/>
-      <c r="H3" s="255"/>
-      <c r="I3" s="255"/>
+      <c r="C3" s="266"/>
+      <c r="D3" s="266"/>
+      <c r="E3" s="266"/>
+      <c r="F3" s="266"/>
+      <c r="G3" s="266"/>
+      <c r="H3" s="266"/>
+      <c r="I3" s="266"/>
     </row>
     <row r="4" spans="1:9" ht="7.8" customHeight="1"/>
     <row r="5" spans="1:9" s="8" customFormat="1" ht="24" customHeight="1">
@@ -5674,10 +5720,10 @@
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="256" t="s">
+      <c r="C5" s="267" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="256"/>
+      <c r="D5" s="267"/>
       <c r="E5" s="11" t="s">
         <v>38</v>
       </c>
@@ -14031,7 +14077,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="23" priority="2">
+    <cfRule type="expression" dxfId="26" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14064,63 +14110,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="147.6" customHeight="1">
-      <c r="B1" s="257"/>
-      <c r="C1" s="257"/>
-      <c r="D1" s="257"/>
-      <c r="E1" s="257"/>
-      <c r="F1" s="257"/>
-      <c r="G1" s="257"/>
-      <c r="H1" s="257"/>
-      <c r="I1" s="257"/>
-      <c r="J1" s="257"/>
-      <c r="K1" s="257"/>
-      <c r="L1" s="257"/>
-      <c r="M1" s="257"/>
-      <c r="N1" s="257"/>
+      <c r="B1" s="268"/>
+      <c r="C1" s="268"/>
+      <c r="D1" s="268"/>
+      <c r="E1" s="268"/>
+      <c r="F1" s="268"/>
+      <c r="G1" s="268"/>
+      <c r="H1" s="268"/>
+      <c r="I1" s="268"/>
+      <c r="J1" s="268"/>
+      <c r="K1" s="268"/>
+      <c r="L1" s="268"/>
+      <c r="M1" s="268"/>
+      <c r="N1" s="268"/>
     </row>
     <row r="2" spans="2:14" ht="25.2" customHeight="1">
-      <c r="B2" s="254" t="s">
+      <c r="B2" s="265" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="254"/>
-      <c r="D2" s="254"/>
-      <c r="E2" s="254"/>
-      <c r="F2" s="254"/>
-      <c r="G2" s="254"/>
-      <c r="H2" s="254"/>
-      <c r="I2" s="254"/>
-      <c r="J2" s="254"/>
-      <c r="K2" s="254"/>
-      <c r="L2" s="254"/>
-      <c r="M2" s="254"/>
-      <c r="N2" s="254"/>
+      <c r="C2" s="265"/>
+      <c r="D2" s="265"/>
+      <c r="E2" s="265"/>
+      <c r="F2" s="265"/>
+      <c r="G2" s="265"/>
+      <c r="H2" s="265"/>
+      <c r="I2" s="265"/>
+      <c r="J2" s="265"/>
+      <c r="K2" s="265"/>
+      <c r="L2" s="265"/>
+      <c r="M2" s="265"/>
+      <c r="N2" s="265"/>
     </row>
     <row r="3" spans="2:14" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="255" t="s">
+      <c r="B3" s="266" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="255"/>
-      <c r="D3" s="255"/>
-      <c r="E3" s="255"/>
-      <c r="F3" s="255"/>
-      <c r="G3" s="255"/>
-      <c r="H3" s="255"/>
-      <c r="I3" s="255"/>
-      <c r="J3" s="255"/>
-      <c r="K3" s="255"/>
-      <c r="L3" s="255"/>
-      <c r="M3" s="255"/>
-      <c r="N3" s="255"/>
+      <c r="C3" s="266"/>
+      <c r="D3" s="266"/>
+      <c r="E3" s="266"/>
+      <c r="F3" s="266"/>
+      <c r="G3" s="266"/>
+      <c r="H3" s="266"/>
+      <c r="I3" s="266"/>
+      <c r="J3" s="266"/>
+      <c r="K3" s="266"/>
+      <c r="L3" s="266"/>
+      <c r="M3" s="266"/>
+      <c r="N3" s="266"/>
     </row>
     <row r="4" spans="2:14" ht="7.2" customHeight="1"/>
     <row r="5" spans="2:14" s="17" customFormat="1" ht="37.200000000000003" customHeight="1">
       <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="258" t="s">
+      <c r="C5" s="269" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="258"/>
+      <c r="D5" s="269"/>
       <c r="E5" s="38" t="s">
         <v>8</v>
       </c>
@@ -16281,23 +16327,23 @@
     <mergeCell ref="B1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:N16997">
-    <cfRule type="expression" dxfId="22" priority="1">
+    <cfRule type="expression" dxfId="25" priority="1">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="2">
+    <cfRule type="expression" dxfId="24" priority="2">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="5">
+    <cfRule type="expression" dxfId="23" priority="5">
       <formula>AND($B6="",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H16997">
-    <cfRule type="expression" dxfId="19" priority="9">
+    <cfRule type="expression" dxfId="22" priority="9">
       <formula>IF(G6&lt;&gt;"", NOT(AND(OR(LEFT($E6,2)="L.", LEFT($E6,2)="A.", LEFT($E6,2)="B.", LEFT($E6,2)="M."), $H6&lt;&gt;"", $E6&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:K16997">
-    <cfRule type="notContainsBlanks" dxfId="18" priority="8">
+    <cfRule type="notContainsBlanks" dxfId="21" priority="8">
       <formula>LEN(TRIM(H6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16324,35 +16370,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="123" customHeight="1">
-      <c r="B1" s="257"/>
-      <c r="C1" s="257"/>
-      <c r="D1" s="257"/>
-      <c r="E1" s="257"/>
-      <c r="F1" s="257"/>
-      <c r="G1" s="257"/>
-      <c r="H1" s="257"/>
+      <c r="B1" s="268"/>
+      <c r="C1" s="268"/>
+      <c r="D1" s="268"/>
+      <c r="E1" s="268"/>
+      <c r="F1" s="268"/>
+      <c r="G1" s="268"/>
+      <c r="H1" s="268"/>
     </row>
     <row r="2" spans="2:10" ht="22.8" customHeight="1">
-      <c r="B2" s="254" t="s">
+      <c r="B2" s="265" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="254"/>
-      <c r="D2" s="254"/>
-      <c r="E2" s="254"/>
-      <c r="F2" s="254"/>
-      <c r="G2" s="254"/>
-      <c r="H2" s="254"/>
+      <c r="C2" s="265"/>
+      <c r="D2" s="265"/>
+      <c r="E2" s="265"/>
+      <c r="F2" s="265"/>
+      <c r="G2" s="265"/>
+      <c r="H2" s="265"/>
     </row>
     <row r="3" spans="2:10" ht="17.399999999999999" customHeight="1">
-      <c r="B3" s="255" t="s">
+      <c r="B3" s="266" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="255"/>
-      <c r="D3" s="255"/>
-      <c r="E3" s="255"/>
-      <c r="F3" s="255"/>
-      <c r="G3" s="255"/>
-      <c r="H3" s="255"/>
+      <c r="C3" s="266"/>
+      <c r="D3" s="266"/>
+      <c r="E3" s="266"/>
+      <c r="F3" s="266"/>
+      <c r="G3" s="266"/>
+      <c r="H3" s="266"/>
     </row>
     <row r="4" spans="2:10" ht="8.4" customHeight="1">
       <c r="G4" s="52"/>
@@ -40400,19 +40446,16 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B995 E6:H995">
-    <cfRule type="expression" dxfId="17" priority="7">
+    <cfRule type="expression" dxfId="6" priority="7">
       <formula>$J6=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:H995">
-    <cfRule type="expression" dxfId="16" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>AND(LEN($B6)=1,$C6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="2">
-      <formula>AND($C6="",$B6&lt;&gt;"")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="3">
-      <formula>AND($B6&lt;&gt;"",$C6&lt;&gt;"")</formula>
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>$C6&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -40446,30 +40489,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="111.6" customHeight="1">
-      <c r="B1" s="261"/>
-      <c r="C1" s="261"/>
-      <c r="D1" s="261"/>
-      <c r="E1" s="261"/>
-      <c r="F1" s="261"/>
-      <c r="G1" s="261"/>
-      <c r="H1" s="261"/>
-      <c r="I1" s="261"/>
-      <c r="J1" s="261"/>
-      <c r="K1" s="261"/>
+      <c r="B1" s="272"/>
+      <c r="C1" s="272"/>
+      <c r="D1" s="272"/>
+      <c r="E1" s="272"/>
+      <c r="F1" s="272"/>
+      <c r="G1" s="272"/>
+      <c r="H1" s="272"/>
+      <c r="I1" s="272"/>
+      <c r="J1" s="272"/>
+      <c r="K1" s="272"/>
     </row>
     <row r="2" spans="2:11" ht="22.95" customHeight="1">
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="270" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="260"/>
-      <c r="D2" s="260"/>
-      <c r="E2" s="260"/>
-      <c r="F2" s="260"/>
-      <c r="G2" s="260"/>
-      <c r="H2" s="260"/>
-      <c r="I2" s="260"/>
-      <c r="J2" s="260"/>
-      <c r="K2" s="260"/>
+      <c r="C2" s="271"/>
+      <c r="D2" s="271"/>
+      <c r="E2" s="271"/>
+      <c r="F2" s="271"/>
+      <c r="G2" s="271"/>
+      <c r="H2" s="271"/>
+      <c r="I2" s="271"/>
+      <c r="J2" s="271"/>
+      <c r="K2" s="271"/>
     </row>
     <row r="3" spans="2:11" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40589,11 +40632,11 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="258" t="s">
+      <c r="C11" s="269" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="258"/>
-      <c r="E11" s="258"/>
+      <c r="D11" s="269"/>
+      <c r="E11" s="269"/>
       <c r="F11" s="38" t="s">
         <v>26</v>
       </c>
@@ -40649,26 +40692,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="111.6" customHeight="1">
-      <c r="B1" s="261"/>
-      <c r="C1" s="261"/>
-      <c r="D1" s="261"/>
-      <c r="E1" s="261"/>
-      <c r="F1" s="261"/>
-      <c r="G1" s="261"/>
-      <c r="H1" s="261"/>
-      <c r="I1" s="261"/>
+      <c r="B1" s="272"/>
+      <c r="C1" s="272"/>
+      <c r="D1" s="272"/>
+      <c r="E1" s="272"/>
+      <c r="F1" s="272"/>
+      <c r="G1" s="272"/>
+      <c r="H1" s="272"/>
+      <c r="I1" s="272"/>
     </row>
     <row r="2" spans="2:9" ht="22.95" customHeight="1">
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="270" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="260"/>
-      <c r="D2" s="260"/>
-      <c r="E2" s="260"/>
-      <c r="F2" s="260"/>
-      <c r="G2" s="260"/>
-      <c r="H2" s="260"/>
-      <c r="I2" s="260"/>
+      <c r="C2" s="271"/>
+      <c r="D2" s="271"/>
+      <c r="E2" s="271"/>
+      <c r="F2" s="271"/>
+      <c r="G2" s="271"/>
+      <c r="H2" s="271"/>
+      <c r="I2" s="271"/>
     </row>
     <row r="3" spans="2:9" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -40778,12 +40821,12 @@
       <c r="B11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="258" t="s">
+      <c r="C11" s="269" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="258"/>
-      <c r="E11" s="258"/>
-      <c r="F11" s="258"/>
+      <c r="D11" s="269"/>
+      <c r="E11" s="269"/>
+      <c r="F11" s="269"/>
       <c r="G11" s="40" t="s">
         <v>29</v>
       </c>
@@ -40821,58 +40864,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="100.05" customHeight="1">
-      <c r="B1" s="261"/>
-      <c r="C1" s="261"/>
-      <c r="D1" s="261"/>
-      <c r="E1" s="261"/>
-      <c r="F1" s="261"/>
+      <c r="B1" s="272"/>
+      <c r="C1" s="272"/>
+      <c r="D1" s="272"/>
+      <c r="E1" s="272"/>
+      <c r="F1" s="272"/>
     </row>
     <row r="2" spans="2:12" ht="18">
-      <c r="B2" s="264" t="s">
+      <c r="B2" s="275" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="264"/>
-      <c r="D2" s="264"/>
-      <c r="E2" s="264"/>
-      <c r="F2" s="264"/>
+      <c r="C2" s="275"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
     </row>
     <row r="3" spans="2:12">
-      <c r="B3" s="261"/>
-      <c r="C3" s="261"/>
-      <c r="D3" s="261"/>
-      <c r="E3" s="261"/>
-      <c r="F3" s="261"/>
+      <c r="B3" s="272"/>
+      <c r="C3" s="272"/>
+      <c r="D3" s="272"/>
+      <c r="E3" s="272"/>
+      <c r="F3" s="272"/>
     </row>
     <row r="5" spans="2:12" s="58" customFormat="1">
-      <c r="B5" s="262" t="s">
+      <c r="B5" s="273" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="262" t="s">
+      <c r="C5" s="273" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="262" t="s">
+      <c r="D5" s="273" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="263" t="s">
+      <c r="E5" s="274" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="263" t="s">
+      <c r="F5" s="274" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="58" customFormat="1">
-      <c r="B6" s="262"/>
-      <c r="C6" s="262"/>
-      <c r="D6" s="262"/>
-      <c r="E6" s="263"/>
-      <c r="F6" s="263"/>
+      <c r="B6" s="273"/>
+      <c r="C6" s="273"/>
+      <c r="D6" s="273"/>
+      <c r="E6" s="274"/>
+      <c r="F6" s="274"/>
     </row>
     <row r="7" spans="2:12" s="72" customFormat="1">
-      <c r="B7" s="262"/>
-      <c r="C7" s="262"/>
-      <c r="D7" s="262"/>
-      <c r="E7" s="263"/>
-      <c r="F7" s="263"/>
+      <c r="B7" s="273"/>
+      <c r="C7" s="273"/>
+      <c r="D7" s="273"/>
+      <c r="E7" s="274"/>
+      <c r="F7" s="274"/>
       <c r="G7" s="75"/>
       <c r="H7" s="75"/>
       <c r="I7" s="75"/>
@@ -40920,39 +40963,39 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:CE7">
-    <cfRule type="expression" dxfId="13" priority="12">
+    <cfRule type="expression" dxfId="20" priority="12">
       <formula>B5&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:CE201">
-    <cfRule type="expression" dxfId="12" priority="1">
+    <cfRule type="expression" dxfId="19" priority="1">
       <formula>AND(G8&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="2">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>AND(G$7&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="3">
+    <cfRule type="expression" dxfId="17" priority="3">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="4">
+    <cfRule type="expression" dxfId="16" priority="4">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="5">
+    <cfRule type="expression" dxfId="15" priority="5">
       <formula>AND(G8&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="14" priority="6">
       <formula>AND(G$7&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="7">
+    <cfRule type="expression" dxfId="13" priority="7">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="8">
+    <cfRule type="expression" dxfId="12" priority="8">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="10">
+    <cfRule type="expression" dxfId="10" priority="10">
       <formula>AND(G$7&lt;&gt;"",$B8="DEVIASI")</formula>
     </cfRule>
     <cfRule type="colorScale" priority="11">
@@ -40993,45 +41036,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="232"/>
-      <c r="C1" s="233"/>
-      <c r="D1" s="233"/>
-      <c r="E1" s="233"/>
-      <c r="F1" s="233"/>
-      <c r="G1" s="233"/>
-      <c r="H1" s="233"/>
-      <c r="I1" s="233"/>
-      <c r="J1" s="233"/>
-      <c r="K1" s="233"/>
-      <c r="L1" s="234"/>
+      <c r="B1" s="160"/>
+      <c r="C1" s="161"/>
+      <c r="D1" s="161"/>
+      <c r="E1" s="161"/>
+      <c r="F1" s="161"/>
+      <c r="G1" s="161"/>
+      <c r="H1" s="161"/>
+      <c r="I1" s="161"/>
+      <c r="J1" s="161"/>
+      <c r="K1" s="161"/>
+      <c r="L1" s="162"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="235" t="s">
+      <c r="B2" s="163" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
-      <c r="F2" s="236"/>
-      <c r="G2" s="236"/>
-      <c r="H2" s="236"/>
-      <c r="I2" s="237"/>
-      <c r="J2" s="241"/>
-      <c r="K2" s="242"/>
-      <c r="L2" s="243"/>
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
+      <c r="F2" s="164"/>
+      <c r="G2" s="164"/>
+      <c r="H2" s="164"/>
+      <c r="I2" s="165"/>
+      <c r="J2" s="169"/>
+      <c r="K2" s="170"/>
+      <c r="L2" s="171"/>
     </row>
     <row r="3" spans="1:13" ht="14.4" customHeight="1">
-      <c r="B3" s="238"/>
-      <c r="C3" s="239"/>
-      <c r="D3" s="239"/>
-      <c r="E3" s="239"/>
-      <c r="F3" s="239"/>
-      <c r="G3" s="239"/>
-      <c r="H3" s="239"/>
-      <c r="I3" s="240"/>
-      <c r="J3" s="244"/>
-      <c r="K3" s="245"/>
-      <c r="L3" s="246"/>
+      <c r="B3" s="166"/>
+      <c r="C3" s="167"/>
+      <c r="D3" s="167"/>
+      <c r="E3" s="167"/>
+      <c r="F3" s="167"/>
+      <c r="G3" s="167"/>
+      <c r="H3" s="167"/>
+      <c r="I3" s="168"/>
+      <c r="J3" s="172"/>
+      <c r="K3" s="173"/>
+      <c r="L3" s="174"/>
     </row>
     <row r="4" spans="1:13" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -41042,9 +41085,9 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="244"/>
-      <c r="K4" s="245"/>
-      <c r="L4" s="246"/>
+      <c r="J4" s="172"/>
+      <c r="K4" s="173"/>
+      <c r="L4" s="174"/>
     </row>
     <row r="5" spans="1:13" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -41059,9 +41102,9 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="244"/>
-      <c r="K5" s="245"/>
-      <c r="L5" s="246"/>
+      <c r="J5" s="172"/>
+      <c r="K5" s="173"/>
+      <c r="L5" s="174"/>
     </row>
     <row r="6" spans="1:13" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -41076,9 +41119,9 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="247"/>
-      <c r="K6" s="248"/>
-      <c r="L6" s="249"/>
+      <c r="J6" s="175"/>
+      <c r="K6" s="176"/>
+      <c r="L6" s="177"/>
     </row>
     <row r="7" spans="1:13" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -41134,41 +41177,41 @@
       <c r="L9" s="89"/>
     </row>
     <row r="10" spans="1:13" ht="15.6">
-      <c r="B10" s="250" t="s">
+      <c r="B10" s="178" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="251"/>
-      <c r="D10" s="251"/>
-      <c r="E10" s="251"/>
-      <c r="F10" s="252"/>
-      <c r="G10" s="251" t="s">
+      <c r="C10" s="179"/>
+      <c r="D10" s="179"/>
+      <c r="E10" s="179"/>
+      <c r="F10" s="180"/>
+      <c r="G10" s="179" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="251"/>
-      <c r="I10" s="251"/>
-      <c r="J10" s="252"/>
-      <c r="K10" s="251" t="s">
+      <c r="H10" s="179"/>
+      <c r="I10" s="179"/>
+      <c r="J10" s="180"/>
+      <c r="K10" s="179" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="253"/>
+      <c r="L10" s="181"/>
     </row>
     <row r="11" spans="1:13" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="200" t="s">
+      <c r="C11" s="204" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="201"/>
-      <c r="E11" s="201"/>
+      <c r="D11" s="205"/>
+      <c r="E11" s="205"/>
       <c r="F11" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="200" t="s">
+      <c r="G11" s="204" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="202"/>
+      <c r="H11" s="206"/>
       <c r="I11" s="92" t="s">
         <v>27</v>
       </c>
@@ -41187,233 +41230,233 @@
       <c r="B12" s="94" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="160" t="s">
+      <c r="C12" s="250" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="161"/>
-      <c r="E12" s="162"/>
-      <c r="F12" s="299"/>
-      <c r="G12" s="209"/>
-      <c r="H12" s="210"/>
-      <c r="I12" s="297"/>
-      <c r="J12" s="304"/>
-      <c r="K12" s="305"/>
-      <c r="L12" s="301"/>
+      <c r="D12" s="251"/>
+      <c r="E12" s="252"/>
+      <c r="F12" s="151"/>
+      <c r="G12" s="213"/>
+      <c r="H12" s="214"/>
+      <c r="I12" s="149"/>
+      <c r="J12" s="156"/>
+      <c r="K12" s="157"/>
+      <c r="L12" s="153"/>
     </row>
     <row r="13" spans="1:13" ht="15.6">
       <c r="B13" s="95">
         <v>1</v>
       </c>
-      <c r="C13" s="154" t="s">
+      <c r="C13" s="253" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="155"/>
-      <c r="E13" s="156"/>
-      <c r="F13" s="300"/>
-      <c r="G13" s="211"/>
-      <c r="H13" s="212"/>
-      <c r="I13" s="298"/>
-      <c r="J13" s="306"/>
-      <c r="K13" s="307"/>
-      <c r="L13" s="302"/>
+      <c r="D13" s="254"/>
+      <c r="E13" s="255"/>
+      <c r="F13" s="152"/>
+      <c r="G13" s="215"/>
+      <c r="H13" s="216"/>
+      <c r="I13" s="150"/>
+      <c r="J13" s="96"/>
+      <c r="K13" s="158"/>
+      <c r="L13" s="154"/>
     </row>
     <row r="14" spans="1:13" ht="15.6">
       <c r="B14" s="95">
         <v>2</v>
       </c>
-      <c r="C14" s="154" t="s">
+      <c r="C14" s="253" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="155"/>
-      <c r="E14" s="156"/>
-      <c r="F14" s="300"/>
-      <c r="G14" s="211"/>
-      <c r="H14" s="212"/>
-      <c r="I14" s="298"/>
-      <c r="J14" s="306"/>
-      <c r="K14" s="307"/>
-      <c r="L14" s="302"/>
+      <c r="D14" s="254"/>
+      <c r="E14" s="255"/>
+      <c r="F14" s="152"/>
+      <c r="G14" s="215"/>
+      <c r="H14" s="216"/>
+      <c r="I14" s="150"/>
+      <c r="J14" s="96"/>
+      <c r="K14" s="158"/>
+      <c r="L14" s="154"/>
     </row>
     <row r="15" spans="1:13" ht="15.6">
       <c r="B15" s="95">
         <v>3</v>
       </c>
-      <c r="C15" s="154" t="s">
+      <c r="C15" s="253" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="155"/>
-      <c r="E15" s="156"/>
-      <c r="F15" s="300"/>
-      <c r="G15" s="211"/>
-      <c r="H15" s="212"/>
-      <c r="I15" s="298"/>
-      <c r="J15" s="306"/>
-      <c r="K15" s="307"/>
-      <c r="L15" s="302"/>
+      <c r="D15" s="254"/>
+      <c r="E15" s="255"/>
+      <c r="F15" s="152"/>
+      <c r="G15" s="215"/>
+      <c r="H15" s="216"/>
+      <c r="I15" s="150"/>
+      <c r="J15" s="96"/>
+      <c r="K15" s="158"/>
+      <c r="L15" s="154"/>
     </row>
     <row r="16" spans="1:13" ht="15.6">
       <c r="B16" s="95">
         <v>4</v>
       </c>
-      <c r="C16" s="154" t="s">
+      <c r="C16" s="253" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="155"/>
-      <c r="E16" s="156"/>
-      <c r="F16" s="300"/>
-      <c r="G16" s="211"/>
-      <c r="H16" s="212"/>
-      <c r="I16" s="298"/>
-      <c r="J16" s="306"/>
-      <c r="K16" s="307"/>
-      <c r="L16" s="302"/>
+      <c r="D16" s="254"/>
+      <c r="E16" s="255"/>
+      <c r="F16" s="152"/>
+      <c r="G16" s="215"/>
+      <c r="H16" s="216"/>
+      <c r="I16" s="150"/>
+      <c r="J16" s="96"/>
+      <c r="K16" s="158"/>
+      <c r="L16" s="154"/>
     </row>
     <row r="17" spans="1:12" ht="15.6">
       <c r="B17" s="95">
         <v>5</v>
       </c>
-      <c r="C17" s="154" t="s">
+      <c r="C17" s="253" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="155"/>
-      <c r="E17" s="156"/>
-      <c r="F17" s="300"/>
-      <c r="G17" s="211"/>
-      <c r="H17" s="212"/>
-      <c r="I17" s="298"/>
-      <c r="J17" s="306"/>
-      <c r="K17" s="307"/>
-      <c r="L17" s="302"/>
+      <c r="D17" s="254"/>
+      <c r="E17" s="255"/>
+      <c r="F17" s="152"/>
+      <c r="G17" s="215"/>
+      <c r="H17" s="216"/>
+      <c r="I17" s="150"/>
+      <c r="J17" s="96"/>
+      <c r="K17" s="158"/>
+      <c r="L17" s="154"/>
     </row>
     <row r="18" spans="1:12" ht="15.6">
       <c r="B18" s="95">
         <v>6</v>
       </c>
-      <c r="C18" s="154" t="s">
+      <c r="C18" s="253" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="155"/>
-      <c r="E18" s="156"/>
-      <c r="F18" s="300"/>
-      <c r="G18" s="211"/>
-      <c r="H18" s="212"/>
-      <c r="I18" s="298"/>
-      <c r="J18" s="306"/>
-      <c r="K18" s="307"/>
-      <c r="L18" s="302"/>
+      <c r="D18" s="254"/>
+      <c r="E18" s="255"/>
+      <c r="F18" s="152"/>
+      <c r="G18" s="215"/>
+      <c r="H18" s="216"/>
+      <c r="I18" s="150"/>
+      <c r="J18" s="96"/>
+      <c r="K18" s="158"/>
+      <c r="L18" s="154"/>
     </row>
     <row r="19" spans="1:12" ht="15.6">
       <c r="B19" s="97" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="157" t="s">
+      <c r="C19" s="259" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="158"/>
-      <c r="E19" s="159"/>
-      <c r="F19" s="300"/>
-      <c r="G19" s="211"/>
-      <c r="H19" s="212"/>
-      <c r="I19" s="298"/>
-      <c r="J19" s="306"/>
-      <c r="K19" s="307"/>
-      <c r="L19" s="302"/>
+      <c r="D19" s="260"/>
+      <c r="E19" s="261"/>
+      <c r="F19" s="152"/>
+      <c r="G19" s="215"/>
+      <c r="H19" s="216"/>
+      <c r="I19" s="150"/>
+      <c r="J19" s="96"/>
+      <c r="K19" s="158"/>
+      <c r="L19" s="154"/>
     </row>
     <row r="20" spans="1:12" ht="15.6">
       <c r="B20" s="95">
         <v>1</v>
       </c>
-      <c r="C20" s="154" t="s">
+      <c r="C20" s="253" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="155"/>
-      <c r="E20" s="156"/>
-      <c r="F20" s="300"/>
-      <c r="G20" s="211"/>
-      <c r="H20" s="212"/>
-      <c r="I20" s="298"/>
-      <c r="J20" s="306"/>
-      <c r="K20" s="307"/>
-      <c r="L20" s="302"/>
+      <c r="D20" s="254"/>
+      <c r="E20" s="255"/>
+      <c r="F20" s="152"/>
+      <c r="G20" s="215"/>
+      <c r="H20" s="216"/>
+      <c r="I20" s="150"/>
+      <c r="J20" s="96"/>
+      <c r="K20" s="158"/>
+      <c r="L20" s="154"/>
     </row>
     <row r="21" spans="1:12" ht="15.6">
       <c r="B21" s="95">
         <v>2</v>
       </c>
-      <c r="C21" s="154" t="s">
+      <c r="C21" s="253" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="155"/>
-      <c r="E21" s="156"/>
-      <c r="F21" s="300"/>
-      <c r="G21" s="211"/>
-      <c r="H21" s="212"/>
-      <c r="I21" s="298"/>
-      <c r="J21" s="306"/>
-      <c r="K21" s="307"/>
-      <c r="L21" s="302"/>
+      <c r="D21" s="254"/>
+      <c r="E21" s="255"/>
+      <c r="F21" s="152"/>
+      <c r="G21" s="215"/>
+      <c r="H21" s="216"/>
+      <c r="I21" s="150"/>
+      <c r="J21" s="96"/>
+      <c r="K21" s="158"/>
+      <c r="L21" s="154"/>
     </row>
     <row r="22" spans="1:12" ht="15.6">
       <c r="B22" s="95">
         <v>3</v>
       </c>
-      <c r="C22" s="149" t="s">
+      <c r="C22" s="256" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="150"/>
-      <c r="E22" s="151"/>
-      <c r="F22" s="300"/>
-      <c r="G22" s="213"/>
-      <c r="H22" s="214"/>
-      <c r="I22" s="298"/>
-      <c r="J22" s="306"/>
-      <c r="K22" s="308"/>
-      <c r="L22" s="303"/>
+      <c r="D22" s="257"/>
+      <c r="E22" s="258"/>
+      <c r="F22" s="152"/>
+      <c r="G22" s="217"/>
+      <c r="H22" s="218"/>
+      <c r="I22" s="150"/>
+      <c r="J22" s="96"/>
+      <c r="K22" s="159"/>
+      <c r="L22" s="155"/>
     </row>
     <row r="23" spans="1:12" ht="16.2" thickBot="1">
-      <c r="B23" s="203"/>
-      <c r="C23" s="204"/>
-      <c r="D23" s="204"/>
-      <c r="E23" s="204"/>
+      <c r="B23" s="207"/>
+      <c r="C23" s="208"/>
+      <c r="D23" s="208"/>
+      <c r="E23" s="208"/>
       <c r="F23" s="98"/>
       <c r="G23" s="98"/>
       <c r="H23" s="99"/>
       <c r="I23" s="99"/>
-      <c r="J23" s="205"/>
-      <c r="K23" s="205"/>
-      <c r="L23" s="206"/>
+      <c r="J23" s="209"/>
+      <c r="K23" s="209"/>
+      <c r="L23" s="210"/>
     </row>
     <row r="24" spans="1:12" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="207" t="s">
+      <c r="B24" s="211" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="215" t="s">
+      <c r="C24" s="182" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="215"/>
-      <c r="E24" s="215"/>
-      <c r="F24" s="215"/>
-      <c r="G24" s="215"/>
-      <c r="H24" s="215"/>
-      <c r="I24" s="215"/>
-      <c r="J24" s="217" t="s">
+      <c r="D24" s="182"/>
+      <c r="E24" s="182"/>
+      <c r="F24" s="182"/>
+      <c r="G24" s="182"/>
+      <c r="H24" s="182"/>
+      <c r="I24" s="182"/>
+      <c r="J24" s="184" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="218"/>
-      <c r="L24" s="219"/>
+      <c r="K24" s="185"/>
+      <c r="L24" s="186"/>
     </row>
     <row r="25" spans="1:12" ht="31.2">
-      <c r="B25" s="208"/>
-      <c r="C25" s="216"/>
-      <c r="D25" s="216"/>
-      <c r="E25" s="216"/>
-      <c r="F25" s="216"/>
-      <c r="G25" s="216"/>
-      <c r="H25" s="216"/>
-      <c r="I25" s="216"/>
+      <c r="B25" s="212"/>
+      <c r="C25" s="183"/>
+      <c r="D25" s="183"/>
+      <c r="E25" s="183"/>
+      <c r="F25" s="183"/>
+      <c r="G25" s="183"/>
+      <c r="H25" s="183"/>
+      <c r="I25" s="183"/>
       <c r="J25" s="137" t="s">
         <v>9</v>
       </c>
@@ -41426,52 +41469,52 @@
     </row>
     <row r="26" spans="1:12" ht="15.6">
       <c r="B26" s="100"/>
-      <c r="C26" s="229"/>
-      <c r="D26" s="230"/>
-      <c r="E26" s="230"/>
-      <c r="F26" s="230"/>
-      <c r="G26" s="230"/>
-      <c r="H26" s="230"/>
-      <c r="I26" s="231"/>
+      <c r="C26" s="198"/>
+      <c r="D26" s="199"/>
+      <c r="E26" s="199"/>
+      <c r="F26" s="199"/>
+      <c r="G26" s="199"/>
+      <c r="H26" s="199"/>
+      <c r="I26" s="200"/>
       <c r="J26" s="138"/>
       <c r="K26" s="146"/>
       <c r="L26" s="144"/>
     </row>
     <row r="27" spans="1:12" ht="15.6">
       <c r="B27" s="100"/>
-      <c r="C27" s="163"/>
-      <c r="D27" s="164"/>
-      <c r="E27" s="164"/>
-      <c r="F27" s="164"/>
-      <c r="G27" s="164"/>
-      <c r="H27" s="164"/>
-      <c r="I27" s="165"/>
+      <c r="C27" s="201"/>
+      <c r="D27" s="202"/>
+      <c r="E27" s="202"/>
+      <c r="F27" s="202"/>
+      <c r="G27" s="202"/>
+      <c r="H27" s="202"/>
+      <c r="I27" s="203"/>
       <c r="J27" s="96"/>
       <c r="K27" s="147"/>
       <c r="L27" s="144"/>
     </row>
     <row r="28" spans="1:12" ht="15.6">
       <c r="B28" s="100"/>
-      <c r="C28" s="163"/>
-      <c r="D28" s="164"/>
-      <c r="E28" s="164"/>
-      <c r="F28" s="164"/>
-      <c r="G28" s="164"/>
-      <c r="H28" s="164"/>
-      <c r="I28" s="165"/>
+      <c r="C28" s="201"/>
+      <c r="D28" s="202"/>
+      <c r="E28" s="202"/>
+      <c r="F28" s="202"/>
+      <c r="G28" s="202"/>
+      <c r="H28" s="202"/>
+      <c r="I28" s="203"/>
       <c r="J28" s="96"/>
       <c r="K28" s="147"/>
       <c r="L28" s="145"/>
     </row>
     <row r="29" spans="1:12" ht="15.6">
       <c r="B29" s="100"/>
-      <c r="C29" s="163"/>
-      <c r="D29" s="164"/>
-      <c r="E29" s="164"/>
-      <c r="F29" s="164"/>
-      <c r="G29" s="164"/>
-      <c r="H29" s="164"/>
-      <c r="I29" s="165"/>
+      <c r="C29" s="201"/>
+      <c r="D29" s="202"/>
+      <c r="E29" s="202"/>
+      <c r="F29" s="202"/>
+      <c r="G29" s="202"/>
+      <c r="H29" s="202"/>
+      <c r="I29" s="203"/>
       <c r="J29" s="96"/>
       <c r="K29" s="147"/>
       <c r="L29" s="145"/>
@@ -41480,15 +41523,15 @@
       <c r="B30" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="163" t="s">
+      <c r="C30" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="164"/>
-      <c r="E30" s="164"/>
-      <c r="F30" s="164"/>
-      <c r="G30" s="164"/>
-      <c r="H30" s="164"/>
-      <c r="I30" s="165"/>
+      <c r="D30" s="202"/>
+      <c r="E30" s="202"/>
+      <c r="F30" s="202"/>
+      <c r="G30" s="202"/>
+      <c r="H30" s="202"/>
+      <c r="I30" s="203"/>
       <c r="J30" s="96" t="s">
         <v>64</v>
       </c>
@@ -41501,15 +41544,15 @@
       <c r="B31" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="163" t="s">
+      <c r="C31" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="164"/>
-      <c r="E31" s="164"/>
-      <c r="F31" s="164"/>
-      <c r="G31" s="164"/>
-      <c r="H31" s="164"/>
-      <c r="I31" s="165"/>
+      <c r="D31" s="202"/>
+      <c r="E31" s="202"/>
+      <c r="F31" s="202"/>
+      <c r="G31" s="202"/>
+      <c r="H31" s="202"/>
+      <c r="I31" s="203"/>
       <c r="J31" s="96" t="s">
         <v>64</v>
       </c>
@@ -41522,15 +41565,15 @@
       <c r="B32" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="163" t="s">
+      <c r="C32" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="164"/>
-      <c r="E32" s="164"/>
-      <c r="F32" s="164"/>
-      <c r="G32" s="164"/>
-      <c r="H32" s="164"/>
-      <c r="I32" s="165"/>
+      <c r="D32" s="202"/>
+      <c r="E32" s="202"/>
+      <c r="F32" s="202"/>
+      <c r="G32" s="202"/>
+      <c r="H32" s="202"/>
+      <c r="I32" s="203"/>
       <c r="J32" s="96" t="s">
         <v>64</v>
       </c>
@@ -41543,15 +41586,15 @@
       <c r="B33" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="163" t="s">
+      <c r="C33" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="164"/>
-      <c r="E33" s="164"/>
-      <c r="F33" s="164"/>
-      <c r="G33" s="164"/>
-      <c r="H33" s="164"/>
-      <c r="I33" s="165"/>
+      <c r="D33" s="202"/>
+      <c r="E33" s="202"/>
+      <c r="F33" s="202"/>
+      <c r="G33" s="202"/>
+      <c r="H33" s="202"/>
+      <c r="I33" s="203"/>
       <c r="J33" s="96" t="s">
         <v>64</v>
       </c>
@@ -41564,15 +41607,15 @@
       <c r="B34" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="163" t="s">
+      <c r="C34" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="164"/>
-      <c r="E34" s="164"/>
-      <c r="F34" s="164"/>
-      <c r="G34" s="164"/>
-      <c r="H34" s="164"/>
-      <c r="I34" s="165"/>
+      <c r="D34" s="202"/>
+      <c r="E34" s="202"/>
+      <c r="F34" s="202"/>
+      <c r="G34" s="202"/>
+      <c r="H34" s="202"/>
+      <c r="I34" s="203"/>
       <c r="J34" s="96" t="s">
         <v>64</v>
       </c>
@@ -41585,15 +41628,15 @@
       <c r="B35" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="163" t="s">
+      <c r="C35" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="164"/>
-      <c r="E35" s="164"/>
-      <c r="F35" s="164"/>
-      <c r="G35" s="164"/>
-      <c r="H35" s="164"/>
-      <c r="I35" s="165"/>
+      <c r="D35" s="202"/>
+      <c r="E35" s="202"/>
+      <c r="F35" s="202"/>
+      <c r="G35" s="202"/>
+      <c r="H35" s="202"/>
+      <c r="I35" s="203"/>
       <c r="J35" s="96" t="s">
         <v>64</v>
       </c>
@@ -41606,15 +41649,15 @@
       <c r="B36" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C36" s="163" t="s">
+      <c r="C36" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="164"/>
-      <c r="E36" s="164"/>
-      <c r="F36" s="164"/>
-      <c r="G36" s="164"/>
-      <c r="H36" s="164"/>
-      <c r="I36" s="165"/>
+      <c r="D36" s="202"/>
+      <c r="E36" s="202"/>
+      <c r="F36" s="202"/>
+      <c r="G36" s="202"/>
+      <c r="H36" s="202"/>
+      <c r="I36" s="203"/>
       <c r="J36" s="96" t="s">
         <v>64</v>
       </c>
@@ -41627,15 +41670,15 @@
       <c r="B37" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="163" t="s">
+      <c r="C37" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="164"/>
-      <c r="E37" s="164"/>
-      <c r="F37" s="164"/>
-      <c r="G37" s="164"/>
-      <c r="H37" s="164"/>
-      <c r="I37" s="165"/>
+      <c r="D37" s="202"/>
+      <c r="E37" s="202"/>
+      <c r="F37" s="202"/>
+      <c r="G37" s="202"/>
+      <c r="H37" s="202"/>
+      <c r="I37" s="203"/>
       <c r="J37" s="96" t="s">
         <v>64</v>
       </c>
@@ -41648,15 +41691,15 @@
       <c r="B38" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="163" t="s">
+      <c r="C38" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="164"/>
-      <c r="E38" s="164"/>
-      <c r="F38" s="164"/>
-      <c r="G38" s="164"/>
-      <c r="H38" s="164"/>
-      <c r="I38" s="165"/>
+      <c r="D38" s="202"/>
+      <c r="E38" s="202"/>
+      <c r="F38" s="202"/>
+      <c r="G38" s="202"/>
+      <c r="H38" s="202"/>
+      <c r="I38" s="203"/>
       <c r="J38" s="96" t="s">
         <v>64</v>
       </c>
@@ -41669,15 +41712,15 @@
       <c r="B39" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="163" t="s">
+      <c r="C39" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D39" s="164"/>
-      <c r="E39" s="164"/>
-      <c r="F39" s="164"/>
-      <c r="G39" s="164"/>
-      <c r="H39" s="164"/>
-      <c r="I39" s="165"/>
+      <c r="D39" s="202"/>
+      <c r="E39" s="202"/>
+      <c r="F39" s="202"/>
+      <c r="G39" s="202"/>
+      <c r="H39" s="202"/>
+      <c r="I39" s="203"/>
       <c r="J39" s="96" t="s">
         <v>64</v>
       </c>
@@ -41690,15 +41733,15 @@
       <c r="B40" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="163" t="s">
+      <c r="C40" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D40" s="164"/>
-      <c r="E40" s="164"/>
-      <c r="F40" s="164"/>
-      <c r="G40" s="164"/>
-      <c r="H40" s="164"/>
-      <c r="I40" s="165"/>
+      <c r="D40" s="202"/>
+      <c r="E40" s="202"/>
+      <c r="F40" s="202"/>
+      <c r="G40" s="202"/>
+      <c r="H40" s="202"/>
+      <c r="I40" s="203"/>
       <c r="J40" s="96" t="s">
         <v>64</v>
       </c>
@@ -41711,15 +41754,15 @@
       <c r="B41" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="163" t="s">
+      <c r="C41" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D41" s="164"/>
-      <c r="E41" s="164"/>
-      <c r="F41" s="164"/>
-      <c r="G41" s="164"/>
-      <c r="H41" s="164"/>
-      <c r="I41" s="165"/>
+      <c r="D41" s="202"/>
+      <c r="E41" s="202"/>
+      <c r="F41" s="202"/>
+      <c r="G41" s="202"/>
+      <c r="H41" s="202"/>
+      <c r="I41" s="203"/>
       <c r="J41" s="96" t="s">
         <v>64</v>
       </c>
@@ -41732,15 +41775,15 @@
       <c r="B42" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="163" t="s">
+      <c r="C42" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="164"/>
-      <c r="E42" s="164"/>
-      <c r="F42" s="164"/>
-      <c r="G42" s="164"/>
-      <c r="H42" s="164"/>
-      <c r="I42" s="165"/>
+      <c r="D42" s="202"/>
+      <c r="E42" s="202"/>
+      <c r="F42" s="202"/>
+      <c r="G42" s="202"/>
+      <c r="H42" s="202"/>
+      <c r="I42" s="203"/>
       <c r="J42" s="96" t="s">
         <v>64</v>
       </c>
@@ -41753,15 +41796,15 @@
       <c r="B43" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="163" t="s">
+      <c r="C43" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="164"/>
-      <c r="E43" s="164"/>
-      <c r="F43" s="164"/>
-      <c r="G43" s="164"/>
-      <c r="H43" s="164"/>
-      <c r="I43" s="165"/>
+      <c r="D43" s="202"/>
+      <c r="E43" s="202"/>
+      <c r="F43" s="202"/>
+      <c r="G43" s="202"/>
+      <c r="H43" s="202"/>
+      <c r="I43" s="203"/>
       <c r="J43" s="96" t="s">
         <v>64</v>
       </c>
@@ -41774,15 +41817,15 @@
       <c r="B44" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="163" t="s">
+      <c r="C44" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D44" s="164"/>
-      <c r="E44" s="164"/>
-      <c r="F44" s="164"/>
-      <c r="G44" s="164"/>
-      <c r="H44" s="164"/>
-      <c r="I44" s="165"/>
+      <c r="D44" s="202"/>
+      <c r="E44" s="202"/>
+      <c r="F44" s="202"/>
+      <c r="G44" s="202"/>
+      <c r="H44" s="202"/>
+      <c r="I44" s="203"/>
       <c r="J44" s="96" t="s">
         <v>64</v>
       </c>
@@ -41795,15 +41838,15 @@
       <c r="B45" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C45" s="163" t="s">
+      <c r="C45" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D45" s="164"/>
-      <c r="E45" s="164"/>
-      <c r="F45" s="164"/>
-      <c r="G45" s="164"/>
-      <c r="H45" s="164"/>
-      <c r="I45" s="165"/>
+      <c r="D45" s="202"/>
+      <c r="E45" s="202"/>
+      <c r="F45" s="202"/>
+      <c r="G45" s="202"/>
+      <c r="H45" s="202"/>
+      <c r="I45" s="203"/>
       <c r="J45" s="96" t="s">
         <v>64</v>
       </c>
@@ -41816,15 +41859,15 @@
       <c r="B46" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C46" s="163" t="s">
+      <c r="C46" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="164"/>
-      <c r="E46" s="164"/>
-      <c r="F46" s="164"/>
-      <c r="G46" s="164"/>
-      <c r="H46" s="164"/>
-      <c r="I46" s="165"/>
+      <c r="D46" s="202"/>
+      <c r="E46" s="202"/>
+      <c r="F46" s="202"/>
+      <c r="G46" s="202"/>
+      <c r="H46" s="202"/>
+      <c r="I46" s="203"/>
       <c r="J46" s="96" t="s">
         <v>64</v>
       </c>
@@ -41837,15 +41880,15 @@
       <c r="B47" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="163" t="s">
+      <c r="C47" s="201" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="164"/>
-      <c r="E47" s="164"/>
-      <c r="F47" s="164"/>
-      <c r="G47" s="164"/>
-      <c r="H47" s="164"/>
-      <c r="I47" s="165"/>
+      <c r="D47" s="202"/>
+      <c r="E47" s="202"/>
+      <c r="F47" s="202"/>
+      <c r="G47" s="202"/>
+      <c r="H47" s="202"/>
+      <c r="I47" s="203"/>
       <c r="J47" s="96" t="s">
         <v>64</v>
       </c>
@@ -41858,15 +41901,15 @@
       <c r="B48" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C48" s="166" t="s">
+      <c r="C48" s="262" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="167"/>
-      <c r="E48" s="167"/>
-      <c r="F48" s="167"/>
-      <c r="G48" s="167"/>
-      <c r="H48" s="167"/>
-      <c r="I48" s="168"/>
+      <c r="D48" s="263"/>
+      <c r="E48" s="263"/>
+      <c r="F48" s="263"/>
+      <c r="G48" s="263"/>
+      <c r="H48" s="263"/>
+      <c r="I48" s="264"/>
       <c r="J48" s="139" t="s">
         <v>64</v>
       </c>
@@ -41876,140 +41919,140 @@
       </c>
     </row>
     <row r="49" spans="2:12" ht="16.2" thickTop="1">
-      <c r="B49" s="182" t="s">
+      <c r="B49" s="232" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="183"/>
-      <c r="D49" s="183"/>
-      <c r="E49" s="183"/>
-      <c r="F49" s="183"/>
-      <c r="G49" s="183"/>
-      <c r="H49" s="183"/>
-      <c r="I49" s="183"/>
-      <c r="J49" s="184"/>
-      <c r="K49" s="227" t="s">
+      <c r="C49" s="233"/>
+      <c r="D49" s="233"/>
+      <c r="E49" s="233"/>
+      <c r="F49" s="233"/>
+      <c r="G49" s="233"/>
+      <c r="H49" s="233"/>
+      <c r="I49" s="233"/>
+      <c r="J49" s="234"/>
+      <c r="K49" s="196" t="s">
         <v>79</v>
       </c>
-      <c r="L49" s="228"/>
+      <c r="L49" s="197"/>
     </row>
     <row r="50" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B50" s="185"/>
-      <c r="C50" s="186"/>
-      <c r="D50" s="186"/>
-      <c r="E50" s="186"/>
-      <c r="F50" s="186"/>
-      <c r="G50" s="186"/>
-      <c r="H50" s="186"/>
-      <c r="I50" s="186"/>
-      <c r="J50" s="187"/>
-      <c r="K50" s="225" t="s">
+      <c r="B50" s="235"/>
+      <c r="C50" s="236"/>
+      <c r="D50" s="236"/>
+      <c r="E50" s="236"/>
+      <c r="F50" s="236"/>
+      <c r="G50" s="236"/>
+      <c r="H50" s="236"/>
+      <c r="I50" s="236"/>
+      <c r="J50" s="237"/>
+      <c r="K50" s="194" t="s">
         <v>103</v>
       </c>
-      <c r="L50" s="226"/>
+      <c r="L50" s="195"/>
     </row>
     <row r="51" spans="2:12" ht="15.6">
       <c r="B51" s="101"/>
-      <c r="C51" s="222"/>
-      <c r="D51" s="222"/>
-      <c r="E51" s="222"/>
-      <c r="F51" s="222"/>
-      <c r="G51" s="222"/>
-      <c r="H51" s="222"/>
-      <c r="I51" s="222"/>
+      <c r="C51" s="191"/>
+      <c r="D51" s="191"/>
+      <c r="E51" s="191"/>
+      <c r="F51" s="191"/>
+      <c r="G51" s="191"/>
+      <c r="H51" s="191"/>
+      <c r="I51" s="191"/>
       <c r="J51" s="102"/>
-      <c r="K51" s="220"/>
-      <c r="L51" s="221"/>
+      <c r="K51" s="189"/>
+      <c r="L51" s="190"/>
     </row>
     <row r="52" spans="2:12" ht="15.6">
       <c r="B52" s="103"/>
-      <c r="C52" s="223"/>
-      <c r="D52" s="223"/>
-      <c r="E52" s="223"/>
-      <c r="F52" s="223"/>
-      <c r="G52" s="223"/>
-      <c r="H52" s="223"/>
-      <c r="I52" s="223"/>
+      <c r="C52" s="192"/>
+      <c r="D52" s="192"/>
+      <c r="E52" s="192"/>
+      <c r="F52" s="192"/>
+      <c r="G52" s="192"/>
+      <c r="H52" s="192"/>
+      <c r="I52" s="192"/>
       <c r="J52" s="104"/>
       <c r="K52" s="115"/>
       <c r="L52" s="105"/>
     </row>
     <row r="53" spans="2:12" ht="15.6">
       <c r="B53" s="106"/>
-      <c r="C53" s="223"/>
-      <c r="D53" s="223"/>
-      <c r="E53" s="223"/>
-      <c r="F53" s="223"/>
-      <c r="G53" s="223"/>
-      <c r="H53" s="223"/>
-      <c r="I53" s="223"/>
+      <c r="C53" s="192"/>
+      <c r="D53" s="192"/>
+      <c r="E53" s="192"/>
+      <c r="F53" s="192"/>
+      <c r="G53" s="192"/>
+      <c r="H53" s="192"/>
+      <c r="I53" s="192"/>
       <c r="J53" s="107"/>
       <c r="K53" s="108"/>
       <c r="L53" s="109"/>
     </row>
     <row r="54" spans="2:12" ht="15.6">
       <c r="B54" s="106"/>
-      <c r="C54" s="223"/>
-      <c r="D54" s="223"/>
-      <c r="E54" s="223"/>
-      <c r="F54" s="223"/>
-      <c r="G54" s="223"/>
-      <c r="H54" s="223"/>
-      <c r="I54" s="223"/>
+      <c r="C54" s="192"/>
+      <c r="D54" s="192"/>
+      <c r="E54" s="192"/>
+      <c r="F54" s="192"/>
+      <c r="G54" s="192"/>
+      <c r="H54" s="192"/>
+      <c r="I54" s="192"/>
       <c r="J54" s="107"/>
       <c r="K54" s="140"/>
       <c r="L54" s="141"/>
     </row>
     <row r="55" spans="2:12" ht="15.6">
       <c r="B55" s="106"/>
-      <c r="C55" s="223"/>
-      <c r="D55" s="223"/>
-      <c r="E55" s="223"/>
-      <c r="F55" s="223"/>
-      <c r="G55" s="223"/>
-      <c r="H55" s="223"/>
-      <c r="I55" s="223"/>
+      <c r="C55" s="192"/>
+      <c r="D55" s="192"/>
+      <c r="E55" s="192"/>
+      <c r="F55" s="192"/>
+      <c r="G55" s="192"/>
+      <c r="H55" s="192"/>
+      <c r="I55" s="192"/>
       <c r="J55" s="107"/>
       <c r="K55" s="140"/>
       <c r="L55" s="141"/>
     </row>
     <row r="56" spans="2:12" ht="15.6">
       <c r="B56" s="106"/>
-      <c r="C56" s="223"/>
-      <c r="D56" s="223"/>
-      <c r="E56" s="223"/>
-      <c r="F56" s="223"/>
-      <c r="G56" s="223"/>
-      <c r="H56" s="223"/>
-      <c r="I56" s="223"/>
+      <c r="C56" s="192"/>
+      <c r="D56" s="192"/>
+      <c r="E56" s="192"/>
+      <c r="F56" s="192"/>
+      <c r="G56" s="192"/>
+      <c r="H56" s="192"/>
+      <c r="I56" s="192"/>
       <c r="J56" s="107"/>
       <c r="K56" s="142"/>
       <c r="L56" s="143"/>
     </row>
     <row r="57" spans="2:12" ht="15.6">
       <c r="B57" s="106"/>
-      <c r="C57" s="223"/>
-      <c r="D57" s="223"/>
-      <c r="E57" s="223"/>
-      <c r="F57" s="223"/>
-      <c r="G57" s="223"/>
-      <c r="H57" s="223"/>
-      <c r="I57" s="223"/>
+      <c r="C57" s="192"/>
+      <c r="D57" s="192"/>
+      <c r="E57" s="192"/>
+      <c r="F57" s="192"/>
+      <c r="G57" s="192"/>
+      <c r="H57" s="192"/>
+      <c r="I57" s="192"/>
       <c r="J57" s="107"/>
       <c r="K57" s="140"/>
       <c r="L57" s="141"/>
     </row>
     <row r="58" spans="2:12" ht="15.6">
       <c r="B58" s="106"/>
-      <c r="C58" s="224"/>
-      <c r="D58" s="224"/>
-      <c r="E58" s="224"/>
-      <c r="F58" s="224"/>
-      <c r="G58" s="224"/>
-      <c r="H58" s="224"/>
-      <c r="I58" s="224"/>
+      <c r="C58" s="193"/>
+      <c r="D58" s="193"/>
+      <c r="E58" s="193"/>
+      <c r="F58" s="193"/>
+      <c r="G58" s="193"/>
+      <c r="H58" s="193"/>
+      <c r="I58" s="193"/>
       <c r="J58" s="107"/>
-      <c r="K58" s="152"/>
-      <c r="L58" s="153"/>
+      <c r="K58" s="187"/>
+      <c r="L58" s="188"/>
     </row>
     <row r="59" spans="2:12" ht="15.6">
       <c r="B59" s="106"/>
@@ -42021,103 +42064,103 @@
       <c r="H59" s="110"/>
       <c r="I59" s="110"/>
       <c r="J59" s="107"/>
-      <c r="K59" s="152"/>
-      <c r="L59" s="153"/>
+      <c r="K59" s="187"/>
+      <c r="L59" s="188"/>
     </row>
     <row r="60" spans="2:12" ht="15.6">
-      <c r="B60" s="169" t="s">
+      <c r="B60" s="219" t="s">
         <v>80</v>
       </c>
-      <c r="C60" s="170"/>
-      <c r="D60" s="170"/>
-      <c r="E60" s="171"/>
-      <c r="F60" s="172" t="s">
+      <c r="C60" s="220"/>
+      <c r="D60" s="220"/>
+      <c r="E60" s="221"/>
+      <c r="F60" s="222" t="s">
         <v>81</v>
       </c>
-      <c r="G60" s="171"/>
-      <c r="H60" s="172" t="s">
+      <c r="G60" s="221"/>
+      <c r="H60" s="222" t="s">
         <v>82</v>
       </c>
-      <c r="I60" s="170"/>
-      <c r="J60" s="171"/>
+      <c r="I60" s="220"/>
+      <c r="J60" s="221"/>
       <c r="K60" s="108"/>
       <c r="L60" s="109"/>
     </row>
     <row r="61" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B61" s="194"/>
-      <c r="C61" s="195"/>
-      <c r="D61" s="195"/>
-      <c r="E61" s="189"/>
-      <c r="F61" s="188"/>
-      <c r="G61" s="189"/>
-      <c r="H61" s="173"/>
-      <c r="I61" s="174"/>
-      <c r="J61" s="175"/>
+      <c r="B61" s="244"/>
+      <c r="C61" s="245"/>
+      <c r="D61" s="245"/>
+      <c r="E61" s="239"/>
+      <c r="F61" s="238"/>
+      <c r="G61" s="239"/>
+      <c r="H61" s="223"/>
+      <c r="I61" s="224"/>
+      <c r="J61" s="225"/>
       <c r="K61" s="108"/>
       <c r="L61" s="109"/>
     </row>
     <row r="62" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B62" s="196"/>
-      <c r="C62" s="197"/>
-      <c r="D62" s="197"/>
-      <c r="E62" s="191"/>
-      <c r="F62" s="190"/>
-      <c r="G62" s="191"/>
-      <c r="H62" s="176"/>
-      <c r="I62" s="177"/>
-      <c r="J62" s="178"/>
+      <c r="B62" s="246"/>
+      <c r="C62" s="247"/>
+      <c r="D62" s="247"/>
+      <c r="E62" s="241"/>
+      <c r="F62" s="240"/>
+      <c r="G62" s="241"/>
+      <c r="H62" s="226"/>
+      <c r="I62" s="227"/>
+      <c r="J62" s="228"/>
       <c r="K62" s="117"/>
       <c r="L62" s="109"/>
     </row>
     <row r="63" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B63" s="196"/>
-      <c r="C63" s="197"/>
-      <c r="D63" s="197"/>
-      <c r="E63" s="191"/>
-      <c r="F63" s="190"/>
-      <c r="G63" s="191"/>
-      <c r="H63" s="176"/>
-      <c r="I63" s="177"/>
-      <c r="J63" s="178"/>
+      <c r="B63" s="246"/>
+      <c r="C63" s="247"/>
+      <c r="D63" s="247"/>
+      <c r="E63" s="241"/>
+      <c r="F63" s="240"/>
+      <c r="G63" s="241"/>
+      <c r="H63" s="226"/>
+      <c r="I63" s="227"/>
+      <c r="J63" s="228"/>
       <c r="K63" s="116"/>
       <c r="L63" s="76"/>
     </row>
     <row r="64" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B64" s="196"/>
-      <c r="C64" s="197"/>
-      <c r="D64" s="197"/>
-      <c r="E64" s="191"/>
-      <c r="F64" s="190"/>
-      <c r="G64" s="191"/>
-      <c r="H64" s="176"/>
-      <c r="I64" s="177"/>
-      <c r="J64" s="178"/>
+      <c r="B64" s="246"/>
+      <c r="C64" s="247"/>
+      <c r="D64" s="247"/>
+      <c r="E64" s="241"/>
+      <c r="F64" s="240"/>
+      <c r="G64" s="241"/>
+      <c r="H64" s="226"/>
+      <c r="I64" s="227"/>
+      <c r="J64" s="228"/>
       <c r="K64" s="118"/>
       <c r="L64" s="119"/>
     </row>
     <row r="65" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B65" s="196"/>
-      <c r="C65" s="197"/>
-      <c r="D65" s="197"/>
-      <c r="E65" s="191"/>
-      <c r="F65" s="190"/>
-      <c r="G65" s="191"/>
-      <c r="H65" s="176"/>
-      <c r="I65" s="177"/>
-      <c r="J65" s="178"/>
+      <c r="B65" s="246"/>
+      <c r="C65" s="247"/>
+      <c r="D65" s="247"/>
+      <c r="E65" s="241"/>
+      <c r="F65" s="240"/>
+      <c r="G65" s="241"/>
+      <c r="H65" s="226"/>
+      <c r="I65" s="227"/>
+      <c r="J65" s="228"/>
       <c r="K65" s="118"/>
       <c r="L65" s="119"/>
     </row>
     <row r="66" spans="2:12" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B66" s="198"/>
-      <c r="C66" s="199"/>
-      <c r="D66" s="199"/>
-      <c r="E66" s="193"/>
-      <c r="F66" s="192"/>
-      <c r="G66" s="193"/>
-      <c r="H66" s="179"/>
-      <c r="I66" s="180"/>
-      <c r="J66" s="181"/>
+      <c r="B66" s="248"/>
+      <c r="C66" s="249"/>
+      <c r="D66" s="249"/>
+      <c r="E66" s="243"/>
+      <c r="F66" s="242"/>
+      <c r="G66" s="243"/>
+      <c r="H66" s="229"/>
+      <c r="I66" s="230"/>
+      <c r="J66" s="231"/>
       <c r="K66" s="111"/>
       <c r="L66" s="112"/>
     </row>
@@ -42128,27 +42171,39 @@
     </row>
   </sheetData>
   <mergeCells count="71">
-    <mergeCell ref="B1:L1"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="J2:L6"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="C24:I25"/>
-    <mergeCell ref="J24:L24"/>
-    <mergeCell ref="K58:L58"/>
-    <mergeCell ref="K51:L51"/>
-    <mergeCell ref="C51:I58"/>
-    <mergeCell ref="K50:L50"/>
-    <mergeCell ref="K49:L49"/>
-    <mergeCell ref="C26:I26"/>
-    <mergeCell ref="C27:I27"/>
-    <mergeCell ref="C28:I28"/>
-    <mergeCell ref="C29:I29"/>
-    <mergeCell ref="C30:I30"/>
-    <mergeCell ref="C31:I31"/>
-    <mergeCell ref="C32:I32"/>
-    <mergeCell ref="C33:I33"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="K59:L59"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C44:I44"/>
+    <mergeCell ref="C45:I45"/>
+    <mergeCell ref="C46:I46"/>
+    <mergeCell ref="C47:I47"/>
+    <mergeCell ref="C48:I48"/>
+    <mergeCell ref="C39:I39"/>
+    <mergeCell ref="C40:I40"/>
+    <mergeCell ref="C41:I41"/>
+    <mergeCell ref="C42:I42"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="C36:I36"/>
+    <mergeCell ref="C37:I37"/>
+    <mergeCell ref="C38:I38"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="H60:J60"/>
+    <mergeCell ref="H61:J66"/>
+    <mergeCell ref="B49:J50"/>
+    <mergeCell ref="F61:G66"/>
+    <mergeCell ref="B61:E66"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="B23:E23"/>
@@ -42165,43 +42220,31 @@
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="G22:H22"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="H60:J60"/>
-    <mergeCell ref="H61:J66"/>
-    <mergeCell ref="B49:J50"/>
-    <mergeCell ref="F61:G66"/>
-    <mergeCell ref="B61:E66"/>
+    <mergeCell ref="C24:I25"/>
+    <mergeCell ref="J24:L24"/>
+    <mergeCell ref="K58:L58"/>
+    <mergeCell ref="K51:L51"/>
+    <mergeCell ref="C51:I58"/>
+    <mergeCell ref="K50:L50"/>
+    <mergeCell ref="K49:L49"/>
+    <mergeCell ref="C26:I26"/>
+    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="C28:I28"/>
+    <mergeCell ref="C29:I29"/>
+    <mergeCell ref="C30:I30"/>
+    <mergeCell ref="C31:I31"/>
+    <mergeCell ref="C32:I32"/>
+    <mergeCell ref="C33:I33"/>
     <mergeCell ref="C43:I43"/>
-    <mergeCell ref="C34:I34"/>
-    <mergeCell ref="C35:I35"/>
-    <mergeCell ref="C36:I36"/>
-    <mergeCell ref="C37:I37"/>
-    <mergeCell ref="C38:I38"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="K59:L59"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C44:I44"/>
-    <mergeCell ref="C45:I45"/>
-    <mergeCell ref="C46:I46"/>
-    <mergeCell ref="C47:I47"/>
-    <mergeCell ref="C48:I48"/>
-    <mergeCell ref="C39:I39"/>
-    <mergeCell ref="C40:I40"/>
-    <mergeCell ref="C41:I41"/>
-    <mergeCell ref="C42:I42"/>
+    <mergeCell ref="B1:L1"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="J2:L6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="K10:L10"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:L48">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>AND($B26&lt;&gt;"",$J26="",$L26&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -42239,40 +42282,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="111.6" customHeight="1">
-      <c r="B1" s="261"/>
-      <c r="C1" s="261"/>
-      <c r="D1" s="261"/>
-      <c r="E1" s="261"/>
-      <c r="F1" s="261"/>
-      <c r="G1" s="261"/>
-      <c r="H1" s="261"/>
-      <c r="I1" s="261"/>
-      <c r="J1" s="261"/>
-      <c r="K1" s="261"/>
-      <c r="L1" s="261"/>
-      <c r="M1" s="261"/>
-      <c r="N1" s="261"/>
-      <c r="O1" s="261"/>
-      <c r="P1" s="261"/>
+      <c r="B1" s="272"/>
+      <c r="C1" s="272"/>
+      <c r="D1" s="272"/>
+      <c r="E1" s="272"/>
+      <c r="F1" s="272"/>
+      <c r="G1" s="272"/>
+      <c r="H1" s="272"/>
+      <c r="I1" s="272"/>
+      <c r="J1" s="272"/>
+      <c r="K1" s="272"/>
+      <c r="L1" s="272"/>
+      <c r="M1" s="272"/>
+      <c r="N1" s="272"/>
+      <c r="O1" s="272"/>
+      <c r="P1" s="272"/>
     </row>
     <row r="2" spans="2:16" ht="22.95" customHeight="1">
-      <c r="B2" s="259" t="s">
+      <c r="B2" s="270" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="260"/>
-      <c r="D2" s="260"/>
-      <c r="E2" s="260"/>
-      <c r="F2" s="260"/>
-      <c r="G2" s="260"/>
-      <c r="H2" s="260"/>
-      <c r="I2" s="260"/>
-      <c r="J2" s="260"/>
-      <c r="K2" s="260"/>
-      <c r="L2" s="260"/>
-      <c r="M2" s="260"/>
-      <c r="N2" s="260"/>
-      <c r="O2" s="260"/>
-      <c r="P2" s="260"/>
+      <c r="C2" s="271"/>
+      <c r="D2" s="271"/>
+      <c r="E2" s="271"/>
+      <c r="F2" s="271"/>
+      <c r="G2" s="271"/>
+      <c r="H2" s="271"/>
+      <c r="I2" s="271"/>
+      <c r="J2" s="271"/>
+      <c r="K2" s="271"/>
+      <c r="L2" s="271"/>
+      <c r="M2" s="271"/>
+      <c r="N2" s="271"/>
+      <c r="O2" s="271"/>
+      <c r="P2" s="271"/>
     </row>
     <row r="3" spans="2:16" ht="4.95" customHeight="1">
       <c r="B3"/>
@@ -42299,16 +42342,16 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" s="267" t="s">
+      <c r="I4" s="278" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="267"/>
-      <c r="K4" s="267"/>
-      <c r="L4" s="267"/>
-      <c r="M4" s="267"/>
-      <c r="N4" s="267"/>
-      <c r="O4" s="267"/>
-      <c r="P4" s="267"/>
+      <c r="J4" s="278"/>
+      <c r="K4" s="278"/>
+      <c r="L4" s="278"/>
+      <c r="M4" s="278"/>
+      <c r="N4" s="278"/>
+      <c r="O4" s="278"/>
+      <c r="P4" s="278"/>
     </row>
     <row r="5" spans="2:16" ht="14.4" customHeight="1">
       <c r="B5" t="s">
@@ -42322,14 +42365,14 @@
       <c r="F5" s="56"/>
       <c r="G5" s="56"/>
       <c r="H5" s="56"/>
-      <c r="I5" s="267"/>
-      <c r="J5" s="267"/>
-      <c r="K5" s="267"/>
-      <c r="L5" s="267"/>
-      <c r="M5" s="267"/>
-      <c r="N5" s="267"/>
-      <c r="O5" s="267"/>
-      <c r="P5" s="267"/>
+      <c r="I5" s="278"/>
+      <c r="J5" s="278"/>
+      <c r="K5" s="278"/>
+      <c r="L5" s="278"/>
+      <c r="M5" s="278"/>
+      <c r="N5" s="278"/>
+      <c r="O5" s="278"/>
+      <c r="P5" s="278"/>
     </row>
     <row r="6" spans="2:16" ht="14.4" customHeight="1">
       <c r="B6" t="s">
@@ -42464,70 +42507,70 @@
       <c r="P11"/>
     </row>
     <row r="12" spans="2:16" s="62" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B12" s="258" t="s">
+      <c r="B12" s="269" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="258" t="s">
+      <c r="C12" s="269" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="258"/>
-      <c r="E12" s="258"/>
-      <c r="F12" s="258" t="s">
+      <c r="D12" s="269"/>
+      <c r="E12" s="269"/>
+      <c r="F12" s="269" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="258" t="s">
+      <c r="G12" s="269" t="s">
         <v>91</v>
       </c>
-      <c r="H12" s="258" t="s">
+      <c r="H12" s="269" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="258" t="s">
+      <c r="I12" s="269" t="s">
         <v>92</v>
       </c>
-      <c r="J12" s="258" t="s">
+      <c r="J12" s="269" t="s">
         <v>96</v>
       </c>
-      <c r="K12" s="258"/>
-      <c r="L12" s="258"/>
-      <c r="M12" s="258"/>
-      <c r="N12" s="258"/>
-      <c r="O12" s="258"/>
-      <c r="P12" s="266" t="s">
+      <c r="K12" s="269"/>
+      <c r="L12" s="269"/>
+      <c r="M12" s="269"/>
+      <c r="N12" s="269"/>
+      <c r="O12" s="269"/>
+      <c r="P12" s="277" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="2:16" s="61" customFormat="1">
-      <c r="B13" s="258"/>
-      <c r="C13" s="258"/>
-      <c r="D13" s="258"/>
-      <c r="E13" s="258"/>
-      <c r="F13" s="258"/>
-      <c r="G13" s="258"/>
-      <c r="H13" s="258"/>
-      <c r="I13" s="258"/>
-      <c r="J13" s="265" t="s">
+      <c r="B13" s="269"/>
+      <c r="C13" s="269"/>
+      <c r="D13" s="269"/>
+      <c r="E13" s="269"/>
+      <c r="F13" s="269"/>
+      <c r="G13" s="269"/>
+      <c r="H13" s="269"/>
+      <c r="I13" s="269"/>
+      <c r="J13" s="276" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="265"/>
-      <c r="L13" s="265" t="s">
+      <c r="K13" s="276"/>
+      <c r="L13" s="276" t="s">
         <v>98</v>
       </c>
-      <c r="M13" s="265"/>
-      <c r="N13" s="265" t="s">
+      <c r="M13" s="276"/>
+      <c r="N13" s="276" t="s">
         <v>99</v>
       </c>
-      <c r="O13" s="265"/>
-      <c r="P13" s="266"/>
+      <c r="O13" s="276"/>
+      <c r="P13" s="277"/>
     </row>
     <row r="14" spans="2:16" s="61" customFormat="1" ht="14.4" customHeight="1">
-      <c r="B14" s="258"/>
-      <c r="C14" s="258"/>
-      <c r="D14" s="258"/>
-      <c r="E14" s="258"/>
-      <c r="F14" s="258"/>
-      <c r="G14" s="258"/>
-      <c r="H14" s="258"/>
-      <c r="I14" s="258"/>
+      <c r="B14" s="269"/>
+      <c r="C14" s="269"/>
+      <c r="D14" s="269"/>
+      <c r="E14" s="269"/>
+      <c r="F14" s="269"/>
+      <c r="G14" s="269"/>
+      <c r="H14" s="269"/>
+      <c r="I14" s="269"/>
       <c r="J14" s="38" t="s">
         <v>76</v>
       </c>
@@ -42546,7 +42589,7 @@
       <c r="O14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="P14" s="266"/>
+      <c r="P14" s="277"/>
     </row>
     <row r="15" spans="2:16">
       <c r="C15" s="59"/>
@@ -42896,7 +42939,7 @@
     <mergeCell ref="I4:P5"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P49">
-    <cfRule type="expression" dxfId="1" priority="13">
+    <cfRule type="expression" dxfId="8" priority="13">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Update Excel export template: master_template_custom.xlsx
</commit_message>
<xml_diff>
--- a/public/templates/master_template_custom.xlsx
+++ b/public/templates/master_template_custom.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE7D67C5-7E0D-4AD0-A98E-DBA967EAD43F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20791560-2224-4B80-A5BF-ACAD31704E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cover" sheetId="21" r:id="rId1"/>
@@ -2664,17 +2664,92 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="39" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="75" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="114" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="26" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2684,29 +2759,47 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="61" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="66" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="59" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="54" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2720,28 +2813,57 @@
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="111" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="112" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2849,187 +2971,65 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="47" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="34" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="37" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="39" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="48" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="114" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="61" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="66" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="59" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="34" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="54" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="37" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="111" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="112" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="52" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="75" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="76" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="77" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="113" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3134,94 +3134,7 @@
     <cellStyle name="Normal 2 2 3" xfId="2" xr:uid="{25DAB206-4C06-437D-BFFA-FD21FFA5A242}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="25">
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color rgb="FFFFC000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0"/>
-          <bgColor theme="7" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="22">
     <dxf>
       <font>
         <b/>
@@ -3374,6 +3287,43 @@
           <bgColor rgb="FF002060"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="0"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <fill>
@@ -4973,7 +4923,7 @@
     <mergeCell ref="G12:G14"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P51">
-    <cfRule type="expression" dxfId="5" priority="14">
+    <cfRule type="expression" dxfId="0" priority="14">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14052,7 +14002,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="24" priority="2">
+    <cfRule type="expression" dxfId="21" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16302,23 +16252,23 @@
     <mergeCell ref="B1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:N16997">
-    <cfRule type="expression" dxfId="23" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="2">
+    <cfRule type="expression" dxfId="19" priority="2">
       <formula>AND(LEN($B6)&lt;&gt;0,$D6&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="5">
+    <cfRule type="expression" dxfId="18" priority="5">
       <formula>AND($B6="",$C6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H16997">
-    <cfRule type="expression" dxfId="20" priority="9">
+    <cfRule type="expression" dxfId="17" priority="9">
       <formula>IF(G6&lt;&gt;"", NOT(AND(OR(LEFT($E6,2)="L.", LEFT($E6,2)="A.", LEFT($E6,2)="B.", LEFT($E6,2)="M."), $H6&lt;&gt;"", $E6&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:K16997">
-    <cfRule type="notContainsBlanks" dxfId="19" priority="8">
+    <cfRule type="notContainsBlanks" dxfId="16" priority="8">
       <formula>LEN(TRIM(H6))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -40421,12 +40371,12 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B995 E6:H995">
-    <cfRule type="expression" dxfId="1" priority="7">
+    <cfRule type="expression" dxfId="15" priority="7">
       <formula>$J6=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:H995">
-    <cfRule type="expression" dxfId="0" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>AND($B6&lt;&gt;"",$C6="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -40655,7 +40605,7 @@
     <col min="6" max="6" width="31.77734375" style="57" customWidth="1"/>
     <col min="7" max="7" width="19.21875" style="68" customWidth="1"/>
     <col min="8" max="8" width="11.44140625" style="60" customWidth="1"/>
-    <col min="9" max="9" width="19.21875" style="68" customWidth="1"/>
+    <col min="9" max="9" width="20" style="68" customWidth="1"/>
     <col min="10" max="10" width="1.21875" customWidth="1"/>
     <col min="11" max="11" width="8.88671875" customWidth="1"/>
     <col min="12" max="12" width="12.21875" bestFit="1" customWidth="1"/>
@@ -40816,7 +40766,7 @@
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="76" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="75" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -40935,39 +40885,39 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:CE7">
-    <cfRule type="expression" dxfId="18" priority="12">
+    <cfRule type="expression" dxfId="13" priority="12">
       <formula>B5&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:CE201">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="12" priority="1">
       <formula>AND(G8&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="2">
+    <cfRule type="expression" dxfId="11" priority="2">
       <formula>AND(G$7&lt;&gt;"",$B8="RENCANA PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="10" priority="3">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="9" priority="4">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>AND(G8&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="6">
+    <cfRule type="expression" dxfId="7" priority="6">
       <formula>AND(G$7&lt;&gt;"",$B8="AKTUAL PROGRESS MINGGUAN")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="7">
+    <cfRule type="expression" dxfId="6" priority="7">
       <formula>AND(G8&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="8">
+    <cfRule type="expression" dxfId="5" priority="8">
       <formula>AND(G$7&lt;&gt;"",$B8="KUMULATIF PROGRESS AKTUAL")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="10">
+    <cfRule type="expression" dxfId="3" priority="10">
       <formula>AND(G$7&lt;&gt;"",$B8="DEVIASI")</formula>
     </cfRule>
     <cfRule type="colorScale" priority="11">
@@ -41008,45 +40958,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="88.8" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B1" s="254"/>
-      <c r="C1" s="255"/>
-      <c r="D1" s="255"/>
-      <c r="E1" s="255"/>
-      <c r="F1" s="255"/>
-      <c r="G1" s="255"/>
-      <c r="H1" s="255"/>
-      <c r="I1" s="255"/>
-      <c r="J1" s="255"/>
-      <c r="K1" s="255"/>
-      <c r="L1" s="256"/>
+      <c r="B1" s="171"/>
+      <c r="C1" s="172"/>
+      <c r="D1" s="172"/>
+      <c r="E1" s="172"/>
+      <c r="F1" s="172"/>
+      <c r="G1" s="172"/>
+      <c r="H1" s="172"/>
+      <c r="I1" s="172"/>
+      <c r="J1" s="172"/>
+      <c r="K1" s="172"/>
+      <c r="L1" s="173"/>
     </row>
     <row r="2" spans="1:13" ht="15" customHeight="1" thickTop="1">
-      <c r="B2" s="257" t="s">
+      <c r="B2" s="174" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="258"/>
-      <c r="D2" s="258"/>
-      <c r="E2" s="258"/>
-      <c r="F2" s="258"/>
-      <c r="G2" s="258"/>
-      <c r="H2" s="258"/>
-      <c r="I2" s="259"/>
-      <c r="J2" s="263"/>
-      <c r="K2" s="264"/>
-      <c r="L2" s="265"/>
+      <c r="C2" s="175"/>
+      <c r="D2" s="175"/>
+      <c r="E2" s="175"/>
+      <c r="F2" s="175"/>
+      <c r="G2" s="175"/>
+      <c r="H2" s="175"/>
+      <c r="I2" s="176"/>
+      <c r="J2" s="180"/>
+      <c r="K2" s="181"/>
+      <c r="L2" s="182"/>
     </row>
     <row r="3" spans="1:13" ht="14.4" customHeight="1">
-      <c r="B3" s="260"/>
-      <c r="C3" s="261"/>
-      <c r="D3" s="261"/>
-      <c r="E3" s="261"/>
-      <c r="F3" s="261"/>
-      <c r="G3" s="261"/>
-      <c r="H3" s="261"/>
-      <c r="I3" s="262"/>
-      <c r="J3" s="266"/>
-      <c r="K3" s="267"/>
-      <c r="L3" s="268"/>
+      <c r="B3" s="177"/>
+      <c r="C3" s="178"/>
+      <c r="D3" s="178"/>
+      <c r="E3" s="178"/>
+      <c r="F3" s="178"/>
+      <c r="G3" s="178"/>
+      <c r="H3" s="178"/>
+      <c r="I3" s="179"/>
+      <c r="J3" s="183"/>
+      <c r="K3" s="184"/>
+      <c r="L3" s="185"/>
     </row>
     <row r="4" spans="1:13" ht="14.4" customHeight="1">
       <c r="B4" s="77"/>
@@ -41057,9 +41007,9 @@
       <c r="G4" s="78"/>
       <c r="H4" s="78"/>
       <c r="I4" s="78"/>
-      <c r="J4" s="266"/>
-      <c r="K4" s="267"/>
-      <c r="L4" s="268"/>
+      <c r="J4" s="183"/>
+      <c r="K4" s="184"/>
+      <c r="L4" s="185"/>
     </row>
     <row r="5" spans="1:13" ht="15.6" customHeight="1">
       <c r="B5" s="79" t="s">
@@ -41074,9 +41024,9 @@
       <c r="G5" s="81"/>
       <c r="H5" s="81"/>
       <c r="I5" s="82"/>
-      <c r="J5" s="266"/>
-      <c r="K5" s="267"/>
-      <c r="L5" s="268"/>
+      <c r="J5" s="183"/>
+      <c r="K5" s="184"/>
+      <c r="L5" s="185"/>
     </row>
     <row r="6" spans="1:13" ht="15.6" customHeight="1">
       <c r="B6" s="79" t="s">
@@ -41091,9 +41041,9 @@
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
       <c r="I6" s="83"/>
-      <c r="J6" s="269"/>
-      <c r="K6" s="270"/>
-      <c r="L6" s="271"/>
+      <c r="J6" s="186"/>
+      <c r="K6" s="187"/>
+      <c r="L6" s="188"/>
     </row>
     <row r="7" spans="1:13" ht="15.6">
       <c r="B7" s="79" t="s">
@@ -41149,41 +41099,41 @@
       <c r="L9" s="89"/>
     </row>
     <row r="10" spans="1:13" ht="15.6">
-      <c r="B10" s="272" t="s">
+      <c r="B10" s="189" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="273"/>
-      <c r="D10" s="273"/>
-      <c r="E10" s="273"/>
-      <c r="F10" s="274"/>
-      <c r="G10" s="273" t="s">
+      <c r="C10" s="190"/>
+      <c r="D10" s="190"/>
+      <c r="E10" s="190"/>
+      <c r="F10" s="191"/>
+      <c r="G10" s="190" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="273"/>
-      <c r="I10" s="273"/>
-      <c r="J10" s="274"/>
-      <c r="K10" s="273" t="s">
+      <c r="H10" s="190"/>
+      <c r="I10" s="190"/>
+      <c r="J10" s="191"/>
+      <c r="K10" s="190" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="275"/>
+      <c r="L10" s="192"/>
     </row>
     <row r="11" spans="1:13" ht="16.2" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="222" t="s">
+      <c r="C11" s="215" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="223"/>
-      <c r="E11" s="223"/>
+      <c r="D11" s="216"/>
+      <c r="E11" s="216"/>
       <c r="F11" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="G11" s="222" t="s">
+      <c r="G11" s="215" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="224"/>
+      <c r="H11" s="217"/>
       <c r="I11" s="92" t="s">
         <v>27</v>
       </c>
@@ -41202,14 +41152,14 @@
       <c r="B12" s="94" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="188" t="s">
+      <c r="C12" s="261" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="189"/>
-      <c r="E12" s="190"/>
+      <c r="D12" s="262"/>
+      <c r="E12" s="263"/>
       <c r="F12" s="151"/>
-      <c r="G12" s="231"/>
-      <c r="H12" s="232"/>
+      <c r="G12" s="224"/>
+      <c r="H12" s="225"/>
       <c r="I12" s="149"/>
       <c r="J12" s="156"/>
       <c r="K12" s="157"/>
@@ -41219,14 +41169,14 @@
       <c r="B13" s="95">
         <v>1</v>
       </c>
-      <c r="C13" s="176" t="s">
+      <c r="C13" s="264" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="177"/>
-      <c r="E13" s="178"/>
+      <c r="D13" s="265"/>
+      <c r="E13" s="266"/>
       <c r="F13" s="152"/>
-      <c r="G13" s="233"/>
-      <c r="H13" s="234"/>
+      <c r="G13" s="226"/>
+      <c r="H13" s="227"/>
       <c r="I13" s="150"/>
       <c r="J13" s="96"/>
       <c r="K13" s="158"/>
@@ -41236,14 +41186,14 @@
       <c r="B14" s="95">
         <v>2</v>
       </c>
-      <c r="C14" s="176" t="s">
+      <c r="C14" s="264" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="177"/>
-      <c r="E14" s="178"/>
+      <c r="D14" s="265"/>
+      <c r="E14" s="266"/>
       <c r="F14" s="152"/>
-      <c r="G14" s="233"/>
-      <c r="H14" s="234"/>
+      <c r="G14" s="226"/>
+      <c r="H14" s="227"/>
       <c r="I14" s="150"/>
       <c r="J14" s="96"/>
       <c r="K14" s="158"/>
@@ -41253,14 +41203,14 @@
       <c r="B15" s="95">
         <v>3</v>
       </c>
-      <c r="C15" s="176" t="s">
+      <c r="C15" s="264" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="177"/>
-      <c r="E15" s="178"/>
+      <c r="D15" s="265"/>
+      <c r="E15" s="266"/>
       <c r="F15" s="152"/>
-      <c r="G15" s="233"/>
-      <c r="H15" s="234"/>
+      <c r="G15" s="226"/>
+      <c r="H15" s="227"/>
       <c r="I15" s="150"/>
       <c r="J15" s="96"/>
       <c r="K15" s="158"/>
@@ -41270,14 +41220,14 @@
       <c r="B16" s="95">
         <v>4</v>
       </c>
-      <c r="C16" s="176" t="s">
+      <c r="C16" s="264" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="177"/>
-      <c r="E16" s="178"/>
+      <c r="D16" s="265"/>
+      <c r="E16" s="266"/>
       <c r="F16" s="152"/>
-      <c r="G16" s="233"/>
-      <c r="H16" s="234"/>
+      <c r="G16" s="226"/>
+      <c r="H16" s="227"/>
       <c r="I16" s="150"/>
       <c r="J16" s="96"/>
       <c r="K16" s="158"/>
@@ -41287,14 +41237,14 @@
       <c r="B17" s="95">
         <v>5</v>
       </c>
-      <c r="C17" s="176" t="s">
+      <c r="C17" s="264" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="177"/>
-      <c r="E17" s="178"/>
+      <c r="D17" s="265"/>
+      <c r="E17" s="266"/>
       <c r="F17" s="152"/>
-      <c r="G17" s="233"/>
-      <c r="H17" s="234"/>
+      <c r="G17" s="226"/>
+      <c r="H17" s="227"/>
       <c r="I17" s="150"/>
       <c r="J17" s="96"/>
       <c r="K17" s="158"/>
@@ -41304,14 +41254,14 @@
       <c r="B18" s="95">
         <v>6</v>
       </c>
-      <c r="C18" s="176" t="s">
+      <c r="C18" s="264" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="177"/>
-      <c r="E18" s="178"/>
+      <c r="D18" s="265"/>
+      <c r="E18" s="266"/>
       <c r="F18" s="152"/>
-      <c r="G18" s="233"/>
-      <c r="H18" s="234"/>
+      <c r="G18" s="226"/>
+      <c r="H18" s="227"/>
       <c r="I18" s="150"/>
       <c r="J18" s="96"/>
       <c r="K18" s="158"/>
@@ -41321,14 +41271,14 @@
       <c r="B19" s="97" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="179" t="s">
+      <c r="C19" s="270" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="180"/>
-      <c r="E19" s="181"/>
+      <c r="D19" s="271"/>
+      <c r="E19" s="272"/>
       <c r="F19" s="152"/>
-      <c r="G19" s="233"/>
-      <c r="H19" s="234"/>
+      <c r="G19" s="226"/>
+      <c r="H19" s="227"/>
       <c r="I19" s="150"/>
       <c r="J19" s="96"/>
       <c r="K19" s="158"/>
@@ -41338,14 +41288,14 @@
       <c r="B20" s="95">
         <v>1</v>
       </c>
-      <c r="C20" s="176" t="s">
+      <c r="C20" s="264" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="177"/>
-      <c r="E20" s="178"/>
+      <c r="D20" s="265"/>
+      <c r="E20" s="266"/>
       <c r="F20" s="152"/>
-      <c r="G20" s="233"/>
-      <c r="H20" s="234"/>
+      <c r="G20" s="226"/>
+      <c r="H20" s="227"/>
       <c r="I20" s="150"/>
       <c r="J20" s="96"/>
       <c r="K20" s="158"/>
@@ -41355,14 +41305,14 @@
       <c r="B21" s="95">
         <v>2</v>
       </c>
-      <c r="C21" s="176" t="s">
+      <c r="C21" s="264" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="177"/>
-      <c r="E21" s="178"/>
+      <c r="D21" s="265"/>
+      <c r="E21" s="266"/>
       <c r="F21" s="152"/>
-      <c r="G21" s="233"/>
-      <c r="H21" s="234"/>
+      <c r="G21" s="226"/>
+      <c r="H21" s="227"/>
       <c r="I21" s="150"/>
       <c r="J21" s="96"/>
       <c r="K21" s="158"/>
@@ -41372,63 +41322,63 @@
       <c r="B22" s="95">
         <v>3</v>
       </c>
-      <c r="C22" s="171" t="s">
+      <c r="C22" s="267" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="172"/>
-      <c r="E22" s="173"/>
+      <c r="D22" s="268"/>
+      <c r="E22" s="269"/>
       <c r="F22" s="152"/>
-      <c r="G22" s="235"/>
-      <c r="H22" s="236"/>
+      <c r="G22" s="228"/>
+      <c r="H22" s="229"/>
       <c r="I22" s="150"/>
       <c r="J22" s="96"/>
       <c r="K22" s="159"/>
       <c r="L22" s="155"/>
     </row>
     <row r="23" spans="1:12" ht="16.2" thickBot="1">
-      <c r="B23" s="225"/>
-      <c r="C23" s="226"/>
-      <c r="D23" s="226"/>
-      <c r="E23" s="226"/>
+      <c r="B23" s="218"/>
+      <c r="C23" s="219"/>
+      <c r="D23" s="219"/>
+      <c r="E23" s="219"/>
       <c r="F23" s="98"/>
       <c r="G23" s="98"/>
       <c r="H23" s="99"/>
       <c r="I23" s="99"/>
-      <c r="J23" s="227"/>
-      <c r="K23" s="227"/>
-      <c r="L23" s="228"/>
+      <c r="J23" s="220"/>
+      <c r="K23" s="220"/>
+      <c r="L23" s="221"/>
     </row>
     <row r="24" spans="1:12" ht="16.2" customHeight="1" thickTop="1">
       <c r="A24" s="113" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="229" t="s">
+      <c r="B24" s="222" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="237" t="s">
+      <c r="C24" s="193" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="237"/>
-      <c r="E24" s="237"/>
-      <c r="F24" s="237"/>
-      <c r="G24" s="237"/>
-      <c r="H24" s="237"/>
-      <c r="I24" s="237"/>
-      <c r="J24" s="239" t="s">
+      <c r="D24" s="193"/>
+      <c r="E24" s="193"/>
+      <c r="F24" s="193"/>
+      <c r="G24" s="193"/>
+      <c r="H24" s="193"/>
+      <c r="I24" s="193"/>
+      <c r="J24" s="195" t="s">
         <v>75</v>
       </c>
-      <c r="K24" s="240"/>
-      <c r="L24" s="241"/>
+      <c r="K24" s="196"/>
+      <c r="L24" s="197"/>
     </row>
     <row r="25" spans="1:12" ht="31.2">
-      <c r="B25" s="230"/>
-      <c r="C25" s="238"/>
-      <c r="D25" s="238"/>
-      <c r="E25" s="238"/>
-      <c r="F25" s="238"/>
-      <c r="G25" s="238"/>
-      <c r="H25" s="238"/>
-      <c r="I25" s="238"/>
+      <c r="B25" s="223"/>
+      <c r="C25" s="194"/>
+      <c r="D25" s="194"/>
+      <c r="E25" s="194"/>
+      <c r="F25" s="194"/>
+      <c r="G25" s="194"/>
+      <c r="H25" s="194"/>
+      <c r="I25" s="194"/>
       <c r="J25" s="137" t="s">
         <v>9</v>
       </c>
@@ -41441,52 +41391,52 @@
     </row>
     <row r="26" spans="1:12" ht="15.6">
       <c r="B26" s="100"/>
-      <c r="C26" s="251"/>
-      <c r="D26" s="252"/>
-      <c r="E26" s="252"/>
-      <c r="F26" s="252"/>
-      <c r="G26" s="252"/>
-      <c r="H26" s="252"/>
-      <c r="I26" s="253"/>
+      <c r="C26" s="209"/>
+      <c r="D26" s="210"/>
+      <c r="E26" s="210"/>
+      <c r="F26" s="210"/>
+      <c r="G26" s="210"/>
+      <c r="H26" s="210"/>
+      <c r="I26" s="211"/>
       <c r="J26" s="138"/>
       <c r="K26" s="146"/>
       <c r="L26" s="144"/>
     </row>
     <row r="27" spans="1:12" ht="15.6">
       <c r="B27" s="100"/>
-      <c r="C27" s="182"/>
-      <c r="D27" s="183"/>
-      <c r="E27" s="183"/>
-      <c r="F27" s="183"/>
-      <c r="G27" s="183"/>
-      <c r="H27" s="183"/>
-      <c r="I27" s="184"/>
+      <c r="C27" s="212"/>
+      <c r="D27" s="213"/>
+      <c r="E27" s="213"/>
+      <c r="F27" s="213"/>
+      <c r="G27" s="213"/>
+      <c r="H27" s="213"/>
+      <c r="I27" s="214"/>
       <c r="J27" s="96"/>
       <c r="K27" s="147"/>
       <c r="L27" s="144"/>
     </row>
     <row r="28" spans="1:12" ht="15.6">
       <c r="B28" s="100"/>
-      <c r="C28" s="182"/>
-      <c r="D28" s="183"/>
-      <c r="E28" s="183"/>
-      <c r="F28" s="183"/>
-      <c r="G28" s="183"/>
-      <c r="H28" s="183"/>
-      <c r="I28" s="184"/>
+      <c r="C28" s="212"/>
+      <c r="D28" s="213"/>
+      <c r="E28" s="213"/>
+      <c r="F28" s="213"/>
+      <c r="G28" s="213"/>
+      <c r="H28" s="213"/>
+      <c r="I28" s="214"/>
       <c r="J28" s="96"/>
       <c r="K28" s="147"/>
       <c r="L28" s="145"/>
     </row>
     <row r="29" spans="1:12" ht="15.6">
       <c r="B29" s="100"/>
-      <c r="C29" s="182"/>
-      <c r="D29" s="183"/>
-      <c r="E29" s="183"/>
-      <c r="F29" s="183"/>
-      <c r="G29" s="183"/>
-      <c r="H29" s="183"/>
-      <c r="I29" s="184"/>
+      <c r="C29" s="212"/>
+      <c r="D29" s="213"/>
+      <c r="E29" s="213"/>
+      <c r="F29" s="213"/>
+      <c r="G29" s="213"/>
+      <c r="H29" s="213"/>
+      <c r="I29" s="214"/>
       <c r="J29" s="96"/>
       <c r="K29" s="147"/>
       <c r="L29" s="145"/>
@@ -41495,15 +41445,15 @@
       <c r="B30" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="182" t="s">
+      <c r="C30" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="183"/>
-      <c r="E30" s="183"/>
-      <c r="F30" s="183"/>
-      <c r="G30" s="183"/>
-      <c r="H30" s="183"/>
-      <c r="I30" s="184"/>
+      <c r="D30" s="213"/>
+      <c r="E30" s="213"/>
+      <c r="F30" s="213"/>
+      <c r="G30" s="213"/>
+      <c r="H30" s="213"/>
+      <c r="I30" s="214"/>
       <c r="J30" s="96" t="s">
         <v>64</v>
       </c>
@@ -41516,15 +41466,15 @@
       <c r="B31" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="182" t="s">
+      <c r="C31" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="183"/>
-      <c r="E31" s="183"/>
-      <c r="F31" s="183"/>
-      <c r="G31" s="183"/>
-      <c r="H31" s="183"/>
-      <c r="I31" s="184"/>
+      <c r="D31" s="213"/>
+      <c r="E31" s="213"/>
+      <c r="F31" s="213"/>
+      <c r="G31" s="213"/>
+      <c r="H31" s="213"/>
+      <c r="I31" s="214"/>
       <c r="J31" s="96" t="s">
         <v>64</v>
       </c>
@@ -41537,15 +41487,15 @@
       <c r="B32" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="182" t="s">
+      <c r="C32" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="183"/>
-      <c r="E32" s="183"/>
-      <c r="F32" s="183"/>
-      <c r="G32" s="183"/>
-      <c r="H32" s="183"/>
-      <c r="I32" s="184"/>
+      <c r="D32" s="213"/>
+      <c r="E32" s="213"/>
+      <c r="F32" s="213"/>
+      <c r="G32" s="213"/>
+      <c r="H32" s="213"/>
+      <c r="I32" s="214"/>
       <c r="J32" s="96" t="s">
         <v>64</v>
       </c>
@@ -41558,15 +41508,15 @@
       <c r="B33" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="182" t="s">
+      <c r="C33" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="183"/>
-      <c r="E33" s="183"/>
-      <c r="F33" s="183"/>
-      <c r="G33" s="183"/>
-      <c r="H33" s="183"/>
-      <c r="I33" s="184"/>
+      <c r="D33" s="213"/>
+      <c r="E33" s="213"/>
+      <c r="F33" s="213"/>
+      <c r="G33" s="213"/>
+      <c r="H33" s="213"/>
+      <c r="I33" s="214"/>
       <c r="J33" s="96" t="s">
         <v>64</v>
       </c>
@@ -41579,15 +41529,15 @@
       <c r="B34" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="182" t="s">
+      <c r="C34" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="183"/>
-      <c r="E34" s="183"/>
-      <c r="F34" s="183"/>
-      <c r="G34" s="183"/>
-      <c r="H34" s="183"/>
-      <c r="I34" s="184"/>
+      <c r="D34" s="213"/>
+      <c r="E34" s="213"/>
+      <c r="F34" s="213"/>
+      <c r="G34" s="213"/>
+      <c r="H34" s="213"/>
+      <c r="I34" s="214"/>
       <c r="J34" s="96" t="s">
         <v>64</v>
       </c>
@@ -41600,15 +41550,15 @@
       <c r="B35" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="182" t="s">
+      <c r="C35" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="183"/>
-      <c r="E35" s="183"/>
-      <c r="F35" s="183"/>
-      <c r="G35" s="183"/>
-      <c r="H35" s="183"/>
-      <c r="I35" s="184"/>
+      <c r="D35" s="213"/>
+      <c r="E35" s="213"/>
+      <c r="F35" s="213"/>
+      <c r="G35" s="213"/>
+      <c r="H35" s="213"/>
+      <c r="I35" s="214"/>
       <c r="J35" s="96" t="s">
         <v>64</v>
       </c>
@@ -41621,15 +41571,15 @@
       <c r="B36" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C36" s="182" t="s">
+      <c r="C36" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D36" s="183"/>
-      <c r="E36" s="183"/>
-      <c r="F36" s="183"/>
-      <c r="G36" s="183"/>
-      <c r="H36" s="183"/>
-      <c r="I36" s="184"/>
+      <c r="D36" s="213"/>
+      <c r="E36" s="213"/>
+      <c r="F36" s="213"/>
+      <c r="G36" s="213"/>
+      <c r="H36" s="213"/>
+      <c r="I36" s="214"/>
       <c r="J36" s="96" t="s">
         <v>64</v>
       </c>
@@ -41642,15 +41592,15 @@
       <c r="B37" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="182" t="s">
+      <c r="C37" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D37" s="183"/>
-      <c r="E37" s="183"/>
-      <c r="F37" s="183"/>
-      <c r="G37" s="183"/>
-      <c r="H37" s="183"/>
-      <c r="I37" s="184"/>
+      <c r="D37" s="213"/>
+      <c r="E37" s="213"/>
+      <c r="F37" s="213"/>
+      <c r="G37" s="213"/>
+      <c r="H37" s="213"/>
+      <c r="I37" s="214"/>
       <c r="J37" s="96" t="s">
         <v>64</v>
       </c>
@@ -41663,15 +41613,15 @@
       <c r="B38" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="182" t="s">
+      <c r="C38" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="183"/>
-      <c r="E38" s="183"/>
-      <c r="F38" s="183"/>
-      <c r="G38" s="183"/>
-      <c r="H38" s="183"/>
-      <c r="I38" s="184"/>
+      <c r="D38" s="213"/>
+      <c r="E38" s="213"/>
+      <c r="F38" s="213"/>
+      <c r="G38" s="213"/>
+      <c r="H38" s="213"/>
+      <c r="I38" s="214"/>
       <c r="J38" s="96" t="s">
         <v>64</v>
       </c>
@@ -41684,15 +41634,15 @@
       <c r="B39" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="182" t="s">
+      <c r="C39" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D39" s="183"/>
-      <c r="E39" s="183"/>
-      <c r="F39" s="183"/>
-      <c r="G39" s="183"/>
-      <c r="H39" s="183"/>
-      <c r="I39" s="184"/>
+      <c r="D39" s="213"/>
+      <c r="E39" s="213"/>
+      <c r="F39" s="213"/>
+      <c r="G39" s="213"/>
+      <c r="H39" s="213"/>
+      <c r="I39" s="214"/>
       <c r="J39" s="96" t="s">
         <v>64</v>
       </c>
@@ -41705,15 +41655,15 @@
       <c r="B40" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="182" t="s">
+      <c r="C40" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D40" s="183"/>
-      <c r="E40" s="183"/>
-      <c r="F40" s="183"/>
-      <c r="G40" s="183"/>
-      <c r="H40" s="183"/>
-      <c r="I40" s="184"/>
+      <c r="D40" s="213"/>
+      <c r="E40" s="213"/>
+      <c r="F40" s="213"/>
+      <c r="G40" s="213"/>
+      <c r="H40" s="213"/>
+      <c r="I40" s="214"/>
       <c r="J40" s="96" t="s">
         <v>64</v>
       </c>
@@ -41726,15 +41676,15 @@
       <c r="B41" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="182" t="s">
+      <c r="C41" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D41" s="183"/>
-      <c r="E41" s="183"/>
-      <c r="F41" s="183"/>
-      <c r="G41" s="183"/>
-      <c r="H41" s="183"/>
-      <c r="I41" s="184"/>
+      <c r="D41" s="213"/>
+      <c r="E41" s="213"/>
+      <c r="F41" s="213"/>
+      <c r="G41" s="213"/>
+      <c r="H41" s="213"/>
+      <c r="I41" s="214"/>
       <c r="J41" s="96" t="s">
         <v>64</v>
       </c>
@@ -41747,15 +41697,15 @@
       <c r="B42" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="182" t="s">
+      <c r="C42" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="183"/>
-      <c r="E42" s="183"/>
-      <c r="F42" s="183"/>
-      <c r="G42" s="183"/>
-      <c r="H42" s="183"/>
-      <c r="I42" s="184"/>
+      <c r="D42" s="213"/>
+      <c r="E42" s="213"/>
+      <c r="F42" s="213"/>
+      <c r="G42" s="213"/>
+      <c r="H42" s="213"/>
+      <c r="I42" s="214"/>
       <c r="J42" s="96" t="s">
         <v>64</v>
       </c>
@@ -41768,15 +41718,15 @@
       <c r="B43" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="182" t="s">
+      <c r="C43" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="183"/>
-      <c r="E43" s="183"/>
-      <c r="F43" s="183"/>
-      <c r="G43" s="183"/>
-      <c r="H43" s="183"/>
-      <c r="I43" s="184"/>
+      <c r="D43" s="213"/>
+      <c r="E43" s="213"/>
+      <c r="F43" s="213"/>
+      <c r="G43" s="213"/>
+      <c r="H43" s="213"/>
+      <c r="I43" s="214"/>
       <c r="J43" s="96" t="s">
         <v>64</v>
       </c>
@@ -41789,15 +41739,15 @@
       <c r="B44" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="182" t="s">
+      <c r="C44" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D44" s="183"/>
-      <c r="E44" s="183"/>
-      <c r="F44" s="183"/>
-      <c r="G44" s="183"/>
-      <c r="H44" s="183"/>
-      <c r="I44" s="184"/>
+      <c r="D44" s="213"/>
+      <c r="E44" s="213"/>
+      <c r="F44" s="213"/>
+      <c r="G44" s="213"/>
+      <c r="H44" s="213"/>
+      <c r="I44" s="214"/>
       <c r="J44" s="96" t="s">
         <v>64</v>
       </c>
@@ -41810,15 +41760,15 @@
       <c r="B45" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C45" s="182" t="s">
+      <c r="C45" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D45" s="183"/>
-      <c r="E45" s="183"/>
-      <c r="F45" s="183"/>
-      <c r="G45" s="183"/>
-      <c r="H45" s="183"/>
-      <c r="I45" s="184"/>
+      <c r="D45" s="213"/>
+      <c r="E45" s="213"/>
+      <c r="F45" s="213"/>
+      <c r="G45" s="213"/>
+      <c r="H45" s="213"/>
+      <c r="I45" s="214"/>
       <c r="J45" s="96" t="s">
         <v>64</v>
       </c>
@@ -41831,15 +41781,15 @@
       <c r="B46" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C46" s="182" t="s">
+      <c r="C46" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="183"/>
-      <c r="E46" s="183"/>
-      <c r="F46" s="183"/>
-      <c r="G46" s="183"/>
-      <c r="H46" s="183"/>
-      <c r="I46" s="184"/>
+      <c r="D46" s="213"/>
+      <c r="E46" s="213"/>
+      <c r="F46" s="213"/>
+      <c r="G46" s="213"/>
+      <c r="H46" s="213"/>
+      <c r="I46" s="214"/>
       <c r="J46" s="96" t="s">
         <v>64</v>
       </c>
@@ -41852,15 +41802,15 @@
       <c r="B47" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="182" t="s">
+      <c r="C47" s="212" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="183"/>
-      <c r="E47" s="183"/>
-      <c r="F47" s="183"/>
-      <c r="G47" s="183"/>
-      <c r="H47" s="183"/>
-      <c r="I47" s="184"/>
+      <c r="D47" s="213"/>
+      <c r="E47" s="213"/>
+      <c r="F47" s="213"/>
+      <c r="G47" s="213"/>
+      <c r="H47" s="213"/>
+      <c r="I47" s="214"/>
       <c r="J47" s="96" t="s">
         <v>64</v>
       </c>
@@ -41873,15 +41823,15 @@
       <c r="B48" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="C48" s="185" t="s">
+      <c r="C48" s="273" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="186"/>
-      <c r="E48" s="186"/>
-      <c r="F48" s="186"/>
-      <c r="G48" s="186"/>
-      <c r="H48" s="186"/>
-      <c r="I48" s="187"/>
+      <c r="D48" s="274"/>
+      <c r="E48" s="274"/>
+      <c r="F48" s="274"/>
+      <c r="G48" s="274"/>
+      <c r="H48" s="274"/>
+      <c r="I48" s="275"/>
       <c r="J48" s="139" t="s">
         <v>64</v>
       </c>
@@ -41891,140 +41841,140 @@
       </c>
     </row>
     <row r="49" spans="2:12" ht="16.2" thickTop="1">
-      <c r="B49" s="204" t="s">
+      <c r="B49" s="243" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="205"/>
-      <c r="D49" s="205"/>
-      <c r="E49" s="205"/>
-      <c r="F49" s="205"/>
-      <c r="G49" s="205"/>
-      <c r="H49" s="205"/>
-      <c r="I49" s="205"/>
-      <c r="J49" s="206"/>
-      <c r="K49" s="249" t="s">
+      <c r="C49" s="244"/>
+      <c r="D49" s="244"/>
+      <c r="E49" s="244"/>
+      <c r="F49" s="244"/>
+      <c r="G49" s="244"/>
+      <c r="H49" s="244"/>
+      <c r="I49" s="244"/>
+      <c r="J49" s="245"/>
+      <c r="K49" s="207" t="s">
         <v>79</v>
       </c>
-      <c r="L49" s="250"/>
+      <c r="L49" s="208"/>
     </row>
     <row r="50" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B50" s="207"/>
-      <c r="C50" s="208"/>
-      <c r="D50" s="208"/>
-      <c r="E50" s="208"/>
-      <c r="F50" s="208"/>
-      <c r="G50" s="208"/>
-      <c r="H50" s="208"/>
-      <c r="I50" s="208"/>
-      <c r="J50" s="209"/>
-      <c r="K50" s="247" t="s">
+      <c r="B50" s="246"/>
+      <c r="C50" s="247"/>
+      <c r="D50" s="247"/>
+      <c r="E50" s="247"/>
+      <c r="F50" s="247"/>
+      <c r="G50" s="247"/>
+      <c r="H50" s="247"/>
+      <c r="I50" s="247"/>
+      <c r="J50" s="248"/>
+      <c r="K50" s="205" t="s">
         <v>103</v>
       </c>
-      <c r="L50" s="248"/>
+      <c r="L50" s="206"/>
     </row>
     <row r="51" spans="2:12" ht="15.6">
       <c r="B51" s="101"/>
-      <c r="C51" s="244"/>
-      <c r="D51" s="244"/>
-      <c r="E51" s="244"/>
-      <c r="F51" s="244"/>
-      <c r="G51" s="244"/>
-      <c r="H51" s="244"/>
-      <c r="I51" s="244"/>
+      <c r="C51" s="202"/>
+      <c r="D51" s="202"/>
+      <c r="E51" s="202"/>
+      <c r="F51" s="202"/>
+      <c r="G51" s="202"/>
+      <c r="H51" s="202"/>
+      <c r="I51" s="202"/>
       <c r="J51" s="102"/>
-      <c r="K51" s="242"/>
-      <c r="L51" s="243"/>
+      <c r="K51" s="200"/>
+      <c r="L51" s="201"/>
     </row>
     <row r="52" spans="2:12" ht="15.6">
       <c r="B52" s="103"/>
-      <c r="C52" s="245"/>
-      <c r="D52" s="245"/>
-      <c r="E52" s="245"/>
-      <c r="F52" s="245"/>
-      <c r="G52" s="245"/>
-      <c r="H52" s="245"/>
-      <c r="I52" s="245"/>
+      <c r="C52" s="203"/>
+      <c r="D52" s="203"/>
+      <c r="E52" s="203"/>
+      <c r="F52" s="203"/>
+      <c r="G52" s="203"/>
+      <c r="H52" s="203"/>
+      <c r="I52" s="203"/>
       <c r="J52" s="104"/>
       <c r="K52" s="115"/>
       <c r="L52" s="105"/>
     </row>
     <row r="53" spans="2:12" ht="15.6">
       <c r="B53" s="106"/>
-      <c r="C53" s="245"/>
-      <c r="D53" s="245"/>
-      <c r="E53" s="245"/>
-      <c r="F53" s="245"/>
-      <c r="G53" s="245"/>
-      <c r="H53" s="245"/>
-      <c r="I53" s="245"/>
+      <c r="C53" s="203"/>
+      <c r="D53" s="203"/>
+      <c r="E53" s="203"/>
+      <c r="F53" s="203"/>
+      <c r="G53" s="203"/>
+      <c r="H53" s="203"/>
+      <c r="I53" s="203"/>
       <c r="J53" s="107"/>
       <c r="K53" s="108"/>
       <c r="L53" s="109"/>
     </row>
     <row r="54" spans="2:12" ht="15.6">
       <c r="B54" s="106"/>
-      <c r="C54" s="245"/>
-      <c r="D54" s="245"/>
-      <c r="E54" s="245"/>
-      <c r="F54" s="245"/>
-      <c r="G54" s="245"/>
-      <c r="H54" s="245"/>
-      <c r="I54" s="245"/>
+      <c r="C54" s="203"/>
+      <c r="D54" s="203"/>
+      <c r="E54" s="203"/>
+      <c r="F54" s="203"/>
+      <c r="G54" s="203"/>
+      <c r="H54" s="203"/>
+      <c r="I54" s="203"/>
       <c r="J54" s="107"/>
       <c r="K54" s="140"/>
       <c r="L54" s="141"/>
     </row>
     <row r="55" spans="2:12" ht="15.6">
       <c r="B55" s="106"/>
-      <c r="C55" s="245"/>
-      <c r="D55" s="245"/>
-      <c r="E55" s="245"/>
-      <c r="F55" s="245"/>
-      <c r="G55" s="245"/>
-      <c r="H55" s="245"/>
-      <c r="I55" s="245"/>
+      <c r="C55" s="203"/>
+      <c r="D55" s="203"/>
+      <c r="E55" s="203"/>
+      <c r="F55" s="203"/>
+      <c r="G55" s="203"/>
+      <c r="H55" s="203"/>
+      <c r="I55" s="203"/>
       <c r="J55" s="107"/>
       <c r="K55" s="140"/>
       <c r="L55" s="141"/>
     </row>
     <row r="56" spans="2:12" ht="15.6">
       <c r="B56" s="106"/>
-      <c r="C56" s="245"/>
-      <c r="D56" s="245"/>
-      <c r="E56" s="245"/>
-      <c r="F56" s="245"/>
-      <c r="G56" s="245"/>
-      <c r="H56" s="245"/>
-      <c r="I56" s="245"/>
+      <c r="C56" s="203"/>
+      <c r="D56" s="203"/>
+      <c r="E56" s="203"/>
+      <c r="F56" s="203"/>
+      <c r="G56" s="203"/>
+      <c r="H56" s="203"/>
+      <c r="I56" s="203"/>
       <c r="J56" s="107"/>
       <c r="K56" s="142"/>
       <c r="L56" s="143"/>
     </row>
     <row r="57" spans="2:12" ht="15.6">
       <c r="B57" s="106"/>
-      <c r="C57" s="245"/>
-      <c r="D57" s="245"/>
-      <c r="E57" s="245"/>
-      <c r="F57" s="245"/>
-      <c r="G57" s="245"/>
-      <c r="H57" s="245"/>
-      <c r="I57" s="245"/>
+      <c r="C57" s="203"/>
+      <c r="D57" s="203"/>
+      <c r="E57" s="203"/>
+      <c r="F57" s="203"/>
+      <c r="G57" s="203"/>
+      <c r="H57" s="203"/>
+      <c r="I57" s="203"/>
       <c r="J57" s="107"/>
       <c r="K57" s="140"/>
       <c r="L57" s="141"/>
     </row>
     <row r="58" spans="2:12" ht="15.6">
       <c r="B58" s="106"/>
-      <c r="C58" s="246"/>
-      <c r="D58" s="246"/>
-      <c r="E58" s="246"/>
-      <c r="F58" s="246"/>
-      <c r="G58" s="246"/>
-      <c r="H58" s="246"/>
-      <c r="I58" s="246"/>
+      <c r="C58" s="204"/>
+      <c r="D58" s="204"/>
+      <c r="E58" s="204"/>
+      <c r="F58" s="204"/>
+      <c r="G58" s="204"/>
+      <c r="H58" s="204"/>
+      <c r="I58" s="204"/>
       <c r="J58" s="107"/>
-      <c r="K58" s="174"/>
-      <c r="L58" s="175"/>
+      <c r="K58" s="198"/>
+      <c r="L58" s="199"/>
     </row>
     <row r="59" spans="2:12" ht="15.6">
       <c r="B59" s="106"/>
@@ -42036,103 +41986,103 @@
       <c r="H59" s="110"/>
       <c r="I59" s="110"/>
       <c r="J59" s="107"/>
-      <c r="K59" s="174"/>
-      <c r="L59" s="175"/>
+      <c r="K59" s="198"/>
+      <c r="L59" s="199"/>
     </row>
     <row r="60" spans="2:12" ht="15.6">
-      <c r="B60" s="191" t="s">
+      <c r="B60" s="230" t="s">
         <v>80</v>
       </c>
-      <c r="C60" s="192"/>
-      <c r="D60" s="192"/>
-      <c r="E60" s="193"/>
-      <c r="F60" s="194" t="s">
+      <c r="C60" s="231"/>
+      <c r="D60" s="231"/>
+      <c r="E60" s="232"/>
+      <c r="F60" s="233" t="s">
         <v>81</v>
       </c>
-      <c r="G60" s="193"/>
-      <c r="H60" s="194" t="s">
+      <c r="G60" s="232"/>
+      <c r="H60" s="233" t="s">
         <v>82</v>
       </c>
-      <c r="I60" s="192"/>
-      <c r="J60" s="193"/>
+      <c r="I60" s="231"/>
+      <c r="J60" s="232"/>
       <c r="K60" s="108"/>
       <c r="L60" s="109"/>
     </row>
     <row r="61" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B61" s="216"/>
-      <c r="C61" s="217"/>
-      <c r="D61" s="217"/>
-      <c r="E61" s="211"/>
-      <c r="F61" s="210"/>
-      <c r="G61" s="211"/>
-      <c r="H61" s="195"/>
-      <c r="I61" s="196"/>
-      <c r="J61" s="197"/>
+      <c r="B61" s="255"/>
+      <c r="C61" s="256"/>
+      <c r="D61" s="256"/>
+      <c r="E61" s="250"/>
+      <c r="F61" s="249"/>
+      <c r="G61" s="250"/>
+      <c r="H61" s="234"/>
+      <c r="I61" s="235"/>
+      <c r="J61" s="236"/>
       <c r="K61" s="108"/>
       <c r="L61" s="109"/>
     </row>
     <row r="62" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B62" s="218"/>
-      <c r="C62" s="219"/>
-      <c r="D62" s="219"/>
-      <c r="E62" s="213"/>
-      <c r="F62" s="212"/>
-      <c r="G62" s="213"/>
-      <c r="H62" s="198"/>
-      <c r="I62" s="199"/>
-      <c r="J62" s="200"/>
+      <c r="B62" s="257"/>
+      <c r="C62" s="258"/>
+      <c r="D62" s="258"/>
+      <c r="E62" s="252"/>
+      <c r="F62" s="251"/>
+      <c r="G62" s="252"/>
+      <c r="H62" s="237"/>
+      <c r="I62" s="238"/>
+      <c r="J62" s="239"/>
       <c r="K62" s="117"/>
       <c r="L62" s="109"/>
     </row>
     <row r="63" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B63" s="218"/>
-      <c r="C63" s="219"/>
-      <c r="D63" s="219"/>
-      <c r="E63" s="213"/>
-      <c r="F63" s="212"/>
-      <c r="G63" s="213"/>
-      <c r="H63" s="198"/>
-      <c r="I63" s="199"/>
-      <c r="J63" s="200"/>
+      <c r="B63" s="257"/>
+      <c r="C63" s="258"/>
+      <c r="D63" s="258"/>
+      <c r="E63" s="252"/>
+      <c r="F63" s="251"/>
+      <c r="G63" s="252"/>
+      <c r="H63" s="237"/>
+      <c r="I63" s="238"/>
+      <c r="J63" s="239"/>
       <c r="K63" s="116"/>
       <c r="L63" s="76"/>
     </row>
     <row r="64" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B64" s="218"/>
-      <c r="C64" s="219"/>
-      <c r="D64" s="219"/>
-      <c r="E64" s="213"/>
-      <c r="F64" s="212"/>
-      <c r="G64" s="213"/>
-      <c r="H64" s="198"/>
-      <c r="I64" s="199"/>
-      <c r="J64" s="200"/>
+      <c r="B64" s="257"/>
+      <c r="C64" s="258"/>
+      <c r="D64" s="258"/>
+      <c r="E64" s="252"/>
+      <c r="F64" s="251"/>
+      <c r="G64" s="252"/>
+      <c r="H64" s="237"/>
+      <c r="I64" s="238"/>
+      <c r="J64" s="239"/>
       <c r="K64" s="118"/>
       <c r="L64" s="119"/>
     </row>
     <row r="65" spans="2:12" ht="15.6" customHeight="1">
-      <c r="B65" s="218"/>
-      <c r="C65" s="219"/>
-      <c r="D65" s="219"/>
-      <c r="E65" s="213"/>
-      <c r="F65" s="212"/>
-      <c r="G65" s="213"/>
-      <c r="H65" s="198"/>
-      <c r="I65" s="199"/>
-      <c r="J65" s="200"/>
+      <c r="B65" s="257"/>
+      <c r="C65" s="258"/>
+      <c r="D65" s="258"/>
+      <c r="E65" s="252"/>
+      <c r="F65" s="251"/>
+      <c r="G65" s="252"/>
+      <c r="H65" s="237"/>
+      <c r="I65" s="238"/>
+      <c r="J65" s="239"/>
       <c r="K65" s="118"/>
       <c r="L65" s="119"/>
     </row>
     <row r="66" spans="2:12" ht="16.2" customHeight="1" thickBot="1">
-      <c r="B66" s="220"/>
-      <c r="C66" s="221"/>
-      <c r="D66" s="221"/>
-      <c r="E66" s="215"/>
-      <c r="F66" s="214"/>
-      <c r="G66" s="215"/>
-      <c r="H66" s="201"/>
-      <c r="I66" s="202"/>
-      <c r="J66" s="203"/>
+      <c r="B66" s="259"/>
+      <c r="C66" s="260"/>
+      <c r="D66" s="260"/>
+      <c r="E66" s="254"/>
+      <c r="F66" s="253"/>
+      <c r="G66" s="254"/>
+      <c r="H66" s="240"/>
+      <c r="I66" s="241"/>
+      <c r="J66" s="242"/>
       <c r="K66" s="111"/>
       <c r="L66" s="112"/>
     </row>
@@ -42143,12 +42093,55 @@
     </row>
   </sheetData>
   <mergeCells count="71">
-    <mergeCell ref="B1:L1"/>
-    <mergeCell ref="B2:I3"/>
-    <mergeCell ref="J2:L6"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="K59:L59"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C44:I44"/>
+    <mergeCell ref="C45:I45"/>
+    <mergeCell ref="C46:I46"/>
+    <mergeCell ref="C47:I47"/>
+    <mergeCell ref="C48:I48"/>
+    <mergeCell ref="C39:I39"/>
+    <mergeCell ref="C40:I40"/>
+    <mergeCell ref="C41:I41"/>
+    <mergeCell ref="C42:I42"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="C36:I36"/>
+    <mergeCell ref="C37:I37"/>
+    <mergeCell ref="C38:I38"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="H60:J60"/>
+    <mergeCell ref="H61:J66"/>
+    <mergeCell ref="B49:J50"/>
+    <mergeCell ref="F61:G66"/>
+    <mergeCell ref="B61:E66"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
     <mergeCell ref="C24:I25"/>
     <mergeCell ref="J24:L24"/>
     <mergeCell ref="K58:L58"/>
@@ -42165,58 +42158,15 @@
     <mergeCell ref="C32:I32"/>
     <mergeCell ref="C33:I33"/>
     <mergeCell ref="C43:I43"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="H60:J60"/>
-    <mergeCell ref="H61:J66"/>
-    <mergeCell ref="B49:J50"/>
-    <mergeCell ref="F61:G66"/>
-    <mergeCell ref="B61:E66"/>
-    <mergeCell ref="C34:I34"/>
-    <mergeCell ref="C35:I35"/>
-    <mergeCell ref="C36:I36"/>
-    <mergeCell ref="C37:I37"/>
-    <mergeCell ref="C38:I38"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="K59:L59"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C44:I44"/>
-    <mergeCell ref="C45:I45"/>
-    <mergeCell ref="C46:I46"/>
-    <mergeCell ref="C47:I47"/>
-    <mergeCell ref="C48:I48"/>
-    <mergeCell ref="C39:I39"/>
-    <mergeCell ref="C40:I40"/>
-    <mergeCell ref="C41:I41"/>
-    <mergeCell ref="C42:I42"/>
+    <mergeCell ref="B1:L1"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="J2:L6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="K10:L10"/>
   </mergeCells>
   <conditionalFormatting sqref="B26:L48">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>AND($B26&lt;&gt;"",$J26="",$L26&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -42911,7 +42861,7 @@
     <mergeCell ref="I4:P5"/>
   </mergeCells>
   <conditionalFormatting sqref="J13 L13 N13 B15:P49">
-    <cfRule type="expression" dxfId="6" priority="13">
+    <cfRule type="expression" dxfId="1" priority="13">
       <formula>AND($B13&lt;&gt;"",$C13&lt;&gt;"",$J13="")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>